<commit_message>
Add missing Harry Potter films (card_309-315)
All 7 theatrical Harry Potter films, scraped director/budget/box
office/runtime/oscars from Wikipedia, Letterboxd + Metacritic user
ratings, and Wikidata genres. First batch of a larger pass adding
missing movies across franchise/director lists.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P309"/>
+  <dimension ref="A1:P316"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -17145,6 +17145,356 @@
         <v>0</v>
       </c>
     </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Philosopher's Stone</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>card_309</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Chris Columbus</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E310" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F310" t="n">
+        <v>79</v>
+      </c>
+      <c r="I310" t="n">
+        <v>1029000000</v>
+      </c>
+      <c r="J310" t="b">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L310" t="b">
+        <v>0</v>
+      </c>
+      <c r="M310" t="n">
+        <v>152</v>
+      </c>
+      <c r="N310" t="n">
+        <v>0</v>
+      </c>
+      <c r="O310" t="n">
+        <v>0</v>
+      </c>
+      <c r="P310" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Chamber of Secrets</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>card_310</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Chris Columbus</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E311" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F311" t="n">
+        <v>77</v>
+      </c>
+      <c r="I311" t="n">
+        <v>883400000</v>
+      </c>
+      <c r="J311" t="b">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L311" t="b">
+        <v>0</v>
+      </c>
+      <c r="M311" t="n">
+        <v>161</v>
+      </c>
+      <c r="N311" t="n">
+        <v>0</v>
+      </c>
+      <c r="O311" t="n">
+        <v>0</v>
+      </c>
+      <c r="P311" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Goblet of Fire</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>card_311</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Mike Newell</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E312" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F312" t="n">
+        <v>79</v>
+      </c>
+      <c r="I312" t="n">
+        <v>900400000</v>
+      </c>
+      <c r="J312" t="b">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L312" t="b">
+        <v>0</v>
+      </c>
+      <c r="M312" t="n">
+        <v>157</v>
+      </c>
+      <c r="N312" t="n">
+        <v>0</v>
+      </c>
+      <c r="O312" t="n">
+        <v>0</v>
+      </c>
+      <c r="P312" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Order of the Phoenix</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>card_312</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>David Yates</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E313" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F313" t="n">
+        <v>75</v>
+      </c>
+      <c r="I313" t="n">
+        <v>942900000</v>
+      </c>
+      <c r="J313" t="b">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L313" t="b">
+        <v>1</v>
+      </c>
+      <c r="M313" t="n">
+        <v>138</v>
+      </c>
+      <c r="N313" t="n">
+        <v>0</v>
+      </c>
+      <c r="O313" t="n">
+        <v>0</v>
+      </c>
+      <c r="P313" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Half-Blood Prince</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>card_313</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>David Yates</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E314" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F314" t="n">
+        <v>76</v>
+      </c>
+      <c r="I314" t="n">
+        <v>941100000</v>
+      </c>
+      <c r="J314" t="b">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="L314" t="b">
+        <v>0</v>
+      </c>
+      <c r="M314" t="n">
+        <v>153</v>
+      </c>
+      <c r="N314" t="n">
+        <v>0</v>
+      </c>
+      <c r="O314" t="n">
+        <v>0</v>
+      </c>
+      <c r="P314" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Deathly Hallows: Part 1</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>card_314</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>David Yates</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E315" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F315" t="n">
+        <v>76</v>
+      </c>
+      <c r="I315" t="n">
+        <v>991200000</v>
+      </c>
+      <c r="J315" t="b">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L315" t="b">
+        <v>1</v>
+      </c>
+      <c r="M315" t="n">
+        <v>146</v>
+      </c>
+      <c r="N315" t="n">
+        <v>0</v>
+      </c>
+      <c r="O315" t="n">
+        <v>0</v>
+      </c>
+      <c r="P315" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Harry Potter and the Deathly Hallows: Part 2</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>card_315</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>David Yates</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E316" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F316" t="n">
+        <v>83</v>
+      </c>
+      <c r="I316" t="n">
+        <v>1380000000</v>
+      </c>
+      <c r="J316" t="b">
+        <v>0</v>
+      </c>
+      <c r="K316" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L316" t="b">
+        <v>1</v>
+      </c>
+      <c r="M316" t="n">
+        <v>130</v>
+      </c>
+      <c r="N316" t="n">
+        <v>0</v>
+      </c>
+      <c r="O316" t="n">
+        <v>0</v>
+      </c>
+      <c r="P316" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Add Warcraft, Ocean's trilogy, Highlander, Twilight, Fifty Shades, Die Hard (card_316-336)
21 films scraped from Wikipedia/Letterboxd/Metacritic/Wikidata. Second
batch of the missing-movies pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P316"/>
+  <dimension ref="A1:P337"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -17146,352 +17146,1402 @@
       </c>
     </row>
     <row r="310">
-      <c r="A310" t="inlineStr">
+      <c r="A310" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Philosopher's Stone</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
+      <c r="B310" s="10" t="inlineStr">
         <is>
           <t>card_309</t>
         </is>
       </c>
-      <c r="C310" t="inlineStr">
+      <c r="C310" s="10" t="inlineStr">
         <is>
           <t>Chris Columbus</t>
         </is>
       </c>
-      <c r="D310" t="n">
+      <c r="D310" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E310" t="n">
+      <c r="E310" s="10" t="n">
         <v>3.84</v>
       </c>
-      <c r="F310" t="n">
+      <c r="F310" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I310" t="n">
+      <c r="I310" s="10" t="n">
         <v>1029000000</v>
       </c>
-      <c r="J310" t="b">
-        <v>0</v>
-      </c>
-      <c r="K310" t="n">
+      <c r="J310" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K310" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L310" t="b">
-        <v>0</v>
-      </c>
-      <c r="M310" t="n">
+      <c r="L310" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M310" s="10" t="n">
         <v>152</v>
       </c>
-      <c r="N310" t="n">
-        <v>0</v>
-      </c>
-      <c r="O310" t="n">
-        <v>0</v>
-      </c>
-      <c r="P310" t="b">
+      <c r="N310" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O310" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P310" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="311">
-      <c r="A311" t="inlineStr">
+      <c r="A311" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Chamber of Secrets</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
+      <c r="B311" s="10" t="inlineStr">
         <is>
           <t>card_310</t>
         </is>
       </c>
-      <c r="C311" t="inlineStr">
+      <c r="C311" s="10" t="inlineStr">
         <is>
           <t>Chris Columbus</t>
         </is>
       </c>
-      <c r="D311" t="n">
+      <c r="D311" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E311" t="n">
+      <c r="E311" s="10" t="n">
         <v>3.65</v>
       </c>
-      <c r="F311" t="n">
+      <c r="F311" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I311" t="n">
+      <c r="I311" s="10" t="n">
         <v>883400000</v>
       </c>
-      <c r="J311" t="b">
-        <v>0</v>
-      </c>
-      <c r="K311" t="n">
+      <c r="J311" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K311" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L311" t="b">
-        <v>0</v>
-      </c>
-      <c r="M311" t="n">
+      <c r="L311" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M311" s="10" t="n">
         <v>161</v>
       </c>
-      <c r="N311" t="n">
-        <v>0</v>
-      </c>
-      <c r="O311" t="n">
-        <v>0</v>
-      </c>
-      <c r="P311" t="b">
+      <c r="N311" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O311" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P311" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="312">
-      <c r="A312" t="inlineStr">
+      <c r="A312" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Goblet of Fire</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr">
+      <c r="B312" s="10" t="inlineStr">
         <is>
           <t>card_311</t>
         </is>
       </c>
-      <c r="C312" t="inlineStr">
+      <c r="C312" s="10" t="inlineStr">
         <is>
           <t>Mike Newell</t>
         </is>
       </c>
-      <c r="D312" t="n">
+      <c r="D312" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E312" t="n">
+      <c r="E312" s="10" t="n">
         <v>3.9</v>
       </c>
-      <c r="F312" t="n">
+      <c r="F312" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I312" t="n">
+      <c r="I312" s="10" t="n">
         <v>900400000</v>
       </c>
-      <c r="J312" t="b">
-        <v>0</v>
-      </c>
-      <c r="K312" t="n">
+      <c r="J312" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K312" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L312" t="b">
-        <v>0</v>
-      </c>
-      <c r="M312" t="n">
+      <c r="L312" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M312" s="10" t="n">
         <v>157</v>
       </c>
-      <c r="N312" t="n">
-        <v>0</v>
-      </c>
-      <c r="O312" t="n">
-        <v>0</v>
-      </c>
-      <c r="P312" t="b">
+      <c r="N312" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O312" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P312" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="313">
-      <c r="A313" t="inlineStr">
+      <c r="A313" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Order of the Phoenix</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr">
+      <c r="B313" s="10" t="inlineStr">
         <is>
           <t>card_312</t>
         </is>
       </c>
-      <c r="C313" t="inlineStr">
+      <c r="C313" s="10" t="inlineStr">
         <is>
           <t>David Yates</t>
         </is>
       </c>
-      <c r="D313" t="n">
+      <c r="D313" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E313" t="n">
+      <c r="E313" s="10" t="n">
         <v>3.72</v>
       </c>
-      <c r="F313" t="n">
+      <c r="F313" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I313" t="n">
+      <c r="I313" s="10" t="n">
         <v>942900000</v>
       </c>
-      <c r="J313" t="b">
-        <v>0</v>
-      </c>
-      <c r="K313" t="n">
+      <c r="J313" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K313" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L313" t="b">
+      <c r="L313" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M313" t="n">
+      <c r="M313" s="10" t="n">
         <v>138</v>
       </c>
-      <c r="N313" t="n">
-        <v>0</v>
-      </c>
-      <c r="O313" t="n">
-        <v>0</v>
-      </c>
-      <c r="P313" t="b">
+      <c r="N313" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O313" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P313" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="314">
-      <c r="A314" t="inlineStr">
+      <c r="A314" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Half-Blood Prince</t>
         </is>
       </c>
-      <c r="B314" t="inlineStr">
+      <c r="B314" s="10" t="inlineStr">
         <is>
           <t>card_313</t>
         </is>
       </c>
-      <c r="C314" t="inlineStr">
+      <c r="C314" s="10" t="inlineStr">
         <is>
           <t>David Yates</t>
         </is>
       </c>
-      <c r="D314" t="n">
+      <c r="D314" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E314" t="n">
+      <c r="E314" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F314" t="n">
+      <c r="F314" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I314" t="n">
+      <c r="I314" s="10" t="n">
         <v>941100000</v>
       </c>
-      <c r="J314" t="b">
-        <v>0</v>
-      </c>
-      <c r="K314" t="n">
+      <c r="J314" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K314" s="10" t="n">
         <v>250000000</v>
       </c>
-      <c r="L314" t="b">
-        <v>0</v>
-      </c>
-      <c r="M314" t="n">
+      <c r="L314" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M314" s="10" t="n">
         <v>153</v>
       </c>
-      <c r="N314" t="n">
-        <v>0</v>
-      </c>
-      <c r="O314" t="n">
-        <v>0</v>
-      </c>
-      <c r="P314" t="b">
+      <c r="N314" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O314" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P314" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="315">
-      <c r="A315" t="inlineStr">
+      <c r="A315" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Deathly Hallows: Part 1</t>
         </is>
       </c>
-      <c r="B315" t="inlineStr">
+      <c r="B315" s="10" t="inlineStr">
         <is>
           <t>card_314</t>
         </is>
       </c>
-      <c r="C315" t="inlineStr">
+      <c r="C315" s="10" t="inlineStr">
         <is>
           <t>David Yates</t>
         </is>
       </c>
-      <c r="D315" t="n">
+      <c r="D315" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E315" t="n">
+      <c r="E315" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F315" t="n">
+      <c r="F315" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I315" t="n">
+      <c r="I315" s="10" t="n">
         <v>991200000</v>
       </c>
-      <c r="J315" t="b">
-        <v>0</v>
-      </c>
-      <c r="K315" t="n">
+      <c r="J315" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K315" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L315" t="b">
+      <c r="L315" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M315" t="n">
+      <c r="M315" s="10" t="n">
         <v>146</v>
       </c>
-      <c r="N315" t="n">
-        <v>0</v>
-      </c>
-      <c r="O315" t="n">
-        <v>0</v>
-      </c>
-      <c r="P315" t="b">
+      <c r="N315" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O315" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P315" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="316">
-      <c r="A316" t="inlineStr">
+      <c r="A316" s="10" t="inlineStr">
         <is>
           <t>Harry Potter and the Deathly Hallows: Part 2</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr">
+      <c r="B316" s="10" t="inlineStr">
         <is>
           <t>card_315</t>
         </is>
       </c>
-      <c r="C316" t="inlineStr">
+      <c r="C316" s="10" t="inlineStr">
         <is>
           <t>David Yates</t>
         </is>
       </c>
-      <c r="D316" t="n">
+      <c r="D316" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E316" t="n">
+      <c r="E316" s="10" t="n">
         <v>4.04</v>
       </c>
-      <c r="F316" t="n">
+      <c r="F316" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I316" t="n">
+      <c r="I316" s="10" t="n">
         <v>1380000000</v>
       </c>
-      <c r="J316" t="b">
-        <v>0</v>
-      </c>
-      <c r="K316" t="n">
+      <c r="J316" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K316" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L316" t="b">
+      <c r="L316" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M316" t="n">
+      <c r="M316" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N316" t="n">
-        <v>0</v>
-      </c>
-      <c r="O316" t="n">
-        <v>0</v>
-      </c>
-      <c r="P316" t="b">
+      <c r="N316" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O316" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P316" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Warcraft</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>card_316</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Duncan Jones</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E317" t="n">
+        <v>2.57</v>
+      </c>
+      <c r="F317" t="n">
+        <v>81</v>
+      </c>
+      <c r="I317" t="n">
+        <v>439100000</v>
+      </c>
+      <c r="J317" t="b">
+        <v>0</v>
+      </c>
+      <c r="K317" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L317" t="b">
+        <v>0</v>
+      </c>
+      <c r="M317" t="n">
+        <v>123</v>
+      </c>
+      <c r="N317" t="n">
+        <v>0</v>
+      </c>
+      <c r="O317" t="n">
+        <v>0</v>
+      </c>
+      <c r="P317" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Ocean's Eleven</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>card_317</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Steven Soderbergh</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E318" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="F318" t="n">
+        <v>80</v>
+      </c>
+      <c r="I318" t="n">
+        <v>450700000</v>
+      </c>
+      <c r="J318" t="b">
+        <v>0</v>
+      </c>
+      <c r="K318" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="L318" t="b">
+        <v>0</v>
+      </c>
+      <c r="M318" t="n">
+        <v>116</v>
+      </c>
+      <c r="N318" t="n">
+        <v>0</v>
+      </c>
+      <c r="O318" t="n">
+        <v>0</v>
+      </c>
+      <c r="P318" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Ocean's Twelve</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>card_318</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Steven Soderbergh</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E319" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="F319" t="n">
+        <v>62</v>
+      </c>
+      <c r="I319" t="n">
+        <v>362900000</v>
+      </c>
+      <c r="J319" t="b">
+        <v>0</v>
+      </c>
+      <c r="K319" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L319" t="b">
+        <v>0</v>
+      </c>
+      <c r="M319" t="n">
+        <v>125</v>
+      </c>
+      <c r="N319" t="n">
+        <v>0</v>
+      </c>
+      <c r="O319" t="n">
+        <v>0</v>
+      </c>
+      <c r="P319" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Ocean's Thirteen</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>card_319</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Steven Soderbergh</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E320" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="F320" t="n">
+        <v>69</v>
+      </c>
+      <c r="I320" t="n">
+        <v>311700000</v>
+      </c>
+      <c r="J320" t="b">
+        <v>0</v>
+      </c>
+      <c r="K320" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="L320" t="b">
+        <v>0</v>
+      </c>
+      <c r="M320" t="n">
+        <v>122</v>
+      </c>
+      <c r="N320" t="n">
+        <v>0</v>
+      </c>
+      <c r="O320" t="n">
+        <v>0</v>
+      </c>
+      <c r="P320" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Highlander</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>card_320</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Russell Mulcahy</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>1986</v>
+      </c>
+      <c r="E321" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="F321" t="n">
+        <v>74</v>
+      </c>
+      <c r="I321" t="n">
+        <v>12800000</v>
+      </c>
+      <c r="J321" t="b">
+        <v>0</v>
+      </c>
+      <c r="K321" t="n">
+        <v>19000000</v>
+      </c>
+      <c r="L321" t="b">
+        <v>0</v>
+      </c>
+      <c r="M321" t="n">
+        <v>111</v>
+      </c>
+      <c r="N321" t="n">
+        <v>0</v>
+      </c>
+      <c r="O321" t="n">
+        <v>0</v>
+      </c>
+      <c r="P321" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Highlander II: The Quickening</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>card_321</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Russell Mulcahy</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>1991</v>
+      </c>
+      <c r="E322" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="F322" t="n">
+        <v>53</v>
+      </c>
+      <c r="I322" t="n">
+        <v>15600000</v>
+      </c>
+      <c r="J322" t="b">
+        <v>1</v>
+      </c>
+      <c r="K322" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="L322" t="b">
+        <v>0</v>
+      </c>
+      <c r="M322" t="n">
+        <v>100</v>
+      </c>
+      <c r="N322" t="n">
+        <v>0</v>
+      </c>
+      <c r="O322" t="n">
+        <v>0</v>
+      </c>
+      <c r="P322" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Highlander III: The Sorcerer</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>card_322</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Andy Morahan</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E323" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F323" t="n">
+        <v>67</v>
+      </c>
+      <c r="I323" t="n">
+        <v>36700000</v>
+      </c>
+      <c r="J323" t="b">
+        <v>0</v>
+      </c>
+      <c r="K323" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L323" t="b">
+        <v>1</v>
+      </c>
+      <c r="M323" t="n">
+        <v>95</v>
+      </c>
+      <c r="N323" t="n">
+        <v>0</v>
+      </c>
+      <c r="O323" t="n">
+        <v>0</v>
+      </c>
+      <c r="P323" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Highlander: Endgame</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>card_323</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Doug Aarniokoski</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E324" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F324" t="n">
+        <v>53</v>
+      </c>
+      <c r="I324" t="n">
+        <v>15800000</v>
+      </c>
+      <c r="J324" t="b">
+        <v>0</v>
+      </c>
+      <c r="K324" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="L324" t="b">
+        <v>0</v>
+      </c>
+      <c r="M324" t="n">
+        <v>87</v>
+      </c>
+      <c r="N324" t="n">
+        <v>0</v>
+      </c>
+      <c r="O324" t="n">
+        <v>0</v>
+      </c>
+      <c r="P324" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Twilight</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>card_324</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Catherine Hardwicke</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E325" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="F325" t="n">
+        <v>42</v>
+      </c>
+      <c r="I325" t="n">
+        <v>412000000</v>
+      </c>
+      <c r="J325" t="b">
+        <v>0</v>
+      </c>
+      <c r="K325" t="n">
+        <v>37000000</v>
+      </c>
+      <c r="L325" t="b">
+        <v>0</v>
+      </c>
+      <c r="M325" t="n">
+        <v>121</v>
+      </c>
+      <c r="N325" t="n">
+        <v>0</v>
+      </c>
+      <c r="O325" t="n">
+        <v>0</v>
+      </c>
+      <c r="P325" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>The Twilight Saga: New Moon</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>card_325</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Chris Weitz</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E326" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="F326" t="n">
+        <v>39</v>
+      </c>
+      <c r="I326" t="n">
+        <v>712000000</v>
+      </c>
+      <c r="J326" t="b">
+        <v>0</v>
+      </c>
+      <c r="K326" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="L326" t="b">
+        <v>0</v>
+      </c>
+      <c r="M326" t="n">
+        <v>130</v>
+      </c>
+      <c r="N326" t="n">
+        <v>0</v>
+      </c>
+      <c r="O326" t="n">
+        <v>0</v>
+      </c>
+      <c r="P326" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>The Twilight Saga: Eclipse</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>card_326</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>David Slade</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E327" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F327" t="n">
+        <v>48</v>
+      </c>
+      <c r="I327" t="n">
+        <v>699000000</v>
+      </c>
+      <c r="J327" t="b">
+        <v>0</v>
+      </c>
+      <c r="K327" t="n">
+        <v>68000000</v>
+      </c>
+      <c r="L327" t="b">
+        <v>0</v>
+      </c>
+      <c r="M327" t="n">
+        <v>124</v>
+      </c>
+      <c r="N327" t="n">
+        <v>0</v>
+      </c>
+      <c r="O327" t="n">
+        <v>0</v>
+      </c>
+      <c r="P327" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>The Twilight Saga: Breaking Dawn - Part 1</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>card_327</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Bill Condon</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E328" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F328" t="n">
+        <v>43</v>
+      </c>
+      <c r="I328" t="n">
+        <v>732000000</v>
+      </c>
+      <c r="J328" t="b">
+        <v>0</v>
+      </c>
+      <c r="K328" t="n">
+        <v>127000000</v>
+      </c>
+      <c r="L328" t="b">
+        <v>0</v>
+      </c>
+      <c r="M328" t="n">
+        <v>117</v>
+      </c>
+      <c r="N328" t="n">
+        <v>0</v>
+      </c>
+      <c r="O328" t="n">
+        <v>0</v>
+      </c>
+      <c r="P328" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>The Twilight Saga: Breaking Dawn - Part 2</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>card_328</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Bill Condon</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E329" t="n">
+        <v>3.01</v>
+      </c>
+      <c r="F329" t="n">
+        <v>45</v>
+      </c>
+      <c r="I329" t="n">
+        <v>868000000</v>
+      </c>
+      <c r="J329" t="b">
+        <v>0</v>
+      </c>
+      <c r="K329" t="n">
+        <v>136000000</v>
+      </c>
+      <c r="L329" t="b">
+        <v>0</v>
+      </c>
+      <c r="M329" t="n">
+        <v>115</v>
+      </c>
+      <c r="N329" t="n">
+        <v>0</v>
+      </c>
+      <c r="O329" t="n">
+        <v>0</v>
+      </c>
+      <c r="P329" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Fifty Shades of Grey</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>card_329</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Sam Taylor-Johnson</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E330" t="n">
+        <v>1.88</v>
+      </c>
+      <c r="F330" t="n">
+        <v>33</v>
+      </c>
+      <c r="I330" t="n">
+        <v>569700000</v>
+      </c>
+      <c r="J330" t="b">
+        <v>0</v>
+      </c>
+      <c r="K330" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L330" t="b">
+        <v>0</v>
+      </c>
+      <c r="M330" t="n">
+        <v>125</v>
+      </c>
+      <c r="N330" t="n">
+        <v>0</v>
+      </c>
+      <c r="O330" t="n">
+        <v>0</v>
+      </c>
+      <c r="P330" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Fifty Shades Darker</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>card_330</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>James Foley</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E331" t="n">
+        <v>2.09</v>
+      </c>
+      <c r="F331" t="n">
+        <v>32</v>
+      </c>
+      <c r="I331" t="n">
+        <v>381000000</v>
+      </c>
+      <c r="J331" t="b">
+        <v>0</v>
+      </c>
+      <c r="K331" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="L331" t="b">
+        <v>0</v>
+      </c>
+      <c r="M331" t="n">
+        <v>118</v>
+      </c>
+      <c r="N331" t="n">
+        <v>0</v>
+      </c>
+      <c r="O331" t="n">
+        <v>0</v>
+      </c>
+      <c r="P331" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Fifty Shades Freed</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>card_331</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>James Foley</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E332" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="F332" t="n">
+        <v>35</v>
+      </c>
+      <c r="I332" t="n">
+        <v>372000000</v>
+      </c>
+      <c r="J332" t="b">
+        <v>0</v>
+      </c>
+      <c r="K332" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="L332" t="b">
+        <v>0</v>
+      </c>
+      <c r="M332" t="n">
+        <v>105</v>
+      </c>
+      <c r="N332" t="n">
+        <v>0</v>
+      </c>
+      <c r="O332" t="n">
+        <v>0</v>
+      </c>
+      <c r="P332" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Die Hard</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>card_332</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>John McTiernan</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E333" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="F333" t="n">
+        <v>86</v>
+      </c>
+      <c r="I333" t="n">
+        <v>141500000</v>
+      </c>
+      <c r="J333" t="b">
+        <v>0</v>
+      </c>
+      <c r="K333" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L333" t="b">
+        <v>1</v>
+      </c>
+      <c r="M333" t="n">
+        <v>132</v>
+      </c>
+      <c r="N333" t="n">
+        <v>0</v>
+      </c>
+      <c r="O333" t="n">
+        <v>0</v>
+      </c>
+      <c r="P333" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Die Hard 2</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>card_333</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Renny Harlin</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E334" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="F334" t="n">
+        <v>73</v>
+      </c>
+      <c r="I334" t="n">
+        <v>240000000</v>
+      </c>
+      <c r="J334" t="b">
+        <v>0</v>
+      </c>
+      <c r="K334" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="L334" t="b">
+        <v>1</v>
+      </c>
+      <c r="M334" t="n">
+        <v>124</v>
+      </c>
+      <c r="N334" t="n">
+        <v>0</v>
+      </c>
+      <c r="O334" t="n">
+        <v>0</v>
+      </c>
+      <c r="P334" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Die Hard with a Vengeance</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>card_334</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>John McTiernan</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E335" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F335" t="n">
+        <v>78</v>
+      </c>
+      <c r="I335" t="n">
+        <v>366000000</v>
+      </c>
+      <c r="J335" t="b">
+        <v>0</v>
+      </c>
+      <c r="K335" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="L335" t="b">
+        <v>0</v>
+      </c>
+      <c r="M335" t="n">
+        <v>128</v>
+      </c>
+      <c r="N335" t="n">
+        <v>0</v>
+      </c>
+      <c r="O335" t="n">
+        <v>0</v>
+      </c>
+      <c r="P335" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Live Free or Die Hard</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>card_335</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Len Wiseman</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E336" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="F336" t="n">
+        <v>73</v>
+      </c>
+      <c r="I336" t="n">
+        <v>383500000</v>
+      </c>
+      <c r="J336" t="b">
+        <v>0</v>
+      </c>
+      <c r="K336" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L336" t="b">
+        <v>0</v>
+      </c>
+      <c r="M336" t="n">
+        <v>128</v>
+      </c>
+      <c r="N336" t="n">
+        <v>0</v>
+      </c>
+      <c r="O336" t="n">
+        <v>0</v>
+      </c>
+      <c r="P336" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>A Good Day to Die Hard</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>card_336</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>John Moore</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E337" t="n">
+        <v>1.87</v>
+      </c>
+      <c r="F337" t="n">
+        <v>44</v>
+      </c>
+      <c r="I337" t="n">
+        <v>304700000</v>
+      </c>
+      <c r="J337" t="b">
+        <v>0</v>
+      </c>
+      <c r="K337" t="n">
+        <v>92000000</v>
+      </c>
+      <c r="L337" t="b">
+        <v>0</v>
+      </c>
+      <c r="M337" t="n">
+        <v>98</v>
+      </c>
+      <c r="N337" t="n">
+        <v>0</v>
+      </c>
+      <c r="O337" t="n">
+        <v>0</v>
+      </c>
+      <c r="P337" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Peter Jackson films (card_337-343)
King Kong, Heavenly Creatures, The Frighteners, Braindead, Bad Taste,
Meet the Feebles, The Lovely Bones. Third batch of the missing-movies
pass. Box office for Braindead/Bad Taste/Meet the Feebles is a rough
estimate (only limited/regional figures are documented for these).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P337"/>
+  <dimension ref="A1:P344"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -17496,1052 +17496,1399 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" t="inlineStr">
+      <c r="A317" s="10" t="inlineStr">
         <is>
           <t>Warcraft</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr">
+      <c r="B317" s="10" t="inlineStr">
         <is>
           <t>card_316</t>
         </is>
       </c>
-      <c r="C317" t="inlineStr">
+      <c r="C317" s="10" t="inlineStr">
         <is>
           <t>Duncan Jones</t>
         </is>
       </c>
-      <c r="D317" t="n">
+      <c r="D317" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E317" t="n">
+      <c r="E317" s="10" t="n">
         <v>2.57</v>
       </c>
-      <c r="F317" t="n">
+      <c r="F317" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I317" t="n">
+      <c r="I317" s="10" t="n">
         <v>439100000</v>
       </c>
-      <c r="J317" t="b">
-        <v>0</v>
-      </c>
-      <c r="K317" t="n">
+      <c r="J317" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K317" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L317" t="b">
-        <v>0</v>
-      </c>
-      <c r="M317" t="n">
+      <c r="L317" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M317" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="N317" t="n">
-        <v>0</v>
-      </c>
-      <c r="O317" t="n">
-        <v>0</v>
-      </c>
-      <c r="P317" t="b">
+      <c r="N317" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O317" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P317" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="318">
-      <c r="A318" t="inlineStr">
+      <c r="A318" s="10" t="inlineStr">
         <is>
           <t>Ocean's Eleven</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
+      <c r="B318" s="10" t="inlineStr">
         <is>
           <t>card_317</t>
         </is>
       </c>
-      <c r="C318" t="inlineStr">
+      <c r="C318" s="10" t="inlineStr">
         <is>
           <t>Steven Soderbergh</t>
         </is>
       </c>
-      <c r="D318" t="n">
+      <c r="D318" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E318" t="n">
+      <c r="E318" s="10" t="n">
         <v>3.07</v>
       </c>
-      <c r="F318" t="n">
+      <c r="F318" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I318" t="n">
+      <c r="I318" s="10" t="n">
         <v>450700000</v>
       </c>
-      <c r="J318" t="b">
-        <v>0</v>
-      </c>
-      <c r="K318" t="n">
+      <c r="J318" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K318" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="L318" t="b">
-        <v>0</v>
-      </c>
-      <c r="M318" t="n">
+      <c r="L318" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M318" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="N318" t="n">
-        <v>0</v>
-      </c>
-      <c r="O318" t="n">
-        <v>0</v>
-      </c>
-      <c r="P318" t="b">
+      <c r="N318" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O318" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P318" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="319">
-      <c r="A319" t="inlineStr">
+      <c r="A319" s="10" t="inlineStr">
         <is>
           <t>Ocean's Twelve</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
+      <c r="B319" s="10" t="inlineStr">
         <is>
           <t>card_318</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr">
+      <c r="C319" s="10" t="inlineStr">
         <is>
           <t>Steven Soderbergh</t>
         </is>
       </c>
-      <c r="D319" t="n">
+      <c r="D319" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E319" t="n">
+      <c r="E319" s="10" t="n">
         <v>3.39</v>
       </c>
-      <c r="F319" t="n">
+      <c r="F319" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I319" t="n">
+      <c r="I319" s="10" t="n">
         <v>362900000</v>
       </c>
-      <c r="J319" t="b">
-        <v>0</v>
-      </c>
-      <c r="K319" t="n">
+      <c r="J319" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K319" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L319" t="b">
-        <v>0</v>
-      </c>
-      <c r="M319" t="n">
+      <c r="L319" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M319" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="N319" t="n">
-        <v>0</v>
-      </c>
-      <c r="O319" t="n">
-        <v>0</v>
-      </c>
-      <c r="P319" t="b">
+      <c r="N319" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O319" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P319" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="320">
-      <c r="A320" t="inlineStr">
+      <c r="A320" s="10" t="inlineStr">
         <is>
           <t>Ocean's Thirteen</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
+      <c r="B320" s="10" t="inlineStr">
         <is>
           <t>card_319</t>
         </is>
       </c>
-      <c r="C320" t="inlineStr">
+      <c r="C320" s="10" t="inlineStr">
         <is>
           <t>Steven Soderbergh</t>
         </is>
       </c>
-      <c r="D320" t="n">
+      <c r="D320" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E320" t="n">
+      <c r="E320" s="10" t="n">
         <v>3.44</v>
       </c>
-      <c r="F320" t="n">
+      <c r="F320" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I320" t="n">
+      <c r="I320" s="10" t="n">
         <v>311700000</v>
       </c>
-      <c r="J320" t="b">
-        <v>0</v>
-      </c>
-      <c r="K320" t="n">
+      <c r="J320" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K320" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="L320" t="b">
-        <v>0</v>
-      </c>
-      <c r="M320" t="n">
+      <c r="L320" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M320" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N320" t="n">
-        <v>0</v>
-      </c>
-      <c r="O320" t="n">
-        <v>0</v>
-      </c>
-      <c r="P320" t="b">
+      <c r="N320" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O320" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P320" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="321">
-      <c r="A321" t="inlineStr">
+      <c r="A321" s="10" t="inlineStr">
         <is>
           <t>Highlander</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
+      <c r="B321" s="10" t="inlineStr">
         <is>
           <t>card_320</t>
         </is>
       </c>
-      <c r="C321" t="inlineStr">
+      <c r="C321" s="10" t="inlineStr">
         <is>
           <t>Russell Mulcahy</t>
         </is>
       </c>
-      <c r="D321" t="n">
+      <c r="D321" s="10" t="n">
         <v>1986</v>
       </c>
-      <c r="E321" t="n">
+      <c r="E321" s="10" t="n">
         <v>3.33</v>
       </c>
-      <c r="F321" t="n">
+      <c r="F321" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I321" t="n">
+      <c r="I321" s="10" t="n">
         <v>12800000</v>
       </c>
-      <c r="J321" t="b">
-        <v>0</v>
-      </c>
-      <c r="K321" t="n">
+      <c r="J321" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K321" s="10" t="n">
         <v>19000000</v>
       </c>
-      <c r="L321" t="b">
-        <v>0</v>
-      </c>
-      <c r="M321" t="n">
+      <c r="L321" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M321" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N321" t="n">
-        <v>0</v>
-      </c>
-      <c r="O321" t="n">
-        <v>0</v>
-      </c>
-      <c r="P321" t="b">
+      <c r="N321" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O321" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P321" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="322">
-      <c r="A322" t="inlineStr">
+      <c r="A322" s="10" t="inlineStr">
         <is>
           <t>Highlander II: The Quickening</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr">
+      <c r="B322" s="10" t="inlineStr">
         <is>
           <t>card_321</t>
         </is>
       </c>
-      <c r="C322" t="inlineStr">
+      <c r="C322" s="10" t="inlineStr">
         <is>
           <t>Russell Mulcahy</t>
         </is>
       </c>
-      <c r="D322" t="n">
+      <c r="D322" s="10" t="n">
         <v>1991</v>
       </c>
-      <c r="E322" t="n">
+      <c r="E322" s="10" t="n">
         <v>2.14</v>
       </c>
-      <c r="F322" t="n">
+      <c r="F322" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="I322" t="n">
+      <c r="I322" s="10" t="n">
         <v>15600000</v>
       </c>
-      <c r="J322" t="b">
+      <c r="J322" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K322" t="n">
+      <c r="K322" s="10" t="n">
         <v>22000000</v>
       </c>
-      <c r="L322" t="b">
-        <v>0</v>
-      </c>
-      <c r="M322" t="n">
+      <c r="L322" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M322" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="N322" t="n">
-        <v>0</v>
-      </c>
-      <c r="O322" t="n">
-        <v>0</v>
-      </c>
-      <c r="P322" t="b">
+      <c r="N322" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O322" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P322" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="323">
-      <c r="A323" t="inlineStr">
+      <c r="A323" s="10" t="inlineStr">
         <is>
           <t>Highlander III: The Sorcerer</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr">
+      <c r="B323" s="10" t="inlineStr">
         <is>
           <t>card_322</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr">
+      <c r="C323" s="10" t="inlineStr">
         <is>
           <t>Andy Morahan</t>
         </is>
       </c>
-      <c r="D323" t="n">
+      <c r="D323" s="10" t="n">
         <v>1994</v>
       </c>
-      <c r="E323" t="n">
+      <c r="E323" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="F323" t="n">
+      <c r="F323" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I323" t="n">
+      <c r="I323" s="10" t="n">
         <v>36700000</v>
       </c>
-      <c r="J323" t="b">
-        <v>0</v>
-      </c>
-      <c r="K323" t="n">
+      <c r="J323" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K323" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L323" t="b">
+      <c r="L323" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M323" t="n">
+      <c r="M323" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N323" t="n">
-        <v>0</v>
-      </c>
-      <c r="O323" t="n">
-        <v>0</v>
-      </c>
-      <c r="P323" t="b">
+      <c r="N323" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O323" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P323" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="324">
-      <c r="A324" t="inlineStr">
+      <c r="A324" s="10" t="inlineStr">
         <is>
           <t>Highlander: Endgame</t>
         </is>
       </c>
-      <c r="B324" t="inlineStr">
+      <c r="B324" s="10" t="inlineStr">
         <is>
           <t>card_323</t>
         </is>
       </c>
-      <c r="C324" t="inlineStr">
+      <c r="C324" s="10" t="inlineStr">
         <is>
           <t>Doug Aarniokoski</t>
         </is>
       </c>
-      <c r="D324" t="n">
+      <c r="D324" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E324" t="n">
+      <c r="E324" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="F324" t="n">
+      <c r="F324" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="I324" t="n">
+      <c r="I324" s="10" t="n">
         <v>15800000</v>
       </c>
-      <c r="J324" t="b">
-        <v>0</v>
-      </c>
-      <c r="K324" t="n">
+      <c r="J324" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K324" s="10" t="n">
         <v>25000000</v>
       </c>
-      <c r="L324" t="b">
-        <v>0</v>
-      </c>
-      <c r="M324" t="n">
+      <c r="L324" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M324" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="N324" t="n">
-        <v>0</v>
-      </c>
-      <c r="O324" t="n">
-        <v>0</v>
-      </c>
-      <c r="P324" t="b">
+      <c r="N324" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O324" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P324" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="325">
-      <c r="A325" t="inlineStr">
+      <c r="A325" s="10" t="inlineStr">
         <is>
           <t>Twilight</t>
         </is>
       </c>
-      <c r="B325" t="inlineStr">
+      <c r="B325" s="10" t="inlineStr">
         <is>
           <t>card_324</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr">
+      <c r="C325" s="10" t="inlineStr">
         <is>
           <t>Catherine Hardwicke</t>
         </is>
       </c>
-      <c r="D325" t="n">
+      <c r="D325" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E325" t="n">
+      <c r="E325" s="10" t="n">
         <v>3.11</v>
       </c>
-      <c r="F325" t="n">
+      <c r="F325" s="10" t="n">
         <v>42</v>
       </c>
-      <c r="I325" t="n">
+      <c r="I325" s="10" t="n">
         <v>412000000</v>
       </c>
-      <c r="J325" t="b">
-        <v>0</v>
-      </c>
-      <c r="K325" t="n">
+      <c r="J325" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K325" s="10" t="n">
         <v>37000000</v>
       </c>
-      <c r="L325" t="b">
-        <v>0</v>
-      </c>
-      <c r="M325" t="n">
+      <c r="L325" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M325" s="10" t="n">
         <v>121</v>
       </c>
-      <c r="N325" t="n">
-        <v>0</v>
-      </c>
-      <c r="O325" t="n">
-        <v>0</v>
-      </c>
-      <c r="P325" t="b">
+      <c r="N325" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O325" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P325" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="326">
-      <c r="A326" t="inlineStr">
+      <c r="A326" s="10" t="inlineStr">
         <is>
           <t>The Twilight Saga: New Moon</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr">
+      <c r="B326" s="10" t="inlineStr">
         <is>
           <t>card_325</t>
         </is>
       </c>
-      <c r="C326" t="inlineStr">
+      <c r="C326" s="10" t="inlineStr">
         <is>
           <t>Chris Weitz</t>
         </is>
       </c>
-      <c r="D326" t="n">
+      <c r="D326" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E326" t="n">
+      <c r="E326" s="10" t="n">
         <v>2.82</v>
       </c>
-      <c r="F326" t="n">
+      <c r="F326" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="I326" t="n">
+      <c r="I326" s="10" t="n">
         <v>712000000</v>
       </c>
-      <c r="J326" t="b">
-        <v>0</v>
-      </c>
-      <c r="K326" t="n">
+      <c r="J326" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K326" s="10" t="n">
         <v>50000000</v>
       </c>
-      <c r="L326" t="b">
-        <v>0</v>
-      </c>
-      <c r="M326" t="n">
+      <c r="L326" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M326" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N326" t="n">
-        <v>0</v>
-      </c>
-      <c r="O326" t="n">
-        <v>0</v>
-      </c>
-      <c r="P326" t="b">
+      <c r="N326" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O326" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P326" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="327">
-      <c r="A327" t="inlineStr">
+      <c r="A327" s="10" t="inlineStr">
         <is>
           <t>The Twilight Saga: Eclipse</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr">
+      <c r="B327" s="10" t="inlineStr">
         <is>
           <t>card_326</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr">
+      <c r="C327" s="10" t="inlineStr">
         <is>
           <t>David Slade</t>
         </is>
       </c>
-      <c r="D327" t="n">
+      <c r="D327" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E327" t="n">
+      <c r="E327" s="10" t="n">
         <v>2.77</v>
       </c>
-      <c r="F327" t="n">
+      <c r="F327" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="I327" t="n">
+      <c r="I327" s="10" t="n">
         <v>699000000</v>
       </c>
-      <c r="J327" t="b">
-        <v>0</v>
-      </c>
-      <c r="K327" t="n">
+      <c r="J327" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K327" s="10" t="n">
         <v>68000000</v>
       </c>
-      <c r="L327" t="b">
-        <v>0</v>
-      </c>
-      <c r="M327" t="n">
+      <c r="L327" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M327" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="N327" t="n">
-        <v>0</v>
-      </c>
-      <c r="O327" t="n">
-        <v>0</v>
-      </c>
-      <c r="P327" t="b">
+      <c r="N327" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O327" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P327" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="328">
-      <c r="A328" t="inlineStr">
+      <c r="A328" s="10" t="inlineStr">
         <is>
           <t>The Twilight Saga: Breaking Dawn - Part 1</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr">
+      <c r="B328" s="10" t="inlineStr">
         <is>
           <t>card_327</t>
         </is>
       </c>
-      <c r="C328" t="inlineStr">
+      <c r="C328" s="10" t="inlineStr">
         <is>
           <t>Bill Condon</t>
         </is>
       </c>
-      <c r="D328" t="n">
+      <c r="D328" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E328" t="n">
+      <c r="E328" s="10" t="n">
         <v>2.77</v>
       </c>
-      <c r="F328" t="n">
+      <c r="F328" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="I328" t="n">
+      <c r="I328" s="10" t="n">
         <v>732000000</v>
       </c>
-      <c r="J328" t="b">
-        <v>0</v>
-      </c>
-      <c r="K328" t="n">
+      <c r="J328" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K328" s="10" t="n">
         <v>127000000</v>
       </c>
-      <c r="L328" t="b">
-        <v>0</v>
-      </c>
-      <c r="M328" t="n">
+      <c r="L328" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M328" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N328" t="n">
-        <v>0</v>
-      </c>
-      <c r="O328" t="n">
-        <v>0</v>
-      </c>
-      <c r="P328" t="b">
+      <c r="N328" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O328" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P328" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="329">
-      <c r="A329" t="inlineStr">
+      <c r="A329" s="10" t="inlineStr">
         <is>
           <t>The Twilight Saga: Breaking Dawn - Part 2</t>
         </is>
       </c>
-      <c r="B329" t="inlineStr">
+      <c r="B329" s="10" t="inlineStr">
         <is>
           <t>card_328</t>
         </is>
       </c>
-      <c r="C329" t="inlineStr">
+      <c r="C329" s="10" t="inlineStr">
         <is>
           <t>Bill Condon</t>
         </is>
       </c>
-      <c r="D329" t="n">
+      <c r="D329" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E329" t="n">
+      <c r="E329" s="10" t="n">
         <v>3.01</v>
       </c>
-      <c r="F329" t="n">
+      <c r="F329" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="I329" t="n">
+      <c r="I329" s="10" t="n">
         <v>868000000</v>
       </c>
-      <c r="J329" t="b">
-        <v>0</v>
-      </c>
-      <c r="K329" t="n">
+      <c r="J329" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K329" s="10" t="n">
         <v>136000000</v>
       </c>
-      <c r="L329" t="b">
-        <v>0</v>
-      </c>
-      <c r="M329" t="n">
+      <c r="L329" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M329" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N329" t="n">
-        <v>0</v>
-      </c>
-      <c r="O329" t="n">
-        <v>0</v>
-      </c>
-      <c r="P329" t="b">
+      <c r="N329" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O329" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P329" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="330">
-      <c r="A330" t="inlineStr">
+      <c r="A330" s="10" t="inlineStr">
         <is>
           <t>Fifty Shades of Grey</t>
         </is>
       </c>
-      <c r="B330" t="inlineStr">
+      <c r="B330" s="10" t="inlineStr">
         <is>
           <t>card_329</t>
         </is>
       </c>
-      <c r="C330" t="inlineStr">
+      <c r="C330" s="10" t="inlineStr">
         <is>
           <t>Sam Taylor-Johnson</t>
         </is>
       </c>
-      <c r="D330" t="n">
+      <c r="D330" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E330" t="n">
+      <c r="E330" s="10" t="n">
         <v>1.88</v>
       </c>
-      <c r="F330" t="n">
+      <c r="F330" s="10" t="n">
         <v>33</v>
       </c>
-      <c r="I330" t="n">
+      <c r="I330" s="10" t="n">
         <v>569700000</v>
       </c>
-      <c r="J330" t="b">
-        <v>0</v>
-      </c>
-      <c r="K330" t="n">
+      <c r="J330" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K330" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L330" t="b">
-        <v>0</v>
-      </c>
-      <c r="M330" t="n">
+      <c r="L330" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M330" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="N330" t="n">
-        <v>0</v>
-      </c>
-      <c r="O330" t="n">
-        <v>0</v>
-      </c>
-      <c r="P330" t="b">
+      <c r="N330" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O330" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P330" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="331">
-      <c r="A331" t="inlineStr">
+      <c r="A331" s="10" t="inlineStr">
         <is>
           <t>Fifty Shades Darker</t>
         </is>
       </c>
-      <c r="B331" t="inlineStr">
+      <c r="B331" s="10" t="inlineStr">
         <is>
           <t>card_330</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr">
+      <c r="C331" s="10" t="inlineStr">
         <is>
           <t>James Foley</t>
         </is>
       </c>
-      <c r="D331" t="n">
+      <c r="D331" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E331" t="n">
+      <c r="E331" s="10" t="n">
         <v>2.09</v>
       </c>
-      <c r="F331" t="n">
+      <c r="F331" s="10" t="n">
         <v>32</v>
       </c>
-      <c r="I331" t="n">
+      <c r="I331" s="10" t="n">
         <v>381000000</v>
       </c>
-      <c r="J331" t="b">
-        <v>0</v>
-      </c>
-      <c r="K331" t="n">
+      <c r="J331" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K331" s="10" t="n">
         <v>55000000</v>
       </c>
-      <c r="L331" t="b">
-        <v>0</v>
-      </c>
-      <c r="M331" t="n">
+      <c r="L331" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M331" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N331" t="n">
-        <v>0</v>
-      </c>
-      <c r="O331" t="n">
-        <v>0</v>
-      </c>
-      <c r="P331" t="b">
+      <c r="N331" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O331" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P331" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="332">
-      <c r="A332" t="inlineStr">
+      <c r="A332" s="10" t="inlineStr">
         <is>
           <t>Fifty Shades Freed</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
+      <c r="B332" s="10" t="inlineStr">
         <is>
           <t>card_331</t>
         </is>
       </c>
-      <c r="C332" t="inlineStr">
+      <c r="C332" s="10" t="inlineStr">
         <is>
           <t>James Foley</t>
         </is>
       </c>
-      <c r="D332" t="n">
+      <c r="D332" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E332" t="n">
+      <c r="E332" s="10" t="n">
         <v>2.06</v>
       </c>
-      <c r="F332" t="n">
+      <c r="F332" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I332" t="n">
+      <c r="I332" s="10" t="n">
         <v>372000000</v>
       </c>
-      <c r="J332" t="b">
-        <v>0</v>
-      </c>
-      <c r="K332" t="n">
+      <c r="J332" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K332" s="10" t="n">
         <v>55000000</v>
       </c>
-      <c r="L332" t="b">
-        <v>0</v>
-      </c>
-      <c r="M332" t="n">
+      <c r="L332" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M332" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="N332" t="n">
-        <v>0</v>
-      </c>
-      <c r="O332" t="n">
-        <v>0</v>
-      </c>
-      <c r="P332" t="b">
+      <c r="N332" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O332" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P332" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="333">
-      <c r="A333" t="inlineStr">
+      <c r="A333" s="10" t="inlineStr">
         <is>
           <t>Die Hard</t>
         </is>
       </c>
-      <c r="B333" t="inlineStr">
+      <c r="B333" s="10" t="inlineStr">
         <is>
           <t>card_332</t>
         </is>
       </c>
-      <c r="C333" t="inlineStr">
+      <c r="C333" s="10" t="inlineStr">
         <is>
           <t>John McTiernan</t>
         </is>
       </c>
-      <c r="D333" t="n">
+      <c r="D333" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E333" t="n">
+      <c r="E333" s="10" t="n">
         <v>4.06</v>
       </c>
-      <c r="F333" t="n">
+      <c r="F333" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="I333" t="n">
+      <c r="I333" s="10" t="n">
         <v>141500000</v>
       </c>
-      <c r="J333" t="b">
-        <v>0</v>
-      </c>
-      <c r="K333" t="n">
+      <c r="J333" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K333" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L333" t="b">
+      <c r="L333" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M333" t="n">
+      <c r="M333" s="10" t="n">
         <v>132</v>
       </c>
-      <c r="N333" t="n">
-        <v>0</v>
-      </c>
-      <c r="O333" t="n">
-        <v>0</v>
-      </c>
-      <c r="P333" t="b">
+      <c r="N333" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O333" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P333" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="334">
-      <c r="A334" t="inlineStr">
+      <c r="A334" s="10" t="inlineStr">
         <is>
           <t>Die Hard 2</t>
         </is>
       </c>
-      <c r="B334" t="inlineStr">
+      <c r="B334" s="10" t="inlineStr">
         <is>
           <t>card_333</t>
         </is>
       </c>
-      <c r="C334" t="inlineStr">
+      <c r="C334" s="10" t="inlineStr">
         <is>
           <t>Renny Harlin</t>
         </is>
       </c>
-      <c r="D334" t="n">
+      <c r="D334" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E334" t="n">
+      <c r="E334" s="10" t="n">
         <v>3.37</v>
       </c>
-      <c r="F334" t="n">
+      <c r="F334" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I334" t="n">
+      <c r="I334" s="10" t="n">
         <v>240000000</v>
       </c>
-      <c r="J334" t="b">
-        <v>0</v>
-      </c>
-      <c r="K334" t="n">
+      <c r="J334" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K334" s="10" t="n">
         <v>65000000</v>
       </c>
-      <c r="L334" t="b">
+      <c r="L334" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M334" t="n">
+      <c r="M334" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="N334" t="n">
-        <v>0</v>
-      </c>
-      <c r="O334" t="n">
-        <v>0</v>
-      </c>
-      <c r="P334" t="b">
+      <c r="N334" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O334" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P334" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="335">
-      <c r="A335" t="inlineStr">
+      <c r="A335" s="10" t="inlineStr">
         <is>
           <t>Die Hard with a Vengeance</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
+      <c r="B335" s="10" t="inlineStr">
         <is>
           <t>card_334</t>
         </is>
       </c>
-      <c r="C335" t="inlineStr">
+      <c r="C335" s="10" t="inlineStr">
         <is>
           <t>John McTiernan</t>
         </is>
       </c>
-      <c r="D335" t="n">
+      <c r="D335" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E335" t="n">
+      <c r="E335" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F335" t="n">
+      <c r="F335" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I335" t="n">
+      <c r="I335" s="10" t="n">
         <v>366000000</v>
       </c>
-      <c r="J335" t="b">
-        <v>0</v>
-      </c>
-      <c r="K335" t="n">
+      <c r="J335" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K335" s="10" t="n">
         <v>90000000</v>
       </c>
-      <c r="L335" t="b">
-        <v>0</v>
-      </c>
-      <c r="M335" t="n">
+      <c r="L335" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M335" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N335" t="n">
-        <v>0</v>
-      </c>
-      <c r="O335" t="n">
-        <v>0</v>
-      </c>
-      <c r="P335" t="b">
+      <c r="N335" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O335" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P335" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="336">
-      <c r="A336" t="inlineStr">
+      <c r="A336" s="10" t="inlineStr">
         <is>
           <t>Live Free or Die Hard</t>
         </is>
       </c>
-      <c r="B336" t="inlineStr">
+      <c r="B336" s="10" t="inlineStr">
         <is>
           <t>card_335</t>
         </is>
       </c>
-      <c r="C336" t="inlineStr">
+      <c r="C336" s="10" t="inlineStr">
         <is>
           <t>Len Wiseman</t>
         </is>
       </c>
-      <c r="D336" t="n">
+      <c r="D336" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E336" t="n">
+      <c r="E336" s="10" t="n">
         <v>2.97</v>
       </c>
-      <c r="F336" t="n">
+      <c r="F336" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I336" t="n">
+      <c r="I336" s="10" t="n">
         <v>383500000</v>
       </c>
-      <c r="J336" t="b">
-        <v>0</v>
-      </c>
-      <c r="K336" t="n">
+      <c r="J336" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K336" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L336" t="b">
-        <v>0</v>
-      </c>
-      <c r="M336" t="n">
+      <c r="L336" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M336" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N336" t="n">
-        <v>0</v>
-      </c>
-      <c r="O336" t="n">
-        <v>0</v>
-      </c>
-      <c r="P336" t="b">
+      <c r="N336" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O336" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P336" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="337">
-      <c r="A337" t="inlineStr">
+      <c r="A337" s="10" t="inlineStr">
         <is>
           <t>A Good Day to Die Hard</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B337" s="10" t="inlineStr">
         <is>
           <t>card_336</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C337" s="10" t="inlineStr">
         <is>
           <t>John Moore</t>
         </is>
       </c>
-      <c r="D337" t="n">
+      <c r="D337" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E337" t="n">
+      <c r="E337" s="10" t="n">
         <v>1.87</v>
       </c>
-      <c r="F337" t="n">
+      <c r="F337" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="I337" t="n">
+      <c r="I337" s="10" t="n">
         <v>304700000</v>
       </c>
-      <c r="J337" t="b">
-        <v>0</v>
-      </c>
-      <c r="K337" t="n">
+      <c r="J337" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K337" s="10" t="n">
         <v>92000000</v>
       </c>
-      <c r="L337" t="b">
-        <v>0</v>
-      </c>
-      <c r="M337" t="n">
+      <c r="L337" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M337" s="10" t="n">
         <v>98</v>
       </c>
-      <c r="N337" t="n">
-        <v>0</v>
-      </c>
-      <c r="O337" t="n">
-        <v>0</v>
-      </c>
-      <c r="P337" t="b">
+      <c r="N337" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O337" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P337" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>King Kong</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>card_337</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E338" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F338" t="n">
+        <v>78</v>
+      </c>
+      <c r="I338" t="n">
+        <v>556900000</v>
+      </c>
+      <c r="J338" t="b">
+        <v>0</v>
+      </c>
+      <c r="K338" t="n">
+        <v>207000000</v>
+      </c>
+      <c r="L338" t="b">
+        <v>0</v>
+      </c>
+      <c r="M338" t="n">
+        <v>187</v>
+      </c>
+      <c r="N338" t="n">
+        <v>3</v>
+      </c>
+      <c r="O338" t="n">
+        <v>3</v>
+      </c>
+      <c r="P338" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Heavenly Creatures</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>card_338</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E339" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F339" t="n">
+        <v>73</v>
+      </c>
+      <c r="I339" t="n">
+        <v>5400000</v>
+      </c>
+      <c r="J339" t="b">
+        <v>0</v>
+      </c>
+      <c r="K339" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L339" t="b">
+        <v>0</v>
+      </c>
+      <c r="M339" t="n">
+        <v>99</v>
+      </c>
+      <c r="N339" t="n">
+        <v>0</v>
+      </c>
+      <c r="O339" t="n">
+        <v>3</v>
+      </c>
+      <c r="P339" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>The Frighteners</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>card_339</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E340" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="F340" t="n">
+        <v>76</v>
+      </c>
+      <c r="I340" t="n">
+        <v>29300000</v>
+      </c>
+      <c r="J340" t="b">
+        <v>0</v>
+      </c>
+      <c r="K340" t="n">
+        <v>26000000</v>
+      </c>
+      <c r="L340" t="b">
+        <v>0</v>
+      </c>
+      <c r="M340" t="n">
+        <v>110</v>
+      </c>
+      <c r="N340" t="n">
+        <v>0</v>
+      </c>
+      <c r="O340" t="n">
+        <v>3</v>
+      </c>
+      <c r="P340" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Braindead</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>card_340</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E341" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="F341" t="n">
+        <v>75</v>
+      </c>
+      <c r="I341" t="n">
+        <v>242623</v>
+      </c>
+      <c r="J341" t="b">
+        <v>1</v>
+      </c>
+      <c r="K341" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="L341" t="b">
+        <v>0</v>
+      </c>
+      <c r="M341" t="n">
+        <v>104</v>
+      </c>
+      <c r="N341" t="n">
+        <v>0</v>
+      </c>
+      <c r="O341" t="n">
+        <v>3</v>
+      </c>
+      <c r="P341" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Bad Taste</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>card_341</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E342" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F342" t="n">
+        <v>54</v>
+      </c>
+      <c r="I342" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J342" t="b">
+        <v>1</v>
+      </c>
+      <c r="K342" t="n">
+        <v>400000</v>
+      </c>
+      <c r="L342" t="b">
+        <v>0</v>
+      </c>
+      <c r="M342" t="n">
+        <v>92</v>
+      </c>
+      <c r="N342" t="n">
+        <v>0</v>
+      </c>
+      <c r="O342" t="n">
+        <v>3</v>
+      </c>
+      <c r="P342" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Meet the Feebles</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>card_342</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E343" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="I343" t="n">
+        <v>80000</v>
+      </c>
+      <c r="J343" t="b">
+        <v>1</v>
+      </c>
+      <c r="K343" t="n">
+        <v>750000</v>
+      </c>
+      <c r="L343" t="b">
+        <v>0</v>
+      </c>
+      <c r="M343" t="n">
+        <v>97</v>
+      </c>
+      <c r="N343" t="n">
+        <v>0</v>
+      </c>
+      <c r="O343" t="n">
+        <v>3</v>
+      </c>
+      <c r="P343" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>The Lovely Bones</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>card_343</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Peter Jackson</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E344" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F344" t="n">
+        <v>62</v>
+      </c>
+      <c r="I344" t="n">
+        <v>93600000</v>
+      </c>
+      <c r="J344" t="b">
+        <v>0</v>
+      </c>
+      <c r="K344" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="L344" t="b">
+        <v>0</v>
+      </c>
+      <c r="M344" t="n">
+        <v>135</v>
+      </c>
+      <c r="N344" t="n">
+        <v>0</v>
+      </c>
+      <c r="O344" t="n">
+        <v>3</v>
+      </c>
+      <c r="P344" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Steven Spielberg films (card_344-365)
22 films: E.T., Close Encounters, Indiana Jones II & IV, The Lost
World, Catch Me If You Can, Minority Report, War of the Worlds,
Munich, Bridge of Spies, The Post, Ready Player One, West Side Story,
The Fabelmans, A.I., Hook, Empire of the Sun, The Color Purple,
Amistad, War Horse, The BFG, Always.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P344"/>
+  <dimension ref="A1:P366"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -18546,349 +18546,1449 @@
       </c>
     </row>
     <row r="338">
-      <c r="A338" t="inlineStr">
+      <c r="A338" s="10" t="inlineStr">
         <is>
           <t>King Kong</t>
         </is>
       </c>
-      <c r="B338" t="inlineStr">
+      <c r="B338" s="10" t="inlineStr">
         <is>
           <t>card_337</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr">
+      <c r="C338" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D338" t="n">
+      <c r="D338" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E338" t="n">
+      <c r="E338" s="10" t="n">
         <v>3.43</v>
       </c>
-      <c r="F338" t="n">
+      <c r="F338" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I338" t="n">
+      <c r="I338" s="10" t="n">
         <v>556900000</v>
       </c>
-      <c r="J338" t="b">
-        <v>0</v>
-      </c>
-      <c r="K338" t="n">
+      <c r="J338" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K338" s="10" t="n">
         <v>207000000</v>
       </c>
-      <c r="L338" t="b">
-        <v>0</v>
-      </c>
-      <c r="M338" t="n">
+      <c r="L338" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M338" s="10" t="n">
         <v>187</v>
       </c>
-      <c r="N338" t="n">
+      <c r="N338" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="O338" t="n">
+      <c r="O338" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P338" t="b">
+      <c r="P338" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="inlineStr">
+      <c r="A339" s="10" t="inlineStr">
         <is>
           <t>Heavenly Creatures</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
+      <c r="B339" s="10" t="inlineStr">
         <is>
           <t>card_338</t>
         </is>
       </c>
-      <c r="C339" t="inlineStr">
+      <c r="C339" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D339" t="n">
+      <c r="D339" s="10" t="n">
         <v>1994</v>
       </c>
-      <c r="E339" t="n">
+      <c r="E339" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F339" t="n">
+      <c r="F339" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I339" t="n">
+      <c r="I339" s="10" t="n">
         <v>5400000</v>
       </c>
-      <c r="J339" t="b">
-        <v>0</v>
-      </c>
-      <c r="K339" t="n">
+      <c r="J339" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K339" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L339" t="b">
-        <v>0</v>
-      </c>
-      <c r="M339" t="n">
+      <c r="L339" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M339" s="10" t="n">
         <v>99</v>
       </c>
-      <c r="N339" t="n">
-        <v>0</v>
-      </c>
-      <c r="O339" t="n">
+      <c r="N339" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O339" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P339" t="b">
+      <c r="P339" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="340">
-      <c r="A340" t="inlineStr">
+      <c r="A340" s="10" t="inlineStr">
         <is>
           <t>The Frighteners</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
+      <c r="B340" s="10" t="inlineStr">
         <is>
           <t>card_339</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr">
+      <c r="C340" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D340" t="n">
+      <c r="D340" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E340" t="n">
+      <c r="E340" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="F340" t="n">
+      <c r="F340" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I340" t="n">
+      <c r="I340" s="10" t="n">
         <v>29300000</v>
       </c>
-      <c r="J340" t="b">
-        <v>0</v>
-      </c>
-      <c r="K340" t="n">
+      <c r="J340" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K340" s="10" t="n">
         <v>26000000</v>
       </c>
-      <c r="L340" t="b">
-        <v>0</v>
-      </c>
-      <c r="M340" t="n">
+      <c r="L340" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M340" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N340" t="n">
-        <v>0</v>
-      </c>
-      <c r="O340" t="n">
+      <c r="N340" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O340" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P340" t="b">
+      <c r="P340" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="341">
-      <c r="A341" t="inlineStr">
+      <c r="A341" s="10" t="inlineStr">
         <is>
           <t>Braindead</t>
         </is>
       </c>
-      <c r="B341" t="inlineStr">
+      <c r="B341" s="10" t="inlineStr">
         <is>
           <t>card_340</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr">
+      <c r="C341" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D341" t="n">
+      <c r="D341" s="10" t="n">
         <v>1992</v>
       </c>
-      <c r="E341" t="n">
+      <c r="E341" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="F341" t="n">
+      <c r="F341" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I341" t="n">
+      <c r="I341" s="10" t="n">
         <v>242623</v>
       </c>
-      <c r="J341" t="b">
+      <c r="J341" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K341" t="n">
+      <c r="K341" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="L341" t="b">
-        <v>0</v>
-      </c>
-      <c r="M341" t="n">
+      <c r="L341" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M341" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="N341" t="n">
-        <v>0</v>
-      </c>
-      <c r="O341" t="n">
+      <c r="N341" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O341" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P341" t="b">
+      <c r="P341" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="342">
-      <c r="A342" t="inlineStr">
+      <c r="A342" s="10" t="inlineStr">
         <is>
           <t>Bad Taste</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B342" s="10" t="inlineStr">
         <is>
           <t>card_341</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C342" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D342" t="n">
+      <c r="D342" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E342" t="n">
+      <c r="E342" s="10" t="n">
         <v>3.29</v>
       </c>
-      <c r="F342" t="n">
+      <c r="F342" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="I342" t="n">
+      <c r="I342" s="10" t="n">
         <v>500000</v>
       </c>
-      <c r="J342" t="b">
+      <c r="J342" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K342" t="n">
+      <c r="K342" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="L342" t="b">
-        <v>0</v>
-      </c>
-      <c r="M342" t="n">
+      <c r="L342" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M342" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="N342" t="n">
-        <v>0</v>
-      </c>
-      <c r="O342" t="n">
+      <c r="N342" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O342" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P342" t="b">
+      <c r="P342" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="343">
-      <c r="A343" t="inlineStr">
+      <c r="A343" s="10" t="inlineStr">
         <is>
           <t>Meet the Feebles</t>
         </is>
       </c>
-      <c r="B343" t="inlineStr">
+      <c r="B343" s="10" t="inlineStr">
         <is>
           <t>card_342</t>
         </is>
       </c>
-      <c r="C343" t="inlineStr">
+      <c r="C343" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D343" t="n">
+      <c r="D343" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E343" t="n">
+      <c r="E343" s="10" t="n">
         <v>3.37</v>
       </c>
-      <c r="I343" t="n">
+      <c r="I343" s="10" t="n">
         <v>80000</v>
       </c>
-      <c r="J343" t="b">
+      <c r="J343" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K343" t="n">
+      <c r="K343" s="10" t="n">
         <v>750000</v>
       </c>
-      <c r="L343" t="b">
-        <v>0</v>
-      </c>
-      <c r="M343" t="n">
+      <c r="L343" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M343" s="10" t="n">
         <v>97</v>
       </c>
-      <c r="N343" t="n">
-        <v>0</v>
-      </c>
-      <c r="O343" t="n">
+      <c r="N343" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O343" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P343" t="b">
+      <c r="P343" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="344">
-      <c r="A344" t="inlineStr">
+      <c r="A344" s="10" t="inlineStr">
         <is>
           <t>The Lovely Bones</t>
         </is>
       </c>
-      <c r="B344" t="inlineStr">
+      <c r="B344" s="10" t="inlineStr">
         <is>
           <t>card_343</t>
         </is>
       </c>
-      <c r="C344" t="inlineStr">
+      <c r="C344" s="10" t="inlineStr">
         <is>
           <t>Peter Jackson</t>
         </is>
       </c>
-      <c r="D344" t="n">
+      <c r="D344" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E344" t="n">
+      <c r="E344" s="10" t="n">
         <v>3.43</v>
       </c>
-      <c r="F344" t="n">
+      <c r="F344" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I344" t="n">
+      <c r="I344" s="10" t="n">
         <v>93600000</v>
       </c>
-      <c r="J344" t="b">
-        <v>0</v>
-      </c>
-      <c r="K344" t="n">
+      <c r="J344" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K344" s="10" t="n">
         <v>65000000</v>
       </c>
-      <c r="L344" t="b">
-        <v>0</v>
-      </c>
-      <c r="M344" t="n">
+      <c r="L344" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M344" s="10" t="n">
         <v>135</v>
       </c>
-      <c r="N344" t="n">
-        <v>0</v>
-      </c>
-      <c r="O344" t="n">
+      <c r="N344" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O344" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="P344" t="b">
+      <c r="P344" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>E.T. the Extra-Terrestrial</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>card_344</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>1982</v>
+      </c>
+      <c r="E345" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F345" t="n">
+        <v>82</v>
+      </c>
+      <c r="I345" t="n">
+        <v>797300000</v>
+      </c>
+      <c r="J345" t="b">
+        <v>0</v>
+      </c>
+      <c r="K345" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="L345" t="b">
+        <v>0</v>
+      </c>
+      <c r="M345" t="n">
+        <v>114</v>
+      </c>
+      <c r="N345" t="n">
+        <v>4</v>
+      </c>
+      <c r="O345" t="n">
+        <v>0</v>
+      </c>
+      <c r="P345" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Close Encounters of the Third Kind</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>card_345</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>1977</v>
+      </c>
+      <c r="E346" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="F346" t="n">
+        <v>79</v>
+      </c>
+      <c r="I346" t="n">
+        <v>306900000</v>
+      </c>
+      <c r="J346" t="b">
+        <v>0</v>
+      </c>
+      <c r="K346" t="n">
+        <v>19400000</v>
+      </c>
+      <c r="L346" t="b">
+        <v>0</v>
+      </c>
+      <c r="M346" t="n">
+        <v>135</v>
+      </c>
+      <c r="N346" t="n">
+        <v>2</v>
+      </c>
+      <c r="O346" t="n">
+        <v>0</v>
+      </c>
+      <c r="P346" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Indiana Jones and the Temple of Doom</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>card_346</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E347" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="F347" t="n">
+        <v>77</v>
+      </c>
+      <c r="I347" t="n">
+        <v>333100000</v>
+      </c>
+      <c r="J347" t="b">
+        <v>0</v>
+      </c>
+      <c r="K347" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="L347" t="b">
+        <v>0</v>
+      </c>
+      <c r="M347" t="n">
+        <v>117</v>
+      </c>
+      <c r="N347" t="n">
+        <v>1</v>
+      </c>
+      <c r="O347" t="n">
+        <v>0</v>
+      </c>
+      <c r="P347" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Indiana Jones and the Kingdom of the Crystal Skull</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>card_347</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E348" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="F348" t="n">
+        <v>59</v>
+      </c>
+      <c r="I348" t="n">
+        <v>786600000</v>
+      </c>
+      <c r="J348" t="b">
+        <v>0</v>
+      </c>
+      <c r="K348" t="n">
+        <v>185000000</v>
+      </c>
+      <c r="L348" t="b">
+        <v>0</v>
+      </c>
+      <c r="M348" t="n">
+        <v>122</v>
+      </c>
+      <c r="N348" t="n">
+        <v>0</v>
+      </c>
+      <c r="O348" t="n">
+        <v>0</v>
+      </c>
+      <c r="P348" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>The Lost World: Jurassic Park</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>card_348</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E349" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F349" t="n">
+        <v>70</v>
+      </c>
+      <c r="I349" t="n">
+        <v>618600000</v>
+      </c>
+      <c r="J349" t="b">
+        <v>0</v>
+      </c>
+      <c r="K349" t="n">
+        <v>73000000</v>
+      </c>
+      <c r="L349" t="b">
+        <v>0</v>
+      </c>
+      <c r="M349" t="n">
+        <v>129</v>
+      </c>
+      <c r="N349" t="n">
+        <v>0</v>
+      </c>
+      <c r="O349" t="n">
+        <v>0</v>
+      </c>
+      <c r="P349" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Catch Me If You Can</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>card_349</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E350" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F350" t="n">
+        <v>83</v>
+      </c>
+      <c r="I350" t="n">
+        <v>352100000</v>
+      </c>
+      <c r="J350" t="b">
+        <v>0</v>
+      </c>
+      <c r="K350" t="n">
+        <v>52000000</v>
+      </c>
+      <c r="L350" t="b">
+        <v>0</v>
+      </c>
+      <c r="M350" t="n">
+        <v>141</v>
+      </c>
+      <c r="N350" t="n">
+        <v>0</v>
+      </c>
+      <c r="O350" t="n">
+        <v>0</v>
+      </c>
+      <c r="P350" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Minority Report</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>card_350</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E351" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F351" t="n">
+        <v>78</v>
+      </c>
+      <c r="I351" t="n">
+        <v>358400000</v>
+      </c>
+      <c r="J351" t="b">
+        <v>0</v>
+      </c>
+      <c r="K351" t="n">
+        <v>102000000</v>
+      </c>
+      <c r="L351" t="b">
+        <v>0</v>
+      </c>
+      <c r="M351" t="n">
+        <v>145</v>
+      </c>
+      <c r="N351" t="n">
+        <v>0</v>
+      </c>
+      <c r="O351" t="n">
+        <v>0</v>
+      </c>
+      <c r="P351" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>War of the Worlds</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>card_351</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E352" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="F352" t="n">
+        <v>69</v>
+      </c>
+      <c r="I352" t="n">
+        <v>604000000</v>
+      </c>
+      <c r="J352" t="b">
+        <v>0</v>
+      </c>
+      <c r="K352" t="n">
+        <v>132000000</v>
+      </c>
+      <c r="L352" t="b">
+        <v>0</v>
+      </c>
+      <c r="M352" t="n">
+        <v>116</v>
+      </c>
+      <c r="N352" t="n">
+        <v>0</v>
+      </c>
+      <c r="O352" t="n">
+        <v>0</v>
+      </c>
+      <c r="P352" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>card_352</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E353" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="F353" t="n">
+        <v>74</v>
+      </c>
+      <c r="I353" t="n">
+        <v>131000000</v>
+      </c>
+      <c r="J353" t="b">
+        <v>0</v>
+      </c>
+      <c r="K353" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="L353" t="b">
+        <v>0</v>
+      </c>
+      <c r="M353" t="n">
+        <v>163</v>
+      </c>
+      <c r="N353" t="n">
+        <v>0</v>
+      </c>
+      <c r="O353" t="n">
+        <v>0</v>
+      </c>
+      <c r="P353" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Bridge of Spies</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>card_353</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E354" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="F354" t="n">
+        <v>76</v>
+      </c>
+      <c r="I354" t="n">
+        <v>165500000</v>
+      </c>
+      <c r="J354" t="b">
+        <v>0</v>
+      </c>
+      <c r="K354" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L354" t="b">
+        <v>0</v>
+      </c>
+      <c r="M354" t="n">
+        <v>141</v>
+      </c>
+      <c r="N354" t="n">
+        <v>1</v>
+      </c>
+      <c r="O354" t="n">
+        <v>0</v>
+      </c>
+      <c r="P354" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>The Post</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>card_354</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E355" t="n">
+        <v>3.51</v>
+      </c>
+      <c r="F355" t="n">
+        <v>70</v>
+      </c>
+      <c r="I355" t="n">
+        <v>179800000</v>
+      </c>
+      <c r="J355" t="b">
+        <v>0</v>
+      </c>
+      <c r="K355" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="L355" t="b">
+        <v>0</v>
+      </c>
+      <c r="M355" t="n">
+        <v>116</v>
+      </c>
+      <c r="N355" t="n">
+        <v>0</v>
+      </c>
+      <c r="O355" t="n">
+        <v>0</v>
+      </c>
+      <c r="P355" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Ready Player One</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>card_355</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E356" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="F356" t="n">
+        <v>74</v>
+      </c>
+      <c r="I356" t="n">
+        <v>608000000</v>
+      </c>
+      <c r="J356" t="b">
+        <v>0</v>
+      </c>
+      <c r="K356" t="n">
+        <v>175000000</v>
+      </c>
+      <c r="L356" t="b">
+        <v>0</v>
+      </c>
+      <c r="M356" t="n">
+        <v>140</v>
+      </c>
+      <c r="N356" t="n">
+        <v>0</v>
+      </c>
+      <c r="O356" t="n">
+        <v>0</v>
+      </c>
+      <c r="P356" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>West Side Story</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>card_356</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E357" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="F357" t="n">
+        <v>73</v>
+      </c>
+      <c r="I357" t="n">
+        <v>76000000</v>
+      </c>
+      <c r="J357" t="b">
+        <v>0</v>
+      </c>
+      <c r="K357" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L357" t="b">
+        <v>0</v>
+      </c>
+      <c r="M357" t="n">
+        <v>156</v>
+      </c>
+      <c r="N357" t="n">
+        <v>1</v>
+      </c>
+      <c r="O357" t="n">
+        <v>0</v>
+      </c>
+      <c r="P357" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>The Fabelmans</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>card_357</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E358" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F358" t="n">
+        <v>74</v>
+      </c>
+      <c r="I358" t="n">
+        <v>45600000</v>
+      </c>
+      <c r="J358" t="b">
+        <v>0</v>
+      </c>
+      <c r="K358" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L358" t="b">
+        <v>0</v>
+      </c>
+      <c r="M358" t="n">
+        <v>151</v>
+      </c>
+      <c r="N358" t="n">
+        <v>0</v>
+      </c>
+      <c r="O358" t="n">
+        <v>0</v>
+      </c>
+      <c r="P358" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>A.I. Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>card_358</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E359" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="F359" t="n">
+        <v>74</v>
+      </c>
+      <c r="I359" t="n">
+        <v>235900000</v>
+      </c>
+      <c r="J359" t="b">
+        <v>0</v>
+      </c>
+      <c r="K359" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L359" t="b">
+        <v>0</v>
+      </c>
+      <c r="M359" t="n">
+        <v>145</v>
+      </c>
+      <c r="N359" t="n">
+        <v>0</v>
+      </c>
+      <c r="O359" t="n">
+        <v>0</v>
+      </c>
+      <c r="P359" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Hook</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>card_359</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>1991</v>
+      </c>
+      <c r="E360" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="F360" t="n">
+        <v>71</v>
+      </c>
+      <c r="I360" t="n">
+        <v>300900000</v>
+      </c>
+      <c r="J360" t="b">
+        <v>0</v>
+      </c>
+      <c r="K360" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="L360" t="b">
+        <v>0</v>
+      </c>
+      <c r="M360" t="n">
+        <v>142</v>
+      </c>
+      <c r="N360" t="n">
+        <v>0</v>
+      </c>
+      <c r="O360" t="n">
+        <v>0</v>
+      </c>
+      <c r="P360" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Empire of the Sun</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>card_360</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E361" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F361" t="n">
+        <v>77</v>
+      </c>
+      <c r="I361" t="n">
+        <v>66700000</v>
+      </c>
+      <c r="J361" t="b">
+        <v>0</v>
+      </c>
+      <c r="K361" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="L361" t="b">
+        <v>0</v>
+      </c>
+      <c r="M361" t="n">
+        <v>154</v>
+      </c>
+      <c r="N361" t="n">
+        <v>0</v>
+      </c>
+      <c r="O361" t="n">
+        <v>0</v>
+      </c>
+      <c r="P361" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>The Color Purple</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>card_361</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E362" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="F362" t="n">
+        <v>82</v>
+      </c>
+      <c r="I362" t="n">
+        <v>98400000</v>
+      </c>
+      <c r="J362" t="b">
+        <v>0</v>
+      </c>
+      <c r="K362" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L362" t="b">
+        <v>0</v>
+      </c>
+      <c r="M362" t="n">
+        <v>154</v>
+      </c>
+      <c r="N362" t="n">
+        <v>0</v>
+      </c>
+      <c r="O362" t="n">
+        <v>0</v>
+      </c>
+      <c r="P362" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Amistad</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>card_362</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E363" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F363" t="n">
+        <v>74</v>
+      </c>
+      <c r="I363" t="n">
+        <v>58300000</v>
+      </c>
+      <c r="J363" t="b">
+        <v>0</v>
+      </c>
+      <c r="K363" t="n">
+        <v>39000000</v>
+      </c>
+      <c r="L363" t="b">
+        <v>0</v>
+      </c>
+      <c r="M363" t="n">
+        <v>154</v>
+      </c>
+      <c r="N363" t="n">
+        <v>0</v>
+      </c>
+      <c r="O363" t="n">
+        <v>0</v>
+      </c>
+      <c r="P363" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>War Horse</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>card_363</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E364" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F364" t="n">
+        <v>67</v>
+      </c>
+      <c r="I364" t="n">
+        <v>177600000</v>
+      </c>
+      <c r="J364" t="b">
+        <v>0</v>
+      </c>
+      <c r="K364" t="n">
+        <v>66000000</v>
+      </c>
+      <c r="L364" t="b">
+        <v>0</v>
+      </c>
+      <c r="M364" t="n">
+        <v>146</v>
+      </c>
+      <c r="N364" t="n">
+        <v>0</v>
+      </c>
+      <c r="O364" t="n">
+        <v>0</v>
+      </c>
+      <c r="P364" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>The BFG</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>card_364</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E365" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F365" t="n">
+        <v>60</v>
+      </c>
+      <c r="I365" t="n">
+        <v>195200000</v>
+      </c>
+      <c r="J365" t="b">
+        <v>0</v>
+      </c>
+      <c r="K365" t="n">
+        <v>140000000</v>
+      </c>
+      <c r="L365" t="b">
+        <v>0</v>
+      </c>
+      <c r="M365" t="n">
+        <v>118</v>
+      </c>
+      <c r="N365" t="n">
+        <v>0</v>
+      </c>
+      <c r="O365" t="n">
+        <v>0</v>
+      </c>
+      <c r="P365" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>card_365</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Steven Spielberg</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E366" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="F366" t="n">
+        <v>64</v>
+      </c>
+      <c r="I366" t="n">
+        <v>74100000</v>
+      </c>
+      <c r="J366" t="b">
+        <v>0</v>
+      </c>
+      <c r="K366" t="n">
+        <v>31000000</v>
+      </c>
+      <c r="L366" t="b">
+        <v>0</v>
+      </c>
+      <c r="M366" t="n">
+        <v>123</v>
+      </c>
+      <c r="N366" t="n">
+        <v>0</v>
+      </c>
+      <c r="O366" t="n">
+        <v>0</v>
+      </c>
+      <c r="P366" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Scorsese, Leone, Nolan, Tarantino films (card_366-394)
29 films rounding out four director filmographies: Taxi Driver, The
Departed, Casino, Wolf of Wall Street, Shutter Island, Mean Streets,
Last Temptation of Christ, The Aviator, Cape Fear, After Hours (10
Scorsese); A Fistful of Dollars, For a Few Dollars More, Once Upon a
Time in America, Duck You Sucker (4 Leone); Following, Insomnia,
Batman Begins, Dark Knight Rises, Inception, Dunkirk, Tenet (7 Nolan);
Kill Bill 1-2, Jackie Brown, Death Proof, Inglourious Basterds, Django
Unchained, The Hateful Eight, Once Upon a Time in Hollywood (8
Tarantino).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P366"/>
+  <dimension ref="A1:P395"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -18893,1102 +18893,2549 @@
       </c>
     </row>
     <row r="345">
-      <c r="A345" t="inlineStr">
+      <c r="A345" s="10" t="inlineStr">
         <is>
           <t>E.T. the Extra-Terrestrial</t>
         </is>
       </c>
-      <c r="B345" t="inlineStr">
+      <c r="B345" s="10" t="inlineStr">
         <is>
           <t>card_344</t>
         </is>
       </c>
-      <c r="C345" t="inlineStr">
+      <c r="C345" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D345" t="n">
+      <c r="D345" s="10" t="n">
         <v>1982</v>
       </c>
-      <c r="E345" t="n">
+      <c r="E345" s="10" t="n">
         <v>3.85</v>
       </c>
-      <c r="F345" t="n">
+      <c r="F345" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I345" t="n">
+      <c r="I345" s="10" t="n">
         <v>797300000</v>
       </c>
-      <c r="J345" t="b">
-        <v>0</v>
-      </c>
-      <c r="K345" t="n">
+      <c r="J345" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K345" s="10" t="n">
         <v>10500000</v>
       </c>
-      <c r="L345" t="b">
-        <v>0</v>
-      </c>
-      <c r="M345" t="n">
+      <c r="L345" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M345" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N345" t="n">
+      <c r="N345" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="O345" t="n">
-        <v>0</v>
-      </c>
-      <c r="P345" t="b">
+      <c r="O345" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P345" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="346">
-      <c r="A346" t="inlineStr">
+      <c r="A346" s="10" t="inlineStr">
         <is>
           <t>Close Encounters of the Third Kind</t>
         </is>
       </c>
-      <c r="B346" t="inlineStr">
+      <c r="B346" s="10" t="inlineStr">
         <is>
           <t>card_345</t>
         </is>
       </c>
-      <c r="C346" t="inlineStr">
+      <c r="C346" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D346" t="n">
+      <c r="D346" s="10" t="n">
         <v>1977</v>
       </c>
-      <c r="E346" t="n">
+      <c r="E346" s="10" t="n">
         <v>3.82</v>
       </c>
-      <c r="F346" t="n">
+      <c r="F346" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I346" t="n">
+      <c r="I346" s="10" t="n">
         <v>306900000</v>
       </c>
-      <c r="J346" t="b">
-        <v>0</v>
-      </c>
-      <c r="K346" t="n">
+      <c r="J346" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K346" s="10" t="n">
         <v>19400000</v>
       </c>
-      <c r="L346" t="b">
-        <v>0</v>
-      </c>
-      <c r="M346" t="n">
+      <c r="L346" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M346" s="10" t="n">
         <v>135</v>
       </c>
-      <c r="N346" t="n">
+      <c r="N346" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O346" t="n">
-        <v>0</v>
-      </c>
-      <c r="P346" t="b">
+      <c r="O346" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P346" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="347">
-      <c r="A347" t="inlineStr">
+      <c r="A347" s="10" t="inlineStr">
         <is>
           <t>Indiana Jones and the Temple of Doom</t>
         </is>
       </c>
-      <c r="B347" t="inlineStr">
+      <c r="B347" s="10" t="inlineStr">
         <is>
           <t>card_346</t>
         </is>
       </c>
-      <c r="C347" t="inlineStr">
+      <c r="C347" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D347" t="n">
+      <c r="D347" s="10" t="n">
         <v>1984</v>
       </c>
-      <c r="E347" t="n">
+      <c r="E347" s="10" t="n">
         <v>3.67</v>
       </c>
-      <c r="F347" t="n">
+      <c r="F347" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I347" t="n">
+      <c r="I347" s="10" t="n">
         <v>333100000</v>
       </c>
-      <c r="J347" t="b">
-        <v>0</v>
-      </c>
-      <c r="K347" t="n">
+      <c r="J347" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K347" s="10" t="n">
         <v>28000000</v>
       </c>
-      <c r="L347" t="b">
-        <v>0</v>
-      </c>
-      <c r="M347" t="n">
+      <c r="L347" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M347" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N347" t="n">
+      <c r="N347" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O347" t="n">
-        <v>0</v>
-      </c>
-      <c r="P347" t="b">
+      <c r="O347" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P347" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="348">
-      <c r="A348" t="inlineStr">
+      <c r="A348" s="10" t="inlineStr">
         <is>
           <t>Indiana Jones and the Kingdom of the Crystal Skull</t>
         </is>
       </c>
-      <c r="B348" t="inlineStr">
+      <c r="B348" s="10" t="inlineStr">
         <is>
           <t>card_347</t>
         </is>
       </c>
-      <c r="C348" t="inlineStr">
+      <c r="C348" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D348" t="n">
+      <c r="D348" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E348" t="n">
+      <c r="E348" s="10" t="n">
         <v>2.82</v>
       </c>
-      <c r="F348" t="n">
+      <c r="F348" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="I348" t="n">
+      <c r="I348" s="10" t="n">
         <v>786600000</v>
       </c>
-      <c r="J348" t="b">
-        <v>0</v>
-      </c>
-      <c r="K348" t="n">
+      <c r="J348" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K348" s="10" t="n">
         <v>185000000</v>
       </c>
-      <c r="L348" t="b">
-        <v>0</v>
-      </c>
-      <c r="M348" t="n">
+      <c r="L348" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M348" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N348" t="n">
-        <v>0</v>
-      </c>
-      <c r="O348" t="n">
-        <v>0</v>
-      </c>
-      <c r="P348" t="b">
+      <c r="N348" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O348" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P348" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="349">
-      <c r="A349" t="inlineStr">
+      <c r="A349" s="10" t="inlineStr">
         <is>
           <t>The Lost World: Jurassic Park</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
+      <c r="B349" s="10" t="inlineStr">
         <is>
           <t>card_348</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
+      <c r="C349" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D349" t="n">
+      <c r="D349" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E349" t="n">
+      <c r="E349" s="10" t="n">
         <v>3.15</v>
       </c>
-      <c r="F349" t="n">
+      <c r="F349" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I349" t="n">
+      <c r="I349" s="10" t="n">
         <v>618600000</v>
       </c>
-      <c r="J349" t="b">
-        <v>0</v>
-      </c>
-      <c r="K349" t="n">
+      <c r="J349" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K349" s="10" t="n">
         <v>73000000</v>
       </c>
-      <c r="L349" t="b">
-        <v>0</v>
-      </c>
-      <c r="M349" t="n">
+      <c r="L349" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M349" s="10" t="n">
         <v>129</v>
       </c>
-      <c r="N349" t="n">
-        <v>0</v>
-      </c>
-      <c r="O349" t="n">
-        <v>0</v>
-      </c>
-      <c r="P349" t="b">
+      <c r="N349" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O349" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P349" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="350">
-      <c r="A350" t="inlineStr">
+      <c r="A350" s="10" t="inlineStr">
         <is>
           <t>Catch Me If You Can</t>
         </is>
       </c>
-      <c r="B350" t="inlineStr">
+      <c r="B350" s="10" t="inlineStr">
         <is>
           <t>card_349</t>
         </is>
       </c>
-      <c r="C350" t="inlineStr">
+      <c r="C350" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D350" t="n">
+      <c r="D350" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E350" t="n">
+      <c r="E350" s="10" t="n">
         <v>3.25</v>
       </c>
-      <c r="F350" t="n">
+      <c r="F350" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I350" t="n">
+      <c r="I350" s="10" t="n">
         <v>352100000</v>
       </c>
-      <c r="J350" t="b">
-        <v>0</v>
-      </c>
-      <c r="K350" t="n">
+      <c r="J350" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K350" s="10" t="n">
         <v>52000000</v>
       </c>
-      <c r="L350" t="b">
-        <v>0</v>
-      </c>
-      <c r="M350" t="n">
+      <c r="L350" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M350" s="10" t="n">
         <v>141</v>
       </c>
-      <c r="N350" t="n">
-        <v>0</v>
-      </c>
-      <c r="O350" t="n">
-        <v>0</v>
-      </c>
-      <c r="P350" t="b">
+      <c r="N350" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O350" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P350" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="351">
-      <c r="A351" t="inlineStr">
+      <c r="A351" s="10" t="inlineStr">
         <is>
           <t>Minority Report</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
+      <c r="B351" s="10" t="inlineStr">
         <is>
           <t>card_350</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
+      <c r="C351" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D351" t="n">
+      <c r="D351" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E351" t="n">
+      <c r="E351" s="10" t="n">
         <v>3.79</v>
       </c>
-      <c r="F351" t="n">
+      <c r="F351" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I351" t="n">
+      <c r="I351" s="10" t="n">
         <v>358400000</v>
       </c>
-      <c r="J351" t="b">
-        <v>0</v>
-      </c>
-      <c r="K351" t="n">
+      <c r="J351" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K351" s="10" t="n">
         <v>102000000</v>
       </c>
-      <c r="L351" t="b">
-        <v>0</v>
-      </c>
-      <c r="M351" t="n">
+      <c r="L351" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M351" s="10" t="n">
         <v>145</v>
       </c>
-      <c r="N351" t="n">
-        <v>0</v>
-      </c>
-      <c r="O351" t="n">
-        <v>0</v>
-      </c>
-      <c r="P351" t="b">
+      <c r="N351" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O351" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P351" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="352">
-      <c r="A352" t="inlineStr">
+      <c r="A352" s="10" t="inlineStr">
         <is>
           <t>War of the Worlds</t>
         </is>
       </c>
-      <c r="B352" t="inlineStr">
+      <c r="B352" s="10" t="inlineStr">
         <is>
           <t>card_351</t>
         </is>
       </c>
-      <c r="C352" t="inlineStr">
+      <c r="C352" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D352" t="n">
+      <c r="D352" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E352" t="n">
+      <c r="E352" s="10" t="n">
         <v>3.37</v>
       </c>
-      <c r="F352" t="n">
+      <c r="F352" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I352" t="n">
+      <c r="I352" s="10" t="n">
         <v>604000000</v>
       </c>
-      <c r="J352" t="b">
-        <v>0</v>
-      </c>
-      <c r="K352" t="n">
+      <c r="J352" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K352" s="10" t="n">
         <v>132000000</v>
       </c>
-      <c r="L352" t="b">
-        <v>0</v>
-      </c>
-      <c r="M352" t="n">
+      <c r="L352" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M352" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="N352" t="n">
-        <v>0</v>
-      </c>
-      <c r="O352" t="n">
-        <v>0</v>
-      </c>
-      <c r="P352" t="b">
+      <c r="N352" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O352" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P352" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="353">
-      <c r="A353" t="inlineStr">
+      <c r="A353" s="10" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="B353" t="inlineStr">
+      <c r="B353" s="10" t="inlineStr">
         <is>
           <t>card_352</t>
         </is>
       </c>
-      <c r="C353" t="inlineStr">
+      <c r="C353" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D353" t="n">
+      <c r="D353" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E353" t="n">
+      <c r="E353" s="10" t="n">
         <v>3.82</v>
       </c>
-      <c r="F353" t="n">
+      <c r="F353" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I353" t="n">
+      <c r="I353" s="10" t="n">
         <v>131000000</v>
       </c>
-      <c r="J353" t="b">
-        <v>0</v>
-      </c>
-      <c r="K353" t="n">
+      <c r="J353" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K353" s="10" t="n">
         <v>70000000</v>
       </c>
-      <c r="L353" t="b">
-        <v>0</v>
-      </c>
-      <c r="M353" t="n">
+      <c r="L353" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M353" s="10" t="n">
         <v>163</v>
       </c>
-      <c r="N353" t="n">
-        <v>0</v>
-      </c>
-      <c r="O353" t="n">
-        <v>0</v>
-      </c>
-      <c r="P353" t="b">
+      <c r="N353" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O353" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P353" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="354">
-      <c r="A354" t="inlineStr">
+      <c r="A354" s="10" t="inlineStr">
         <is>
           <t>Bridge of Spies</t>
         </is>
       </c>
-      <c r="B354" t="inlineStr">
+      <c r="B354" s="10" t="inlineStr">
         <is>
           <t>card_353</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr">
+      <c r="C354" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D354" t="n">
+      <c r="D354" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E354" t="n">
+      <c r="E354" s="10" t="n">
         <v>3.63</v>
       </c>
-      <c r="F354" t="n">
+      <c r="F354" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I354" t="n">
+      <c r="I354" s="10" t="n">
         <v>165500000</v>
       </c>
-      <c r="J354" t="b">
-        <v>0</v>
-      </c>
-      <c r="K354" t="n">
+      <c r="J354" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K354" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L354" t="b">
-        <v>0</v>
-      </c>
-      <c r="M354" t="n">
+      <c r="L354" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M354" s="10" t="n">
         <v>141</v>
       </c>
-      <c r="N354" t="n">
+      <c r="N354" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O354" t="n">
-        <v>0</v>
-      </c>
-      <c r="P354" t="b">
+      <c r="O354" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P354" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="355">
-      <c r="A355" t="inlineStr">
+      <c r="A355" s="10" t="inlineStr">
         <is>
           <t>The Post</t>
         </is>
       </c>
-      <c r="B355" t="inlineStr">
+      <c r="B355" s="10" t="inlineStr">
         <is>
           <t>card_354</t>
         </is>
       </c>
-      <c r="C355" t="inlineStr">
+      <c r="C355" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D355" t="n">
+      <c r="D355" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E355" t="n">
+      <c r="E355" s="10" t="n">
         <v>3.51</v>
       </c>
-      <c r="F355" t="n">
+      <c r="F355" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I355" t="n">
+      <c r="I355" s="10" t="n">
         <v>179800000</v>
       </c>
-      <c r="J355" t="b">
-        <v>0</v>
-      </c>
-      <c r="K355" t="n">
+      <c r="J355" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K355" s="10" t="n">
         <v>50000000</v>
       </c>
-      <c r="L355" t="b">
-        <v>0</v>
-      </c>
-      <c r="M355" t="n">
+      <c r="L355" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M355" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="N355" t="n">
-        <v>0</v>
-      </c>
-      <c r="O355" t="n">
-        <v>0</v>
-      </c>
-      <c r="P355" t="b">
+      <c r="N355" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O355" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P355" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="356">
-      <c r="A356" t="inlineStr">
+      <c r="A356" s="10" t="inlineStr">
         <is>
           <t>Ready Player One</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
+      <c r="B356" s="10" t="inlineStr">
         <is>
           <t>card_355</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C356" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D356" t="n">
+      <c r="D356" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E356" t="n">
+      <c r="E356" s="10" t="n">
         <v>3.37</v>
       </c>
-      <c r="F356" t="n">
+      <c r="F356" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I356" t="n">
+      <c r="I356" s="10" t="n">
         <v>608000000</v>
       </c>
-      <c r="J356" t="b">
-        <v>0</v>
-      </c>
-      <c r="K356" t="n">
+      <c r="J356" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K356" s="10" t="n">
         <v>175000000</v>
       </c>
-      <c r="L356" t="b">
-        <v>0</v>
-      </c>
-      <c r="M356" t="n">
+      <c r="L356" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M356" s="10" t="n">
         <v>140</v>
       </c>
-      <c r="N356" t="n">
-        <v>0</v>
-      </c>
-      <c r="O356" t="n">
-        <v>0</v>
-      </c>
-      <c r="P356" t="b">
+      <c r="N356" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O356" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P356" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="357">
-      <c r="A357" t="inlineStr">
+      <c r="A357" s="10" t="inlineStr">
         <is>
           <t>West Side Story</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr">
+      <c r="B357" s="10" t="inlineStr">
         <is>
           <t>card_356</t>
         </is>
       </c>
-      <c r="C357" t="inlineStr">
+      <c r="C357" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D357" t="n">
+      <c r="D357" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E357" t="n">
+      <c r="E357" s="10" t="n">
         <v>3.63</v>
       </c>
-      <c r="F357" t="n">
+      <c r="F357" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I357" t="n">
+      <c r="I357" s="10" t="n">
         <v>76000000</v>
       </c>
-      <c r="J357" t="b">
-        <v>0</v>
-      </c>
-      <c r="K357" t="n">
+      <c r="J357" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K357" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L357" t="b">
-        <v>0</v>
-      </c>
-      <c r="M357" t="n">
+      <c r="L357" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M357" s="10" t="n">
         <v>156</v>
       </c>
-      <c r="N357" t="n">
+      <c r="N357" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O357" t="n">
-        <v>0</v>
-      </c>
-      <c r="P357" t="b">
+      <c r="O357" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P357" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="358">
-      <c r="A358" t="inlineStr">
+      <c r="A358" s="10" t="inlineStr">
         <is>
           <t>The Fabelmans</t>
         </is>
       </c>
-      <c r="B358" t="inlineStr">
+      <c r="B358" s="10" t="inlineStr">
         <is>
           <t>card_357</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr">
+      <c r="C358" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D358" t="n">
+      <c r="D358" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E358" t="n">
+      <c r="E358" s="10" t="n">
         <v>4.01</v>
       </c>
-      <c r="F358" t="n">
+      <c r="F358" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I358" t="n">
+      <c r="I358" s="10" t="n">
         <v>45600000</v>
       </c>
-      <c r="J358" t="b">
-        <v>0</v>
-      </c>
-      <c r="K358" t="n">
+      <c r="J358" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K358" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L358" t="b">
-        <v>0</v>
-      </c>
-      <c r="M358" t="n">
+      <c r="L358" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M358" s="10" t="n">
         <v>151</v>
       </c>
-      <c r="N358" t="n">
-        <v>0</v>
-      </c>
-      <c r="O358" t="n">
-        <v>0</v>
-      </c>
-      <c r="P358" t="b">
+      <c r="N358" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O358" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P358" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="359">
-      <c r="A359" t="inlineStr">
+      <c r="A359" s="10" t="inlineStr">
         <is>
           <t>A.I. Artificial Intelligence</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B359" s="10" t="inlineStr">
         <is>
           <t>card_358</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr">
+      <c r="C359" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D359" t="n">
+      <c r="D359" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E359" t="n">
+      <c r="E359" s="10" t="n">
         <v>3.66</v>
       </c>
-      <c r="F359" t="n">
+      <c r="F359" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I359" t="n">
+      <c r="I359" s="10" t="n">
         <v>235900000</v>
       </c>
-      <c r="J359" t="b">
-        <v>0</v>
-      </c>
-      <c r="K359" t="n">
+      <c r="J359" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K359" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L359" t="b">
-        <v>0</v>
-      </c>
-      <c r="M359" t="n">
+      <c r="L359" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M359" s="10" t="n">
         <v>145</v>
       </c>
-      <c r="N359" t="n">
-        <v>0</v>
-      </c>
-      <c r="O359" t="n">
-        <v>0</v>
-      </c>
-      <c r="P359" t="b">
+      <c r="N359" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O359" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P359" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="360">
-      <c r="A360" t="inlineStr">
+      <c r="A360" s="10" t="inlineStr">
         <is>
           <t>Hook</t>
         </is>
       </c>
-      <c r="B360" t="inlineStr">
+      <c r="B360" s="10" t="inlineStr">
         <is>
           <t>card_359</t>
         </is>
       </c>
-      <c r="C360" t="inlineStr">
+      <c r="C360" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D360" t="n">
+      <c r="D360" s="10" t="n">
         <v>1991</v>
       </c>
-      <c r="E360" t="n">
+      <c r="E360" s="10" t="n">
         <v>3.48</v>
       </c>
-      <c r="F360" t="n">
+      <c r="F360" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I360" t="n">
+      <c r="I360" s="10" t="n">
         <v>300900000</v>
       </c>
-      <c r="J360" t="b">
-        <v>0</v>
-      </c>
-      <c r="K360" t="n">
+      <c r="J360" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K360" s="10" t="n">
         <v>70000000</v>
       </c>
-      <c r="L360" t="b">
-        <v>0</v>
-      </c>
-      <c r="M360" t="n">
+      <c r="L360" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M360" s="10" t="n">
         <v>142</v>
       </c>
-      <c r="N360" t="n">
-        <v>0</v>
-      </c>
-      <c r="O360" t="n">
-        <v>0</v>
-      </c>
-      <c r="P360" t="b">
+      <c r="N360" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O360" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P360" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="361">
-      <c r="A361" t="inlineStr">
+      <c r="A361" s="10" t="inlineStr">
         <is>
           <t>Empire of the Sun</t>
         </is>
       </c>
-      <c r="B361" t="inlineStr">
+      <c r="B361" s="10" t="inlineStr">
         <is>
           <t>card_360</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
+      <c r="C361" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D361" t="n">
+      <c r="D361" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E361" t="n">
+      <c r="E361" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="F361" t="n">
+      <c r="F361" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I361" t="n">
+      <c r="I361" s="10" t="n">
         <v>66700000</v>
       </c>
-      <c r="J361" t="b">
-        <v>0</v>
-      </c>
-      <c r="K361" t="n">
+      <c r="J361" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K361" s="10" t="n">
         <v>25000000</v>
       </c>
-      <c r="L361" t="b">
-        <v>0</v>
-      </c>
-      <c r="M361" t="n">
+      <c r="L361" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M361" s="10" t="n">
         <v>154</v>
       </c>
-      <c r="N361" t="n">
-        <v>0</v>
-      </c>
-      <c r="O361" t="n">
-        <v>0</v>
-      </c>
-      <c r="P361" t="b">
+      <c r="N361" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O361" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P361" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="362">
-      <c r="A362" t="inlineStr">
+      <c r="A362" s="10" t="inlineStr">
         <is>
           <t>The Color Purple</t>
         </is>
       </c>
-      <c r="B362" t="inlineStr">
+      <c r="B362" s="10" t="inlineStr">
         <is>
           <t>card_361</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr">
+      <c r="C362" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D362" t="n">
+      <c r="D362" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E362" t="n">
+      <c r="E362" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="F362" t="n">
+      <c r="F362" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I362" t="n">
+      <c r="I362" s="10" t="n">
         <v>98400000</v>
       </c>
-      <c r="J362" t="b">
-        <v>0</v>
-      </c>
-      <c r="K362" t="n">
+      <c r="J362" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K362" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L362" t="b">
-        <v>0</v>
-      </c>
-      <c r="M362" t="n">
+      <c r="L362" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M362" s="10" t="n">
         <v>154</v>
       </c>
-      <c r="N362" t="n">
-        <v>0</v>
-      </c>
-      <c r="O362" t="n">
-        <v>0</v>
-      </c>
-      <c r="P362" t="b">
+      <c r="N362" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O362" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P362" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="363">
-      <c r="A363" t="inlineStr">
+      <c r="A363" s="10" t="inlineStr">
         <is>
           <t>Amistad</t>
         </is>
       </c>
-      <c r="B363" t="inlineStr">
+      <c r="B363" s="10" t="inlineStr">
         <is>
           <t>card_362</t>
         </is>
       </c>
-      <c r="C363" t="inlineStr">
+      <c r="C363" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D363" t="n">
+      <c r="D363" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E363" t="n">
+      <c r="E363" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="F363" t="n">
+      <c r="F363" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I363" t="n">
+      <c r="I363" s="10" t="n">
         <v>58300000</v>
       </c>
-      <c r="J363" t="b">
-        <v>0</v>
-      </c>
-      <c r="K363" t="n">
+      <c r="J363" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K363" s="10" t="n">
         <v>39000000</v>
       </c>
-      <c r="L363" t="b">
-        <v>0</v>
-      </c>
-      <c r="M363" t="n">
+      <c r="L363" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M363" s="10" t="n">
         <v>154</v>
       </c>
-      <c r="N363" t="n">
-        <v>0</v>
-      </c>
-      <c r="O363" t="n">
-        <v>0</v>
-      </c>
-      <c r="P363" t="b">
+      <c r="N363" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O363" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P363" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="364">
-      <c r="A364" t="inlineStr">
+      <c r="A364" s="10" t="inlineStr">
         <is>
           <t>War Horse</t>
         </is>
       </c>
-      <c r="B364" t="inlineStr">
+      <c r="B364" s="10" t="inlineStr">
         <is>
           <t>card_363</t>
         </is>
       </c>
-      <c r="C364" t="inlineStr">
+      <c r="C364" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D364" t="n">
+      <c r="D364" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E364" t="n">
+      <c r="E364" s="10" t="n">
         <v>3.41</v>
       </c>
-      <c r="F364" t="n">
+      <c r="F364" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I364" t="n">
+      <c r="I364" s="10" t="n">
         <v>177600000</v>
       </c>
-      <c r="J364" t="b">
-        <v>0</v>
-      </c>
-      <c r="K364" t="n">
+      <c r="J364" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K364" s="10" t="n">
         <v>66000000</v>
       </c>
-      <c r="L364" t="b">
-        <v>0</v>
-      </c>
-      <c r="M364" t="n">
+      <c r="L364" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M364" s="10" t="n">
         <v>146</v>
       </c>
-      <c r="N364" t="n">
-        <v>0</v>
-      </c>
-      <c r="O364" t="n">
-        <v>0</v>
-      </c>
-      <c r="P364" t="b">
+      <c r="N364" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O364" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P364" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="365">
-      <c r="A365" t="inlineStr">
+      <c r="A365" s="10" t="inlineStr">
         <is>
           <t>The BFG</t>
         </is>
       </c>
-      <c r="B365" t="inlineStr">
+      <c r="B365" s="10" t="inlineStr">
         <is>
           <t>card_364</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr">
+      <c r="C365" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D365" t="n">
+      <c r="D365" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E365" t="n">
+      <c r="E365" s="10" t="n">
         <v>3.29</v>
       </c>
-      <c r="F365" t="n">
+      <c r="F365" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I365" t="n">
+      <c r="I365" s="10" t="n">
         <v>195200000</v>
       </c>
-      <c r="J365" t="b">
-        <v>0</v>
-      </c>
-      <c r="K365" t="n">
+      <c r="J365" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K365" s="10" t="n">
         <v>140000000</v>
       </c>
-      <c r="L365" t="b">
-        <v>0</v>
-      </c>
-      <c r="M365" t="n">
+      <c r="L365" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M365" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N365" t="n">
-        <v>0</v>
-      </c>
-      <c r="O365" t="n">
-        <v>0</v>
-      </c>
-      <c r="P365" t="b">
+      <c r="N365" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O365" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P365" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="366">
-      <c r="A366" t="inlineStr">
+      <c r="A366" s="10" t="inlineStr">
         <is>
           <t>Always</t>
         </is>
       </c>
-      <c r="B366" t="inlineStr">
+      <c r="B366" s="10" t="inlineStr">
         <is>
           <t>card_365</t>
         </is>
       </c>
-      <c r="C366" t="inlineStr">
+      <c r="C366" s="10" t="inlineStr">
         <is>
           <t>Steven Spielberg</t>
         </is>
       </c>
-      <c r="D366" t="n">
+      <c r="D366" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E366" t="n">
+      <c r="E366" s="10" t="n">
         <v>2.92</v>
       </c>
-      <c r="F366" t="n">
+      <c r="F366" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="I366" t="n">
+      <c r="I366" s="10" t="n">
         <v>74100000</v>
       </c>
-      <c r="J366" t="b">
-        <v>0</v>
-      </c>
-      <c r="K366" t="n">
+      <c r="J366" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K366" s="10" t="n">
         <v>31000000</v>
       </c>
-      <c r="L366" t="b">
-        <v>0</v>
-      </c>
-      <c r="M366" t="n">
+      <c r="L366" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M366" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="N366" t="n">
-        <v>0</v>
-      </c>
-      <c r="O366" t="n">
-        <v>0</v>
-      </c>
-      <c r="P366" t="b">
+      <c r="N366" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O366" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P366" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Taxi Driver</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>card_366</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>1976</v>
+      </c>
+      <c r="E367" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F367" t="n">
+        <v>86</v>
+      </c>
+      <c r="I367" t="n">
+        <v>29000000</v>
+      </c>
+      <c r="J367" t="b">
+        <v>0</v>
+      </c>
+      <c r="K367" t="n">
+        <v>1900000</v>
+      </c>
+      <c r="L367" t="b">
+        <v>0</v>
+      </c>
+      <c r="M367" t="n">
+        <v>114</v>
+      </c>
+      <c r="N367" t="n">
+        <v>0</v>
+      </c>
+      <c r="O367" t="n">
+        <v>1</v>
+      </c>
+      <c r="P367" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>The Departed</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>card_367</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E368" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="F368" t="n">
+        <v>86</v>
+      </c>
+      <c r="I368" t="n">
+        <v>291500000</v>
+      </c>
+      <c r="J368" t="b">
+        <v>0</v>
+      </c>
+      <c r="K368" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="L368" t="b">
+        <v>0</v>
+      </c>
+      <c r="M368" t="n">
+        <v>151</v>
+      </c>
+      <c r="N368" t="n">
+        <v>4</v>
+      </c>
+      <c r="O368" t="n">
+        <v>1</v>
+      </c>
+      <c r="P368" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Casino</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>card_368</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E369" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="F369" t="n">
+        <v>83</v>
+      </c>
+      <c r="I369" t="n">
+        <v>116100000</v>
+      </c>
+      <c r="J369" t="b">
+        <v>0</v>
+      </c>
+      <c r="K369" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="L369" t="b">
+        <v>0</v>
+      </c>
+      <c r="M369" t="n">
+        <v>178</v>
+      </c>
+      <c r="N369" t="n">
+        <v>0</v>
+      </c>
+      <c r="O369" t="n">
+        <v>1</v>
+      </c>
+      <c r="P369" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>The Wolf of Wall Street</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>card_369</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E370" t="n">
+        <v>4</v>
+      </c>
+      <c r="F370" t="n">
+        <v>81</v>
+      </c>
+      <c r="I370" t="n">
+        <v>407000000</v>
+      </c>
+      <c r="J370" t="b">
+        <v>0</v>
+      </c>
+      <c r="K370" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L370" t="b">
+        <v>0</v>
+      </c>
+      <c r="M370" t="n">
+        <v>179</v>
+      </c>
+      <c r="N370" t="n">
+        <v>0</v>
+      </c>
+      <c r="O370" t="n">
+        <v>1</v>
+      </c>
+      <c r="P370" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Shutter Island</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>card_370</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E371" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F371" t="n">
+        <v>83</v>
+      </c>
+      <c r="I371" t="n">
+        <v>294800000</v>
+      </c>
+      <c r="J371" t="b">
+        <v>0</v>
+      </c>
+      <c r="K371" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L371" t="b">
+        <v>0</v>
+      </c>
+      <c r="M371" t="n">
+        <v>138</v>
+      </c>
+      <c r="N371" t="n">
+        <v>0</v>
+      </c>
+      <c r="O371" t="n">
+        <v>1</v>
+      </c>
+      <c r="P371" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Mean Streets</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>card_371</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>1973</v>
+      </c>
+      <c r="E372" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F372" t="n">
+        <v>75</v>
+      </c>
+      <c r="I372" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J372" t="b">
+        <v>0</v>
+      </c>
+      <c r="K372" t="n">
+        <v>650000</v>
+      </c>
+      <c r="L372" t="b">
+        <v>0</v>
+      </c>
+      <c r="M372" t="n">
+        <v>112</v>
+      </c>
+      <c r="N372" t="n">
+        <v>0</v>
+      </c>
+      <c r="O372" t="n">
+        <v>1</v>
+      </c>
+      <c r="P372" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>The Last Temptation of Christ</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>card_372</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E373" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="F373" t="n">
+        <v>76</v>
+      </c>
+      <c r="I373" t="n">
+        <v>33800000</v>
+      </c>
+      <c r="J373" t="b">
+        <v>0</v>
+      </c>
+      <c r="K373" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="L373" t="b">
+        <v>0</v>
+      </c>
+      <c r="M373" t="n">
+        <v>163</v>
+      </c>
+      <c r="N373" t="n">
+        <v>0</v>
+      </c>
+      <c r="O373" t="n">
+        <v>1</v>
+      </c>
+      <c r="P373" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>The Aviator</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>card_373</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E374" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="F374" t="n">
+        <v>79</v>
+      </c>
+      <c r="I374" t="n">
+        <v>214000000</v>
+      </c>
+      <c r="J374" t="b">
+        <v>0</v>
+      </c>
+      <c r="K374" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L374" t="b">
+        <v>0</v>
+      </c>
+      <c r="M374" t="n">
+        <v>170</v>
+      </c>
+      <c r="N374" t="n">
+        <v>5</v>
+      </c>
+      <c r="O374" t="n">
+        <v>1</v>
+      </c>
+      <c r="P374" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Cape Fear</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>card_374</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>1991</v>
+      </c>
+      <c r="E375" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F375" t="n">
+        <v>75</v>
+      </c>
+      <c r="I375" t="n">
+        <v>182300000</v>
+      </c>
+      <c r="J375" t="b">
+        <v>0</v>
+      </c>
+      <c r="K375" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="L375" t="b">
+        <v>0</v>
+      </c>
+      <c r="M375" t="n">
+        <v>128</v>
+      </c>
+      <c r="N375" t="n">
+        <v>0</v>
+      </c>
+      <c r="O375" t="n">
+        <v>1</v>
+      </c>
+      <c r="P375" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>After Hours</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>card_375</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Martin Scorsese</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E376" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="F376" t="n">
+        <v>81</v>
+      </c>
+      <c r="I376" t="n">
+        <v>10600000</v>
+      </c>
+      <c r="J376" t="b">
+        <v>0</v>
+      </c>
+      <c r="K376" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L376" t="b">
+        <v>0</v>
+      </c>
+      <c r="M376" t="n">
+        <v>97</v>
+      </c>
+      <c r="N376" t="n">
+        <v>0</v>
+      </c>
+      <c r="O376" t="n">
+        <v>1</v>
+      </c>
+      <c r="P376" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>A Fistful of Dollars</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>card_376</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Sergio Leone</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>1964</v>
+      </c>
+      <c r="E377" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="F377" t="n">
+        <v>79</v>
+      </c>
+      <c r="I377" t="n">
+        <v>19900000</v>
+      </c>
+      <c r="J377" t="b">
+        <v>0</v>
+      </c>
+      <c r="K377" t="n">
+        <v>220000</v>
+      </c>
+      <c r="L377" t="b">
+        <v>0</v>
+      </c>
+      <c r="M377" t="n">
+        <v>99</v>
+      </c>
+      <c r="N377" t="n">
+        <v>0</v>
+      </c>
+      <c r="O377" t="n">
+        <v>0</v>
+      </c>
+      <c r="P377" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>For a Few Dollars More</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>card_377</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Sergio Leone</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>1965</v>
+      </c>
+      <c r="E378" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="F378" t="n">
+        <v>83</v>
+      </c>
+      <c r="I378" t="n">
+        <v>25500000</v>
+      </c>
+      <c r="J378" t="b">
+        <v>0</v>
+      </c>
+      <c r="K378" t="n">
+        <v>600000</v>
+      </c>
+      <c r="L378" t="b">
+        <v>0</v>
+      </c>
+      <c r="M378" t="n">
+        <v>132</v>
+      </c>
+      <c r="N378" t="n">
+        <v>0</v>
+      </c>
+      <c r="O378" t="n">
+        <v>0</v>
+      </c>
+      <c r="P378" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Once Upon a Time in America</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>card_378</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Sergio Leone</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E379" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="F379" t="n">
+        <v>83</v>
+      </c>
+      <c r="I379" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="J379" t="b">
+        <v>0</v>
+      </c>
+      <c r="K379" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L379" t="b">
+        <v>0</v>
+      </c>
+      <c r="M379" t="n">
+        <v>229</v>
+      </c>
+      <c r="N379" t="n">
+        <v>0</v>
+      </c>
+      <c r="O379" t="n">
+        <v>0</v>
+      </c>
+      <c r="P379" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Duck, You Sucker!</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>card_379</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Sergio Leone</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>1971</v>
+      </c>
+      <c r="E380" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F380" t="n">
+        <v>79</v>
+      </c>
+      <c r="I380" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="J380" t="b">
+        <v>1</v>
+      </c>
+      <c r="K380" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="L380" t="b">
+        <v>1</v>
+      </c>
+      <c r="M380" t="n">
+        <v>157</v>
+      </c>
+      <c r="N380" t="n">
+        <v>0</v>
+      </c>
+      <c r="O380" t="n">
+        <v>0</v>
+      </c>
+      <c r="P380" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Following</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>card_380</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E381" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="F381" t="n">
+        <v>75</v>
+      </c>
+      <c r="I381" t="n">
+        <v>126052</v>
+      </c>
+      <c r="J381" t="b">
+        <v>0</v>
+      </c>
+      <c r="K381" t="n">
+        <v>6000</v>
+      </c>
+      <c r="L381" t="b">
+        <v>0</v>
+      </c>
+      <c r="M381" t="n">
+        <v>70</v>
+      </c>
+      <c r="N381" t="n">
+        <v>0</v>
+      </c>
+      <c r="O381" t="n">
+        <v>2</v>
+      </c>
+      <c r="P381" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Insomnia</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>card_381</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E382" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F382" t="n">
+        <v>76</v>
+      </c>
+      <c r="I382" t="n">
+        <v>113800000</v>
+      </c>
+      <c r="J382" t="b">
+        <v>0</v>
+      </c>
+      <c r="K382" t="n">
+        <v>46000000</v>
+      </c>
+      <c r="L382" t="b">
+        <v>0</v>
+      </c>
+      <c r="M382" t="n">
+        <v>118</v>
+      </c>
+      <c r="N382" t="n">
+        <v>0</v>
+      </c>
+      <c r="O382" t="n">
+        <v>2</v>
+      </c>
+      <c r="P382" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Batman Begins</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>card_382</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E383" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="F383" t="n">
+        <v>83</v>
+      </c>
+      <c r="I383" t="n">
+        <v>375600000</v>
+      </c>
+      <c r="J383" t="b">
+        <v>0</v>
+      </c>
+      <c r="K383" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L383" t="b">
+        <v>0</v>
+      </c>
+      <c r="M383" t="n">
+        <v>140</v>
+      </c>
+      <c r="N383" t="n">
+        <v>0</v>
+      </c>
+      <c r="O383" t="n">
+        <v>2</v>
+      </c>
+      <c r="P383" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>The Dark Knight Rises</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>card_383</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E384" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F384" t="n">
+        <v>84</v>
+      </c>
+      <c r="I384" t="n">
+        <v>1085000000</v>
+      </c>
+      <c r="J384" t="b">
+        <v>0</v>
+      </c>
+      <c r="K384" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="L384" t="b">
+        <v>0</v>
+      </c>
+      <c r="M384" t="n">
+        <v>164</v>
+      </c>
+      <c r="N384" t="n">
+        <v>0</v>
+      </c>
+      <c r="O384" t="n">
+        <v>2</v>
+      </c>
+      <c r="P384" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Inception</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>card_384</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E385" t="n">
+        <v>4.24</v>
+      </c>
+      <c r="F385" t="n">
+        <v>88</v>
+      </c>
+      <c r="I385" t="n">
+        <v>839000000</v>
+      </c>
+      <c r="J385" t="b">
+        <v>0</v>
+      </c>
+      <c r="K385" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L385" t="b">
+        <v>0</v>
+      </c>
+      <c r="M385" t="n">
+        <v>148</v>
+      </c>
+      <c r="N385" t="n">
+        <v>4</v>
+      </c>
+      <c r="O385" t="n">
+        <v>2</v>
+      </c>
+      <c r="P385" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Dunkirk</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>card_385</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E386" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F386" t="n">
+        <v>82</v>
+      </c>
+      <c r="I386" t="n">
+        <v>549900000</v>
+      </c>
+      <c r="J386" t="b">
+        <v>0</v>
+      </c>
+      <c r="K386" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L386" t="b">
+        <v>0</v>
+      </c>
+      <c r="M386" t="n">
+        <v>106</v>
+      </c>
+      <c r="N386" t="n">
+        <v>3</v>
+      </c>
+      <c r="O386" t="n">
+        <v>2</v>
+      </c>
+      <c r="P386" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Tenet</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>card_386</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Christopher Nolan</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E387" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="F387" t="n">
+        <v>72</v>
+      </c>
+      <c r="I387" t="n">
+        <v>376600000</v>
+      </c>
+      <c r="J387" t="b">
+        <v>0</v>
+      </c>
+      <c r="K387" t="n">
+        <v>205000000</v>
+      </c>
+      <c r="L387" t="b">
+        <v>0</v>
+      </c>
+      <c r="M387" t="n">
+        <v>150</v>
+      </c>
+      <c r="N387" t="n">
+        <v>1</v>
+      </c>
+      <c r="O387" t="n">
+        <v>2</v>
+      </c>
+      <c r="P387" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Kill Bill: Volume 1</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>card_387</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E388" t="n">
+        <v>4.22</v>
+      </c>
+      <c r="F388" t="n">
+        <v>83</v>
+      </c>
+      <c r="I388" t="n">
+        <v>180900000</v>
+      </c>
+      <c r="J388" t="b">
+        <v>0</v>
+      </c>
+      <c r="K388" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L388" t="b">
+        <v>0</v>
+      </c>
+      <c r="M388" t="n">
+        <v>110</v>
+      </c>
+      <c r="N388" t="n">
+        <v>0</v>
+      </c>
+      <c r="O388" t="n">
+        <v>2</v>
+      </c>
+      <c r="P388" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Kill Bill: Volume 2</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>card_388</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E389" t="n">
+        <v>4.11</v>
+      </c>
+      <c r="F389" t="n">
+        <v>82</v>
+      </c>
+      <c r="I389" t="n">
+        <v>152300000</v>
+      </c>
+      <c r="J389" t="b">
+        <v>0</v>
+      </c>
+      <c r="K389" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L389" t="b">
+        <v>0</v>
+      </c>
+      <c r="M389" t="n">
+        <v>137</v>
+      </c>
+      <c r="N389" t="n">
+        <v>0</v>
+      </c>
+      <c r="O389" t="n">
+        <v>2</v>
+      </c>
+      <c r="P389" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Jackie Brown</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>card_389</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E390" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="F390" t="n">
+        <v>76</v>
+      </c>
+      <c r="I390" t="n">
+        <v>74700000</v>
+      </c>
+      <c r="J390" t="b">
+        <v>0</v>
+      </c>
+      <c r="K390" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="L390" t="b">
+        <v>0</v>
+      </c>
+      <c r="M390" t="n">
+        <v>154</v>
+      </c>
+      <c r="N390" t="n">
+        <v>0</v>
+      </c>
+      <c r="O390" t="n">
+        <v>2</v>
+      </c>
+      <c r="P390" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Death Proof</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>card_390</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E391" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="I391" t="n">
+        <v>31100000</v>
+      </c>
+      <c r="J391" t="b">
+        <v>0</v>
+      </c>
+      <c r="K391" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L391" t="b">
+        <v>0</v>
+      </c>
+      <c r="M391" t="n">
+        <v>113</v>
+      </c>
+      <c r="N391" t="n">
+        <v>0</v>
+      </c>
+      <c r="O391" t="n">
+        <v>2</v>
+      </c>
+      <c r="P391" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Inglourious Basterds</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>card_391</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E392" t="n">
+        <v>4.37</v>
+      </c>
+      <c r="F392" t="n">
+        <v>83</v>
+      </c>
+      <c r="I392" t="n">
+        <v>321500000</v>
+      </c>
+      <c r="J392" t="b">
+        <v>0</v>
+      </c>
+      <c r="K392" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="L392" t="b">
+        <v>0</v>
+      </c>
+      <c r="M392" t="n">
+        <v>153</v>
+      </c>
+      <c r="N392" t="n">
+        <v>1</v>
+      </c>
+      <c r="O392" t="n">
+        <v>2</v>
+      </c>
+      <c r="P392" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Django Unchained</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>card_392</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D393" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E393" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="F393" t="n">
+        <v>86</v>
+      </c>
+      <c r="I393" t="n">
+        <v>449800000</v>
+      </c>
+      <c r="J393" t="b">
+        <v>0</v>
+      </c>
+      <c r="K393" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L393" t="b">
+        <v>0</v>
+      </c>
+      <c r="M393" t="n">
+        <v>165</v>
+      </c>
+      <c r="N393" t="n">
+        <v>2</v>
+      </c>
+      <c r="O393" t="n">
+        <v>2</v>
+      </c>
+      <c r="P393" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>The Hateful Eight</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>card_393</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E394" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F394" t="n">
+        <v>76</v>
+      </c>
+      <c r="I394" t="n">
+        <v>161200000</v>
+      </c>
+      <c r="J394" t="b">
+        <v>0</v>
+      </c>
+      <c r="K394" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="L394" t="b">
+        <v>0</v>
+      </c>
+      <c r="M394" t="n">
+        <v>168</v>
+      </c>
+      <c r="N394" t="n">
+        <v>1</v>
+      </c>
+      <c r="O394" t="n">
+        <v>2</v>
+      </c>
+      <c r="P394" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Once Upon a Time in Hollywood</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>card_394</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Quentin Tarantino</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E395" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F395" t="n">
+        <v>75</v>
+      </c>
+      <c r="I395" t="n">
+        <v>393900000</v>
+      </c>
+      <c r="J395" t="b">
+        <v>0</v>
+      </c>
+      <c r="K395" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="L395" t="b">
+        <v>0</v>
+      </c>
+      <c r="M395" t="n">
+        <v>161</v>
+      </c>
+      <c r="N395" t="n">
+        <v>2</v>
+      </c>
+      <c r="O395" t="n">
+        <v>2</v>
+      </c>
+      <c r="P395" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Monty Python, The Martian, Project Hail Mary, Asterix films (card_395-404)
Life of Brian, Meaning of Life, And Now for Something Completely
Different; The Martian; Project Hail Mary (2026); all 5 live-action
Asterix & Obelix films.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P395"/>
+  <dimension ref="A1:P405"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -19993,1449 +19993,1928 @@
       </c>
     </row>
     <row r="367">
-      <c r="A367" t="inlineStr">
+      <c r="A367" s="10" t="inlineStr">
         <is>
           <t>Taxi Driver</t>
         </is>
       </c>
-      <c r="B367" t="inlineStr">
+      <c r="B367" s="10" t="inlineStr">
         <is>
           <t>card_366</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
+      <c r="C367" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D367" t="n">
+      <c r="D367" s="10" t="n">
         <v>1976</v>
       </c>
-      <c r="E367" t="n">
+      <c r="E367" s="10" t="n">
         <v>4.1</v>
       </c>
-      <c r="F367" t="n">
+      <c r="F367" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="I367" t="n">
+      <c r="I367" s="10" t="n">
         <v>29000000</v>
       </c>
-      <c r="J367" t="b">
-        <v>0</v>
-      </c>
-      <c r="K367" t="n">
+      <c r="J367" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K367" s="10" t="n">
         <v>1900000</v>
       </c>
-      <c r="L367" t="b">
-        <v>0</v>
-      </c>
-      <c r="M367" t="n">
+      <c r="L367" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M367" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N367" t="n">
-        <v>0</v>
-      </c>
-      <c r="O367" t="n">
+      <c r="N367" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O367" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P367" t="b">
+      <c r="P367" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="368">
-      <c r="A368" t="inlineStr">
+      <c r="A368" s="10" t="inlineStr">
         <is>
           <t>The Departed</t>
         </is>
       </c>
-      <c r="B368" t="inlineStr">
+      <c r="B368" s="10" t="inlineStr">
         <is>
           <t>card_367</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C368" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D368" t="n">
+      <c r="D368" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E368" t="n">
+      <c r="E368" s="10" t="n">
         <v>4.35</v>
       </c>
-      <c r="F368" t="n">
+      <c r="F368" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="I368" t="n">
+      <c r="I368" s="10" t="n">
         <v>291500000</v>
       </c>
-      <c r="J368" t="b">
-        <v>0</v>
-      </c>
-      <c r="K368" t="n">
+      <c r="J368" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K368" s="10" t="n">
         <v>90000000</v>
       </c>
-      <c r="L368" t="b">
-        <v>0</v>
-      </c>
-      <c r="M368" t="n">
+      <c r="L368" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M368" s="10" t="n">
         <v>151</v>
       </c>
-      <c r="N368" t="n">
+      <c r="N368" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="O368" t="n">
+      <c r="O368" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P368" t="b">
+      <c r="P368" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="369">
-      <c r="A369" t="inlineStr">
+      <c r="A369" s="10" t="inlineStr">
         <is>
           <t>Casino</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr">
+      <c r="B369" s="10" t="inlineStr">
         <is>
           <t>card_368</t>
         </is>
       </c>
-      <c r="C369" t="inlineStr">
+      <c r="C369" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D369" t="n">
+      <c r="D369" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E369" t="n">
+      <c r="E369" s="10" t="n">
         <v>4.22</v>
       </c>
-      <c r="F369" t="n">
+      <c r="F369" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I369" t="n">
+      <c r="I369" s="10" t="n">
         <v>116100000</v>
       </c>
-      <c r="J369" t="b">
-        <v>0</v>
-      </c>
-      <c r="K369" t="n">
+      <c r="J369" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K369" s="10" t="n">
         <v>45000000</v>
       </c>
-      <c r="L369" t="b">
-        <v>0</v>
-      </c>
-      <c r="M369" t="n">
+      <c r="L369" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M369" s="10" t="n">
         <v>178</v>
       </c>
-      <c r="N369" t="n">
-        <v>0</v>
-      </c>
-      <c r="O369" t="n">
+      <c r="N369" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O369" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P369" t="b">
+      <c r="P369" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="370">
-      <c r="A370" t="inlineStr">
+      <c r="A370" s="10" t="inlineStr">
         <is>
           <t>The Wolf of Wall Street</t>
         </is>
       </c>
-      <c r="B370" t="inlineStr">
+      <c r="B370" s="10" t="inlineStr">
         <is>
           <t>card_369</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
+      <c r="C370" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D370" t="n">
+      <c r="D370" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E370" t="n">
+      <c r="E370" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F370" t="n">
+      <c r="F370" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I370" t="n">
+      <c r="I370" s="10" t="n">
         <v>407000000</v>
       </c>
-      <c r="J370" t="b">
-        <v>0</v>
-      </c>
-      <c r="K370" t="n">
+      <c r="J370" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K370" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L370" t="b">
-        <v>0</v>
-      </c>
-      <c r="M370" t="n">
+      <c r="L370" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M370" s="10" t="n">
         <v>179</v>
       </c>
-      <c r="N370" t="n">
-        <v>0</v>
-      </c>
-      <c r="O370" t="n">
+      <c r="N370" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O370" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P370" t="b">
+      <c r="P370" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="371">
-      <c r="A371" t="inlineStr">
+      <c r="A371" s="10" t="inlineStr">
         <is>
           <t>Shutter Island</t>
         </is>
       </c>
-      <c r="B371" t="inlineStr">
+      <c r="B371" s="10" t="inlineStr">
         <is>
           <t>card_370</t>
         </is>
       </c>
-      <c r="C371" t="inlineStr">
+      <c r="C371" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D371" t="n">
+      <c r="D371" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E371" t="n">
+      <c r="E371" s="10" t="n">
         <v>4.2</v>
       </c>
-      <c r="F371" t="n">
+      <c r="F371" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I371" t="n">
+      <c r="I371" s="10" t="n">
         <v>294800000</v>
       </c>
-      <c r="J371" t="b">
-        <v>0</v>
-      </c>
-      <c r="K371" t="n">
+      <c r="J371" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K371" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L371" t="b">
-        <v>0</v>
-      </c>
-      <c r="M371" t="n">
+      <c r="L371" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M371" s="10" t="n">
         <v>138</v>
       </c>
-      <c r="N371" t="n">
-        <v>0</v>
-      </c>
-      <c r="O371" t="n">
+      <c r="N371" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O371" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P371" t="b">
+      <c r="P371" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="372">
-      <c r="A372" t="inlineStr">
+      <c r="A372" s="10" t="inlineStr">
         <is>
           <t>Mean Streets</t>
         </is>
       </c>
-      <c r="B372" t="inlineStr">
+      <c r="B372" s="10" t="inlineStr">
         <is>
           <t>card_371</t>
         </is>
       </c>
-      <c r="C372" t="inlineStr">
+      <c r="C372" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D372" t="n">
+      <c r="D372" s="10" t="n">
         <v>1973</v>
       </c>
-      <c r="E372" t="n">
+      <c r="E372" s="10" t="n">
         <v>3.71</v>
       </c>
-      <c r="F372" t="n">
+      <c r="F372" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I372" t="n">
+      <c r="I372" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="J372" t="b">
-        <v>0</v>
-      </c>
-      <c r="K372" t="n">
+      <c r="J372" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K372" s="10" t="n">
         <v>650000</v>
       </c>
-      <c r="L372" t="b">
-        <v>0</v>
-      </c>
-      <c r="M372" t="n">
+      <c r="L372" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M372" s="10" t="n">
         <v>112</v>
       </c>
-      <c r="N372" t="n">
-        <v>0</v>
-      </c>
-      <c r="O372" t="n">
+      <c r="N372" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O372" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P372" t="b">
+      <c r="P372" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="373">
-      <c r="A373" t="inlineStr">
+      <c r="A373" s="10" t="inlineStr">
         <is>
           <t>The Last Temptation of Christ</t>
         </is>
       </c>
-      <c r="B373" t="inlineStr">
+      <c r="B373" s="10" t="inlineStr">
         <is>
           <t>card_372</t>
         </is>
       </c>
-      <c r="C373" t="inlineStr">
+      <c r="C373" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D373" t="n">
+      <c r="D373" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E373" t="n">
+      <c r="E373" s="10" t="n">
         <v>3.92</v>
       </c>
-      <c r="F373" t="n">
+      <c r="F373" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I373" t="n">
+      <c r="I373" s="10" t="n">
         <v>33800000</v>
       </c>
-      <c r="J373" t="b">
-        <v>0</v>
-      </c>
-      <c r="K373" t="n">
+      <c r="J373" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K373" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="L373" t="b">
-        <v>0</v>
-      </c>
-      <c r="M373" t="n">
+      <c r="L373" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M373" s="10" t="n">
         <v>163</v>
       </c>
-      <c r="N373" t="n">
-        <v>0</v>
-      </c>
-      <c r="O373" t="n">
+      <c r="N373" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O373" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P373" t="b">
+      <c r="P373" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="374">
-      <c r="A374" t="inlineStr">
+      <c r="A374" s="10" t="inlineStr">
         <is>
           <t>The Aviator</t>
         </is>
       </c>
-      <c r="B374" t="inlineStr">
+      <c r="B374" s="10" t="inlineStr">
         <is>
           <t>card_373</t>
         </is>
       </c>
-      <c r="C374" t="inlineStr">
+      <c r="C374" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D374" t="n">
+      <c r="D374" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E374" t="n">
+      <c r="E374" s="10" t="n">
         <v>3.76</v>
       </c>
-      <c r="F374" t="n">
+      <c r="F374" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I374" t="n">
+      <c r="I374" s="10" t="n">
         <v>214000000</v>
       </c>
-      <c r="J374" t="b">
-        <v>0</v>
-      </c>
-      <c r="K374" t="n">
+      <c r="J374" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K374" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L374" t="b">
-        <v>0</v>
-      </c>
-      <c r="M374" t="n">
+      <c r="L374" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M374" s="10" t="n">
         <v>170</v>
       </c>
-      <c r="N374" t="n">
+      <c r="N374" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="O374" t="n">
+      <c r="O374" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P374" t="b">
+      <c r="P374" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="375">
-      <c r="A375" t="inlineStr">
+      <c r="A375" s="10" t="inlineStr">
         <is>
           <t>Cape Fear</t>
         </is>
       </c>
-      <c r="B375" t="inlineStr">
+      <c r="B375" s="10" t="inlineStr">
         <is>
           <t>card_374</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr">
+      <c r="C375" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D375" t="n">
+      <c r="D375" s="10" t="n">
         <v>1991</v>
       </c>
-      <c r="E375" t="n">
+      <c r="E375" s="10" t="n">
         <v>3.72</v>
       </c>
-      <c r="F375" t="n">
+      <c r="F375" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I375" t="n">
+      <c r="I375" s="10" t="n">
         <v>182300000</v>
       </c>
-      <c r="J375" t="b">
-        <v>0</v>
-      </c>
-      <c r="K375" t="n">
+      <c r="J375" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K375" s="10" t="n">
         <v>35000000</v>
       </c>
-      <c r="L375" t="b">
-        <v>0</v>
-      </c>
-      <c r="M375" t="n">
+      <c r="L375" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M375" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N375" t="n">
-        <v>0</v>
-      </c>
-      <c r="O375" t="n">
+      <c r="N375" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O375" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P375" t="b">
+      <c r="P375" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="376">
-      <c r="A376" t="inlineStr">
+      <c r="A376" s="10" t="inlineStr">
         <is>
           <t>After Hours</t>
         </is>
       </c>
-      <c r="B376" t="inlineStr">
+      <c r="B376" s="10" t="inlineStr">
         <is>
           <t>card_375</t>
         </is>
       </c>
-      <c r="C376" t="inlineStr">
+      <c r="C376" s="10" t="inlineStr">
         <is>
           <t>Martin Scorsese</t>
         </is>
       </c>
-      <c r="D376" t="n">
+      <c r="D376" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E376" t="n">
+      <c r="E376" s="10" t="n">
         <v>4.13</v>
       </c>
-      <c r="F376" t="n">
+      <c r="F376" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I376" t="n">
+      <c r="I376" s="10" t="n">
         <v>10600000</v>
       </c>
-      <c r="J376" t="b">
-        <v>0</v>
-      </c>
-      <c r="K376" t="n">
+      <c r="J376" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K376" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L376" t="b">
-        <v>0</v>
-      </c>
-      <c r="M376" t="n">
+      <c r="L376" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M376" s="10" t="n">
         <v>97</v>
       </c>
-      <c r="N376" t="n">
-        <v>0</v>
-      </c>
-      <c r="O376" t="n">
+      <c r="N376" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O376" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P376" t="b">
+      <c r="P376" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="377">
-      <c r="A377" t="inlineStr">
+      <c r="A377" s="10" t="inlineStr">
         <is>
           <t>A Fistful of Dollars</t>
         </is>
       </c>
-      <c r="B377" t="inlineStr">
+      <c r="B377" s="10" t="inlineStr">
         <is>
           <t>card_376</t>
         </is>
       </c>
-      <c r="C377" t="inlineStr">
+      <c r="C377" s="10" t="inlineStr">
         <is>
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="D377" t="n">
+      <c r="D377" s="10" t="n">
         <v>1964</v>
       </c>
-      <c r="E377" t="n">
+      <c r="E377" s="10" t="n">
         <v>3.98</v>
       </c>
-      <c r="F377" t="n">
+      <c r="F377" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I377" t="n">
+      <c r="I377" s="10" t="n">
         <v>19900000</v>
       </c>
-      <c r="J377" t="b">
-        <v>0</v>
-      </c>
-      <c r="K377" t="n">
+      <c r="J377" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K377" s="10" t="n">
         <v>220000</v>
       </c>
-      <c r="L377" t="b">
-        <v>0</v>
-      </c>
-      <c r="M377" t="n">
+      <c r="L377" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M377" s="10" t="n">
         <v>99</v>
       </c>
-      <c r="N377" t="n">
-        <v>0</v>
-      </c>
-      <c r="O377" t="n">
-        <v>0</v>
-      </c>
-      <c r="P377" t="b">
+      <c r="N377" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O377" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P377" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="378">
-      <c r="A378" t="inlineStr">
+      <c r="A378" s="10" t="inlineStr">
         <is>
           <t>For a Few Dollars More</t>
         </is>
       </c>
-      <c r="B378" t="inlineStr">
+      <c r="B378" s="10" t="inlineStr">
         <is>
           <t>card_377</t>
         </is>
       </c>
-      <c r="C378" t="inlineStr">
+      <c r="C378" s="10" t="inlineStr">
         <is>
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="D378" t="n">
+      <c r="D378" s="10" t="n">
         <v>1965</v>
       </c>
-      <c r="E378" t="n">
+      <c r="E378" s="10" t="n">
         <v>4.25</v>
       </c>
-      <c r="F378" t="n">
+      <c r="F378" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I378" t="n">
+      <c r="I378" s="10" t="n">
         <v>25500000</v>
       </c>
-      <c r="J378" t="b">
-        <v>0</v>
-      </c>
-      <c r="K378" t="n">
+      <c r="J378" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K378" s="10" t="n">
         <v>600000</v>
       </c>
-      <c r="L378" t="b">
-        <v>0</v>
-      </c>
-      <c r="M378" t="n">
+      <c r="L378" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M378" s="10" t="n">
         <v>132</v>
       </c>
-      <c r="N378" t="n">
-        <v>0</v>
-      </c>
-      <c r="O378" t="n">
-        <v>0</v>
-      </c>
-      <c r="P378" t="b">
+      <c r="N378" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O378" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P378" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="379">
-      <c r="A379" t="inlineStr">
+      <c r="A379" s="10" t="inlineStr">
         <is>
           <t>Once Upon a Time in America</t>
         </is>
       </c>
-      <c r="B379" t="inlineStr">
+      <c r="B379" s="10" t="inlineStr">
         <is>
           <t>card_378</t>
         </is>
       </c>
-      <c r="C379" t="inlineStr">
+      <c r="C379" s="10" t="inlineStr">
         <is>
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="D379" t="n">
+      <c r="D379" s="10" t="n">
         <v>1984</v>
       </c>
-      <c r="E379" t="n">
+      <c r="E379" s="10" t="n">
         <v>4.22</v>
       </c>
-      <c r="F379" t="n">
+      <c r="F379" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I379" t="n">
+      <c r="I379" s="10" t="n">
         <v>5500000</v>
       </c>
-      <c r="J379" t="b">
-        <v>0</v>
-      </c>
-      <c r="K379" t="n">
+      <c r="J379" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K379" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L379" t="b">
-        <v>0</v>
-      </c>
-      <c r="M379" t="n">
+      <c r="L379" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M379" s="10" t="n">
         <v>229</v>
       </c>
-      <c r="N379" t="n">
-        <v>0</v>
-      </c>
-      <c r="O379" t="n">
-        <v>0</v>
-      </c>
-      <c r="P379" t="b">
+      <c r="N379" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O379" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P379" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="380">
-      <c r="A380" t="inlineStr">
+      <c r="A380" s="10" t="inlineStr">
         <is>
           <t>Duck, You Sucker!</t>
         </is>
       </c>
-      <c r="B380" t="inlineStr">
+      <c r="B380" s="10" t="inlineStr">
         <is>
           <t>card_379</t>
         </is>
       </c>
-      <c r="C380" t="inlineStr">
+      <c r="C380" s="10" t="inlineStr">
         <is>
           <t>Sergio Leone</t>
         </is>
       </c>
-      <c r="D380" t="n">
+      <c r="D380" s="10" t="n">
         <v>1971</v>
       </c>
-      <c r="E380" t="n">
+      <c r="E380" s="10" t="n">
         <v>3.96</v>
       </c>
-      <c r="F380" t="n">
+      <c r="F380" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I380" t="n">
+      <c r="I380" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="J380" t="b">
+      <c r="J380" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K380" t="n">
+      <c r="K380" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="L380" t="b">
+      <c r="L380" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M380" t="n">
+      <c r="M380" s="10" t="n">
         <v>157</v>
       </c>
-      <c r="N380" t="n">
-        <v>0</v>
-      </c>
-      <c r="O380" t="n">
-        <v>0</v>
-      </c>
-      <c r="P380" t="b">
+      <c r="N380" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O380" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P380" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="381">
-      <c r="A381" t="inlineStr">
+      <c r="A381" s="10" t="inlineStr">
         <is>
           <t>Following</t>
         </is>
       </c>
-      <c r="B381" t="inlineStr">
+      <c r="B381" s="10" t="inlineStr">
         <is>
           <t>card_380</t>
         </is>
       </c>
-      <c r="C381" t="inlineStr">
+      <c r="C381" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D381" t="n">
+      <c r="D381" s="10" t="n">
         <v>1998</v>
       </c>
-      <c r="E381" t="n">
+      <c r="E381" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="F381" t="n">
+      <c r="F381" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I381" t="n">
+      <c r="I381" s="10" t="n">
         <v>126052</v>
       </c>
-      <c r="J381" t="b">
-        <v>0</v>
-      </c>
-      <c r="K381" t="n">
+      <c r="J381" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K381" s="10" t="n">
         <v>6000</v>
       </c>
-      <c r="L381" t="b">
-        <v>0</v>
-      </c>
-      <c r="M381" t="n">
+      <c r="L381" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M381" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="N381" t="n">
-        <v>0</v>
-      </c>
-      <c r="O381" t="n">
+      <c r="N381" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O381" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P381" t="b">
+      <c r="P381" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="382">
-      <c r="A382" t="inlineStr">
+      <c r="A382" s="10" t="inlineStr">
         <is>
           <t>Insomnia</t>
         </is>
       </c>
-      <c r="B382" t="inlineStr">
+      <c r="B382" s="10" t="inlineStr">
         <is>
           <t>card_381</t>
         </is>
       </c>
-      <c r="C382" t="inlineStr">
+      <c r="C382" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D382" t="n">
+      <c r="D382" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E382" t="n">
+      <c r="E382" s="10" t="n">
         <v>3.55</v>
       </c>
-      <c r="F382" t="n">
+      <c r="F382" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I382" t="n">
+      <c r="I382" s="10" t="n">
         <v>113800000</v>
       </c>
-      <c r="J382" t="b">
-        <v>0</v>
-      </c>
-      <c r="K382" t="n">
+      <c r="J382" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K382" s="10" t="n">
         <v>46000000</v>
       </c>
-      <c r="L382" t="b">
-        <v>0</v>
-      </c>
-      <c r="M382" t="n">
+      <c r="L382" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M382" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N382" t="n">
-        <v>0</v>
-      </c>
-      <c r="O382" t="n">
+      <c r="N382" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O382" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P382" t="b">
+      <c r="P382" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="383">
-      <c r="A383" t="inlineStr">
+      <c r="A383" s="10" t="inlineStr">
         <is>
           <t>Batman Begins</t>
         </is>
       </c>
-      <c r="B383" t="inlineStr">
+      <c r="B383" s="10" t="inlineStr">
         <is>
           <t>card_382</t>
         </is>
       </c>
-      <c r="C383" t="inlineStr">
+      <c r="C383" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D383" t="n">
+      <c r="D383" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E383" t="n">
+      <c r="E383" s="10" t="n">
         <v>3.85</v>
       </c>
-      <c r="F383" t="n">
+      <c r="F383" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I383" t="n">
+      <c r="I383" s="10" t="n">
         <v>375600000</v>
       </c>
-      <c r="J383" t="b">
-        <v>0</v>
-      </c>
-      <c r="K383" t="n">
+      <c r="J383" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K383" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L383" t="b">
-        <v>0</v>
-      </c>
-      <c r="M383" t="n">
+      <c r="L383" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M383" s="10" t="n">
         <v>140</v>
       </c>
-      <c r="N383" t="n">
-        <v>0</v>
-      </c>
-      <c r="O383" t="n">
+      <c r="N383" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O383" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P383" t="b">
+      <c r="P383" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="384">
-      <c r="A384" t="inlineStr">
+      <c r="A384" s="10" t="inlineStr">
         <is>
           <t>The Dark Knight Rises</t>
         </is>
       </c>
-      <c r="B384" t="inlineStr">
+      <c r="B384" s="10" t="inlineStr">
         <is>
           <t>card_383</t>
         </is>
       </c>
-      <c r="C384" t="inlineStr">
+      <c r="C384" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D384" t="n">
+      <c r="D384" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E384" t="n">
+      <c r="E384" s="10" t="n">
         <v>3.83</v>
       </c>
-      <c r="F384" t="n">
+      <c r="F384" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="I384" t="n">
+      <c r="I384" s="10" t="n">
         <v>1085000000</v>
       </c>
-      <c r="J384" t="b">
-        <v>0</v>
-      </c>
-      <c r="K384" t="n">
+      <c r="J384" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K384" s="10" t="n">
         <v>250000000</v>
       </c>
-      <c r="L384" t="b">
-        <v>0</v>
-      </c>
-      <c r="M384" t="n">
+      <c r="L384" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M384" s="10" t="n">
         <v>164</v>
       </c>
-      <c r="N384" t="n">
-        <v>0</v>
-      </c>
-      <c r="O384" t="n">
+      <c r="N384" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O384" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P384" t="b">
+      <c r="P384" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="385">
-      <c r="A385" t="inlineStr">
+      <c r="A385" s="10" t="inlineStr">
         <is>
           <t>Inception</t>
         </is>
       </c>
-      <c r="B385" t="inlineStr">
+      <c r="B385" s="10" t="inlineStr">
         <is>
           <t>card_384</t>
         </is>
       </c>
-      <c r="C385" t="inlineStr">
+      <c r="C385" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D385" t="n">
+      <c r="D385" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E385" t="n">
+      <c r="E385" s="10" t="n">
         <v>4.24</v>
       </c>
-      <c r="F385" t="n">
+      <c r="F385" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="I385" t="n">
+      <c r="I385" s="10" t="n">
         <v>839000000</v>
       </c>
-      <c r="J385" t="b">
-        <v>0</v>
-      </c>
-      <c r="K385" t="n">
+      <c r="J385" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K385" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L385" t="b">
-        <v>0</v>
-      </c>
-      <c r="M385" t="n">
+      <c r="L385" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M385" s="10" t="n">
         <v>148</v>
       </c>
-      <c r="N385" t="n">
+      <c r="N385" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="O385" t="n">
+      <c r="O385" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P385" t="b">
+      <c r="P385" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="386">
-      <c r="A386" t="inlineStr">
+      <c r="A386" s="10" t="inlineStr">
         <is>
           <t>Dunkirk</t>
         </is>
       </c>
-      <c r="B386" t="inlineStr">
+      <c r="B386" s="10" t="inlineStr">
         <is>
           <t>card_385</t>
         </is>
       </c>
-      <c r="C386" t="inlineStr">
+      <c r="C386" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D386" t="n">
+      <c r="D386" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E386" t="n">
+      <c r="E386" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F386" t="n">
+      <c r="F386" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I386" t="n">
+      <c r="I386" s="10" t="n">
         <v>549900000</v>
       </c>
-      <c r="J386" t="b">
-        <v>0</v>
-      </c>
-      <c r="K386" t="n">
+      <c r="J386" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K386" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L386" t="b">
-        <v>0</v>
-      </c>
-      <c r="M386" t="n">
+      <c r="L386" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M386" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="N386" t="n">
+      <c r="N386" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="O386" t="n">
+      <c r="O386" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P386" t="b">
+      <c r="P386" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="387">
-      <c r="A387" t="inlineStr">
+      <c r="A387" s="10" t="inlineStr">
         <is>
           <t>Tenet</t>
         </is>
       </c>
-      <c r="B387" t="inlineStr">
+      <c r="B387" s="10" t="inlineStr">
         <is>
           <t>card_386</t>
         </is>
       </c>
-      <c r="C387" t="inlineStr">
+      <c r="C387" s="10" t="inlineStr">
         <is>
           <t>Christopher Nolan</t>
         </is>
       </c>
-      <c r="D387" t="n">
+      <c r="D387" s="10" t="n">
         <v>2020</v>
       </c>
-      <c r="E387" t="n">
+      <c r="E387" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="F387" t="n">
+      <c r="F387" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I387" t="n">
+      <c r="I387" s="10" t="n">
         <v>376600000</v>
       </c>
-      <c r="J387" t="b">
-        <v>0</v>
-      </c>
-      <c r="K387" t="n">
+      <c r="J387" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K387" s="10" t="n">
         <v>205000000</v>
       </c>
-      <c r="L387" t="b">
-        <v>0</v>
-      </c>
-      <c r="M387" t="n">
+      <c r="L387" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M387" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="N387" t="n">
+      <c r="N387" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O387" t="n">
+      <c r="O387" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P387" t="b">
+      <c r="P387" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="388">
-      <c r="A388" t="inlineStr">
+      <c r="A388" s="10" t="inlineStr">
         <is>
           <t>Kill Bill: Volume 1</t>
         </is>
       </c>
-      <c r="B388" t="inlineStr">
+      <c r="B388" s="10" t="inlineStr">
         <is>
           <t>card_387</t>
         </is>
       </c>
-      <c r="C388" t="inlineStr">
+      <c r="C388" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D388" t="n">
+      <c r="D388" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E388" t="n">
+      <c r="E388" s="10" t="n">
         <v>4.22</v>
       </c>
-      <c r="F388" t="n">
+      <c r="F388" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I388" t="n">
+      <c r="I388" s="10" t="n">
         <v>180900000</v>
       </c>
-      <c r="J388" t="b">
-        <v>0</v>
-      </c>
-      <c r="K388" t="n">
+      <c r="J388" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K388" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L388" t="b">
-        <v>0</v>
-      </c>
-      <c r="M388" t="n">
+      <c r="L388" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M388" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N388" t="n">
-        <v>0</v>
-      </c>
-      <c r="O388" t="n">
+      <c r="N388" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O388" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P388" t="b">
+      <c r="P388" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="389">
-      <c r="A389" t="inlineStr">
+      <c r="A389" s="10" t="inlineStr">
         <is>
           <t>Kill Bill: Volume 2</t>
         </is>
       </c>
-      <c r="B389" t="inlineStr">
+      <c r="B389" s="10" t="inlineStr">
         <is>
           <t>card_388</t>
         </is>
       </c>
-      <c r="C389" t="inlineStr">
+      <c r="C389" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D389" t="n">
+      <c r="D389" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E389" t="n">
+      <c r="E389" s="10" t="n">
         <v>4.11</v>
       </c>
-      <c r="F389" t="n">
+      <c r="F389" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I389" t="n">
+      <c r="I389" s="10" t="n">
         <v>152300000</v>
       </c>
-      <c r="J389" t="b">
-        <v>0</v>
-      </c>
-      <c r="K389" t="n">
+      <c r="J389" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K389" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L389" t="b">
-        <v>0</v>
-      </c>
-      <c r="M389" t="n">
+      <c r="L389" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M389" s="10" t="n">
         <v>137</v>
       </c>
-      <c r="N389" t="n">
-        <v>0</v>
-      </c>
-      <c r="O389" t="n">
+      <c r="N389" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O389" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P389" t="b">
+      <c r="P389" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="390">
-      <c r="A390" t="inlineStr">
+      <c r="A390" s="10" t="inlineStr">
         <is>
           <t>Jackie Brown</t>
         </is>
       </c>
-      <c r="B390" t="inlineStr">
+      <c r="B390" s="10" t="inlineStr">
         <is>
           <t>card_389</t>
         </is>
       </c>
-      <c r="C390" t="inlineStr">
+      <c r="C390" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D390" t="n">
+      <c r="D390" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E390" t="n">
+      <c r="E390" s="10" t="n">
         <v>3.88</v>
       </c>
-      <c r="F390" t="n">
+      <c r="F390" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I390" t="n">
+      <c r="I390" s="10" t="n">
         <v>74700000</v>
       </c>
-      <c r="J390" t="b">
-        <v>0</v>
-      </c>
-      <c r="K390" t="n">
+      <c r="J390" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K390" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="L390" t="b">
-        <v>0</v>
-      </c>
-      <c r="M390" t="n">
+      <c r="L390" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M390" s="10" t="n">
         <v>154</v>
       </c>
-      <c r="N390" t="n">
-        <v>0</v>
-      </c>
-      <c r="O390" t="n">
+      <c r="N390" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O390" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P390" t="b">
+      <c r="P390" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="391">
-      <c r="A391" t="inlineStr">
+      <c r="A391" s="10" t="inlineStr">
         <is>
           <t>Death Proof</t>
         </is>
       </c>
-      <c r="B391" t="inlineStr">
+      <c r="B391" s="10" t="inlineStr">
         <is>
           <t>card_390</t>
         </is>
       </c>
-      <c r="C391" t="inlineStr">
+      <c r="C391" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D391" t="n">
+      <c r="D391" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E391" t="n">
+      <c r="E391" s="10" t="n">
         <v>3.59</v>
       </c>
-      <c r="I391" t="n">
+      <c r="I391" s="10" t="n">
         <v>31100000</v>
       </c>
-      <c r="J391" t="b">
-        <v>0</v>
-      </c>
-      <c r="K391" t="n">
+      <c r="J391" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K391" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L391" t="b">
-        <v>0</v>
-      </c>
-      <c r="M391" t="n">
+      <c r="L391" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M391" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="N391" t="n">
-        <v>0</v>
-      </c>
-      <c r="O391" t="n">
+      <c r="N391" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O391" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P391" t="b">
+      <c r="P391" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="392">
-      <c r="A392" t="inlineStr">
+      <c r="A392" s="10" t="inlineStr">
         <is>
           <t>Inglourious Basterds</t>
         </is>
       </c>
-      <c r="B392" t="inlineStr">
+      <c r="B392" s="10" t="inlineStr">
         <is>
           <t>card_391</t>
         </is>
       </c>
-      <c r="C392" t="inlineStr">
+      <c r="C392" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D392" t="n">
+      <c r="D392" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E392" t="n">
+      <c r="E392" s="10" t="n">
         <v>4.37</v>
       </c>
-      <c r="F392" t="n">
+      <c r="F392" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I392" t="n">
+      <c r="I392" s="10" t="n">
         <v>321500000</v>
       </c>
-      <c r="J392" t="b">
-        <v>0</v>
-      </c>
-      <c r="K392" t="n">
+      <c r="J392" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K392" s="10" t="n">
         <v>70000000</v>
       </c>
-      <c r="L392" t="b">
-        <v>0</v>
-      </c>
-      <c r="M392" t="n">
+      <c r="L392" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M392" s="10" t="n">
         <v>153</v>
       </c>
-      <c r="N392" t="n">
+      <c r="N392" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O392" t="n">
+      <c r="O392" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P392" t="b">
+      <c r="P392" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="393">
-      <c r="A393" t="inlineStr">
+      <c r="A393" s="10" t="inlineStr">
         <is>
           <t>Django Unchained</t>
         </is>
       </c>
-      <c r="B393" t="inlineStr">
+      <c r="B393" s="10" t="inlineStr">
         <is>
           <t>card_392</t>
         </is>
       </c>
-      <c r="C393" t="inlineStr">
+      <c r="C393" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D393" t="n">
+      <c r="D393" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E393" t="n">
+      <c r="E393" s="10" t="n">
         <v>4.34</v>
       </c>
-      <c r="F393" t="n">
+      <c r="F393" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="I393" t="n">
+      <c r="I393" s="10" t="n">
         <v>449800000</v>
       </c>
-      <c r="J393" t="b">
-        <v>0</v>
-      </c>
-      <c r="K393" t="n">
+      <c r="J393" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K393" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L393" t="b">
-        <v>0</v>
-      </c>
-      <c r="M393" t="n">
+      <c r="L393" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M393" s="10" t="n">
         <v>165</v>
       </c>
-      <c r="N393" t="n">
+      <c r="N393" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O393" t="n">
+      <c r="O393" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P393" t="b">
+      <c r="P393" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="394">
-      <c r="A394" t="inlineStr">
+      <c r="A394" s="10" t="inlineStr">
         <is>
           <t>The Hateful Eight</t>
         </is>
       </c>
-      <c r="B394" t="inlineStr">
+      <c r="B394" s="10" t="inlineStr">
         <is>
           <t>card_393</t>
         </is>
       </c>
-      <c r="C394" t="inlineStr">
+      <c r="C394" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D394" t="n">
+      <c r="D394" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E394" t="n">
+      <c r="E394" s="10" t="n">
         <v>4.04</v>
       </c>
-      <c r="F394" t="n">
+      <c r="F394" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I394" t="n">
+      <c r="I394" s="10" t="n">
         <v>161200000</v>
       </c>
-      <c r="J394" t="b">
-        <v>0</v>
-      </c>
-      <c r="K394" t="n">
+      <c r="J394" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K394" s="10" t="n">
         <v>44000000</v>
       </c>
-      <c r="L394" t="b">
-        <v>0</v>
-      </c>
-      <c r="M394" t="n">
+      <c r="L394" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M394" s="10" t="n">
         <v>168</v>
       </c>
-      <c r="N394" t="n">
+      <c r="N394" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O394" t="n">
+      <c r="O394" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P394" t="b">
+      <c r="P394" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="395">
-      <c r="A395" t="inlineStr">
+      <c r="A395" s="10" t="inlineStr">
         <is>
           <t>Once Upon a Time in Hollywood</t>
         </is>
       </c>
-      <c r="B395" t="inlineStr">
+      <c r="B395" s="10" t="inlineStr">
         <is>
           <t>card_394</t>
         </is>
       </c>
-      <c r="C395" t="inlineStr">
+      <c r="C395" s="10" t="inlineStr">
         <is>
           <t>Quentin Tarantino</t>
         </is>
       </c>
-      <c r="D395" t="n">
+      <c r="D395" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E395" t="n">
+      <c r="E395" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F395" t="n">
+      <c r="F395" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I395" t="n">
+      <c r="I395" s="10" t="n">
         <v>393900000</v>
       </c>
-      <c r="J395" t="b">
-        <v>0</v>
-      </c>
-      <c r="K395" t="n">
+      <c r="J395" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K395" s="10" t="n">
         <v>90000000</v>
       </c>
-      <c r="L395" t="b">
-        <v>0</v>
-      </c>
-      <c r="M395" t="n">
+      <c r="L395" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M395" s="10" t="n">
         <v>161</v>
       </c>
-      <c r="N395" t="n">
+      <c r="N395" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O395" t="n">
+      <c r="O395" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P395" t="b">
+      <c r="P395" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Monty Python's Life of Brian</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>card_395</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Terry Jones</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>1979</v>
+      </c>
+      <c r="E396" t="n">
+        <v>4</v>
+      </c>
+      <c r="F396" t="n">
+        <v>81</v>
+      </c>
+      <c r="I396" t="n">
+        <v>20700000</v>
+      </c>
+      <c r="J396" t="b">
+        <v>0</v>
+      </c>
+      <c r="K396" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L396" t="b">
+        <v>0</v>
+      </c>
+      <c r="M396" t="n">
+        <v>94</v>
+      </c>
+      <c r="N396" t="n">
+        <v>0</v>
+      </c>
+      <c r="O396" t="n">
+        <v>0</v>
+      </c>
+      <c r="P396" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Monty Python's The Meaning of Life</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>card_396</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Terry Jones</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>1983</v>
+      </c>
+      <c r="E397" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="I397" t="n">
+        <v>42700000</v>
+      </c>
+      <c r="J397" t="b">
+        <v>0</v>
+      </c>
+      <c r="K397" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="L397" t="b">
+        <v>0</v>
+      </c>
+      <c r="M397" t="n">
+        <v>90</v>
+      </c>
+      <c r="N397" t="n">
+        <v>0</v>
+      </c>
+      <c r="O397" t="n">
+        <v>0</v>
+      </c>
+      <c r="P397" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>And Now for Something Completely Different</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>card_397</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Ian MacNaughton</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>1971</v>
+      </c>
+      <c r="E398" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="I398" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J398" t="b">
+        <v>1</v>
+      </c>
+      <c r="K398" t="n">
+        <v>220000</v>
+      </c>
+      <c r="L398" t="b">
+        <v>0</v>
+      </c>
+      <c r="M398" t="n">
+        <v>88</v>
+      </c>
+      <c r="N398" t="n">
+        <v>0</v>
+      </c>
+      <c r="O398" t="n">
+        <v>0</v>
+      </c>
+      <c r="P398" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>The Martian</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>card_398</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Ridley Scott</t>
+        </is>
+      </c>
+      <c r="D399" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E399" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F399" t="n">
+        <v>79</v>
+      </c>
+      <c r="I399" t="n">
+        <v>630600000</v>
+      </c>
+      <c r="J399" t="b">
+        <v>0</v>
+      </c>
+      <c r="K399" t="n">
+        <v>108000000</v>
+      </c>
+      <c r="L399" t="b">
+        <v>0</v>
+      </c>
+      <c r="M399" t="n">
+        <v>142</v>
+      </c>
+      <c r="N399" t="n">
+        <v>0</v>
+      </c>
+      <c r="O399" t="n">
+        <v>0</v>
+      </c>
+      <c r="P399" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Project Hail Mary</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>card_399</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Phil Lord and Christopher Miller</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E400" t="n">
+        <v>4.31</v>
+      </c>
+      <c r="F400" t="n">
+        <v>82</v>
+      </c>
+      <c r="I400" t="n">
+        <v>685000000</v>
+      </c>
+      <c r="J400" t="b">
+        <v>0</v>
+      </c>
+      <c r="K400" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L400" t="b">
+        <v>0</v>
+      </c>
+      <c r="M400" t="n">
+        <v>156</v>
+      </c>
+      <c r="N400" t="n">
+        <v>0</v>
+      </c>
+      <c r="O400" t="n">
+        <v>0</v>
+      </c>
+      <c r="P400" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Asterix and Obelix vs. Caesar</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>card_400</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Claude Zidi</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E401" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="I401" t="n">
+        <v>101600000</v>
+      </c>
+      <c r="J401" t="b">
+        <v>0</v>
+      </c>
+      <c r="K401" t="n">
+        <v>48500000</v>
+      </c>
+      <c r="L401" t="b">
+        <v>0</v>
+      </c>
+      <c r="M401" t="n">
+        <v>110</v>
+      </c>
+      <c r="N401" t="n">
+        <v>0</v>
+      </c>
+      <c r="O401" t="n">
+        <v>0</v>
+      </c>
+      <c r="P401" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Asterix &amp; Obelix: Mission Cleopatra</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>card_401</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Alain Chabat</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E402" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="I402" t="n">
+        <v>131000000</v>
+      </c>
+      <c r="J402" t="b">
+        <v>0</v>
+      </c>
+      <c r="K402" t="n">
+        <v>54400000</v>
+      </c>
+      <c r="L402" t="b">
+        <v>0</v>
+      </c>
+      <c r="M402" t="n">
+        <v>107</v>
+      </c>
+      <c r="N402" t="n">
+        <v>0</v>
+      </c>
+      <c r="O402" t="n">
+        <v>0</v>
+      </c>
+      <c r="P402" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Asterix at the Olympic Games</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>card_402</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Frederic Forestier and Thomas Langmann</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E403" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="I403" t="n">
+        <v>133000000</v>
+      </c>
+      <c r="J403" t="b">
+        <v>0</v>
+      </c>
+      <c r="K403" t="n">
+        <v>113500000</v>
+      </c>
+      <c r="L403" t="b">
+        <v>0</v>
+      </c>
+      <c r="M403" t="n">
+        <v>117</v>
+      </c>
+      <c r="N403" t="n">
+        <v>0</v>
+      </c>
+      <c r="O403" t="n">
+        <v>0</v>
+      </c>
+      <c r="P403" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Asterix and Obelix: God Save Britannia</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>card_403</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Laurent Tirard</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E404" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="I404" t="n">
+        <v>61319383</v>
+      </c>
+      <c r="J404" t="b">
+        <v>0</v>
+      </c>
+      <c r="K404" t="n">
+        <v>78000000</v>
+      </c>
+      <c r="L404" t="b">
+        <v>0</v>
+      </c>
+      <c r="M404" t="n">
+        <v>110</v>
+      </c>
+      <c r="N404" t="n">
+        <v>0</v>
+      </c>
+      <c r="O404" t="n">
+        <v>0</v>
+      </c>
+      <c r="P404" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Asterix &amp; Obelix: The Middle Kingdom</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>card_404</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Guillaume Canet</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E405" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="I405" t="n">
+        <v>46500000</v>
+      </c>
+      <c r="J405" t="b">
+        <v>0</v>
+      </c>
+      <c r="K405" t="n">
+        <v>72400000</v>
+      </c>
+      <c r="L405" t="b">
+        <v>0</v>
+      </c>
+      <c r="M405" t="n">
+        <v>111</v>
+      </c>
+      <c r="N405" t="n">
+        <v>0</v>
+      </c>
+      <c r="O405" t="n">
+        <v>0</v>
+      </c>
+      <c r="P405" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Matrix, Terminator, Back to the Future, Mad Max sequels (card_405-417)
13 films: Matrix Reloaded/Revolutions/Resurrections; Terminator 3/
Salvation/Genisys/Dark Fate; Back to the Future II & III; Mad Max
(1979), Mad Max 2, Beyond Thunderdome, Furiosa.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P405"/>
+  <dimension ref="A1:P418"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -21440,481 +21440,1131 @@
       </c>
     </row>
     <row r="396">
-      <c r="A396" t="inlineStr">
+      <c r="A396" s="10" t="inlineStr">
         <is>
           <t>Monty Python's Life of Brian</t>
         </is>
       </c>
-      <c r="B396" t="inlineStr">
+      <c r="B396" s="10" t="inlineStr">
         <is>
           <t>card_395</t>
         </is>
       </c>
-      <c r="C396" t="inlineStr">
+      <c r="C396" s="10" t="inlineStr">
         <is>
           <t>Terry Jones</t>
         </is>
       </c>
-      <c r="D396" t="n">
+      <c r="D396" s="10" t="n">
         <v>1979</v>
       </c>
-      <c r="E396" t="n">
+      <c r="E396" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F396" t="n">
+      <c r="F396" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I396" t="n">
+      <c r="I396" s="10" t="n">
         <v>20700000</v>
       </c>
-      <c r="J396" t="b">
-        <v>0</v>
-      </c>
-      <c r="K396" t="n">
+      <c r="J396" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K396" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L396" t="b">
-        <v>0</v>
-      </c>
-      <c r="M396" t="n">
+      <c r="L396" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M396" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="N396" t="n">
-        <v>0</v>
-      </c>
-      <c r="O396" t="n">
-        <v>0</v>
-      </c>
-      <c r="P396" t="b">
+      <c r="N396" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O396" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P396" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="397">
-      <c r="A397" t="inlineStr">
+      <c r="A397" s="10" t="inlineStr">
         <is>
           <t>Monty Python's The Meaning of Life</t>
         </is>
       </c>
-      <c r="B397" t="inlineStr">
+      <c r="B397" s="10" t="inlineStr">
         <is>
           <t>card_396</t>
         </is>
       </c>
-      <c r="C397" t="inlineStr">
+      <c r="C397" s="10" t="inlineStr">
         <is>
           <t>Terry Jones</t>
         </is>
       </c>
-      <c r="D397" t="n">
+      <c r="D397" s="10" t="n">
         <v>1983</v>
       </c>
-      <c r="E397" t="n">
+      <c r="E397" s="10" t="n">
         <v>3.8</v>
       </c>
-      <c r="I397" t="n">
+      <c r="I397" s="10" t="n">
         <v>42700000</v>
       </c>
-      <c r="J397" t="b">
-        <v>0</v>
-      </c>
-      <c r="K397" t="n">
+      <c r="J397" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K397" s="10" t="n">
         <v>9000000</v>
       </c>
-      <c r="L397" t="b">
-        <v>0</v>
-      </c>
-      <c r="M397" t="n">
+      <c r="L397" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M397" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="N397" t="n">
-        <v>0</v>
-      </c>
-      <c r="O397" t="n">
-        <v>0</v>
-      </c>
-      <c r="P397" t="b">
+      <c r="N397" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O397" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P397" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="398">
-      <c r="A398" t="inlineStr">
+      <c r="A398" s="10" t="inlineStr">
         <is>
           <t>And Now for Something Completely Different</t>
         </is>
       </c>
-      <c r="B398" t="inlineStr">
+      <c r="B398" s="10" t="inlineStr">
         <is>
           <t>card_397</t>
         </is>
       </c>
-      <c r="C398" t="inlineStr">
+      <c r="C398" s="10" t="inlineStr">
         <is>
           <t>Ian MacNaughton</t>
         </is>
       </c>
-      <c r="D398" t="n">
+      <c r="D398" s="10" t="n">
         <v>1971</v>
       </c>
-      <c r="E398" t="n">
+      <c r="E398" s="10" t="n">
         <v>3.79</v>
       </c>
-      <c r="I398" t="n">
+      <c r="I398" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="J398" t="b">
+      <c r="J398" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K398" t="n">
+      <c r="K398" s="10" t="n">
         <v>220000</v>
       </c>
-      <c r="L398" t="b">
-        <v>0</v>
-      </c>
-      <c r="M398" t="n">
+      <c r="L398" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M398" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N398" t="n">
-        <v>0</v>
-      </c>
-      <c r="O398" t="n">
-        <v>0</v>
-      </c>
-      <c r="P398" t="b">
+      <c r="N398" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O398" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P398" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="399">
-      <c r="A399" t="inlineStr">
+      <c r="A399" s="10" t="inlineStr">
         <is>
           <t>The Martian</t>
         </is>
       </c>
-      <c r="B399" t="inlineStr">
+      <c r="B399" s="10" t="inlineStr">
         <is>
           <t>card_398</t>
         </is>
       </c>
-      <c r="C399" t="inlineStr">
+      <c r="C399" s="10" t="inlineStr">
         <is>
           <t>Ridley Scott</t>
         </is>
       </c>
-      <c r="D399" t="n">
+      <c r="D399" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E399" t="n">
+      <c r="E399" s="10" t="n">
         <v>3.83</v>
       </c>
-      <c r="F399" t="n">
+      <c r="F399" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I399" t="n">
+      <c r="I399" s="10" t="n">
         <v>630600000</v>
       </c>
-      <c r="J399" t="b">
-        <v>0</v>
-      </c>
-      <c r="K399" t="n">
+      <c r="J399" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K399" s="10" t="n">
         <v>108000000</v>
       </c>
-      <c r="L399" t="b">
-        <v>0</v>
-      </c>
-      <c r="M399" t="n">
+      <c r="L399" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M399" s="10" t="n">
         <v>142</v>
       </c>
-      <c r="N399" t="n">
-        <v>0</v>
-      </c>
-      <c r="O399" t="n">
-        <v>0</v>
-      </c>
-      <c r="P399" t="b">
+      <c r="N399" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O399" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P399" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="400">
-      <c r="A400" t="inlineStr">
+      <c r="A400" s="10" t="inlineStr">
         <is>
           <t>Project Hail Mary</t>
         </is>
       </c>
-      <c r="B400" t="inlineStr">
+      <c r="B400" s="10" t="inlineStr">
         <is>
           <t>card_399</t>
         </is>
       </c>
-      <c r="C400" t="inlineStr">
+      <c r="C400" s="10" t="inlineStr">
         <is>
           <t>Phil Lord and Christopher Miller</t>
         </is>
       </c>
-      <c r="D400" t="n">
+      <c r="D400" s="10" t="n">
         <v>2026</v>
       </c>
-      <c r="E400" t="n">
+      <c r="E400" s="10" t="n">
         <v>4.31</v>
       </c>
-      <c r="F400" t="n">
+      <c r="F400" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I400" t="n">
+      <c r="I400" s="10" t="n">
         <v>685000000</v>
       </c>
-      <c r="J400" t="b">
-        <v>0</v>
-      </c>
-      <c r="K400" t="n">
+      <c r="J400" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K400" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L400" t="b">
-        <v>0</v>
-      </c>
-      <c r="M400" t="n">
+      <c r="L400" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M400" s="10" t="n">
         <v>156</v>
       </c>
-      <c r="N400" t="n">
-        <v>0</v>
-      </c>
-      <c r="O400" t="n">
-        <v>0</v>
-      </c>
-      <c r="P400" t="b">
+      <c r="N400" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O400" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P400" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="401">
-      <c r="A401" t="inlineStr">
+      <c r="A401" s="10" t="inlineStr">
         <is>
           <t>Asterix and Obelix vs. Caesar</t>
         </is>
       </c>
-      <c r="B401" t="inlineStr">
+      <c r="B401" s="10" t="inlineStr">
         <is>
           <t>card_400</t>
         </is>
       </c>
-      <c r="C401" t="inlineStr">
+      <c r="C401" s="10" t="inlineStr">
         <is>
           <t>Claude Zidi</t>
         </is>
       </c>
-      <c r="D401" t="n">
+      <c r="D401" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E401" t="n">
+      <c r="E401" s="10" t="n">
         <v>2.99</v>
       </c>
-      <c r="I401" t="n">
+      <c r="I401" s="10" t="n">
         <v>101600000</v>
       </c>
-      <c r="J401" t="b">
-        <v>0</v>
-      </c>
-      <c r="K401" t="n">
+      <c r="J401" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K401" s="10" t="n">
         <v>48500000</v>
       </c>
-      <c r="L401" t="b">
-        <v>0</v>
-      </c>
-      <c r="M401" t="n">
+      <c r="L401" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M401" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N401" t="n">
-        <v>0</v>
-      </c>
-      <c r="O401" t="n">
-        <v>0</v>
-      </c>
-      <c r="P401" t="b">
+      <c r="N401" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O401" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P401" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="402">
-      <c r="A402" t="inlineStr">
+      <c r="A402" s="10" t="inlineStr">
         <is>
           <t>Asterix &amp; Obelix: Mission Cleopatra</t>
         </is>
       </c>
-      <c r="B402" t="inlineStr">
+      <c r="B402" s="10" t="inlineStr">
         <is>
           <t>card_401</t>
         </is>
       </c>
-      <c r="C402" t="inlineStr">
+      <c r="C402" s="10" t="inlineStr">
         <is>
           <t>Alain Chabat</t>
         </is>
       </c>
-      <c r="D402" t="n">
+      <c r="D402" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E402" t="n">
+      <c r="E402" s="10" t="n">
         <v>3.67</v>
       </c>
-      <c r="I402" t="n">
+      <c r="I402" s="10" t="n">
         <v>131000000</v>
       </c>
-      <c r="J402" t="b">
-        <v>0</v>
-      </c>
-      <c r="K402" t="n">
+      <c r="J402" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K402" s="10" t="n">
         <v>54400000</v>
       </c>
-      <c r="L402" t="b">
-        <v>0</v>
-      </c>
-      <c r="M402" t="n">
+      <c r="L402" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M402" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N402" t="n">
-        <v>0</v>
-      </c>
-      <c r="O402" t="n">
-        <v>0</v>
-      </c>
-      <c r="P402" t="b">
+      <c r="N402" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O402" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P402" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="403">
-      <c r="A403" t="inlineStr">
+      <c r="A403" s="10" t="inlineStr">
         <is>
           <t>Asterix at the Olympic Games</t>
         </is>
       </c>
-      <c r="B403" t="inlineStr">
+      <c r="B403" s="10" t="inlineStr">
         <is>
           <t>card_402</t>
         </is>
       </c>
-      <c r="C403" t="inlineStr">
+      <c r="C403" s="10" t="inlineStr">
         <is>
           <t>Frederic Forestier and Thomas Langmann</t>
         </is>
       </c>
-      <c r="D403" t="n">
+      <c r="D403" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E403" t="n">
+      <c r="E403" s="10" t="n">
         <v>2.68</v>
       </c>
-      <c r="I403" t="n">
+      <c r="I403" s="10" t="n">
         <v>133000000</v>
       </c>
-      <c r="J403" t="b">
-        <v>0</v>
-      </c>
-      <c r="K403" t="n">
+      <c r="J403" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K403" s="10" t="n">
         <v>113500000</v>
       </c>
-      <c r="L403" t="b">
-        <v>0</v>
-      </c>
-      <c r="M403" t="n">
+      <c r="L403" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M403" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N403" t="n">
-        <v>0</v>
-      </c>
-      <c r="O403" t="n">
-        <v>0</v>
-      </c>
-      <c r="P403" t="b">
+      <c r="N403" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O403" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P403" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="404">
-      <c r="A404" t="inlineStr">
+      <c r="A404" s="10" t="inlineStr">
         <is>
           <t>Asterix and Obelix: God Save Britannia</t>
         </is>
       </c>
-      <c r="B404" t="inlineStr">
+      <c r="B404" s="10" t="inlineStr">
         <is>
           <t>card_403</t>
         </is>
       </c>
-      <c r="C404" t="inlineStr">
+      <c r="C404" s="10" t="inlineStr">
         <is>
           <t>Laurent Tirard</t>
         </is>
       </c>
-      <c r="D404" t="n">
+      <c r="D404" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E404" t="n">
+      <c r="E404" s="10" t="n">
         <v>2.44</v>
       </c>
-      <c r="I404" t="n">
+      <c r="I404" s="10" t="n">
         <v>61319383</v>
       </c>
-      <c r="J404" t="b">
-        <v>0</v>
-      </c>
-      <c r="K404" t="n">
+      <c r="J404" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K404" s="10" t="n">
         <v>78000000</v>
       </c>
-      <c r="L404" t="b">
-        <v>0</v>
-      </c>
-      <c r="M404" t="n">
+      <c r="L404" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M404" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N404" t="n">
-        <v>0</v>
-      </c>
-      <c r="O404" t="n">
-        <v>0</v>
-      </c>
-      <c r="P404" t="b">
+      <c r="N404" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O404" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P404" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="405">
-      <c r="A405" t="inlineStr">
+      <c r="A405" s="10" t="inlineStr">
         <is>
           <t>Asterix &amp; Obelix: The Middle Kingdom</t>
         </is>
       </c>
-      <c r="B405" t="inlineStr">
+      <c r="B405" s="10" t="inlineStr">
         <is>
           <t>card_404</t>
         </is>
       </c>
-      <c r="C405" t="inlineStr">
+      <c r="C405" s="10" t="inlineStr">
         <is>
           <t>Guillaume Canet</t>
         </is>
       </c>
-      <c r="D405" t="n">
+      <c r="D405" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E405" t="n">
+      <c r="E405" s="10" t="n">
         <v>2.25</v>
       </c>
-      <c r="I405" t="n">
+      <c r="I405" s="10" t="n">
         <v>46500000</v>
       </c>
-      <c r="J405" t="b">
-        <v>0</v>
-      </c>
-      <c r="K405" t="n">
+      <c r="J405" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K405" s="10" t="n">
         <v>72400000</v>
       </c>
-      <c r="L405" t="b">
-        <v>0</v>
-      </c>
-      <c r="M405" t="n">
+      <c r="L405" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M405" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N405" t="n">
-        <v>0</v>
-      </c>
-      <c r="O405" t="n">
-        <v>0</v>
-      </c>
-      <c r="P405" t="b">
+      <c r="N405" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O405" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P405" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>The Matrix Reloaded</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>card_405</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Lana Wachowski and Lilly Wachowski</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E406" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F406" t="n">
+        <v>75</v>
+      </c>
+      <c r="I406" t="n">
+        <v>741800000</v>
+      </c>
+      <c r="J406" t="b">
+        <v>0</v>
+      </c>
+      <c r="K406" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L406" t="b">
+        <v>0</v>
+      </c>
+      <c r="M406" t="n">
+        <v>138</v>
+      </c>
+      <c r="N406" t="n">
+        <v>0</v>
+      </c>
+      <c r="O406" t="n">
+        <v>0</v>
+      </c>
+      <c r="P406" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>The Matrix Revolutions</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>card_406</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Lana Wachowski and Lilly Wachowski</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E407" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F407" t="n">
+        <v>66</v>
+      </c>
+      <c r="I407" t="n">
+        <v>427300000</v>
+      </c>
+      <c r="J407" t="b">
+        <v>0</v>
+      </c>
+      <c r="K407" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L407" t="b">
+        <v>0</v>
+      </c>
+      <c r="M407" t="n">
+        <v>129</v>
+      </c>
+      <c r="N407" t="n">
+        <v>0</v>
+      </c>
+      <c r="O407" t="n">
+        <v>0</v>
+      </c>
+      <c r="P407" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>The Matrix Resurrections</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>card_407</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Lana Wachowski</t>
+        </is>
+      </c>
+      <c r="D408" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E408" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F408" t="n">
+        <v>39</v>
+      </c>
+      <c r="I408" t="n">
+        <v>160200000</v>
+      </c>
+      <c r="J408" t="b">
+        <v>0</v>
+      </c>
+      <c r="K408" t="n">
+        <v>190000000</v>
+      </c>
+      <c r="L408" t="b">
+        <v>0</v>
+      </c>
+      <c r="M408" t="n">
+        <v>148</v>
+      </c>
+      <c r="N408" t="n">
+        <v>0</v>
+      </c>
+      <c r="O408" t="n">
+        <v>0</v>
+      </c>
+      <c r="P408" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Terminator 3: Rise of the Machines</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>card_408</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Jonathan Mostow</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E409" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="F409" t="n">
+        <v>63</v>
+      </c>
+      <c r="I409" t="n">
+        <v>433400000</v>
+      </c>
+      <c r="J409" t="b">
+        <v>0</v>
+      </c>
+      <c r="K409" t="n">
+        <v>187300000</v>
+      </c>
+      <c r="L409" t="b">
+        <v>0</v>
+      </c>
+      <c r="M409" t="n">
+        <v>109</v>
+      </c>
+      <c r="N409" t="n">
+        <v>0</v>
+      </c>
+      <c r="O409" t="n">
+        <v>0</v>
+      </c>
+      <c r="P409" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Terminator Salvation</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>card_409</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>McG</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E410" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="F410" t="n">
+        <v>60</v>
+      </c>
+      <c r="I410" t="n">
+        <v>371400000</v>
+      </c>
+      <c r="J410" t="b">
+        <v>0</v>
+      </c>
+      <c r="K410" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L410" t="b">
+        <v>0</v>
+      </c>
+      <c r="M410" t="n">
+        <v>115</v>
+      </c>
+      <c r="N410" t="n">
+        <v>0</v>
+      </c>
+      <c r="O410" t="n">
+        <v>0</v>
+      </c>
+      <c r="P410" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Terminator Genisys</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>card_410</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Alan Taylor</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E411" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="F411" t="n">
+        <v>59</v>
+      </c>
+      <c r="I411" t="n">
+        <v>440600000</v>
+      </c>
+      <c r="J411" t="b">
+        <v>0</v>
+      </c>
+      <c r="K411" t="n">
+        <v>155000000</v>
+      </c>
+      <c r="L411" t="b">
+        <v>0</v>
+      </c>
+      <c r="M411" t="n">
+        <v>126</v>
+      </c>
+      <c r="N411" t="n">
+        <v>0</v>
+      </c>
+      <c r="O411" t="n">
+        <v>0</v>
+      </c>
+      <c r="P411" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Terminator: Dark Fate</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>card_411</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Tim Miller</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E412" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F412" t="n">
+        <v>40</v>
+      </c>
+      <c r="I412" t="n">
+        <v>261100000</v>
+      </c>
+      <c r="J412" t="b">
+        <v>0</v>
+      </c>
+      <c r="K412" t="n">
+        <v>185000000</v>
+      </c>
+      <c r="L412" t="b">
+        <v>0</v>
+      </c>
+      <c r="M412" t="n">
+        <v>128</v>
+      </c>
+      <c r="N412" t="n">
+        <v>0</v>
+      </c>
+      <c r="O412" t="n">
+        <v>0</v>
+      </c>
+      <c r="P412" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Back to the Future Part II</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>card_412</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Robert Zemeckis</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E413" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="F413" t="n">
+        <v>82</v>
+      </c>
+      <c r="I413" t="n">
+        <v>333000000</v>
+      </c>
+      <c r="J413" t="b">
+        <v>0</v>
+      </c>
+      <c r="K413" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L413" t="b">
+        <v>0</v>
+      </c>
+      <c r="M413" t="n">
+        <v>108</v>
+      </c>
+      <c r="N413" t="n">
+        <v>0</v>
+      </c>
+      <c r="O413" t="n">
+        <v>1</v>
+      </c>
+      <c r="P413" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Back to the Future Part III</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>card_413</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Robert Zemeckis</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E414" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="F414" t="n">
+        <v>79</v>
+      </c>
+      <c r="I414" t="n">
+        <v>245100000</v>
+      </c>
+      <c r="J414" t="b">
+        <v>0</v>
+      </c>
+      <c r="K414" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L414" t="b">
+        <v>0</v>
+      </c>
+      <c r="M414" t="n">
+        <v>118</v>
+      </c>
+      <c r="N414" t="n">
+        <v>0</v>
+      </c>
+      <c r="O414" t="n">
+        <v>1</v>
+      </c>
+      <c r="P414" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Mad Max</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>card_414</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>George Miller</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>1979</v>
+      </c>
+      <c r="E415" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F415" t="n">
+        <v>69</v>
+      </c>
+      <c r="I415" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="J415" t="b">
+        <v>1</v>
+      </c>
+      <c r="K415" t="n">
+        <v>400000</v>
+      </c>
+      <c r="L415" t="b">
+        <v>0</v>
+      </c>
+      <c r="M415" t="n">
+        <v>93</v>
+      </c>
+      <c r="N415" t="n">
+        <v>0</v>
+      </c>
+      <c r="O415" t="n">
+        <v>0</v>
+      </c>
+      <c r="P415" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Mad Max 2</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>card_415</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>George Miller</t>
+        </is>
+      </c>
+      <c r="D416" t="n">
+        <v>1981</v>
+      </c>
+      <c r="E416" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F416" t="n">
+        <v>82</v>
+      </c>
+      <c r="I416" t="n">
+        <v>23700000</v>
+      </c>
+      <c r="J416" t="b">
+        <v>0</v>
+      </c>
+      <c r="K416" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="L416" t="b">
+        <v>0</v>
+      </c>
+      <c r="M416" t="n">
+        <v>96</v>
+      </c>
+      <c r="N416" t="n">
+        <v>0</v>
+      </c>
+      <c r="O416" t="n">
+        <v>0</v>
+      </c>
+      <c r="P416" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Mad Max Beyond Thunderdome</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>card_416</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>George Miller and George Ogilvie</t>
+        </is>
+      </c>
+      <c r="D417" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E417" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F417" t="n">
+        <v>62</v>
+      </c>
+      <c r="I417" t="n">
+        <v>36200000</v>
+      </c>
+      <c r="J417" t="b">
+        <v>0</v>
+      </c>
+      <c r="K417" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L417" t="b">
+        <v>0</v>
+      </c>
+      <c r="M417" t="n">
+        <v>107</v>
+      </c>
+      <c r="N417" t="n">
+        <v>0</v>
+      </c>
+      <c r="O417" t="n">
+        <v>0</v>
+      </c>
+      <c r="P417" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Furiosa: A Mad Max Saga</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>card_417</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>George Miller</t>
+        </is>
+      </c>
+      <c r="D418" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E418" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F418" t="n">
+        <v>72</v>
+      </c>
+      <c r="I418" t="n">
+        <v>174400000</v>
+      </c>
+      <c r="J418" t="b">
+        <v>0</v>
+      </c>
+      <c r="K418" t="n">
+        <v>168000000</v>
+      </c>
+      <c r="L418" t="b">
+        <v>0</v>
+      </c>
+      <c r="M418" t="n">
+        <v>148</v>
+      </c>
+      <c r="N418" t="n">
+        <v>0</v>
+      </c>
+      <c r="O418" t="n">
+        <v>0</v>
+      </c>
+      <c r="P418" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Rocky and Creed films (card_418-425)
Rocky II-V, Rocky Balboa, Creed I-III.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P418"/>
+  <dimension ref="A1:P426"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -21919,652 +21919,1052 @@
       </c>
     </row>
     <row r="406">
-      <c r="A406" t="inlineStr">
+      <c r="A406" s="10" t="inlineStr">
         <is>
           <t>The Matrix Reloaded</t>
         </is>
       </c>
-      <c r="B406" t="inlineStr">
+      <c r="B406" s="10" t="inlineStr">
         <is>
           <t>card_405</t>
         </is>
       </c>
-      <c r="C406" t="inlineStr">
+      <c r="C406" s="10" t="inlineStr">
         <is>
           <t>Lana Wachowski and Lilly Wachowski</t>
         </is>
       </c>
-      <c r="D406" t="n">
+      <c r="D406" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E406" t="n">
+      <c r="E406" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F406" t="n">
+      <c r="F406" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I406" t="n">
+      <c r="I406" s="10" t="n">
         <v>741800000</v>
       </c>
-      <c r="J406" t="b">
-        <v>0</v>
-      </c>
-      <c r="K406" t="n">
+      <c r="J406" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K406" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L406" t="b">
-        <v>0</v>
-      </c>
-      <c r="M406" t="n">
+      <c r="L406" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M406" s="10" t="n">
         <v>138</v>
       </c>
-      <c r="N406" t="n">
-        <v>0</v>
-      </c>
-      <c r="O406" t="n">
-        <v>0</v>
-      </c>
-      <c r="P406" t="b">
+      <c r="N406" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O406" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P406" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="407">
-      <c r="A407" t="inlineStr">
+      <c r="A407" s="10" t="inlineStr">
         <is>
           <t>The Matrix Revolutions</t>
         </is>
       </c>
-      <c r="B407" t="inlineStr">
+      <c r="B407" s="10" t="inlineStr">
         <is>
           <t>card_406</t>
         </is>
       </c>
-      <c r="C407" t="inlineStr">
+      <c r="C407" s="10" t="inlineStr">
         <is>
           <t>Lana Wachowski and Lilly Wachowski</t>
         </is>
       </c>
-      <c r="D407" t="n">
+      <c r="D407" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E407" t="n">
+      <c r="E407" s="10" t="n">
         <v>3.19</v>
       </c>
-      <c r="F407" t="n">
+      <c r="F407" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I407" t="n">
+      <c r="I407" s="10" t="n">
         <v>427300000</v>
       </c>
-      <c r="J407" t="b">
-        <v>0</v>
-      </c>
-      <c r="K407" t="n">
+      <c r="J407" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K407" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L407" t="b">
-        <v>0</v>
-      </c>
-      <c r="M407" t="n">
+      <c r="L407" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M407" s="10" t="n">
         <v>129</v>
       </c>
-      <c r="N407" t="n">
-        <v>0</v>
-      </c>
-      <c r="O407" t="n">
-        <v>0</v>
-      </c>
-      <c r="P407" t="b">
+      <c r="N407" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O407" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P407" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="408">
-      <c r="A408" t="inlineStr">
+      <c r="A408" s="10" t="inlineStr">
         <is>
           <t>The Matrix Resurrections</t>
         </is>
       </c>
-      <c r="B408" t="inlineStr">
+      <c r="B408" s="10" t="inlineStr">
         <is>
           <t>card_407</t>
         </is>
       </c>
-      <c r="C408" t="inlineStr">
+      <c r="C408" s="10" t="inlineStr">
         <is>
           <t>Lana Wachowski</t>
         </is>
       </c>
-      <c r="D408" t="n">
+      <c r="D408" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E408" t="n">
+      <c r="E408" s="10" t="n">
         <v>2.67</v>
       </c>
-      <c r="F408" t="n">
+      <c r="F408" s="10" t="n">
         <v>39</v>
       </c>
-      <c r="I408" t="n">
+      <c r="I408" s="10" t="n">
         <v>160200000</v>
       </c>
-      <c r="J408" t="b">
-        <v>0</v>
-      </c>
-      <c r="K408" t="n">
+      <c r="J408" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K408" s="10" t="n">
         <v>190000000</v>
       </c>
-      <c r="L408" t="b">
-        <v>0</v>
-      </c>
-      <c r="M408" t="n">
+      <c r="L408" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M408" s="10" t="n">
         <v>148</v>
       </c>
-      <c r="N408" t="n">
-        <v>0</v>
-      </c>
-      <c r="O408" t="n">
-        <v>0</v>
-      </c>
-      <c r="P408" t="b">
+      <c r="N408" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O408" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P408" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="409">
-      <c r="A409" t="inlineStr">
+      <c r="A409" s="10" t="inlineStr">
         <is>
           <t>Terminator 3: Rise of the Machines</t>
         </is>
       </c>
-      <c r="B409" t="inlineStr">
+      <c r="B409" s="10" t="inlineStr">
         <is>
           <t>card_408</t>
         </is>
       </c>
-      <c r="C409" t="inlineStr">
+      <c r="C409" s="10" t="inlineStr">
         <is>
           <t>Jonathan Mostow</t>
         </is>
       </c>
-      <c r="D409" t="n">
+      <c r="D409" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E409" t="n">
+      <c r="E409" s="10" t="n">
         <v>2.76</v>
       </c>
-      <c r="F409" t="n">
+      <c r="F409" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I409" t="n">
+      <c r="I409" s="10" t="n">
         <v>433400000</v>
       </c>
-      <c r="J409" t="b">
-        <v>0</v>
-      </c>
-      <c r="K409" t="n">
+      <c r="J409" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K409" s="10" t="n">
         <v>187300000</v>
       </c>
-      <c r="L409" t="b">
-        <v>0</v>
-      </c>
-      <c r="M409" t="n">
+      <c r="L409" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M409" s="10" t="n">
         <v>109</v>
       </c>
-      <c r="N409" t="n">
-        <v>0</v>
-      </c>
-      <c r="O409" t="n">
-        <v>0</v>
-      </c>
-      <c r="P409" t="b">
+      <c r="N409" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O409" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P409" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="410">
-      <c r="A410" t="inlineStr">
+      <c r="A410" s="10" t="inlineStr">
         <is>
           <t>Terminator Salvation</t>
         </is>
       </c>
-      <c r="B410" t="inlineStr">
+      <c r="B410" s="10" t="inlineStr">
         <is>
           <t>card_409</t>
         </is>
       </c>
-      <c r="C410" t="inlineStr">
+      <c r="C410" s="10" t="inlineStr">
         <is>
           <t>McG</t>
         </is>
       </c>
-      <c r="D410" t="n">
+      <c r="D410" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E410" t="n">
+      <c r="E410" s="10" t="n">
         <v>2.64</v>
       </c>
-      <c r="F410" t="n">
+      <c r="F410" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I410" t="n">
+      <c r="I410" s="10" t="n">
         <v>371400000</v>
       </c>
-      <c r="J410" t="b">
-        <v>0</v>
-      </c>
-      <c r="K410" t="n">
+      <c r="J410" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K410" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L410" t="b">
-        <v>0</v>
-      </c>
-      <c r="M410" t="n">
+      <c r="L410" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M410" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N410" t="n">
-        <v>0</v>
-      </c>
-      <c r="O410" t="n">
-        <v>0</v>
-      </c>
-      <c r="P410" t="b">
+      <c r="N410" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O410" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P410" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="411">
-      <c r="A411" t="inlineStr">
+      <c r="A411" s="10" t="inlineStr">
         <is>
           <t>Terminator Genisys</t>
         </is>
       </c>
-      <c r="B411" t="inlineStr">
+      <c r="B411" s="10" t="inlineStr">
         <is>
           <t>card_410</t>
         </is>
       </c>
-      <c r="C411" t="inlineStr">
+      <c r="C411" s="10" t="inlineStr">
         <is>
           <t>Alan Taylor</t>
         </is>
       </c>
-      <c r="D411" t="n">
+      <c r="D411" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E411" t="n">
+      <c r="E411" s="10" t="n">
         <v>2.26</v>
       </c>
-      <c r="F411" t="n">
+      <c r="F411" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="I411" t="n">
+      <c r="I411" s="10" t="n">
         <v>440600000</v>
       </c>
-      <c r="J411" t="b">
-        <v>0</v>
-      </c>
-      <c r="K411" t="n">
+      <c r="J411" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K411" s="10" t="n">
         <v>155000000</v>
       </c>
-      <c r="L411" t="b">
-        <v>0</v>
-      </c>
-      <c r="M411" t="n">
+      <c r="L411" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M411" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="N411" t="n">
-        <v>0</v>
-      </c>
-      <c r="O411" t="n">
-        <v>0</v>
-      </c>
-      <c r="P411" t="b">
+      <c r="N411" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O411" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P411" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="412">
-      <c r="A412" t="inlineStr">
+      <c r="A412" s="10" t="inlineStr">
         <is>
           <t>Terminator: Dark Fate</t>
         </is>
       </c>
-      <c r="B412" t="inlineStr">
+      <c r="B412" s="10" t="inlineStr">
         <is>
           <t>card_411</t>
         </is>
       </c>
-      <c r="C412" t="inlineStr">
+      <c r="C412" s="10" t="inlineStr">
         <is>
           <t>Tim Miller</t>
         </is>
       </c>
-      <c r="D412" t="n">
+      <c r="D412" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E412" t="n">
+      <c r="E412" s="10" t="n">
         <v>2.59</v>
       </c>
-      <c r="F412" t="n">
+      <c r="F412" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="I412" t="n">
+      <c r="I412" s="10" t="n">
         <v>261100000</v>
       </c>
-      <c r="J412" t="b">
-        <v>0</v>
-      </c>
-      <c r="K412" t="n">
+      <c r="J412" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K412" s="10" t="n">
         <v>185000000</v>
       </c>
-      <c r="L412" t="b">
-        <v>0</v>
-      </c>
-      <c r="M412" t="n">
+      <c r="L412" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M412" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N412" t="n">
-        <v>0</v>
-      </c>
-      <c r="O412" t="n">
-        <v>0</v>
-      </c>
-      <c r="P412" t="b">
+      <c r="N412" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O412" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P412" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="413">
-      <c r="A413" t="inlineStr">
+      <c r="A413" s="10" t="inlineStr">
         <is>
           <t>Back to the Future Part II</t>
         </is>
       </c>
-      <c r="B413" t="inlineStr">
+      <c r="B413" s="10" t="inlineStr">
         <is>
           <t>card_412</t>
         </is>
       </c>
-      <c r="C413" t="inlineStr">
+      <c r="C413" s="10" t="inlineStr">
         <is>
           <t>Robert Zemeckis</t>
         </is>
       </c>
-      <c r="D413" t="n">
+      <c r="D413" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E413" t="n">
+      <c r="E413" s="10" t="n">
         <v>3.91</v>
       </c>
-      <c r="F413" t="n">
+      <c r="F413" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I413" t="n">
+      <c r="I413" s="10" t="n">
         <v>333000000</v>
       </c>
-      <c r="J413" t="b">
-        <v>0</v>
-      </c>
-      <c r="K413" t="n">
+      <c r="J413" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K413" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L413" t="b">
-        <v>0</v>
-      </c>
-      <c r="M413" t="n">
+      <c r="L413" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M413" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="N413" t="n">
-        <v>0</v>
-      </c>
-      <c r="O413" t="n">
+      <c r="N413" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O413" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P413" t="b">
+      <c r="P413" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="414">
-      <c r="A414" t="inlineStr">
+      <c r="A414" s="10" t="inlineStr">
         <is>
           <t>Back to the Future Part III</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
+      <c r="B414" s="10" t="inlineStr">
         <is>
           <t>card_413</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr">
+      <c r="C414" s="10" t="inlineStr">
         <is>
           <t>Robert Zemeckis</t>
         </is>
       </c>
-      <c r="D414" t="n">
+      <c r="D414" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E414" t="n">
+      <c r="E414" s="10" t="n">
         <v>3.61</v>
       </c>
-      <c r="F414" t="n">
+      <c r="F414" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I414" t="n">
+      <c r="I414" s="10" t="n">
         <v>245100000</v>
       </c>
-      <c r="J414" t="b">
-        <v>0</v>
-      </c>
-      <c r="K414" t="n">
+      <c r="J414" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K414" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L414" t="b">
-        <v>0</v>
-      </c>
-      <c r="M414" t="n">
+      <c r="L414" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M414" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N414" t="n">
-        <v>0</v>
-      </c>
-      <c r="O414" t="n">
+      <c r="N414" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O414" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P414" t="b">
+      <c r="P414" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="415">
-      <c r="A415" t="inlineStr">
+      <c r="A415" s="10" t="inlineStr">
         <is>
           <t>Mad Max</t>
         </is>
       </c>
-      <c r="B415" t="inlineStr">
+      <c r="B415" s="10" t="inlineStr">
         <is>
           <t>card_414</t>
         </is>
       </c>
-      <c r="C415" t="inlineStr">
+      <c r="C415" s="10" t="inlineStr">
         <is>
           <t>George Miller</t>
         </is>
       </c>
-      <c r="D415" t="n">
+      <c r="D415" s="10" t="n">
         <v>1979</v>
       </c>
-      <c r="E415" t="n">
+      <c r="E415" s="10" t="n">
         <v>3.29</v>
       </c>
-      <c r="F415" t="n">
+      <c r="F415" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I415" t="n">
+      <c r="I415" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="J415" t="b">
+      <c r="J415" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K415" t="n">
+      <c r="K415" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="L415" t="b">
-        <v>0</v>
-      </c>
-      <c r="M415" t="n">
+      <c r="L415" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M415" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N415" t="n">
-        <v>0</v>
-      </c>
-      <c r="O415" t="n">
-        <v>0</v>
-      </c>
-      <c r="P415" t="b">
+      <c r="N415" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O415" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P415" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="416">
-      <c r="A416" t="inlineStr">
+      <c r="A416" s="10" t="inlineStr">
         <is>
           <t>Mad Max 2</t>
         </is>
       </c>
-      <c r="B416" t="inlineStr">
+      <c r="B416" s="10" t="inlineStr">
         <is>
           <t>card_415</t>
         </is>
       </c>
-      <c r="C416" t="inlineStr">
+      <c r="C416" s="10" t="inlineStr">
         <is>
           <t>George Miller</t>
         </is>
       </c>
-      <c r="D416" t="n">
+      <c r="D416" s="10" t="n">
         <v>1981</v>
       </c>
-      <c r="E416" t="n">
+      <c r="E416" s="10" t="n">
         <v>3.89</v>
       </c>
-      <c r="F416" t="n">
+      <c r="F416" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I416" t="n">
+      <c r="I416" s="10" t="n">
         <v>23700000</v>
       </c>
-      <c r="J416" t="b">
-        <v>0</v>
-      </c>
-      <c r="K416" t="n">
+      <c r="J416" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K416" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="L416" t="b">
-        <v>0</v>
-      </c>
-      <c r="M416" t="n">
+      <c r="L416" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M416" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N416" t="n">
-        <v>0</v>
-      </c>
-      <c r="O416" t="n">
-        <v>0</v>
-      </c>
-      <c r="P416" t="b">
+      <c r="N416" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O416" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P416" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="417">
-      <c r="A417" t="inlineStr">
+      <c r="A417" s="10" t="inlineStr">
         <is>
           <t>Mad Max Beyond Thunderdome</t>
         </is>
       </c>
-      <c r="B417" t="inlineStr">
+      <c r="B417" s="10" t="inlineStr">
         <is>
           <t>card_416</t>
         </is>
       </c>
-      <c r="C417" t="inlineStr">
+      <c r="C417" s="10" t="inlineStr">
         <is>
           <t>George Miller and George Ogilvie</t>
         </is>
       </c>
-      <c r="D417" t="n">
+      <c r="D417" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E417" t="n">
+      <c r="E417" s="10" t="n">
         <v>2.98</v>
       </c>
-      <c r="F417" t="n">
+      <c r="F417" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I417" t="n">
+      <c r="I417" s="10" t="n">
         <v>36200000</v>
       </c>
-      <c r="J417" t="b">
-        <v>0</v>
-      </c>
-      <c r="K417" t="n">
+      <c r="J417" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K417" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L417" t="b">
-        <v>0</v>
-      </c>
-      <c r="M417" t="n">
+      <c r="L417" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M417" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N417" t="n">
-        <v>0</v>
-      </c>
-      <c r="O417" t="n">
-        <v>0</v>
-      </c>
-      <c r="P417" t="b">
+      <c r="N417" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O417" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P417" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="418">
-      <c r="A418" t="inlineStr">
+      <c r="A418" s="10" t="inlineStr">
         <is>
           <t>Furiosa: A Mad Max Saga</t>
         </is>
       </c>
-      <c r="B418" t="inlineStr">
+      <c r="B418" s="10" t="inlineStr">
         <is>
           <t>card_417</t>
         </is>
       </c>
-      <c r="C418" t="inlineStr">
+      <c r="C418" s="10" t="inlineStr">
         <is>
           <t>George Miller</t>
         </is>
       </c>
-      <c r="D418" t="n">
+      <c r="D418" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="E418" t="n">
+      <c r="E418" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F418" t="n">
+      <c r="F418" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I418" t="n">
+      <c r="I418" s="10" t="n">
         <v>174400000</v>
       </c>
-      <c r="J418" t="b">
-        <v>0</v>
-      </c>
-      <c r="K418" t="n">
+      <c r="J418" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K418" s="10" t="n">
         <v>168000000</v>
       </c>
-      <c r="L418" t="b">
-        <v>0</v>
-      </c>
-      <c r="M418" t="n">
+      <c r="L418" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M418" s="10" t="n">
         <v>148</v>
       </c>
-      <c r="N418" t="n">
-        <v>0</v>
-      </c>
-      <c r="O418" t="n">
-        <v>0</v>
-      </c>
-      <c r="P418" t="b">
+      <c r="N418" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O418" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P418" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Rocky II</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>card_418</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>Sylvester Stallone</t>
+        </is>
+      </c>
+      <c r="D419" t="n">
+        <v>1979</v>
+      </c>
+      <c r="E419" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F419" t="n">
+        <v>82</v>
+      </c>
+      <c r="I419" t="n">
+        <v>200100000</v>
+      </c>
+      <c r="J419" t="b">
+        <v>0</v>
+      </c>
+      <c r="K419" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="L419" t="b">
+        <v>0</v>
+      </c>
+      <c r="M419" t="n">
+        <v>119</v>
+      </c>
+      <c r="N419" t="n">
+        <v>0</v>
+      </c>
+      <c r="O419" t="n">
+        <v>0</v>
+      </c>
+      <c r="P419" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Rocky III</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>card_419</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Sylvester Stallone</t>
+        </is>
+      </c>
+      <c r="D420" t="n">
+        <v>1982</v>
+      </c>
+      <c r="E420" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="F420" t="n">
+        <v>76</v>
+      </c>
+      <c r="I420" t="n">
+        <v>270000000</v>
+      </c>
+      <c r="J420" t="b">
+        <v>0</v>
+      </c>
+      <c r="K420" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="L420" t="b">
+        <v>0</v>
+      </c>
+      <c r="M420" t="n">
+        <v>100</v>
+      </c>
+      <c r="N420" t="n">
+        <v>0</v>
+      </c>
+      <c r="O420" t="n">
+        <v>0</v>
+      </c>
+      <c r="P420" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Rocky IV</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>card_420</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Sylvester Stallone</t>
+        </is>
+      </c>
+      <c r="D421" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E421" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F421" t="n">
+        <v>73</v>
+      </c>
+      <c r="I421" t="n">
+        <v>300500000</v>
+      </c>
+      <c r="J421" t="b">
+        <v>0</v>
+      </c>
+      <c r="K421" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="L421" t="b">
+        <v>0</v>
+      </c>
+      <c r="M421" t="n">
+        <v>91</v>
+      </c>
+      <c r="N421" t="n">
+        <v>0</v>
+      </c>
+      <c r="O421" t="n">
+        <v>0</v>
+      </c>
+      <c r="P421" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Rocky V</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>card_421</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>John G. Avildsen</t>
+        </is>
+      </c>
+      <c r="D422" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E422" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F422" t="n">
+        <v>56</v>
+      </c>
+      <c r="I422" t="n">
+        <v>119900000</v>
+      </c>
+      <c r="J422" t="b">
+        <v>0</v>
+      </c>
+      <c r="K422" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="L422" t="b">
+        <v>1</v>
+      </c>
+      <c r="M422" t="n">
+        <v>104</v>
+      </c>
+      <c r="N422" t="n">
+        <v>0</v>
+      </c>
+      <c r="O422" t="n">
+        <v>0</v>
+      </c>
+      <c r="P422" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Rocky Balboa</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>card_422</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Sylvester Stallone</t>
+        </is>
+      </c>
+      <c r="D423" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E423" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F423" t="n">
+        <v>77</v>
+      </c>
+      <c r="I423" t="n">
+        <v>156000000</v>
+      </c>
+      <c r="J423" t="b">
+        <v>0</v>
+      </c>
+      <c r="K423" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="L423" t="b">
+        <v>0</v>
+      </c>
+      <c r="M423" t="n">
+        <v>102</v>
+      </c>
+      <c r="N423" t="n">
+        <v>0</v>
+      </c>
+      <c r="O423" t="n">
+        <v>0</v>
+      </c>
+      <c r="P423" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Creed</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>card_423</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Ryan Coogler</t>
+        </is>
+      </c>
+      <c r="D424" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E424" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F424" t="n">
+        <v>80</v>
+      </c>
+      <c r="I424" t="n">
+        <v>174100000</v>
+      </c>
+      <c r="J424" t="b">
+        <v>0</v>
+      </c>
+      <c r="K424" t="n">
+        <v>37000000</v>
+      </c>
+      <c r="L424" t="b">
+        <v>0</v>
+      </c>
+      <c r="M424" t="n">
+        <v>133</v>
+      </c>
+      <c r="N424" t="n">
+        <v>0</v>
+      </c>
+      <c r="O424" t="n">
+        <v>0</v>
+      </c>
+      <c r="P424" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Creed II</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>card_424</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Steven Caple Jr.</t>
+        </is>
+      </c>
+      <c r="D425" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E425" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F425" t="n">
+        <v>71</v>
+      </c>
+      <c r="I425" t="n">
+        <v>214200000</v>
+      </c>
+      <c r="J425" t="b">
+        <v>0</v>
+      </c>
+      <c r="K425" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="L425" t="b">
+        <v>0</v>
+      </c>
+      <c r="M425" t="n">
+        <v>130</v>
+      </c>
+      <c r="N425" t="n">
+        <v>0</v>
+      </c>
+      <c r="O425" t="n">
+        <v>0</v>
+      </c>
+      <c r="P425" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Creed III</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>card_425</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Michael B. Jordan</t>
+        </is>
+      </c>
+      <c r="D426" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E426" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="F426" t="n">
+        <v>68</v>
+      </c>
+      <c r="I426" t="n">
+        <v>276100000</v>
+      </c>
+      <c r="J426" t="b">
+        <v>0</v>
+      </c>
+      <c r="K426" t="n">
+        <v>75000000</v>
+      </c>
+      <c r="L426" t="b">
+        <v>0</v>
+      </c>
+      <c r="M426" t="n">
+        <v>116</v>
+      </c>
+      <c r="N426" t="n">
+        <v>0</v>
+      </c>
+      <c r="O426" t="n">
+        <v>0</v>
+      </c>
+      <c r="P426" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add John Wick, Lethal Weapon, Bourne series (card_426-438)
John Wick 1-4, Lethal Weapon 1-4, Bourne Identity/Supremacy/
Ultimatum/Legacy, Jason Bourne.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P426"/>
+  <dimension ref="A1:P439"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -22569,402 +22569,1052 @@
       </c>
     </row>
     <row r="419">
-      <c r="A419" t="inlineStr">
+      <c r="A419" s="10" t="inlineStr">
         <is>
           <t>Rocky II</t>
         </is>
       </c>
-      <c r="B419" t="inlineStr">
+      <c r="B419" s="10" t="inlineStr">
         <is>
           <t>card_418</t>
         </is>
       </c>
-      <c r="C419" t="inlineStr">
+      <c r="C419" s="10" t="inlineStr">
         <is>
           <t>Sylvester Stallone</t>
         </is>
       </c>
-      <c r="D419" t="n">
+      <c r="D419" s="10" t="n">
         <v>1979</v>
       </c>
-      <c r="E419" t="n">
+      <c r="E419" s="10" t="n">
         <v>3.84</v>
       </c>
-      <c r="F419" t="n">
+      <c r="F419" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I419" t="n">
+      <c r="I419" s="10" t="n">
         <v>200100000</v>
       </c>
-      <c r="J419" t="b">
-        <v>0</v>
-      </c>
-      <c r="K419" t="n">
+      <c r="J419" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K419" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="L419" t="b">
-        <v>0</v>
-      </c>
-      <c r="M419" t="n">
+      <c r="L419" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M419" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="N419" t="n">
-        <v>0</v>
-      </c>
-      <c r="O419" t="n">
-        <v>0</v>
-      </c>
-      <c r="P419" t="b">
+      <c r="N419" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O419" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P419" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="420">
-      <c r="A420" t="inlineStr">
+      <c r="A420" s="10" t="inlineStr">
         <is>
           <t>Rocky III</t>
         </is>
       </c>
-      <c r="B420" t="inlineStr">
+      <c r="B420" s="10" t="inlineStr">
         <is>
           <t>card_419</t>
         </is>
       </c>
-      <c r="C420" t="inlineStr">
+      <c r="C420" s="10" t="inlineStr">
         <is>
           <t>Sylvester Stallone</t>
         </is>
       </c>
-      <c r="D420" t="n">
+      <c r="D420" s="10" t="n">
         <v>1982</v>
       </c>
-      <c r="E420" t="n">
+      <c r="E420" s="10" t="n">
         <v>3.58</v>
       </c>
-      <c r="F420" t="n">
+      <c r="F420" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I420" t="n">
+      <c r="I420" s="10" t="n">
         <v>270000000</v>
       </c>
-      <c r="J420" t="b">
-        <v>0</v>
-      </c>
-      <c r="K420" t="n">
+      <c r="J420" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K420" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="L420" t="b">
-        <v>0</v>
-      </c>
-      <c r="M420" t="n">
+      <c r="L420" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M420" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="N420" t="n">
-        <v>0</v>
-      </c>
-      <c r="O420" t="n">
-        <v>0</v>
-      </c>
-      <c r="P420" t="b">
+      <c r="N420" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O420" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P420" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="421">
-      <c r="A421" t="inlineStr">
+      <c r="A421" s="10" t="inlineStr">
         <is>
           <t>Rocky IV</t>
         </is>
       </c>
-      <c r="B421" t="inlineStr">
+      <c r="B421" s="10" t="inlineStr">
         <is>
           <t>card_420</t>
         </is>
       </c>
-      <c r="C421" t="inlineStr">
+      <c r="C421" s="10" t="inlineStr">
         <is>
           <t>Sylvester Stallone</t>
         </is>
       </c>
-      <c r="D421" t="n">
+      <c r="D421" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E421" t="n">
+      <c r="E421" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F421" t="n">
+      <c r="F421" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I421" t="n">
+      <c r="I421" s="10" t="n">
         <v>300500000</v>
       </c>
-      <c r="J421" t="b">
-        <v>0</v>
-      </c>
-      <c r="K421" t="n">
+      <c r="J421" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K421" s="10" t="n">
         <v>28000000</v>
       </c>
-      <c r="L421" t="b">
-        <v>0</v>
-      </c>
-      <c r="M421" t="n">
+      <c r="L421" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M421" s="10" t="n">
         <v>91</v>
       </c>
-      <c r="N421" t="n">
-        <v>0</v>
-      </c>
-      <c r="O421" t="n">
-        <v>0</v>
-      </c>
-      <c r="P421" t="b">
+      <c r="N421" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O421" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P421" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="422">
-      <c r="A422" t="inlineStr">
+      <c r="A422" s="10" t="inlineStr">
         <is>
           <t>Rocky V</t>
         </is>
       </c>
-      <c r="B422" t="inlineStr">
+      <c r="B422" s="10" t="inlineStr">
         <is>
           <t>card_421</t>
         </is>
       </c>
-      <c r="C422" t="inlineStr">
+      <c r="C422" s="10" t="inlineStr">
         <is>
           <t>John G. Avildsen</t>
         </is>
       </c>
-      <c r="D422" t="n">
+      <c r="D422" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E422" t="n">
+      <c r="E422" s="10" t="n">
         <v>2.55</v>
       </c>
-      <c r="F422" t="n">
+      <c r="F422" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="I422" t="n">
+      <c r="I422" s="10" t="n">
         <v>119900000</v>
       </c>
-      <c r="J422" t="b">
-        <v>0</v>
-      </c>
-      <c r="K422" t="n">
+      <c r="J422" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K422" s="10" t="n">
         <v>36000000</v>
       </c>
-      <c r="L422" t="b">
+      <c r="L422" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M422" t="n">
+      <c r="M422" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="N422" t="n">
-        <v>0</v>
-      </c>
-      <c r="O422" t="n">
-        <v>0</v>
-      </c>
-      <c r="P422" t="b">
+      <c r="N422" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O422" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P422" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="423">
-      <c r="A423" t="inlineStr">
+      <c r="A423" s="10" t="inlineStr">
         <is>
           <t>Rocky Balboa</t>
         </is>
       </c>
-      <c r="B423" t="inlineStr">
+      <c r="B423" s="10" t="inlineStr">
         <is>
           <t>card_422</t>
         </is>
       </c>
-      <c r="C423" t="inlineStr">
+      <c r="C423" s="10" t="inlineStr">
         <is>
           <t>Sylvester Stallone</t>
         </is>
       </c>
-      <c r="D423" t="n">
+      <c r="D423" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E423" t="n">
+      <c r="E423" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="F423" t="n">
+      <c r="F423" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I423" t="n">
+      <c r="I423" s="10" t="n">
         <v>156000000</v>
       </c>
-      <c r="J423" t="b">
-        <v>0</v>
-      </c>
-      <c r="K423" t="n">
+      <c r="J423" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K423" s="10" t="n">
         <v>24000000</v>
       </c>
-      <c r="L423" t="b">
-        <v>0</v>
-      </c>
-      <c r="M423" t="n">
+      <c r="L423" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M423" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="N423" t="n">
-        <v>0</v>
-      </c>
-      <c r="O423" t="n">
-        <v>0</v>
-      </c>
-      <c r="P423" t="b">
+      <c r="N423" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O423" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P423" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="424">
-      <c r="A424" t="inlineStr">
+      <c r="A424" s="10" t="inlineStr">
         <is>
           <t>Creed</t>
         </is>
       </c>
-      <c r="B424" t="inlineStr">
+      <c r="B424" s="10" t="inlineStr">
         <is>
           <t>card_423</t>
         </is>
       </c>
-      <c r="C424" t="inlineStr">
+      <c r="C424" s="10" t="inlineStr">
         <is>
           <t>Ryan Coogler</t>
         </is>
       </c>
-      <c r="D424" t="n">
+      <c r="D424" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E424" t="n">
+      <c r="E424" s="10" t="n">
         <v>3.83</v>
       </c>
-      <c r="F424" t="n">
+      <c r="F424" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I424" t="n">
+      <c r="I424" s="10" t="n">
         <v>174100000</v>
       </c>
-      <c r="J424" t="b">
-        <v>0</v>
-      </c>
-      <c r="K424" t="n">
+      <c r="J424" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K424" s="10" t="n">
         <v>37000000</v>
       </c>
-      <c r="L424" t="b">
-        <v>0</v>
-      </c>
-      <c r="M424" t="n">
+      <c r="L424" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M424" s="10" t="n">
         <v>133</v>
       </c>
-      <c r="N424" t="n">
-        <v>0</v>
-      </c>
-      <c r="O424" t="n">
-        <v>0</v>
-      </c>
-      <c r="P424" t="b">
+      <c r="N424" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O424" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P424" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="425">
-      <c r="A425" t="inlineStr">
+      <c r="A425" s="10" t="inlineStr">
         <is>
           <t>Creed II</t>
         </is>
       </c>
-      <c r="B425" t="inlineStr">
+      <c r="B425" s="10" t="inlineStr">
         <is>
           <t>card_424</t>
         </is>
       </c>
-      <c r="C425" t="inlineStr">
+      <c r="C425" s="10" t="inlineStr">
         <is>
           <t>Steven Caple Jr.</t>
         </is>
       </c>
-      <c r="D425" t="n">
+      <c r="D425" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E425" t="n">
+      <c r="E425" s="10" t="n">
         <v>3.59</v>
       </c>
-      <c r="F425" t="n">
+      <c r="F425" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I425" t="n">
+      <c r="I425" s="10" t="n">
         <v>214200000</v>
       </c>
-      <c r="J425" t="b">
-        <v>0</v>
-      </c>
-      <c r="K425" t="n">
+      <c r="J425" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K425" s="10" t="n">
         <v>50000000</v>
       </c>
-      <c r="L425" t="b">
-        <v>0</v>
-      </c>
-      <c r="M425" t="n">
+      <c r="L425" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M425" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N425" t="n">
-        <v>0</v>
-      </c>
-      <c r="O425" t="n">
-        <v>0</v>
-      </c>
-      <c r="P425" t="b">
+      <c r="N425" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O425" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P425" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="426">
-      <c r="A426" t="inlineStr">
+      <c r="A426" s="10" t="inlineStr">
         <is>
           <t>Creed III</t>
         </is>
       </c>
-      <c r="B426" t="inlineStr">
+      <c r="B426" s="10" t="inlineStr">
         <is>
           <t>card_425</t>
         </is>
       </c>
-      <c r="C426" t="inlineStr">
+      <c r="C426" s="10" t="inlineStr">
         <is>
           <t>Michael B. Jordan</t>
         </is>
       </c>
-      <c r="D426" t="n">
+      <c r="D426" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E426" t="n">
+      <c r="E426" s="10" t="n">
         <v>3.44</v>
       </c>
-      <c r="F426" t="n">
+      <c r="F426" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I426" t="n">
+      <c r="I426" s="10" t="n">
         <v>276100000</v>
       </c>
-      <c r="J426" t="b">
-        <v>0</v>
-      </c>
-      <c r="K426" t="n">
+      <c r="J426" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K426" s="10" t="n">
         <v>75000000</v>
       </c>
-      <c r="L426" t="b">
-        <v>0</v>
-      </c>
-      <c r="M426" t="n">
+      <c r="L426" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M426" s="10" t="n">
         <v>116</v>
       </c>
-      <c r="N426" t="n">
-        <v>0</v>
-      </c>
-      <c r="O426" t="n">
-        <v>0</v>
-      </c>
-      <c r="P426" t="b">
+      <c r="N426" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O426" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P426" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>John Wick</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>card_426</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Chad Stahelski</t>
+        </is>
+      </c>
+      <c r="D427" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E427" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F427" t="n">
+        <v>78</v>
+      </c>
+      <c r="I427" t="n">
+        <v>86100000</v>
+      </c>
+      <c r="J427" t="b">
+        <v>0</v>
+      </c>
+      <c r="K427" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L427" t="b">
+        <v>0</v>
+      </c>
+      <c r="M427" t="n">
+        <v>101</v>
+      </c>
+      <c r="N427" t="n">
+        <v>0</v>
+      </c>
+      <c r="O427" t="n">
+        <v>0</v>
+      </c>
+      <c r="P427" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>John Wick: Chapter 2</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>card_427</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Chad Stahelski</t>
+        </is>
+      </c>
+      <c r="D428" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E428" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F428" t="n">
+        <v>80</v>
+      </c>
+      <c r="I428" t="n">
+        <v>174300000</v>
+      </c>
+      <c r="J428" t="b">
+        <v>0</v>
+      </c>
+      <c r="K428" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L428" t="b">
+        <v>0</v>
+      </c>
+      <c r="M428" t="n">
+        <v>122</v>
+      </c>
+      <c r="N428" t="n">
+        <v>0</v>
+      </c>
+      <c r="O428" t="n">
+        <v>0</v>
+      </c>
+      <c r="P428" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>John Wick: Chapter 3 - Parabellum</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>card_428</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Chad Stahelski</t>
+        </is>
+      </c>
+      <c r="D429" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E429" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F429" t="n">
+        <v>84</v>
+      </c>
+      <c r="I429" t="n">
+        <v>328300000</v>
+      </c>
+      <c r="J429" t="b">
+        <v>0</v>
+      </c>
+      <c r="K429" t="n">
+        <v>75000000</v>
+      </c>
+      <c r="L429" t="b">
+        <v>0</v>
+      </c>
+      <c r="M429" t="n">
+        <v>131</v>
+      </c>
+      <c r="N429" t="n">
+        <v>0</v>
+      </c>
+      <c r="O429" t="n">
+        <v>0</v>
+      </c>
+      <c r="P429" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>John Wick: Chapter 4</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>card_429</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Chad Stahelski</t>
+        </is>
+      </c>
+      <c r="D430" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E430" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F430" t="n">
+        <v>80</v>
+      </c>
+      <c r="I430" t="n">
+        <v>447300000</v>
+      </c>
+      <c r="J430" t="b">
+        <v>0</v>
+      </c>
+      <c r="K430" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L430" t="b">
+        <v>0</v>
+      </c>
+      <c r="M430" t="n">
+        <v>169</v>
+      </c>
+      <c r="N430" t="n">
+        <v>0</v>
+      </c>
+      <c r="O430" t="n">
+        <v>0</v>
+      </c>
+      <c r="P430" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Lethal Weapon</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>card_430</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Richard Donner</t>
+        </is>
+      </c>
+      <c r="D431" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E431" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F431" t="n">
+        <v>77</v>
+      </c>
+      <c r="I431" t="n">
+        <v>120100000</v>
+      </c>
+      <c r="J431" t="b">
+        <v>0</v>
+      </c>
+      <c r="K431" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L431" t="b">
+        <v>0</v>
+      </c>
+      <c r="M431" t="n">
+        <v>109</v>
+      </c>
+      <c r="N431" t="n">
+        <v>0</v>
+      </c>
+      <c r="O431" t="n">
+        <v>0</v>
+      </c>
+      <c r="P431" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Lethal Weapon 2</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>card_431</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Richard Donner</t>
+        </is>
+      </c>
+      <c r="D432" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E432" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F432" t="n">
+        <v>76</v>
+      </c>
+      <c r="I432" t="n">
+        <v>227300000</v>
+      </c>
+      <c r="J432" t="b">
+        <v>0</v>
+      </c>
+      <c r="K432" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L432" t="b">
+        <v>0</v>
+      </c>
+      <c r="M432" t="n">
+        <v>114</v>
+      </c>
+      <c r="N432" t="n">
+        <v>0</v>
+      </c>
+      <c r="O432" t="n">
+        <v>0</v>
+      </c>
+      <c r="P432" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Lethal Weapon 3</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>card_432</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Richard Donner</t>
+        </is>
+      </c>
+      <c r="D433" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E433" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F433" t="n">
+        <v>68</v>
+      </c>
+      <c r="I433" t="n">
+        <v>321700000</v>
+      </c>
+      <c r="J433" t="b">
+        <v>0</v>
+      </c>
+      <c r="K433" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="L433" t="b">
+        <v>0</v>
+      </c>
+      <c r="M433" t="n">
+        <v>118</v>
+      </c>
+      <c r="N433" t="n">
+        <v>0</v>
+      </c>
+      <c r="O433" t="n">
+        <v>0</v>
+      </c>
+      <c r="P433" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Lethal Weapon 4</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>card_433</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Richard Donner</t>
+        </is>
+      </c>
+      <c r="D434" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E434" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F434" t="n">
+        <v>63</v>
+      </c>
+      <c r="I434" t="n">
+        <v>285400000</v>
+      </c>
+      <c r="J434" t="b">
+        <v>0</v>
+      </c>
+      <c r="K434" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L434" t="b">
+        <v>1</v>
+      </c>
+      <c r="M434" t="n">
+        <v>127</v>
+      </c>
+      <c r="N434" t="n">
+        <v>0</v>
+      </c>
+      <c r="O434" t="n">
+        <v>0</v>
+      </c>
+      <c r="P434" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>The Bourne Identity</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>card_434</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Doug Liman</t>
+        </is>
+      </c>
+      <c r="D435" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E435" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F435" t="n">
+        <v>80</v>
+      </c>
+      <c r="I435" t="n">
+        <v>214000000</v>
+      </c>
+      <c r="J435" t="b">
+        <v>0</v>
+      </c>
+      <c r="K435" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="L435" t="b">
+        <v>0</v>
+      </c>
+      <c r="M435" t="n">
+        <v>119</v>
+      </c>
+      <c r="N435" t="n">
+        <v>0</v>
+      </c>
+      <c r="O435" t="n">
+        <v>0</v>
+      </c>
+      <c r="P435" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>The Bourne Supremacy</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>card_435</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Paul Greengrass</t>
+        </is>
+      </c>
+      <c r="D436" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E436" t="n">
+        <v>3.63</v>
+      </c>
+      <c r="F436" t="n">
+        <v>79</v>
+      </c>
+      <c r="I436" t="n">
+        <v>311000000</v>
+      </c>
+      <c r="J436" t="b">
+        <v>0</v>
+      </c>
+      <c r="K436" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L436" t="b">
+        <v>0</v>
+      </c>
+      <c r="M436" t="n">
+        <v>108</v>
+      </c>
+      <c r="N436" t="n">
+        <v>0</v>
+      </c>
+      <c r="O436" t="n">
+        <v>0</v>
+      </c>
+      <c r="P436" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>The Bourne Ultimatum</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>card_436</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>Paul Greengrass</t>
+        </is>
+      </c>
+      <c r="D437" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E437" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="F437" t="n">
+        <v>83</v>
+      </c>
+      <c r="I437" t="n">
+        <v>444000000</v>
+      </c>
+      <c r="J437" t="b">
+        <v>0</v>
+      </c>
+      <c r="K437" t="n">
+        <v>120000000</v>
+      </c>
+      <c r="L437" t="b">
+        <v>0</v>
+      </c>
+      <c r="M437" t="n">
+        <v>115</v>
+      </c>
+      <c r="N437" t="n">
+        <v>3</v>
+      </c>
+      <c r="O437" t="n">
+        <v>0</v>
+      </c>
+      <c r="P437" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>The Bourne Legacy</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>card_437</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Tony Gilroy</t>
+        </is>
+      </c>
+      <c r="D438" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E438" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F438" t="n">
+        <v>62</v>
+      </c>
+      <c r="I438" t="n">
+        <v>276100000</v>
+      </c>
+      <c r="J438" t="b">
+        <v>0</v>
+      </c>
+      <c r="K438" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L438" t="b">
+        <v>0</v>
+      </c>
+      <c r="M438" t="n">
+        <v>135</v>
+      </c>
+      <c r="N438" t="n">
+        <v>0</v>
+      </c>
+      <c r="O438" t="n">
+        <v>0</v>
+      </c>
+      <c r="P438" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Jason Bourne</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>card_438</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Paul Greengrass</t>
+        </is>
+      </c>
+      <c r="D439" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E439" t="n">
+        <v>3</v>
+      </c>
+      <c r="F439" t="n">
+        <v>64</v>
+      </c>
+      <c r="I439" t="n">
+        <v>416200000</v>
+      </c>
+      <c r="J439" t="b">
+        <v>0</v>
+      </c>
+      <c r="K439" t="n">
+        <v>120000000</v>
+      </c>
+      <c r="L439" t="b">
+        <v>0</v>
+      </c>
+      <c r="M439" t="n">
+        <v>123</v>
+      </c>
+      <c r="N439" t="n">
+        <v>0</v>
+      </c>
+      <c r="O439" t="n">
+        <v>0</v>
+      </c>
+      <c r="P439" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Pirates of the Caribbean series (card_439-443)
All 5 films: Curse of the Black Pearl, Dead Man's Chest, At World's
End, On Stranger Tides, Dead Men Tell No Tales.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P439"/>
+  <dimension ref="A1:P444"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -22969,652 +22969,902 @@
       </c>
     </row>
     <row r="427">
-      <c r="A427" t="inlineStr">
+      <c r="A427" s="10" t="inlineStr">
         <is>
           <t>John Wick</t>
         </is>
       </c>
-      <c r="B427" t="inlineStr">
+      <c r="B427" s="10" t="inlineStr">
         <is>
           <t>card_426</t>
         </is>
       </c>
-      <c r="C427" t="inlineStr">
+      <c r="C427" s="10" t="inlineStr">
         <is>
           <t>Chad Stahelski</t>
         </is>
       </c>
-      <c r="D427" t="n">
+      <c r="D427" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E427" t="n">
+      <c r="E427" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="F427" t="n">
+      <c r="F427" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I427" t="n">
+      <c r="I427" s="10" t="n">
         <v>86100000</v>
       </c>
-      <c r="J427" t="b">
-        <v>0</v>
-      </c>
-      <c r="K427" t="n">
+      <c r="J427" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K427" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L427" t="b">
-        <v>0</v>
-      </c>
-      <c r="M427" t="n">
+      <c r="L427" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M427" s="10" t="n">
         <v>101</v>
       </c>
-      <c r="N427" t="n">
-        <v>0</v>
-      </c>
-      <c r="O427" t="n">
-        <v>0</v>
-      </c>
-      <c r="P427" t="b">
+      <c r="N427" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O427" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P427" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="428">
-      <c r="A428" t="inlineStr">
+      <c r="A428" s="10" t="inlineStr">
         <is>
           <t>John Wick: Chapter 2</t>
         </is>
       </c>
-      <c r="B428" t="inlineStr">
+      <c r="B428" s="10" t="inlineStr">
         <is>
           <t>card_427</t>
         </is>
       </c>
-      <c r="C428" t="inlineStr">
+      <c r="C428" s="10" t="inlineStr">
         <is>
           <t>Chad Stahelski</t>
         </is>
       </c>
-      <c r="D428" t="n">
+      <c r="D428" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E428" t="n">
+      <c r="E428" s="10" t="n">
         <v>3.72</v>
       </c>
-      <c r="F428" t="n">
+      <c r="F428" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I428" t="n">
+      <c r="I428" s="10" t="n">
         <v>174300000</v>
       </c>
-      <c r="J428" t="b">
-        <v>0</v>
-      </c>
-      <c r="K428" t="n">
+      <c r="J428" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K428" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L428" t="b">
-        <v>0</v>
-      </c>
-      <c r="M428" t="n">
+      <c r="L428" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M428" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N428" t="n">
-        <v>0</v>
-      </c>
-      <c r="O428" t="n">
-        <v>0</v>
-      </c>
-      <c r="P428" t="b">
+      <c r="N428" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O428" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P428" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="429">
-      <c r="A429" t="inlineStr">
+      <c r="A429" s="10" t="inlineStr">
         <is>
           <t>John Wick: Chapter 3 - Parabellum</t>
         </is>
       </c>
-      <c r="B429" t="inlineStr">
+      <c r="B429" s="10" t="inlineStr">
         <is>
           <t>card_428</t>
         </is>
       </c>
-      <c r="C429" t="inlineStr">
+      <c r="C429" s="10" t="inlineStr">
         <is>
           <t>Chad Stahelski</t>
         </is>
       </c>
-      <c r="D429" t="n">
+      <c r="D429" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E429" t="n">
+      <c r="E429" s="10" t="n">
         <v>3.71</v>
       </c>
-      <c r="F429" t="n">
+      <c r="F429" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="I429" t="n">
+      <c r="I429" s="10" t="n">
         <v>328300000</v>
       </c>
-      <c r="J429" t="b">
-        <v>0</v>
-      </c>
-      <c r="K429" t="n">
+      <c r="J429" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K429" s="10" t="n">
         <v>75000000</v>
       </c>
-      <c r="L429" t="b">
-        <v>0</v>
-      </c>
-      <c r="M429" t="n">
+      <c r="L429" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M429" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N429" t="n">
-        <v>0</v>
-      </c>
-      <c r="O429" t="n">
-        <v>0</v>
-      </c>
-      <c r="P429" t="b">
+      <c r="N429" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O429" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P429" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="430">
-      <c r="A430" t="inlineStr">
+      <c r="A430" s="10" t="inlineStr">
         <is>
           <t>John Wick: Chapter 4</t>
         </is>
       </c>
-      <c r="B430" t="inlineStr">
+      <c r="B430" s="10" t="inlineStr">
         <is>
           <t>card_429</t>
         </is>
       </c>
-      <c r="C430" t="inlineStr">
+      <c r="C430" s="10" t="inlineStr">
         <is>
           <t>Chad Stahelski</t>
         </is>
       </c>
-      <c r="D430" t="n">
+      <c r="D430" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E430" t="n">
+      <c r="E430" s="10" t="n">
         <v>3.9</v>
       </c>
-      <c r="F430" t="n">
+      <c r="F430" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I430" t="n">
+      <c r="I430" s="10" t="n">
         <v>447300000</v>
       </c>
-      <c r="J430" t="b">
-        <v>0</v>
-      </c>
-      <c r="K430" t="n">
+      <c r="J430" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K430" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L430" t="b">
-        <v>0</v>
-      </c>
-      <c r="M430" t="n">
+      <c r="L430" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M430" s="10" t="n">
         <v>169</v>
       </c>
-      <c r="N430" t="n">
-        <v>0</v>
-      </c>
-      <c r="O430" t="n">
-        <v>0</v>
-      </c>
-      <c r="P430" t="b">
+      <c r="N430" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O430" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P430" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="431">
-      <c r="A431" t="inlineStr">
+      <c r="A431" s="10" t="inlineStr">
         <is>
           <t>Lethal Weapon</t>
         </is>
       </c>
-      <c r="B431" t="inlineStr">
+      <c r="B431" s="10" t="inlineStr">
         <is>
           <t>card_430</t>
         </is>
       </c>
-      <c r="C431" t="inlineStr">
+      <c r="C431" s="10" t="inlineStr">
         <is>
           <t>Richard Donner</t>
         </is>
       </c>
-      <c r="D431" t="n">
+      <c r="D431" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E431" t="n">
+      <c r="E431" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F431" t="n">
+      <c r="F431" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I431" t="n">
+      <c r="I431" s="10" t="n">
         <v>120100000</v>
       </c>
-      <c r="J431" t="b">
-        <v>0</v>
-      </c>
-      <c r="K431" t="n">
+      <c r="J431" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K431" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L431" t="b">
-        <v>0</v>
-      </c>
-      <c r="M431" t="n">
+      <c r="L431" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M431" s="10" t="n">
         <v>109</v>
       </c>
-      <c r="N431" t="n">
-        <v>0</v>
-      </c>
-      <c r="O431" t="n">
-        <v>0</v>
-      </c>
-      <c r="P431" t="b">
+      <c r="N431" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O431" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P431" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="432">
-      <c r="A432" t="inlineStr">
+      <c r="A432" s="10" t="inlineStr">
         <is>
           <t>Lethal Weapon 2</t>
         </is>
       </c>
-      <c r="B432" t="inlineStr">
+      <c r="B432" s="10" t="inlineStr">
         <is>
           <t>card_431</t>
         </is>
       </c>
-      <c r="C432" t="inlineStr">
+      <c r="C432" s="10" t="inlineStr">
         <is>
           <t>Richard Donner</t>
         </is>
       </c>
-      <c r="D432" t="n">
+      <c r="D432" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E432" t="n">
+      <c r="E432" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F432" t="n">
+      <c r="F432" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I432" t="n">
+      <c r="I432" s="10" t="n">
         <v>227300000</v>
       </c>
-      <c r="J432" t="b">
-        <v>0</v>
-      </c>
-      <c r="K432" t="n">
+      <c r="J432" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K432" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L432" t="b">
-        <v>0</v>
-      </c>
-      <c r="M432" t="n">
+      <c r="L432" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M432" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N432" t="n">
-        <v>0</v>
-      </c>
-      <c r="O432" t="n">
-        <v>0</v>
-      </c>
-      <c r="P432" t="b">
+      <c r="N432" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O432" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P432" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="433">
-      <c r="A433" t="inlineStr">
+      <c r="A433" s="10" t="inlineStr">
         <is>
           <t>Lethal Weapon 3</t>
         </is>
       </c>
-      <c r="B433" t="inlineStr">
+      <c r="B433" s="10" t="inlineStr">
         <is>
           <t>card_432</t>
         </is>
       </c>
-      <c r="C433" t="inlineStr">
+      <c r="C433" s="10" t="inlineStr">
         <is>
           <t>Richard Donner</t>
         </is>
       </c>
-      <c r="D433" t="n">
+      <c r="D433" s="10" t="n">
         <v>1992</v>
       </c>
-      <c r="E433" t="n">
+      <c r="E433" s="10" t="n">
         <v>3.26</v>
       </c>
-      <c r="F433" t="n">
+      <c r="F433" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I433" t="n">
+      <c r="I433" s="10" t="n">
         <v>321700000</v>
       </c>
-      <c r="J433" t="b">
-        <v>0</v>
-      </c>
-      <c r="K433" t="n">
+      <c r="J433" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K433" s="10" t="n">
         <v>35000000</v>
       </c>
-      <c r="L433" t="b">
-        <v>0</v>
-      </c>
-      <c r="M433" t="n">
+      <c r="L433" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M433" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N433" t="n">
-        <v>0</v>
-      </c>
-      <c r="O433" t="n">
-        <v>0</v>
-      </c>
-      <c r="P433" t="b">
+      <c r="N433" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O433" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P433" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="434">
-      <c r="A434" t="inlineStr">
+      <c r="A434" s="10" t="inlineStr">
         <is>
           <t>Lethal Weapon 4</t>
         </is>
       </c>
-      <c r="B434" t="inlineStr">
+      <c r="B434" s="10" t="inlineStr">
         <is>
           <t>card_433</t>
         </is>
       </c>
-      <c r="C434" t="inlineStr">
+      <c r="C434" s="10" t="inlineStr">
         <is>
           <t>Richard Donner</t>
         </is>
       </c>
-      <c r="D434" t="n">
+      <c r="D434" s="10" t="n">
         <v>1998</v>
       </c>
-      <c r="E434" t="n">
+      <c r="E434" s="10" t="n">
         <v>3.16</v>
       </c>
-      <c r="F434" t="n">
+      <c r="F434" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I434" t="n">
+      <c r="I434" s="10" t="n">
         <v>285400000</v>
       </c>
-      <c r="J434" t="b">
-        <v>0</v>
-      </c>
-      <c r="K434" t="n">
+      <c r="J434" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K434" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L434" t="b">
+      <c r="L434" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M434" t="n">
+      <c r="M434" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="N434" t="n">
-        <v>0</v>
-      </c>
-      <c r="O434" t="n">
-        <v>0</v>
-      </c>
-      <c r="P434" t="b">
+      <c r="N434" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O434" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P434" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="435">
-      <c r="A435" t="inlineStr">
+      <c r="A435" s="10" t="inlineStr">
         <is>
           <t>The Bourne Identity</t>
         </is>
       </c>
-      <c r="B435" t="inlineStr">
+      <c r="B435" s="10" t="inlineStr">
         <is>
           <t>card_434</t>
         </is>
       </c>
-      <c r="C435" t="inlineStr">
+      <c r="C435" s="10" t="inlineStr">
         <is>
           <t>Doug Liman</t>
         </is>
       </c>
-      <c r="D435" t="n">
+      <c r="D435" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E435" t="n">
+      <c r="E435" s="10" t="n">
         <v>3.27</v>
       </c>
-      <c r="F435" t="n">
+      <c r="F435" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I435" t="n">
+      <c r="I435" s="10" t="n">
         <v>214000000</v>
       </c>
-      <c r="J435" t="b">
-        <v>0</v>
-      </c>
-      <c r="K435" t="n">
+      <c r="J435" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K435" s="10" t="n">
         <v>60000000</v>
       </c>
-      <c r="L435" t="b">
-        <v>0</v>
-      </c>
-      <c r="M435" t="n">
+      <c r="L435" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M435" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="N435" t="n">
-        <v>0</v>
-      </c>
-      <c r="O435" t="n">
-        <v>0</v>
-      </c>
-      <c r="P435" t="b">
+      <c r="N435" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O435" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P435" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="436">
-      <c r="A436" t="inlineStr">
+      <c r="A436" s="10" t="inlineStr">
         <is>
           <t>The Bourne Supremacy</t>
         </is>
       </c>
-      <c r="B436" t="inlineStr">
+      <c r="B436" s="10" t="inlineStr">
         <is>
           <t>card_435</t>
         </is>
       </c>
-      <c r="C436" t="inlineStr">
+      <c r="C436" s="10" t="inlineStr">
         <is>
           <t>Paul Greengrass</t>
         </is>
       </c>
-      <c r="D436" t="n">
+      <c r="D436" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E436" t="n">
+      <c r="E436" s="10" t="n">
         <v>3.63</v>
       </c>
-      <c r="F436" t="n">
+      <c r="F436" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I436" t="n">
+      <c r="I436" s="10" t="n">
         <v>311000000</v>
       </c>
-      <c r="J436" t="b">
-        <v>0</v>
-      </c>
-      <c r="K436" t="n">
+      <c r="J436" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K436" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L436" t="b">
-        <v>0</v>
-      </c>
-      <c r="M436" t="n">
+      <c r="L436" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M436" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="N436" t="n">
-        <v>0</v>
-      </c>
-      <c r="O436" t="n">
-        <v>0</v>
-      </c>
-      <c r="P436" t="b">
+      <c r="N436" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O436" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P436" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="437">
-      <c r="A437" t="inlineStr">
+      <c r="A437" s="10" t="inlineStr">
         <is>
           <t>The Bourne Ultimatum</t>
         </is>
       </c>
-      <c r="B437" t="inlineStr">
+      <c r="B437" s="10" t="inlineStr">
         <is>
           <t>card_436</t>
         </is>
       </c>
-      <c r="C437" t="inlineStr">
+      <c r="C437" s="10" t="inlineStr">
         <is>
           <t>Paul Greengrass</t>
         </is>
       </c>
-      <c r="D437" t="n">
+      <c r="D437" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E437" t="n">
+      <c r="E437" s="10" t="n">
         <v>3.74</v>
       </c>
-      <c r="F437" t="n">
+      <c r="F437" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I437" t="n">
+      <c r="I437" s="10" t="n">
         <v>444000000</v>
       </c>
-      <c r="J437" t="b">
-        <v>0</v>
-      </c>
-      <c r="K437" t="n">
+      <c r="J437" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K437" s="10" t="n">
         <v>120000000</v>
       </c>
-      <c r="L437" t="b">
-        <v>0</v>
-      </c>
-      <c r="M437" t="n">
+      <c r="L437" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M437" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N437" t="n">
+      <c r="N437" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="O437" t="n">
-        <v>0</v>
-      </c>
-      <c r="P437" t="b">
+      <c r="O437" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P437" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="438">
-      <c r="A438" t="inlineStr">
+      <c r="A438" s="10" t="inlineStr">
         <is>
           <t>The Bourne Legacy</t>
         </is>
       </c>
-      <c r="B438" t="inlineStr">
+      <c r="B438" s="10" t="inlineStr">
         <is>
           <t>card_437</t>
         </is>
       </c>
-      <c r="C438" t="inlineStr">
+      <c r="C438" s="10" t="inlineStr">
         <is>
           <t>Tony Gilroy</t>
         </is>
       </c>
-      <c r="D438" t="n">
+      <c r="D438" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E438" t="n">
+      <c r="E438" s="10" t="n">
         <v>2.85</v>
       </c>
-      <c r="F438" t="n">
+      <c r="F438" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I438" t="n">
+      <c r="I438" s="10" t="n">
         <v>276100000</v>
       </c>
-      <c r="J438" t="b">
-        <v>0</v>
-      </c>
-      <c r="K438" t="n">
+      <c r="J438" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K438" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L438" t="b">
-        <v>0</v>
-      </c>
-      <c r="M438" t="n">
+      <c r="L438" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M438" s="10" t="n">
         <v>135</v>
       </c>
-      <c r="N438" t="n">
-        <v>0</v>
-      </c>
-      <c r="O438" t="n">
-        <v>0</v>
-      </c>
-      <c r="P438" t="b">
+      <c r="N438" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O438" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P438" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="439">
-      <c r="A439" t="inlineStr">
+      <c r="A439" s="10" t="inlineStr">
         <is>
           <t>Jason Bourne</t>
         </is>
       </c>
-      <c r="B439" t="inlineStr">
+      <c r="B439" s="10" t="inlineStr">
         <is>
           <t>card_438</t>
         </is>
       </c>
-      <c r="C439" t="inlineStr">
+      <c r="C439" s="10" t="inlineStr">
         <is>
           <t>Paul Greengrass</t>
         </is>
       </c>
-      <c r="D439" t="n">
+      <c r="D439" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E439" t="n">
+      <c r="E439" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F439" t="n">
+      <c r="F439" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="I439" t="n">
+      <c r="I439" s="10" t="n">
         <v>416200000</v>
       </c>
-      <c r="J439" t="b">
-        <v>0</v>
-      </c>
-      <c r="K439" t="n">
+      <c r="J439" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K439" s="10" t="n">
         <v>120000000</v>
       </c>
-      <c r="L439" t="b">
-        <v>0</v>
-      </c>
-      <c r="M439" t="n">
+      <c r="L439" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M439" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="N439" t="n">
-        <v>0</v>
-      </c>
-      <c r="O439" t="n">
-        <v>0</v>
-      </c>
-      <c r="P439" t="b">
+      <c r="N439" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O439" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P439" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Pirates of the Caribbean: The Curse of the Black Pearl</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>card_439</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Gore Verbinski</t>
+        </is>
+      </c>
+      <c r="D440" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E440" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F440" t="n">
+        <v>84</v>
+      </c>
+      <c r="I440" t="n">
+        <v>654300000</v>
+      </c>
+      <c r="J440" t="b">
+        <v>0</v>
+      </c>
+      <c r="K440" t="n">
+        <v>140000000</v>
+      </c>
+      <c r="L440" t="b">
+        <v>0</v>
+      </c>
+      <c r="M440" t="n">
+        <v>143</v>
+      </c>
+      <c r="N440" t="n">
+        <v>0</v>
+      </c>
+      <c r="O440" t="n">
+        <v>0</v>
+      </c>
+      <c r="P440" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Pirates of the Caribbean: Dead Man's Chest</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>card_440</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Gore Verbinski</t>
+        </is>
+      </c>
+      <c r="D441" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E441" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="F441" t="n">
+        <v>77</v>
+      </c>
+      <c r="I441" t="n">
+        <v>1066000000</v>
+      </c>
+      <c r="J441" t="b">
+        <v>0</v>
+      </c>
+      <c r="K441" t="n">
+        <v>225000000</v>
+      </c>
+      <c r="L441" t="b">
+        <v>0</v>
+      </c>
+      <c r="M441" t="n">
+        <v>150</v>
+      </c>
+      <c r="N441" t="n">
+        <v>1</v>
+      </c>
+      <c r="O441" t="n">
+        <v>0</v>
+      </c>
+      <c r="P441" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Pirates of the Caribbean: At World's End</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>card_441</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Gore Verbinski</t>
+        </is>
+      </c>
+      <c r="D442" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E442" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F442" t="n">
+        <v>73</v>
+      </c>
+      <c r="I442" t="n">
+        <v>963400000</v>
+      </c>
+      <c r="J442" t="b">
+        <v>0</v>
+      </c>
+      <c r="K442" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="L442" t="b">
+        <v>0</v>
+      </c>
+      <c r="M442" t="n">
+        <v>168</v>
+      </c>
+      <c r="N442" t="n">
+        <v>0</v>
+      </c>
+      <c r="O442" t="n">
+        <v>0</v>
+      </c>
+      <c r="P442" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Pirates of the Caribbean: On Stranger Tides</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>card_442</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Rob Marshall</t>
+        </is>
+      </c>
+      <c r="D443" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E443" t="n">
+        <v>3</v>
+      </c>
+      <c r="F443" t="n">
+        <v>63</v>
+      </c>
+      <c r="I443" t="n">
+        <v>1046000000</v>
+      </c>
+      <c r="J443" t="b">
+        <v>0</v>
+      </c>
+      <c r="K443" t="n">
+        <v>378500000</v>
+      </c>
+      <c r="L443" t="b">
+        <v>0</v>
+      </c>
+      <c r="M443" t="n">
+        <v>136</v>
+      </c>
+      <c r="N443" t="n">
+        <v>0</v>
+      </c>
+      <c r="O443" t="n">
+        <v>0</v>
+      </c>
+      <c r="P443" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Pirates of the Caribbean: Dead Men Tell No Tales</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>card_443</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Joachim Ronning and Espen Sandberg</t>
+        </is>
+      </c>
+      <c r="D444" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E444" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="F444" t="n">
+        <v>62</v>
+      </c>
+      <c r="I444" t="n">
+        <v>795900000</v>
+      </c>
+      <c r="J444" t="b">
+        <v>0</v>
+      </c>
+      <c r="K444" t="n">
+        <v>230000000</v>
+      </c>
+      <c r="L444" t="b">
+        <v>0</v>
+      </c>
+      <c r="M444" t="n">
+        <v>129</v>
+      </c>
+      <c r="N444" t="n">
+        <v>0</v>
+      </c>
+      <c r="O444" t="n">
+        <v>0</v>
+      </c>
+      <c r="P444" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Mission: Impossible series (card_444-451)
All 8 films, 1996 through The Final Reckoning (2025).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P444"/>
+  <dimension ref="A1:P452"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -23619,252 +23619,652 @@
       </c>
     </row>
     <row r="440">
-      <c r="A440" t="inlineStr">
+      <c r="A440" s="10" t="inlineStr">
         <is>
           <t>Pirates of the Caribbean: The Curse of the Black Pearl</t>
         </is>
       </c>
-      <c r="B440" t="inlineStr">
+      <c r="B440" s="10" t="inlineStr">
         <is>
           <t>card_439</t>
         </is>
       </c>
-      <c r="C440" t="inlineStr">
+      <c r="C440" s="10" t="inlineStr">
         <is>
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="D440" t="n">
+      <c r="D440" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E440" t="n">
+      <c r="E440" s="10" t="n">
         <v>4.02</v>
       </c>
-      <c r="F440" t="n">
+      <c r="F440" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="I440" t="n">
+      <c r="I440" s="10" t="n">
         <v>654300000</v>
       </c>
-      <c r="J440" t="b">
-        <v>0</v>
-      </c>
-      <c r="K440" t="n">
+      <c r="J440" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K440" s="10" t="n">
         <v>140000000</v>
       </c>
-      <c r="L440" t="b">
-        <v>0</v>
-      </c>
-      <c r="M440" t="n">
+      <c r="L440" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M440" s="10" t="n">
         <v>143</v>
       </c>
-      <c r="N440" t="n">
-        <v>0</v>
-      </c>
-      <c r="O440" t="n">
-        <v>0</v>
-      </c>
-      <c r="P440" t="b">
+      <c r="N440" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O440" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P440" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="441">
-      <c r="A441" t="inlineStr">
+      <c r="A441" s="10" t="inlineStr">
         <is>
           <t>Pirates of the Caribbean: Dead Man's Chest</t>
         </is>
       </c>
-      <c r="B441" t="inlineStr">
+      <c r="B441" s="10" t="inlineStr">
         <is>
           <t>card_440</t>
         </is>
       </c>
-      <c r="C441" t="inlineStr">
+      <c r="C441" s="10" t="inlineStr">
         <is>
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="D441" t="n">
+      <c r="D441" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E441" t="n">
+      <c r="E441" s="10" t="n">
         <v>3.79</v>
       </c>
-      <c r="F441" t="n">
+      <c r="F441" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I441" t="n">
+      <c r="I441" s="10" t="n">
         <v>1066000000</v>
       </c>
-      <c r="J441" t="b">
-        <v>0</v>
-      </c>
-      <c r="K441" t="n">
+      <c r="J441" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K441" s="10" t="n">
         <v>225000000</v>
       </c>
-      <c r="L441" t="b">
-        <v>0</v>
-      </c>
-      <c r="M441" t="n">
+      <c r="L441" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M441" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="N441" t="n">
+      <c r="N441" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O441" t="n">
-        <v>0</v>
-      </c>
-      <c r="P441" t="b">
+      <c r="O441" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P441" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="442">
-      <c r="A442" t="inlineStr">
+      <c r="A442" s="10" t="inlineStr">
         <is>
           <t>Pirates of the Caribbean: At World's End</t>
         </is>
       </c>
-      <c r="B442" t="inlineStr">
+      <c r="B442" s="10" t="inlineStr">
         <is>
           <t>card_441</t>
         </is>
       </c>
-      <c r="C442" t="inlineStr">
+      <c r="C442" s="10" t="inlineStr">
         <is>
           <t>Gore Verbinski</t>
         </is>
       </c>
-      <c r="D442" t="n">
+      <c r="D442" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E442" t="n">
+      <c r="E442" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F442" t="n">
+      <c r="F442" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I442" t="n">
+      <c r="I442" s="10" t="n">
         <v>963400000</v>
       </c>
-      <c r="J442" t="b">
-        <v>0</v>
-      </c>
-      <c r="K442" t="n">
+      <c r="J442" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K442" s="10" t="n">
         <v>300000000</v>
       </c>
-      <c r="L442" t="b">
-        <v>0</v>
-      </c>
-      <c r="M442" t="n">
+      <c r="L442" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M442" s="10" t="n">
         <v>168</v>
       </c>
-      <c r="N442" t="n">
-        <v>0</v>
-      </c>
-      <c r="O442" t="n">
-        <v>0</v>
-      </c>
-      <c r="P442" t="b">
+      <c r="N442" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O442" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P442" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="443">
-      <c r="A443" t="inlineStr">
+      <c r="A443" s="10" t="inlineStr">
         <is>
           <t>Pirates of the Caribbean: On Stranger Tides</t>
         </is>
       </c>
-      <c r="B443" t="inlineStr">
+      <c r="B443" s="10" t="inlineStr">
         <is>
           <t>card_442</t>
         </is>
       </c>
-      <c r="C443" t="inlineStr">
+      <c r="C443" s="10" t="inlineStr">
         <is>
           <t>Rob Marshall</t>
         </is>
       </c>
-      <c r="D443" t="n">
+      <c r="D443" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E443" t="n">
+      <c r="E443" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F443" t="n">
+      <c r="F443" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I443" t="n">
+      <c r="I443" s="10" t="n">
         <v>1046000000</v>
       </c>
-      <c r="J443" t="b">
-        <v>0</v>
-      </c>
-      <c r="K443" t="n">
+      <c r="J443" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K443" s="10" t="n">
         <v>378500000</v>
       </c>
-      <c r="L443" t="b">
-        <v>0</v>
-      </c>
-      <c r="M443" t="n">
+      <c r="L443" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M443" s="10" t="n">
         <v>136</v>
       </c>
-      <c r="N443" t="n">
-        <v>0</v>
-      </c>
-      <c r="O443" t="n">
-        <v>0</v>
-      </c>
-      <c r="P443" t="b">
+      <c r="N443" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O443" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P443" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="444">
-      <c r="A444" t="inlineStr">
+      <c r="A444" s="10" t="inlineStr">
         <is>
           <t>Pirates of the Caribbean: Dead Men Tell No Tales</t>
         </is>
       </c>
-      <c r="B444" t="inlineStr">
+      <c r="B444" s="10" t="inlineStr">
         <is>
           <t>card_443</t>
         </is>
       </c>
-      <c r="C444" t="inlineStr">
+      <c r="C444" s="10" t="inlineStr">
         <is>
           <t>Joachim Ronning and Espen Sandberg</t>
         </is>
       </c>
-      <c r="D444" t="n">
+      <c r="D444" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E444" t="n">
+      <c r="E444" s="10" t="n">
         <v>2.81</v>
       </c>
-      <c r="F444" t="n">
+      <c r="F444" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I444" t="n">
+      <c r="I444" s="10" t="n">
         <v>795900000</v>
       </c>
-      <c r="J444" t="b">
-        <v>0</v>
-      </c>
-      <c r="K444" t="n">
+      <c r="J444" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K444" s="10" t="n">
         <v>230000000</v>
       </c>
-      <c r="L444" t="b">
-        <v>0</v>
-      </c>
-      <c r="M444" t="n">
+      <c r="L444" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M444" s="10" t="n">
         <v>129</v>
       </c>
-      <c r="N444" t="n">
-        <v>0</v>
-      </c>
-      <c r="O444" t="n">
-        <v>0</v>
-      </c>
-      <c r="P444" t="b">
+      <c r="N444" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O444" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P444" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Mission: Impossible</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>card_444</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Brian De Palma</t>
+        </is>
+      </c>
+      <c r="D445" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E445" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F445" t="n">
+        <v>73</v>
+      </c>
+      <c r="I445" t="n">
+        <v>457700000</v>
+      </c>
+      <c r="J445" t="b">
+        <v>0</v>
+      </c>
+      <c r="K445" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L445" t="b">
+        <v>0</v>
+      </c>
+      <c r="M445" t="n">
+        <v>110</v>
+      </c>
+      <c r="N445" t="n">
+        <v>0</v>
+      </c>
+      <c r="O445" t="n">
+        <v>0</v>
+      </c>
+      <c r="P445" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Mission: Impossible 2</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>card_445</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>John Woo</t>
+        </is>
+      </c>
+      <c r="D446" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E446" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F446" t="n">
+        <v>58</v>
+      </c>
+      <c r="I446" t="n">
+        <v>546400000</v>
+      </c>
+      <c r="J446" t="b">
+        <v>0</v>
+      </c>
+      <c r="K446" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L446" t="b">
+        <v>0</v>
+      </c>
+      <c r="M446" t="n">
+        <v>124</v>
+      </c>
+      <c r="N446" t="n">
+        <v>0</v>
+      </c>
+      <c r="O446" t="n">
+        <v>0</v>
+      </c>
+      <c r="P446" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Mission: Impossible III</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>card_446</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>J.J. Abrams</t>
+        </is>
+      </c>
+      <c r="D447" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E447" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="F447" t="n">
+        <v>72</v>
+      </c>
+      <c r="I447" t="n">
+        <v>398500000</v>
+      </c>
+      <c r="J447" t="b">
+        <v>0</v>
+      </c>
+      <c r="K447" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L447" t="b">
+        <v>0</v>
+      </c>
+      <c r="M447" t="n">
+        <v>126</v>
+      </c>
+      <c r="N447" t="n">
+        <v>0</v>
+      </c>
+      <c r="O447" t="n">
+        <v>0</v>
+      </c>
+      <c r="P447" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Mission: Impossible - Ghost Protocol</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>card_447</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Brad Bird</t>
+        </is>
+      </c>
+      <c r="D448" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E448" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="F448" t="n">
+        <v>79</v>
+      </c>
+      <c r="I448" t="n">
+        <v>694700000</v>
+      </c>
+      <c r="J448" t="b">
+        <v>0</v>
+      </c>
+      <c r="K448" t="n">
+        <v>145000000</v>
+      </c>
+      <c r="L448" t="b">
+        <v>0</v>
+      </c>
+      <c r="M448" t="n">
+        <v>133</v>
+      </c>
+      <c r="N448" t="n">
+        <v>0</v>
+      </c>
+      <c r="O448" t="n">
+        <v>0</v>
+      </c>
+      <c r="P448" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Mission: Impossible - Rogue Nation</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>card_448</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Christopher McQuarrie</t>
+        </is>
+      </c>
+      <c r="D449" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E449" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F449" t="n">
+        <v>78</v>
+      </c>
+      <c r="I449" t="n">
+        <v>710900000</v>
+      </c>
+      <c r="J449" t="b">
+        <v>0</v>
+      </c>
+      <c r="K449" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L449" t="b">
+        <v>0</v>
+      </c>
+      <c r="M449" t="n">
+        <v>131</v>
+      </c>
+      <c r="N449" t="n">
+        <v>0</v>
+      </c>
+      <c r="O449" t="n">
+        <v>0</v>
+      </c>
+      <c r="P449" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Mission: Impossible - Fallout</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>card_449</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Christopher McQuarrie</t>
+        </is>
+      </c>
+      <c r="D450" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E450" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F450" t="n">
+        <v>83</v>
+      </c>
+      <c r="I450" t="n">
+        <v>791100000</v>
+      </c>
+      <c r="J450" t="b">
+        <v>0</v>
+      </c>
+      <c r="K450" t="n">
+        <v>178000000</v>
+      </c>
+      <c r="L450" t="b">
+        <v>0</v>
+      </c>
+      <c r="M450" t="n">
+        <v>147</v>
+      </c>
+      <c r="N450" t="n">
+        <v>0</v>
+      </c>
+      <c r="O450" t="n">
+        <v>0</v>
+      </c>
+      <c r="P450" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Mission: Impossible - Dead Reckoning Part One</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>card_450</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>Christopher McQuarrie</t>
+        </is>
+      </c>
+      <c r="D451" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E451" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F451" t="n">
+        <v>78</v>
+      </c>
+      <c r="I451" t="n">
+        <v>571100000</v>
+      </c>
+      <c r="J451" t="b">
+        <v>0</v>
+      </c>
+      <c r="K451" t="n">
+        <v>291000000</v>
+      </c>
+      <c r="L451" t="b">
+        <v>0</v>
+      </c>
+      <c r="M451" t="n">
+        <v>163</v>
+      </c>
+      <c r="N451" t="n">
+        <v>0</v>
+      </c>
+      <c r="O451" t="n">
+        <v>0</v>
+      </c>
+      <c r="P451" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Mission: Impossible - The Final Reckoning</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>card_451</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Christopher McQuarrie</t>
+        </is>
+      </c>
+      <c r="D452" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E452" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="F452" t="n">
+        <v>68</v>
+      </c>
+      <c r="I452" t="n">
+        <v>598800000</v>
+      </c>
+      <c r="J452" t="b">
+        <v>0</v>
+      </c>
+      <c r="K452" t="n">
+        <v>350000000</v>
+      </c>
+      <c r="L452" t="b">
+        <v>0</v>
+      </c>
+      <c r="M452" t="n">
+        <v>170</v>
+      </c>
+      <c r="N452" t="n">
+        <v>0</v>
+      </c>
+      <c r="O452" t="n">
+        <v>0</v>
+      </c>
+      <c r="P452" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Hunger Games series (card_452-456)
The Hunger Games, Catching Fire, Mockingjay Part 1 & 2, The Ballad of
Songbirds and Snakes. Sunrise on the Reaping (Nov 2026) isn't released
yet, so it's not included.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P452"/>
+  <dimension ref="A1:P457"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -23869,402 +23869,652 @@
       </c>
     </row>
     <row r="445">
-      <c r="A445" t="inlineStr">
+      <c r="A445" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible</t>
         </is>
       </c>
-      <c r="B445" t="inlineStr">
+      <c r="B445" s="10" t="inlineStr">
         <is>
           <t>card_444</t>
         </is>
       </c>
-      <c r="C445" t="inlineStr">
+      <c r="C445" s="10" t="inlineStr">
         <is>
           <t>Brian De Palma</t>
         </is>
       </c>
-      <c r="D445" t="n">
+      <c r="D445" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E445" t="n">
+      <c r="E445" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F445" t="n">
+      <c r="F445" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I445" t="n">
+      <c r="I445" s="10" t="n">
         <v>457700000</v>
       </c>
-      <c r="J445" t="b">
-        <v>0</v>
-      </c>
-      <c r="K445" t="n">
+      <c r="J445" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K445" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L445" t="b">
-        <v>0</v>
-      </c>
-      <c r="M445" t="n">
+      <c r="L445" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M445" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N445" t="n">
-        <v>0</v>
-      </c>
-      <c r="O445" t="n">
-        <v>0</v>
-      </c>
-      <c r="P445" t="b">
+      <c r="N445" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O445" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P445" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="446">
-      <c r="A446" t="inlineStr">
+      <c r="A446" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible 2</t>
         </is>
       </c>
-      <c r="B446" t="inlineStr">
+      <c r="B446" s="10" t="inlineStr">
         <is>
           <t>card_445</t>
         </is>
       </c>
-      <c r="C446" t="inlineStr">
+      <c r="C446" s="10" t="inlineStr">
         <is>
           <t>John Woo</t>
         </is>
       </c>
-      <c r="D446" t="n">
+      <c r="D446" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E446" t="n">
+      <c r="E446" s="10" t="n">
         <v>2.7</v>
       </c>
-      <c r="F446" t="n">
+      <c r="F446" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="I446" t="n">
+      <c r="I446" s="10" t="n">
         <v>546400000</v>
       </c>
-      <c r="J446" t="b">
-        <v>0</v>
-      </c>
-      <c r="K446" t="n">
+      <c r="J446" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K446" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L446" t="b">
-        <v>0</v>
-      </c>
-      <c r="M446" t="n">
+      <c r="L446" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M446" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="N446" t="n">
-        <v>0</v>
-      </c>
-      <c r="O446" t="n">
-        <v>0</v>
-      </c>
-      <c r="P446" t="b">
+      <c r="N446" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O446" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P446" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="447">
-      <c r="A447" t="inlineStr">
+      <c r="A447" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible III</t>
         </is>
       </c>
-      <c r="B447" t="inlineStr">
+      <c r="B447" s="10" t="inlineStr">
         <is>
           <t>card_446</t>
         </is>
       </c>
-      <c r="C447" t="inlineStr">
+      <c r="C447" s="10" t="inlineStr">
         <is>
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="D447" t="n">
+      <c r="D447" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E447" t="n">
+      <c r="E447" s="10" t="n">
         <v>3.42</v>
       </c>
-      <c r="F447" t="n">
+      <c r="F447" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I447" t="n">
+      <c r="I447" s="10" t="n">
         <v>398500000</v>
       </c>
-      <c r="J447" t="b">
-        <v>0</v>
-      </c>
-      <c r="K447" t="n">
+      <c r="J447" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K447" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L447" t="b">
-        <v>0</v>
-      </c>
-      <c r="M447" t="n">
+      <c r="L447" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M447" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="N447" t="n">
-        <v>0</v>
-      </c>
-      <c r="O447" t="n">
-        <v>0</v>
-      </c>
-      <c r="P447" t="b">
+      <c r="N447" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O447" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P447" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="448">
-      <c r="A448" t="inlineStr">
+      <c r="A448" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible - Ghost Protocol</t>
         </is>
       </c>
-      <c r="B448" t="inlineStr">
+      <c r="B448" s="10" t="inlineStr">
         <is>
           <t>card_447</t>
         </is>
       </c>
-      <c r="C448" t="inlineStr">
+      <c r="C448" s="10" t="inlineStr">
         <is>
           <t>Brad Bird</t>
         </is>
       </c>
-      <c r="D448" t="n">
+      <c r="D448" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E448" t="n">
+      <c r="E448" s="10" t="n">
         <v>3.76</v>
       </c>
-      <c r="F448" t="n">
+      <c r="F448" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I448" t="n">
+      <c r="I448" s="10" t="n">
         <v>694700000</v>
       </c>
-      <c r="J448" t="b">
-        <v>0</v>
-      </c>
-      <c r="K448" t="n">
+      <c r="J448" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K448" s="10" t="n">
         <v>145000000</v>
       </c>
-      <c r="L448" t="b">
-        <v>0</v>
-      </c>
-      <c r="M448" t="n">
+      <c r="L448" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M448" s="10" t="n">
         <v>133</v>
       </c>
-      <c r="N448" t="n">
-        <v>0</v>
-      </c>
-      <c r="O448" t="n">
-        <v>0</v>
-      </c>
-      <c r="P448" t="b">
+      <c r="N448" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O448" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P448" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="449">
-      <c r="A449" t="inlineStr">
+      <c r="A449" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible - Rogue Nation</t>
         </is>
       </c>
-      <c r="B449" t="inlineStr">
+      <c r="B449" s="10" t="inlineStr">
         <is>
           <t>card_448</t>
         </is>
       </c>
-      <c r="C449" t="inlineStr">
+      <c r="C449" s="10" t="inlineStr">
         <is>
           <t>Christopher McQuarrie</t>
         </is>
       </c>
-      <c r="D449" t="n">
+      <c r="D449" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E449" t="n">
+      <c r="E449" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F449" t="n">
+      <c r="F449" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I449" t="n">
+      <c r="I449" s="10" t="n">
         <v>710900000</v>
       </c>
-      <c r="J449" t="b">
-        <v>0</v>
-      </c>
-      <c r="K449" t="n">
+      <c r="J449" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K449" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L449" t="b">
-        <v>0</v>
-      </c>
-      <c r="M449" t="n">
+      <c r="L449" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M449" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N449" t="n">
-        <v>0</v>
-      </c>
-      <c r="O449" t="n">
-        <v>0</v>
-      </c>
-      <c r="P449" t="b">
+      <c r="N449" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O449" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P449" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="450">
-      <c r="A450" t="inlineStr">
+      <c r="A450" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible - Fallout</t>
         </is>
       </c>
-      <c r="B450" t="inlineStr">
+      <c r="B450" s="10" t="inlineStr">
         <is>
           <t>card_449</t>
         </is>
       </c>
-      <c r="C450" t="inlineStr">
+      <c r="C450" s="10" t="inlineStr">
         <is>
           <t>Christopher McQuarrie</t>
         </is>
       </c>
-      <c r="D450" t="n">
+      <c r="D450" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E450" t="n">
+      <c r="E450" s="10" t="n">
         <v>4.01</v>
       </c>
-      <c r="F450" t="n">
+      <c r="F450" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I450" t="n">
+      <c r="I450" s="10" t="n">
         <v>791100000</v>
       </c>
-      <c r="J450" t="b">
-        <v>0</v>
-      </c>
-      <c r="K450" t="n">
+      <c r="J450" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K450" s="10" t="n">
         <v>178000000</v>
       </c>
-      <c r="L450" t="b">
-        <v>0</v>
-      </c>
-      <c r="M450" t="n">
+      <c r="L450" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M450" s="10" t="n">
         <v>147</v>
       </c>
-      <c r="N450" t="n">
-        <v>0</v>
-      </c>
-      <c r="O450" t="n">
-        <v>0</v>
-      </c>
-      <c r="P450" t="b">
+      <c r="N450" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O450" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P450" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="451">
-      <c r="A451" t="inlineStr">
+      <c r="A451" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible - Dead Reckoning Part One</t>
         </is>
       </c>
-      <c r="B451" t="inlineStr">
+      <c r="B451" s="10" t="inlineStr">
         <is>
           <t>card_450</t>
         </is>
       </c>
-      <c r="C451" t="inlineStr">
+      <c r="C451" s="10" t="inlineStr">
         <is>
           <t>Christopher McQuarrie</t>
         </is>
       </c>
-      <c r="D451" t="n">
+      <c r="D451" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E451" t="n">
+      <c r="E451" s="10" t="n">
         <v>3.7</v>
       </c>
-      <c r="F451" t="n">
+      <c r="F451" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I451" t="n">
+      <c r="I451" s="10" t="n">
         <v>571100000</v>
       </c>
-      <c r="J451" t="b">
-        <v>0</v>
-      </c>
-      <c r="K451" t="n">
+      <c r="J451" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K451" s="10" t="n">
         <v>291000000</v>
       </c>
-      <c r="L451" t="b">
-        <v>0</v>
-      </c>
-      <c r="M451" t="n">
+      <c r="L451" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M451" s="10" t="n">
         <v>163</v>
       </c>
-      <c r="N451" t="n">
-        <v>0</v>
-      </c>
-      <c r="O451" t="n">
-        <v>0</v>
-      </c>
-      <c r="P451" t="b">
+      <c r="N451" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O451" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P451" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="452">
-      <c r="A452" t="inlineStr">
+      <c r="A452" s="10" t="inlineStr">
         <is>
           <t>Mission: Impossible - The Final Reckoning</t>
         </is>
       </c>
-      <c r="B452" t="inlineStr">
+      <c r="B452" s="10" t="inlineStr">
         <is>
           <t>card_451</t>
         </is>
       </c>
-      <c r="C452" t="inlineStr">
+      <c r="C452" s="10" t="inlineStr">
         <is>
           <t>Christopher McQuarrie</t>
         </is>
       </c>
-      <c r="D452" t="n">
+      <c r="D452" s="10" t="n">
         <v>2025</v>
       </c>
-      <c r="E452" t="n">
+      <c r="E452" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="F452" t="n">
+      <c r="F452" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I452" t="n">
+      <c r="I452" s="10" t="n">
         <v>598800000</v>
       </c>
-      <c r="J452" t="b">
-        <v>0</v>
-      </c>
-      <c r="K452" t="n">
+      <c r="J452" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K452" s="10" t="n">
         <v>350000000</v>
       </c>
-      <c r="L452" t="b">
-        <v>0</v>
-      </c>
-      <c r="M452" t="n">
+      <c r="L452" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M452" s="10" t="n">
         <v>170</v>
       </c>
-      <c r="N452" t="n">
-        <v>0</v>
-      </c>
-      <c r="O452" t="n">
-        <v>0</v>
-      </c>
-      <c r="P452" t="b">
+      <c r="N452" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O452" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P452" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>The Hunger Games</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>card_452</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Gary Ross</t>
+        </is>
+      </c>
+      <c r="D453" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E453" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F453" t="n">
+        <v>71</v>
+      </c>
+      <c r="I453" t="n">
+        <v>695200000</v>
+      </c>
+      <c r="J453" t="b">
+        <v>0</v>
+      </c>
+      <c r="K453" t="n">
+        <v>78000000</v>
+      </c>
+      <c r="L453" t="b">
+        <v>0</v>
+      </c>
+      <c r="M453" t="n">
+        <v>142</v>
+      </c>
+      <c r="N453" t="n">
+        <v>0</v>
+      </c>
+      <c r="O453" t="n">
+        <v>0</v>
+      </c>
+      <c r="P453" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>The Hunger Games: Catching Fire</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>card_453</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Francis Lawrence</t>
+        </is>
+      </c>
+      <c r="D454" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E454" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="F454" t="n">
+        <v>79</v>
+      </c>
+      <c r="I454" t="n">
+        <v>865000000</v>
+      </c>
+      <c r="J454" t="b">
+        <v>0</v>
+      </c>
+      <c r="K454" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="L454" t="b">
+        <v>0</v>
+      </c>
+      <c r="M454" t="n">
+        <v>146</v>
+      </c>
+      <c r="N454" t="n">
+        <v>0</v>
+      </c>
+      <c r="O454" t="n">
+        <v>0</v>
+      </c>
+      <c r="P454" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>The Hunger Games: Mockingjay - Part 1</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>card_454</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Francis Lawrence</t>
+        </is>
+      </c>
+      <c r="D455" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E455" t="n">
+        <v>3.42</v>
+      </c>
+      <c r="F455" t="n">
+        <v>63</v>
+      </c>
+      <c r="I455" t="n">
+        <v>755400000</v>
+      </c>
+      <c r="J455" t="b">
+        <v>0</v>
+      </c>
+      <c r="K455" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L455" t="b">
+        <v>0</v>
+      </c>
+      <c r="M455" t="n">
+        <v>123</v>
+      </c>
+      <c r="N455" t="n">
+        <v>0</v>
+      </c>
+      <c r="O455" t="n">
+        <v>0</v>
+      </c>
+      <c r="P455" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>The Hunger Games: Mockingjay - Part 2</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>card_455</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Francis Lawrence</t>
+        </is>
+      </c>
+      <c r="D456" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E456" t="n">
+        <v>3.52</v>
+      </c>
+      <c r="F456" t="n">
+        <v>66</v>
+      </c>
+      <c r="I456" t="n">
+        <v>661400000</v>
+      </c>
+      <c r="J456" t="b">
+        <v>0</v>
+      </c>
+      <c r="K456" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L456" t="b">
+        <v>0</v>
+      </c>
+      <c r="M456" t="n">
+        <v>137</v>
+      </c>
+      <c r="N456" t="n">
+        <v>0</v>
+      </c>
+      <c r="O456" t="n">
+        <v>0</v>
+      </c>
+      <c r="P456" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>The Hunger Games: The Ballad of Songbirds and Snakes</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>card_456</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Francis Lawrence</t>
+        </is>
+      </c>
+      <c r="D457" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E457" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F457" t="n">
+        <v>57</v>
+      </c>
+      <c r="I457" t="n">
+        <v>361800000</v>
+      </c>
+      <c r="J457" t="b">
+        <v>0</v>
+      </c>
+      <c r="K457" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L457" t="b">
+        <v>0</v>
+      </c>
+      <c r="M457" t="n">
+        <v>157</v>
+      </c>
+      <c r="N457" t="n">
+        <v>0</v>
+      </c>
+      <c r="O457" t="n">
+        <v>0</v>
+      </c>
+      <c r="P457" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Scream series (card_457-462)
Scream 1-4 (Wes Craven), Scream (2022), Scream VI.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P457"/>
+  <dimension ref="A1:P463"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -24269,252 +24269,552 @@
       </c>
     </row>
     <row r="453">
-      <c r="A453" t="inlineStr">
+      <c r="A453" s="10" t="inlineStr">
         <is>
           <t>The Hunger Games</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr">
+      <c r="B453" s="10" t="inlineStr">
         <is>
           <t>card_452</t>
         </is>
       </c>
-      <c r="C453" t="inlineStr">
+      <c r="C453" s="10" t="inlineStr">
         <is>
           <t>Gary Ross</t>
         </is>
       </c>
-      <c r="D453" t="n">
+      <c r="D453" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E453" t="n">
+      <c r="E453" s="10" t="n">
         <v>3.84</v>
       </c>
-      <c r="F453" t="n">
+      <c r="F453" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I453" t="n">
+      <c r="I453" s="10" t="n">
         <v>695200000</v>
       </c>
-      <c r="J453" t="b">
-        <v>0</v>
-      </c>
-      <c r="K453" t="n">
+      <c r="J453" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K453" s="10" t="n">
         <v>78000000</v>
       </c>
-      <c r="L453" t="b">
-        <v>0</v>
-      </c>
-      <c r="M453" t="n">
+      <c r="L453" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M453" s="10" t="n">
         <v>142</v>
       </c>
-      <c r="N453" t="n">
-        <v>0</v>
-      </c>
-      <c r="O453" t="n">
-        <v>0</v>
-      </c>
-      <c r="P453" t="b">
+      <c r="N453" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O453" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P453" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="454">
-      <c r="A454" t="inlineStr">
+      <c r="A454" s="10" t="inlineStr">
         <is>
           <t>The Hunger Games: Catching Fire</t>
         </is>
       </c>
-      <c r="B454" t="inlineStr">
+      <c r="B454" s="10" t="inlineStr">
         <is>
           <t>card_453</t>
         </is>
       </c>
-      <c r="C454" t="inlineStr">
+      <c r="C454" s="10" t="inlineStr">
         <is>
           <t>Francis Lawrence</t>
         </is>
       </c>
-      <c r="D454" t="n">
+      <c r="D454" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E454" t="n">
+      <c r="E454" s="10" t="n">
         <v>3.97</v>
       </c>
-      <c r="F454" t="n">
+      <c r="F454" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I454" t="n">
+      <c r="I454" s="10" t="n">
         <v>865000000</v>
       </c>
-      <c r="J454" t="b">
-        <v>0</v>
-      </c>
-      <c r="K454" t="n">
+      <c r="J454" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K454" s="10" t="n">
         <v>130000000</v>
       </c>
-      <c r="L454" t="b">
-        <v>0</v>
-      </c>
-      <c r="M454" t="n">
+      <c r="L454" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M454" s="10" t="n">
         <v>146</v>
       </c>
-      <c r="N454" t="n">
-        <v>0</v>
-      </c>
-      <c r="O454" t="n">
-        <v>0</v>
-      </c>
-      <c r="P454" t="b">
+      <c r="N454" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O454" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P454" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="455">
-      <c r="A455" t="inlineStr">
+      <c r="A455" s="10" t="inlineStr">
         <is>
           <t>The Hunger Games: Mockingjay - Part 1</t>
         </is>
       </c>
-      <c r="B455" t="inlineStr">
+      <c r="B455" s="10" t="inlineStr">
         <is>
           <t>card_454</t>
         </is>
       </c>
-      <c r="C455" t="inlineStr">
+      <c r="C455" s="10" t="inlineStr">
         <is>
           <t>Francis Lawrence</t>
         </is>
       </c>
-      <c r="D455" t="n">
+      <c r="D455" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E455" t="n">
+      <c r="E455" s="10" t="n">
         <v>3.42</v>
       </c>
-      <c r="F455" t="n">
+      <c r="F455" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I455" t="n">
+      <c r="I455" s="10" t="n">
         <v>755400000</v>
       </c>
-      <c r="J455" t="b">
-        <v>0</v>
-      </c>
-      <c r="K455" t="n">
+      <c r="J455" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K455" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L455" t="b">
-        <v>0</v>
-      </c>
-      <c r="M455" t="n">
+      <c r="L455" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M455" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="N455" t="n">
-        <v>0</v>
-      </c>
-      <c r="O455" t="n">
-        <v>0</v>
-      </c>
-      <c r="P455" t="b">
+      <c r="N455" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O455" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P455" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="456">
-      <c r="A456" t="inlineStr">
+      <c r="A456" s="10" t="inlineStr">
         <is>
           <t>The Hunger Games: Mockingjay - Part 2</t>
         </is>
       </c>
-      <c r="B456" t="inlineStr">
+      <c r="B456" s="10" t="inlineStr">
         <is>
           <t>card_455</t>
         </is>
       </c>
-      <c r="C456" t="inlineStr">
+      <c r="C456" s="10" t="inlineStr">
         <is>
           <t>Francis Lawrence</t>
         </is>
       </c>
-      <c r="D456" t="n">
+      <c r="D456" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E456" t="n">
+      <c r="E456" s="10" t="n">
         <v>3.52</v>
       </c>
-      <c r="F456" t="n">
+      <c r="F456" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I456" t="n">
+      <c r="I456" s="10" t="n">
         <v>661400000</v>
       </c>
-      <c r="J456" t="b">
-        <v>0</v>
-      </c>
-      <c r="K456" t="n">
+      <c r="J456" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K456" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L456" t="b">
-        <v>0</v>
-      </c>
-      <c r="M456" t="n">
+      <c r="L456" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M456" s="10" t="n">
         <v>137</v>
       </c>
-      <c r="N456" t="n">
-        <v>0</v>
-      </c>
-      <c r="O456" t="n">
-        <v>0</v>
-      </c>
-      <c r="P456" t="b">
+      <c r="N456" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O456" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P456" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="457">
-      <c r="A457" t="inlineStr">
+      <c r="A457" s="10" t="inlineStr">
         <is>
           <t>The Hunger Games: The Ballad of Songbirds and Snakes</t>
         </is>
       </c>
-      <c r="B457" t="inlineStr">
+      <c r="B457" s="10" t="inlineStr">
         <is>
           <t>card_456</t>
         </is>
       </c>
-      <c r="C457" t="inlineStr">
+      <c r="C457" s="10" t="inlineStr">
         <is>
           <t>Francis Lawrence</t>
         </is>
       </c>
-      <c r="D457" t="n">
+      <c r="D457" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E457" t="n">
+      <c r="E457" s="10" t="n">
         <v>3.59</v>
       </c>
-      <c r="F457" t="n">
+      <c r="F457" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I457" t="n">
+      <c r="I457" s="10" t="n">
         <v>361800000</v>
       </c>
-      <c r="J457" t="b">
-        <v>0</v>
-      </c>
-      <c r="K457" t="n">
+      <c r="J457" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K457" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L457" t="b">
-        <v>0</v>
-      </c>
-      <c r="M457" t="n">
+      <c r="L457" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M457" s="10" t="n">
         <v>157</v>
       </c>
-      <c r="N457" t="n">
-        <v>0</v>
-      </c>
-      <c r="O457" t="n">
-        <v>0</v>
-      </c>
-      <c r="P457" t="b">
+      <c r="N457" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O457" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P457" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Scream</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>card_457</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>Wes Craven</t>
+        </is>
+      </c>
+      <c r="D458" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E458" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="F458" t="n">
+        <v>83</v>
+      </c>
+      <c r="I458" t="n">
+        <v>173000000</v>
+      </c>
+      <c r="J458" t="b">
+        <v>0</v>
+      </c>
+      <c r="K458" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="L458" t="b">
+        <v>0</v>
+      </c>
+      <c r="M458" t="n">
+        <v>111</v>
+      </c>
+      <c r="N458" t="n">
+        <v>0</v>
+      </c>
+      <c r="O458" t="n">
+        <v>0</v>
+      </c>
+      <c r="P458" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Scream 2</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>card_458</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Wes Craven</t>
+        </is>
+      </c>
+      <c r="D459" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E459" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F459" t="n">
+        <v>73</v>
+      </c>
+      <c r="I459" t="n">
+        <v>172000000</v>
+      </c>
+      <c r="J459" t="b">
+        <v>0</v>
+      </c>
+      <c r="K459" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="L459" t="b">
+        <v>0</v>
+      </c>
+      <c r="M459" t="n">
+        <v>120</v>
+      </c>
+      <c r="N459" t="n">
+        <v>0</v>
+      </c>
+      <c r="O459" t="n">
+        <v>0</v>
+      </c>
+      <c r="P459" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Scream 3</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>card_459</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Wes Craven</t>
+        </is>
+      </c>
+      <c r="D460" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E460" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="F460" t="n">
+        <v>63</v>
+      </c>
+      <c r="I460" t="n">
+        <v>162000000</v>
+      </c>
+      <c r="J460" t="b">
+        <v>0</v>
+      </c>
+      <c r="K460" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L460" t="b">
+        <v>0</v>
+      </c>
+      <c r="M460" t="n">
+        <v>117</v>
+      </c>
+      <c r="N460" t="n">
+        <v>0</v>
+      </c>
+      <c r="O460" t="n">
+        <v>0</v>
+      </c>
+      <c r="P460" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Scream 4</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>card_460</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Wes Craven</t>
+        </is>
+      </c>
+      <c r="D461" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E461" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="F461" t="n">
+        <v>70</v>
+      </c>
+      <c r="I461" t="n">
+        <v>97000000</v>
+      </c>
+      <c r="J461" t="b">
+        <v>0</v>
+      </c>
+      <c r="K461" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L461" t="b">
+        <v>0</v>
+      </c>
+      <c r="M461" t="n">
+        <v>111</v>
+      </c>
+      <c r="N461" t="n">
+        <v>0</v>
+      </c>
+      <c r="O461" t="n">
+        <v>0</v>
+      </c>
+      <c r="P461" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Scream (2022)</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>card_461</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Matt Bettinelli-Olpin and Tyler Gillett</t>
+        </is>
+      </c>
+      <c r="D462" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E462" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F462" t="n">
+        <v>67</v>
+      </c>
+      <c r="I462" t="n">
+        <v>138000000</v>
+      </c>
+      <c r="J462" t="b">
+        <v>0</v>
+      </c>
+      <c r="K462" t="n">
+        <v>24000000</v>
+      </c>
+      <c r="L462" t="b">
+        <v>0</v>
+      </c>
+      <c r="M462" t="n">
+        <v>114</v>
+      </c>
+      <c r="N462" t="n">
+        <v>0</v>
+      </c>
+      <c r="O462" t="n">
+        <v>0</v>
+      </c>
+      <c r="P462" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Scream VI</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>card_462</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Matt Bettinelli-Olpin and Tyler Gillett</t>
+        </is>
+      </c>
+      <c r="D463" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E463" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="F463" t="n">
+        <v>66</v>
+      </c>
+      <c r="I463" t="n">
+        <v>167000000</v>
+      </c>
+      <c r="J463" t="b">
+        <v>0</v>
+      </c>
+      <c r="K463" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="L463" t="b">
+        <v>0</v>
+      </c>
+      <c r="M463" t="n">
+        <v>122</v>
+      </c>
+      <c r="N463" t="n">
+        <v>0</v>
+      </c>
+      <c r="O463" t="n">
+        <v>0</v>
+      </c>
+      <c r="P463" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Evil Dead series (card_463-467)
The Evil Dead, Evil Dead II, Army of Darkness, Evil Dead (2013), Evil
Dead Rise.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P463"/>
+  <dimension ref="A1:P468"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -24519,302 +24519,552 @@
       </c>
     </row>
     <row r="458">
-      <c r="A458" t="inlineStr">
+      <c r="A458" s="10" t="inlineStr">
         <is>
           <t>Scream</t>
         </is>
       </c>
-      <c r="B458" t="inlineStr">
+      <c r="B458" s="10" t="inlineStr">
         <is>
           <t>card_457</t>
         </is>
       </c>
-      <c r="C458" t="inlineStr">
+      <c r="C458" s="10" t="inlineStr">
         <is>
           <t>Wes Craven</t>
         </is>
       </c>
-      <c r="D458" t="n">
+      <c r="D458" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E458" t="n">
+      <c r="E458" s="10" t="n">
         <v>4.02</v>
       </c>
-      <c r="F458" t="n">
+      <c r="F458" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I458" t="n">
+      <c r="I458" s="10" t="n">
         <v>173000000</v>
       </c>
-      <c r="J458" t="b">
-        <v>0</v>
-      </c>
-      <c r="K458" t="n">
+      <c r="J458" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K458" s="10" t="n">
         <v>14000000</v>
       </c>
-      <c r="L458" t="b">
-        <v>0</v>
-      </c>
-      <c r="M458" t="n">
+      <c r="L458" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M458" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N458" t="n">
-        <v>0</v>
-      </c>
-      <c r="O458" t="n">
-        <v>0</v>
-      </c>
-      <c r="P458" t="b">
+      <c r="N458" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O458" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P458" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="459">
-      <c r="A459" t="inlineStr">
+      <c r="A459" s="10" t="inlineStr">
         <is>
           <t>Scream 2</t>
         </is>
       </c>
-      <c r="B459" t="inlineStr">
+      <c r="B459" s="10" t="inlineStr">
         <is>
           <t>card_458</t>
         </is>
       </c>
-      <c r="C459" t="inlineStr">
+      <c r="C459" s="10" t="inlineStr">
         <is>
           <t>Wes Craven</t>
         </is>
       </c>
-      <c r="D459" t="n">
+      <c r="D459" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E459" t="n">
+      <c r="E459" s="10" t="n">
         <v>3.27</v>
       </c>
-      <c r="F459" t="n">
+      <c r="F459" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I459" t="n">
+      <c r="I459" s="10" t="n">
         <v>172000000</v>
       </c>
-      <c r="J459" t="b">
-        <v>0</v>
-      </c>
-      <c r="K459" t="n">
+      <c r="J459" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K459" s="10" t="n">
         <v>24000000</v>
       </c>
-      <c r="L459" t="b">
-        <v>0</v>
-      </c>
-      <c r="M459" t="n">
+      <c r="L459" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M459" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="N459" t="n">
-        <v>0</v>
-      </c>
-      <c r="O459" t="n">
-        <v>0</v>
-      </c>
-      <c r="P459" t="b">
+      <c r="N459" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O459" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P459" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="460">
-      <c r="A460" t="inlineStr">
+      <c r="A460" s="10" t="inlineStr">
         <is>
           <t>Scream 3</t>
         </is>
       </c>
-      <c r="B460" t="inlineStr">
+      <c r="B460" s="10" t="inlineStr">
         <is>
           <t>card_459</t>
         </is>
       </c>
-      <c r="C460" t="inlineStr">
+      <c r="C460" s="10" t="inlineStr">
         <is>
           <t>Wes Craven</t>
         </is>
       </c>
-      <c r="D460" t="n">
+      <c r="D460" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E460" t="n">
+      <c r="E460" s="10" t="n">
         <v>2.91</v>
       </c>
-      <c r="F460" t="n">
+      <c r="F460" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I460" t="n">
+      <c r="I460" s="10" t="n">
         <v>162000000</v>
       </c>
-      <c r="J460" t="b">
-        <v>0</v>
-      </c>
-      <c r="K460" t="n">
+      <c r="J460" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K460" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L460" t="b">
-        <v>0</v>
-      </c>
-      <c r="M460" t="n">
+      <c r="L460" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M460" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N460" t="n">
-        <v>0</v>
-      </c>
-      <c r="O460" t="n">
-        <v>0</v>
-      </c>
-      <c r="P460" t="b">
+      <c r="N460" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O460" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P460" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="461">
-      <c r="A461" t="inlineStr">
+      <c r="A461" s="10" t="inlineStr">
         <is>
           <t>Scream 4</t>
         </is>
       </c>
-      <c r="B461" t="inlineStr">
+      <c r="B461" s="10" t="inlineStr">
         <is>
           <t>card_460</t>
         </is>
       </c>
-      <c r="C461" t="inlineStr">
+      <c r="C461" s="10" t="inlineStr">
         <is>
           <t>Wes Craven</t>
         </is>
       </c>
-      <c r="D461" t="n">
+      <c r="D461" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E461" t="n">
+      <c r="E461" s="10" t="n">
         <v>3.39</v>
       </c>
-      <c r="F461" t="n">
+      <c r="F461" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I461" t="n">
+      <c r="I461" s="10" t="n">
         <v>97000000</v>
       </c>
-      <c r="J461" t="b">
-        <v>0</v>
-      </c>
-      <c r="K461" t="n">
+      <c r="J461" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K461" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L461" t="b">
-        <v>0</v>
-      </c>
-      <c r="M461" t="n">
+      <c r="L461" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M461" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N461" t="n">
-        <v>0</v>
-      </c>
-      <c r="O461" t="n">
-        <v>0</v>
-      </c>
-      <c r="P461" t="b">
+      <c r="N461" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O461" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P461" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="462">
-      <c r="A462" t="inlineStr">
+      <c r="A462" s="10" t="inlineStr">
         <is>
           <t>Scream (2022)</t>
         </is>
       </c>
-      <c r="B462" t="inlineStr">
+      <c r="B462" s="10" t="inlineStr">
         <is>
           <t>card_461</t>
         </is>
       </c>
-      <c r="C462" t="inlineStr">
+      <c r="C462" s="10" t="inlineStr">
         <is>
           <t>Matt Bettinelli-Olpin and Tyler Gillett</t>
         </is>
       </c>
-      <c r="D462" t="n">
+      <c r="D462" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E462" t="n">
+      <c r="E462" s="10" t="n">
         <v>3.26</v>
       </c>
-      <c r="F462" t="n">
+      <c r="F462" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I462" t="n">
+      <c r="I462" s="10" t="n">
         <v>138000000</v>
       </c>
-      <c r="J462" t="b">
-        <v>0</v>
-      </c>
-      <c r="K462" t="n">
+      <c r="J462" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K462" s="10" t="n">
         <v>24000000</v>
       </c>
-      <c r="L462" t="b">
-        <v>0</v>
-      </c>
-      <c r="M462" t="n">
+      <c r="L462" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M462" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N462" t="n">
-        <v>0</v>
-      </c>
-      <c r="O462" t="n">
-        <v>0</v>
-      </c>
-      <c r="P462" t="b">
+      <c r="N462" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O462" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P462" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="463">
-      <c r="A463" t="inlineStr">
+      <c r="A463" s="10" t="inlineStr">
         <is>
           <t>Scream VI</t>
         </is>
       </c>
-      <c r="B463" t="inlineStr">
+      <c r="B463" s="10" t="inlineStr">
         <is>
           <t>card_462</t>
         </is>
       </c>
-      <c r="C463" t="inlineStr">
+      <c r="C463" s="10" t="inlineStr">
         <is>
           <t>Matt Bettinelli-Olpin and Tyler Gillett</t>
         </is>
       </c>
-      <c r="D463" t="n">
+      <c r="D463" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E463" t="n">
+      <c r="E463" s="10" t="n">
         <v>3.35</v>
       </c>
-      <c r="F463" t="n">
+      <c r="F463" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I463" t="n">
+      <c r="I463" s="10" t="n">
         <v>167000000</v>
       </c>
-      <c r="J463" t="b">
-        <v>0</v>
-      </c>
-      <c r="K463" t="n">
+      <c r="J463" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K463" s="10" t="n">
         <v>35000000</v>
       </c>
-      <c r="L463" t="b">
-        <v>0</v>
-      </c>
-      <c r="M463" t="n">
+      <c r="L463" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M463" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N463" t="n">
-        <v>0</v>
-      </c>
-      <c r="O463" t="n">
-        <v>0</v>
-      </c>
-      <c r="P463" t="b">
+      <c r="N463" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O463" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P463" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>The Evil Dead</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>card_463</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>Sam Raimi</t>
+        </is>
+      </c>
+      <c r="D464" t="n">
+        <v>1981</v>
+      </c>
+      <c r="E464" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="F464" t="n">
+        <v>79</v>
+      </c>
+      <c r="I464" t="n">
+        <v>29400000</v>
+      </c>
+      <c r="J464" t="b">
+        <v>0</v>
+      </c>
+      <c r="K464" t="n">
+        <v>375000</v>
+      </c>
+      <c r="L464" t="b">
+        <v>0</v>
+      </c>
+      <c r="M464" t="n">
+        <v>85</v>
+      </c>
+      <c r="N464" t="n">
+        <v>0</v>
+      </c>
+      <c r="O464" t="n">
+        <v>0</v>
+      </c>
+      <c r="P464" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Evil Dead II</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>card_464</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Sam Raimi</t>
+        </is>
+      </c>
+      <c r="D465" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E465" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="F465" t="n">
+        <v>82</v>
+      </c>
+      <c r="I465" t="n">
+        <v>5900000</v>
+      </c>
+      <c r="J465" t="b">
+        <v>0</v>
+      </c>
+      <c r="K465" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="L465" t="b">
+        <v>0</v>
+      </c>
+      <c r="M465" t="n">
+        <v>84</v>
+      </c>
+      <c r="N465" t="n">
+        <v>0</v>
+      </c>
+      <c r="O465" t="n">
+        <v>0</v>
+      </c>
+      <c r="P465" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Army of Darkness</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>card_465</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Sam Raimi</t>
+        </is>
+      </c>
+      <c r="D466" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E466" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F466" t="n">
+        <v>79</v>
+      </c>
+      <c r="I466" t="n">
+        <v>21500000</v>
+      </c>
+      <c r="J466" t="b">
+        <v>0</v>
+      </c>
+      <c r="K466" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="L466" t="b">
+        <v>0</v>
+      </c>
+      <c r="M466" t="n">
+        <v>81</v>
+      </c>
+      <c r="N466" t="n">
+        <v>0</v>
+      </c>
+      <c r="O466" t="n">
+        <v>0</v>
+      </c>
+      <c r="P466" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Evil Dead</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>card_466</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Fede Alvarez</t>
+        </is>
+      </c>
+      <c r="D467" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E467" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F467" t="n">
+        <v>72</v>
+      </c>
+      <c r="I467" t="n">
+        <v>97500000</v>
+      </c>
+      <c r="J467" t="b">
+        <v>0</v>
+      </c>
+      <c r="K467" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="L467" t="b">
+        <v>0</v>
+      </c>
+      <c r="M467" t="n">
+        <v>92</v>
+      </c>
+      <c r="N467" t="n">
+        <v>0</v>
+      </c>
+      <c r="O467" t="n">
+        <v>0</v>
+      </c>
+      <c r="P467" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Evil Dead Rise</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>card_467</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Lee Cronin</t>
+        </is>
+      </c>
+      <c r="D468" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E468" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F468" t="n">
+        <v>69</v>
+      </c>
+      <c r="I468" t="n">
+        <v>147000000</v>
+      </c>
+      <c r="J468" t="b">
+        <v>0</v>
+      </c>
+      <c r="K468" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="L468" t="b">
+        <v>0</v>
+      </c>
+      <c r="M468" t="n">
+        <v>96</v>
+      </c>
+      <c r="N468" t="n">
+        <v>0</v>
+      </c>
+      <c r="O468" t="n">
+        <v>0</v>
+      </c>
+      <c r="P468" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Planet of the Apes series (card_468-476)
All 5 original films plus the Rise/Dawn/War/Kingdom reboot tetralogy.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P468"/>
+  <dimension ref="A1:P477"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -24819,252 +24819,702 @@
       </c>
     </row>
     <row r="464">
-      <c r="A464" t="inlineStr">
+      <c r="A464" s="10" t="inlineStr">
         <is>
           <t>The Evil Dead</t>
         </is>
       </c>
-      <c r="B464" t="inlineStr">
+      <c r="B464" s="10" t="inlineStr">
         <is>
           <t>card_463</t>
         </is>
       </c>
-      <c r="C464" t="inlineStr">
+      <c r="C464" s="10" t="inlineStr">
         <is>
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="D464" t="n">
+      <c r="D464" s="10" t="n">
         <v>1981</v>
       </c>
-      <c r="E464" t="n">
+      <c r="E464" s="10" t="n">
         <v>3.62</v>
       </c>
-      <c r="F464" t="n">
+      <c r="F464" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I464" t="n">
+      <c r="I464" s="10" t="n">
         <v>29400000</v>
       </c>
-      <c r="J464" t="b">
-        <v>0</v>
-      </c>
-      <c r="K464" t="n">
+      <c r="J464" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K464" s="10" t="n">
         <v>375000</v>
       </c>
-      <c r="L464" t="b">
-        <v>0</v>
-      </c>
-      <c r="M464" t="n">
+      <c r="L464" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M464" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="N464" t="n">
-        <v>0</v>
-      </c>
-      <c r="O464" t="n">
-        <v>0</v>
-      </c>
-      <c r="P464" t="b">
+      <c r="N464" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O464" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P464" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="465">
-      <c r="A465" t="inlineStr">
+      <c r="A465" s="10" t="inlineStr">
         <is>
           <t>Evil Dead II</t>
         </is>
       </c>
-      <c r="B465" t="inlineStr">
+      <c r="B465" s="10" t="inlineStr">
         <is>
           <t>card_464</t>
         </is>
       </c>
-      <c r="C465" t="inlineStr">
+      <c r="C465" s="10" t="inlineStr">
         <is>
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="D465" t="n">
+      <c r="D465" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E465" t="n">
+      <c r="E465" s="10" t="n">
         <v>3.99</v>
       </c>
-      <c r="F465" t="n">
+      <c r="F465" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I465" t="n">
+      <c r="I465" s="10" t="n">
         <v>5900000</v>
       </c>
-      <c r="J465" t="b">
-        <v>0</v>
-      </c>
-      <c r="K465" t="n">
+      <c r="J465" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K465" s="10" t="n">
         <v>3500000</v>
       </c>
-      <c r="L465" t="b">
-        <v>0</v>
-      </c>
-      <c r="M465" t="n">
+      <c r="L465" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M465" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="N465" t="n">
-        <v>0</v>
-      </c>
-      <c r="O465" t="n">
-        <v>0</v>
-      </c>
-      <c r="P465" t="b">
+      <c r="N465" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O465" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P465" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="466">
-      <c r="A466" t="inlineStr">
+      <c r="A466" s="10" t="inlineStr">
         <is>
           <t>Army of Darkness</t>
         </is>
       </c>
-      <c r="B466" t="inlineStr">
+      <c r="B466" s="10" t="inlineStr">
         <is>
           <t>card_465</t>
         </is>
       </c>
-      <c r="C466" t="inlineStr">
+      <c r="C466" s="10" t="inlineStr">
         <is>
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="D466" t="n">
+      <c r="D466" s="10" t="n">
         <v>1992</v>
       </c>
-      <c r="E466" t="n">
+      <c r="E466" s="10" t="n">
         <v>3.71</v>
       </c>
-      <c r="F466" t="n">
+      <c r="F466" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I466" t="n">
+      <c r="I466" s="10" t="n">
         <v>21500000</v>
       </c>
-      <c r="J466" t="b">
-        <v>0</v>
-      </c>
-      <c r="K466" t="n">
+      <c r="J466" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K466" s="10" t="n">
         <v>11000000</v>
       </c>
-      <c r="L466" t="b">
-        <v>0</v>
-      </c>
-      <c r="M466" t="n">
+      <c r="L466" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M466" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="N466" t="n">
-        <v>0</v>
-      </c>
-      <c r="O466" t="n">
-        <v>0</v>
-      </c>
-      <c r="P466" t="b">
+      <c r="N466" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O466" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P466" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="467">
-      <c r="A467" t="inlineStr">
+      <c r="A467" s="10" t="inlineStr">
         <is>
           <t>Evil Dead</t>
         </is>
       </c>
-      <c r="B467" t="inlineStr">
+      <c r="B467" s="10" t="inlineStr">
         <is>
           <t>card_466</t>
         </is>
       </c>
-      <c r="C467" t="inlineStr">
+      <c r="C467" s="10" t="inlineStr">
         <is>
           <t>Fede Alvarez</t>
         </is>
       </c>
-      <c r="D467" t="n">
+      <c r="D467" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E467" t="n">
+      <c r="E467" s="10" t="n">
         <v>3.41</v>
       </c>
-      <c r="F467" t="n">
+      <c r="F467" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I467" t="n">
+      <c r="I467" s="10" t="n">
         <v>97500000</v>
       </c>
-      <c r="J467" t="b">
-        <v>0</v>
-      </c>
-      <c r="K467" t="n">
+      <c r="J467" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K467" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="L467" t="b">
-        <v>0</v>
-      </c>
-      <c r="M467" t="n">
+      <c r="L467" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M467" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="N467" t="n">
-        <v>0</v>
-      </c>
-      <c r="O467" t="n">
-        <v>0</v>
-      </c>
-      <c r="P467" t="b">
+      <c r="N467" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O467" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P467" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="468">
-      <c r="A468" t="inlineStr">
+      <c r="A468" s="10" t="inlineStr">
         <is>
           <t>Evil Dead Rise</t>
         </is>
       </c>
-      <c r="B468" t="inlineStr">
+      <c r="B468" s="10" t="inlineStr">
         <is>
           <t>card_467</t>
         </is>
       </c>
-      <c r="C468" t="inlineStr">
+      <c r="C468" s="10" t="inlineStr">
         <is>
           <t>Lee Cronin</t>
         </is>
       </c>
-      <c r="D468" t="n">
+      <c r="D468" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E468" t="n">
+      <c r="E468" s="10" t="n">
         <v>3.15</v>
       </c>
-      <c r="F468" t="n">
+      <c r="F468" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I468" t="n">
+      <c r="I468" s="10" t="n">
         <v>147000000</v>
       </c>
-      <c r="J468" t="b">
-        <v>0</v>
-      </c>
-      <c r="K468" t="n">
+      <c r="J468" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K468" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="L468" t="b">
-        <v>0</v>
-      </c>
-      <c r="M468" t="n">
+      <c r="L468" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M468" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N468" t="n">
-        <v>0</v>
-      </c>
-      <c r="O468" t="n">
-        <v>0</v>
-      </c>
-      <c r="P468" t="b">
+      <c r="N468" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O468" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P468" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>card_468</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Franklin J. Schaffner</t>
+        </is>
+      </c>
+      <c r="D469" t="n">
+        <v>1968</v>
+      </c>
+      <c r="E469" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F469" t="n">
+        <v>83</v>
+      </c>
+      <c r="I469" t="n">
+        <v>33300000</v>
+      </c>
+      <c r="J469" t="b">
+        <v>1</v>
+      </c>
+      <c r="K469" t="n">
+        <v>5800000</v>
+      </c>
+      <c r="L469" t="b">
+        <v>0</v>
+      </c>
+      <c r="M469" t="n">
+        <v>112</v>
+      </c>
+      <c r="N469" t="n">
+        <v>1</v>
+      </c>
+      <c r="O469" t="n">
+        <v>1</v>
+      </c>
+      <c r="P469" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Beneath the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>card_469</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Ted Post</t>
+        </is>
+      </c>
+      <c r="D470" t="n">
+        <v>1970</v>
+      </c>
+      <c r="E470" t="n">
+        <v>2.78</v>
+      </c>
+      <c r="F470" t="n">
+        <v>53</v>
+      </c>
+      <c r="I470" t="n">
+        <v>19000000</v>
+      </c>
+      <c r="J470" t="b">
+        <v>1</v>
+      </c>
+      <c r="K470" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="L470" t="b">
+        <v>0</v>
+      </c>
+      <c r="M470" t="n">
+        <v>95</v>
+      </c>
+      <c r="N470" t="n">
+        <v>0</v>
+      </c>
+      <c r="O470" t="n">
+        <v>0</v>
+      </c>
+      <c r="P470" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Escape from the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>card_470</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Don Taylor</t>
+        </is>
+      </c>
+      <c r="D471" t="n">
+        <v>1971</v>
+      </c>
+      <c r="E471" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F471" t="n">
+        <v>67</v>
+      </c>
+      <c r="I471" t="n">
+        <v>12300000</v>
+      </c>
+      <c r="J471" t="b">
+        <v>0</v>
+      </c>
+      <c r="K471" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="L471" t="b">
+        <v>0</v>
+      </c>
+      <c r="M471" t="n">
+        <v>98</v>
+      </c>
+      <c r="N471" t="n">
+        <v>0</v>
+      </c>
+      <c r="O471" t="n">
+        <v>0</v>
+      </c>
+      <c r="P471" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Conquest of the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>card_471</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>J. Lee Thompson</t>
+        </is>
+      </c>
+      <c r="D472" t="n">
+        <v>1972</v>
+      </c>
+      <c r="E472" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F472" t="n">
+        <v>62</v>
+      </c>
+      <c r="I472" t="n">
+        <v>9700000</v>
+      </c>
+      <c r="J472" t="b">
+        <v>0</v>
+      </c>
+      <c r="K472" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="L472" t="b">
+        <v>0</v>
+      </c>
+      <c r="M472" t="n">
+        <v>88</v>
+      </c>
+      <c r="N472" t="n">
+        <v>0</v>
+      </c>
+      <c r="O472" t="n">
+        <v>0</v>
+      </c>
+      <c r="P472" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Battle for the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>card_472</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>J. Lee Thompson</t>
+        </is>
+      </c>
+      <c r="D473" t="n">
+        <v>1973</v>
+      </c>
+      <c r="E473" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F473" t="n">
+        <v>53</v>
+      </c>
+      <c r="I473" t="n">
+        <v>8800000</v>
+      </c>
+      <c r="J473" t="b">
+        <v>0</v>
+      </c>
+      <c r="K473" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="L473" t="b">
+        <v>0</v>
+      </c>
+      <c r="M473" t="n">
+        <v>87</v>
+      </c>
+      <c r="N473" t="n">
+        <v>0</v>
+      </c>
+      <c r="O473" t="n">
+        <v>0</v>
+      </c>
+      <c r="P473" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Rise of the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>card_473</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Rupert Wyatt</t>
+        </is>
+      </c>
+      <c r="D474" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E474" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F474" t="n">
+        <v>78</v>
+      </c>
+      <c r="I474" t="n">
+        <v>481800000</v>
+      </c>
+      <c r="J474" t="b">
+        <v>0</v>
+      </c>
+      <c r="K474" t="n">
+        <v>93000000</v>
+      </c>
+      <c r="L474" t="b">
+        <v>0</v>
+      </c>
+      <c r="M474" t="n">
+        <v>105</v>
+      </c>
+      <c r="N474" t="n">
+        <v>0</v>
+      </c>
+      <c r="O474" t="n">
+        <v>0</v>
+      </c>
+      <c r="P474" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Dawn of the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>card_474</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Matt Reeves</t>
+        </is>
+      </c>
+      <c r="D475" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E475" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F475" t="n">
+        <v>82</v>
+      </c>
+      <c r="I475" t="n">
+        <v>710600000</v>
+      </c>
+      <c r="J475" t="b">
+        <v>0</v>
+      </c>
+      <c r="K475" t="n">
+        <v>170000000</v>
+      </c>
+      <c r="L475" t="b">
+        <v>0</v>
+      </c>
+      <c r="M475" t="n">
+        <v>130</v>
+      </c>
+      <c r="N475" t="n">
+        <v>0</v>
+      </c>
+      <c r="O475" t="n">
+        <v>0</v>
+      </c>
+      <c r="P475" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>War for the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>card_475</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>Matt Reeves</t>
+        </is>
+      </c>
+      <c r="D476" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E476" t="n">
+        <v>3.83</v>
+      </c>
+      <c r="F476" t="n">
+        <v>79</v>
+      </c>
+      <c r="I476" t="n">
+        <v>490700000</v>
+      </c>
+      <c r="J476" t="b">
+        <v>0</v>
+      </c>
+      <c r="K476" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L476" t="b">
+        <v>0</v>
+      </c>
+      <c r="M476" t="n">
+        <v>140</v>
+      </c>
+      <c r="N476" t="n">
+        <v>0</v>
+      </c>
+      <c r="O476" t="n">
+        <v>0</v>
+      </c>
+      <c r="P476" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Kingdom of the Planet of the Apes</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>card_476</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>Wes Ball</t>
+        </is>
+      </c>
+      <c r="D477" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E477" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="F477" t="n">
+        <v>70</v>
+      </c>
+      <c r="I477" t="n">
+        <v>397300000</v>
+      </c>
+      <c r="J477" t="b">
+        <v>0</v>
+      </c>
+      <c r="K477" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L477" t="b">
+        <v>0</v>
+      </c>
+      <c r="M477" t="n">
+        <v>145</v>
+      </c>
+      <c r="N477" t="n">
+        <v>0</v>
+      </c>
+      <c r="O477" t="n">
+        <v>0</v>
+      </c>
+      <c r="P477" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Saw series (card_477-486)
All 10 films: Saw through Saw X, including Jigsaw and Spiral.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P477"/>
+  <dimension ref="A1:P487"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -25069,452 +25069,952 @@
       </c>
     </row>
     <row r="469">
-      <c r="A469" t="inlineStr">
+      <c r="A469" s="10" t="inlineStr">
         <is>
           <t>Planet of the Apes</t>
         </is>
       </c>
-      <c r="B469" t="inlineStr">
+      <c r="B469" s="10" t="inlineStr">
         <is>
           <t>card_468</t>
         </is>
       </c>
-      <c r="C469" t="inlineStr">
+      <c r="C469" s="10" t="inlineStr">
         <is>
           <t>Franklin J. Schaffner</t>
         </is>
       </c>
-      <c r="D469" t="n">
+      <c r="D469" s="10" t="n">
         <v>1968</v>
       </c>
-      <c r="E469" t="n">
+      <c r="E469" s="10" t="n">
         <v>4.01</v>
       </c>
-      <c r="F469" t="n">
+      <c r="F469" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I469" t="n">
+      <c r="I469" s="10" t="n">
         <v>33300000</v>
       </c>
-      <c r="J469" t="b">
+      <c r="J469" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K469" t="n">
+      <c r="K469" s="10" t="n">
         <v>5800000</v>
       </c>
-      <c r="L469" t="b">
-        <v>0</v>
-      </c>
-      <c r="M469" t="n">
+      <c r="L469" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M469" s="10" t="n">
         <v>112</v>
       </c>
-      <c r="N469" t="n">
+      <c r="N469" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O469" t="n">
+      <c r="O469" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P469" t="b">
+      <c r="P469" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="470">
-      <c r="A470" t="inlineStr">
+      <c r="A470" s="10" t="inlineStr">
         <is>
           <t>Beneath the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B470" t="inlineStr">
+      <c r="B470" s="10" t="inlineStr">
         <is>
           <t>card_469</t>
         </is>
       </c>
-      <c r="C470" t="inlineStr">
+      <c r="C470" s="10" t="inlineStr">
         <is>
           <t>Ted Post</t>
         </is>
       </c>
-      <c r="D470" t="n">
+      <c r="D470" s="10" t="n">
         <v>1970</v>
       </c>
-      <c r="E470" t="n">
+      <c r="E470" s="10" t="n">
         <v>2.78</v>
       </c>
-      <c r="F470" t="n">
+      <c r="F470" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="I470" t="n">
+      <c r="I470" s="10" t="n">
         <v>19000000</v>
       </c>
-      <c r="J470" t="b">
+      <c r="J470" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K470" t="n">
+      <c r="K470" s="10" t="n">
         <v>2500000</v>
       </c>
-      <c r="L470" t="b">
-        <v>0</v>
-      </c>
-      <c r="M470" t="n">
+      <c r="L470" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M470" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N470" t="n">
-        <v>0</v>
-      </c>
-      <c r="O470" t="n">
-        <v>0</v>
-      </c>
-      <c r="P470" t="b">
+      <c r="N470" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O470" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P470" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="471">
-      <c r="A471" t="inlineStr">
+      <c r="A471" s="10" t="inlineStr">
         <is>
           <t>Escape from the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B471" t="inlineStr">
+      <c r="B471" s="10" t="inlineStr">
         <is>
           <t>card_470</t>
         </is>
       </c>
-      <c r="C471" t="inlineStr">
+      <c r="C471" s="10" t="inlineStr">
         <is>
           <t>Don Taylor</t>
         </is>
       </c>
-      <c r="D471" t="n">
+      <c r="D471" s="10" t="n">
         <v>1971</v>
       </c>
-      <c r="E471" t="n">
+      <c r="E471" s="10" t="n">
         <v>3.25</v>
       </c>
-      <c r="F471" t="n">
+      <c r="F471" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I471" t="n">
+      <c r="I471" s="10" t="n">
         <v>12300000</v>
       </c>
-      <c r="J471" t="b">
-        <v>0</v>
-      </c>
-      <c r="K471" t="n">
+      <c r="J471" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K471" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="L471" t="b">
-        <v>0</v>
-      </c>
-      <c r="M471" t="n">
+      <c r="L471" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M471" s="10" t="n">
         <v>98</v>
       </c>
-      <c r="N471" t="n">
-        <v>0</v>
-      </c>
-      <c r="O471" t="n">
-        <v>0</v>
-      </c>
-      <c r="P471" t="b">
+      <c r="N471" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O471" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P471" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="472">
-      <c r="A472" t="inlineStr">
+      <c r="A472" s="10" t="inlineStr">
         <is>
           <t>Conquest of the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B472" t="inlineStr">
+      <c r="B472" s="10" t="inlineStr">
         <is>
           <t>card_471</t>
         </is>
       </c>
-      <c r="C472" t="inlineStr">
+      <c r="C472" s="10" t="inlineStr">
         <is>
           <t>J. Lee Thompson</t>
         </is>
       </c>
-      <c r="D472" t="n">
+      <c r="D472" s="10" t="n">
         <v>1972</v>
       </c>
-      <c r="E472" t="n">
+      <c r="E472" s="10" t="n">
         <v>3.16</v>
       </c>
-      <c r="F472" t="n">
+      <c r="F472" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I472" t="n">
+      <c r="I472" s="10" t="n">
         <v>9700000</v>
       </c>
-      <c r="J472" t="b">
-        <v>0</v>
-      </c>
-      <c r="K472" t="n">
+      <c r="J472" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K472" s="10" t="n">
         <v>1700000</v>
       </c>
-      <c r="L472" t="b">
-        <v>0</v>
-      </c>
-      <c r="M472" t="n">
+      <c r="L472" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M472" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N472" t="n">
-        <v>0</v>
-      </c>
-      <c r="O472" t="n">
-        <v>0</v>
-      </c>
-      <c r="P472" t="b">
+      <c r="N472" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O472" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P472" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="473">
-      <c r="A473" t="inlineStr">
+      <c r="A473" s="10" t="inlineStr">
         <is>
           <t>Battle for the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B473" t="inlineStr">
+      <c r="B473" s="10" t="inlineStr">
         <is>
           <t>card_472</t>
         </is>
       </c>
-      <c r="C473" t="inlineStr">
+      <c r="C473" s="10" t="inlineStr">
         <is>
           <t>J. Lee Thompson</t>
         </is>
       </c>
-      <c r="D473" t="n">
+      <c r="D473" s="10" t="n">
         <v>1973</v>
       </c>
-      <c r="E473" t="n">
+      <c r="E473" s="10" t="n">
         <v>2.6</v>
       </c>
-      <c r="F473" t="n">
+      <c r="F473" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="I473" t="n">
+      <c r="I473" s="10" t="n">
         <v>8800000</v>
       </c>
-      <c r="J473" t="b">
-        <v>0</v>
-      </c>
-      <c r="K473" t="n">
+      <c r="J473" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K473" s="10" t="n">
         <v>1700000</v>
       </c>
-      <c r="L473" t="b">
-        <v>0</v>
-      </c>
-      <c r="M473" t="n">
+      <c r="L473" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M473" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="N473" t="n">
-        <v>0</v>
-      </c>
-      <c r="O473" t="n">
-        <v>0</v>
-      </c>
-      <c r="P473" t="b">
+      <c r="N473" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O473" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P473" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="474">
-      <c r="A474" t="inlineStr">
+      <c r="A474" s="10" t="inlineStr">
         <is>
           <t>Rise of the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B474" t="inlineStr">
+      <c r="B474" s="10" t="inlineStr">
         <is>
           <t>card_473</t>
         </is>
       </c>
-      <c r="C474" t="inlineStr">
+      <c r="C474" s="10" t="inlineStr">
         <is>
           <t>Rupert Wyatt</t>
         </is>
       </c>
-      <c r="D474" t="n">
+      <c r="D474" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E474" t="n">
+      <c r="E474" s="10" t="n">
         <v>3.69</v>
       </c>
-      <c r="F474" t="n">
+      <c r="F474" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I474" t="n">
+      <c r="I474" s="10" t="n">
         <v>481800000</v>
       </c>
-      <c r="J474" t="b">
-        <v>0</v>
-      </c>
-      <c r="K474" t="n">
+      <c r="J474" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K474" s="10" t="n">
         <v>93000000</v>
       </c>
-      <c r="L474" t="b">
-        <v>0</v>
-      </c>
-      <c r="M474" t="n">
+      <c r="L474" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M474" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="N474" t="n">
-        <v>0</v>
-      </c>
-      <c r="O474" t="n">
-        <v>0</v>
-      </c>
-      <c r="P474" t="b">
+      <c r="N474" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O474" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P474" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="475">
-      <c r="A475" t="inlineStr">
+      <c r="A475" s="10" t="inlineStr">
         <is>
           <t>Dawn of the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B475" t="inlineStr">
+      <c r="B475" s="10" t="inlineStr">
         <is>
           <t>card_474</t>
         </is>
       </c>
-      <c r="C475" t="inlineStr">
+      <c r="C475" s="10" t="inlineStr">
         <is>
           <t>Matt Reeves</t>
         </is>
       </c>
-      <c r="D475" t="n">
+      <c r="D475" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E475" t="n">
+      <c r="E475" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="F475" t="n">
+      <c r="F475" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I475" t="n">
+      <c r="I475" s="10" t="n">
         <v>710600000</v>
       </c>
-      <c r="J475" t="b">
-        <v>0</v>
-      </c>
-      <c r="K475" t="n">
+      <c r="J475" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K475" s="10" t="n">
         <v>170000000</v>
       </c>
-      <c r="L475" t="b">
-        <v>0</v>
-      </c>
-      <c r="M475" t="n">
+      <c r="L475" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M475" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N475" t="n">
-        <v>0</v>
-      </c>
-      <c r="O475" t="n">
-        <v>0</v>
-      </c>
-      <c r="P475" t="b">
+      <c r="N475" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O475" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P475" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="476">
-      <c r="A476" t="inlineStr">
+      <c r="A476" s="10" t="inlineStr">
         <is>
           <t>War for the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B476" t="inlineStr">
+      <c r="B476" s="10" t="inlineStr">
         <is>
           <t>card_475</t>
         </is>
       </c>
-      <c r="C476" t="inlineStr">
+      <c r="C476" s="10" t="inlineStr">
         <is>
           <t>Matt Reeves</t>
         </is>
       </c>
-      <c r="D476" t="n">
+      <c r="D476" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E476" t="n">
+      <c r="E476" s="10" t="n">
         <v>3.83</v>
       </c>
-      <c r="F476" t="n">
+      <c r="F476" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I476" t="n">
+      <c r="I476" s="10" t="n">
         <v>490700000</v>
       </c>
-      <c r="J476" t="b">
-        <v>0</v>
-      </c>
-      <c r="K476" t="n">
+      <c r="J476" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K476" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L476" t="b">
-        <v>0</v>
-      </c>
-      <c r="M476" t="n">
+      <c r="L476" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M476" s="10" t="n">
         <v>140</v>
       </c>
-      <c r="N476" t="n">
-        <v>0</v>
-      </c>
-      <c r="O476" t="n">
-        <v>0</v>
-      </c>
-      <c r="P476" t="b">
+      <c r="N476" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O476" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P476" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="477">
-      <c r="A477" t="inlineStr">
+      <c r="A477" s="10" t="inlineStr">
         <is>
           <t>Kingdom of the Planet of the Apes</t>
         </is>
       </c>
-      <c r="B477" t="inlineStr">
+      <c r="B477" s="10" t="inlineStr">
         <is>
           <t>card_476</t>
         </is>
       </c>
-      <c r="C477" t="inlineStr">
+      <c r="C477" s="10" t="inlineStr">
         <is>
           <t>Wes Ball</t>
         </is>
       </c>
-      <c r="D477" t="n">
+      <c r="D477" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="E477" t="n">
+      <c r="E477" s="10" t="n">
         <v>3.32</v>
       </c>
-      <c r="F477" t="n">
+      <c r="F477" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I477" t="n">
+      <c r="I477" s="10" t="n">
         <v>397300000</v>
       </c>
-      <c r="J477" t="b">
-        <v>0</v>
-      </c>
-      <c r="K477" t="n">
+      <c r="J477" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K477" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L477" t="b">
-        <v>0</v>
-      </c>
-      <c r="M477" t="n">
+      <c r="L477" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M477" s="10" t="n">
         <v>145</v>
       </c>
-      <c r="N477" t="n">
-        <v>0</v>
-      </c>
-      <c r="O477" t="n">
-        <v>0</v>
-      </c>
-      <c r="P477" t="b">
+      <c r="N477" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O477" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P477" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Saw</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>card_477</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>James Wan</t>
+        </is>
+      </c>
+      <c r="D478" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E478" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F478" t="n">
+        <v>77</v>
+      </c>
+      <c r="I478" t="n">
+        <v>104000000</v>
+      </c>
+      <c r="J478" t="b">
+        <v>0</v>
+      </c>
+      <c r="K478" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="L478" t="b">
+        <v>0</v>
+      </c>
+      <c r="M478" t="n">
+        <v>103</v>
+      </c>
+      <c r="N478" t="n">
+        <v>0</v>
+      </c>
+      <c r="O478" t="n">
+        <v>0</v>
+      </c>
+      <c r="P478" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Saw II</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>card_478</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Darren Lynn Bousman</t>
+        </is>
+      </c>
+      <c r="D479" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E479" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F479" t="n">
+        <v>69</v>
+      </c>
+      <c r="I479" t="n">
+        <v>152900000</v>
+      </c>
+      <c r="J479" t="b">
+        <v>0</v>
+      </c>
+      <c r="K479" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L479" t="b">
+        <v>0</v>
+      </c>
+      <c r="M479" t="n">
+        <v>93</v>
+      </c>
+      <c r="N479" t="n">
+        <v>0</v>
+      </c>
+      <c r="O479" t="n">
+        <v>0</v>
+      </c>
+      <c r="P479" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Saw III</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>card_479</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Darren Lynn Bousman</t>
+        </is>
+      </c>
+      <c r="D480" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E480" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="F480" t="n">
+        <v>66</v>
+      </c>
+      <c r="I480" t="n">
+        <v>164900000</v>
+      </c>
+      <c r="J480" t="b">
+        <v>0</v>
+      </c>
+      <c r="K480" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L480" t="b">
+        <v>0</v>
+      </c>
+      <c r="M480" t="n">
+        <v>108</v>
+      </c>
+      <c r="N480" t="n">
+        <v>0</v>
+      </c>
+      <c r="O480" t="n">
+        <v>0</v>
+      </c>
+      <c r="P480" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Saw IV</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>card_480</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Darren Lynn Bousman</t>
+        </is>
+      </c>
+      <c r="D481" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E481" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="F481" t="n">
+        <v>59</v>
+      </c>
+      <c r="I481" t="n">
+        <v>139400000</v>
+      </c>
+      <c r="J481" t="b">
+        <v>0</v>
+      </c>
+      <c r="K481" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L481" t="b">
+        <v>0</v>
+      </c>
+      <c r="M481" t="n">
+        <v>92</v>
+      </c>
+      <c r="N481" t="n">
+        <v>0</v>
+      </c>
+      <c r="O481" t="n">
+        <v>0</v>
+      </c>
+      <c r="P481" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Saw V</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>card_481</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>David Hackl</t>
+        </is>
+      </c>
+      <c r="D482" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E482" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="F482" t="n">
+        <v>55</v>
+      </c>
+      <c r="I482" t="n">
+        <v>118200000</v>
+      </c>
+      <c r="J482" t="b">
+        <v>0</v>
+      </c>
+      <c r="K482" t="n">
+        <v>10800000</v>
+      </c>
+      <c r="L482" t="b">
+        <v>0</v>
+      </c>
+      <c r="M482" t="n">
+        <v>92</v>
+      </c>
+      <c r="N482" t="n">
+        <v>0</v>
+      </c>
+      <c r="O482" t="n">
+        <v>0</v>
+      </c>
+      <c r="P482" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Saw VI</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>card_482</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Kevin Greutert</t>
+        </is>
+      </c>
+      <c r="D483" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E483" t="n">
+        <v>2.97</v>
+      </c>
+      <c r="F483" t="n">
+        <v>65</v>
+      </c>
+      <c r="I483" t="n">
+        <v>69800000</v>
+      </c>
+      <c r="J483" t="b">
+        <v>0</v>
+      </c>
+      <c r="K483" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="L483" t="b">
+        <v>0</v>
+      </c>
+      <c r="M483" t="n">
+        <v>90</v>
+      </c>
+      <c r="N483" t="n">
+        <v>0</v>
+      </c>
+      <c r="O483" t="n">
+        <v>0</v>
+      </c>
+      <c r="P483" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Saw 3D</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>card_483</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Kevin Greutert</t>
+        </is>
+      </c>
+      <c r="D484" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E484" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="F484" t="n">
+        <v>52</v>
+      </c>
+      <c r="I484" t="n">
+        <v>136200000</v>
+      </c>
+      <c r="J484" t="b">
+        <v>0</v>
+      </c>
+      <c r="K484" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="L484" t="b">
+        <v>0</v>
+      </c>
+      <c r="M484" t="n">
+        <v>90</v>
+      </c>
+      <c r="N484" t="n">
+        <v>0</v>
+      </c>
+      <c r="O484" t="n">
+        <v>0</v>
+      </c>
+      <c r="P484" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Jigsaw</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>card_484</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Michael Spierig and Peter Spierig</t>
+        </is>
+      </c>
+      <c r="D485" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E485" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="F485" t="n">
+        <v>59</v>
+      </c>
+      <c r="I485" t="n">
+        <v>104200000</v>
+      </c>
+      <c r="J485" t="b">
+        <v>0</v>
+      </c>
+      <c r="K485" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L485" t="b">
+        <v>0</v>
+      </c>
+      <c r="M485" t="n">
+        <v>92</v>
+      </c>
+      <c r="N485" t="n">
+        <v>0</v>
+      </c>
+      <c r="O485" t="n">
+        <v>0</v>
+      </c>
+      <c r="P485" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Spiral: From the Book of Saw</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>card_485</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Darren Lynn Bousman</t>
+        </is>
+      </c>
+      <c r="D486" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E486" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="F486" t="n">
+        <v>50</v>
+      </c>
+      <c r="I486" t="n">
+        <v>40600000</v>
+      </c>
+      <c r="J486" t="b">
+        <v>0</v>
+      </c>
+      <c r="K486" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L486" t="b">
+        <v>0</v>
+      </c>
+      <c r="M486" t="n">
+        <v>93</v>
+      </c>
+      <c r="N486" t="n">
+        <v>0</v>
+      </c>
+      <c r="O486" t="n">
+        <v>0</v>
+      </c>
+      <c r="P486" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Saw X</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>card_486</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Kevin Greutert</t>
+        </is>
+      </c>
+      <c r="D487" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E487" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="F487" t="n">
+        <v>73</v>
+      </c>
+      <c r="I487" t="n">
+        <v>125300000</v>
+      </c>
+      <c r="J487" t="b">
+        <v>0</v>
+      </c>
+      <c r="K487" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="L487" t="b">
+        <v>0</v>
+      </c>
+      <c r="M487" t="n">
+        <v>118</v>
+      </c>
+      <c r="N487" t="n">
+        <v>0</v>
+      </c>
+      <c r="O487" t="n">
+        <v>0</v>
+      </c>
+      <c r="P487" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Halloween films (card_487-498)
Halloween II (1981) through Halloween Ends (2022), 12 films spanning
the original, Thorn, and Rob Zombie/David Gordon Green timelines.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P487"/>
+  <dimension ref="A1:P499"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -25519,502 +25519,1102 @@
       </c>
     </row>
     <row r="478">
-      <c r="A478" t="inlineStr">
+      <c r="A478" s="10" t="inlineStr">
         <is>
           <t>Saw</t>
         </is>
       </c>
-      <c r="B478" t="inlineStr">
+      <c r="B478" s="10" t="inlineStr">
         <is>
           <t>card_477</t>
         </is>
       </c>
-      <c r="C478" t="inlineStr">
+      <c r="C478" s="10" t="inlineStr">
         <is>
           <t>James Wan</t>
         </is>
       </c>
-      <c r="D478" t="n">
+      <c r="D478" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E478" t="n">
+      <c r="E478" s="10" t="n">
         <v>3.69</v>
       </c>
-      <c r="F478" t="n">
+      <c r="F478" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I478" t="n">
+      <c r="I478" s="10" t="n">
         <v>104000000</v>
       </c>
-      <c r="J478" t="b">
-        <v>0</v>
-      </c>
-      <c r="K478" t="n">
+      <c r="J478" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K478" s="10" t="n">
         <v>1200000</v>
       </c>
-      <c r="L478" t="b">
-        <v>0</v>
-      </c>
-      <c r="M478" t="n">
+      <c r="L478" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M478" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="N478" t="n">
-        <v>0</v>
-      </c>
-      <c r="O478" t="n">
-        <v>0</v>
-      </c>
-      <c r="P478" t="b">
+      <c r="N478" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O478" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P478" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="479">
-      <c r="A479" t="inlineStr">
+      <c r="A479" s="10" t="inlineStr">
         <is>
           <t>Saw II</t>
         </is>
       </c>
-      <c r="B479" t="inlineStr">
+      <c r="B479" s="10" t="inlineStr">
         <is>
           <t>card_478</t>
         </is>
       </c>
-      <c r="C479" t="inlineStr">
+      <c r="C479" s="10" t="inlineStr">
         <is>
           <t>Darren Lynn Bousman</t>
         </is>
       </c>
-      <c r="D479" t="n">
+      <c r="D479" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E479" t="n">
+      <c r="E479" s="10" t="n">
         <v>3.29</v>
       </c>
-      <c r="F479" t="n">
+      <c r="F479" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I479" t="n">
+      <c r="I479" s="10" t="n">
         <v>152900000</v>
       </c>
-      <c r="J479" t="b">
-        <v>0</v>
-      </c>
-      <c r="K479" t="n">
+      <c r="J479" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K479" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L479" t="b">
-        <v>0</v>
-      </c>
-      <c r="M479" t="n">
+      <c r="L479" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M479" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N479" t="n">
-        <v>0</v>
-      </c>
-      <c r="O479" t="n">
-        <v>0</v>
-      </c>
-      <c r="P479" t="b">
+      <c r="N479" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O479" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P479" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="480">
-      <c r="A480" t="inlineStr">
+      <c r="A480" s="10" t="inlineStr">
         <is>
           <t>Saw III</t>
         </is>
       </c>
-      <c r="B480" t="inlineStr">
+      <c r="B480" s="10" t="inlineStr">
         <is>
           <t>card_479</t>
         </is>
       </c>
-      <c r="C480" t="inlineStr">
+      <c r="C480" s="10" t="inlineStr">
         <is>
           <t>Darren Lynn Bousman</t>
         </is>
       </c>
-      <c r="D480" t="n">
+      <c r="D480" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E480" t="n">
+      <c r="E480" s="10" t="n">
         <v>3.07</v>
       </c>
-      <c r="F480" t="n">
+      <c r="F480" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I480" t="n">
+      <c r="I480" s="10" t="n">
         <v>164900000</v>
       </c>
-      <c r="J480" t="b">
-        <v>0</v>
-      </c>
-      <c r="K480" t="n">
+      <c r="J480" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K480" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L480" t="b">
-        <v>0</v>
-      </c>
-      <c r="M480" t="n">
+      <c r="L480" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M480" s="10" t="n">
         <v>108</v>
       </c>
-      <c r="N480" t="n">
-        <v>0</v>
-      </c>
-      <c r="O480" t="n">
-        <v>0</v>
-      </c>
-      <c r="P480" t="b">
+      <c r="N480" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O480" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P480" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="481">
-      <c r="A481" t="inlineStr">
+      <c r="A481" s="10" t="inlineStr">
         <is>
           <t>Saw IV</t>
         </is>
       </c>
-      <c r="B481" t="inlineStr">
+      <c r="B481" s="10" t="inlineStr">
         <is>
           <t>card_480</t>
         </is>
       </c>
-      <c r="C481" t="inlineStr">
+      <c r="C481" s="10" t="inlineStr">
         <is>
           <t>Darren Lynn Bousman</t>
         </is>
       </c>
-      <c r="D481" t="n">
+      <c r="D481" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E481" t="n">
+      <c r="E481" s="10" t="n">
         <v>2.81</v>
       </c>
-      <c r="F481" t="n">
+      <c r="F481" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="I481" t="n">
+      <c r="I481" s="10" t="n">
         <v>139400000</v>
       </c>
-      <c r="J481" t="b">
-        <v>0</v>
-      </c>
-      <c r="K481" t="n">
+      <c r="J481" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K481" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L481" t="b">
-        <v>0</v>
-      </c>
-      <c r="M481" t="n">
+      <c r="L481" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M481" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="N481" t="n">
-        <v>0</v>
-      </c>
-      <c r="O481" t="n">
-        <v>0</v>
-      </c>
-      <c r="P481" t="b">
+      <c r="N481" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O481" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P481" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="482">
-      <c r="A482" t="inlineStr">
+      <c r="A482" s="10" t="inlineStr">
         <is>
           <t>Saw V</t>
         </is>
       </c>
-      <c r="B482" t="inlineStr">
+      <c r="B482" s="10" t="inlineStr">
         <is>
           <t>card_481</t>
         </is>
       </c>
-      <c r="C482" t="inlineStr">
+      <c r="C482" s="10" t="inlineStr">
         <is>
           <t>David Hackl</t>
         </is>
       </c>
-      <c r="D482" t="n">
+      <c r="D482" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E482" t="n">
+      <c r="E482" s="10" t="n">
         <v>2.76</v>
       </c>
-      <c r="F482" t="n">
+      <c r="F482" s="10" t="n">
         <v>55</v>
       </c>
-      <c r="I482" t="n">
+      <c r="I482" s="10" t="n">
         <v>118200000</v>
       </c>
-      <c r="J482" t="b">
-        <v>0</v>
-      </c>
-      <c r="K482" t="n">
+      <c r="J482" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K482" s="10" t="n">
         <v>10800000</v>
       </c>
-      <c r="L482" t="b">
-        <v>0</v>
-      </c>
-      <c r="M482" t="n">
+      <c r="L482" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M482" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="N482" t="n">
-        <v>0</v>
-      </c>
-      <c r="O482" t="n">
-        <v>0</v>
-      </c>
-      <c r="P482" t="b">
+      <c r="N482" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O482" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P482" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="483">
-      <c r="A483" t="inlineStr">
+      <c r="A483" s="10" t="inlineStr">
         <is>
           <t>Saw VI</t>
         </is>
       </c>
-      <c r="B483" t="inlineStr">
+      <c r="B483" s="10" t="inlineStr">
         <is>
           <t>card_482</t>
         </is>
       </c>
-      <c r="C483" t="inlineStr">
+      <c r="C483" s="10" t="inlineStr">
         <is>
           <t>Kevin Greutert</t>
         </is>
       </c>
-      <c r="D483" t="n">
+      <c r="D483" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E483" t="n">
+      <c r="E483" s="10" t="n">
         <v>2.97</v>
       </c>
-      <c r="F483" t="n">
+      <c r="F483" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="I483" t="n">
+      <c r="I483" s="10" t="n">
         <v>69800000</v>
       </c>
-      <c r="J483" t="b">
-        <v>0</v>
-      </c>
-      <c r="K483" t="n">
+      <c r="J483" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K483" s="10" t="n">
         <v>11000000</v>
       </c>
-      <c r="L483" t="b">
-        <v>0</v>
-      </c>
-      <c r="M483" t="n">
+      <c r="L483" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M483" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="N483" t="n">
-        <v>0</v>
-      </c>
-      <c r="O483" t="n">
-        <v>0</v>
-      </c>
-      <c r="P483" t="b">
+      <c r="N483" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O483" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P483" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="484">
-      <c r="A484" t="inlineStr">
+      <c r="A484" s="10" t="inlineStr">
         <is>
           <t>Saw 3D</t>
         </is>
       </c>
-      <c r="B484" t="inlineStr">
+      <c r="B484" s="10" t="inlineStr">
         <is>
           <t>card_483</t>
         </is>
       </c>
-      <c r="C484" t="inlineStr">
+      <c r="C484" s="10" t="inlineStr">
         <is>
           <t>Kevin Greutert</t>
         </is>
       </c>
-      <c r="D484" t="n">
+      <c r="D484" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E484" t="n">
+      <c r="E484" s="10" t="n">
         <v>2.43</v>
       </c>
-      <c r="F484" t="n">
+      <c r="F484" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="I484" t="n">
+      <c r="I484" s="10" t="n">
         <v>136200000</v>
       </c>
-      <c r="J484" t="b">
-        <v>0</v>
-      </c>
-      <c r="K484" t="n">
+      <c r="J484" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K484" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="L484" t="b">
-        <v>0</v>
-      </c>
-      <c r="M484" t="n">
+      <c r="L484" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M484" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="N484" t="n">
-        <v>0</v>
-      </c>
-      <c r="O484" t="n">
-        <v>0</v>
-      </c>
-      <c r="P484" t="b">
+      <c r="N484" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O484" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P484" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="485">
-      <c r="A485" t="inlineStr">
+      <c r="A485" s="10" t="inlineStr">
         <is>
           <t>Jigsaw</t>
         </is>
       </c>
-      <c r="B485" t="inlineStr">
+      <c r="B485" s="10" t="inlineStr">
         <is>
           <t>card_484</t>
         </is>
       </c>
-      <c r="C485" t="inlineStr">
+      <c r="C485" s="10" t="inlineStr">
         <is>
           <t>Michael Spierig and Peter Spierig</t>
         </is>
       </c>
-      <c r="D485" t="n">
+      <c r="D485" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E485" t="n">
+      <c r="E485" s="10" t="n">
         <v>2.96</v>
       </c>
-      <c r="F485" t="n">
+      <c r="F485" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="I485" t="n">
+      <c r="I485" s="10" t="n">
         <v>104200000</v>
       </c>
-      <c r="J485" t="b">
-        <v>0</v>
-      </c>
-      <c r="K485" t="n">
+      <c r="J485" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K485" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L485" t="b">
-        <v>0</v>
-      </c>
-      <c r="M485" t="n">
+      <c r="L485" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M485" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="N485" t="n">
-        <v>0</v>
-      </c>
-      <c r="O485" t="n">
-        <v>0</v>
-      </c>
-      <c r="P485" t="b">
+      <c r="N485" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O485" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P485" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="486">
-      <c r="A486" t="inlineStr">
+      <c r="A486" s="10" t="inlineStr">
         <is>
           <t>Spiral: From the Book of Saw</t>
         </is>
       </c>
-      <c r="B486" t="inlineStr">
+      <c r="B486" s="10" t="inlineStr">
         <is>
           <t>card_485</t>
         </is>
       </c>
-      <c r="C486" t="inlineStr">
+      <c r="C486" s="10" t="inlineStr">
         <is>
           <t>Darren Lynn Bousman</t>
         </is>
       </c>
-      <c r="D486" t="n">
+      <c r="D486" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E486" t="n">
+      <c r="E486" s="10" t="n">
         <v>2.05</v>
       </c>
-      <c r="F486" t="n">
+      <c r="F486" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I486" t="n">
+      <c r="I486" s="10" t="n">
         <v>40600000</v>
       </c>
-      <c r="J486" t="b">
-        <v>0</v>
-      </c>
-      <c r="K486" t="n">
+      <c r="J486" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K486" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L486" t="b">
-        <v>0</v>
-      </c>
-      <c r="M486" t="n">
+      <c r="L486" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M486" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N486" t="n">
-        <v>0</v>
-      </c>
-      <c r="O486" t="n">
-        <v>0</v>
-      </c>
-      <c r="P486" t="b">
+      <c r="N486" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O486" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P486" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="487">
-      <c r="A487" t="inlineStr">
+      <c r="A487" s="10" t="inlineStr">
         <is>
           <t>Saw X</t>
         </is>
       </c>
-      <c r="B487" t="inlineStr">
+      <c r="B487" s="10" t="inlineStr">
         <is>
           <t>card_486</t>
         </is>
       </c>
-      <c r="C487" t="inlineStr">
+      <c r="C487" s="10" t="inlineStr">
         <is>
           <t>Kevin Greutert</t>
         </is>
       </c>
-      <c r="D487" t="n">
+      <c r="D487" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E487" t="n">
+      <c r="E487" s="10" t="n">
         <v>3.26</v>
       </c>
-      <c r="F487" t="n">
+      <c r="F487" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I487" t="n">
+      <c r="I487" s="10" t="n">
         <v>125300000</v>
       </c>
-      <c r="J487" t="b">
-        <v>0</v>
-      </c>
-      <c r="K487" t="n">
+      <c r="J487" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K487" s="10" t="n">
         <v>13000000</v>
       </c>
-      <c r="L487" t="b">
-        <v>0</v>
-      </c>
-      <c r="M487" t="n">
+      <c r="L487" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M487" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N487" t="n">
-        <v>0</v>
-      </c>
-      <c r="O487" t="n">
-        <v>0</v>
-      </c>
-      <c r="P487" t="b">
+      <c r="N487" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O487" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P487" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Halloween II (1981)</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>card_487</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Rick Rosenthal</t>
+        </is>
+      </c>
+      <c r="D488" t="n">
+        <v>1981</v>
+      </c>
+      <c r="E488" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F488" t="n">
+        <v>73</v>
+      </c>
+      <c r="I488" t="n">
+        <v>25500000</v>
+      </c>
+      <c r="J488" t="b">
+        <v>0</v>
+      </c>
+      <c r="K488" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="L488" t="b">
+        <v>0</v>
+      </c>
+      <c r="M488" t="n">
+        <v>92</v>
+      </c>
+      <c r="N488" t="n">
+        <v>0</v>
+      </c>
+      <c r="O488" t="n">
+        <v>0</v>
+      </c>
+      <c r="P488" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Halloween III: Season of the Witch</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>card_488</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Tommy Lee Wallace</t>
+        </is>
+      </c>
+      <c r="D489" t="n">
+        <v>1982</v>
+      </c>
+      <c r="E489" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="F489" t="n">
+        <v>62</v>
+      </c>
+      <c r="I489" t="n">
+        <v>14400000</v>
+      </c>
+      <c r="J489" t="b">
+        <v>1</v>
+      </c>
+      <c r="K489" t="n">
+        <v>4600000</v>
+      </c>
+      <c r="L489" t="b">
+        <v>0</v>
+      </c>
+      <c r="M489" t="n">
+        <v>99</v>
+      </c>
+      <c r="N489" t="n">
+        <v>0</v>
+      </c>
+      <c r="O489" t="n">
+        <v>0</v>
+      </c>
+      <c r="P489" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Halloween 4: The Return of Michael Myers</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>card_489</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>Dwight H. Little</t>
+        </is>
+      </c>
+      <c r="D490" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E490" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="F490" t="n">
+        <v>64</v>
+      </c>
+      <c r="I490" t="n">
+        <v>17800000</v>
+      </c>
+      <c r="J490" t="b">
+        <v>0</v>
+      </c>
+      <c r="K490" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L490" t="b">
+        <v>0</v>
+      </c>
+      <c r="M490" t="n">
+        <v>88</v>
+      </c>
+      <c r="N490" t="n">
+        <v>0</v>
+      </c>
+      <c r="O490" t="n">
+        <v>0</v>
+      </c>
+      <c r="P490" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Halloween 5: The Revenge of Michael Myers</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>card_490</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Dominique Othenin-Girard</t>
+        </is>
+      </c>
+      <c r="D491" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E491" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F491" t="n">
+        <v>47</v>
+      </c>
+      <c r="I491" t="n">
+        <v>11600000</v>
+      </c>
+      <c r="J491" t="b">
+        <v>0</v>
+      </c>
+      <c r="K491" t="n">
+        <v>5500000</v>
+      </c>
+      <c r="L491" t="b">
+        <v>0</v>
+      </c>
+      <c r="M491" t="n">
+        <v>96</v>
+      </c>
+      <c r="N491" t="n">
+        <v>0</v>
+      </c>
+      <c r="O491" t="n">
+        <v>0</v>
+      </c>
+      <c r="P491" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Halloween: The Curse of Michael Myers</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>card_491</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Joe Chappelle</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E492" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="F492" t="n">
+        <v>45</v>
+      </c>
+      <c r="I492" t="n">
+        <v>15100000</v>
+      </c>
+      <c r="J492" t="b">
+        <v>1</v>
+      </c>
+      <c r="K492" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L492" t="b">
+        <v>0</v>
+      </c>
+      <c r="M492" t="n">
+        <v>88</v>
+      </c>
+      <c r="N492" t="n">
+        <v>0</v>
+      </c>
+      <c r="O492" t="n">
+        <v>0</v>
+      </c>
+      <c r="P492" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Halloween H20: 20 Years Later</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>card_492</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Steve Miner</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E493" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="F493" t="n">
+        <v>68</v>
+      </c>
+      <c r="I493" t="n">
+        <v>75000000</v>
+      </c>
+      <c r="J493" t="b">
+        <v>0</v>
+      </c>
+      <c r="K493" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="L493" t="b">
+        <v>0</v>
+      </c>
+      <c r="M493" t="n">
+        <v>86</v>
+      </c>
+      <c r="N493" t="n">
+        <v>0</v>
+      </c>
+      <c r="O493" t="n">
+        <v>0</v>
+      </c>
+      <c r="P493" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Halloween: Resurrection</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>card_493</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Rick Rosenthal</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E494" t="n">
+        <v>1.66</v>
+      </c>
+      <c r="F494" t="n">
+        <v>35</v>
+      </c>
+      <c r="I494" t="n">
+        <v>37600000</v>
+      </c>
+      <c r="J494" t="b">
+        <v>0</v>
+      </c>
+      <c r="K494" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L494" t="b">
+        <v>0</v>
+      </c>
+      <c r="M494" t="n">
+        <v>90</v>
+      </c>
+      <c r="N494" t="n">
+        <v>0</v>
+      </c>
+      <c r="O494" t="n">
+        <v>0</v>
+      </c>
+      <c r="P494" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Halloween (2007)</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>card_494</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Rob Zombie</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E495" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="F495" t="n">
+        <v>54</v>
+      </c>
+      <c r="I495" t="n">
+        <v>80400000</v>
+      </c>
+      <c r="J495" t="b">
+        <v>0</v>
+      </c>
+      <c r="K495" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L495" t="b">
+        <v>0</v>
+      </c>
+      <c r="M495" t="n">
+        <v>110</v>
+      </c>
+      <c r="N495" t="n">
+        <v>0</v>
+      </c>
+      <c r="O495" t="n">
+        <v>0</v>
+      </c>
+      <c r="P495" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Halloween II (2009)</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>card_495</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Rob Zombie</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E496" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="F496" t="n">
+        <v>40</v>
+      </c>
+      <c r="I496" t="n">
+        <v>39400000</v>
+      </c>
+      <c r="J496" t="b">
+        <v>0</v>
+      </c>
+      <c r="K496" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L496" t="b">
+        <v>0</v>
+      </c>
+      <c r="M496" t="n">
+        <v>105</v>
+      </c>
+      <c r="N496" t="n">
+        <v>0</v>
+      </c>
+      <c r="O496" t="n">
+        <v>0</v>
+      </c>
+      <c r="P496" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Halloween (2018)</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>card_496</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>David Gordon Green</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E497" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="F497" t="n">
+        <v>70</v>
+      </c>
+      <c r="I497" t="n">
+        <v>259900000</v>
+      </c>
+      <c r="J497" t="b">
+        <v>0</v>
+      </c>
+      <c r="K497" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L497" t="b">
+        <v>0</v>
+      </c>
+      <c r="M497" t="n">
+        <v>106</v>
+      </c>
+      <c r="N497" t="n">
+        <v>0</v>
+      </c>
+      <c r="O497" t="n">
+        <v>0</v>
+      </c>
+      <c r="P497" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Halloween Kills</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>card_497</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>David Gordon Green</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E498" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="F498" t="n">
+        <v>57</v>
+      </c>
+      <c r="I498" t="n">
+        <v>133400000</v>
+      </c>
+      <c r="J498" t="b">
+        <v>0</v>
+      </c>
+      <c r="K498" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L498" t="b">
+        <v>0</v>
+      </c>
+      <c r="M498" t="n">
+        <v>105</v>
+      </c>
+      <c r="N498" t="n">
+        <v>0</v>
+      </c>
+      <c r="O498" t="n">
+        <v>0</v>
+      </c>
+      <c r="P498" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Halloween Ends</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>card_498</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>David Gordon Green</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E499" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="F499" t="n">
+        <v>45</v>
+      </c>
+      <c r="I499" t="n">
+        <v>105400000</v>
+      </c>
+      <c r="J499" t="b">
+        <v>0</v>
+      </c>
+      <c r="K499" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="L499" t="b">
+        <v>0</v>
+      </c>
+      <c r="M499" t="n">
+        <v>111</v>
+      </c>
+      <c r="N499" t="n">
+        <v>0</v>
+      </c>
+      <c r="O499" t="n">
+        <v>0</v>
+      </c>
+      <c r="P499" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Star Trek films (card_499-510)
The Motion Picture, III-VI, Generations, First Contact, Insurrection,
Nemesis, the 2009 reboot, Into Darkness, Beyond.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P499"/>
+  <dimension ref="A1:P511"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -26019,602 +26019,1202 @@
       </c>
     </row>
     <row r="488">
-      <c r="A488" t="inlineStr">
+      <c r="A488" s="10" t="inlineStr">
         <is>
           <t>Halloween II (1981)</t>
         </is>
       </c>
-      <c r="B488" t="inlineStr">
+      <c r="B488" s="10" t="inlineStr">
         <is>
           <t>card_487</t>
         </is>
       </c>
-      <c r="C488" t="inlineStr">
+      <c r="C488" s="10" t="inlineStr">
         <is>
           <t>Rick Rosenthal</t>
         </is>
       </c>
-      <c r="D488" t="n">
+      <c r="D488" s="10" t="n">
         <v>1981</v>
       </c>
-      <c r="E488" t="n">
+      <c r="E488" s="10" t="n">
         <v>3.2</v>
       </c>
-      <c r="F488" t="n">
+      <c r="F488" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I488" t="n">
+      <c r="I488" s="10" t="n">
         <v>25500000</v>
       </c>
-      <c r="J488" t="b">
-        <v>0</v>
-      </c>
-      <c r="K488" t="n">
+      <c r="J488" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K488" s="10" t="n">
         <v>2500000</v>
       </c>
-      <c r="L488" t="b">
-        <v>0</v>
-      </c>
-      <c r="M488" t="n">
+      <c r="L488" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M488" s="10" t="n">
         <v>92</v>
       </c>
-      <c r="N488" t="n">
-        <v>0</v>
-      </c>
-      <c r="O488" t="n">
-        <v>0</v>
-      </c>
-      <c r="P488" t="b">
+      <c r="N488" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O488" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P488" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="489">
-      <c r="A489" t="inlineStr">
+      <c r="A489" s="10" t="inlineStr">
         <is>
           <t>Halloween III: Season of the Witch</t>
         </is>
       </c>
-      <c r="B489" t="inlineStr">
+      <c r="B489" s="10" t="inlineStr">
         <is>
           <t>card_488</t>
         </is>
       </c>
-      <c r="C489" t="inlineStr">
+      <c r="C489" s="10" t="inlineStr">
         <is>
           <t>Tommy Lee Wallace</t>
         </is>
       </c>
-      <c r="D489" t="n">
+      <c r="D489" s="10" t="n">
         <v>1982</v>
       </c>
-      <c r="E489" t="n">
+      <c r="E489" s="10" t="n">
         <v>2.82</v>
       </c>
-      <c r="F489" t="n">
+      <c r="F489" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I489" t="n">
+      <c r="I489" s="10" t="n">
         <v>14400000</v>
       </c>
-      <c r="J489" t="b">
+      <c r="J489" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K489" t="n">
+      <c r="K489" s="10" t="n">
         <v>4600000</v>
       </c>
-      <c r="L489" t="b">
-        <v>0</v>
-      </c>
-      <c r="M489" t="n">
+      <c r="L489" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M489" s="10" t="n">
         <v>99</v>
       </c>
-      <c r="N489" t="n">
-        <v>0</v>
-      </c>
-      <c r="O489" t="n">
-        <v>0</v>
-      </c>
-      <c r="P489" t="b">
+      <c r="N489" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O489" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P489" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="490">
-      <c r="A490" t="inlineStr">
+      <c r="A490" s="10" t="inlineStr">
         <is>
           <t>Halloween 4: The Return of Michael Myers</t>
         </is>
       </c>
-      <c r="B490" t="inlineStr">
+      <c r="B490" s="10" t="inlineStr">
         <is>
           <t>card_489</t>
         </is>
       </c>
-      <c r="C490" t="inlineStr">
+      <c r="C490" s="10" t="inlineStr">
         <is>
           <t>Dwight H. Little</t>
         </is>
       </c>
-      <c r="D490" t="n">
+      <c r="D490" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E490" t="n">
+      <c r="E490" s="10" t="n">
         <v>2.81</v>
       </c>
-      <c r="F490" t="n">
+      <c r="F490" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="I490" t="n">
+      <c r="I490" s="10" t="n">
         <v>17800000</v>
       </c>
-      <c r="J490" t="b">
-        <v>0</v>
-      </c>
-      <c r="K490" t="n">
+      <c r="J490" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K490" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L490" t="b">
-        <v>0</v>
-      </c>
-      <c r="M490" t="n">
+      <c r="L490" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M490" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N490" t="n">
-        <v>0</v>
-      </c>
-      <c r="O490" t="n">
-        <v>0</v>
-      </c>
-      <c r="P490" t="b">
+      <c r="N490" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O490" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P490" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="491">
-      <c r="A491" t="inlineStr">
+      <c r="A491" s="10" t="inlineStr">
         <is>
           <t>Halloween 5: The Revenge of Michael Myers</t>
         </is>
       </c>
-      <c r="B491" t="inlineStr">
+      <c r="B491" s="10" t="inlineStr">
         <is>
           <t>card_490</t>
         </is>
       </c>
-      <c r="C491" t="inlineStr">
+      <c r="C491" s="10" t="inlineStr">
         <is>
           <t>Dominique Othenin-Girard</t>
         </is>
       </c>
-      <c r="D491" t="n">
+      <c r="D491" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E491" t="n">
+      <c r="E491" s="10" t="n">
         <v>2.16</v>
       </c>
-      <c r="F491" t="n">
+      <c r="F491" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="I491" t="n">
+      <c r="I491" s="10" t="n">
         <v>11600000</v>
       </c>
-      <c r="J491" t="b">
-        <v>0</v>
-      </c>
-      <c r="K491" t="n">
+      <c r="J491" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K491" s="10" t="n">
         <v>5500000</v>
       </c>
-      <c r="L491" t="b">
-        <v>0</v>
-      </c>
-      <c r="M491" t="n">
+      <c r="L491" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M491" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N491" t="n">
-        <v>0</v>
-      </c>
-      <c r="O491" t="n">
-        <v>0</v>
-      </c>
-      <c r="P491" t="b">
+      <c r="N491" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O491" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P491" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="492">
-      <c r="A492" t="inlineStr">
+      <c r="A492" s="10" t="inlineStr">
         <is>
           <t>Halloween: The Curse of Michael Myers</t>
         </is>
       </c>
-      <c r="B492" t="inlineStr">
+      <c r="B492" s="10" t="inlineStr">
         <is>
           <t>card_491</t>
         </is>
       </c>
-      <c r="C492" t="inlineStr">
+      <c r="C492" s="10" t="inlineStr">
         <is>
           <t>Joe Chappelle</t>
         </is>
       </c>
-      <c r="D492" t="n">
+      <c r="D492" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E492" t="n">
+      <c r="E492" s="10" t="n">
         <v>2.05</v>
       </c>
-      <c r="F492" t="n">
+      <c r="F492" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="I492" t="n">
+      <c r="I492" s="10" t="n">
         <v>15100000</v>
       </c>
-      <c r="J492" t="b">
+      <c r="J492" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K492" t="n">
+      <c r="K492" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L492" t="b">
-        <v>0</v>
-      </c>
-      <c r="M492" t="n">
+      <c r="L492" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M492" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N492" t="n">
-        <v>0</v>
-      </c>
-      <c r="O492" t="n">
-        <v>0</v>
-      </c>
-      <c r="P492" t="b">
+      <c r="N492" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O492" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P492" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="493">
-      <c r="A493" t="inlineStr">
+      <c r="A493" s="10" t="inlineStr">
         <is>
           <t>Halloween H20: 20 Years Later</t>
         </is>
       </c>
-      <c r="B493" t="inlineStr">
+      <c r="B493" s="10" t="inlineStr">
         <is>
           <t>card_492</t>
         </is>
       </c>
-      <c r="C493" t="inlineStr">
+      <c r="C493" s="10" t="inlineStr">
         <is>
           <t>Steve Miner</t>
         </is>
       </c>
-      <c r="D493" t="n">
+      <c r="D493" s="10" t="n">
         <v>1998</v>
       </c>
-      <c r="E493" t="n">
+      <c r="E493" s="10" t="n">
         <v>2.85</v>
       </c>
-      <c r="F493" t="n">
+      <c r="F493" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I493" t="n">
+      <c r="I493" s="10" t="n">
         <v>75000000</v>
       </c>
-      <c r="J493" t="b">
-        <v>0</v>
-      </c>
-      <c r="K493" t="n">
+      <c r="J493" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K493" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="L493" t="b">
-        <v>0</v>
-      </c>
-      <c r="M493" t="n">
+      <c r="L493" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M493" s="10" t="n">
         <v>86</v>
       </c>
-      <c r="N493" t="n">
-        <v>0</v>
-      </c>
-      <c r="O493" t="n">
-        <v>0</v>
-      </c>
-      <c r="P493" t="b">
+      <c r="N493" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O493" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P493" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="494">
-      <c r="A494" t="inlineStr">
+      <c r="A494" s="10" t="inlineStr">
         <is>
           <t>Halloween: Resurrection</t>
         </is>
       </c>
-      <c r="B494" t="inlineStr">
+      <c r="B494" s="10" t="inlineStr">
         <is>
           <t>card_493</t>
         </is>
       </c>
-      <c r="C494" t="inlineStr">
+      <c r="C494" s="10" t="inlineStr">
         <is>
           <t>Rick Rosenthal</t>
         </is>
       </c>
-      <c r="D494" t="n">
+      <c r="D494" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E494" t="n">
+      <c r="E494" s="10" t="n">
         <v>1.66</v>
       </c>
-      <c r="F494" t="n">
+      <c r="F494" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I494" t="n">
+      <c r="I494" s="10" t="n">
         <v>37600000</v>
       </c>
-      <c r="J494" t="b">
-        <v>0</v>
-      </c>
-      <c r="K494" t="n">
+      <c r="J494" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K494" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L494" t="b">
-        <v>0</v>
-      </c>
-      <c r="M494" t="n">
+      <c r="L494" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M494" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="N494" t="n">
-        <v>0</v>
-      </c>
-      <c r="O494" t="n">
-        <v>0</v>
-      </c>
-      <c r="P494" t="b">
+      <c r="N494" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O494" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P494" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="495">
-      <c r="A495" t="inlineStr">
+      <c r="A495" s="10" t="inlineStr">
         <is>
           <t>Halloween (2007)</t>
         </is>
       </c>
-      <c r="B495" t="inlineStr">
+      <c r="B495" s="10" t="inlineStr">
         <is>
           <t>card_494</t>
         </is>
       </c>
-      <c r="C495" t="inlineStr">
+      <c r="C495" s="10" t="inlineStr">
         <is>
           <t>Rob Zombie</t>
         </is>
       </c>
-      <c r="D495" t="n">
+      <c r="D495" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E495" t="n">
+      <c r="E495" s="10" t="n">
         <v>2.81</v>
       </c>
-      <c r="F495" t="n">
+      <c r="F495" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="I495" t="n">
+      <c r="I495" s="10" t="n">
         <v>80400000</v>
       </c>
-      <c r="J495" t="b">
-        <v>0</v>
-      </c>
-      <c r="K495" t="n">
+      <c r="J495" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K495" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L495" t="b">
-        <v>0</v>
-      </c>
-      <c r="M495" t="n">
+      <c r="L495" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M495" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N495" t="n">
-        <v>0</v>
-      </c>
-      <c r="O495" t="n">
-        <v>0</v>
-      </c>
-      <c r="P495" t="b">
+      <c r="N495" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O495" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P495" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="496">
-      <c r="A496" t="inlineStr">
+      <c r="A496" s="10" t="inlineStr">
         <is>
           <t>Halloween II (2009)</t>
         </is>
       </c>
-      <c r="B496" t="inlineStr">
+      <c r="B496" s="10" t="inlineStr">
         <is>
           <t>card_495</t>
         </is>
       </c>
-      <c r="C496" t="inlineStr">
+      <c r="C496" s="10" t="inlineStr">
         <is>
           <t>Rob Zombie</t>
         </is>
       </c>
-      <c r="D496" t="n">
+      <c r="D496" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E496" t="n">
+      <c r="E496" s="10" t="n">
         <v>2.35</v>
       </c>
-      <c r="F496" t="n">
+      <c r="F496" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="I496" t="n">
+      <c r="I496" s="10" t="n">
         <v>39400000</v>
       </c>
-      <c r="J496" t="b">
-        <v>0</v>
-      </c>
-      <c r="K496" t="n">
+      <c r="J496" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K496" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L496" t="b">
-        <v>0</v>
-      </c>
-      <c r="M496" t="n">
+      <c r="L496" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M496" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="N496" t="n">
-        <v>0</v>
-      </c>
-      <c r="O496" t="n">
-        <v>0</v>
-      </c>
-      <c r="P496" t="b">
+      <c r="N496" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O496" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P496" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="497">
-      <c r="A497" t="inlineStr">
+      <c r="A497" s="10" t="inlineStr">
         <is>
           <t>Halloween (2018)</t>
         </is>
       </c>
-      <c r="B497" t="inlineStr">
+      <c r="B497" s="10" t="inlineStr">
         <is>
           <t>card_496</t>
         </is>
       </c>
-      <c r="C497" t="inlineStr">
+      <c r="C497" s="10" t="inlineStr">
         <is>
           <t>David Gordon Green</t>
         </is>
       </c>
-      <c r="D497" t="n">
+      <c r="D497" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E497" t="n">
+      <c r="E497" s="10" t="n">
         <v>3.22</v>
       </c>
-      <c r="F497" t="n">
+      <c r="F497" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I497" t="n">
+      <c r="I497" s="10" t="n">
         <v>259900000</v>
       </c>
-      <c r="J497" t="b">
-        <v>0</v>
-      </c>
-      <c r="K497" t="n">
+      <c r="J497" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K497" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L497" t="b">
-        <v>0</v>
-      </c>
-      <c r="M497" t="n">
+      <c r="L497" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M497" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="N497" t="n">
-        <v>0</v>
-      </c>
-      <c r="O497" t="n">
-        <v>0</v>
-      </c>
-      <c r="P497" t="b">
+      <c r="N497" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O497" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P497" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="498">
-      <c r="A498" t="inlineStr">
+      <c r="A498" s="10" t="inlineStr">
         <is>
           <t>Halloween Kills</t>
         </is>
       </c>
-      <c r="B498" t="inlineStr">
+      <c r="B498" s="10" t="inlineStr">
         <is>
           <t>card_497</t>
         </is>
       </c>
-      <c r="C498" t="inlineStr">
+      <c r="C498" s="10" t="inlineStr">
         <is>
           <t>David Gordon Green</t>
         </is>
       </c>
-      <c r="D498" t="n">
+      <c r="D498" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E498" t="n">
+      <c r="E498" s="10" t="n">
         <v>2.56</v>
       </c>
-      <c r="F498" t="n">
+      <c r="F498" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I498" t="n">
+      <c r="I498" s="10" t="n">
         <v>133400000</v>
       </c>
-      <c r="J498" t="b">
-        <v>0</v>
-      </c>
-      <c r="K498" t="n">
+      <c r="J498" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K498" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L498" t="b">
-        <v>0</v>
-      </c>
-      <c r="M498" t="n">
+      <c r="L498" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M498" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="N498" t="n">
-        <v>0</v>
-      </c>
-      <c r="O498" t="n">
-        <v>0</v>
-      </c>
-      <c r="P498" t="b">
+      <c r="N498" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O498" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P498" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="499">
-      <c r="A499" t="inlineStr">
+      <c r="A499" s="10" t="inlineStr">
         <is>
           <t>Halloween Ends</t>
         </is>
       </c>
-      <c r="B499" t="inlineStr">
+      <c r="B499" s="10" t="inlineStr">
         <is>
           <t>card_498</t>
         </is>
       </c>
-      <c r="C499" t="inlineStr">
+      <c r="C499" s="10" t="inlineStr">
         <is>
           <t>David Gordon Green</t>
         </is>
       </c>
-      <c r="D499" t="n">
+      <c r="D499" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E499" t="n">
+      <c r="E499" s="10" t="n">
         <v>2.16</v>
       </c>
-      <c r="F499" t="n">
+      <c r="F499" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="I499" t="n">
+      <c r="I499" s="10" t="n">
         <v>105400000</v>
       </c>
-      <c r="J499" t="b">
-        <v>0</v>
-      </c>
-      <c r="K499" t="n">
+      <c r="J499" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K499" s="10" t="n">
         <v>33000000</v>
       </c>
-      <c r="L499" t="b">
-        <v>0</v>
-      </c>
-      <c r="M499" t="n">
+      <c r="L499" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M499" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N499" t="n">
-        <v>0</v>
-      </c>
-      <c r="O499" t="n">
-        <v>0</v>
-      </c>
-      <c r="P499" t="b">
+      <c r="N499" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O499" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P499" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Star Trek: The Motion Picture</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>card_499</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Robert Wise</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>1979</v>
+      </c>
+      <c r="E500" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="F500" t="n">
+        <v>67</v>
+      </c>
+      <c r="I500" t="n">
+        <v>139000000</v>
+      </c>
+      <c r="J500" t="b">
+        <v>0</v>
+      </c>
+      <c r="K500" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="L500" t="b">
+        <v>0</v>
+      </c>
+      <c r="M500" t="n">
+        <v>132</v>
+      </c>
+      <c r="N500" t="n">
+        <v>0</v>
+      </c>
+      <c r="O500" t="n">
+        <v>2</v>
+      </c>
+      <c r="P500" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Star Trek III: The Search for Spock</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>card_500</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Leonard Nimoy</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E501" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="F501" t="n">
+        <v>68</v>
+      </c>
+      <c r="I501" t="n">
+        <v>87000000</v>
+      </c>
+      <c r="J501" t="b">
+        <v>0</v>
+      </c>
+      <c r="K501" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="L501" t="b">
+        <v>0</v>
+      </c>
+      <c r="M501" t="n">
+        <v>105</v>
+      </c>
+      <c r="N501" t="n">
+        <v>0</v>
+      </c>
+      <c r="O501" t="n">
+        <v>0</v>
+      </c>
+      <c r="P501" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Star Trek IV: The Voyage Home</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>card_501</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Leonard Nimoy</t>
+        </is>
+      </c>
+      <c r="D502" t="n">
+        <v>1986</v>
+      </c>
+      <c r="E502" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="F502" t="n">
+        <v>80</v>
+      </c>
+      <c r="I502" t="n">
+        <v>133000000</v>
+      </c>
+      <c r="J502" t="b">
+        <v>0</v>
+      </c>
+      <c r="K502" t="n">
+        <v>21000000</v>
+      </c>
+      <c r="L502" t="b">
+        <v>0</v>
+      </c>
+      <c r="M502" t="n">
+        <v>122</v>
+      </c>
+      <c r="N502" t="n">
+        <v>0</v>
+      </c>
+      <c r="O502" t="n">
+        <v>0</v>
+      </c>
+      <c r="P502" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Star Trek V: The Final Frontier</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>card_502</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>William Shatner</t>
+        </is>
+      </c>
+      <c r="D503" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E503" t="n">
+        <v>2.61</v>
+      </c>
+      <c r="F503" t="n">
+        <v>56</v>
+      </c>
+      <c r="I503" t="n">
+        <v>63000000</v>
+      </c>
+      <c r="J503" t="b">
+        <v>0</v>
+      </c>
+      <c r="K503" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="L503" t="b">
+        <v>0</v>
+      </c>
+      <c r="M503" t="n">
+        <v>106</v>
+      </c>
+      <c r="N503" t="n">
+        <v>0</v>
+      </c>
+      <c r="O503" t="n">
+        <v>0</v>
+      </c>
+      <c r="P503" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Star Trek VI: The Undiscovered Country</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>card_503</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Nicholas Meyer</t>
+        </is>
+      </c>
+      <c r="D504" t="n">
+        <v>1991</v>
+      </c>
+      <c r="E504" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F504" t="n">
+        <v>83</v>
+      </c>
+      <c r="I504" t="n">
+        <v>96800000</v>
+      </c>
+      <c r="J504" t="b">
+        <v>0</v>
+      </c>
+      <c r="K504" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L504" t="b">
+        <v>0</v>
+      </c>
+      <c r="M504" t="n">
+        <v>110</v>
+      </c>
+      <c r="N504" t="n">
+        <v>0</v>
+      </c>
+      <c r="O504" t="n">
+        <v>0</v>
+      </c>
+      <c r="P504" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Star Trek Generations</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>card_504</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>David Carson</t>
+        </is>
+      </c>
+      <c r="D505" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E505" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="F505" t="n">
+        <v>65</v>
+      </c>
+      <c r="I505" t="n">
+        <v>118000000</v>
+      </c>
+      <c r="J505" t="b">
+        <v>0</v>
+      </c>
+      <c r="K505" t="n">
+        <v>35000000</v>
+      </c>
+      <c r="L505" t="b">
+        <v>0</v>
+      </c>
+      <c r="M505" t="n">
+        <v>118</v>
+      </c>
+      <c r="N505" t="n">
+        <v>0</v>
+      </c>
+      <c r="O505" t="n">
+        <v>0</v>
+      </c>
+      <c r="P505" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Star Trek: First Contact</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>card_505</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Jonathan Frakes</t>
+        </is>
+      </c>
+      <c r="D506" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E506" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F506" t="n">
+        <v>81</v>
+      </c>
+      <c r="I506" t="n">
+        <v>146000000</v>
+      </c>
+      <c r="J506" t="b">
+        <v>0</v>
+      </c>
+      <c r="K506" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="L506" t="b">
+        <v>0</v>
+      </c>
+      <c r="M506" t="n">
+        <v>111</v>
+      </c>
+      <c r="N506" t="n">
+        <v>0</v>
+      </c>
+      <c r="O506" t="n">
+        <v>0</v>
+      </c>
+      <c r="P506" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Star Trek: Insurrection</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>card_506</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Jonathan Frakes</t>
+        </is>
+      </c>
+      <c r="D507" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E507" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="F507" t="n">
+        <v>60</v>
+      </c>
+      <c r="I507" t="n">
+        <v>118000000</v>
+      </c>
+      <c r="J507" t="b">
+        <v>0</v>
+      </c>
+      <c r="K507" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="L507" t="b">
+        <v>0</v>
+      </c>
+      <c r="M507" t="n">
+        <v>103</v>
+      </c>
+      <c r="N507" t="n">
+        <v>0</v>
+      </c>
+      <c r="O507" t="n">
+        <v>0</v>
+      </c>
+      <c r="P507" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Star Trek: Nemesis</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>card_507</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Stuart Baird</t>
+        </is>
+      </c>
+      <c r="D508" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E508" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="F508" t="n">
+        <v>57</v>
+      </c>
+      <c r="I508" t="n">
+        <v>67300000</v>
+      </c>
+      <c r="J508" t="b">
+        <v>0</v>
+      </c>
+      <c r="K508" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="L508" t="b">
+        <v>0</v>
+      </c>
+      <c r="M508" t="n">
+        <v>117</v>
+      </c>
+      <c r="N508" t="n">
+        <v>0</v>
+      </c>
+      <c r="O508" t="n">
+        <v>0</v>
+      </c>
+      <c r="P508" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Star Trek</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>card_508</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>J.J. Abrams</t>
+        </is>
+      </c>
+      <c r="D509" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E509" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F509" t="n">
+        <v>77</v>
+      </c>
+      <c r="I509" t="n">
+        <v>385700000</v>
+      </c>
+      <c r="J509" t="b">
+        <v>0</v>
+      </c>
+      <c r="K509" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L509" t="b">
+        <v>0</v>
+      </c>
+      <c r="M509" t="n">
+        <v>127</v>
+      </c>
+      <c r="N509" t="n">
+        <v>1</v>
+      </c>
+      <c r="O509" t="n">
+        <v>0</v>
+      </c>
+      <c r="P509" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Star Trek Into Darkness</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>card_509</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>J.J. Abrams</t>
+        </is>
+      </c>
+      <c r="D510" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E510" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F510" t="n">
+        <v>76</v>
+      </c>
+      <c r="I510" t="n">
+        <v>467400000</v>
+      </c>
+      <c r="J510" t="b">
+        <v>0</v>
+      </c>
+      <c r="K510" t="n">
+        <v>190000000</v>
+      </c>
+      <c r="L510" t="b">
+        <v>0</v>
+      </c>
+      <c r="M510" t="n">
+        <v>132</v>
+      </c>
+      <c r="N510" t="n">
+        <v>0</v>
+      </c>
+      <c r="O510" t="n">
+        <v>0</v>
+      </c>
+      <c r="P510" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Star Trek Beyond</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>card_510</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>Justin Lin</t>
+        </is>
+      </c>
+      <c r="D511" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E511" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F511" t="n">
+        <v>66</v>
+      </c>
+      <c r="I511" t="n">
+        <v>343500000</v>
+      </c>
+      <c r="J511" t="b">
+        <v>0</v>
+      </c>
+      <c r="K511" t="n">
+        <v>185000000</v>
+      </c>
+      <c r="L511" t="b">
+        <v>0</v>
+      </c>
+      <c r="M511" t="n">
+        <v>122</v>
+      </c>
+      <c r="N511" t="n">
+        <v>0</v>
+      </c>
+      <c r="O511" t="n">
+        <v>0</v>
+      </c>
+      <c r="P511" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add a curated set of notable Godzilla films (card_511-521)
Gojira (1954), Mothra vs. Godzilla, Ghidorah the Three-Headed Monster,
Godzilla vs. Mechagodzilla, The Return of Godzilla, Godzilla (1998),
Shin Godzilla, Godzilla (2014), King of the Monsters, vs. Kong, x Kong:
The New Empire. Not exhaustive -- the full Toho catalog runs 30+ films;
this covers the best-known/highest-grossing entries per era.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P511"/>
+  <dimension ref="A1:P522"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -26619,602 +26619,1140 @@
       </c>
     </row>
     <row r="500">
-      <c r="A500" t="inlineStr">
+      <c r="A500" s="10" t="inlineStr">
         <is>
           <t>Star Trek: The Motion Picture</t>
         </is>
       </c>
-      <c r="B500" t="inlineStr">
+      <c r="B500" s="10" t="inlineStr">
         <is>
           <t>card_499</t>
         </is>
       </c>
-      <c r="C500" t="inlineStr">
+      <c r="C500" s="10" t="inlineStr">
         <is>
           <t>Robert Wise</t>
         </is>
       </c>
-      <c r="D500" t="n">
+      <c r="D500" s="10" t="n">
         <v>1979</v>
       </c>
-      <c r="E500" t="n">
+      <c r="E500" s="10" t="n">
         <v>3.22</v>
       </c>
-      <c r="F500" t="n">
+      <c r="F500" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I500" t="n">
+      <c r="I500" s="10" t="n">
         <v>139000000</v>
       </c>
-      <c r="J500" t="b">
-        <v>0</v>
-      </c>
-      <c r="K500" t="n">
+      <c r="J500" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K500" s="10" t="n">
         <v>44000000</v>
       </c>
-      <c r="L500" t="b">
-        <v>0</v>
-      </c>
-      <c r="M500" t="n">
+      <c r="L500" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M500" s="10" t="n">
         <v>132</v>
       </c>
-      <c r="N500" t="n">
-        <v>0</v>
-      </c>
-      <c r="O500" t="n">
+      <c r="N500" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O500" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P500" t="b">
+      <c r="P500" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="501">
-      <c r="A501" t="inlineStr">
+      <c r="A501" s="10" t="inlineStr">
         <is>
           <t>Star Trek III: The Search for Spock</t>
         </is>
       </c>
-      <c r="B501" t="inlineStr">
+      <c r="B501" s="10" t="inlineStr">
         <is>
           <t>card_500</t>
         </is>
       </c>
-      <c r="C501" t="inlineStr">
+      <c r="C501" s="10" t="inlineStr">
         <is>
           <t>Leonard Nimoy</t>
         </is>
       </c>
-      <c r="D501" t="n">
+      <c r="D501" s="10" t="n">
         <v>1984</v>
       </c>
-      <c r="E501" t="n">
+      <c r="E501" s="10" t="n">
         <v>3.29</v>
       </c>
-      <c r="F501" t="n">
+      <c r="F501" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I501" t="n">
+      <c r="I501" s="10" t="n">
         <v>87000000</v>
       </c>
-      <c r="J501" t="b">
-        <v>0</v>
-      </c>
-      <c r="K501" t="n">
+      <c r="J501" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K501" s="10" t="n">
         <v>16000000</v>
       </c>
-      <c r="L501" t="b">
-        <v>0</v>
-      </c>
-      <c r="M501" t="n">
+      <c r="L501" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M501" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="N501" t="n">
-        <v>0</v>
-      </c>
-      <c r="O501" t="n">
-        <v>0</v>
-      </c>
-      <c r="P501" t="b">
+      <c r="N501" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O501" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P501" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="502">
-      <c r="A502" t="inlineStr">
+      <c r="A502" s="10" t="inlineStr">
         <is>
           <t>Star Trek IV: The Voyage Home</t>
         </is>
       </c>
-      <c r="B502" t="inlineStr">
+      <c r="B502" s="10" t="inlineStr">
         <is>
           <t>card_501</t>
         </is>
       </c>
-      <c r="C502" t="inlineStr">
+      <c r="C502" s="10" t="inlineStr">
         <is>
           <t>Leonard Nimoy</t>
         </is>
       </c>
-      <c r="D502" t="n">
+      <c r="D502" s="10" t="n">
         <v>1986</v>
       </c>
-      <c r="E502" t="n">
+      <c r="E502" s="10" t="n">
         <v>3.74</v>
       </c>
-      <c r="F502" t="n">
+      <c r="F502" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I502" t="n">
+      <c r="I502" s="10" t="n">
         <v>133000000</v>
       </c>
-      <c r="J502" t="b">
-        <v>0</v>
-      </c>
-      <c r="K502" t="n">
+      <c r="J502" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K502" s="10" t="n">
         <v>21000000</v>
       </c>
-      <c r="L502" t="b">
-        <v>0</v>
-      </c>
-      <c r="M502" t="n">
+      <c r="L502" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M502" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N502" t="n">
-        <v>0</v>
-      </c>
-      <c r="O502" t="n">
-        <v>0</v>
-      </c>
-      <c r="P502" t="b">
+      <c r="N502" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O502" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P502" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="503">
-      <c r="A503" t="inlineStr">
+      <c r="A503" s="10" t="inlineStr">
         <is>
           <t>Star Trek V: The Final Frontier</t>
         </is>
       </c>
-      <c r="B503" t="inlineStr">
+      <c r="B503" s="10" t="inlineStr">
         <is>
           <t>card_502</t>
         </is>
       </c>
-      <c r="C503" t="inlineStr">
+      <c r="C503" s="10" t="inlineStr">
         <is>
           <t>William Shatner</t>
         </is>
       </c>
-      <c r="D503" t="n">
+      <c r="D503" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E503" t="n">
+      <c r="E503" s="10" t="n">
         <v>2.61</v>
       </c>
-      <c r="F503" t="n">
+      <c r="F503" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="I503" t="n">
+      <c r="I503" s="10" t="n">
         <v>63000000</v>
       </c>
-      <c r="J503" t="b">
-        <v>0</v>
-      </c>
-      <c r="K503" t="n">
+      <c r="J503" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K503" s="10" t="n">
         <v>33000000</v>
       </c>
-      <c r="L503" t="b">
-        <v>0</v>
-      </c>
-      <c r="M503" t="n">
+      <c r="L503" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M503" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="N503" t="n">
-        <v>0</v>
-      </c>
-      <c r="O503" t="n">
-        <v>0</v>
-      </c>
-      <c r="P503" t="b">
+      <c r="N503" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O503" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P503" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="504">
-      <c r="A504" t="inlineStr">
+      <c r="A504" s="10" t="inlineStr">
         <is>
           <t>Star Trek VI: The Undiscovered Country</t>
         </is>
       </c>
-      <c r="B504" t="inlineStr">
+      <c r="B504" s="10" t="inlineStr">
         <is>
           <t>card_503</t>
         </is>
       </c>
-      <c r="C504" t="inlineStr">
+      <c r="C504" s="10" t="inlineStr">
         <is>
           <t>Nicholas Meyer</t>
         </is>
       </c>
-      <c r="D504" t="n">
+      <c r="D504" s="10" t="n">
         <v>1991</v>
       </c>
-      <c r="E504" t="n">
+      <c r="E504" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F504" t="n">
+      <c r="F504" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I504" t="n">
+      <c r="I504" s="10" t="n">
         <v>96800000</v>
       </c>
-      <c r="J504" t="b">
-        <v>0</v>
-      </c>
-      <c r="K504" t="n">
+      <c r="J504" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K504" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L504" t="b">
-        <v>0</v>
-      </c>
-      <c r="M504" t="n">
+      <c r="L504" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M504" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N504" t="n">
-        <v>0</v>
-      </c>
-      <c r="O504" t="n">
-        <v>0</v>
-      </c>
-      <c r="P504" t="b">
+      <c r="N504" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O504" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P504" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="505">
-      <c r="A505" t="inlineStr">
+      <c r="A505" s="10" t="inlineStr">
         <is>
           <t>Star Trek Generations</t>
         </is>
       </c>
-      <c r="B505" t="inlineStr">
+      <c r="B505" s="10" t="inlineStr">
         <is>
           <t>card_504</t>
         </is>
       </c>
-      <c r="C505" t="inlineStr">
+      <c r="C505" s="10" t="inlineStr">
         <is>
           <t>David Carson</t>
         </is>
       </c>
-      <c r="D505" t="n">
+      <c r="D505" s="10" t="n">
         <v>1994</v>
       </c>
-      <c r="E505" t="n">
+      <c r="E505" s="10" t="n">
         <v>3.05</v>
       </c>
-      <c r="F505" t="n">
+      <c r="F505" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="I505" t="n">
+      <c r="I505" s="10" t="n">
         <v>118000000</v>
       </c>
-      <c r="J505" t="b">
-        <v>0</v>
-      </c>
-      <c r="K505" t="n">
+      <c r="J505" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K505" s="10" t="n">
         <v>35000000</v>
       </c>
-      <c r="L505" t="b">
-        <v>0</v>
-      </c>
-      <c r="M505" t="n">
+      <c r="L505" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M505" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N505" t="n">
-        <v>0</v>
-      </c>
-      <c r="O505" t="n">
-        <v>0</v>
-      </c>
-      <c r="P505" t="b">
+      <c r="N505" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O505" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P505" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="506">
-      <c r="A506" t="inlineStr">
+      <c r="A506" s="10" t="inlineStr">
         <is>
           <t>Star Trek: First Contact</t>
         </is>
       </c>
-      <c r="B506" t="inlineStr">
+      <c r="B506" s="10" t="inlineStr">
         <is>
           <t>card_505</t>
         </is>
       </c>
-      <c r="C506" t="inlineStr">
+      <c r="C506" s="10" t="inlineStr">
         <is>
           <t>Jonathan Frakes</t>
         </is>
       </c>
-      <c r="D506" t="n">
+      <c r="D506" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E506" t="n">
+      <c r="E506" s="10" t="n">
         <v>3.69</v>
       </c>
-      <c r="F506" t="n">
+      <c r="F506" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I506" t="n">
+      <c r="I506" s="10" t="n">
         <v>146000000</v>
       </c>
-      <c r="J506" t="b">
-        <v>0</v>
-      </c>
-      <c r="K506" t="n">
+      <c r="J506" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K506" s="10" t="n">
         <v>45000000</v>
       </c>
-      <c r="L506" t="b">
-        <v>0</v>
-      </c>
-      <c r="M506" t="n">
+      <c r="L506" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M506" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N506" t="n">
-        <v>0</v>
-      </c>
-      <c r="O506" t="n">
-        <v>0</v>
-      </c>
-      <c r="P506" t="b">
+      <c r="N506" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O506" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P506" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="507">
-      <c r="A507" t="inlineStr">
+      <c r="A507" s="10" t="inlineStr">
         <is>
           <t>Star Trek: Insurrection</t>
         </is>
       </c>
-      <c r="B507" t="inlineStr">
+      <c r="B507" s="10" t="inlineStr">
         <is>
           <t>card_506</t>
         </is>
       </c>
-      <c r="C507" t="inlineStr">
+      <c r="C507" s="10" t="inlineStr">
         <is>
           <t>Jonathan Frakes</t>
         </is>
       </c>
-      <c r="D507" t="n">
+      <c r="D507" s="10" t="n">
         <v>1998</v>
       </c>
-      <c r="E507" t="n">
+      <c r="E507" s="10" t="n">
         <v>2.84</v>
       </c>
-      <c r="F507" t="n">
+      <c r="F507" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I507" t="n">
+      <c r="I507" s="10" t="n">
         <v>118000000</v>
       </c>
-      <c r="J507" t="b">
-        <v>0</v>
-      </c>
-      <c r="K507" t="n">
+      <c r="J507" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K507" s="10" t="n">
         <v>70000000</v>
       </c>
-      <c r="L507" t="b">
-        <v>0</v>
-      </c>
-      <c r="M507" t="n">
+      <c r="L507" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M507" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="N507" t="n">
-        <v>0</v>
-      </c>
-      <c r="O507" t="n">
-        <v>0</v>
-      </c>
-      <c r="P507" t="b">
+      <c r="N507" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O507" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P507" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="508">
-      <c r="A508" t="inlineStr">
+      <c r="A508" s="10" t="inlineStr">
         <is>
           <t>Star Trek: Nemesis</t>
         </is>
       </c>
-      <c r="B508" t="inlineStr">
+      <c r="B508" s="10" t="inlineStr">
         <is>
           <t>card_507</t>
         </is>
       </c>
-      <c r="C508" t="inlineStr">
+      <c r="C508" s="10" t="inlineStr">
         <is>
           <t>Stuart Baird</t>
         </is>
       </c>
-      <c r="D508" t="n">
+      <c r="D508" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E508" t="n">
+      <c r="E508" s="10" t="n">
         <v>2.7</v>
       </c>
-      <c r="F508" t="n">
+      <c r="F508" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I508" t="n">
+      <c r="I508" s="10" t="n">
         <v>67300000</v>
       </c>
-      <c r="J508" t="b">
-        <v>0</v>
-      </c>
-      <c r="K508" t="n">
+      <c r="J508" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K508" s="10" t="n">
         <v>60000000</v>
       </c>
-      <c r="L508" t="b">
-        <v>0</v>
-      </c>
-      <c r="M508" t="n">
+      <c r="L508" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M508" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N508" t="n">
-        <v>0</v>
-      </c>
-      <c r="O508" t="n">
-        <v>0</v>
-      </c>
-      <c r="P508" t="b">
+      <c r="N508" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O508" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P508" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="509">
-      <c r="A509" t="inlineStr">
+      <c r="A509" s="10" t="inlineStr">
         <is>
           <t>Star Trek</t>
         </is>
       </c>
-      <c r="B509" t="inlineStr">
+      <c r="B509" s="10" t="inlineStr">
         <is>
           <t>card_508</t>
         </is>
       </c>
-      <c r="C509" t="inlineStr">
+      <c r="C509" s="10" t="inlineStr">
         <is>
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="D509" t="n">
+      <c r="D509" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E509" t="n">
+      <c r="E509" s="10" t="n">
         <v>3.65</v>
       </c>
-      <c r="F509" t="n">
+      <c r="F509" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I509" t="n">
+      <c r="I509" s="10" t="n">
         <v>385700000</v>
       </c>
-      <c r="J509" t="b">
-        <v>0</v>
-      </c>
-      <c r="K509" t="n">
+      <c r="J509" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K509" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L509" t="b">
-        <v>0</v>
-      </c>
-      <c r="M509" t="n">
+      <c r="L509" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M509" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="N509" t="n">
+      <c r="N509" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O509" t="n">
-        <v>0</v>
-      </c>
-      <c r="P509" t="b">
+      <c r="O509" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P509" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="510">
-      <c r="A510" t="inlineStr">
+      <c r="A510" s="10" t="inlineStr">
         <is>
           <t>Star Trek Into Darkness</t>
         </is>
       </c>
-      <c r="B510" t="inlineStr">
+      <c r="B510" s="10" t="inlineStr">
         <is>
           <t>card_509</t>
         </is>
       </c>
-      <c r="C510" t="inlineStr">
+      <c r="C510" s="10" t="inlineStr">
         <is>
           <t>J.J. Abrams</t>
         </is>
       </c>
-      <c r="D510" t="n">
+      <c r="D510" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E510" t="n">
+      <c r="E510" s="10" t="n">
         <v>3.4</v>
       </c>
-      <c r="F510" t="n">
+      <c r="F510" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I510" t="n">
+      <c r="I510" s="10" t="n">
         <v>467400000</v>
       </c>
-      <c r="J510" t="b">
-        <v>0</v>
-      </c>
-      <c r="K510" t="n">
+      <c r="J510" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K510" s="10" t="n">
         <v>190000000</v>
       </c>
-      <c r="L510" t="b">
-        <v>0</v>
-      </c>
-      <c r="M510" t="n">
+      <c r="L510" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M510" s="10" t="n">
         <v>132</v>
       </c>
-      <c r="N510" t="n">
-        <v>0</v>
-      </c>
-      <c r="O510" t="n">
-        <v>0</v>
-      </c>
-      <c r="P510" t="b">
+      <c r="N510" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O510" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P510" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="511">
-      <c r="A511" t="inlineStr">
+      <c r="A511" s="10" t="inlineStr">
         <is>
           <t>Star Trek Beyond</t>
         </is>
       </c>
-      <c r="B511" t="inlineStr">
+      <c r="B511" s="10" t="inlineStr">
         <is>
           <t>card_510</t>
         </is>
       </c>
-      <c r="C511" t="inlineStr">
+      <c r="C511" s="10" t="inlineStr">
         <is>
           <t>Justin Lin</t>
         </is>
       </c>
-      <c r="D511" t="n">
+      <c r="D511" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E511" t="n">
+      <c r="E511" s="10" t="n">
         <v>3.28</v>
       </c>
-      <c r="F511" t="n">
+      <c r="F511" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I511" t="n">
+      <c r="I511" s="10" t="n">
         <v>343500000</v>
       </c>
-      <c r="J511" t="b">
-        <v>0</v>
-      </c>
-      <c r="K511" t="n">
+      <c r="J511" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K511" s="10" t="n">
         <v>185000000</v>
       </c>
-      <c r="L511" t="b">
-        <v>0</v>
-      </c>
-      <c r="M511" t="n">
+      <c r="L511" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M511" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N511" t="n">
-        <v>0</v>
-      </c>
-      <c r="O511" t="n">
-        <v>0</v>
-      </c>
-      <c r="P511" t="b">
+      <c r="N511" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O511" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P511" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Godzilla</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>card_511</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Ishiro Honda</t>
+        </is>
+      </c>
+      <c r="D512" t="n">
+        <v>1954</v>
+      </c>
+      <c r="E512" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="F512" t="n">
+        <v>83</v>
+      </c>
+      <c r="I512" t="n">
+        <v>2250000</v>
+      </c>
+      <c r="J512" t="b">
+        <v>0</v>
+      </c>
+      <c r="K512" t="n">
+        <v>900000</v>
+      </c>
+      <c r="L512" t="b">
+        <v>0</v>
+      </c>
+      <c r="M512" t="n">
+        <v>96</v>
+      </c>
+      <c r="N512" t="n">
+        <v>0</v>
+      </c>
+      <c r="O512" t="n">
+        <v>0</v>
+      </c>
+      <c r="P512" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Mothra vs. Godzilla</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>card_512</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Ishiro Honda</t>
+        </is>
+      </c>
+      <c r="D513" t="n">
+        <v>1964</v>
+      </c>
+      <c r="E513" t="n">
+        <v>3.46</v>
+      </c>
+      <c r="I513" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="J513" t="b">
+        <v>1</v>
+      </c>
+      <c r="K513" t="n">
+        <v>400000</v>
+      </c>
+      <c r="L513" t="b">
+        <v>1</v>
+      </c>
+      <c r="M513" t="n">
+        <v>88</v>
+      </c>
+      <c r="N513" t="n">
+        <v>0</v>
+      </c>
+      <c r="O513" t="n">
+        <v>0</v>
+      </c>
+      <c r="P513" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Ghidorah, the Three-Headed Monster</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>card_513</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Ishiro Honda</t>
+        </is>
+      </c>
+      <c r="D514" t="n">
+        <v>1964</v>
+      </c>
+      <c r="E514" t="n">
+        <v>3.39</v>
+      </c>
+      <c r="I514" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="J514" t="b">
+        <v>0</v>
+      </c>
+      <c r="K514" t="n">
+        <v>370000</v>
+      </c>
+      <c r="L514" t="b">
+        <v>0</v>
+      </c>
+      <c r="M514" t="n">
+        <v>93</v>
+      </c>
+      <c r="N514" t="n">
+        <v>0</v>
+      </c>
+      <c r="O514" t="n">
+        <v>0</v>
+      </c>
+      <c r="P514" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Godzilla vs. Mechagodzilla</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>card_514</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Jun Fukuda</t>
+        </is>
+      </c>
+      <c r="D515" t="n">
+        <v>1974</v>
+      </c>
+      <c r="E515" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="I515" t="n">
+        <v>17100000</v>
+      </c>
+      <c r="J515" t="b">
+        <v>0</v>
+      </c>
+      <c r="K515" t="n">
+        <v>380000</v>
+      </c>
+      <c r="L515" t="b">
+        <v>0</v>
+      </c>
+      <c r="M515" t="n">
+        <v>84</v>
+      </c>
+      <c r="N515" t="n">
+        <v>0</v>
+      </c>
+      <c r="O515" t="n">
+        <v>0</v>
+      </c>
+      <c r="P515" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>The Return of Godzilla</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>card_515</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Koji Hashimoto</t>
+        </is>
+      </c>
+      <c r="D516" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E516" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="I516" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="J516" t="b">
+        <v>0</v>
+      </c>
+      <c r="K516" t="n">
+        <v>6250000</v>
+      </c>
+      <c r="L516" t="b">
+        <v>0</v>
+      </c>
+      <c r="M516" t="n">
+        <v>103</v>
+      </c>
+      <c r="N516" t="n">
+        <v>0</v>
+      </c>
+      <c r="O516" t="n">
+        <v>0</v>
+      </c>
+      <c r="P516" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Godzilla (1998)</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>card_516</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Roland Emmerich</t>
+        </is>
+      </c>
+      <c r="D517" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E517" t="n">
+        <v>2.31</v>
+      </c>
+      <c r="F517" t="n">
+        <v>50</v>
+      </c>
+      <c r="I517" t="n">
+        <v>379000000</v>
+      </c>
+      <c r="J517" t="b">
+        <v>0</v>
+      </c>
+      <c r="K517" t="n">
+        <v>140000000</v>
+      </c>
+      <c r="L517" t="b">
+        <v>0</v>
+      </c>
+      <c r="M517" t="n">
+        <v>139</v>
+      </c>
+      <c r="N517" t="n">
+        <v>0</v>
+      </c>
+      <c r="O517" t="n">
+        <v>0</v>
+      </c>
+      <c r="P517" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Shin Godzilla</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>card_517</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Hideaki Anno and Shinji Higuchi</t>
+        </is>
+      </c>
+      <c r="D518" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E518" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="F518" t="n">
+        <v>74</v>
+      </c>
+      <c r="I518" t="n">
+        <v>83300000</v>
+      </c>
+      <c r="J518" t="b">
+        <v>0</v>
+      </c>
+      <c r="K518" t="n">
+        <v>12600000</v>
+      </c>
+      <c r="L518" t="b">
+        <v>0</v>
+      </c>
+      <c r="M518" t="n">
+        <v>120</v>
+      </c>
+      <c r="N518" t="n">
+        <v>0</v>
+      </c>
+      <c r="O518" t="n">
+        <v>0</v>
+      </c>
+      <c r="P518" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Godzilla (2014)</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>card_518</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Gareth Edwards</t>
+        </is>
+      </c>
+      <c r="D519" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E519" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="F519" t="n">
+        <v>69</v>
+      </c>
+      <c r="I519" t="n">
+        <v>529100000</v>
+      </c>
+      <c r="J519" t="b">
+        <v>0</v>
+      </c>
+      <c r="K519" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L519" t="b">
+        <v>0</v>
+      </c>
+      <c r="M519" t="n">
+        <v>123</v>
+      </c>
+      <c r="N519" t="n">
+        <v>0</v>
+      </c>
+      <c r="O519" t="n">
+        <v>0</v>
+      </c>
+      <c r="P519" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Godzilla: King of the Monsters</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>card_519</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Michael Dougherty</t>
+        </is>
+      </c>
+      <c r="D520" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E520" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="F520" t="n">
+        <v>70</v>
+      </c>
+      <c r="I520" t="n">
+        <v>387300000</v>
+      </c>
+      <c r="J520" t="b">
+        <v>0</v>
+      </c>
+      <c r="K520" t="n">
+        <v>185000000</v>
+      </c>
+      <c r="L520" t="b">
+        <v>0</v>
+      </c>
+      <c r="M520" t="n">
+        <v>131</v>
+      </c>
+      <c r="N520" t="n">
+        <v>0</v>
+      </c>
+      <c r="O520" t="n">
+        <v>0</v>
+      </c>
+      <c r="P520" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Godzilla vs. Kong</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>card_520</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>Adam Wingard</t>
+        </is>
+      </c>
+      <c r="D521" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E521" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="F521" t="n">
+        <v>68</v>
+      </c>
+      <c r="I521" t="n">
+        <v>470000000</v>
+      </c>
+      <c r="J521" t="b">
+        <v>0</v>
+      </c>
+      <c r="K521" t="n">
+        <v>155000000</v>
+      </c>
+      <c r="L521" t="b">
+        <v>0</v>
+      </c>
+      <c r="M521" t="n">
+        <v>113</v>
+      </c>
+      <c r="N521" t="n">
+        <v>0</v>
+      </c>
+      <c r="O521" t="n">
+        <v>0</v>
+      </c>
+      <c r="P521" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Godzilla x Kong: The New Empire</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>card_521</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Adam Wingard</t>
+        </is>
+      </c>
+      <c r="D522" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E522" t="n">
+        <v>2.72</v>
+      </c>
+      <c r="F522" t="n">
+        <v>70</v>
+      </c>
+      <c r="I522" t="n">
+        <v>572500000</v>
+      </c>
+      <c r="J522" t="b">
+        <v>0</v>
+      </c>
+      <c r="K522" t="n">
+        <v>135000000</v>
+      </c>
+      <c r="L522" t="b">
+        <v>0</v>
+      </c>
+      <c r="M522" t="n">
+        <v>115</v>
+      </c>
+      <c r="N522" t="n">
+        <v>0</v>
+      </c>
+      <c r="O522" t="n">
+        <v>0</v>
+      </c>
+      <c r="P522" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the complete James Bond series (card_522-546)
All 25 Eon-produced films, Dr. No (1962) through No Time to Die
(2021).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P522"/>
+  <dimension ref="A1:P547"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -27219,540 +27219,1790 @@
       </c>
     </row>
     <row r="512">
-      <c r="A512" t="inlineStr">
+      <c r="A512" s="10" t="inlineStr">
         <is>
           <t>Godzilla</t>
         </is>
       </c>
-      <c r="B512" t="inlineStr">
+      <c r="B512" s="10" t="inlineStr">
         <is>
           <t>card_511</t>
         </is>
       </c>
-      <c r="C512" t="inlineStr">
+      <c r="C512" s="10" t="inlineStr">
         <is>
           <t>Ishiro Honda</t>
         </is>
       </c>
-      <c r="D512" t="n">
+      <c r="D512" s="10" t="n">
         <v>1954</v>
       </c>
-      <c r="E512" t="n">
+      <c r="E512" s="10" t="n">
         <v>4.07</v>
       </c>
-      <c r="F512" t="n">
+      <c r="F512" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I512" t="n">
+      <c r="I512" s="10" t="n">
         <v>2250000</v>
       </c>
-      <c r="J512" t="b">
-        <v>0</v>
-      </c>
-      <c r="K512" t="n">
+      <c r="J512" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K512" s="10" t="n">
         <v>900000</v>
       </c>
-      <c r="L512" t="b">
-        <v>0</v>
-      </c>
-      <c r="M512" t="n">
+      <c r="L512" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M512" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N512" t="n">
-        <v>0</v>
-      </c>
-      <c r="O512" t="n">
-        <v>0</v>
-      </c>
-      <c r="P512" t="b">
+      <c r="N512" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O512" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P512" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="513">
-      <c r="A513" t="inlineStr">
+      <c r="A513" s="10" t="inlineStr">
         <is>
           <t>Mothra vs. Godzilla</t>
         </is>
       </c>
-      <c r="B513" t="inlineStr">
+      <c r="B513" s="10" t="inlineStr">
         <is>
           <t>card_512</t>
         </is>
       </c>
-      <c r="C513" t="inlineStr">
+      <c r="C513" s="10" t="inlineStr">
         <is>
           <t>Ishiro Honda</t>
         </is>
       </c>
-      <c r="D513" t="n">
+      <c r="D513" s="10" t="n">
         <v>1964</v>
       </c>
-      <c r="E513" t="n">
+      <c r="E513" s="10" t="n">
         <v>3.46</v>
       </c>
-      <c r="I513" t="n">
+      <c r="I513" s="10" t="n">
         <v>3500000</v>
       </c>
-      <c r="J513" t="b">
+      <c r="J513" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K513" t="n">
+      <c r="K513" s="10" t="n">
         <v>400000</v>
       </c>
-      <c r="L513" t="b">
+      <c r="L513" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M513" t="n">
+      <c r="M513" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N513" t="n">
-        <v>0</v>
-      </c>
-      <c r="O513" t="n">
-        <v>0</v>
-      </c>
-      <c r="P513" t="b">
+      <c r="N513" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O513" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P513" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="514">
-      <c r="A514" t="inlineStr">
+      <c r="A514" s="10" t="inlineStr">
         <is>
           <t>Ghidorah, the Three-Headed Monster</t>
         </is>
       </c>
-      <c r="B514" t="inlineStr">
+      <c r="B514" s="10" t="inlineStr">
         <is>
           <t>card_513</t>
         </is>
       </c>
-      <c r="C514" t="inlineStr">
+      <c r="C514" s="10" t="inlineStr">
         <is>
           <t>Ishiro Honda</t>
         </is>
       </c>
-      <c r="D514" t="n">
+      <c r="D514" s="10" t="n">
         <v>1964</v>
       </c>
-      <c r="E514" t="n">
+      <c r="E514" s="10" t="n">
         <v>3.39</v>
       </c>
-      <c r="I514" t="n">
+      <c r="I514" s="10" t="n">
         <v>2300000</v>
       </c>
-      <c r="J514" t="b">
-        <v>0</v>
-      </c>
-      <c r="K514" t="n">
+      <c r="J514" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K514" s="10" t="n">
         <v>370000</v>
       </c>
-      <c r="L514" t="b">
-        <v>0</v>
-      </c>
-      <c r="M514" t="n">
+      <c r="L514" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M514" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N514" t="n">
-        <v>0</v>
-      </c>
-      <c r="O514" t="n">
-        <v>0</v>
-      </c>
-      <c r="P514" t="b">
+      <c r="N514" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O514" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P514" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="515">
-      <c r="A515" t="inlineStr">
+      <c r="A515" s="10" t="inlineStr">
         <is>
           <t>Godzilla vs. Mechagodzilla</t>
         </is>
       </c>
-      <c r="B515" t="inlineStr">
+      <c r="B515" s="10" t="inlineStr">
         <is>
           <t>card_514</t>
         </is>
       </c>
-      <c r="C515" t="inlineStr">
+      <c r="C515" s="10" t="inlineStr">
         <is>
           <t>Jun Fukuda</t>
         </is>
       </c>
-      <c r="D515" t="n">
+      <c r="D515" s="10" t="n">
         <v>1974</v>
       </c>
-      <c r="E515" t="n">
+      <c r="E515" s="10" t="n">
         <v>3.3</v>
       </c>
-      <c r="I515" t="n">
+      <c r="I515" s="10" t="n">
         <v>17100000</v>
       </c>
-      <c r="J515" t="b">
-        <v>0</v>
-      </c>
-      <c r="K515" t="n">
+      <c r="J515" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K515" s="10" t="n">
         <v>380000</v>
       </c>
-      <c r="L515" t="b">
-        <v>0</v>
-      </c>
-      <c r="M515" t="n">
+      <c r="L515" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M515" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="N515" t="n">
-        <v>0</v>
-      </c>
-      <c r="O515" t="n">
-        <v>0</v>
-      </c>
-      <c r="P515" t="b">
+      <c r="N515" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O515" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P515" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="516">
-      <c r="A516" t="inlineStr">
+      <c r="A516" s="10" t="inlineStr">
         <is>
           <t>The Return of Godzilla</t>
         </is>
       </c>
-      <c r="B516" t="inlineStr">
+      <c r="B516" s="10" t="inlineStr">
         <is>
           <t>card_515</t>
         </is>
       </c>
-      <c r="C516" t="inlineStr">
+      <c r="C516" s="10" t="inlineStr">
         <is>
           <t>Koji Hashimoto</t>
         </is>
       </c>
-      <c r="D516" t="n">
+      <c r="D516" s="10" t="n">
         <v>1984</v>
       </c>
-      <c r="E516" t="n">
+      <c r="E516" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="I516" t="n">
+      <c r="I516" s="10" t="n">
         <v>14000000</v>
       </c>
-      <c r="J516" t="b">
-        <v>0</v>
-      </c>
-      <c r="K516" t="n">
+      <c r="J516" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K516" s="10" t="n">
         <v>6250000</v>
       </c>
-      <c r="L516" t="b">
-        <v>0</v>
-      </c>
-      <c r="M516" t="n">
+      <c r="L516" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M516" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="N516" t="n">
-        <v>0</v>
-      </c>
-      <c r="O516" t="n">
-        <v>0</v>
-      </c>
-      <c r="P516" t="b">
+      <c r="N516" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O516" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P516" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="517">
-      <c r="A517" t="inlineStr">
+      <c r="A517" s="10" t="inlineStr">
         <is>
           <t>Godzilla (1998)</t>
         </is>
       </c>
-      <c r="B517" t="inlineStr">
+      <c r="B517" s="10" t="inlineStr">
         <is>
           <t>card_516</t>
         </is>
       </c>
-      <c r="C517" t="inlineStr">
+      <c r="C517" s="10" t="inlineStr">
         <is>
           <t>Roland Emmerich</t>
         </is>
       </c>
-      <c r="D517" t="n">
+      <c r="D517" s="10" t="n">
         <v>1998</v>
       </c>
-      <c r="E517" t="n">
+      <c r="E517" s="10" t="n">
         <v>2.31</v>
       </c>
-      <c r="F517" t="n">
+      <c r="F517" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I517" t="n">
+      <c r="I517" s="10" t="n">
         <v>379000000</v>
       </c>
-      <c r="J517" t="b">
-        <v>0</v>
-      </c>
-      <c r="K517" t="n">
+      <c r="J517" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K517" s="10" t="n">
         <v>140000000</v>
       </c>
-      <c r="L517" t="b">
-        <v>0</v>
-      </c>
-      <c r="M517" t="n">
+      <c r="L517" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M517" s="10" t="n">
         <v>139</v>
       </c>
-      <c r="N517" t="n">
-        <v>0</v>
-      </c>
-      <c r="O517" t="n">
-        <v>0</v>
-      </c>
-      <c r="P517" t="b">
+      <c r="N517" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O517" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P517" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="518">
-      <c r="A518" t="inlineStr">
+      <c r="A518" s="10" t="inlineStr">
         <is>
           <t>Shin Godzilla</t>
         </is>
       </c>
-      <c r="B518" t="inlineStr">
+      <c r="B518" s="10" t="inlineStr">
         <is>
           <t>card_517</t>
         </is>
       </c>
-      <c r="C518" t="inlineStr">
+      <c r="C518" s="10" t="inlineStr">
         <is>
           <t>Hideaki Anno and Shinji Higuchi</t>
         </is>
       </c>
-      <c r="D518" t="n">
+      <c r="D518" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E518" t="n">
+      <c r="E518" s="10" t="n">
         <v>3.89</v>
       </c>
-      <c r="F518" t="n">
+      <c r="F518" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I518" t="n">
+      <c r="I518" s="10" t="n">
         <v>83300000</v>
       </c>
-      <c r="J518" t="b">
-        <v>0</v>
-      </c>
-      <c r="K518" t="n">
+      <c r="J518" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K518" s="10" t="n">
         <v>12600000</v>
       </c>
-      <c r="L518" t="b">
-        <v>0</v>
-      </c>
-      <c r="M518" t="n">
+      <c r="L518" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M518" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="N518" t="n">
-        <v>0</v>
-      </c>
-      <c r="O518" t="n">
-        <v>0</v>
-      </c>
-      <c r="P518" t="b">
+      <c r="N518" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O518" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P518" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="519">
-      <c r="A519" t="inlineStr">
+      <c r="A519" s="10" t="inlineStr">
         <is>
           <t>Godzilla (2014)</t>
         </is>
       </c>
-      <c r="B519" t="inlineStr">
+      <c r="B519" s="10" t="inlineStr">
         <is>
           <t>card_518</t>
         </is>
       </c>
-      <c r="C519" t="inlineStr">
+      <c r="C519" s="10" t="inlineStr">
         <is>
           <t>Gareth Edwards</t>
         </is>
       </c>
-      <c r="D519" t="n">
+      <c r="D519" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E519" t="n">
+      <c r="E519" s="10" t="n">
         <v>3.14</v>
       </c>
-      <c r="F519" t="n">
+      <c r="F519" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I519" t="n">
+      <c r="I519" s="10" t="n">
         <v>529100000</v>
       </c>
-      <c r="J519" t="b">
-        <v>0</v>
-      </c>
-      <c r="K519" t="n">
+      <c r="J519" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K519" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L519" t="b">
-        <v>0</v>
-      </c>
-      <c r="M519" t="n">
+      <c r="L519" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M519" s="10" t="n">
         <v>123</v>
       </c>
-      <c r="N519" t="n">
-        <v>0</v>
-      </c>
-      <c r="O519" t="n">
-        <v>0</v>
-      </c>
-      <c r="P519" t="b">
+      <c r="N519" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O519" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P519" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="520">
-      <c r="A520" t="inlineStr">
+      <c r="A520" s="10" t="inlineStr">
         <is>
           <t>Godzilla: King of the Monsters</t>
         </is>
       </c>
-      <c r="B520" t="inlineStr">
+      <c r="B520" s="10" t="inlineStr">
         <is>
           <t>card_519</t>
         </is>
       </c>
-      <c r="C520" t="inlineStr">
+      <c r="C520" s="10" t="inlineStr">
         <is>
           <t>Michael Dougherty</t>
         </is>
       </c>
-      <c r="D520" t="n">
+      <c r="D520" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E520" t="n">
+      <c r="E520" s="10" t="n">
         <v>2.93</v>
       </c>
-      <c r="F520" t="n">
+      <c r="F520" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I520" t="n">
+      <c r="I520" s="10" t="n">
         <v>387300000</v>
       </c>
-      <c r="J520" t="b">
-        <v>0</v>
-      </c>
-      <c r="K520" t="n">
+      <c r="J520" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K520" s="10" t="n">
         <v>185000000</v>
       </c>
-      <c r="L520" t="b">
-        <v>0</v>
-      </c>
-      <c r="M520" t="n">
+      <c r="L520" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M520" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N520" t="n">
-        <v>0</v>
-      </c>
-      <c r="O520" t="n">
-        <v>0</v>
-      </c>
-      <c r="P520" t="b">
+      <c r="N520" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O520" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P520" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="521">
-      <c r="A521" t="inlineStr">
+      <c r="A521" s="10" t="inlineStr">
         <is>
           <t>Godzilla vs. Kong</t>
         </is>
       </c>
-      <c r="B521" t="inlineStr">
+      <c r="B521" s="10" t="inlineStr">
         <is>
           <t>card_520</t>
         </is>
       </c>
-      <c r="C521" t="inlineStr">
+      <c r="C521" s="10" t="inlineStr">
         <is>
           <t>Adam Wingard</t>
         </is>
       </c>
-      <c r="D521" t="n">
+      <c r="D521" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E521" t="n">
+      <c r="E521" s="10" t="n">
         <v>2.84</v>
       </c>
-      <c r="F521" t="n">
+      <c r="F521" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I521" t="n">
+      <c r="I521" s="10" t="n">
         <v>470000000</v>
       </c>
-      <c r="J521" t="b">
-        <v>0</v>
-      </c>
-      <c r="K521" t="n">
+      <c r="J521" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K521" s="10" t="n">
         <v>155000000</v>
       </c>
-      <c r="L521" t="b">
-        <v>0</v>
-      </c>
-      <c r="M521" t="n">
+      <c r="L521" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M521" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="N521" t="n">
-        <v>0</v>
-      </c>
-      <c r="O521" t="n">
-        <v>0</v>
-      </c>
-      <c r="P521" t="b">
+      <c r="N521" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O521" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P521" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="522">
-      <c r="A522" t="inlineStr">
+      <c r="A522" s="10" t="inlineStr">
         <is>
           <t>Godzilla x Kong: The New Empire</t>
         </is>
       </c>
-      <c r="B522" t="inlineStr">
+      <c r="B522" s="10" t="inlineStr">
         <is>
           <t>card_521</t>
         </is>
       </c>
-      <c r="C522" t="inlineStr">
+      <c r="C522" s="10" t="inlineStr">
         <is>
           <t>Adam Wingard</t>
         </is>
       </c>
-      <c r="D522" t="n">
+      <c r="D522" s="10" t="n">
         <v>2024</v>
       </c>
-      <c r="E522" t="n">
+      <c r="E522" s="10" t="n">
         <v>2.72</v>
       </c>
-      <c r="F522" t="n">
+      <c r="F522" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I522" t="n">
+      <c r="I522" s="10" t="n">
         <v>572500000</v>
       </c>
-      <c r="J522" t="b">
-        <v>0</v>
-      </c>
-      <c r="K522" t="n">
+      <c r="J522" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K522" s="10" t="n">
         <v>135000000</v>
       </c>
-      <c r="L522" t="b">
-        <v>0</v>
-      </c>
-      <c r="M522" t="n">
+      <c r="L522" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M522" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N522" t="n">
-        <v>0</v>
-      </c>
-      <c r="O522" t="n">
-        <v>0</v>
-      </c>
-      <c r="P522" t="b">
+      <c r="N522" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O522" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P522" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Dr. No</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>card_522</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Terence Young</t>
+        </is>
+      </c>
+      <c r="D523" t="n">
+        <v>1962</v>
+      </c>
+      <c r="E523" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F523" t="n">
+        <v>74</v>
+      </c>
+      <c r="I523" t="n">
+        <v>59500000</v>
+      </c>
+      <c r="J523" t="b">
+        <v>0</v>
+      </c>
+      <c r="K523" t="n">
+        <v>1100000</v>
+      </c>
+      <c r="L523" t="b">
+        <v>0</v>
+      </c>
+      <c r="M523" t="n">
+        <v>110</v>
+      </c>
+      <c r="N523" t="n">
+        <v>0</v>
+      </c>
+      <c r="O523" t="n">
+        <v>0</v>
+      </c>
+      <c r="P523" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>From Russia with Love</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>card_523</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Terence Young</t>
+        </is>
+      </c>
+      <c r="D524" t="n">
+        <v>1963</v>
+      </c>
+      <c r="E524" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F524" t="n">
+        <v>78</v>
+      </c>
+      <c r="I524" t="n">
+        <v>79000000</v>
+      </c>
+      <c r="J524" t="b">
+        <v>0</v>
+      </c>
+      <c r="K524" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="L524" t="b">
+        <v>0</v>
+      </c>
+      <c r="M524" t="n">
+        <v>115</v>
+      </c>
+      <c r="N524" t="n">
+        <v>0</v>
+      </c>
+      <c r="O524" t="n">
+        <v>0</v>
+      </c>
+      <c r="P524" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Goldfinger</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>card_524</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Guy Hamilton</t>
+        </is>
+      </c>
+      <c r="D525" t="n">
+        <v>1964</v>
+      </c>
+      <c r="E525" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F525" t="n">
+        <v>80</v>
+      </c>
+      <c r="I525" t="n">
+        <v>124900000</v>
+      </c>
+      <c r="J525" t="b">
+        <v>0</v>
+      </c>
+      <c r="K525" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="L525" t="b">
+        <v>0</v>
+      </c>
+      <c r="M525" t="n">
+        <v>110</v>
+      </c>
+      <c r="N525" t="n">
+        <v>1</v>
+      </c>
+      <c r="O525" t="n">
+        <v>0</v>
+      </c>
+      <c r="P525" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Thunderball</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>card_525</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Terence Young</t>
+        </is>
+      </c>
+      <c r="D526" t="n">
+        <v>1965</v>
+      </c>
+      <c r="E526" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="F526" t="n">
+        <v>67</v>
+      </c>
+      <c r="I526" t="n">
+        <v>141200000</v>
+      </c>
+      <c r="J526" t="b">
+        <v>0</v>
+      </c>
+      <c r="K526" t="n">
+        <v>9000000</v>
+      </c>
+      <c r="L526" t="b">
+        <v>0</v>
+      </c>
+      <c r="M526" t="n">
+        <v>130</v>
+      </c>
+      <c r="N526" t="n">
+        <v>1</v>
+      </c>
+      <c r="O526" t="n">
+        <v>0</v>
+      </c>
+      <c r="P526" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>You Only Live Twice</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>card_526</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Lewis Gilbert</t>
+        </is>
+      </c>
+      <c r="D527" t="n">
+        <v>1967</v>
+      </c>
+      <c r="E527" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F527" t="n">
+        <v>68</v>
+      </c>
+      <c r="I527" t="n">
+        <v>111600000</v>
+      </c>
+      <c r="J527" t="b">
+        <v>0</v>
+      </c>
+      <c r="K527" t="n">
+        <v>9500000</v>
+      </c>
+      <c r="L527" t="b">
+        <v>0</v>
+      </c>
+      <c r="M527" t="n">
+        <v>117</v>
+      </c>
+      <c r="N527" t="n">
+        <v>0</v>
+      </c>
+      <c r="O527" t="n">
+        <v>0</v>
+      </c>
+      <c r="P527" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>On Her Majesty's Secret Service</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>card_527</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Peter R. Hunt</t>
+        </is>
+      </c>
+      <c r="D528" t="n">
+        <v>1969</v>
+      </c>
+      <c r="E528" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="F528" t="n">
+        <v>72</v>
+      </c>
+      <c r="I528" t="n">
+        <v>82000000</v>
+      </c>
+      <c r="J528" t="b">
+        <v>0</v>
+      </c>
+      <c r="K528" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="L528" t="b">
+        <v>0</v>
+      </c>
+      <c r="M528" t="n">
+        <v>142</v>
+      </c>
+      <c r="N528" t="n">
+        <v>0</v>
+      </c>
+      <c r="O528" t="n">
+        <v>0</v>
+      </c>
+      <c r="P528" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Diamonds Are Forever</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>card_528</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Guy Hamilton</t>
+        </is>
+      </c>
+      <c r="D529" t="n">
+        <v>1971</v>
+      </c>
+      <c r="E529" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="F529" t="n">
+        <v>57</v>
+      </c>
+      <c r="I529" t="n">
+        <v>116000000</v>
+      </c>
+      <c r="J529" t="b">
+        <v>0</v>
+      </c>
+      <c r="K529" t="n">
+        <v>7200000</v>
+      </c>
+      <c r="L529" t="b">
+        <v>0</v>
+      </c>
+      <c r="M529" t="n">
+        <v>120</v>
+      </c>
+      <c r="N529" t="n">
+        <v>0</v>
+      </c>
+      <c r="O529" t="n">
+        <v>0</v>
+      </c>
+      <c r="P529" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Live and Let Die</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>card_529</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Guy Hamilton</t>
+        </is>
+      </c>
+      <c r="D530" t="n">
+        <v>1973</v>
+      </c>
+      <c r="E530" t="n">
+        <v>3.17</v>
+      </c>
+      <c r="F530" t="n">
+        <v>62</v>
+      </c>
+      <c r="I530" t="n">
+        <v>161800000</v>
+      </c>
+      <c r="J530" t="b">
+        <v>0</v>
+      </c>
+      <c r="K530" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="L530" t="b">
+        <v>0</v>
+      </c>
+      <c r="M530" t="n">
+        <v>121</v>
+      </c>
+      <c r="N530" t="n">
+        <v>0</v>
+      </c>
+      <c r="O530" t="n">
+        <v>0</v>
+      </c>
+      <c r="P530" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>The Man with the Golden Gun</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>card_530</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Guy Hamilton</t>
+        </is>
+      </c>
+      <c r="D531" t="n">
+        <v>1974</v>
+      </c>
+      <c r="E531" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="F531" t="n">
+        <v>60</v>
+      </c>
+      <c r="I531" t="n">
+        <v>97600000</v>
+      </c>
+      <c r="J531" t="b">
+        <v>0</v>
+      </c>
+      <c r="K531" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="L531" t="b">
+        <v>0</v>
+      </c>
+      <c r="M531" t="n">
+        <v>125</v>
+      </c>
+      <c r="N531" t="n">
+        <v>0</v>
+      </c>
+      <c r="O531" t="n">
+        <v>0</v>
+      </c>
+      <c r="P531" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>The Spy Who Loved Me</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>card_531</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Lewis Gilbert</t>
+        </is>
+      </c>
+      <c r="D532" t="n">
+        <v>1977</v>
+      </c>
+      <c r="E532" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F532" t="n">
+        <v>69</v>
+      </c>
+      <c r="I532" t="n">
+        <v>185400000</v>
+      </c>
+      <c r="J532" t="b">
+        <v>0</v>
+      </c>
+      <c r="K532" t="n">
+        <v>13500000</v>
+      </c>
+      <c r="L532" t="b">
+        <v>0</v>
+      </c>
+      <c r="M532" t="n">
+        <v>125</v>
+      </c>
+      <c r="N532" t="n">
+        <v>0</v>
+      </c>
+      <c r="O532" t="n">
+        <v>0</v>
+      </c>
+      <c r="P532" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Moonraker</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>card_532</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Lewis Gilbert</t>
+        </is>
+      </c>
+      <c r="D533" t="n">
+        <v>1979</v>
+      </c>
+      <c r="E533" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="F533" t="n">
+        <v>60</v>
+      </c>
+      <c r="I533" t="n">
+        <v>210300000</v>
+      </c>
+      <c r="J533" t="b">
+        <v>0</v>
+      </c>
+      <c r="K533" t="n">
+        <v>34000000</v>
+      </c>
+      <c r="L533" t="b">
+        <v>0</v>
+      </c>
+      <c r="M533" t="n">
+        <v>126</v>
+      </c>
+      <c r="N533" t="n">
+        <v>0</v>
+      </c>
+      <c r="O533" t="n">
+        <v>0</v>
+      </c>
+      <c r="P533" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>For Your Eyes Only</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>card_533</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>John Glen</t>
+        </is>
+      </c>
+      <c r="D534" t="n">
+        <v>1981</v>
+      </c>
+      <c r="E534" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F534" t="n">
+        <v>65</v>
+      </c>
+      <c r="I534" t="n">
+        <v>202800000</v>
+      </c>
+      <c r="J534" t="b">
+        <v>0</v>
+      </c>
+      <c r="K534" t="n">
+        <v>28000000</v>
+      </c>
+      <c r="L534" t="b">
+        <v>0</v>
+      </c>
+      <c r="M534" t="n">
+        <v>127</v>
+      </c>
+      <c r="N534" t="n">
+        <v>0</v>
+      </c>
+      <c r="O534" t="n">
+        <v>0</v>
+      </c>
+      <c r="P534" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Octopussy</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>card_534</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>John Glen</t>
+        </is>
+      </c>
+      <c r="D535" t="n">
+        <v>1983</v>
+      </c>
+      <c r="E535" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="F535" t="n">
+        <v>63</v>
+      </c>
+      <c r="I535" t="n">
+        <v>187500000</v>
+      </c>
+      <c r="J535" t="b">
+        <v>0</v>
+      </c>
+      <c r="K535" t="n">
+        <v>27500000</v>
+      </c>
+      <c r="L535" t="b">
+        <v>0</v>
+      </c>
+      <c r="M535" t="n">
+        <v>131</v>
+      </c>
+      <c r="N535" t="n">
+        <v>0</v>
+      </c>
+      <c r="O535" t="n">
+        <v>0</v>
+      </c>
+      <c r="P535" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>A View to a Kill</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>card_535</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>John Glen</t>
+        </is>
+      </c>
+      <c r="D536" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E536" t="n">
+        <v>2.89</v>
+      </c>
+      <c r="F536" t="n">
+        <v>57</v>
+      </c>
+      <c r="I536" t="n">
+        <v>152400000</v>
+      </c>
+      <c r="J536" t="b">
+        <v>0</v>
+      </c>
+      <c r="K536" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L536" t="b">
+        <v>0</v>
+      </c>
+      <c r="M536" t="n">
+        <v>131</v>
+      </c>
+      <c r="N536" t="n">
+        <v>0</v>
+      </c>
+      <c r="O536" t="n">
+        <v>0</v>
+      </c>
+      <c r="P536" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>The Living Daylights</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>card_536</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>John Glen</t>
+        </is>
+      </c>
+      <c r="D537" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E537" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="F537" t="n">
+        <v>69</v>
+      </c>
+      <c r="I537" t="n">
+        <v>191200000</v>
+      </c>
+      <c r="J537" t="b">
+        <v>0</v>
+      </c>
+      <c r="K537" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L537" t="b">
+        <v>0</v>
+      </c>
+      <c r="M537" t="n">
+        <v>131</v>
+      </c>
+      <c r="N537" t="n">
+        <v>0</v>
+      </c>
+      <c r="O537" t="n">
+        <v>0</v>
+      </c>
+      <c r="P537" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Licence to Kill</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>card_537</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>John Glen</t>
+        </is>
+      </c>
+      <c r="D538" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E538" t="n">
+        <v>3.38</v>
+      </c>
+      <c r="F538" t="n">
+        <v>68</v>
+      </c>
+      <c r="I538" t="n">
+        <v>156100000</v>
+      </c>
+      <c r="J538" t="b">
+        <v>0</v>
+      </c>
+      <c r="K538" t="n">
+        <v>32000000</v>
+      </c>
+      <c r="L538" t="b">
+        <v>0</v>
+      </c>
+      <c r="M538" t="n">
+        <v>133</v>
+      </c>
+      <c r="N538" t="n">
+        <v>0</v>
+      </c>
+      <c r="O538" t="n">
+        <v>0</v>
+      </c>
+      <c r="P538" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>GoldenEye</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>card_538</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Martin Campbell</t>
+        </is>
+      </c>
+      <c r="D539" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E539" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="F539" t="n">
+        <v>77</v>
+      </c>
+      <c r="I539" t="n">
+        <v>356400000</v>
+      </c>
+      <c r="J539" t="b">
+        <v>0</v>
+      </c>
+      <c r="K539" t="n">
+        <v>60000000</v>
+      </c>
+      <c r="L539" t="b">
+        <v>0</v>
+      </c>
+      <c r="M539" t="n">
+        <v>130</v>
+      </c>
+      <c r="N539" t="n">
+        <v>0</v>
+      </c>
+      <c r="O539" t="n">
+        <v>0</v>
+      </c>
+      <c r="P539" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Tomorrow Never Dies</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>card_539</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Roger Spottiswoode</t>
+        </is>
+      </c>
+      <c r="D540" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E540" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="F540" t="n">
+        <v>67</v>
+      </c>
+      <c r="I540" t="n">
+        <v>339500000</v>
+      </c>
+      <c r="J540" t="b">
+        <v>0</v>
+      </c>
+      <c r="K540" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L540" t="b">
+        <v>0</v>
+      </c>
+      <c r="M540" t="n">
+        <v>119</v>
+      </c>
+      <c r="N540" t="n">
+        <v>0</v>
+      </c>
+      <c r="O540" t="n">
+        <v>0</v>
+      </c>
+      <c r="P540" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>The World Is Not Enough</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>card_540</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Michael Apted</t>
+        </is>
+      </c>
+      <c r="D541" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E541" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="F541" t="n">
+        <v>62</v>
+      </c>
+      <c r="I541" t="n">
+        <v>361000000</v>
+      </c>
+      <c r="J541" t="b">
+        <v>0</v>
+      </c>
+      <c r="K541" t="n">
+        <v>135000000</v>
+      </c>
+      <c r="L541" t="b">
+        <v>0</v>
+      </c>
+      <c r="M541" t="n">
+        <v>128</v>
+      </c>
+      <c r="N541" t="n">
+        <v>0</v>
+      </c>
+      <c r="O541" t="n">
+        <v>0</v>
+      </c>
+      <c r="P541" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Die Another Day</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>card_541</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Lee Tamahori</t>
+        </is>
+      </c>
+      <c r="D542" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E542" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="F542" t="n">
+        <v>55</v>
+      </c>
+      <c r="I542" t="n">
+        <v>432000000</v>
+      </c>
+      <c r="J542" t="b">
+        <v>0</v>
+      </c>
+      <c r="K542" t="n">
+        <v>142000000</v>
+      </c>
+      <c r="L542" t="b">
+        <v>0</v>
+      </c>
+      <c r="M542" t="n">
+        <v>133</v>
+      </c>
+      <c r="N542" t="n">
+        <v>0</v>
+      </c>
+      <c r="O542" t="n">
+        <v>0</v>
+      </c>
+      <c r="P542" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Casino Royale</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>card_542</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Martin Campbell</t>
+        </is>
+      </c>
+      <c r="D543" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E543" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F543" t="n">
+        <v>84</v>
+      </c>
+      <c r="I543" t="n">
+        <v>606000000</v>
+      </c>
+      <c r="J543" t="b">
+        <v>0</v>
+      </c>
+      <c r="K543" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L543" t="b">
+        <v>0</v>
+      </c>
+      <c r="M543" t="n">
+        <v>144</v>
+      </c>
+      <c r="N543" t="n">
+        <v>0</v>
+      </c>
+      <c r="O543" t="n">
+        <v>0</v>
+      </c>
+      <c r="P543" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Quantum of Solace</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>card_543</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Marc Forster</t>
+        </is>
+      </c>
+      <c r="D544" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E544" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="F544" t="n">
+        <v>62</v>
+      </c>
+      <c r="I544" t="n">
+        <v>589600000</v>
+      </c>
+      <c r="J544" t="b">
+        <v>0</v>
+      </c>
+      <c r="K544" t="n">
+        <v>230000000</v>
+      </c>
+      <c r="L544" t="b">
+        <v>0</v>
+      </c>
+      <c r="M544" t="n">
+        <v>106</v>
+      </c>
+      <c r="N544" t="n">
+        <v>0</v>
+      </c>
+      <c r="O544" t="n">
+        <v>0</v>
+      </c>
+      <c r="P544" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Skyfall</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>card_544</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Sam Mendes</t>
+        </is>
+      </c>
+      <c r="D545" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E545" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="F545" t="n">
+        <v>76</v>
+      </c>
+      <c r="I545" t="n">
+        <v>1109000000</v>
+      </c>
+      <c r="J545" t="b">
+        <v>0</v>
+      </c>
+      <c r="K545" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L545" t="b">
+        <v>0</v>
+      </c>
+      <c r="M545" t="n">
+        <v>143</v>
+      </c>
+      <c r="N545" t="n">
+        <v>2</v>
+      </c>
+      <c r="O545" t="n">
+        <v>0</v>
+      </c>
+      <c r="P545" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Spectre</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>card_545</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Sam Mendes</t>
+        </is>
+      </c>
+      <c r="D546" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E546" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="F546" t="n">
+        <v>65</v>
+      </c>
+      <c r="I546" t="n">
+        <v>880700000</v>
+      </c>
+      <c r="J546" t="b">
+        <v>0</v>
+      </c>
+      <c r="K546" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="L546" t="b">
+        <v>0</v>
+      </c>
+      <c r="M546" t="n">
+        <v>148</v>
+      </c>
+      <c r="N546" t="n">
+        <v>1</v>
+      </c>
+      <c r="O546" t="n">
+        <v>0</v>
+      </c>
+      <c r="P546" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>No Time to Die</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>card_546</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Cary Joji Fukunaga</t>
+        </is>
+      </c>
+      <c r="D547" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E547" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F547" t="n">
+        <v>63</v>
+      </c>
+      <c r="I547" t="n">
+        <v>774200000</v>
+      </c>
+      <c r="J547" t="b">
+        <v>0</v>
+      </c>
+      <c r="K547" t="n">
+        <v>301000000</v>
+      </c>
+      <c r="L547" t="b">
+        <v>0</v>
+      </c>
+      <c r="M547" t="n">
+        <v>163</v>
+      </c>
+      <c r="N547" t="n">
+        <v>1</v>
+      </c>
+      <c r="O547" t="n">
+        <v>0</v>
+      </c>
+      <c r="P547" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing Batman films (card_547-552)
Batman (1989), Batman Returns, Batman Forever, Batman & Robin, Batman
v Superman: Dawn of Justice, The Batman.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P547"/>
+  <dimension ref="A1:P553"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -27757,1252 +27757,1552 @@
       </c>
     </row>
     <row r="523">
-      <c r="A523" t="inlineStr">
+      <c r="A523" s="10" t="inlineStr">
         <is>
           <t>Dr. No</t>
         </is>
       </c>
-      <c r="B523" t="inlineStr">
+      <c r="B523" s="10" t="inlineStr">
         <is>
           <t>card_522</t>
         </is>
       </c>
-      <c r="C523" t="inlineStr">
+      <c r="C523" s="10" t="inlineStr">
         <is>
           <t>Terence Young</t>
         </is>
       </c>
-      <c r="D523" t="n">
+      <c r="D523" s="10" t="n">
         <v>1962</v>
       </c>
-      <c r="E523" t="n">
+      <c r="E523" s="10" t="n">
         <v>3.41</v>
       </c>
-      <c r="F523" t="n">
+      <c r="F523" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I523" t="n">
+      <c r="I523" s="10" t="n">
         <v>59500000</v>
       </c>
-      <c r="J523" t="b">
-        <v>0</v>
-      </c>
-      <c r="K523" t="n">
+      <c r="J523" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K523" s="10" t="n">
         <v>1100000</v>
       </c>
-      <c r="L523" t="b">
-        <v>0</v>
-      </c>
-      <c r="M523" t="n">
+      <c r="L523" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M523" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N523" t="n">
-        <v>0</v>
-      </c>
-      <c r="O523" t="n">
-        <v>0</v>
-      </c>
-      <c r="P523" t="b">
+      <c r="N523" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O523" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P523" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="524">
-      <c r="A524" t="inlineStr">
+      <c r="A524" s="10" t="inlineStr">
         <is>
           <t>From Russia with Love</t>
         </is>
       </c>
-      <c r="B524" t="inlineStr">
+      <c r="B524" s="10" t="inlineStr">
         <is>
           <t>card_523</t>
         </is>
       </c>
-      <c r="C524" t="inlineStr">
+      <c r="C524" s="10" t="inlineStr">
         <is>
           <t>Terence Young</t>
         </is>
       </c>
-      <c r="D524" t="n">
+      <c r="D524" s="10" t="n">
         <v>1963</v>
       </c>
-      <c r="E524" t="n">
+      <c r="E524" s="10" t="n">
         <v>3.59</v>
       </c>
-      <c r="F524" t="n">
+      <c r="F524" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I524" t="n">
+      <c r="I524" s="10" t="n">
         <v>79000000</v>
       </c>
-      <c r="J524" t="b">
-        <v>0</v>
-      </c>
-      <c r="K524" t="n">
+      <c r="J524" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K524" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="L524" t="b">
-        <v>0</v>
-      </c>
-      <c r="M524" t="n">
+      <c r="L524" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M524" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N524" t="n">
-        <v>0</v>
-      </c>
-      <c r="O524" t="n">
-        <v>0</v>
-      </c>
-      <c r="P524" t="b">
+      <c r="N524" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O524" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P524" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="525">
-      <c r="A525" t="inlineStr">
+      <c r="A525" s="10" t="inlineStr">
         <is>
           <t>Goldfinger</t>
         </is>
       </c>
-      <c r="B525" t="inlineStr">
+      <c r="B525" s="10" t="inlineStr">
         <is>
           <t>card_524</t>
         </is>
       </c>
-      <c r="C525" t="inlineStr">
+      <c r="C525" s="10" t="inlineStr">
         <is>
           <t>Guy Hamilton</t>
         </is>
       </c>
-      <c r="D525" t="n">
+      <c r="D525" s="10" t="n">
         <v>1964</v>
       </c>
-      <c r="E525" t="n">
+      <c r="E525" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F525" t="n">
+      <c r="F525" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I525" t="n">
+      <c r="I525" s="10" t="n">
         <v>124900000</v>
       </c>
-      <c r="J525" t="b">
-        <v>0</v>
-      </c>
-      <c r="K525" t="n">
+      <c r="J525" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K525" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="L525" t="b">
-        <v>0</v>
-      </c>
-      <c r="M525" t="n">
+      <c r="L525" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M525" s="10" t="n">
         <v>110</v>
       </c>
-      <c r="N525" t="n">
+      <c r="N525" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O525" t="n">
-        <v>0</v>
-      </c>
-      <c r="P525" t="b">
+      <c r="O525" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P525" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="526">
-      <c r="A526" t="inlineStr">
+      <c r="A526" s="10" t="inlineStr">
         <is>
           <t>Thunderball</t>
         </is>
       </c>
-      <c r="B526" t="inlineStr">
+      <c r="B526" s="10" t="inlineStr">
         <is>
           <t>card_525</t>
         </is>
       </c>
-      <c r="C526" t="inlineStr">
+      <c r="C526" s="10" t="inlineStr">
         <is>
           <t>Terence Young</t>
         </is>
       </c>
-      <c r="D526" t="n">
+      <c r="D526" s="10" t="n">
         <v>1965</v>
       </c>
-      <c r="E526" t="n">
+      <c r="E526" s="10" t="n">
         <v>3.21</v>
       </c>
-      <c r="F526" t="n">
+      <c r="F526" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I526" t="n">
+      <c r="I526" s="10" t="n">
         <v>141200000</v>
       </c>
-      <c r="J526" t="b">
-        <v>0</v>
-      </c>
-      <c r="K526" t="n">
+      <c r="J526" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K526" s="10" t="n">
         <v>9000000</v>
       </c>
-      <c r="L526" t="b">
-        <v>0</v>
-      </c>
-      <c r="M526" t="n">
+      <c r="L526" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M526" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N526" t="n">
+      <c r="N526" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O526" t="n">
-        <v>0</v>
-      </c>
-      <c r="P526" t="b">
+      <c r="O526" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P526" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="527">
-      <c r="A527" t="inlineStr">
+      <c r="A527" s="10" t="inlineStr">
         <is>
           <t>You Only Live Twice</t>
         </is>
       </c>
-      <c r="B527" t="inlineStr">
+      <c r="B527" s="10" t="inlineStr">
         <is>
           <t>card_526</t>
         </is>
       </c>
-      <c r="C527" t="inlineStr">
+      <c r="C527" s="10" t="inlineStr">
         <is>
           <t>Lewis Gilbert</t>
         </is>
       </c>
-      <c r="D527" t="n">
+      <c r="D527" s="10" t="n">
         <v>1967</v>
       </c>
-      <c r="E527" t="n">
+      <c r="E527" s="10" t="n">
         <v>3.19</v>
       </c>
-      <c r="F527" t="n">
+      <c r="F527" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I527" t="n">
+      <c r="I527" s="10" t="n">
         <v>111600000</v>
       </c>
-      <c r="J527" t="b">
-        <v>0</v>
-      </c>
-      <c r="K527" t="n">
+      <c r="J527" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K527" s="10" t="n">
         <v>9500000</v>
       </c>
-      <c r="L527" t="b">
-        <v>0</v>
-      </c>
-      <c r="M527" t="n">
+      <c r="L527" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M527" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N527" t="n">
-        <v>0</v>
-      </c>
-      <c r="O527" t="n">
-        <v>0</v>
-      </c>
-      <c r="P527" t="b">
+      <c r="N527" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O527" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P527" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="528">
-      <c r="A528" t="inlineStr">
+      <c r="A528" s="10" t="inlineStr">
         <is>
           <t>On Her Majesty's Secret Service</t>
         </is>
       </c>
-      <c r="B528" t="inlineStr">
+      <c r="B528" s="10" t="inlineStr">
         <is>
           <t>card_527</t>
         </is>
       </c>
-      <c r="C528" t="inlineStr">
+      <c r="C528" s="10" t="inlineStr">
         <is>
           <t>Peter R. Hunt</t>
         </is>
       </c>
-      <c r="D528" t="n">
+      <c r="D528" s="10" t="n">
         <v>1969</v>
       </c>
-      <c r="E528" t="n">
+      <c r="E528" s="10" t="n">
         <v>3.44</v>
       </c>
-      <c r="F528" t="n">
+      <c r="F528" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I528" t="n">
+      <c r="I528" s="10" t="n">
         <v>82000000</v>
       </c>
-      <c r="J528" t="b">
-        <v>0</v>
-      </c>
-      <c r="K528" t="n">
+      <c r="J528" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K528" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="L528" t="b">
-        <v>0</v>
-      </c>
-      <c r="M528" t="n">
+      <c r="L528" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M528" s="10" t="n">
         <v>142</v>
       </c>
-      <c r="N528" t="n">
-        <v>0</v>
-      </c>
-      <c r="O528" t="n">
-        <v>0</v>
-      </c>
-      <c r="P528" t="b">
+      <c r="N528" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O528" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P528" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="529">
-      <c r="A529" t="inlineStr">
+      <c r="A529" s="10" t="inlineStr">
         <is>
           <t>Diamonds Are Forever</t>
         </is>
       </c>
-      <c r="B529" t="inlineStr">
+      <c r="B529" s="10" t="inlineStr">
         <is>
           <t>card_528</t>
         </is>
       </c>
-      <c r="C529" t="inlineStr">
+      <c r="C529" s="10" t="inlineStr">
         <is>
           <t>Guy Hamilton</t>
         </is>
       </c>
-      <c r="D529" t="n">
+      <c r="D529" s="10" t="n">
         <v>1971</v>
       </c>
-      <c r="E529" t="n">
+      <c r="E529" s="10" t="n">
         <v>2.86</v>
       </c>
-      <c r="F529" t="n">
+      <c r="F529" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I529" t="n">
+      <c r="I529" s="10" t="n">
         <v>116000000</v>
       </c>
-      <c r="J529" t="b">
-        <v>0</v>
-      </c>
-      <c r="K529" t="n">
+      <c r="J529" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K529" s="10" t="n">
         <v>7200000</v>
       </c>
-      <c r="L529" t="b">
-        <v>0</v>
-      </c>
-      <c r="M529" t="n">
+      <c r="L529" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M529" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="N529" t="n">
-        <v>0</v>
-      </c>
-      <c r="O529" t="n">
-        <v>0</v>
-      </c>
-      <c r="P529" t="b">
+      <c r="N529" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O529" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P529" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="530">
-      <c r="A530" t="inlineStr">
+      <c r="A530" s="10" t="inlineStr">
         <is>
           <t>Live and Let Die</t>
         </is>
       </c>
-      <c r="B530" t="inlineStr">
+      <c r="B530" s="10" t="inlineStr">
         <is>
           <t>card_529</t>
         </is>
       </c>
-      <c r="C530" t="inlineStr">
+      <c r="C530" s="10" t="inlineStr">
         <is>
           <t>Guy Hamilton</t>
         </is>
       </c>
-      <c r="D530" t="n">
+      <c r="D530" s="10" t="n">
         <v>1973</v>
       </c>
-      <c r="E530" t="n">
+      <c r="E530" s="10" t="n">
         <v>3.17</v>
       </c>
-      <c r="F530" t="n">
+      <c r="F530" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I530" t="n">
+      <c r="I530" s="10" t="n">
         <v>161800000</v>
       </c>
-      <c r="J530" t="b">
-        <v>0</v>
-      </c>
-      <c r="K530" t="n">
+      <c r="J530" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K530" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="L530" t="b">
-        <v>0</v>
-      </c>
-      <c r="M530" t="n">
+      <c r="L530" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M530" s="10" t="n">
         <v>121</v>
       </c>
-      <c r="N530" t="n">
-        <v>0</v>
-      </c>
-      <c r="O530" t="n">
-        <v>0</v>
-      </c>
-      <c r="P530" t="b">
+      <c r="N530" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O530" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P530" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="531">
-      <c r="A531" t="inlineStr">
+      <c r="A531" s="10" t="inlineStr">
         <is>
           <t>The Man with the Golden Gun</t>
         </is>
       </c>
-      <c r="B531" t="inlineStr">
+      <c r="B531" s="10" t="inlineStr">
         <is>
           <t>card_530</t>
         </is>
       </c>
-      <c r="C531" t="inlineStr">
+      <c r="C531" s="10" t="inlineStr">
         <is>
           <t>Guy Hamilton</t>
         </is>
       </c>
-      <c r="D531" t="n">
+      <c r="D531" s="10" t="n">
         <v>1974</v>
       </c>
-      <c r="E531" t="n">
+      <c r="E531" s="10" t="n">
         <v>3.12</v>
       </c>
-      <c r="F531" t="n">
+      <c r="F531" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I531" t="n">
+      <c r="I531" s="10" t="n">
         <v>97600000</v>
       </c>
-      <c r="J531" t="b">
-        <v>0</v>
-      </c>
-      <c r="K531" t="n">
+      <c r="J531" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K531" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="L531" t="b">
-        <v>0</v>
-      </c>
-      <c r="M531" t="n">
+      <c r="L531" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M531" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="N531" t="n">
-        <v>0</v>
-      </c>
-      <c r="O531" t="n">
-        <v>0</v>
-      </c>
-      <c r="P531" t="b">
+      <c r="N531" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O531" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P531" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="532">
-      <c r="A532" t="inlineStr">
+      <c r="A532" s="10" t="inlineStr">
         <is>
           <t>The Spy Who Loved Me</t>
         </is>
       </c>
-      <c r="B532" t="inlineStr">
+      <c r="B532" s="10" t="inlineStr">
         <is>
           <t>card_531</t>
         </is>
       </c>
-      <c r="C532" t="inlineStr">
+      <c r="C532" s="10" t="inlineStr">
         <is>
           <t>Lewis Gilbert</t>
         </is>
       </c>
-      <c r="D532" t="n">
+      <c r="D532" s="10" t="n">
         <v>1977</v>
       </c>
-      <c r="E532" t="n">
+      <c r="E532" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="F532" t="n">
+      <c r="F532" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I532" t="n">
+      <c r="I532" s="10" t="n">
         <v>185400000</v>
       </c>
-      <c r="J532" t="b">
-        <v>0</v>
-      </c>
-      <c r="K532" t="n">
+      <c r="J532" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K532" s="10" t="n">
         <v>13500000</v>
       </c>
-      <c r="L532" t="b">
-        <v>0</v>
-      </c>
-      <c r="M532" t="n">
+      <c r="L532" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M532" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="N532" t="n">
-        <v>0</v>
-      </c>
-      <c r="O532" t="n">
-        <v>0</v>
-      </c>
-      <c r="P532" t="b">
+      <c r="N532" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O532" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P532" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="533">
-      <c r="A533" t="inlineStr">
+      <c r="A533" s="10" t="inlineStr">
         <is>
           <t>Moonraker</t>
         </is>
       </c>
-      <c r="B533" t="inlineStr">
+      <c r="B533" s="10" t="inlineStr">
         <is>
           <t>card_532</t>
         </is>
       </c>
-      <c r="C533" t="inlineStr">
+      <c r="C533" s="10" t="inlineStr">
         <is>
           <t>Lewis Gilbert</t>
         </is>
       </c>
-      <c r="D533" t="n">
+      <c r="D533" s="10" t="n">
         <v>1979</v>
       </c>
-      <c r="E533" t="n">
+      <c r="E533" s="10" t="n">
         <v>2.87</v>
       </c>
-      <c r="F533" t="n">
+      <c r="F533" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I533" t="n">
+      <c r="I533" s="10" t="n">
         <v>210300000</v>
       </c>
-      <c r="J533" t="b">
-        <v>0</v>
-      </c>
-      <c r="K533" t="n">
+      <c r="J533" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K533" s="10" t="n">
         <v>34000000</v>
       </c>
-      <c r="L533" t="b">
-        <v>0</v>
-      </c>
-      <c r="M533" t="n">
+      <c r="L533" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M533" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="N533" t="n">
-        <v>0</v>
-      </c>
-      <c r="O533" t="n">
-        <v>0</v>
-      </c>
-      <c r="P533" t="b">
+      <c r="N533" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O533" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P533" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="534">
-      <c r="A534" t="inlineStr">
+      <c r="A534" s="10" t="inlineStr">
         <is>
           <t>For Your Eyes Only</t>
         </is>
       </c>
-      <c r="B534" t="inlineStr">
+      <c r="B534" s="10" t="inlineStr">
         <is>
           <t>card_533</t>
         </is>
       </c>
-      <c r="C534" t="inlineStr">
+      <c r="C534" s="10" t="inlineStr">
         <is>
           <t>John Glen</t>
         </is>
       </c>
-      <c r="D534" t="n">
+      <c r="D534" s="10" t="n">
         <v>1981</v>
       </c>
-      <c r="E534" t="n">
+      <c r="E534" s="10" t="n">
         <v>3.1</v>
       </c>
-      <c r="F534" t="n">
+      <c r="F534" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="I534" t="n">
+      <c r="I534" s="10" t="n">
         <v>202800000</v>
       </c>
-      <c r="J534" t="b">
-        <v>0</v>
-      </c>
-      <c r="K534" t="n">
+      <c r="J534" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K534" s="10" t="n">
         <v>28000000</v>
       </c>
-      <c r="L534" t="b">
-        <v>0</v>
-      </c>
-      <c r="M534" t="n">
+      <c r="L534" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M534" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="N534" t="n">
-        <v>0</v>
-      </c>
-      <c r="O534" t="n">
-        <v>0</v>
-      </c>
-      <c r="P534" t="b">
+      <c r="N534" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O534" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P534" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="535">
-      <c r="A535" t="inlineStr">
+      <c r="A535" s="10" t="inlineStr">
         <is>
           <t>Octopussy</t>
         </is>
       </c>
-      <c r="B535" t="inlineStr">
+      <c r="B535" s="10" t="inlineStr">
         <is>
           <t>card_534</t>
         </is>
       </c>
-      <c r="C535" t="inlineStr">
+      <c r="C535" s="10" t="inlineStr">
         <is>
           <t>John Glen</t>
         </is>
       </c>
-      <c r="D535" t="n">
+      <c r="D535" s="10" t="n">
         <v>1983</v>
       </c>
-      <c r="E535" t="n">
+      <c r="E535" s="10" t="n">
         <v>2.91</v>
       </c>
-      <c r="F535" t="n">
+      <c r="F535" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I535" t="n">
+      <c r="I535" s="10" t="n">
         <v>187500000</v>
       </c>
-      <c r="J535" t="b">
-        <v>0</v>
-      </c>
-      <c r="K535" t="n">
+      <c r="J535" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K535" s="10" t="n">
         <v>27500000</v>
       </c>
-      <c r="L535" t="b">
-        <v>0</v>
-      </c>
-      <c r="M535" t="n">
+      <c r="L535" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M535" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N535" t="n">
-        <v>0</v>
-      </c>
-      <c r="O535" t="n">
-        <v>0</v>
-      </c>
-      <c r="P535" t="b">
+      <c r="N535" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O535" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P535" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="536">
-      <c r="A536" t="inlineStr">
+      <c r="A536" s="10" t="inlineStr">
         <is>
           <t>A View to a Kill</t>
         </is>
       </c>
-      <c r="B536" t="inlineStr">
+      <c r="B536" s="10" t="inlineStr">
         <is>
           <t>card_535</t>
         </is>
       </c>
-      <c r="C536" t="inlineStr">
+      <c r="C536" s="10" t="inlineStr">
         <is>
           <t>John Glen</t>
         </is>
       </c>
-      <c r="D536" t="n">
+      <c r="D536" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E536" t="n">
+      <c r="E536" s="10" t="n">
         <v>2.89</v>
       </c>
-      <c r="F536" t="n">
+      <c r="F536" s="10" t="n">
         <v>57</v>
       </c>
-      <c r="I536" t="n">
+      <c r="I536" s="10" t="n">
         <v>152400000</v>
       </c>
-      <c r="J536" t="b">
-        <v>0</v>
-      </c>
-      <c r="K536" t="n">
+      <c r="J536" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K536" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L536" t="b">
-        <v>0</v>
-      </c>
-      <c r="M536" t="n">
+      <c r="L536" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M536" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N536" t="n">
-        <v>0</v>
-      </c>
-      <c r="O536" t="n">
-        <v>0</v>
-      </c>
-      <c r="P536" t="b">
+      <c r="N536" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O536" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P536" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="537">
-      <c r="A537" t="inlineStr">
+      <c r="A537" s="10" t="inlineStr">
         <is>
           <t>The Living Daylights</t>
         </is>
       </c>
-      <c r="B537" t="inlineStr">
+      <c r="B537" s="10" t="inlineStr">
         <is>
           <t>card_536</t>
         </is>
       </c>
-      <c r="C537" t="inlineStr">
+      <c r="C537" s="10" t="inlineStr">
         <is>
           <t>John Glen</t>
         </is>
       </c>
-      <c r="D537" t="n">
+      <c r="D537" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E537" t="n">
+      <c r="E537" s="10" t="n">
         <v>3.35</v>
       </c>
-      <c r="F537" t="n">
+      <c r="F537" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I537" t="n">
+      <c r="I537" s="10" t="n">
         <v>191200000</v>
       </c>
-      <c r="J537" t="b">
-        <v>0</v>
-      </c>
-      <c r="K537" t="n">
+      <c r="J537" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K537" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L537" t="b">
-        <v>0</v>
-      </c>
-      <c r="M537" t="n">
+      <c r="L537" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M537" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N537" t="n">
-        <v>0</v>
-      </c>
-      <c r="O537" t="n">
-        <v>0</v>
-      </c>
-      <c r="P537" t="b">
+      <c r="N537" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O537" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P537" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="538">
-      <c r="A538" t="inlineStr">
+      <c r="A538" s="10" t="inlineStr">
         <is>
           <t>Licence to Kill</t>
         </is>
       </c>
-      <c r="B538" t="inlineStr">
+      <c r="B538" s="10" t="inlineStr">
         <is>
           <t>card_537</t>
         </is>
       </c>
-      <c r="C538" t="inlineStr">
+      <c r="C538" s="10" t="inlineStr">
         <is>
           <t>John Glen</t>
         </is>
       </c>
-      <c r="D538" t="n">
+      <c r="D538" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E538" t="n">
+      <c r="E538" s="10" t="n">
         <v>3.38</v>
       </c>
-      <c r="F538" t="n">
+      <c r="F538" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I538" t="n">
+      <c r="I538" s="10" t="n">
         <v>156100000</v>
       </c>
-      <c r="J538" t="b">
-        <v>0</v>
-      </c>
-      <c r="K538" t="n">
+      <c r="J538" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K538" s="10" t="n">
         <v>32000000</v>
       </c>
-      <c r="L538" t="b">
-        <v>0</v>
-      </c>
-      <c r="M538" t="n">
+      <c r="L538" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M538" s="10" t="n">
         <v>133</v>
       </c>
-      <c r="N538" t="n">
-        <v>0</v>
-      </c>
-      <c r="O538" t="n">
-        <v>0</v>
-      </c>
-      <c r="P538" t="b">
+      <c r="N538" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O538" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P538" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="539">
-      <c r="A539" t="inlineStr">
+      <c r="A539" s="10" t="inlineStr">
         <is>
           <t>GoldenEye</t>
         </is>
       </c>
-      <c r="B539" t="inlineStr">
+      <c r="B539" s="10" t="inlineStr">
         <is>
           <t>card_538</t>
         </is>
       </c>
-      <c r="C539" t="inlineStr">
+      <c r="C539" s="10" t="inlineStr">
         <is>
           <t>Martin Campbell</t>
         </is>
       </c>
-      <c r="D539" t="n">
+      <c r="D539" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E539" t="n">
+      <c r="E539" s="10" t="n">
         <v>3.58</v>
       </c>
-      <c r="F539" t="n">
+      <c r="F539" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I539" t="n">
+      <c r="I539" s="10" t="n">
         <v>356400000</v>
       </c>
-      <c r="J539" t="b">
-        <v>0</v>
-      </c>
-      <c r="K539" t="n">
+      <c r="J539" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K539" s="10" t="n">
         <v>60000000</v>
       </c>
-      <c r="L539" t="b">
-        <v>0</v>
-      </c>
-      <c r="M539" t="n">
+      <c r="L539" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M539" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N539" t="n">
-        <v>0</v>
-      </c>
-      <c r="O539" t="n">
-        <v>0</v>
-      </c>
-      <c r="P539" t="b">
+      <c r="N539" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O539" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P539" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="540">
-      <c r="A540" t="inlineStr">
+      <c r="A540" s="10" t="inlineStr">
         <is>
           <t>Tomorrow Never Dies</t>
         </is>
       </c>
-      <c r="B540" t="inlineStr">
+      <c r="B540" s="10" t="inlineStr">
         <is>
           <t>card_539</t>
         </is>
       </c>
-      <c r="C540" t="inlineStr">
+      <c r="C540" s="10" t="inlineStr">
         <is>
           <t>Roger Spottiswoode</t>
         </is>
       </c>
-      <c r="D540" t="n">
+      <c r="D540" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E540" t="n">
+      <c r="E540" s="10" t="n">
         <v>3.11</v>
       </c>
-      <c r="F540" t="n">
+      <c r="F540" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I540" t="n">
+      <c r="I540" s="10" t="n">
         <v>339500000</v>
       </c>
-      <c r="J540" t="b">
-        <v>0</v>
-      </c>
-      <c r="K540" t="n">
+      <c r="J540" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K540" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L540" t="b">
-        <v>0</v>
-      </c>
-      <c r="M540" t="n">
+      <c r="L540" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M540" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="N540" t="n">
-        <v>0</v>
-      </c>
-      <c r="O540" t="n">
-        <v>0</v>
-      </c>
-      <c r="P540" t="b">
+      <c r="N540" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O540" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P540" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="541">
-      <c r="A541" t="inlineStr">
+      <c r="A541" s="10" t="inlineStr">
         <is>
           <t>The World Is Not Enough</t>
         </is>
       </c>
-      <c r="B541" t="inlineStr">
+      <c r="B541" s="10" t="inlineStr">
         <is>
           <t>card_540</t>
         </is>
       </c>
-      <c r="C541" t="inlineStr">
+      <c r="C541" s="10" t="inlineStr">
         <is>
           <t>Michael Apted</t>
         </is>
       </c>
-      <c r="D541" t="n">
+      <c r="D541" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E541" t="n">
+      <c r="E541" s="10" t="n">
         <v>2.94</v>
       </c>
-      <c r="F541" t="n">
+      <c r="F541" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I541" t="n">
+      <c r="I541" s="10" t="n">
         <v>361000000</v>
       </c>
-      <c r="J541" t="b">
-        <v>0</v>
-      </c>
-      <c r="K541" t="n">
+      <c r="J541" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K541" s="10" t="n">
         <v>135000000</v>
       </c>
-      <c r="L541" t="b">
-        <v>0</v>
-      </c>
-      <c r="M541" t="n">
+      <c r="L541" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M541" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N541" t="n">
-        <v>0</v>
-      </c>
-      <c r="O541" t="n">
-        <v>0</v>
-      </c>
-      <c r="P541" t="b">
+      <c r="N541" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O541" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P541" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="542">
-      <c r="A542" t="inlineStr">
+      <c r="A542" s="10" t="inlineStr">
         <is>
           <t>Die Another Day</t>
         </is>
       </c>
-      <c r="B542" t="inlineStr">
+      <c r="B542" s="10" t="inlineStr">
         <is>
           <t>card_541</t>
         </is>
       </c>
-      <c r="C542" t="inlineStr">
+      <c r="C542" s="10" t="inlineStr">
         <is>
           <t>Lee Tamahori</t>
         </is>
       </c>
-      <c r="D542" t="n">
+      <c r="D542" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E542" t="n">
+      <c r="E542" s="10" t="n">
         <v>2.59</v>
       </c>
-      <c r="F542" t="n">
+      <c r="F542" s="10" t="n">
         <v>55</v>
       </c>
-      <c r="I542" t="n">
+      <c r="I542" s="10" t="n">
         <v>432000000</v>
       </c>
-      <c r="J542" t="b">
-        <v>0</v>
-      </c>
-      <c r="K542" t="n">
+      <c r="J542" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K542" s="10" t="n">
         <v>142000000</v>
       </c>
-      <c r="L542" t="b">
-        <v>0</v>
-      </c>
-      <c r="M542" t="n">
+      <c r="L542" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M542" s="10" t="n">
         <v>133</v>
       </c>
-      <c r="N542" t="n">
-        <v>0</v>
-      </c>
-      <c r="O542" t="n">
-        <v>0</v>
-      </c>
-      <c r="P542" t="b">
+      <c r="N542" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O542" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P542" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="543">
-      <c r="A543" t="inlineStr">
+      <c r="A543" s="10" t="inlineStr">
         <is>
           <t>Casino Royale</t>
         </is>
       </c>
-      <c r="B543" t="inlineStr">
+      <c r="B543" s="10" t="inlineStr">
         <is>
           <t>card_542</t>
         </is>
       </c>
-      <c r="C543" t="inlineStr">
+      <c r="C543" s="10" t="inlineStr">
         <is>
           <t>Martin Campbell</t>
         </is>
       </c>
-      <c r="D543" t="n">
+      <c r="D543" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E543" t="n">
+      <c r="E543" s="10" t="n">
         <v>4.04</v>
       </c>
-      <c r="F543" t="n">
+      <c r="F543" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="I543" t="n">
+      <c r="I543" s="10" t="n">
         <v>606000000</v>
       </c>
-      <c r="J543" t="b">
-        <v>0</v>
-      </c>
-      <c r="K543" t="n">
+      <c r="J543" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K543" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L543" t="b">
-        <v>0</v>
-      </c>
-      <c r="M543" t="n">
+      <c r="L543" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M543" s="10" t="n">
         <v>144</v>
       </c>
-      <c r="N543" t="n">
-        <v>0</v>
-      </c>
-      <c r="O543" t="n">
-        <v>0</v>
-      </c>
-      <c r="P543" t="b">
+      <c r="N543" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O543" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P543" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="544">
-      <c r="A544" t="inlineStr">
+      <c r="A544" s="10" t="inlineStr">
         <is>
           <t>Quantum of Solace</t>
         </is>
       </c>
-      <c r="B544" t="inlineStr">
+      <c r="B544" s="10" t="inlineStr">
         <is>
           <t>card_543</t>
         </is>
       </c>
-      <c r="C544" t="inlineStr">
+      <c r="C544" s="10" t="inlineStr">
         <is>
           <t>Marc Forster</t>
         </is>
       </c>
-      <c r="D544" t="n">
+      <c r="D544" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E544" t="n">
+      <c r="E544" s="10" t="n">
         <v>2.88</v>
       </c>
-      <c r="F544" t="n">
+      <c r="F544" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I544" t="n">
+      <c r="I544" s="10" t="n">
         <v>589600000</v>
       </c>
-      <c r="J544" t="b">
-        <v>0</v>
-      </c>
-      <c r="K544" t="n">
+      <c r="J544" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K544" s="10" t="n">
         <v>230000000</v>
       </c>
-      <c r="L544" t="b">
-        <v>0</v>
-      </c>
-      <c r="M544" t="n">
+      <c r="L544" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M544" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="N544" t="n">
-        <v>0</v>
-      </c>
-      <c r="O544" t="n">
-        <v>0</v>
-      </c>
-      <c r="P544" t="b">
+      <c r="N544" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O544" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P544" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="545">
-      <c r="A545" t="inlineStr">
+      <c r="A545" s="10" t="inlineStr">
         <is>
           <t>Skyfall</t>
         </is>
       </c>
-      <c r="B545" t="inlineStr">
+      <c r="B545" s="10" t="inlineStr">
         <is>
           <t>card_544</t>
         </is>
       </c>
-      <c r="C545" t="inlineStr">
+      <c r="C545" s="10" t="inlineStr">
         <is>
           <t>Sam Mendes</t>
         </is>
       </c>
-      <c r="D545" t="n">
+      <c r="D545" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E545" t="n">
+      <c r="E545" s="10" t="n">
         <v>3.96</v>
       </c>
-      <c r="F545" t="n">
+      <c r="F545" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I545" t="n">
+      <c r="I545" s="10" t="n">
         <v>1109000000</v>
       </c>
-      <c r="J545" t="b">
-        <v>0</v>
-      </c>
-      <c r="K545" t="n">
+      <c r="J545" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K545" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L545" t="b">
-        <v>0</v>
-      </c>
-      <c r="M545" t="n">
+      <c r="L545" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M545" s="10" t="n">
         <v>143</v>
       </c>
-      <c r="N545" t="n">
+      <c r="N545" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O545" t="n">
-        <v>0</v>
-      </c>
-      <c r="P545" t="b">
+      <c r="O545" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P545" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="546">
-      <c r="A546" t="inlineStr">
+      <c r="A546" s="10" t="inlineStr">
         <is>
           <t>Spectre</t>
         </is>
       </c>
-      <c r="B546" t="inlineStr">
+      <c r="B546" s="10" t="inlineStr">
         <is>
           <t>card_545</t>
         </is>
       </c>
-      <c r="C546" t="inlineStr">
+      <c r="C546" s="10" t="inlineStr">
         <is>
           <t>Sam Mendes</t>
         </is>
       </c>
-      <c r="D546" t="n">
+      <c r="D546" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E546" t="n">
+      <c r="E546" s="10" t="n">
         <v>3.16</v>
       </c>
-      <c r="F546" t="n">
+      <c r="F546" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="I546" t="n">
+      <c r="I546" s="10" t="n">
         <v>880700000</v>
       </c>
-      <c r="J546" t="b">
-        <v>0</v>
-      </c>
-      <c r="K546" t="n">
+      <c r="J546" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K546" s="10" t="n">
         <v>300000000</v>
       </c>
-      <c r="L546" t="b">
-        <v>0</v>
-      </c>
-      <c r="M546" t="n">
+      <c r="L546" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M546" s="10" t="n">
         <v>148</v>
       </c>
-      <c r="N546" t="n">
+      <c r="N546" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O546" t="n">
-        <v>0</v>
-      </c>
-      <c r="P546" t="b">
+      <c r="O546" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P546" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="547">
-      <c r="A547" t="inlineStr">
+      <c r="A547" s="10" t="inlineStr">
         <is>
           <t>No Time to Die</t>
         </is>
       </c>
-      <c r="B547" t="inlineStr">
+      <c r="B547" s="10" t="inlineStr">
         <is>
           <t>card_546</t>
         </is>
       </c>
-      <c r="C547" t="inlineStr">
+      <c r="C547" s="10" t="inlineStr">
         <is>
           <t>Cary Joji Fukunaga</t>
         </is>
       </c>
-      <c r="D547" t="n">
+      <c r="D547" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E547" t="n">
+      <c r="E547" s="10" t="n">
         <v>3.56</v>
       </c>
-      <c r="F547" t="n">
+      <c r="F547" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I547" t="n">
+      <c r="I547" s="10" t="n">
         <v>774200000</v>
       </c>
-      <c r="J547" t="b">
-        <v>0</v>
-      </c>
-      <c r="K547" t="n">
+      <c r="J547" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K547" s="10" t="n">
         <v>301000000</v>
       </c>
-      <c r="L547" t="b">
-        <v>0</v>
-      </c>
-      <c r="M547" t="n">
+      <c r="L547" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M547" s="10" t="n">
         <v>163</v>
       </c>
-      <c r="N547" t="n">
+      <c r="N547" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O547" t="n">
-        <v>0</v>
-      </c>
-      <c r="P547" t="b">
+      <c r="O547" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P547" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Batman</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>card_547</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Tim Burton</t>
+        </is>
+      </c>
+      <c r="D548" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E548" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F548" t="n">
+        <v>78</v>
+      </c>
+      <c r="I548" t="n">
+        <v>411600000</v>
+      </c>
+      <c r="J548" t="b">
+        <v>0</v>
+      </c>
+      <c r="K548" t="n">
+        <v>48000000</v>
+      </c>
+      <c r="L548" t="b">
+        <v>0</v>
+      </c>
+      <c r="M548" t="n">
+        <v>126</v>
+      </c>
+      <c r="N548" t="n">
+        <v>1</v>
+      </c>
+      <c r="O548" t="n">
+        <v>0</v>
+      </c>
+      <c r="P548" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Batman Returns</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>card_548</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Tim Burton</t>
+        </is>
+      </c>
+      <c r="D549" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E549" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F549" t="n">
+        <v>77</v>
+      </c>
+      <c r="I549" t="n">
+        <v>266800000</v>
+      </c>
+      <c r="J549" t="b">
+        <v>0</v>
+      </c>
+      <c r="K549" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="L549" t="b">
+        <v>0</v>
+      </c>
+      <c r="M549" t="n">
+        <v>126</v>
+      </c>
+      <c r="N549" t="n">
+        <v>0</v>
+      </c>
+      <c r="O549" t="n">
+        <v>0</v>
+      </c>
+      <c r="P549" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Batman Forever</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>card_549</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Joel Schumacher</t>
+        </is>
+      </c>
+      <c r="D550" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E550" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="F550" t="n">
+        <v>53</v>
+      </c>
+      <c r="I550" t="n">
+        <v>336600000</v>
+      </c>
+      <c r="J550" t="b">
+        <v>0</v>
+      </c>
+      <c r="K550" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L550" t="b">
+        <v>0</v>
+      </c>
+      <c r="M550" t="n">
+        <v>121</v>
+      </c>
+      <c r="N550" t="n">
+        <v>0</v>
+      </c>
+      <c r="O550" t="n">
+        <v>0</v>
+      </c>
+      <c r="P550" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Batman &amp; Robin</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>card_550</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Joel Schumacher</t>
+        </is>
+      </c>
+      <c r="D551" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E551" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="F551" t="n">
+        <v>30</v>
+      </c>
+      <c r="I551" t="n">
+        <v>238300000</v>
+      </c>
+      <c r="J551" t="b">
+        <v>0</v>
+      </c>
+      <c r="K551" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L551" t="b">
+        <v>0</v>
+      </c>
+      <c r="M551" t="n">
+        <v>125</v>
+      </c>
+      <c r="N551" t="n">
+        <v>0</v>
+      </c>
+      <c r="O551" t="n">
+        <v>0</v>
+      </c>
+      <c r="P551" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Batman v Superman: Dawn of Justice</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>card_551</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Zack Snyder</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E552" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F552" t="n">
+        <v>69</v>
+      </c>
+      <c r="I552" t="n">
+        <v>874400000</v>
+      </c>
+      <c r="J552" t="b">
+        <v>0</v>
+      </c>
+      <c r="K552" t="n">
+        <v>300000000</v>
+      </c>
+      <c r="L552" t="b">
+        <v>0</v>
+      </c>
+      <c r="M552" t="n">
+        <v>151</v>
+      </c>
+      <c r="N552" t="n">
+        <v>0</v>
+      </c>
+      <c r="O552" t="n">
+        <v>0</v>
+      </c>
+      <c r="P552" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>The Batman</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>card_552</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Matt Reeves</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E553" t="n">
+        <v>4.05</v>
+      </c>
+      <c r="F553" t="n">
+        <v>79</v>
+      </c>
+      <c r="I553" t="n">
+        <v>772300000</v>
+      </c>
+      <c r="J553" t="b">
+        <v>0</v>
+      </c>
+      <c r="K553" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L553" t="b">
+        <v>0</v>
+      </c>
+      <c r="M553" t="n">
+        <v>176</v>
+      </c>
+      <c r="N553" t="n">
+        <v>0</v>
+      </c>
+      <c r="O553" t="n">
+        <v>0</v>
+      </c>
+      <c r="P553" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add missing X-Men films (card_553-563)
X-Men through The New Mutants, 11 films (Deadpool 1-2 already in DB).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P553"/>
+  <dimension ref="A1:P564"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -29007,302 +29007,852 @@
       </c>
     </row>
     <row r="548">
-      <c r="A548" t="inlineStr">
+      <c r="A548" s="10" t="inlineStr">
         <is>
           <t>Batman</t>
         </is>
       </c>
-      <c r="B548" t="inlineStr">
+      <c r="B548" s="10" t="inlineStr">
         <is>
           <t>card_547</t>
         </is>
       </c>
-      <c r="C548" t="inlineStr">
+      <c r="C548" s="10" t="inlineStr">
         <is>
           <t>Tim Burton</t>
         </is>
       </c>
-      <c r="D548" t="n">
+      <c r="D548" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E548" t="n">
+      <c r="E548" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F548" t="n">
+      <c r="F548" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I548" t="n">
+      <c r="I548" s="10" t="n">
         <v>411600000</v>
       </c>
-      <c r="J548" t="b">
-        <v>0</v>
-      </c>
-      <c r="K548" t="n">
+      <c r="J548" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K548" s="10" t="n">
         <v>48000000</v>
       </c>
-      <c r="L548" t="b">
-        <v>0</v>
-      </c>
-      <c r="M548" t="n">
+      <c r="L548" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M548" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="N548" t="n">
+      <c r="N548" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O548" t="n">
-        <v>0</v>
-      </c>
-      <c r="P548" t="b">
+      <c r="O548" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P548" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="549">
-      <c r="A549" t="inlineStr">
+      <c r="A549" s="10" t="inlineStr">
         <is>
           <t>Batman Returns</t>
         </is>
       </c>
-      <c r="B549" t="inlineStr">
+      <c r="B549" s="10" t="inlineStr">
         <is>
           <t>card_548</t>
         </is>
       </c>
-      <c r="C549" t="inlineStr">
+      <c r="C549" s="10" t="inlineStr">
         <is>
           <t>Tim Burton</t>
         </is>
       </c>
-      <c r="D549" t="n">
+      <c r="D549" s="10" t="n">
         <v>1992</v>
       </c>
-      <c r="E549" t="n">
+      <c r="E549" s="10" t="n">
         <v>3.6</v>
       </c>
-      <c r="F549" t="n">
+      <c r="F549" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I549" t="n">
+      <c r="I549" s="10" t="n">
         <v>266800000</v>
       </c>
-      <c r="J549" t="b">
-        <v>0</v>
-      </c>
-      <c r="K549" t="n">
+      <c r="J549" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K549" s="10" t="n">
         <v>55000000</v>
       </c>
-      <c r="L549" t="b">
-        <v>0</v>
-      </c>
-      <c r="M549" t="n">
+      <c r="L549" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M549" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="N549" t="n">
-        <v>0</v>
-      </c>
-      <c r="O549" t="n">
-        <v>0</v>
-      </c>
-      <c r="P549" t="b">
+      <c r="N549" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O549" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P549" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="550">
-      <c r="A550" t="inlineStr">
+      <c r="A550" s="10" t="inlineStr">
         <is>
           <t>Batman Forever</t>
         </is>
       </c>
-      <c r="B550" t="inlineStr">
+      <c r="B550" s="10" t="inlineStr">
         <is>
           <t>card_549</t>
         </is>
       </c>
-      <c r="C550" t="inlineStr">
+      <c r="C550" s="10" t="inlineStr">
         <is>
           <t>Joel Schumacher</t>
         </is>
       </c>
-      <c r="D550" t="n">
+      <c r="D550" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E550" t="n">
+      <c r="E550" s="10" t="n">
         <v>2.58</v>
       </c>
-      <c r="F550" t="n">
+      <c r="F550" s="10" t="n">
         <v>53</v>
       </c>
-      <c r="I550" t="n">
+      <c r="I550" s="10" t="n">
         <v>336600000</v>
       </c>
-      <c r="J550" t="b">
-        <v>0</v>
-      </c>
-      <c r="K550" t="n">
+      <c r="J550" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K550" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L550" t="b">
-        <v>0</v>
-      </c>
-      <c r="M550" t="n">
+      <c r="L550" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M550" s="10" t="n">
         <v>121</v>
       </c>
-      <c r="N550" t="n">
-        <v>0</v>
-      </c>
-      <c r="O550" t="n">
-        <v>0</v>
-      </c>
-      <c r="P550" t="b">
+      <c r="N550" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O550" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P550" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="551">
-      <c r="A551" t="inlineStr">
+      <c r="A551" s="10" t="inlineStr">
         <is>
           <t>Batman &amp; Robin</t>
         </is>
       </c>
-      <c r="B551" t="inlineStr">
+      <c r="B551" s="10" t="inlineStr">
         <is>
           <t>card_550</t>
         </is>
       </c>
-      <c r="C551" t="inlineStr">
+      <c r="C551" s="10" t="inlineStr">
         <is>
           <t>Joel Schumacher</t>
         </is>
       </c>
-      <c r="D551" t="n">
+      <c r="D551" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E551" t="n">
+      <c r="E551" s="10" t="n">
         <v>1.96</v>
       </c>
-      <c r="F551" t="n">
+      <c r="F551" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="I551" t="n">
+      <c r="I551" s="10" t="n">
         <v>238300000</v>
       </c>
-      <c r="J551" t="b">
-        <v>0</v>
-      </c>
-      <c r="K551" t="n">
+      <c r="J551" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K551" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L551" t="b">
-        <v>0</v>
-      </c>
-      <c r="M551" t="n">
+      <c r="L551" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M551" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="N551" t="n">
-        <v>0</v>
-      </c>
-      <c r="O551" t="n">
-        <v>0</v>
-      </c>
-      <c r="P551" t="b">
+      <c r="N551" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O551" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P551" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="552">
-      <c r="A552" t="inlineStr">
+      <c r="A552" s="10" t="inlineStr">
         <is>
           <t>Batman v Superman: Dawn of Justice</t>
         </is>
       </c>
-      <c r="B552" t="inlineStr">
+      <c r="B552" s="10" t="inlineStr">
         <is>
           <t>card_551</t>
         </is>
       </c>
-      <c r="C552" t="inlineStr">
+      <c r="C552" s="10" t="inlineStr">
         <is>
           <t>Zack Snyder</t>
         </is>
       </c>
-      <c r="D552" t="n">
+      <c r="D552" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E552" t="n">
+      <c r="E552" s="10" t="n">
         <v>2.5</v>
       </c>
-      <c r="F552" t="n">
+      <c r="F552" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I552" t="n">
+      <c r="I552" s="10" t="n">
         <v>874400000</v>
       </c>
-      <c r="J552" t="b">
-        <v>0</v>
-      </c>
-      <c r="K552" t="n">
+      <c r="J552" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K552" s="10" t="n">
         <v>300000000</v>
       </c>
-      <c r="L552" t="b">
-        <v>0</v>
-      </c>
-      <c r="M552" t="n">
+      <c r="L552" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M552" s="10" t="n">
         <v>151</v>
       </c>
-      <c r="N552" t="n">
-        <v>0</v>
-      </c>
-      <c r="O552" t="n">
-        <v>0</v>
-      </c>
-      <c r="P552" t="b">
+      <c r="N552" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O552" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P552" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="553">
-      <c r="A553" t="inlineStr">
+      <c r="A553" s="10" t="inlineStr">
         <is>
           <t>The Batman</t>
         </is>
       </c>
-      <c r="B553" t="inlineStr">
+      <c r="B553" s="10" t="inlineStr">
         <is>
           <t>card_552</t>
         </is>
       </c>
-      <c r="C553" t="inlineStr">
+      <c r="C553" s="10" t="inlineStr">
         <is>
           <t>Matt Reeves</t>
         </is>
       </c>
-      <c r="D553" t="n">
+      <c r="D553" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E553" t="n">
+      <c r="E553" s="10" t="n">
         <v>4.05</v>
       </c>
-      <c r="F553" t="n">
+      <c r="F553" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I553" t="n">
+      <c r="I553" s="10" t="n">
         <v>772300000</v>
       </c>
-      <c r="J553" t="b">
-        <v>0</v>
-      </c>
-      <c r="K553" t="n">
+      <c r="J553" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K553" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L553" t="b">
-        <v>0</v>
-      </c>
-      <c r="M553" t="n">
+      <c r="L553" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M553" s="10" t="n">
         <v>176</v>
       </c>
-      <c r="N553" t="n">
-        <v>0</v>
-      </c>
-      <c r="O553" t="n">
-        <v>0</v>
-      </c>
-      <c r="P553" t="b">
+      <c r="N553" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O553" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P553" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>X-Men</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>card_553</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Bryan Singer</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E554" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="F554" t="n">
+        <v>73</v>
+      </c>
+      <c r="I554" t="n">
+        <v>296300000</v>
+      </c>
+      <c r="J554" t="b">
+        <v>0</v>
+      </c>
+      <c r="K554" t="n">
+        <v>75000000</v>
+      </c>
+      <c r="L554" t="b">
+        <v>0</v>
+      </c>
+      <c r="M554" t="n">
+        <v>104</v>
+      </c>
+      <c r="N554" t="n">
+        <v>0</v>
+      </c>
+      <c r="O554" t="n">
+        <v>0</v>
+      </c>
+      <c r="P554" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>X2</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>card_554</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Bryan Singer</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E555" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F555" t="n">
+        <v>78</v>
+      </c>
+      <c r="I555" t="n">
+        <v>407700000</v>
+      </c>
+      <c r="J555" t="b">
+        <v>0</v>
+      </c>
+      <c r="K555" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L555" t="b">
+        <v>0</v>
+      </c>
+      <c r="M555" t="n">
+        <v>133</v>
+      </c>
+      <c r="N555" t="n">
+        <v>0</v>
+      </c>
+      <c r="O555" t="n">
+        <v>0</v>
+      </c>
+      <c r="P555" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>X-Men: The Last Stand</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>card_555</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Brett Ratner</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E556" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F556" t="n">
+        <v>58</v>
+      </c>
+      <c r="I556" t="n">
+        <v>460000000</v>
+      </c>
+      <c r="J556" t="b">
+        <v>0</v>
+      </c>
+      <c r="K556" t="n">
+        <v>210000000</v>
+      </c>
+      <c r="L556" t="b">
+        <v>0</v>
+      </c>
+      <c r="M556" t="n">
+        <v>104</v>
+      </c>
+      <c r="N556" t="n">
+        <v>0</v>
+      </c>
+      <c r="O556" t="n">
+        <v>0</v>
+      </c>
+      <c r="P556" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>X-Men Origins: Wolverine</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>card_556</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Gavin Hood</t>
+        </is>
+      </c>
+      <c r="D557" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E557" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F557" t="n">
+        <v>54</v>
+      </c>
+      <c r="I557" t="n">
+        <v>373000000</v>
+      </c>
+      <c r="J557" t="b">
+        <v>0</v>
+      </c>
+      <c r="K557" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L557" t="b">
+        <v>0</v>
+      </c>
+      <c r="M557" t="n">
+        <v>107</v>
+      </c>
+      <c r="N557" t="n">
+        <v>0</v>
+      </c>
+      <c r="O557" t="n">
+        <v>0</v>
+      </c>
+      <c r="P557" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>X-Men: First Class</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>card_557</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Matthew Vaughn</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E558" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="F558" t="n">
+        <v>78</v>
+      </c>
+      <c r="I558" t="n">
+        <v>353000000</v>
+      </c>
+      <c r="J558" t="b">
+        <v>0</v>
+      </c>
+      <c r="K558" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L558" t="b">
+        <v>0</v>
+      </c>
+      <c r="M558" t="n">
+        <v>132</v>
+      </c>
+      <c r="N558" t="n">
+        <v>0</v>
+      </c>
+      <c r="O558" t="n">
+        <v>0</v>
+      </c>
+      <c r="P558" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>The Wolverine</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>card_558</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>James Mangold</t>
+        </is>
+      </c>
+      <c r="D559" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E559" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="F559" t="n">
+        <v>66</v>
+      </c>
+      <c r="I559" t="n">
+        <v>414800000</v>
+      </c>
+      <c r="J559" t="b">
+        <v>0</v>
+      </c>
+      <c r="K559" t="n">
+        <v>120000000</v>
+      </c>
+      <c r="L559" t="b">
+        <v>0</v>
+      </c>
+      <c r="M559" t="n">
+        <v>126</v>
+      </c>
+      <c r="N559" t="n">
+        <v>0</v>
+      </c>
+      <c r="O559" t="n">
+        <v>0</v>
+      </c>
+      <c r="P559" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>X-Men: Days of Future Past</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>card_559</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Bryan Singer</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E560" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F560" t="n">
+        <v>81</v>
+      </c>
+      <c r="I560" t="n">
+        <v>747900000</v>
+      </c>
+      <c r="J560" t="b">
+        <v>0</v>
+      </c>
+      <c r="K560" t="n">
+        <v>205000000</v>
+      </c>
+      <c r="L560" t="b">
+        <v>0</v>
+      </c>
+      <c r="M560" t="n">
+        <v>131</v>
+      </c>
+      <c r="N560" t="n">
+        <v>0</v>
+      </c>
+      <c r="O560" t="n">
+        <v>0</v>
+      </c>
+      <c r="P560" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>X-Men: Apocalypse</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>card_560</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Bryan Singer</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E561" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="F561" t="n">
+        <v>63</v>
+      </c>
+      <c r="I561" t="n">
+        <v>544000000</v>
+      </c>
+      <c r="J561" t="b">
+        <v>0</v>
+      </c>
+      <c r="K561" t="n">
+        <v>178000000</v>
+      </c>
+      <c r="L561" t="b">
+        <v>0</v>
+      </c>
+      <c r="M561" t="n">
+        <v>144</v>
+      </c>
+      <c r="N561" t="n">
+        <v>0</v>
+      </c>
+      <c r="O561" t="n">
+        <v>0</v>
+      </c>
+      <c r="P561" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Logan</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>card_561</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>James Mangold</t>
+        </is>
+      </c>
+      <c r="D562" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E562" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="F562" t="n">
+        <v>84</v>
+      </c>
+      <c r="I562" t="n">
+        <v>619200000</v>
+      </c>
+      <c r="J562" t="b">
+        <v>0</v>
+      </c>
+      <c r="K562" t="n">
+        <v>97000000</v>
+      </c>
+      <c r="L562" t="b">
+        <v>0</v>
+      </c>
+      <c r="M562" t="n">
+        <v>137</v>
+      </c>
+      <c r="N562" t="n">
+        <v>0</v>
+      </c>
+      <c r="O562" t="n">
+        <v>0</v>
+      </c>
+      <c r="P562" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Dark Phoenix</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>card_562</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Simon Kinberg</t>
+        </is>
+      </c>
+      <c r="D563" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E563" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F563" t="n">
+        <v>49</v>
+      </c>
+      <c r="I563" t="n">
+        <v>252400000</v>
+      </c>
+      <c r="J563" t="b">
+        <v>0</v>
+      </c>
+      <c r="K563" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L563" t="b">
+        <v>0</v>
+      </c>
+      <c r="M563" t="n">
+        <v>114</v>
+      </c>
+      <c r="N563" t="n">
+        <v>0</v>
+      </c>
+      <c r="O563" t="n">
+        <v>0</v>
+      </c>
+      <c r="P563" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>The New Mutants</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>card_563</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Josh Boone</t>
+        </is>
+      </c>
+      <c r="D564" t="n">
+        <v>2020</v>
+      </c>
+      <c r="E564" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F564" t="n">
+        <v>43</v>
+      </c>
+      <c r="I564" t="n">
+        <v>49200000</v>
+      </c>
+      <c r="J564" t="b">
+        <v>0</v>
+      </c>
+      <c r="K564" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L564" t="b">
+        <v>0</v>
+      </c>
+      <c r="M564" t="n">
+        <v>94</v>
+      </c>
+      <c r="N564" t="n">
+        <v>0</v>
+      </c>
+      <c r="O564" t="n">
+        <v>0</v>
+      </c>
+      <c r="P564" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Fast & Furious series (card_564-574)
All 10 mainline films plus Hobbs & Shaw.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P564"/>
+  <dimension ref="A1:P575"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -29307,552 +29307,1102 @@
       </c>
     </row>
     <row r="554">
-      <c r="A554" t="inlineStr">
+      <c r="A554" s="10" t="inlineStr">
         <is>
           <t>X-Men</t>
         </is>
       </c>
-      <c r="B554" t="inlineStr">
+      <c r="B554" s="10" t="inlineStr">
         <is>
           <t>card_553</t>
         </is>
       </c>
-      <c r="C554" t="inlineStr">
+      <c r="C554" s="10" t="inlineStr">
         <is>
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="D554" t="n">
+      <c r="D554" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E554" t="n">
+      <c r="E554" s="10" t="n">
         <v>3.35</v>
       </c>
-      <c r="F554" t="n">
+      <c r="F554" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I554" t="n">
+      <c r="I554" s="10" t="n">
         <v>296300000</v>
       </c>
-      <c r="J554" t="b">
-        <v>0</v>
-      </c>
-      <c r="K554" t="n">
+      <c r="J554" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K554" s="10" t="n">
         <v>75000000</v>
       </c>
-      <c r="L554" t="b">
-        <v>0</v>
-      </c>
-      <c r="M554" t="n">
+      <c r="L554" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M554" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="N554" t="n">
-        <v>0</v>
-      </c>
-      <c r="O554" t="n">
-        <v>0</v>
-      </c>
-      <c r="P554" t="b">
+      <c r="N554" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O554" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P554" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="555">
-      <c r="A555" t="inlineStr">
+      <c r="A555" s="10" t="inlineStr">
         <is>
           <t>X2</t>
         </is>
       </c>
-      <c r="B555" t="inlineStr">
+      <c r="B555" s="10" t="inlineStr">
         <is>
           <t>card_554</t>
         </is>
       </c>
-      <c r="C555" t="inlineStr">
+      <c r="C555" s="10" t="inlineStr">
         <is>
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="D555" t="n">
+      <c r="D555" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E555" t="n">
+      <c r="E555" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F555" t="n">
+      <c r="F555" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I555" t="n">
+      <c r="I555" s="10" t="n">
         <v>407700000</v>
       </c>
-      <c r="J555" t="b">
-        <v>0</v>
-      </c>
-      <c r="K555" t="n">
+      <c r="J555" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K555" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L555" t="b">
-        <v>0</v>
-      </c>
-      <c r="M555" t="n">
+      <c r="L555" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M555" s="10" t="n">
         <v>133</v>
       </c>
-      <c r="N555" t="n">
-        <v>0</v>
-      </c>
-      <c r="O555" t="n">
-        <v>0</v>
-      </c>
-      <c r="P555" t="b">
+      <c r="N555" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O555" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P555" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="556">
-      <c r="A556" t="inlineStr">
+      <c r="A556" s="10" t="inlineStr">
         <is>
           <t>X-Men: The Last Stand</t>
         </is>
       </c>
-      <c r="B556" t="inlineStr">
+      <c r="B556" s="10" t="inlineStr">
         <is>
           <t>card_555</t>
         </is>
       </c>
-      <c r="C556" t="inlineStr">
+      <c r="C556" s="10" t="inlineStr">
         <is>
           <t>Brett Ratner</t>
         </is>
       </c>
-      <c r="D556" t="n">
+      <c r="D556" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E556" t="n">
+      <c r="E556" s="10" t="n">
         <v>2.73</v>
       </c>
-      <c r="F556" t="n">
+      <c r="F556" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="I556" t="n">
+      <c r="I556" s="10" t="n">
         <v>460000000</v>
       </c>
-      <c r="J556" t="b">
-        <v>0</v>
-      </c>
-      <c r="K556" t="n">
+      <c r="J556" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K556" s="10" t="n">
         <v>210000000</v>
       </c>
-      <c r="L556" t="b">
-        <v>0</v>
-      </c>
-      <c r="M556" t="n">
+      <c r="L556" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M556" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="N556" t="n">
-        <v>0</v>
-      </c>
-      <c r="O556" t="n">
-        <v>0</v>
-      </c>
-      <c r="P556" t="b">
+      <c r="N556" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O556" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P556" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="557">
-      <c r="A557" t="inlineStr">
+      <c r="A557" s="10" t="inlineStr">
         <is>
           <t>X-Men Origins: Wolverine</t>
         </is>
       </c>
-      <c r="B557" t="inlineStr">
+      <c r="B557" s="10" t="inlineStr">
         <is>
           <t>card_556</t>
         </is>
       </c>
-      <c r="C557" t="inlineStr">
+      <c r="C557" s="10" t="inlineStr">
         <is>
           <t>Gavin Hood</t>
         </is>
       </c>
-      <c r="D557" t="n">
+      <c r="D557" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E557" t="n">
+      <c r="E557" s="10" t="n">
         <v>2.6</v>
       </c>
-      <c r="F557" t="n">
+      <c r="F557" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="I557" t="n">
+      <c r="I557" s="10" t="n">
         <v>373000000</v>
       </c>
-      <c r="J557" t="b">
-        <v>0</v>
-      </c>
-      <c r="K557" t="n">
+      <c r="J557" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K557" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L557" t="b">
-        <v>0</v>
-      </c>
-      <c r="M557" t="n">
+      <c r="L557" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M557" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N557" t="n">
-        <v>0</v>
-      </c>
-      <c r="O557" t="n">
-        <v>0</v>
-      </c>
-      <c r="P557" t="b">
+      <c r="N557" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O557" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P557" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="558">
-      <c r="A558" t="inlineStr">
+      <c r="A558" s="10" t="inlineStr">
         <is>
           <t>X-Men: First Class</t>
         </is>
       </c>
-      <c r="B558" t="inlineStr">
+      <c r="B558" s="10" t="inlineStr">
         <is>
           <t>card_557</t>
         </is>
       </c>
-      <c r="C558" t="inlineStr">
+      <c r="C558" s="10" t="inlineStr">
         <is>
           <t>Matthew Vaughn</t>
         </is>
       </c>
-      <c r="D558" t="n">
+      <c r="D558" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E558" t="n">
+      <c r="E558" s="10" t="n">
         <v>3.62</v>
       </c>
-      <c r="F558" t="n">
+      <c r="F558" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I558" t="n">
+      <c r="I558" s="10" t="n">
         <v>353000000</v>
       </c>
-      <c r="J558" t="b">
-        <v>0</v>
-      </c>
-      <c r="K558" t="n">
+      <c r="J558" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K558" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L558" t="b">
-        <v>0</v>
-      </c>
-      <c r="M558" t="n">
+      <c r="L558" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M558" s="10" t="n">
         <v>132</v>
       </c>
-      <c r="N558" t="n">
-        <v>0</v>
-      </c>
-      <c r="O558" t="n">
-        <v>0</v>
-      </c>
-      <c r="P558" t="b">
+      <c r="N558" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O558" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P558" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="559">
-      <c r="A559" t="inlineStr">
+      <c r="A559" s="10" t="inlineStr">
         <is>
           <t>The Wolverine</t>
         </is>
       </c>
-      <c r="B559" t="inlineStr">
+      <c r="B559" s="10" t="inlineStr">
         <is>
           <t>card_558</t>
         </is>
       </c>
-      <c r="C559" t="inlineStr">
+      <c r="C559" s="10" t="inlineStr">
         <is>
           <t>James Mangold</t>
         </is>
       </c>
-      <c r="D559" t="n">
+      <c r="D559" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E559" t="n">
+      <c r="E559" s="10" t="n">
         <v>3.04</v>
       </c>
-      <c r="F559" t="n">
+      <c r="F559" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I559" t="n">
+      <c r="I559" s="10" t="n">
         <v>414800000</v>
       </c>
-      <c r="J559" t="b">
-        <v>0</v>
-      </c>
-      <c r="K559" t="n">
+      <c r="J559" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K559" s="10" t="n">
         <v>120000000</v>
       </c>
-      <c r="L559" t="b">
-        <v>0</v>
-      </c>
-      <c r="M559" t="n">
+      <c r="L559" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M559" s="10" t="n">
         <v>126</v>
       </c>
-      <c r="N559" t="n">
-        <v>0</v>
-      </c>
-      <c r="O559" t="n">
-        <v>0</v>
-      </c>
-      <c r="P559" t="b">
+      <c r="N559" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O559" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P559" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="560">
-      <c r="A560" t="inlineStr">
+      <c r="A560" s="10" t="inlineStr">
         <is>
           <t>X-Men: Days of Future Past</t>
         </is>
       </c>
-      <c r="B560" t="inlineStr">
+      <c r="B560" s="10" t="inlineStr">
         <is>
           <t>card_559</t>
         </is>
       </c>
-      <c r="C560" t="inlineStr">
+      <c r="C560" s="10" t="inlineStr">
         <is>
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="D560" t="n">
+      <c r="D560" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E560" t="n">
+      <c r="E560" s="10" t="n">
         <v>3.72</v>
       </c>
-      <c r="F560" t="n">
+      <c r="F560" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I560" t="n">
+      <c r="I560" s="10" t="n">
         <v>747900000</v>
       </c>
-      <c r="J560" t="b">
-        <v>0</v>
-      </c>
-      <c r="K560" t="n">
+      <c r="J560" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K560" s="10" t="n">
         <v>205000000</v>
       </c>
-      <c r="L560" t="b">
-        <v>0</v>
-      </c>
-      <c r="M560" t="n">
+      <c r="L560" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M560" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N560" t="n">
-        <v>0</v>
-      </c>
-      <c r="O560" t="n">
-        <v>0</v>
-      </c>
-      <c r="P560" t="b">
+      <c r="N560" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O560" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P560" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="561">
-      <c r="A561" t="inlineStr">
+      <c r="A561" s="10" t="inlineStr">
         <is>
           <t>X-Men: Apocalypse</t>
         </is>
       </c>
-      <c r="B561" t="inlineStr">
+      <c r="B561" s="10" t="inlineStr">
         <is>
           <t>card_560</t>
         </is>
       </c>
-      <c r="C561" t="inlineStr">
+      <c r="C561" s="10" t="inlineStr">
         <is>
           <t>Bryan Singer</t>
         </is>
       </c>
-      <c r="D561" t="n">
+      <c r="D561" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E561" t="n">
+      <c r="E561" s="10" t="n">
         <v>2.71</v>
       </c>
-      <c r="F561" t="n">
+      <c r="F561" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I561" t="n">
+      <c r="I561" s="10" t="n">
         <v>544000000</v>
       </c>
-      <c r="J561" t="b">
-        <v>0</v>
-      </c>
-      <c r="K561" t="n">
+      <c r="J561" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K561" s="10" t="n">
         <v>178000000</v>
       </c>
-      <c r="L561" t="b">
-        <v>0</v>
-      </c>
-      <c r="M561" t="n">
+      <c r="L561" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M561" s="10" t="n">
         <v>144</v>
       </c>
-      <c r="N561" t="n">
-        <v>0</v>
-      </c>
-      <c r="O561" t="n">
-        <v>0</v>
-      </c>
-      <c r="P561" t="b">
+      <c r="N561" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O561" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P561" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="562">
-      <c r="A562" t="inlineStr">
+      <c r="A562" s="10" t="inlineStr">
         <is>
           <t>Logan</t>
         </is>
       </c>
-      <c r="B562" t="inlineStr">
+      <c r="B562" s="10" t="inlineStr">
         <is>
           <t>card_561</t>
         </is>
       </c>
-      <c r="C562" t="inlineStr">
+      <c r="C562" s="10" t="inlineStr">
         <is>
           <t>James Mangold</t>
         </is>
       </c>
-      <c r="D562" t="n">
+      <c r="D562" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E562" t="n">
+      <c r="E562" s="10" t="n">
         <v>4.13</v>
       </c>
-      <c r="F562" t="n">
+      <c r="F562" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="I562" t="n">
+      <c r="I562" s="10" t="n">
         <v>619200000</v>
       </c>
-      <c r="J562" t="b">
-        <v>0</v>
-      </c>
-      <c r="K562" t="n">
+      <c r="J562" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K562" s="10" t="n">
         <v>97000000</v>
       </c>
-      <c r="L562" t="b">
-        <v>0</v>
-      </c>
-      <c r="M562" t="n">
+      <c r="L562" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M562" s="10" t="n">
         <v>137</v>
       </c>
-      <c r="N562" t="n">
-        <v>0</v>
-      </c>
-      <c r="O562" t="n">
-        <v>0</v>
-      </c>
-      <c r="P562" t="b">
+      <c r="N562" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O562" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P562" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="563">
-      <c r="A563" t="inlineStr">
+      <c r="A563" s="10" t="inlineStr">
         <is>
           <t>Dark Phoenix</t>
         </is>
       </c>
-      <c r="B563" t="inlineStr">
+      <c r="B563" s="10" t="inlineStr">
         <is>
           <t>card_562</t>
         </is>
       </c>
-      <c r="C563" t="inlineStr">
+      <c r="C563" s="10" t="inlineStr">
         <is>
           <t>Simon Kinberg</t>
         </is>
       </c>
-      <c r="D563" t="n">
+      <c r="D563" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E563" t="n">
+      <c r="E563" s="10" t="n">
         <v>2.13</v>
       </c>
-      <c r="F563" t="n">
+      <c r="F563" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="I563" t="n">
+      <c r="I563" s="10" t="n">
         <v>252400000</v>
       </c>
-      <c r="J563" t="b">
-        <v>0</v>
-      </c>
-      <c r="K563" t="n">
+      <c r="J563" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K563" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L563" t="b">
-        <v>0</v>
-      </c>
-      <c r="M563" t="n">
+      <c r="L563" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M563" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N563" t="n">
-        <v>0</v>
-      </c>
-      <c r="O563" t="n">
-        <v>0</v>
-      </c>
-      <c r="P563" t="b">
+      <c r="N563" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O563" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P563" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="564">
-      <c r="A564" t="inlineStr">
+      <c r="A564" s="10" t="inlineStr">
         <is>
           <t>The New Mutants</t>
         </is>
       </c>
-      <c r="B564" t="inlineStr">
+      <c r="B564" s="10" t="inlineStr">
         <is>
           <t>card_563</t>
         </is>
       </c>
-      <c r="C564" t="inlineStr">
+      <c r="C564" s="10" t="inlineStr">
         <is>
           <t>Josh Boone</t>
         </is>
       </c>
-      <c r="D564" t="n">
+      <c r="D564" s="10" t="n">
         <v>2020</v>
       </c>
-      <c r="E564" t="n">
+      <c r="E564" s="10" t="n">
         <v>2.13</v>
       </c>
-      <c r="F564" t="n">
+      <c r="F564" s="10" t="n">
         <v>43</v>
       </c>
-      <c r="I564" t="n">
+      <c r="I564" s="10" t="n">
         <v>49200000</v>
       </c>
-      <c r="J564" t="b">
-        <v>0</v>
-      </c>
-      <c r="K564" t="n">
+      <c r="J564" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K564" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L564" t="b">
-        <v>0</v>
-      </c>
-      <c r="M564" t="n">
+      <c r="L564" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M564" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="N564" t="n">
-        <v>0</v>
-      </c>
-      <c r="O564" t="n">
-        <v>0</v>
-      </c>
-      <c r="P564" t="b">
+      <c r="N564" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O564" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P564" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>The Fast and the Furious</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>card_564</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Rob Cohen</t>
+        </is>
+      </c>
+      <c r="D565" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E565" t="n">
+        <v>2.69</v>
+      </c>
+      <c r="F565" t="n">
+        <v>72</v>
+      </c>
+      <c r="I565" t="n">
+        <v>207500000</v>
+      </c>
+      <c r="J565" t="b">
+        <v>0</v>
+      </c>
+      <c r="K565" t="n">
+        <v>38000000</v>
+      </c>
+      <c r="L565" t="b">
+        <v>0</v>
+      </c>
+      <c r="M565" t="n">
+        <v>106</v>
+      </c>
+      <c r="N565" t="n">
+        <v>0</v>
+      </c>
+      <c r="O565" t="n">
+        <v>0</v>
+      </c>
+      <c r="P565" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2 Fast 2 Furious</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>card_565</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>John Singleton</t>
+        </is>
+      </c>
+      <c r="D566" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E566" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="F566" t="n">
+        <v>60</v>
+      </c>
+      <c r="I566" t="n">
+        <v>236400000</v>
+      </c>
+      <c r="J566" t="b">
+        <v>0</v>
+      </c>
+      <c r="K566" t="n">
+        <v>76000000</v>
+      </c>
+      <c r="L566" t="b">
+        <v>0</v>
+      </c>
+      <c r="M566" t="n">
+        <v>107</v>
+      </c>
+      <c r="N566" t="n">
+        <v>0</v>
+      </c>
+      <c r="O566" t="n">
+        <v>0</v>
+      </c>
+      <c r="P566" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>The Fast and the Furious: Tokyo Drift</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>card_566</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Justin Lin</t>
+        </is>
+      </c>
+      <c r="D567" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E567" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="F567" t="n">
+        <v>66</v>
+      </c>
+      <c r="I567" t="n">
+        <v>159000000</v>
+      </c>
+      <c r="J567" t="b">
+        <v>0</v>
+      </c>
+      <c r="K567" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="L567" t="b">
+        <v>0</v>
+      </c>
+      <c r="M567" t="n">
+        <v>104</v>
+      </c>
+      <c r="N567" t="n">
+        <v>0</v>
+      </c>
+      <c r="O567" t="n">
+        <v>0</v>
+      </c>
+      <c r="P567" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Fast &amp; Furious</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>card_567</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Justin Lin</t>
+        </is>
+      </c>
+      <c r="D568" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E568" t="n">
+        <v>3.03</v>
+      </c>
+      <c r="F568" t="n">
+        <v>63</v>
+      </c>
+      <c r="I568" t="n">
+        <v>360400000</v>
+      </c>
+      <c r="J568" t="b">
+        <v>0</v>
+      </c>
+      <c r="K568" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="L568" t="b">
+        <v>0</v>
+      </c>
+      <c r="M568" t="n">
+        <v>107</v>
+      </c>
+      <c r="N568" t="n">
+        <v>0</v>
+      </c>
+      <c r="O568" t="n">
+        <v>0</v>
+      </c>
+      <c r="P568" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Fast Five</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>card_568</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Justin Lin</t>
+        </is>
+      </c>
+      <c r="D569" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E569" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F569" t="n">
+        <v>74</v>
+      </c>
+      <c r="I569" t="n">
+        <v>630000000</v>
+      </c>
+      <c r="J569" t="b">
+        <v>0</v>
+      </c>
+      <c r="K569" t="n">
+        <v>125000000</v>
+      </c>
+      <c r="L569" t="b">
+        <v>0</v>
+      </c>
+      <c r="M569" t="n">
+        <v>130</v>
+      </c>
+      <c r="N569" t="n">
+        <v>0</v>
+      </c>
+      <c r="O569" t="n">
+        <v>0</v>
+      </c>
+      <c r="P569" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Fast &amp; Furious 6</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>card_569</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Justin Lin</t>
+        </is>
+      </c>
+      <c r="D570" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E570" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="F570" t="n">
+        <v>70</v>
+      </c>
+      <c r="I570" t="n">
+        <v>788700000</v>
+      </c>
+      <c r="J570" t="b">
+        <v>0</v>
+      </c>
+      <c r="K570" t="n">
+        <v>160000000</v>
+      </c>
+      <c r="L570" t="b">
+        <v>0</v>
+      </c>
+      <c r="M570" t="n">
+        <v>130</v>
+      </c>
+      <c r="N570" t="n">
+        <v>0</v>
+      </c>
+      <c r="O570" t="n">
+        <v>0</v>
+      </c>
+      <c r="P570" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Furious 7</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>card_570</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>James Wan</t>
+        </is>
+      </c>
+      <c r="D571" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E571" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="F571" t="n">
+        <v>68</v>
+      </c>
+      <c r="I571" t="n">
+        <v>1515000000</v>
+      </c>
+      <c r="J571" t="b">
+        <v>0</v>
+      </c>
+      <c r="K571" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="L571" t="b">
+        <v>0</v>
+      </c>
+      <c r="M571" t="n">
+        <v>137</v>
+      </c>
+      <c r="N571" t="n">
+        <v>0</v>
+      </c>
+      <c r="O571" t="n">
+        <v>0</v>
+      </c>
+      <c r="P571" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>The Fate of the Furious</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>card_571</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>F. Gary Gray</t>
+        </is>
+      </c>
+      <c r="D572" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E572" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F572" t="n">
+        <v>68</v>
+      </c>
+      <c r="I572" t="n">
+        <v>1236000000</v>
+      </c>
+      <c r="J572" t="b">
+        <v>0</v>
+      </c>
+      <c r="K572" t="n">
+        <v>250000000</v>
+      </c>
+      <c r="L572" t="b">
+        <v>0</v>
+      </c>
+      <c r="M572" t="n">
+        <v>136</v>
+      </c>
+      <c r="N572" t="n">
+        <v>0</v>
+      </c>
+      <c r="O572" t="n">
+        <v>0</v>
+      </c>
+      <c r="P572" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Fast &amp; Furious Presents: Hobbs &amp; Shaw</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>card_572</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>David Leitch</t>
+        </is>
+      </c>
+      <c r="D573" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E573" t="n">
+        <v>2.73</v>
+      </c>
+      <c r="F573" t="n">
+        <v>64</v>
+      </c>
+      <c r="I573" t="n">
+        <v>760000000</v>
+      </c>
+      <c r="J573" t="b">
+        <v>0</v>
+      </c>
+      <c r="K573" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L573" t="b">
+        <v>0</v>
+      </c>
+      <c r="M573" t="n">
+        <v>137</v>
+      </c>
+      <c r="N573" t="n">
+        <v>0</v>
+      </c>
+      <c r="O573" t="n">
+        <v>0</v>
+      </c>
+      <c r="P573" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>card_573</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Justin Lin</t>
+        </is>
+      </c>
+      <c r="D574" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E574" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F574" t="n">
+        <v>47</v>
+      </c>
+      <c r="I574" t="n">
+        <v>726200000</v>
+      </c>
+      <c r="J574" t="b">
+        <v>0</v>
+      </c>
+      <c r="K574" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L574" t="b">
+        <v>0</v>
+      </c>
+      <c r="M574" t="n">
+        <v>143</v>
+      </c>
+      <c r="N574" t="n">
+        <v>0</v>
+      </c>
+      <c r="O574" t="n">
+        <v>0</v>
+      </c>
+      <c r="P574" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Fast X</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>card_574</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Louis Leterrier</t>
+        </is>
+      </c>
+      <c r="D575" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E575" t="n">
+        <v>2.49</v>
+      </c>
+      <c r="F575" t="n">
+        <v>49</v>
+      </c>
+      <c r="I575" t="n">
+        <v>714400000</v>
+      </c>
+      <c r="J575" t="b">
+        <v>0</v>
+      </c>
+      <c r="K575" t="n">
+        <v>340000000</v>
+      </c>
+      <c r="L575" t="b">
+        <v>0</v>
+      </c>
+      <c r="M575" t="n">
+        <v>141</v>
+      </c>
+      <c r="N575" t="n">
+        <v>0</v>
+      </c>
+      <c r="O575" t="n">
+        <v>0</v>
+      </c>
+      <c r="P575" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add remaining Spider-Man films (card_575-579)
Spider-Man (2002), Spider-Man 3, The Amazing Spider-Man 1-2, Into the
Spider-Verse.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P575"/>
+  <dimension ref="A1:P580"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -29857,552 +29857,802 @@
       </c>
     </row>
     <row r="565">
-      <c r="A565" t="inlineStr">
+      <c r="A565" s="10" t="inlineStr">
         <is>
           <t>The Fast and the Furious</t>
         </is>
       </c>
-      <c r="B565" t="inlineStr">
+      <c r="B565" s="10" t="inlineStr">
         <is>
           <t>card_564</t>
         </is>
       </c>
-      <c r="C565" t="inlineStr">
+      <c r="C565" s="10" t="inlineStr">
         <is>
           <t>Rob Cohen</t>
         </is>
       </c>
-      <c r="D565" t="n">
+      <c r="D565" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E565" t="n">
+      <c r="E565" s="10" t="n">
         <v>2.69</v>
       </c>
-      <c r="F565" t="n">
+      <c r="F565" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I565" t="n">
+      <c r="I565" s="10" t="n">
         <v>207500000</v>
       </c>
-      <c r="J565" t="b">
-        <v>0</v>
-      </c>
-      <c r="K565" t="n">
+      <c r="J565" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K565" s="10" t="n">
         <v>38000000</v>
       </c>
-      <c r="L565" t="b">
-        <v>0</v>
-      </c>
-      <c r="M565" t="n">
+      <c r="L565" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M565" s="10" t="n">
         <v>106</v>
       </c>
-      <c r="N565" t="n">
-        <v>0</v>
-      </c>
-      <c r="O565" t="n">
-        <v>0</v>
-      </c>
-      <c r="P565" t="b">
+      <c r="N565" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O565" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P565" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="566">
-      <c r="A566" t="inlineStr">
+      <c r="A566" s="10" t="inlineStr">
         <is>
           <t>2 Fast 2 Furious</t>
         </is>
       </c>
-      <c r="B566" t="inlineStr">
+      <c r="B566" s="10" t="inlineStr">
         <is>
           <t>card_565</t>
         </is>
       </c>
-      <c r="C566" t="inlineStr">
+      <c r="C566" s="10" t="inlineStr">
         <is>
           <t>John Singleton</t>
         </is>
       </c>
-      <c r="D566" t="n">
+      <c r="D566" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E566" t="n">
+      <c r="E566" s="10" t="n">
         <v>3.28</v>
       </c>
-      <c r="F566" t="n">
+      <c r="F566" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I566" t="n">
+      <c r="I566" s="10" t="n">
         <v>236400000</v>
       </c>
-      <c r="J566" t="b">
-        <v>0</v>
-      </c>
-      <c r="K566" t="n">
+      <c r="J566" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K566" s="10" t="n">
         <v>76000000</v>
       </c>
-      <c r="L566" t="b">
-        <v>0</v>
-      </c>
-      <c r="M566" t="n">
+      <c r="L566" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M566" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N566" t="n">
-        <v>0</v>
-      </c>
-      <c r="O566" t="n">
-        <v>0</v>
-      </c>
-      <c r="P566" t="b">
+      <c r="N566" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O566" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P566" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="567">
-      <c r="A567" t="inlineStr">
+      <c r="A567" s="10" t="inlineStr">
         <is>
           <t>The Fast and the Furious: Tokyo Drift</t>
         </is>
       </c>
-      <c r="B567" t="inlineStr">
+      <c r="B567" s="10" t="inlineStr">
         <is>
           <t>card_566</t>
         </is>
       </c>
-      <c r="C567" t="inlineStr">
+      <c r="C567" s="10" t="inlineStr">
         <is>
           <t>Justin Lin</t>
         </is>
       </c>
-      <c r="D567" t="n">
+      <c r="D567" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E567" t="n">
+      <c r="E567" s="10" t="n">
         <v>3.41</v>
       </c>
-      <c r="F567" t="n">
+      <c r="F567" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I567" t="n">
+      <c r="I567" s="10" t="n">
         <v>159000000</v>
       </c>
-      <c r="J567" t="b">
-        <v>0</v>
-      </c>
-      <c r="K567" t="n">
+      <c r="J567" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K567" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="L567" t="b">
-        <v>0</v>
-      </c>
-      <c r="M567" t="n">
+      <c r="L567" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M567" s="10" t="n">
         <v>104</v>
       </c>
-      <c r="N567" t="n">
-        <v>0</v>
-      </c>
-      <c r="O567" t="n">
-        <v>0</v>
-      </c>
-      <c r="P567" t="b">
+      <c r="N567" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O567" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P567" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="568">
-      <c r="A568" t="inlineStr">
+      <c r="A568" s="10" t="inlineStr">
         <is>
           <t>Fast &amp; Furious</t>
         </is>
       </c>
-      <c r="B568" t="inlineStr">
+      <c r="B568" s="10" t="inlineStr">
         <is>
           <t>card_567</t>
         </is>
       </c>
-      <c r="C568" t="inlineStr">
+      <c r="C568" s="10" t="inlineStr">
         <is>
           <t>Justin Lin</t>
         </is>
       </c>
-      <c r="D568" t="n">
+      <c r="D568" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E568" t="n">
+      <c r="E568" s="10" t="n">
         <v>3.03</v>
       </c>
-      <c r="F568" t="n">
+      <c r="F568" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I568" t="n">
+      <c r="I568" s="10" t="n">
         <v>360400000</v>
       </c>
-      <c r="J568" t="b">
-        <v>0</v>
-      </c>
-      <c r="K568" t="n">
+      <c r="J568" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K568" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="L568" t="b">
-        <v>0</v>
-      </c>
-      <c r="M568" t="n">
+      <c r="L568" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M568" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N568" t="n">
-        <v>0</v>
-      </c>
-      <c r="O568" t="n">
-        <v>0</v>
-      </c>
-      <c r="P568" t="b">
+      <c r="N568" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O568" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P568" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="569">
-      <c r="A569" t="inlineStr">
+      <c r="A569" s="10" t="inlineStr">
         <is>
           <t>Fast Five</t>
         </is>
       </c>
-      <c r="B569" t="inlineStr">
+      <c r="B569" s="10" t="inlineStr">
         <is>
           <t>card_568</t>
         </is>
       </c>
-      <c r="C569" t="inlineStr">
+      <c r="C569" s="10" t="inlineStr">
         <is>
           <t>Justin Lin</t>
         </is>
       </c>
-      <c r="D569" t="n">
+      <c r="D569" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E569" t="n">
+      <c r="E569" s="10" t="n">
         <v>3.55</v>
       </c>
-      <c r="F569" t="n">
+      <c r="F569" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I569" t="n">
+      <c r="I569" s="10" t="n">
         <v>630000000</v>
       </c>
-      <c r="J569" t="b">
-        <v>0</v>
-      </c>
-      <c r="K569" t="n">
+      <c r="J569" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K569" s="10" t="n">
         <v>125000000</v>
       </c>
-      <c r="L569" t="b">
-        <v>0</v>
-      </c>
-      <c r="M569" t="n">
+      <c r="L569" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M569" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N569" t="n">
-        <v>0</v>
-      </c>
-      <c r="O569" t="n">
-        <v>0</v>
-      </c>
-      <c r="P569" t="b">
+      <c r="N569" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O569" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P569" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="570">
-      <c r="A570" t="inlineStr">
+      <c r="A570" s="10" t="inlineStr">
         <is>
           <t>Fast &amp; Furious 6</t>
         </is>
       </c>
-      <c r="B570" t="inlineStr">
+      <c r="B570" s="10" t="inlineStr">
         <is>
           <t>card_569</t>
         </is>
       </c>
-      <c r="C570" t="inlineStr">
+      <c r="C570" s="10" t="inlineStr">
         <is>
           <t>Justin Lin</t>
         </is>
       </c>
-      <c r="D570" t="n">
+      <c r="D570" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E570" t="n">
+      <c r="E570" s="10" t="n">
         <v>3.13</v>
       </c>
-      <c r="F570" t="n">
+      <c r="F570" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I570" t="n">
+      <c r="I570" s="10" t="n">
         <v>788700000</v>
       </c>
-      <c r="J570" t="b">
-        <v>0</v>
-      </c>
-      <c r="K570" t="n">
+      <c r="J570" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K570" s="10" t="n">
         <v>160000000</v>
       </c>
-      <c r="L570" t="b">
-        <v>0</v>
-      </c>
-      <c r="M570" t="n">
+      <c r="L570" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M570" s="10" t="n">
         <v>130</v>
       </c>
-      <c r="N570" t="n">
-        <v>0</v>
-      </c>
-      <c r="O570" t="n">
-        <v>0</v>
-      </c>
-      <c r="P570" t="b">
+      <c r="N570" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O570" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P570" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="571">
-      <c r="A571" t="inlineStr">
+      <c r="A571" s="10" t="inlineStr">
         <is>
           <t>Furious 7</t>
         </is>
       </c>
-      <c r="B571" t="inlineStr">
+      <c r="B571" s="10" t="inlineStr">
         <is>
           <t>card_570</t>
         </is>
       </c>
-      <c r="C571" t="inlineStr">
+      <c r="C571" s="10" t="inlineStr">
         <is>
           <t>James Wan</t>
         </is>
       </c>
-      <c r="D571" t="n">
+      <c r="D571" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E571" t="n">
+      <c r="E571" s="10" t="n">
         <v>3.35</v>
       </c>
-      <c r="F571" t="n">
+      <c r="F571" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I571" t="n">
+      <c r="I571" s="10" t="n">
         <v>1515000000</v>
       </c>
-      <c r="J571" t="b">
-        <v>0</v>
-      </c>
-      <c r="K571" t="n">
+      <c r="J571" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K571" s="10" t="n">
         <v>250000000</v>
       </c>
-      <c r="L571" t="b">
-        <v>0</v>
-      </c>
-      <c r="M571" t="n">
+      <c r="L571" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M571" s="10" t="n">
         <v>137</v>
       </c>
-      <c r="N571" t="n">
-        <v>0</v>
-      </c>
-      <c r="O571" t="n">
-        <v>0</v>
-      </c>
-      <c r="P571" t="b">
+      <c r="N571" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O571" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P571" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="572">
-      <c r="A572" t="inlineStr">
+      <c r="A572" s="10" t="inlineStr">
         <is>
           <t>The Fate of the Furious</t>
         </is>
       </c>
-      <c r="B572" t="inlineStr">
+      <c r="B572" s="10" t="inlineStr">
         <is>
           <t>card_571</t>
         </is>
       </c>
-      <c r="C572" t="inlineStr">
+      <c r="C572" s="10" t="inlineStr">
         <is>
           <t>F. Gary Gray</t>
         </is>
       </c>
-      <c r="D572" t="n">
+      <c r="D572" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E572" t="n">
+      <c r="E572" s="10" t="n">
         <v>2.77</v>
       </c>
-      <c r="F572" t="n">
+      <c r="F572" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I572" t="n">
+      <c r="I572" s="10" t="n">
         <v>1236000000</v>
       </c>
-      <c r="J572" t="b">
-        <v>0</v>
-      </c>
-      <c r="K572" t="n">
+      <c r="J572" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K572" s="10" t="n">
         <v>250000000</v>
       </c>
-      <c r="L572" t="b">
-        <v>0</v>
-      </c>
-      <c r="M572" t="n">
+      <c r="L572" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M572" s="10" t="n">
         <v>136</v>
       </c>
-      <c r="N572" t="n">
-        <v>0</v>
-      </c>
-      <c r="O572" t="n">
-        <v>0</v>
-      </c>
-      <c r="P572" t="b">
+      <c r="N572" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O572" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P572" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="573">
-      <c r="A573" t="inlineStr">
+      <c r="A573" s="10" t="inlineStr">
         <is>
           <t>Fast &amp; Furious Presents: Hobbs &amp; Shaw</t>
         </is>
       </c>
-      <c r="B573" t="inlineStr">
+      <c r="B573" s="10" t="inlineStr">
         <is>
           <t>card_572</t>
         </is>
       </c>
-      <c r="C573" t="inlineStr">
+      <c r="C573" s="10" t="inlineStr">
         <is>
           <t>David Leitch</t>
         </is>
       </c>
-      <c r="D573" t="n">
+      <c r="D573" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E573" t="n">
+      <c r="E573" s="10" t="n">
         <v>2.73</v>
       </c>
-      <c r="F573" t="n">
+      <c r="F573" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="I573" t="n">
+      <c r="I573" s="10" t="n">
         <v>760000000</v>
       </c>
-      <c r="J573" t="b">
-        <v>0</v>
-      </c>
-      <c r="K573" t="n">
+      <c r="J573" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K573" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L573" t="b">
-        <v>0</v>
-      </c>
-      <c r="M573" t="n">
+      <c r="L573" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M573" s="10" t="n">
         <v>137</v>
       </c>
-      <c r="N573" t="n">
-        <v>0</v>
-      </c>
-      <c r="O573" t="n">
-        <v>0</v>
-      </c>
-      <c r="P573" t="b">
+      <c r="N573" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O573" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P573" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="574">
-      <c r="A574" t="inlineStr">
+      <c r="A574" s="10" t="inlineStr">
         <is>
           <t>F9</t>
         </is>
       </c>
-      <c r="B574" t="inlineStr">
+      <c r="B574" s="10" t="inlineStr">
         <is>
           <t>card_573</t>
         </is>
       </c>
-      <c r="C574" t="inlineStr">
+      <c r="C574" s="10" t="inlineStr">
         <is>
           <t>Justin Lin</t>
         </is>
       </c>
-      <c r="D574" t="n">
+      <c r="D574" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E574" t="n">
+      <c r="E574" s="10" t="n">
         <v>2.4</v>
       </c>
-      <c r="F574" t="n">
+      <c r="F574" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="I574" t="n">
+      <c r="I574" s="10" t="n">
         <v>726200000</v>
       </c>
-      <c r="J574" t="b">
-        <v>0</v>
-      </c>
-      <c r="K574" t="n">
+      <c r="J574" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K574" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L574" t="b">
-        <v>0</v>
-      </c>
-      <c r="M574" t="n">
+      <c r="L574" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M574" s="10" t="n">
         <v>143</v>
       </c>
-      <c r="N574" t="n">
-        <v>0</v>
-      </c>
-      <c r="O574" t="n">
-        <v>0</v>
-      </c>
-      <c r="P574" t="b">
+      <c r="N574" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O574" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P574" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="575">
-      <c r="A575" t="inlineStr">
+      <c r="A575" s="10" t="inlineStr">
         <is>
           <t>Fast X</t>
         </is>
       </c>
-      <c r="B575" t="inlineStr">
+      <c r="B575" s="10" t="inlineStr">
         <is>
           <t>card_574</t>
         </is>
       </c>
-      <c r="C575" t="inlineStr">
+      <c r="C575" s="10" t="inlineStr">
         <is>
           <t>Louis Leterrier</t>
         </is>
       </c>
-      <c r="D575" t="n">
+      <c r="D575" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E575" t="n">
+      <c r="E575" s="10" t="n">
         <v>2.49</v>
       </c>
-      <c r="F575" t="n">
+      <c r="F575" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="I575" t="n">
+      <c r="I575" s="10" t="n">
         <v>714400000</v>
       </c>
-      <c r="J575" t="b">
-        <v>0</v>
-      </c>
-      <c r="K575" t="n">
+      <c r="J575" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K575" s="10" t="n">
         <v>340000000</v>
       </c>
-      <c r="L575" t="b">
-        <v>0</v>
-      </c>
-      <c r="M575" t="n">
+      <c r="L575" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M575" s="10" t="n">
         <v>141</v>
       </c>
-      <c r="N575" t="n">
-        <v>0</v>
-      </c>
-      <c r="O575" t="n">
-        <v>0</v>
-      </c>
-      <c r="P575" t="b">
+      <c r="N575" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O575" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P575" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Spider-Man</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>card_575</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Sam Raimi</t>
+        </is>
+      </c>
+      <c r="D576" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E576" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="F576" t="n">
+        <v>83</v>
+      </c>
+      <c r="I576" t="n">
+        <v>826800000</v>
+      </c>
+      <c r="J576" t="b">
+        <v>0</v>
+      </c>
+      <c r="K576" t="n">
+        <v>139000000</v>
+      </c>
+      <c r="L576" t="b">
+        <v>0</v>
+      </c>
+      <c r="M576" t="n">
+        <v>121</v>
+      </c>
+      <c r="N576" t="n">
+        <v>0</v>
+      </c>
+      <c r="O576" t="n">
+        <v>0</v>
+      </c>
+      <c r="P576" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Spider-Man 3</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>card_576</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Sam Raimi</t>
+        </is>
+      </c>
+      <c r="D577" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E577" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F577" t="n">
+        <v>67</v>
+      </c>
+      <c r="I577" t="n">
+        <v>896300000</v>
+      </c>
+      <c r="J577" t="b">
+        <v>0</v>
+      </c>
+      <c r="K577" t="n">
+        <v>258000000</v>
+      </c>
+      <c r="L577" t="b">
+        <v>0</v>
+      </c>
+      <c r="M577" t="n">
+        <v>139</v>
+      </c>
+      <c r="N577" t="n">
+        <v>0</v>
+      </c>
+      <c r="O577" t="n">
+        <v>0</v>
+      </c>
+      <c r="P577" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>The Amazing Spider-Man</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>card_577</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Marc Webb</t>
+        </is>
+      </c>
+      <c r="D578" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E578" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="F578" t="n">
+        <v>71</v>
+      </c>
+      <c r="I578" t="n">
+        <v>758700000</v>
+      </c>
+      <c r="J578" t="b">
+        <v>0</v>
+      </c>
+      <c r="K578" t="n">
+        <v>230000000</v>
+      </c>
+      <c r="L578" t="b">
+        <v>0</v>
+      </c>
+      <c r="M578" t="n">
+        <v>136</v>
+      </c>
+      <c r="N578" t="n">
+        <v>0</v>
+      </c>
+      <c r="O578" t="n">
+        <v>0</v>
+      </c>
+      <c r="P578" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>The Amazing Spider-Man 2</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>card_578</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>Marc Webb</t>
+        </is>
+      </c>
+      <c r="D579" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E579" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="F579" t="n">
+        <v>64</v>
+      </c>
+      <c r="I579" t="n">
+        <v>717000000</v>
+      </c>
+      <c r="J579" t="b">
+        <v>0</v>
+      </c>
+      <c r="K579" t="n">
+        <v>293000000</v>
+      </c>
+      <c r="L579" t="b">
+        <v>0</v>
+      </c>
+      <c r="M579" t="n">
+        <v>142</v>
+      </c>
+      <c r="N579" t="n">
+        <v>0</v>
+      </c>
+      <c r="O579" t="n">
+        <v>0</v>
+      </c>
+      <c r="P579" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Spider-Man: Into the Spider-Verse</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>card_579</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Bob Persichetti and Peter Ramsey and Rodney Rothman</t>
+        </is>
+      </c>
+      <c r="D580" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E580" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F580" t="n">
+        <v>88</v>
+      </c>
+      <c r="I580" t="n">
+        <v>395000000</v>
+      </c>
+      <c r="J580" t="b">
+        <v>0</v>
+      </c>
+      <c r="K580" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="L580" t="b">
+        <v>0</v>
+      </c>
+      <c r="M580" t="n">
+        <v>117</v>
+      </c>
+      <c r="N580" t="n">
+        <v>1</v>
+      </c>
+      <c r="O580" t="n">
+        <v>0</v>
+      </c>
+      <c r="P580" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Arnold Schwarzenegger films (card_580-590)
Conan the Barbarian, Commando, The Running Man, Twins, Total Recall,
Kindergarten Cop, True Lies, Last Action Hero, Eraser, The 6th Day,
End of Days. Terminator/Predator series were already in the DB.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P580"/>
+  <dimension ref="A1:P591"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -30407,252 +30407,802 @@
       </c>
     </row>
     <row r="576">
-      <c r="A576" t="inlineStr">
+      <c r="A576" s="10" t="inlineStr">
         <is>
           <t>Spider-Man</t>
         </is>
       </c>
-      <c r="B576" t="inlineStr">
+      <c r="B576" s="10" t="inlineStr">
         <is>
           <t>card_575</t>
         </is>
       </c>
-      <c r="C576" t="inlineStr">
+      <c r="C576" s="10" t="inlineStr">
         <is>
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="D576" t="n">
+      <c r="D576" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E576" t="n">
+      <c r="E576" s="10" t="n">
         <v>3.88</v>
       </c>
-      <c r="F576" t="n">
+      <c r="F576" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I576" t="n">
+      <c r="I576" s="10" t="n">
         <v>826800000</v>
       </c>
-      <c r="J576" t="b">
-        <v>0</v>
-      </c>
-      <c r="K576" t="n">
+      <c r="J576" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K576" s="10" t="n">
         <v>139000000</v>
       </c>
-      <c r="L576" t="b">
-        <v>0</v>
-      </c>
-      <c r="M576" t="n">
+      <c r="L576" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M576" s="10" t="n">
         <v>121</v>
       </c>
-      <c r="N576" t="n">
-        <v>0</v>
-      </c>
-      <c r="O576" t="n">
-        <v>0</v>
-      </c>
-      <c r="P576" t="b">
+      <c r="N576" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O576" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P576" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="577">
-      <c r="A577" t="inlineStr">
+      <c r="A577" s="10" t="inlineStr">
         <is>
           <t>Spider-Man 3</t>
         </is>
       </c>
-      <c r="B577" t="inlineStr">
+      <c r="B577" s="10" t="inlineStr">
         <is>
           <t>card_576</t>
         </is>
       </c>
-      <c r="C577" t="inlineStr">
+      <c r="C577" s="10" t="inlineStr">
         <is>
           <t>Sam Raimi</t>
         </is>
       </c>
-      <c r="D577" t="n">
+      <c r="D577" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E577" t="n">
+      <c r="E577" s="10" t="n">
         <v>3.27</v>
       </c>
-      <c r="F577" t="n">
+      <c r="F577" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I577" t="n">
+      <c r="I577" s="10" t="n">
         <v>896300000</v>
       </c>
-      <c r="J577" t="b">
-        <v>0</v>
-      </c>
-      <c r="K577" t="n">
+      <c r="J577" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K577" s="10" t="n">
         <v>258000000</v>
       </c>
-      <c r="L577" t="b">
-        <v>0</v>
-      </c>
-      <c r="M577" t="n">
+      <c r="L577" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M577" s="10" t="n">
         <v>139</v>
       </c>
-      <c r="N577" t="n">
-        <v>0</v>
-      </c>
-      <c r="O577" t="n">
-        <v>0</v>
-      </c>
-      <c r="P577" t="b">
+      <c r="N577" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O577" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P577" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="578">
-      <c r="A578" t="inlineStr">
+      <c r="A578" s="10" t="inlineStr">
         <is>
           <t>The Amazing Spider-Man</t>
         </is>
       </c>
-      <c r="B578" t="inlineStr">
+      <c r="B578" s="10" t="inlineStr">
         <is>
           <t>card_577</t>
         </is>
       </c>
-      <c r="C578" t="inlineStr">
+      <c r="C578" s="10" t="inlineStr">
         <is>
           <t>Marc Webb</t>
         </is>
       </c>
-      <c r="D578" t="n">
+      <c r="D578" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E578" t="n">
+      <c r="E578" s="10" t="n">
         <v>3.59</v>
       </c>
-      <c r="F578" t="n">
+      <c r="F578" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I578" t="n">
+      <c r="I578" s="10" t="n">
         <v>758700000</v>
       </c>
-      <c r="J578" t="b">
-        <v>0</v>
-      </c>
-      <c r="K578" t="n">
+      <c r="J578" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K578" s="10" t="n">
         <v>230000000</v>
       </c>
-      <c r="L578" t="b">
-        <v>0</v>
-      </c>
-      <c r="M578" t="n">
+      <c r="L578" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M578" s="10" t="n">
         <v>136</v>
       </c>
-      <c r="N578" t="n">
-        <v>0</v>
-      </c>
-      <c r="O578" t="n">
-        <v>0</v>
-      </c>
-      <c r="P578" t="b">
+      <c r="N578" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O578" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P578" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="579">
-      <c r="A579" t="inlineStr">
+      <c r="A579" s="10" t="inlineStr">
         <is>
           <t>The Amazing Spider-Man 2</t>
         </is>
       </c>
-      <c r="B579" t="inlineStr">
+      <c r="B579" s="10" t="inlineStr">
         <is>
           <t>card_578</t>
         </is>
       </c>
-      <c r="C579" t="inlineStr">
+      <c r="C579" s="10" t="inlineStr">
         <is>
           <t>Marc Webb</t>
         </is>
       </c>
-      <c r="D579" t="n">
+      <c r="D579" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E579" t="n">
+      <c r="E579" s="10" t="n">
         <v>3.27</v>
       </c>
-      <c r="F579" t="n">
+      <c r="F579" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="I579" t="n">
+      <c r="I579" s="10" t="n">
         <v>717000000</v>
       </c>
-      <c r="J579" t="b">
-        <v>0</v>
-      </c>
-      <c r="K579" t="n">
+      <c r="J579" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K579" s="10" t="n">
         <v>293000000</v>
       </c>
-      <c r="L579" t="b">
-        <v>0</v>
-      </c>
-      <c r="M579" t="n">
+      <c r="L579" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M579" s="10" t="n">
         <v>142</v>
       </c>
-      <c r="N579" t="n">
-        <v>0</v>
-      </c>
-      <c r="O579" t="n">
-        <v>0</v>
-      </c>
-      <c r="P579" t="b">
+      <c r="N579" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O579" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P579" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="580">
-      <c r="A580" t="inlineStr">
+      <c r="A580" s="10" t="inlineStr">
         <is>
           <t>Spider-Man: Into the Spider-Verse</t>
         </is>
       </c>
-      <c r="B580" t="inlineStr">
+      <c r="B580" s="10" t="inlineStr">
         <is>
           <t>card_579</t>
         </is>
       </c>
-      <c r="C580" t="inlineStr">
+      <c r="C580" s="10" t="inlineStr">
         <is>
           <t>Bob Persichetti and Peter Ramsey and Rodney Rothman</t>
         </is>
       </c>
-      <c r="D580" t="n">
+      <c r="D580" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E580" t="n">
+      <c r="E580" s="10" t="n">
         <v>4.4</v>
       </c>
-      <c r="F580" t="n">
+      <c r="F580" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="I580" t="n">
+      <c r="I580" s="10" t="n">
         <v>395000000</v>
       </c>
-      <c r="J580" t="b">
-        <v>0</v>
-      </c>
-      <c r="K580" t="n">
+      <c r="J580" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K580" s="10" t="n">
         <v>90000000</v>
       </c>
-      <c r="L580" t="b">
-        <v>0</v>
-      </c>
-      <c r="M580" t="n">
+      <c r="L580" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M580" s="10" t="n">
         <v>117</v>
       </c>
-      <c r="N580" t="n">
+      <c r="N580" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O580" t="n">
-        <v>0</v>
-      </c>
-      <c r="P580" t="b">
+      <c r="O580" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P580" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Conan the Barbarian</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>card_580</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>John Milius</t>
+        </is>
+      </c>
+      <c r="D581" t="n">
+        <v>1982</v>
+      </c>
+      <c r="E581" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="F581" t="n">
+        <v>78</v>
+      </c>
+      <c r="I581" t="n">
+        <v>79100000</v>
+      </c>
+      <c r="J581" t="b">
+        <v>0</v>
+      </c>
+      <c r="K581" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L581" t="b">
+        <v>0</v>
+      </c>
+      <c r="M581" t="n">
+        <v>129</v>
+      </c>
+      <c r="N581" t="n">
+        <v>0</v>
+      </c>
+      <c r="O581" t="n">
+        <v>0</v>
+      </c>
+      <c r="P581" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Commando</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>card_581</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Mark L. Lester</t>
+        </is>
+      </c>
+      <c r="D582" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E582" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F582" t="n">
+        <v>71</v>
+      </c>
+      <c r="I582" t="n">
+        <v>57500000</v>
+      </c>
+      <c r="J582" t="b">
+        <v>0</v>
+      </c>
+      <c r="K582" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L582" t="b">
+        <v>0</v>
+      </c>
+      <c r="M582" t="n">
+        <v>90</v>
+      </c>
+      <c r="N582" t="n">
+        <v>0</v>
+      </c>
+      <c r="O582" t="n">
+        <v>0</v>
+      </c>
+      <c r="P582" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>The Running Man</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>card_582</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Paul Michael Glaser</t>
+        </is>
+      </c>
+      <c r="D583" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E583" t="n">
+        <v>3.15</v>
+      </c>
+      <c r="F583" t="n">
+        <v>69</v>
+      </c>
+      <c r="I583" t="n">
+        <v>38100000</v>
+      </c>
+      <c r="J583" t="b">
+        <v>0</v>
+      </c>
+      <c r="K583" t="n">
+        <v>27000000</v>
+      </c>
+      <c r="L583" t="b">
+        <v>0</v>
+      </c>
+      <c r="M583" t="n">
+        <v>101</v>
+      </c>
+      <c r="N583" t="n">
+        <v>0</v>
+      </c>
+      <c r="O583" t="n">
+        <v>0</v>
+      </c>
+      <c r="P583" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Twins</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>card_583</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>Ivan Reitman</t>
+        </is>
+      </c>
+      <c r="D584" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E584" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="F584" t="n">
+        <v>68</v>
+      </c>
+      <c r="I584" t="n">
+        <v>216600000</v>
+      </c>
+      <c r="J584" t="b">
+        <v>0</v>
+      </c>
+      <c r="K584" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="L584" t="b">
+        <v>0</v>
+      </c>
+      <c r="M584" t="n">
+        <v>107</v>
+      </c>
+      <c r="N584" t="n">
+        <v>0</v>
+      </c>
+      <c r="O584" t="n">
+        <v>0</v>
+      </c>
+      <c r="P584" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Total Recall</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>card_584</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Paul Verhoeven</t>
+        </is>
+      </c>
+      <c r="D585" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E585" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="F585" t="n">
+        <v>81</v>
+      </c>
+      <c r="I585" t="n">
+        <v>261400000</v>
+      </c>
+      <c r="J585" t="b">
+        <v>0</v>
+      </c>
+      <c r="K585" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="L585" t="b">
+        <v>0</v>
+      </c>
+      <c r="M585" t="n">
+        <v>113</v>
+      </c>
+      <c r="N585" t="n">
+        <v>1</v>
+      </c>
+      <c r="O585" t="n">
+        <v>0</v>
+      </c>
+      <c r="P585" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Kindergarten Cop</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>card_585</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Ivan Reitman</t>
+        </is>
+      </c>
+      <c r="D586" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E586" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F586" t="n">
+        <v>67</v>
+      </c>
+      <c r="I586" t="n">
+        <v>202000000</v>
+      </c>
+      <c r="J586" t="b">
+        <v>0</v>
+      </c>
+      <c r="K586" t="n">
+        <v>26000000</v>
+      </c>
+      <c r="L586" t="b">
+        <v>0</v>
+      </c>
+      <c r="M586" t="n">
+        <v>111</v>
+      </c>
+      <c r="N586" t="n">
+        <v>0</v>
+      </c>
+      <c r="O586" t="n">
+        <v>0</v>
+      </c>
+      <c r="P586" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>True Lies</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>card_586</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>James Cameron</t>
+        </is>
+      </c>
+      <c r="D587" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E587" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F587" t="n">
+        <v>75</v>
+      </c>
+      <c r="I587" t="n">
+        <v>378900000</v>
+      </c>
+      <c r="J587" t="b">
+        <v>0</v>
+      </c>
+      <c r="K587" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L587" t="b">
+        <v>0</v>
+      </c>
+      <c r="M587" t="n">
+        <v>141</v>
+      </c>
+      <c r="N587" t="n">
+        <v>0</v>
+      </c>
+      <c r="O587" t="n">
+        <v>0</v>
+      </c>
+      <c r="P587" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Last Action Hero</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>card_587</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>John McTiernan</t>
+        </is>
+      </c>
+      <c r="D588" t="n">
+        <v>1993</v>
+      </c>
+      <c r="E588" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="F588" t="n">
+        <v>73</v>
+      </c>
+      <c r="I588" t="n">
+        <v>137300000</v>
+      </c>
+      <c r="J588" t="b">
+        <v>0</v>
+      </c>
+      <c r="K588" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="L588" t="b">
+        <v>0</v>
+      </c>
+      <c r="M588" t="n">
+        <v>131</v>
+      </c>
+      <c r="N588" t="n">
+        <v>0</v>
+      </c>
+      <c r="O588" t="n">
+        <v>0</v>
+      </c>
+      <c r="P588" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Eraser</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>card_588</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Chuck Russell</t>
+        </is>
+      </c>
+      <c r="D589" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E589" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="F589" t="n">
+        <v>66</v>
+      </c>
+      <c r="I589" t="n">
+        <v>242000000</v>
+      </c>
+      <c r="J589" t="b">
+        <v>0</v>
+      </c>
+      <c r="K589" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L589" t="b">
+        <v>0</v>
+      </c>
+      <c r="M589" t="n">
+        <v>114</v>
+      </c>
+      <c r="N589" t="n">
+        <v>0</v>
+      </c>
+      <c r="O589" t="n">
+        <v>0</v>
+      </c>
+      <c r="P589" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>The 6th Day</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>card_589</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Roger Spottiswoode</t>
+        </is>
+      </c>
+      <c r="D590" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E590" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="F590" t="n">
+        <v>63</v>
+      </c>
+      <c r="I590" t="n">
+        <v>96000000</v>
+      </c>
+      <c r="J590" t="b">
+        <v>0</v>
+      </c>
+      <c r="K590" t="n">
+        <v>82000000</v>
+      </c>
+      <c r="L590" t="b">
+        <v>0</v>
+      </c>
+      <c r="M590" t="n">
+        <v>124</v>
+      </c>
+      <c r="N590" t="n">
+        <v>0</v>
+      </c>
+      <c r="O590" t="n">
+        <v>0</v>
+      </c>
+      <c r="P590" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>End of Days</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>card_590</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Peter Hyams</t>
+        </is>
+      </c>
+      <c r="D591" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E591" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="F591" t="n">
+        <v>62</v>
+      </c>
+      <c r="I591" t="n">
+        <v>212000000</v>
+      </c>
+      <c r="J591" t="b">
+        <v>0</v>
+      </c>
+      <c r="K591" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L591" t="b">
+        <v>0</v>
+      </c>
+      <c r="M591" t="n">
+        <v>122</v>
+      </c>
+      <c r="N591" t="n">
+        <v>0</v>
+      </c>
+      <c r="O591" t="n">
+        <v>0</v>
+      </c>
+      <c r="P591" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Police Academy series (card_591-597)
All 7 films, Police Academy (1984) through Mission to Moscow (1994).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P591"/>
+  <dimension ref="A1:P598"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -30657,552 +30657,902 @@
       </c>
     </row>
     <row r="581">
-      <c r="A581" t="inlineStr">
+      <c r="A581" s="10" t="inlineStr">
         <is>
           <t>Conan the Barbarian</t>
         </is>
       </c>
-      <c r="B581" t="inlineStr">
+      <c r="B581" s="10" t="inlineStr">
         <is>
           <t>card_580</t>
         </is>
       </c>
-      <c r="C581" t="inlineStr">
+      <c r="C581" s="10" t="inlineStr">
         <is>
           <t>John Milius</t>
         </is>
       </c>
-      <c r="D581" t="n">
+      <c r="D581" s="10" t="n">
         <v>1982</v>
       </c>
-      <c r="E581" t="n">
+      <c r="E581" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="F581" t="n">
+      <c r="F581" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I581" t="n">
+      <c r="I581" s="10" t="n">
         <v>79100000</v>
       </c>
-      <c r="J581" t="b">
-        <v>0</v>
-      </c>
-      <c r="K581" t="n">
+      <c r="J581" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K581" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L581" t="b">
-        <v>0</v>
-      </c>
-      <c r="M581" t="n">
+      <c r="L581" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M581" s="10" t="n">
         <v>129</v>
       </c>
-      <c r="N581" t="n">
-        <v>0</v>
-      </c>
-      <c r="O581" t="n">
-        <v>0</v>
-      </c>
-      <c r="P581" t="b">
+      <c r="N581" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O581" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P581" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="582">
-      <c r="A582" t="inlineStr">
+      <c r="A582" s="10" t="inlineStr">
         <is>
           <t>Commando</t>
         </is>
       </c>
-      <c r="B582" t="inlineStr">
+      <c r="B582" s="10" t="inlineStr">
         <is>
           <t>card_581</t>
         </is>
       </c>
-      <c r="C582" t="inlineStr">
+      <c r="C582" s="10" t="inlineStr">
         <is>
           <t>Mark L. Lester</t>
         </is>
       </c>
-      <c r="D582" t="n">
+      <c r="D582" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E582" t="n">
+      <c r="E582" s="10" t="n">
         <v>3.4</v>
       </c>
-      <c r="F582" t="n">
+      <c r="F582" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I582" t="n">
+      <c r="I582" s="10" t="n">
         <v>57500000</v>
       </c>
-      <c r="J582" t="b">
-        <v>0</v>
-      </c>
-      <c r="K582" t="n">
+      <c r="J582" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K582" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L582" t="b">
-        <v>0</v>
-      </c>
-      <c r="M582" t="n">
+      <c r="L582" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M582" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="N582" t="n">
-        <v>0</v>
-      </c>
-      <c r="O582" t="n">
-        <v>0</v>
-      </c>
-      <c r="P582" t="b">
+      <c r="N582" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O582" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P582" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="583">
-      <c r="A583" t="inlineStr">
+      <c r="A583" s="10" t="inlineStr">
         <is>
           <t>The Running Man</t>
         </is>
       </c>
-      <c r="B583" t="inlineStr">
+      <c r="B583" s="10" t="inlineStr">
         <is>
           <t>card_582</t>
         </is>
       </c>
-      <c r="C583" t="inlineStr">
+      <c r="C583" s="10" t="inlineStr">
         <is>
           <t>Paul Michael Glaser</t>
         </is>
       </c>
-      <c r="D583" t="n">
+      <c r="D583" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E583" t="n">
+      <c r="E583" s="10" t="n">
         <v>3.15</v>
       </c>
-      <c r="F583" t="n">
+      <c r="F583" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I583" t="n">
+      <c r="I583" s="10" t="n">
         <v>38100000</v>
       </c>
-      <c r="J583" t="b">
-        <v>0</v>
-      </c>
-      <c r="K583" t="n">
+      <c r="J583" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K583" s="10" t="n">
         <v>27000000</v>
       </c>
-      <c r="L583" t="b">
-        <v>0</v>
-      </c>
-      <c r="M583" t="n">
+      <c r="L583" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M583" s="10" t="n">
         <v>101</v>
       </c>
-      <c r="N583" t="n">
-        <v>0</v>
-      </c>
-      <c r="O583" t="n">
-        <v>0</v>
-      </c>
-      <c r="P583" t="b">
+      <c r="N583" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O583" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P583" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="584">
-      <c r="A584" t="inlineStr">
+      <c r="A584" s="10" t="inlineStr">
         <is>
           <t>Twins</t>
         </is>
       </c>
-      <c r="B584" t="inlineStr">
+      <c r="B584" s="10" t="inlineStr">
         <is>
           <t>card_583</t>
         </is>
       </c>
-      <c r="C584" t="inlineStr">
+      <c r="C584" s="10" t="inlineStr">
         <is>
           <t>Ivan Reitman</t>
         </is>
       </c>
-      <c r="D584" t="n">
+      <c r="D584" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E584" t="n">
+      <c r="E584" s="10" t="n">
         <v>3.05</v>
       </c>
-      <c r="F584" t="n">
+      <c r="F584" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I584" t="n">
+      <c r="I584" s="10" t="n">
         <v>216600000</v>
       </c>
-      <c r="J584" t="b">
-        <v>0</v>
-      </c>
-      <c r="K584" t="n">
+      <c r="J584" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K584" s="10" t="n">
         <v>18000000</v>
       </c>
-      <c r="L584" t="b">
-        <v>0</v>
-      </c>
-      <c r="M584" t="n">
+      <c r="L584" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M584" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N584" t="n">
-        <v>0</v>
-      </c>
-      <c r="O584" t="n">
-        <v>0</v>
-      </c>
-      <c r="P584" t="b">
+      <c r="N584" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O584" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P584" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="585">
-      <c r="A585" t="inlineStr">
+      <c r="A585" s="10" t="inlineStr">
         <is>
           <t>Total Recall</t>
         </is>
       </c>
-      <c r="B585" t="inlineStr">
+      <c r="B585" s="10" t="inlineStr">
         <is>
           <t>card_584</t>
         </is>
       </c>
-      <c r="C585" t="inlineStr">
+      <c r="C585" s="10" t="inlineStr">
         <is>
           <t>Paul Verhoeven</t>
         </is>
       </c>
-      <c r="D585" t="n">
+      <c r="D585" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E585" t="n">
+      <c r="E585" s="10" t="n">
         <v>3.82</v>
       </c>
-      <c r="F585" t="n">
+      <c r="F585" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I585" t="n">
+      <c r="I585" s="10" t="n">
         <v>261400000</v>
       </c>
-      <c r="J585" t="b">
-        <v>0</v>
-      </c>
-      <c r="K585" t="n">
+      <c r="J585" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K585" s="10" t="n">
         <v>65000000</v>
       </c>
-      <c r="L585" t="b">
-        <v>0</v>
-      </c>
-      <c r="M585" t="n">
+      <c r="L585" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M585" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="N585" t="n">
+      <c r="N585" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O585" t="n">
-        <v>0</v>
-      </c>
-      <c r="P585" t="b">
+      <c r="O585" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P585" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="586">
-      <c r="A586" t="inlineStr">
+      <c r="A586" s="10" t="inlineStr">
         <is>
           <t>Kindergarten Cop</t>
         </is>
       </c>
-      <c r="B586" t="inlineStr">
+      <c r="B586" s="10" t="inlineStr">
         <is>
           <t>card_585</t>
         </is>
       </c>
-      <c r="C586" t="inlineStr">
+      <c r="C586" s="10" t="inlineStr">
         <is>
           <t>Ivan Reitman</t>
         </is>
       </c>
-      <c r="D586" t="n">
+      <c r="D586" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E586" t="n">
+      <c r="E586" s="10" t="n">
         <v>3.19</v>
       </c>
-      <c r="F586" t="n">
+      <c r="F586" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I586" t="n">
+      <c r="I586" s="10" t="n">
         <v>202000000</v>
       </c>
-      <c r="J586" t="b">
-        <v>0</v>
-      </c>
-      <c r="K586" t="n">
+      <c r="J586" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K586" s="10" t="n">
         <v>26000000</v>
       </c>
-      <c r="L586" t="b">
-        <v>0</v>
-      </c>
-      <c r="M586" t="n">
+      <c r="L586" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M586" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N586" t="n">
-        <v>0</v>
-      </c>
-      <c r="O586" t="n">
-        <v>0</v>
-      </c>
-      <c r="P586" t="b">
+      <c r="N586" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O586" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P586" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="587">
-      <c r="A587" t="inlineStr">
+      <c r="A587" s="10" t="inlineStr">
         <is>
           <t>True Lies</t>
         </is>
       </c>
-      <c r="B587" t="inlineStr">
+      <c r="B587" s="10" t="inlineStr">
         <is>
           <t>card_586</t>
         </is>
       </c>
-      <c r="C587" t="inlineStr">
+      <c r="C587" s="10" t="inlineStr">
         <is>
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="D587" t="n">
+      <c r="D587" s="10" t="n">
         <v>1994</v>
       </c>
-      <c r="E587" t="n">
+      <c r="E587" s="10" t="n">
         <v>3.6</v>
       </c>
-      <c r="F587" t="n">
+      <c r="F587" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I587" t="n">
+      <c r="I587" s="10" t="n">
         <v>378900000</v>
       </c>
-      <c r="J587" t="b">
-        <v>0</v>
-      </c>
-      <c r="K587" t="n">
+      <c r="J587" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K587" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L587" t="b">
-        <v>0</v>
-      </c>
-      <c r="M587" t="n">
+      <c r="L587" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M587" s="10" t="n">
         <v>141</v>
       </c>
-      <c r="N587" t="n">
-        <v>0</v>
-      </c>
-      <c r="O587" t="n">
-        <v>0</v>
-      </c>
-      <c r="P587" t="b">
+      <c r="N587" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O587" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P587" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="588">
-      <c r="A588" t="inlineStr">
+      <c r="A588" s="10" t="inlineStr">
         <is>
           <t>Last Action Hero</t>
         </is>
       </c>
-      <c r="B588" t="inlineStr">
+      <c r="B588" s="10" t="inlineStr">
         <is>
           <t>card_587</t>
         </is>
       </c>
-      <c r="C588" t="inlineStr">
+      <c r="C588" s="10" t="inlineStr">
         <is>
           <t>John McTiernan</t>
         </is>
       </c>
-      <c r="D588" t="n">
+      <c r="D588" s="10" t="n">
         <v>1993</v>
       </c>
-      <c r="E588" t="n">
+      <c r="E588" s="10" t="n">
         <v>3.44</v>
       </c>
-      <c r="F588" t="n">
+      <c r="F588" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I588" t="n">
+      <c r="I588" s="10" t="n">
         <v>137300000</v>
       </c>
-      <c r="J588" t="b">
-        <v>0</v>
-      </c>
-      <c r="K588" t="n">
+      <c r="J588" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K588" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="L588" t="b">
-        <v>0</v>
-      </c>
-      <c r="M588" t="n">
+      <c r="L588" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M588" s="10" t="n">
         <v>131</v>
       </c>
-      <c r="N588" t="n">
-        <v>0</v>
-      </c>
-      <c r="O588" t="n">
-        <v>0</v>
-      </c>
-      <c r="P588" t="b">
+      <c r="N588" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O588" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P588" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="589">
-      <c r="A589" t="inlineStr">
+      <c r="A589" s="10" t="inlineStr">
         <is>
           <t>Eraser</t>
         </is>
       </c>
-      <c r="B589" t="inlineStr">
+      <c r="B589" s="10" t="inlineStr">
         <is>
           <t>card_588</t>
         </is>
       </c>
-      <c r="C589" t="inlineStr">
+      <c r="C589" s="10" t="inlineStr">
         <is>
           <t>Chuck Russell</t>
         </is>
       </c>
-      <c r="D589" t="n">
+      <c r="D589" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E589" t="n">
+      <c r="E589" s="10" t="n">
         <v>2.93</v>
       </c>
-      <c r="F589" t="n">
+      <c r="F589" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I589" t="n">
+      <c r="I589" s="10" t="n">
         <v>242000000</v>
       </c>
-      <c r="J589" t="b">
-        <v>0</v>
-      </c>
-      <c r="K589" t="n">
+      <c r="J589" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K589" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L589" t="b">
-        <v>0</v>
-      </c>
-      <c r="M589" t="n">
+      <c r="L589" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M589" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N589" t="n">
-        <v>0</v>
-      </c>
-      <c r="O589" t="n">
-        <v>0</v>
-      </c>
-      <c r="P589" t="b">
+      <c r="N589" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O589" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P589" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="590">
-      <c r="A590" t="inlineStr">
+      <c r="A590" s="10" t="inlineStr">
         <is>
           <t>The 6th Day</t>
         </is>
       </c>
-      <c r="B590" t="inlineStr">
+      <c r="B590" s="10" t="inlineStr">
         <is>
           <t>card_589</t>
         </is>
       </c>
-      <c r="C590" t="inlineStr">
+      <c r="C590" s="10" t="inlineStr">
         <is>
           <t>Roger Spottiswoode</t>
         </is>
       </c>
-      <c r="D590" t="n">
+      <c r="D590" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E590" t="n">
+      <c r="E590" s="10" t="n">
         <v>2.79</v>
       </c>
-      <c r="F590" t="n">
+      <c r="F590" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I590" t="n">
+      <c r="I590" s="10" t="n">
         <v>96000000</v>
       </c>
-      <c r="J590" t="b">
-        <v>0</v>
-      </c>
-      <c r="K590" t="n">
+      <c r="J590" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K590" s="10" t="n">
         <v>82000000</v>
       </c>
-      <c r="L590" t="b">
-        <v>0</v>
-      </c>
-      <c r="M590" t="n">
+      <c r="L590" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M590" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="N590" t="n">
-        <v>0</v>
-      </c>
-      <c r="O590" t="n">
-        <v>0</v>
-      </c>
-      <c r="P590" t="b">
+      <c r="N590" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O590" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P590" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="591">
-      <c r="A591" t="inlineStr">
+      <c r="A591" s="10" t="inlineStr">
         <is>
           <t>End of Days</t>
         </is>
       </c>
-      <c r="B591" t="inlineStr">
+      <c r="B591" s="10" t="inlineStr">
         <is>
           <t>card_590</t>
         </is>
       </c>
-      <c r="C591" t="inlineStr">
+      <c r="C591" s="10" t="inlineStr">
         <is>
           <t>Peter Hyams</t>
         </is>
       </c>
-      <c r="D591" t="n">
+      <c r="D591" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E591" t="n">
+      <c r="E591" s="10" t="n">
         <v>2.74</v>
       </c>
-      <c r="F591" t="n">
+      <c r="F591" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I591" t="n">
+      <c r="I591" s="10" t="n">
         <v>212000000</v>
       </c>
-      <c r="J591" t="b">
-        <v>0</v>
-      </c>
-      <c r="K591" t="n">
+      <c r="J591" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K591" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L591" t="b">
-        <v>0</v>
-      </c>
-      <c r="M591" t="n">
+      <c r="L591" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M591" s="10" t="n">
         <v>122</v>
       </c>
-      <c r="N591" t="n">
-        <v>0</v>
-      </c>
-      <c r="O591" t="n">
-        <v>0</v>
-      </c>
-      <c r="P591" t="b">
+      <c r="N591" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O591" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P591" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Police Academy</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>card_591</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Hugh Wilson</t>
+        </is>
+      </c>
+      <c r="D592" t="n">
+        <v>1984</v>
+      </c>
+      <c r="E592" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="F592" t="n">
+        <v>71</v>
+      </c>
+      <c r="I592" t="n">
+        <v>149800000</v>
+      </c>
+      <c r="J592" t="b">
+        <v>0</v>
+      </c>
+      <c r="K592" t="n">
+        <v>4800000</v>
+      </c>
+      <c r="L592" t="b">
+        <v>0</v>
+      </c>
+      <c r="M592" t="n">
+        <v>96</v>
+      </c>
+      <c r="N592" t="n">
+        <v>0</v>
+      </c>
+      <c r="O592" t="n">
+        <v>0</v>
+      </c>
+      <c r="P592" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Police Academy 2: Their First Assignment</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>card_592</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Jerry Paris</t>
+        </is>
+      </c>
+      <c r="D593" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E593" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="F593" t="n">
+        <v>65</v>
+      </c>
+      <c r="I593" t="n">
+        <v>115000000</v>
+      </c>
+      <c r="J593" t="b">
+        <v>0</v>
+      </c>
+      <c r="K593" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="L593" t="b">
+        <v>0</v>
+      </c>
+      <c r="M593" t="n">
+        <v>87</v>
+      </c>
+      <c r="N593" t="n">
+        <v>0</v>
+      </c>
+      <c r="O593" t="n">
+        <v>0</v>
+      </c>
+      <c r="P593" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Police Academy 3: Back in Training</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>card_593</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>Jerry Paris</t>
+        </is>
+      </c>
+      <c r="D594" t="n">
+        <v>1986</v>
+      </c>
+      <c r="E594" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="F594" t="n">
+        <v>60</v>
+      </c>
+      <c r="I594" t="n">
+        <v>107600000</v>
+      </c>
+      <c r="J594" t="b">
+        <v>0</v>
+      </c>
+      <c r="K594" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="L594" t="b">
+        <v>0</v>
+      </c>
+      <c r="M594" t="n">
+        <v>84</v>
+      </c>
+      <c r="N594" t="n">
+        <v>0</v>
+      </c>
+      <c r="O594" t="n">
+        <v>0</v>
+      </c>
+      <c r="P594" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Police Academy 4: Citizens on Patrol</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>card_594</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>Jim Drake</t>
+        </is>
+      </c>
+      <c r="D595" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E595" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="F595" t="n">
+        <v>58</v>
+      </c>
+      <c r="I595" t="n">
+        <v>76800000</v>
+      </c>
+      <c r="J595" t="b">
+        <v>0</v>
+      </c>
+      <c r="K595" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="L595" t="b">
+        <v>0</v>
+      </c>
+      <c r="M595" t="n">
+        <v>87</v>
+      </c>
+      <c r="N595" t="n">
+        <v>0</v>
+      </c>
+      <c r="O595" t="n">
+        <v>0</v>
+      </c>
+      <c r="P595" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Police Academy 5: Assignment: Miami Beach</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>card_595</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>Alan Myerson</t>
+        </is>
+      </c>
+      <c r="D596" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E596" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="F596" t="n">
+        <v>58</v>
+      </c>
+      <c r="I596" t="n">
+        <v>54500000</v>
+      </c>
+      <c r="J596" t="b">
+        <v>0</v>
+      </c>
+      <c r="K596" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="L596" t="b">
+        <v>0</v>
+      </c>
+      <c r="M596" t="n">
+        <v>90</v>
+      </c>
+      <c r="N596" t="n">
+        <v>0</v>
+      </c>
+      <c r="O596" t="n">
+        <v>0</v>
+      </c>
+      <c r="P596" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Police Academy 6: City Under Siege</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>card_596</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Peter Bonerz</t>
+        </is>
+      </c>
+      <c r="D597" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E597" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="F597" t="n">
+        <v>56</v>
+      </c>
+      <c r="I597" t="n">
+        <v>33200000</v>
+      </c>
+      <c r="J597" t="b">
+        <v>0</v>
+      </c>
+      <c r="K597" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L597" t="b">
+        <v>0</v>
+      </c>
+      <c r="M597" t="n">
+        <v>84</v>
+      </c>
+      <c r="N597" t="n">
+        <v>0</v>
+      </c>
+      <c r="O597" t="n">
+        <v>0</v>
+      </c>
+      <c r="P597" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Police Academy: Mission to Moscow</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>card_597</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Alan Metter</t>
+        </is>
+      </c>
+      <c r="D598" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E598" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="F598" t="n">
+        <v>45</v>
+      </c>
+      <c r="I598" t="n">
+        <v>4300000</v>
+      </c>
+      <c r="J598" t="b">
+        <v>0</v>
+      </c>
+      <c r="K598" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="L598" t="b">
+        <v>0</v>
+      </c>
+      <c r="M598" t="n">
+        <v>83</v>
+      </c>
+      <c r="N598" t="n">
+        <v>0</v>
+      </c>
+      <c r="O598" t="n">
+        <v>0</v>
+      </c>
+      <c r="P598" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Sean Connery non-Bond films (card_598-604)
The Hunt for Red October, The Untouchables, The Rock, Entrapment,
Finding Forrester, The Man Who Would Be King, Murder on the Orient
Express (1974). Bond films and Highlander/Last Crusade already in DB.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P598"/>
+  <dimension ref="A1:P605"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -31207,352 +31207,702 @@
       </c>
     </row>
     <row r="592">
-      <c r="A592" t="inlineStr">
+      <c r="A592" s="10" t="inlineStr">
         <is>
           <t>Police Academy</t>
         </is>
       </c>
-      <c r="B592" t="inlineStr">
+      <c r="B592" s="10" t="inlineStr">
         <is>
           <t>card_591</t>
         </is>
       </c>
-      <c r="C592" t="inlineStr">
+      <c r="C592" s="10" t="inlineStr">
         <is>
           <t>Hugh Wilson</t>
         </is>
       </c>
-      <c r="D592" t="n">
+      <c r="D592" s="10" t="n">
         <v>1984</v>
       </c>
-      <c r="E592" t="n">
+      <c r="E592" s="10" t="n">
         <v>3.23</v>
       </c>
-      <c r="F592" t="n">
+      <c r="F592" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I592" t="n">
+      <c r="I592" s="10" t="n">
         <v>149800000</v>
       </c>
-      <c r="J592" t="b">
-        <v>0</v>
-      </c>
-      <c r="K592" t="n">
+      <c r="J592" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K592" s="10" t="n">
         <v>4800000</v>
       </c>
-      <c r="L592" t="b">
-        <v>0</v>
-      </c>
-      <c r="M592" t="n">
+      <c r="L592" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M592" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N592" t="n">
-        <v>0</v>
-      </c>
-      <c r="O592" t="n">
-        <v>0</v>
-      </c>
-      <c r="P592" t="b">
+      <c r="N592" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O592" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P592" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="593">
-      <c r="A593" t="inlineStr">
+      <c r="A593" s="10" t="inlineStr">
         <is>
           <t>Police Academy 2: Their First Assignment</t>
         </is>
       </c>
-      <c r="B593" t="inlineStr">
+      <c r="B593" s="10" t="inlineStr">
         <is>
           <t>card_592</t>
         </is>
       </c>
-      <c r="C593" t="inlineStr">
+      <c r="C593" s="10" t="inlineStr">
         <is>
           <t>Jerry Paris</t>
         </is>
       </c>
-      <c r="D593" t="n">
+      <c r="D593" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E593" t="n">
+      <c r="E593" s="10" t="n">
         <v>2.88</v>
       </c>
-      <c r="F593" t="n">
+      <c r="F593" s="10" t="n">
         <v>65</v>
       </c>
-      <c r="I593" t="n">
+      <c r="I593" s="10" t="n">
         <v>115000000</v>
       </c>
-      <c r="J593" t="b">
-        <v>0</v>
-      </c>
-      <c r="K593" t="n">
+      <c r="J593" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K593" s="10" t="n">
         <v>7500000</v>
       </c>
-      <c r="L593" t="b">
-        <v>0</v>
-      </c>
-      <c r="M593" t="n">
+      <c r="L593" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M593" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="N593" t="n">
-        <v>0</v>
-      </c>
-      <c r="O593" t="n">
-        <v>0</v>
-      </c>
-      <c r="P593" t="b">
+      <c r="N593" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O593" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P593" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="594">
-      <c r="A594" t="inlineStr">
+      <c r="A594" s="10" t="inlineStr">
         <is>
           <t>Police Academy 3: Back in Training</t>
         </is>
       </c>
-      <c r="B594" t="inlineStr">
+      <c r="B594" s="10" t="inlineStr">
         <is>
           <t>card_593</t>
         </is>
       </c>
-      <c r="C594" t="inlineStr">
+      <c r="C594" s="10" t="inlineStr">
         <is>
           <t>Jerry Paris</t>
         </is>
       </c>
-      <c r="D594" t="n">
+      <c r="D594" s="10" t="n">
         <v>1986</v>
       </c>
-      <c r="E594" t="n">
+      <c r="E594" s="10" t="n">
         <v>2.74</v>
       </c>
-      <c r="F594" t="n">
+      <c r="F594" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="I594" t="n">
+      <c r="I594" s="10" t="n">
         <v>107600000</v>
       </c>
-      <c r="J594" t="b">
-        <v>0</v>
-      </c>
-      <c r="K594" t="n">
+      <c r="J594" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K594" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="L594" t="b">
-        <v>0</v>
-      </c>
-      <c r="M594" t="n">
+      <c r="L594" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M594" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="N594" t="n">
-        <v>0</v>
-      </c>
-      <c r="O594" t="n">
-        <v>0</v>
-      </c>
-      <c r="P594" t="b">
+      <c r="N594" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O594" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P594" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="595">
-      <c r="A595" t="inlineStr">
+      <c r="A595" s="10" t="inlineStr">
         <is>
           <t>Police Academy 4: Citizens on Patrol</t>
         </is>
       </c>
-      <c r="B595" t="inlineStr">
+      <c r="B595" s="10" t="inlineStr">
         <is>
           <t>card_594</t>
         </is>
       </c>
-      <c r="C595" t="inlineStr">
+      <c r="C595" s="10" t="inlineStr">
         <is>
           <t>Jim Drake</t>
         </is>
       </c>
-      <c r="D595" t="n">
+      <c r="D595" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E595" t="n">
+      <c r="E595" s="10" t="n">
         <v>2.62</v>
       </c>
-      <c r="F595" t="n">
+      <c r="F595" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="I595" t="n">
+      <c r="I595" s="10" t="n">
         <v>76800000</v>
       </c>
-      <c r="J595" t="b">
-        <v>0</v>
-      </c>
-      <c r="K595" t="n">
+      <c r="J595" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K595" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="L595" t="b">
-        <v>0</v>
-      </c>
-      <c r="M595" t="n">
+      <c r="L595" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M595" s="10" t="n">
         <v>87</v>
       </c>
-      <c r="N595" t="n">
-        <v>0</v>
-      </c>
-      <c r="O595" t="n">
-        <v>0</v>
-      </c>
-      <c r="P595" t="b">
+      <c r="N595" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O595" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P595" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="596">
-      <c r="A596" t="inlineStr">
+      <c r="A596" s="10" t="inlineStr">
         <is>
           <t>Police Academy 5: Assignment: Miami Beach</t>
         </is>
       </c>
-      <c r="B596" t="inlineStr">
+      <c r="B596" s="10" t="inlineStr">
         <is>
           <t>card_595</t>
         </is>
       </c>
-      <c r="C596" t="inlineStr">
+      <c r="C596" s="10" t="inlineStr">
         <is>
           <t>Alan Myerson</t>
         </is>
       </c>
-      <c r="D596" t="n">
+      <c r="D596" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E596" t="n">
+      <c r="E596" s="10" t="n">
         <v>2.37</v>
       </c>
-      <c r="F596" t="n">
+      <c r="F596" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="I596" t="n">
+      <c r="I596" s="10" t="n">
         <v>54500000</v>
       </c>
-      <c r="J596" t="b">
-        <v>0</v>
-      </c>
-      <c r="K596" t="n">
+      <c r="J596" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K596" s="10" t="n">
         <v>14000000</v>
       </c>
-      <c r="L596" t="b">
-        <v>0</v>
-      </c>
-      <c r="M596" t="n">
+      <c r="L596" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M596" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="N596" t="n">
-        <v>0</v>
-      </c>
-      <c r="O596" t="n">
-        <v>0</v>
-      </c>
-      <c r="P596" t="b">
+      <c r="N596" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O596" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P596" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="597">
-      <c r="A597" t="inlineStr">
+      <c r="A597" s="10" t="inlineStr">
         <is>
           <t>Police Academy 6: City Under Siege</t>
         </is>
       </c>
-      <c r="B597" t="inlineStr">
+      <c r="B597" s="10" t="inlineStr">
         <is>
           <t>card_596</t>
         </is>
       </c>
-      <c r="C597" t="inlineStr">
+      <c r="C597" s="10" t="inlineStr">
         <is>
           <t>Peter Bonerz</t>
         </is>
       </c>
-      <c r="D597" t="n">
+      <c r="D597" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E597" t="n">
+      <c r="E597" s="10" t="n">
         <v>2.26</v>
       </c>
-      <c r="F597" t="n">
+      <c r="F597" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="I597" t="n">
+      <c r="I597" s="10" t="n">
         <v>33200000</v>
       </c>
-      <c r="J597" t="b">
-        <v>0</v>
-      </c>
-      <c r="K597" t="n">
+      <c r="J597" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K597" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L597" t="b">
-        <v>0</v>
-      </c>
-      <c r="M597" t="n">
+      <c r="L597" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M597" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="N597" t="n">
-        <v>0</v>
-      </c>
-      <c r="O597" t="n">
-        <v>0</v>
-      </c>
-      <c r="P597" t="b">
+      <c r="N597" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O597" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P597" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="598">
-      <c r="A598" t="inlineStr">
+      <c r="A598" s="10" t="inlineStr">
         <is>
           <t>Police Academy: Mission to Moscow</t>
         </is>
       </c>
-      <c r="B598" t="inlineStr">
+      <c r="B598" s="10" t="inlineStr">
         <is>
           <t>card_597</t>
         </is>
       </c>
-      <c r="C598" t="inlineStr">
+      <c r="C598" s="10" t="inlineStr">
         <is>
           <t>Alan Metter</t>
         </is>
       </c>
-      <c r="D598" t="n">
+      <c r="D598" s="10" t="n">
         <v>1994</v>
       </c>
-      <c r="E598" t="n">
+      <c r="E598" s="10" t="n">
         <v>1.83</v>
       </c>
-      <c r="F598" t="n">
+      <c r="F598" s="10" t="n">
         <v>45</v>
       </c>
-      <c r="I598" t="n">
+      <c r="I598" s="10" t="n">
         <v>4300000</v>
       </c>
-      <c r="J598" t="b">
-        <v>0</v>
-      </c>
-      <c r="K598" t="n">
+      <c r="J598" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K598" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="L598" t="b">
-        <v>0</v>
-      </c>
-      <c r="M598" t="n">
+      <c r="L598" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M598" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="N598" t="n">
-        <v>0</v>
-      </c>
-      <c r="O598" t="n">
-        <v>0</v>
-      </c>
-      <c r="P598" t="b">
+      <c r="N598" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O598" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P598" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>The Hunt for Red October</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>card_598</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>John McTiernan</t>
+        </is>
+      </c>
+      <c r="D599" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E599" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F599" t="n">
+        <v>76</v>
+      </c>
+      <c r="I599" t="n">
+        <v>200500000</v>
+      </c>
+      <c r="J599" t="b">
+        <v>0</v>
+      </c>
+      <c r="K599" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L599" t="b">
+        <v>0</v>
+      </c>
+      <c r="M599" t="n">
+        <v>135</v>
+      </c>
+      <c r="N599" t="n">
+        <v>1</v>
+      </c>
+      <c r="O599" t="n">
+        <v>0</v>
+      </c>
+      <c r="P599" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>The Untouchables</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>card_599</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Brian De Palma</t>
+        </is>
+      </c>
+      <c r="D600" t="n">
+        <v>1987</v>
+      </c>
+      <c r="E600" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F600" t="n">
+        <v>80</v>
+      </c>
+      <c r="I600" t="n">
+        <v>187000000</v>
+      </c>
+      <c r="J600" t="b">
+        <v>0</v>
+      </c>
+      <c r="K600" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="L600" t="b">
+        <v>0</v>
+      </c>
+      <c r="M600" t="n">
+        <v>119</v>
+      </c>
+      <c r="N600" t="n">
+        <v>1</v>
+      </c>
+      <c r="O600" t="n">
+        <v>0</v>
+      </c>
+      <c r="P600" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>The Rock</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>card_600</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Michael Bay</t>
+        </is>
+      </c>
+      <c r="D601" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E601" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="F601" t="n">
+        <v>75</v>
+      </c>
+      <c r="I601" t="n">
+        <v>335600000</v>
+      </c>
+      <c r="J601" t="b">
+        <v>0</v>
+      </c>
+      <c r="K601" t="n">
+        <v>75000000</v>
+      </c>
+      <c r="L601" t="b">
+        <v>0</v>
+      </c>
+      <c r="M601" t="n">
+        <v>136</v>
+      </c>
+      <c r="N601" t="n">
+        <v>0</v>
+      </c>
+      <c r="O601" t="n">
+        <v>0</v>
+      </c>
+      <c r="P601" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Entrapment</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>card_601</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>Jon Amiel</t>
+        </is>
+      </c>
+      <c r="D602" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E602" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F602" t="n">
+        <v>64</v>
+      </c>
+      <c r="I602" t="n">
+        <v>212000000</v>
+      </c>
+      <c r="J602" t="b">
+        <v>0</v>
+      </c>
+      <c r="K602" t="n">
+        <v>66000000</v>
+      </c>
+      <c r="L602" t="b">
+        <v>0</v>
+      </c>
+      <c r="M602" t="n">
+        <v>113</v>
+      </c>
+      <c r="N602" t="n">
+        <v>0</v>
+      </c>
+      <c r="O602" t="n">
+        <v>0</v>
+      </c>
+      <c r="P602" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Finding Forrester</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>card_602</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Gus Van Sant</t>
+        </is>
+      </c>
+      <c r="D603" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E603" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="F603" t="n">
+        <v>69</v>
+      </c>
+      <c r="I603" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="J603" t="b">
+        <v>0</v>
+      </c>
+      <c r="K603" t="n">
+        <v>43000000</v>
+      </c>
+      <c r="L603" t="b">
+        <v>0</v>
+      </c>
+      <c r="M603" t="n">
+        <v>136</v>
+      </c>
+      <c r="N603" t="n">
+        <v>0</v>
+      </c>
+      <c r="O603" t="n">
+        <v>0</v>
+      </c>
+      <c r="P603" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>The Man Who Would Be King</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>card_603</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>John Huston</t>
+        </is>
+      </c>
+      <c r="D604" t="n">
+        <v>1975</v>
+      </c>
+      <c r="E604" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F604" t="n">
+        <v>76</v>
+      </c>
+      <c r="I604" t="n">
+        <v>11000000</v>
+      </c>
+      <c r="J604" t="b">
+        <v>0</v>
+      </c>
+      <c r="K604" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="L604" t="b">
+        <v>0</v>
+      </c>
+      <c r="M604" t="n">
+        <v>129</v>
+      </c>
+      <c r="N604" t="n">
+        <v>0</v>
+      </c>
+      <c r="O604" t="n">
+        <v>0</v>
+      </c>
+      <c r="P604" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Murder on the Orient Express</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>card_604</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>Sidney Lumet</t>
+        </is>
+      </c>
+      <c r="D605" t="n">
+        <v>1974</v>
+      </c>
+      <c r="E605" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="F605" t="n">
+        <v>74</v>
+      </c>
+      <c r="I605" t="n">
+        <v>37700000</v>
+      </c>
+      <c r="J605" t="b">
+        <v>0</v>
+      </c>
+      <c r="K605" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="L605" t="b">
+        <v>0</v>
+      </c>
+      <c r="M605" t="n">
+        <v>128</v>
+      </c>
+      <c r="N605" t="n">
+        <v>1</v>
+      </c>
+      <c r="O605" t="n">
+        <v>0</v>
+      </c>
+      <c r="P605" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add classic Dracula, Frankenstein, and Mummy films (card_605-613)
Nosferatu, Dracula (1931), Dracula (1958), Bram Stoker's Dracula,
Frankenstein (1931), Bride of Frankenstein, Young Frankenstein, The
Mummy (1932), The Mummy (1999). Box office/budget for the silent and
early-Universal titles are rough period estimates where exact figures
aren't documented.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P605"/>
+  <dimension ref="A1:P614"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -31557,352 +31557,790 @@
       </c>
     </row>
     <row r="599">
-      <c r="A599" t="inlineStr">
+      <c r="A599" s="10" t="inlineStr">
         <is>
           <t>The Hunt for Red October</t>
         </is>
       </c>
-      <c r="B599" t="inlineStr">
+      <c r="B599" s="10" t="inlineStr">
         <is>
           <t>card_598</t>
         </is>
       </c>
-      <c r="C599" t="inlineStr">
+      <c r="C599" s="10" t="inlineStr">
         <is>
           <t>John McTiernan</t>
         </is>
       </c>
-      <c r="D599" t="n">
+      <c r="D599" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E599" t="n">
+      <c r="E599" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F599" t="n">
+      <c r="F599" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I599" t="n">
+      <c r="I599" s="10" t="n">
         <v>200500000</v>
       </c>
-      <c r="J599" t="b">
-        <v>0</v>
-      </c>
-      <c r="K599" t="n">
+      <c r="J599" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K599" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L599" t="b">
-        <v>0</v>
-      </c>
-      <c r="M599" t="n">
+      <c r="L599" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M599" s="10" t="n">
         <v>135</v>
       </c>
-      <c r="N599" t="n">
+      <c r="N599" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O599" t="n">
-        <v>0</v>
-      </c>
-      <c r="P599" t="b">
+      <c r="O599" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P599" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="600">
-      <c r="A600" t="inlineStr">
+      <c r="A600" s="10" t="inlineStr">
         <is>
           <t>The Untouchables</t>
         </is>
       </c>
-      <c r="B600" t="inlineStr">
+      <c r="B600" s="10" t="inlineStr">
         <is>
           <t>card_599</t>
         </is>
       </c>
-      <c r="C600" t="inlineStr">
+      <c r="C600" s="10" t="inlineStr">
         <is>
           <t>Brian De Palma</t>
         </is>
       </c>
-      <c r="D600" t="n">
+      <c r="D600" s="10" t="n">
         <v>1987</v>
       </c>
-      <c r="E600" t="n">
+      <c r="E600" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="F600" t="n">
+      <c r="F600" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I600" t="n">
+      <c r="I600" s="10" t="n">
         <v>187000000</v>
       </c>
-      <c r="J600" t="b">
-        <v>0</v>
-      </c>
-      <c r="K600" t="n">
+      <c r="J600" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K600" s="10" t="n">
         <v>25000000</v>
       </c>
-      <c r="L600" t="b">
-        <v>0</v>
-      </c>
-      <c r="M600" t="n">
+      <c r="L600" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M600" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="N600" t="n">
+      <c r="N600" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O600" t="n">
-        <v>0</v>
-      </c>
-      <c r="P600" t="b">
+      <c r="O600" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P600" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="601">
-      <c r="A601" t="inlineStr">
+      <c r="A601" s="10" t="inlineStr">
         <is>
           <t>The Rock</t>
         </is>
       </c>
-      <c r="B601" t="inlineStr">
+      <c r="B601" s="10" t="inlineStr">
         <is>
           <t>card_600</t>
         </is>
       </c>
-      <c r="C601" t="inlineStr">
+      <c r="C601" s="10" t="inlineStr">
         <is>
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="D601" t="n">
+      <c r="D601" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E601" t="n">
+      <c r="E601" s="10" t="n">
         <v>3.6</v>
       </c>
-      <c r="F601" t="n">
+      <c r="F601" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="I601" t="n">
+      <c r="I601" s="10" t="n">
         <v>335600000</v>
       </c>
-      <c r="J601" t="b">
-        <v>0</v>
-      </c>
-      <c r="K601" t="n">
+      <c r="J601" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K601" s="10" t="n">
         <v>75000000</v>
       </c>
-      <c r="L601" t="b">
-        <v>0</v>
-      </c>
-      <c r="M601" t="n">
+      <c r="L601" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M601" s="10" t="n">
         <v>136</v>
       </c>
-      <c r="N601" t="n">
-        <v>0</v>
-      </c>
-      <c r="O601" t="n">
-        <v>0</v>
-      </c>
-      <c r="P601" t="b">
+      <c r="N601" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O601" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P601" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="602">
-      <c r="A602" t="inlineStr">
+      <c r="A602" s="10" t="inlineStr">
         <is>
           <t>Entrapment</t>
         </is>
       </c>
-      <c r="B602" t="inlineStr">
+      <c r="B602" s="10" t="inlineStr">
         <is>
           <t>card_601</t>
         </is>
       </c>
-      <c r="C602" t="inlineStr">
+      <c r="C602" s="10" t="inlineStr">
         <is>
           <t>Jon Amiel</t>
         </is>
       </c>
-      <c r="D602" t="n">
+      <c r="D602" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E602" t="n">
+      <c r="E602" s="10" t="n">
         <v>2.9</v>
       </c>
-      <c r="F602" t="n">
+      <c r="F602" s="10" t="n">
         <v>64</v>
       </c>
-      <c r="I602" t="n">
+      <c r="I602" s="10" t="n">
         <v>212000000</v>
       </c>
-      <c r="J602" t="b">
-        <v>0</v>
-      </c>
-      <c r="K602" t="n">
+      <c r="J602" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K602" s="10" t="n">
         <v>66000000</v>
       </c>
-      <c r="L602" t="b">
-        <v>0</v>
-      </c>
-      <c r="M602" t="n">
+      <c r="L602" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M602" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="N602" t="n">
-        <v>0</v>
-      </c>
-      <c r="O602" t="n">
-        <v>0</v>
-      </c>
-      <c r="P602" t="b">
+      <c r="N602" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O602" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P602" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="603">
-      <c r="A603" t="inlineStr">
+      <c r="A603" s="10" t="inlineStr">
         <is>
           <t>Finding Forrester</t>
         </is>
       </c>
-      <c r="B603" t="inlineStr">
+      <c r="B603" s="10" t="inlineStr">
         <is>
           <t>card_602</t>
         </is>
       </c>
-      <c r="C603" t="inlineStr">
+      <c r="C603" s="10" t="inlineStr">
         <is>
           <t>Gus Van Sant</t>
         </is>
       </c>
-      <c r="D603" t="n">
+      <c r="D603" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E603" t="n">
+      <c r="E603" s="10" t="n">
         <v>3.56</v>
       </c>
-      <c r="F603" t="n">
+      <c r="F603" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I603" t="n">
+      <c r="I603" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="J603" t="b">
-        <v>0</v>
-      </c>
-      <c r="K603" t="n">
+      <c r="J603" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K603" s="10" t="n">
         <v>43000000</v>
       </c>
-      <c r="L603" t="b">
-        <v>0</v>
-      </c>
-      <c r="M603" t="n">
+      <c r="L603" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M603" s="10" t="n">
         <v>136</v>
       </c>
-      <c r="N603" t="n">
-        <v>0</v>
-      </c>
-      <c r="O603" t="n">
-        <v>0</v>
-      </c>
-      <c r="P603" t="b">
+      <c r="N603" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O603" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P603" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="604">
-      <c r="A604" t="inlineStr">
+      <c r="A604" s="10" t="inlineStr">
         <is>
           <t>The Man Who Would Be King</t>
         </is>
       </c>
-      <c r="B604" t="inlineStr">
+      <c r="B604" s="10" t="inlineStr">
         <is>
           <t>card_603</t>
         </is>
       </c>
-      <c r="C604" t="inlineStr">
+      <c r="C604" s="10" t="inlineStr">
         <is>
           <t>John Huston</t>
         </is>
       </c>
-      <c r="D604" t="n">
+      <c r="D604" s="10" t="n">
         <v>1975</v>
       </c>
-      <c r="E604" t="n">
+      <c r="E604" s="10" t="n">
         <v>3.9</v>
       </c>
-      <c r="F604" t="n">
+      <c r="F604" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I604" t="n">
+      <c r="I604" s="10" t="n">
         <v>11000000</v>
       </c>
-      <c r="J604" t="b">
-        <v>0</v>
-      </c>
-      <c r="K604" t="n">
+      <c r="J604" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K604" s="10" t="n">
         <v>8500000</v>
       </c>
-      <c r="L604" t="b">
-        <v>0</v>
-      </c>
-      <c r="M604" t="n">
+      <c r="L604" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M604" s="10" t="n">
         <v>129</v>
       </c>
-      <c r="N604" t="n">
-        <v>0</v>
-      </c>
-      <c r="O604" t="n">
-        <v>0</v>
-      </c>
-      <c r="P604" t="b">
+      <c r="N604" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O604" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P604" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="605">
-      <c r="A605" t="inlineStr">
+      <c r="A605" s="10" t="inlineStr">
         <is>
           <t>Murder on the Orient Express</t>
         </is>
       </c>
-      <c r="B605" t="inlineStr">
+      <c r="B605" s="10" t="inlineStr">
         <is>
           <t>card_604</t>
         </is>
       </c>
-      <c r="C605" t="inlineStr">
+      <c r="C605" s="10" t="inlineStr">
         <is>
           <t>Sidney Lumet</t>
         </is>
       </c>
-      <c r="D605" t="n">
+      <c r="D605" s="10" t="n">
         <v>1974</v>
       </c>
-      <c r="E605" t="n">
+      <c r="E605" s="10" t="n">
         <v>3.58</v>
       </c>
-      <c r="F605" t="n">
+      <c r="F605" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I605" t="n">
+      <c r="I605" s="10" t="n">
         <v>37700000</v>
       </c>
-      <c r="J605" t="b">
-        <v>0</v>
-      </c>
-      <c r="K605" t="n">
+      <c r="J605" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K605" s="10" t="n">
         <v>1400000</v>
       </c>
-      <c r="L605" t="b">
-        <v>0</v>
-      </c>
-      <c r="M605" t="n">
+      <c r="L605" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M605" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N605" t="n">
+      <c r="N605" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O605" t="n">
-        <v>0</v>
-      </c>
-      <c r="P605" t="b">
+      <c r="O605" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P605" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Nosferatu</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>card_605</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>F. W. Murnau</t>
+        </is>
+      </c>
+      <c r="D606" t="n">
+        <v>1922</v>
+      </c>
+      <c r="E606" t="n">
+        <v>3.82</v>
+      </c>
+      <c r="F606" t="n">
+        <v>79</v>
+      </c>
+      <c r="I606" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J606" t="b">
+        <v>1</v>
+      </c>
+      <c r="K606" t="n">
+        <v>100000</v>
+      </c>
+      <c r="L606" t="b">
+        <v>1</v>
+      </c>
+      <c r="M606" t="n">
+        <v>94</v>
+      </c>
+      <c r="N606" t="n">
+        <v>0</v>
+      </c>
+      <c r="O606" t="n">
+        <v>0</v>
+      </c>
+      <c r="P606" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Dracula</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>card_606</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Tod Browning</t>
+        </is>
+      </c>
+      <c r="D607" t="n">
+        <v>1931</v>
+      </c>
+      <c r="E607" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F607" t="n">
+        <v>72</v>
+      </c>
+      <c r="I607" t="n">
+        <v>700000</v>
+      </c>
+      <c r="J607" t="b">
+        <v>1</v>
+      </c>
+      <c r="K607" t="n">
+        <v>341191</v>
+      </c>
+      <c r="L607" t="b">
+        <v>0</v>
+      </c>
+      <c r="M607" t="n">
+        <v>74</v>
+      </c>
+      <c r="N607" t="n">
+        <v>0</v>
+      </c>
+      <c r="O607" t="n">
+        <v>0</v>
+      </c>
+      <c r="P607" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Dracula (1958)</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>card_607</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Terence Fisher</t>
+        </is>
+      </c>
+      <c r="D608" t="n">
+        <v>1958</v>
+      </c>
+      <c r="E608" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="I608" t="n">
+        <v>3500000</v>
+      </c>
+      <c r="J608" t="b">
+        <v>0</v>
+      </c>
+      <c r="K608" t="n">
+        <v>228000</v>
+      </c>
+      <c r="L608" t="b">
+        <v>0</v>
+      </c>
+      <c r="M608" t="n">
+        <v>82</v>
+      </c>
+      <c r="N608" t="n">
+        <v>0</v>
+      </c>
+      <c r="O608" t="n">
+        <v>0</v>
+      </c>
+      <c r="P608" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Bram Stoker's Dracula</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>card_608</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Francis Ford Coppola</t>
+        </is>
+      </c>
+      <c r="D609" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E609" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="F609" t="n">
+        <v>71</v>
+      </c>
+      <c r="I609" t="n">
+        <v>215900000</v>
+      </c>
+      <c r="J609" t="b">
+        <v>0</v>
+      </c>
+      <c r="K609" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L609" t="b">
+        <v>0</v>
+      </c>
+      <c r="M609" t="n">
+        <v>128</v>
+      </c>
+      <c r="N609" t="n">
+        <v>3</v>
+      </c>
+      <c r="O609" t="n">
+        <v>5</v>
+      </c>
+      <c r="P609" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Frankenstein</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>card_609</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>James Whale</t>
+        </is>
+      </c>
+      <c r="D610" t="n">
+        <v>1931</v>
+      </c>
+      <c r="E610" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="I610" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="J610" t="b">
+        <v>0</v>
+      </c>
+      <c r="K610" t="n">
+        <v>262007</v>
+      </c>
+      <c r="L610" t="b">
+        <v>0</v>
+      </c>
+      <c r="M610" t="n">
+        <v>70</v>
+      </c>
+      <c r="N610" t="n">
+        <v>0</v>
+      </c>
+      <c r="O610" t="n">
+        <v>0</v>
+      </c>
+      <c r="P610" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Bride of Frankenstein</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>card_610</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>James Whale</t>
+        </is>
+      </c>
+      <c r="D611" t="n">
+        <v>1935</v>
+      </c>
+      <c r="E611" t="n">
+        <v>3.96</v>
+      </c>
+      <c r="I611" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="J611" t="b">
+        <v>0</v>
+      </c>
+      <c r="K611" t="n">
+        <v>397000</v>
+      </c>
+      <c r="L611" t="b">
+        <v>0</v>
+      </c>
+      <c r="M611" t="n">
+        <v>75</v>
+      </c>
+      <c r="N611" t="n">
+        <v>0</v>
+      </c>
+      <c r="O611" t="n">
+        <v>0</v>
+      </c>
+      <c r="P611" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Young Frankenstein</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>card_611</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Mel Brooks</t>
+        </is>
+      </c>
+      <c r="D612" t="n">
+        <v>1974</v>
+      </c>
+      <c r="E612" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="F612" t="n">
+        <v>82</v>
+      </c>
+      <c r="I612" t="n">
+        <v>86200000</v>
+      </c>
+      <c r="J612" t="b">
+        <v>0</v>
+      </c>
+      <c r="K612" t="n">
+        <v>2780000</v>
+      </c>
+      <c r="L612" t="b">
+        <v>0</v>
+      </c>
+      <c r="M612" t="n">
+        <v>105</v>
+      </c>
+      <c r="N612" t="n">
+        <v>0</v>
+      </c>
+      <c r="O612" t="n">
+        <v>0</v>
+      </c>
+      <c r="P612" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>The Mummy</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>card_612</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Karl Freund</t>
+        </is>
+      </c>
+      <c r="D613" t="n">
+        <v>1932</v>
+      </c>
+      <c r="E613" t="n">
+        <v>3.27</v>
+      </c>
+      <c r="I613" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J613" t="b">
+        <v>1</v>
+      </c>
+      <c r="K613" t="n">
+        <v>196000</v>
+      </c>
+      <c r="L613" t="b">
+        <v>0</v>
+      </c>
+      <c r="M613" t="n">
+        <v>73</v>
+      </c>
+      <c r="N613" t="n">
+        <v>0</v>
+      </c>
+      <c r="O613" t="n">
+        <v>0</v>
+      </c>
+      <c r="P613" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>The Mummy (1999)</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>card_613</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Stephen Sommers</t>
+        </is>
+      </c>
+      <c r="D614" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E614" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="F614" t="n">
+        <v>77</v>
+      </c>
+      <c r="I614" t="n">
+        <v>422500000</v>
+      </c>
+      <c r="J614" t="b">
+        <v>0</v>
+      </c>
+      <c r="K614" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L614" t="b">
+        <v>0</v>
+      </c>
+      <c r="M614" t="n">
+        <v>125</v>
+      </c>
+      <c r="N614" t="n">
+        <v>0</v>
+      </c>
+      <c r="O614" t="n">
+        <v>0</v>
+      </c>
+      <c r="P614" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disney animated canon, part 1: 1961-1991 (card_614-627)
101 Dalmatians through Beauty and the Beast, 14 films. First of
several batches covering the Disney animated canon since 1960.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P614"/>
+  <dimension ref="A1:P628"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -31907,440 +31907,1140 @@
       </c>
     </row>
     <row r="606">
-      <c r="A606" t="inlineStr">
+      <c r="A606" s="10" t="inlineStr">
         <is>
           <t>Nosferatu</t>
         </is>
       </c>
-      <c r="B606" t="inlineStr">
+      <c r="B606" s="10" t="inlineStr">
         <is>
           <t>card_605</t>
         </is>
       </c>
-      <c r="C606" t="inlineStr">
+      <c r="C606" s="10" t="inlineStr">
         <is>
           <t>F. W. Murnau</t>
         </is>
       </c>
-      <c r="D606" t="n">
+      <c r="D606" s="10" t="n">
         <v>1922</v>
       </c>
-      <c r="E606" t="n">
+      <c r="E606" s="10" t="n">
         <v>3.82</v>
       </c>
-      <c r="F606" t="n">
+      <c r="F606" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I606" t="n">
+      <c r="I606" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="J606" t="b">
+      <c r="J606" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K606" t="n">
+      <c r="K606" s="10" t="n">
         <v>100000</v>
       </c>
-      <c r="L606" t="b">
+      <c r="L606" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M606" t="n">
+      <c r="M606" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="N606" t="n">
-        <v>0</v>
-      </c>
-      <c r="O606" t="n">
-        <v>0</v>
-      </c>
-      <c r="P606" t="b">
+      <c r="N606" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O606" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P606" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="607">
-      <c r="A607" t="inlineStr">
+      <c r="A607" s="10" t="inlineStr">
         <is>
           <t>Dracula</t>
         </is>
       </c>
-      <c r="B607" t="inlineStr">
+      <c r="B607" s="10" t="inlineStr">
         <is>
           <t>card_606</t>
         </is>
       </c>
-      <c r="C607" t="inlineStr">
+      <c r="C607" s="10" t="inlineStr">
         <is>
           <t>Tod Browning</t>
         </is>
       </c>
-      <c r="D607" t="n">
+      <c r="D607" s="10" t="n">
         <v>1931</v>
       </c>
-      <c r="E607" t="n">
+      <c r="E607" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F607" t="n">
+      <c r="F607" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I607" t="n">
+      <c r="I607" s="10" t="n">
         <v>700000</v>
       </c>
-      <c r="J607" t="b">
+      <c r="J607" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K607" t="n">
+      <c r="K607" s="10" t="n">
         <v>341191</v>
       </c>
-      <c r="L607" t="b">
-        <v>0</v>
-      </c>
-      <c r="M607" t="n">
+      <c r="L607" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M607" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="N607" t="n">
-        <v>0</v>
-      </c>
-      <c r="O607" t="n">
-        <v>0</v>
-      </c>
-      <c r="P607" t="b">
+      <c r="N607" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O607" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P607" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="608">
-      <c r="A608" t="inlineStr">
+      <c r="A608" s="10" t="inlineStr">
         <is>
           <t>Dracula (1958)</t>
         </is>
       </c>
-      <c r="B608" t="inlineStr">
+      <c r="B608" s="10" t="inlineStr">
         <is>
           <t>card_607</t>
         </is>
       </c>
-      <c r="C608" t="inlineStr">
+      <c r="C608" s="10" t="inlineStr">
         <is>
           <t>Terence Fisher</t>
         </is>
       </c>
-      <c r="D608" t="n">
+      <c r="D608" s="10" t="n">
         <v>1958</v>
       </c>
-      <c r="E608" t="n">
+      <c r="E608" s="10" t="n">
         <v>3.6</v>
       </c>
-      <c r="I608" t="n">
+      <c r="I608" s="10" t="n">
         <v>3500000</v>
       </c>
-      <c r="J608" t="b">
-        <v>0</v>
-      </c>
-      <c r="K608" t="n">
+      <c r="J608" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K608" s="10" t="n">
         <v>228000</v>
       </c>
-      <c r="L608" t="b">
-        <v>0</v>
-      </c>
-      <c r="M608" t="n">
+      <c r="L608" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M608" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="N608" t="n">
-        <v>0</v>
-      </c>
-      <c r="O608" t="n">
-        <v>0</v>
-      </c>
-      <c r="P608" t="b">
+      <c r="N608" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O608" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P608" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="609">
-      <c r="A609" t="inlineStr">
+      <c r="A609" s="10" t="inlineStr">
         <is>
           <t>Bram Stoker's Dracula</t>
         </is>
       </c>
-      <c r="B609" t="inlineStr">
+      <c r="B609" s="10" t="inlineStr">
         <is>
           <t>card_608</t>
         </is>
       </c>
-      <c r="C609" t="inlineStr">
+      <c r="C609" s="10" t="inlineStr">
         <is>
           <t>Francis Ford Coppola</t>
         </is>
       </c>
-      <c r="D609" t="n">
+      <c r="D609" s="10" t="n">
         <v>1992</v>
       </c>
-      <c r="E609" t="n">
+      <c r="E609" s="10" t="n">
         <v>3.74</v>
       </c>
-      <c r="F609" t="n">
+      <c r="F609" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I609" t="n">
+      <c r="I609" s="10" t="n">
         <v>215900000</v>
       </c>
-      <c r="J609" t="b">
-        <v>0</v>
-      </c>
-      <c r="K609" t="n">
+      <c r="J609" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K609" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L609" t="b">
-        <v>0</v>
-      </c>
-      <c r="M609" t="n">
+      <c r="L609" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M609" s="10" t="n">
         <v>128</v>
       </c>
-      <c r="N609" t="n">
+      <c r="N609" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="O609" t="n">
+      <c r="O609" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="P609" t="b">
+      <c r="P609" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="610">
-      <c r="A610" t="inlineStr">
+      <c r="A610" s="10" t="inlineStr">
         <is>
           <t>Frankenstein</t>
         </is>
       </c>
-      <c r="B610" t="inlineStr">
+      <c r="B610" s="10" t="inlineStr">
         <is>
           <t>card_609</t>
         </is>
       </c>
-      <c r="C610" t="inlineStr">
+      <c r="C610" s="10" t="inlineStr">
         <is>
           <t>James Whale</t>
         </is>
       </c>
-      <c r="D610" t="n">
+      <c r="D610" s="10" t="n">
         <v>1931</v>
       </c>
-      <c r="E610" t="n">
+      <c r="E610" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="I610" t="n">
+      <c r="I610" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="J610" t="b">
-        <v>0</v>
-      </c>
-      <c r="K610" t="n">
+      <c r="J610" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K610" s="10" t="n">
         <v>262007</v>
       </c>
-      <c r="L610" t="b">
-        <v>0</v>
-      </c>
-      <c r="M610" t="n">
+      <c r="L610" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M610" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="N610" t="n">
-        <v>0</v>
-      </c>
-      <c r="O610" t="n">
-        <v>0</v>
-      </c>
-      <c r="P610" t="b">
+      <c r="N610" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O610" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P610" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="611">
-      <c r="A611" t="inlineStr">
+      <c r="A611" s="10" t="inlineStr">
         <is>
           <t>Bride of Frankenstein</t>
         </is>
       </c>
-      <c r="B611" t="inlineStr">
+      <c r="B611" s="10" t="inlineStr">
         <is>
           <t>card_610</t>
         </is>
       </c>
-      <c r="C611" t="inlineStr">
+      <c r="C611" s="10" t="inlineStr">
         <is>
           <t>James Whale</t>
         </is>
       </c>
-      <c r="D611" t="n">
+      <c r="D611" s="10" t="n">
         <v>1935</v>
       </c>
-      <c r="E611" t="n">
+      <c r="E611" s="10" t="n">
         <v>3.96</v>
       </c>
-      <c r="I611" t="n">
+      <c r="I611" s="10" t="n">
         <v>2000000</v>
       </c>
-      <c r="J611" t="b">
-        <v>0</v>
-      </c>
-      <c r="K611" t="n">
+      <c r="J611" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K611" s="10" t="n">
         <v>397000</v>
       </c>
-      <c r="L611" t="b">
-        <v>0</v>
-      </c>
-      <c r="M611" t="n">
+      <c r="L611" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M611" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="N611" t="n">
-        <v>0</v>
-      </c>
-      <c r="O611" t="n">
-        <v>0</v>
-      </c>
-      <c r="P611" t="b">
+      <c r="N611" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O611" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P611" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="612">
-      <c r="A612" t="inlineStr">
+      <c r="A612" s="10" t="inlineStr">
         <is>
           <t>Young Frankenstein</t>
         </is>
       </c>
-      <c r="B612" t="inlineStr">
+      <c r="B612" s="10" t="inlineStr">
         <is>
           <t>card_611</t>
         </is>
       </c>
-      <c r="C612" t="inlineStr">
+      <c r="C612" s="10" t="inlineStr">
         <is>
           <t>Mel Brooks</t>
         </is>
       </c>
-      <c r="D612" t="n">
+      <c r="D612" s="10" t="n">
         <v>1974</v>
       </c>
-      <c r="E612" t="n">
+      <c r="E612" s="10" t="n">
         <v>4.01</v>
       </c>
-      <c r="F612" t="n">
+      <c r="F612" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I612" t="n">
+      <c r="I612" s="10" t="n">
         <v>86200000</v>
       </c>
-      <c r="J612" t="b">
-        <v>0</v>
-      </c>
-      <c r="K612" t="n">
+      <c r="J612" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K612" s="10" t="n">
         <v>2780000</v>
       </c>
-      <c r="L612" t="b">
-        <v>0</v>
-      </c>
-      <c r="M612" t="n">
+      <c r="L612" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M612" s="10" t="n">
         <v>105</v>
       </c>
-      <c r="N612" t="n">
-        <v>0</v>
-      </c>
-      <c r="O612" t="n">
-        <v>0</v>
-      </c>
-      <c r="P612" t="b">
+      <c r="N612" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O612" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P612" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="613">
-      <c r="A613" t="inlineStr">
+      <c r="A613" s="10" t="inlineStr">
         <is>
           <t>The Mummy</t>
         </is>
       </c>
-      <c r="B613" t="inlineStr">
+      <c r="B613" s="10" t="inlineStr">
         <is>
           <t>card_612</t>
         </is>
       </c>
-      <c r="C613" t="inlineStr">
+      <c r="C613" s="10" t="inlineStr">
         <is>
           <t>Karl Freund</t>
         </is>
       </c>
-      <c r="D613" t="n">
+      <c r="D613" s="10" t="n">
         <v>1932</v>
       </c>
-      <c r="E613" t="n">
+      <c r="E613" s="10" t="n">
         <v>3.27</v>
       </c>
-      <c r="I613" t="n">
+      <c r="I613" s="10" t="n">
         <v>1000000</v>
       </c>
-      <c r="J613" t="b">
+      <c r="J613" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K613" t="n">
+      <c r="K613" s="10" t="n">
         <v>196000</v>
       </c>
-      <c r="L613" t="b">
-        <v>0</v>
-      </c>
-      <c r="M613" t="n">
+      <c r="L613" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M613" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="N613" t="n">
-        <v>0</v>
-      </c>
-      <c r="O613" t="n">
-        <v>0</v>
-      </c>
-      <c r="P613" t="b">
+      <c r="N613" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O613" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P613" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="614">
-      <c r="A614" t="inlineStr">
+      <c r="A614" s="10" t="inlineStr">
         <is>
           <t>The Mummy (1999)</t>
         </is>
       </c>
-      <c r="B614" t="inlineStr">
+      <c r="B614" s="10" t="inlineStr">
         <is>
           <t>card_613</t>
         </is>
       </c>
-      <c r="C614" t="inlineStr">
+      <c r="C614" s="10" t="inlineStr">
         <is>
           <t>Stephen Sommers</t>
         </is>
       </c>
-      <c r="D614" t="n">
+      <c r="D614" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E614" t="n">
+      <c r="E614" s="10" t="n">
         <v>3.61</v>
       </c>
-      <c r="F614" t="n">
+      <c r="F614" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I614" t="n">
+      <c r="I614" s="10" t="n">
         <v>422500000</v>
       </c>
-      <c r="J614" t="b">
-        <v>0</v>
-      </c>
-      <c r="K614" t="n">
+      <c r="J614" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K614" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L614" t="b">
-        <v>0</v>
-      </c>
-      <c r="M614" t="n">
+      <c r="L614" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M614" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="N614" t="n">
-        <v>0</v>
-      </c>
-      <c r="O614" t="n">
-        <v>0</v>
-      </c>
-      <c r="P614" t="b">
+      <c r="N614" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O614" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P614" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>One Hundred and One Dalmatians</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>card_614</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman, Hamilton Luske and Clyde Geronimi</t>
+        </is>
+      </c>
+      <c r="D615" t="n">
+        <v>1961</v>
+      </c>
+      <c r="E615" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F615" t="n">
+        <v>69</v>
+      </c>
+      <c r="I615" t="n">
+        <v>303000000</v>
+      </c>
+      <c r="J615" t="b">
+        <v>0</v>
+      </c>
+      <c r="K615" t="n">
+        <v>3900000</v>
+      </c>
+      <c r="L615" t="b">
+        <v>0</v>
+      </c>
+      <c r="M615" t="n">
+        <v>79</v>
+      </c>
+      <c r="N615" t="n">
+        <v>0</v>
+      </c>
+      <c r="O615" t="n">
+        <v>0</v>
+      </c>
+      <c r="P615" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>The Sword in the Stone</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>card_615</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman</t>
+        </is>
+      </c>
+      <c r="D616" t="n">
+        <v>1963</v>
+      </c>
+      <c r="E616" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F616" t="n">
+        <v>72</v>
+      </c>
+      <c r="I616" t="n">
+        <v>22200000</v>
+      </c>
+      <c r="J616" t="b">
+        <v>1</v>
+      </c>
+      <c r="K616" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="L616" t="b">
+        <v>0</v>
+      </c>
+      <c r="M616" t="n">
+        <v>79</v>
+      </c>
+      <c r="N616" t="n">
+        <v>0</v>
+      </c>
+      <c r="O616" t="n">
+        <v>0</v>
+      </c>
+      <c r="P616" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>The Jungle Book</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>card_616</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman</t>
+        </is>
+      </c>
+      <c r="D617" t="n">
+        <v>1967</v>
+      </c>
+      <c r="E617" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F617" t="n">
+        <v>77</v>
+      </c>
+      <c r="I617" t="n">
+        <v>378000000</v>
+      </c>
+      <c r="J617" t="b">
+        <v>0</v>
+      </c>
+      <c r="K617" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L617" t="b">
+        <v>0</v>
+      </c>
+      <c r="M617" t="n">
+        <v>78</v>
+      </c>
+      <c r="N617" t="n">
+        <v>0</v>
+      </c>
+      <c r="O617" t="n">
+        <v>0</v>
+      </c>
+      <c r="P617" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>The Aristocats</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>card_617</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman</t>
+        </is>
+      </c>
+      <c r="D618" t="n">
+        <v>1970</v>
+      </c>
+      <c r="E618" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F618" t="n">
+        <v>67</v>
+      </c>
+      <c r="I618" t="n">
+        <v>191000000</v>
+      </c>
+      <c r="J618" t="b">
+        <v>0</v>
+      </c>
+      <c r="K618" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L618" t="b">
+        <v>0</v>
+      </c>
+      <c r="M618" t="n">
+        <v>79</v>
+      </c>
+      <c r="N618" t="n">
+        <v>0</v>
+      </c>
+      <c r="O618" t="n">
+        <v>0</v>
+      </c>
+      <c r="P618" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Robin Hood</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>card_618</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman</t>
+        </is>
+      </c>
+      <c r="D619" t="n">
+        <v>1973</v>
+      </c>
+      <c r="E619" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F619" t="n">
+        <v>63</v>
+      </c>
+      <c r="I619" t="n">
+        <v>33000000</v>
+      </c>
+      <c r="J619" t="b">
+        <v>0</v>
+      </c>
+      <c r="K619" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L619" t="b">
+        <v>0</v>
+      </c>
+      <c r="M619" t="n">
+        <v>83</v>
+      </c>
+      <c r="N619" t="n">
+        <v>0</v>
+      </c>
+      <c r="O619" t="n">
+        <v>0</v>
+      </c>
+      <c r="P619" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>The Many Adventures of Winnie the Pooh</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>card_619</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman and John Lounsbery</t>
+        </is>
+      </c>
+      <c r="D620" t="n">
+        <v>1977</v>
+      </c>
+      <c r="E620" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F620" t="n">
+        <v>80</v>
+      </c>
+      <c r="I620" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="J620" t="b">
+        <v>1</v>
+      </c>
+      <c r="K620" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L620" t="b">
+        <v>1</v>
+      </c>
+      <c r="M620" t="n">
+        <v>74</v>
+      </c>
+      <c r="N620" t="n">
+        <v>0</v>
+      </c>
+      <c r="O620" t="n">
+        <v>0</v>
+      </c>
+      <c r="P620" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>The Rescuers</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>card_620</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>Wolfgang Reitherman, John Lounsbery and Art Stevens</t>
+        </is>
+      </c>
+      <c r="D621" t="n">
+        <v>1977</v>
+      </c>
+      <c r="E621" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="F621" t="n">
+        <v>69</v>
+      </c>
+      <c r="I621" t="n">
+        <v>169000000</v>
+      </c>
+      <c r="J621" t="b">
+        <v>0</v>
+      </c>
+      <c r="K621" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="L621" t="b">
+        <v>0</v>
+      </c>
+      <c r="M621" t="n">
+        <v>77</v>
+      </c>
+      <c r="N621" t="n">
+        <v>0</v>
+      </c>
+      <c r="O621" t="n">
+        <v>0</v>
+      </c>
+      <c r="P621" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>The Fox and the Hound</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>card_621</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Ted Berman, Richard Rich and Art Stevens</t>
+        </is>
+      </c>
+      <c r="D622" t="n">
+        <v>1981</v>
+      </c>
+      <c r="E622" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F622" t="n">
+        <v>78</v>
+      </c>
+      <c r="I622" t="n">
+        <v>63500000</v>
+      </c>
+      <c r="J622" t="b">
+        <v>0</v>
+      </c>
+      <c r="K622" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="L622" t="b">
+        <v>0</v>
+      </c>
+      <c r="M622" t="n">
+        <v>83</v>
+      </c>
+      <c r="N622" t="n">
+        <v>0</v>
+      </c>
+      <c r="O622" t="n">
+        <v>0</v>
+      </c>
+      <c r="P622" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>The Black Cauldron</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>card_622</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Ted Berman and Richard Rich</t>
+        </is>
+      </c>
+      <c r="D623" t="n">
+        <v>1985</v>
+      </c>
+      <c r="E623" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F623" t="n">
+        <v>58</v>
+      </c>
+      <c r="I623" t="n">
+        <v>21300000</v>
+      </c>
+      <c r="J623" t="b">
+        <v>0</v>
+      </c>
+      <c r="K623" t="n">
+        <v>44000000</v>
+      </c>
+      <c r="L623" t="b">
+        <v>0</v>
+      </c>
+      <c r="M623" t="n">
+        <v>80</v>
+      </c>
+      <c r="N623" t="n">
+        <v>0</v>
+      </c>
+      <c r="O623" t="n">
+        <v>0</v>
+      </c>
+      <c r="P623" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>The Great Mouse Detective</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>card_623</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>John Musker, Ron Clements, Dave Michener and Burny Mattinson</t>
+        </is>
+      </c>
+      <c r="D624" t="n">
+        <v>1986</v>
+      </c>
+      <c r="E624" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F624" t="n">
+        <v>77</v>
+      </c>
+      <c r="I624" t="n">
+        <v>50000000</v>
+      </c>
+      <c r="J624" t="b">
+        <v>0</v>
+      </c>
+      <c r="K624" t="n">
+        <v>14000000</v>
+      </c>
+      <c r="L624" t="b">
+        <v>0</v>
+      </c>
+      <c r="M624" t="n">
+        <v>74</v>
+      </c>
+      <c r="N624" t="n">
+        <v>0</v>
+      </c>
+      <c r="O624" t="n">
+        <v>0</v>
+      </c>
+      <c r="P624" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Oliver &amp; Company</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>card_624</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>George Scribner</t>
+        </is>
+      </c>
+      <c r="D625" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E625" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="F625" t="n">
+        <v>70</v>
+      </c>
+      <c r="I625" t="n">
+        <v>121000000</v>
+      </c>
+      <c r="J625" t="b">
+        <v>0</v>
+      </c>
+      <c r="K625" t="n">
+        <v>31000000</v>
+      </c>
+      <c r="L625" t="b">
+        <v>0</v>
+      </c>
+      <c r="M625" t="n">
+        <v>74</v>
+      </c>
+      <c r="N625" t="n">
+        <v>0</v>
+      </c>
+      <c r="O625" t="n">
+        <v>0</v>
+      </c>
+      <c r="P625" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>The Little Mermaid</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>card_625</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>John Musker and Ron Clements</t>
+        </is>
+      </c>
+      <c r="D626" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E626" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F626" t="n">
+        <v>73</v>
+      </c>
+      <c r="I626" t="n">
+        <v>235000000</v>
+      </c>
+      <c r="J626" t="b">
+        <v>0</v>
+      </c>
+      <c r="K626" t="n">
+        <v>40000000</v>
+      </c>
+      <c r="L626" t="b">
+        <v>0</v>
+      </c>
+      <c r="M626" t="n">
+        <v>83</v>
+      </c>
+      <c r="N626" t="n">
+        <v>2</v>
+      </c>
+      <c r="O626" t="n">
+        <v>0</v>
+      </c>
+      <c r="P626" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>The Rescuers Down Under</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>card_626</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Hendel Butoy and Mike Gabriel</t>
+        </is>
+      </c>
+      <c r="D627" t="n">
+        <v>1990</v>
+      </c>
+      <c r="E627" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F627" t="n">
+        <v>69</v>
+      </c>
+      <c r="I627" t="n">
+        <v>47400000</v>
+      </c>
+      <c r="J627" t="b">
+        <v>0</v>
+      </c>
+      <c r="K627" t="n">
+        <v>38000000</v>
+      </c>
+      <c r="L627" t="b">
+        <v>0</v>
+      </c>
+      <c r="M627" t="n">
+        <v>77</v>
+      </c>
+      <c r="N627" t="n">
+        <v>0</v>
+      </c>
+      <c r="O627" t="n">
+        <v>0</v>
+      </c>
+      <c r="P627" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Beauty and the Beast</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>card_627</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>Gary Trousdale and Kirk Wise</t>
+        </is>
+      </c>
+      <c r="D628" t="n">
+        <v>1991</v>
+      </c>
+      <c r="E628" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="F628" t="n">
+        <v>84</v>
+      </c>
+      <c r="I628" t="n">
+        <v>451200000</v>
+      </c>
+      <c r="J628" t="b">
+        <v>0</v>
+      </c>
+      <c r="K628" t="n">
+        <v>25000000</v>
+      </c>
+      <c r="L628" t="b">
+        <v>0</v>
+      </c>
+      <c r="M628" t="n">
+        <v>84</v>
+      </c>
+      <c r="N628" t="n">
+        <v>2</v>
+      </c>
+      <c r="O628" t="n">
+        <v>0</v>
+      </c>
+      <c r="P628" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disney animated canon, part 2: 1995-2001 (card_628-636)
Pocahontas through Atlantis: The Lost Empire, 9 films. Ralph Zondag's
birth year isn't documented anywhere, so Dinosaur's director_age_at_release
stays null (same nullability as every other unresolved case).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P628"/>
+  <dimension ref="A1:P637"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -32345,702 +32345,1152 @@
       </c>
     </row>
     <row r="615">
-      <c r="A615" t="inlineStr">
+      <c r="A615" s="10" t="inlineStr">
         <is>
           <t>One Hundred and One Dalmatians</t>
         </is>
       </c>
-      <c r="B615" t="inlineStr">
+      <c r="B615" s="10" t="inlineStr">
         <is>
           <t>card_614</t>
         </is>
       </c>
-      <c r="C615" t="inlineStr">
+      <c r="C615" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman, Hamilton Luske and Clyde Geronimi</t>
         </is>
       </c>
-      <c r="D615" t="n">
+      <c r="D615" s="10" t="n">
         <v>1961</v>
       </c>
-      <c r="E615" t="n">
+      <c r="E615" s="10" t="n">
         <v>3.75</v>
       </c>
-      <c r="F615" t="n">
+      <c r="F615" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I615" t="n">
+      <c r="I615" s="10" t="n">
         <v>303000000</v>
       </c>
-      <c r="J615" t="b">
-        <v>0</v>
-      </c>
-      <c r="K615" t="n">
+      <c r="J615" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K615" s="10" t="n">
         <v>3900000</v>
       </c>
-      <c r="L615" t="b">
-        <v>0</v>
-      </c>
-      <c r="M615" t="n">
+      <c r="L615" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M615" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="N615" t="n">
-        <v>0</v>
-      </c>
-      <c r="O615" t="n">
-        <v>0</v>
-      </c>
-      <c r="P615" t="b">
+      <c r="N615" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O615" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P615" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="616">
-      <c r="A616" t="inlineStr">
+      <c r="A616" s="10" t="inlineStr">
         <is>
           <t>The Sword in the Stone</t>
         </is>
       </c>
-      <c r="B616" t="inlineStr">
+      <c r="B616" s="10" t="inlineStr">
         <is>
           <t>card_615</t>
         </is>
       </c>
-      <c r="C616" t="inlineStr">
+      <c r="C616" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman</t>
         </is>
       </c>
-      <c r="D616" t="n">
+      <c r="D616" s="10" t="n">
         <v>1963</v>
       </c>
-      <c r="E616" t="n">
+      <c r="E616" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F616" t="n">
+      <c r="F616" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I616" t="n">
+      <c r="I616" s="10" t="n">
         <v>22200000</v>
       </c>
-      <c r="J616" t="b">
+      <c r="J616" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K616" t="n">
+      <c r="K616" s="10" t="n">
         <v>3000000</v>
       </c>
-      <c r="L616" t="b">
-        <v>0</v>
-      </c>
-      <c r="M616" t="n">
+      <c r="L616" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M616" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="N616" t="n">
-        <v>0</v>
-      </c>
-      <c r="O616" t="n">
-        <v>0</v>
-      </c>
-      <c r="P616" t="b">
+      <c r="N616" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O616" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P616" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="617">
-      <c r="A617" t="inlineStr">
+      <c r="A617" s="10" t="inlineStr">
         <is>
           <t>The Jungle Book</t>
         </is>
       </c>
-      <c r="B617" t="inlineStr">
+      <c r="B617" s="10" t="inlineStr">
         <is>
           <t>card_616</t>
         </is>
       </c>
-      <c r="C617" t="inlineStr">
+      <c r="C617" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman</t>
         </is>
       </c>
-      <c r="D617" t="n">
+      <c r="D617" s="10" t="n">
         <v>1967</v>
       </c>
-      <c r="E617" t="n">
+      <c r="E617" s="10" t="n">
         <v>3.71</v>
       </c>
-      <c r="F617" t="n">
+      <c r="F617" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I617" t="n">
+      <c r="I617" s="10" t="n">
         <v>378000000</v>
       </c>
-      <c r="J617" t="b">
-        <v>0</v>
-      </c>
-      <c r="K617" t="n">
+      <c r="J617" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K617" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L617" t="b">
-        <v>0</v>
-      </c>
-      <c r="M617" t="n">
+      <c r="L617" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M617" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="N617" t="n">
-        <v>0</v>
-      </c>
-      <c r="O617" t="n">
-        <v>0</v>
-      </c>
-      <c r="P617" t="b">
+      <c r="N617" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O617" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P617" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="618">
-      <c r="A618" t="inlineStr">
+      <c r="A618" s="10" t="inlineStr">
         <is>
           <t>The Aristocats</t>
         </is>
       </c>
-      <c r="B618" t="inlineStr">
+      <c r="B618" s="10" t="inlineStr">
         <is>
           <t>card_617</t>
         </is>
       </c>
-      <c r="C618" t="inlineStr">
+      <c r="C618" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman</t>
         </is>
       </c>
-      <c r="D618" t="n">
+      <c r="D618" s="10" t="n">
         <v>1970</v>
       </c>
-      <c r="E618" t="n">
+      <c r="E618" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F618" t="n">
+      <c r="F618" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I618" t="n">
+      <c r="I618" s="10" t="n">
         <v>191000000</v>
       </c>
-      <c r="J618" t="b">
-        <v>0</v>
-      </c>
-      <c r="K618" t="n">
+      <c r="J618" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K618" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L618" t="b">
-        <v>0</v>
-      </c>
-      <c r="M618" t="n">
+      <c r="L618" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M618" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="N618" t="n">
-        <v>0</v>
-      </c>
-      <c r="O618" t="n">
-        <v>0</v>
-      </c>
-      <c r="P618" t="b">
+      <c r="N618" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O618" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P618" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="619">
-      <c r="A619" t="inlineStr">
+      <c r="A619" s="10" t="inlineStr">
         <is>
           <t>Robin Hood</t>
         </is>
       </c>
-      <c r="B619" t="inlineStr">
+      <c r="B619" s="10" t="inlineStr">
         <is>
           <t>card_618</t>
         </is>
       </c>
-      <c r="C619" t="inlineStr">
+      <c r="C619" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman</t>
         </is>
       </c>
-      <c r="D619" t="n">
+      <c r="D619" s="10" t="n">
         <v>1973</v>
       </c>
-      <c r="E619" t="n">
+      <c r="E619" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F619" t="n">
+      <c r="F619" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I619" t="n">
+      <c r="I619" s="10" t="n">
         <v>33000000</v>
       </c>
-      <c r="J619" t="b">
-        <v>0</v>
-      </c>
-      <c r="K619" t="n">
+      <c r="J619" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K619" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L619" t="b">
-        <v>0</v>
-      </c>
-      <c r="M619" t="n">
+      <c r="L619" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M619" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="N619" t="n">
-        <v>0</v>
-      </c>
-      <c r="O619" t="n">
-        <v>0</v>
-      </c>
-      <c r="P619" t="b">
+      <c r="N619" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O619" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P619" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="620">
-      <c r="A620" t="inlineStr">
+      <c r="A620" s="10" t="inlineStr">
         <is>
           <t>The Many Adventures of Winnie the Pooh</t>
         </is>
       </c>
-      <c r="B620" t="inlineStr">
+      <c r="B620" s="10" t="inlineStr">
         <is>
           <t>card_619</t>
         </is>
       </c>
-      <c r="C620" t="inlineStr">
+      <c r="C620" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman and John Lounsbery</t>
         </is>
       </c>
-      <c r="D620" t="n">
+      <c r="D620" s="10" t="n">
         <v>1977</v>
       </c>
-      <c r="E620" t="n">
+      <c r="E620" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F620" t="n">
+      <c r="F620" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I620" t="n">
+      <c r="I620" s="10" t="n">
         <v>25000000</v>
       </c>
-      <c r="J620" t="b">
+      <c r="J620" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K620" t="n">
+      <c r="K620" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L620" t="b">
+      <c r="L620" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M620" t="n">
+      <c r="M620" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="N620" t="n">
-        <v>0</v>
-      </c>
-      <c r="O620" t="n">
-        <v>0</v>
-      </c>
-      <c r="P620" t="b">
+      <c r="N620" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O620" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P620" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="621">
-      <c r="A621" t="inlineStr">
+      <c r="A621" s="10" t="inlineStr">
         <is>
           <t>The Rescuers</t>
         </is>
       </c>
-      <c r="B621" t="inlineStr">
+      <c r="B621" s="10" t="inlineStr">
         <is>
           <t>card_620</t>
         </is>
       </c>
-      <c r="C621" t="inlineStr">
+      <c r="C621" s="10" t="inlineStr">
         <is>
           <t>Wolfgang Reitherman, John Lounsbery and Art Stevens</t>
         </is>
       </c>
-      <c r="D621" t="n">
+      <c r="D621" s="10" t="n">
         <v>1977</v>
       </c>
-      <c r="E621" t="n">
+      <c r="E621" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="F621" t="n">
+      <c r="F621" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I621" t="n">
+      <c r="I621" s="10" t="n">
         <v>169000000</v>
       </c>
-      <c r="J621" t="b">
-        <v>0</v>
-      </c>
-      <c r="K621" t="n">
+      <c r="J621" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K621" s="10" t="n">
         <v>7500000</v>
       </c>
-      <c r="L621" t="b">
-        <v>0</v>
-      </c>
-      <c r="M621" t="n">
+      <c r="L621" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M621" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="N621" t="n">
-        <v>0</v>
-      </c>
-      <c r="O621" t="n">
-        <v>0</v>
-      </c>
-      <c r="P621" t="b">
+      <c r="N621" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O621" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P621" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="622">
-      <c r="A622" t="inlineStr">
+      <c r="A622" s="10" t="inlineStr">
         <is>
           <t>The Fox and the Hound</t>
         </is>
       </c>
-      <c r="B622" t="inlineStr">
+      <c r="B622" s="10" t="inlineStr">
         <is>
           <t>card_621</t>
         </is>
       </c>
-      <c r="C622" t="inlineStr">
+      <c r="C622" s="10" t="inlineStr">
         <is>
           <t>Ted Berman, Richard Rich and Art Stevens</t>
         </is>
       </c>
-      <c r="D622" t="n">
+      <c r="D622" s="10" t="n">
         <v>1981</v>
       </c>
-      <c r="E622" t="n">
+      <c r="E622" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F622" t="n">
+      <c r="F622" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I622" t="n">
+      <c r="I622" s="10" t="n">
         <v>63500000</v>
       </c>
-      <c r="J622" t="b">
-        <v>0</v>
-      </c>
-      <c r="K622" t="n">
+      <c r="J622" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K622" s="10" t="n">
         <v>12000000</v>
       </c>
-      <c r="L622" t="b">
-        <v>0</v>
-      </c>
-      <c r="M622" t="n">
+      <c r="L622" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M622" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="N622" t="n">
-        <v>0</v>
-      </c>
-      <c r="O622" t="n">
-        <v>0</v>
-      </c>
-      <c r="P622" t="b">
+      <c r="N622" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O622" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P622" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="623">
-      <c r="A623" t="inlineStr">
+      <c r="A623" s="10" t="inlineStr">
         <is>
           <t>The Black Cauldron</t>
         </is>
       </c>
-      <c r="B623" t="inlineStr">
+      <c r="B623" s="10" t="inlineStr">
         <is>
           <t>card_622</t>
         </is>
       </c>
-      <c r="C623" t="inlineStr">
+      <c r="C623" s="10" t="inlineStr">
         <is>
           <t>Ted Berman and Richard Rich</t>
         </is>
       </c>
-      <c r="D623" t="n">
+      <c r="D623" s="10" t="n">
         <v>1985</v>
       </c>
-      <c r="E623" t="n">
+      <c r="E623" s="10" t="n">
         <v>3.1</v>
       </c>
-      <c r="F623" t="n">
+      <c r="F623" s="10" t="n">
         <v>58</v>
       </c>
-      <c r="I623" t="n">
+      <c r="I623" s="10" t="n">
         <v>21300000</v>
       </c>
-      <c r="J623" t="b">
-        <v>0</v>
-      </c>
-      <c r="K623" t="n">
+      <c r="J623" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K623" s="10" t="n">
         <v>44000000</v>
       </c>
-      <c r="L623" t="b">
-        <v>0</v>
-      </c>
-      <c r="M623" t="n">
+      <c r="L623" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M623" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="N623" t="n">
-        <v>0</v>
-      </c>
-      <c r="O623" t="n">
-        <v>0</v>
-      </c>
-      <c r="P623" t="b">
+      <c r="N623" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O623" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P623" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="624">
-      <c r="A624" t="inlineStr">
+      <c r="A624" s="10" t="inlineStr">
         <is>
           <t>The Great Mouse Detective</t>
         </is>
       </c>
-      <c r="B624" t="inlineStr">
+      <c r="B624" s="10" t="inlineStr">
         <is>
           <t>card_623</t>
         </is>
       </c>
-      <c r="C624" t="inlineStr">
+      <c r="C624" s="10" t="inlineStr">
         <is>
           <t>John Musker, Ron Clements, Dave Michener and Burny Mattinson</t>
         </is>
       </c>
-      <c r="D624" t="n">
+      <c r="D624" s="10" t="n">
         <v>1986</v>
       </c>
-      <c r="E624" t="n">
+      <c r="E624" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F624" t="n">
+      <c r="F624" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="I624" t="n">
+      <c r="I624" s="10" t="n">
         <v>50000000</v>
       </c>
-      <c r="J624" t="b">
-        <v>0</v>
-      </c>
-      <c r="K624" t="n">
+      <c r="J624" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K624" s="10" t="n">
         <v>14000000</v>
       </c>
-      <c r="L624" t="b">
-        <v>0</v>
-      </c>
-      <c r="M624" t="n">
+      <c r="L624" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M624" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="N624" t="n">
-        <v>0</v>
-      </c>
-      <c r="O624" t="n">
-        <v>0</v>
-      </c>
-      <c r="P624" t="b">
+      <c r="N624" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O624" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P624" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="625">
-      <c r="A625" t="inlineStr">
+      <c r="A625" s="10" t="inlineStr">
         <is>
           <t>Oliver &amp; Company</t>
         </is>
       </c>
-      <c r="B625" t="inlineStr">
+      <c r="B625" s="10" t="inlineStr">
         <is>
           <t>card_624</t>
         </is>
       </c>
-      <c r="C625" t="inlineStr">
+      <c r="C625" s="10" t="inlineStr">
         <is>
           <t>George Scribner</t>
         </is>
       </c>
-      <c r="D625" t="n">
+      <c r="D625" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E625" t="n">
+      <c r="E625" s="10" t="n">
         <v>3.31</v>
       </c>
-      <c r="F625" t="n">
+      <c r="F625" s="10" t="n">
         <v>70</v>
       </c>
-      <c r="I625" t="n">
+      <c r="I625" s="10" t="n">
         <v>121000000</v>
       </c>
-      <c r="J625" t="b">
-        <v>0</v>
-      </c>
-      <c r="K625" t="n">
+      <c r="J625" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K625" s="10" t="n">
         <v>31000000</v>
       </c>
-      <c r="L625" t="b">
-        <v>0</v>
-      </c>
-      <c r="M625" t="n">
+      <c r="L625" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M625" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="N625" t="n">
-        <v>0</v>
-      </c>
-      <c r="O625" t="n">
-        <v>0</v>
-      </c>
-      <c r="P625" t="b">
+      <c r="N625" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O625" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P625" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="626">
-      <c r="A626" t="inlineStr">
+      <c r="A626" s="10" t="inlineStr">
         <is>
           <t>The Little Mermaid</t>
         </is>
       </c>
-      <c r="B626" t="inlineStr">
+      <c r="B626" s="10" t="inlineStr">
         <is>
           <t>card_625</t>
         </is>
       </c>
-      <c r="C626" t="inlineStr">
+      <c r="C626" s="10" t="inlineStr">
         <is>
           <t>John Musker and Ron Clements</t>
         </is>
       </c>
-      <c r="D626" t="n">
+      <c r="D626" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E626" t="n">
+      <c r="E626" s="10" t="n">
         <v>3.71</v>
       </c>
-      <c r="F626" t="n">
+      <c r="F626" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I626" t="n">
+      <c r="I626" s="10" t="n">
         <v>235000000</v>
       </c>
-      <c r="J626" t="b">
-        <v>0</v>
-      </c>
-      <c r="K626" t="n">
+      <c r="J626" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K626" s="10" t="n">
         <v>40000000</v>
       </c>
-      <c r="L626" t="b">
-        <v>0</v>
-      </c>
-      <c r="M626" t="n">
+      <c r="L626" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M626" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="N626" t="n">
+      <c r="N626" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O626" t="n">
-        <v>0</v>
-      </c>
-      <c r="P626" t="b">
+      <c r="O626" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P626" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="627">
-      <c r="A627" t="inlineStr">
+      <c r="A627" s="10" t="inlineStr">
         <is>
           <t>The Rescuers Down Under</t>
         </is>
       </c>
-      <c r="B627" t="inlineStr">
+      <c r="B627" s="10" t="inlineStr">
         <is>
           <t>card_626</t>
         </is>
       </c>
-      <c r="C627" t="inlineStr">
+      <c r="C627" s="10" t="inlineStr">
         <is>
           <t>Hendel Butoy and Mike Gabriel</t>
         </is>
       </c>
-      <c r="D627" t="n">
+      <c r="D627" s="10" t="n">
         <v>1990</v>
       </c>
-      <c r="E627" t="n">
+      <c r="E627" s="10" t="n">
         <v>3.24</v>
       </c>
-      <c r="F627" t="n">
+      <c r="F627" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I627" t="n">
+      <c r="I627" s="10" t="n">
         <v>47400000</v>
       </c>
-      <c r="J627" t="b">
-        <v>0</v>
-      </c>
-      <c r="K627" t="n">
+      <c r="J627" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K627" s="10" t="n">
         <v>38000000</v>
       </c>
-      <c r="L627" t="b">
-        <v>0</v>
-      </c>
-      <c r="M627" t="n">
+      <c r="L627" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M627" s="10" t="n">
         <v>77</v>
       </c>
-      <c r="N627" t="n">
-        <v>0</v>
-      </c>
-      <c r="O627" t="n">
-        <v>0</v>
-      </c>
-      <c r="P627" t="b">
+      <c r="N627" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O627" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P627" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="628">
-      <c r="A628" t="inlineStr">
+      <c r="A628" s="10" t="inlineStr">
         <is>
           <t>Beauty and the Beast</t>
         </is>
       </c>
-      <c r="B628" t="inlineStr">
+      <c r="B628" s="10" t="inlineStr">
         <is>
           <t>card_627</t>
         </is>
       </c>
-      <c r="C628" t="inlineStr">
+      <c r="C628" s="10" t="inlineStr">
         <is>
           <t>Gary Trousdale and Kirk Wise</t>
         </is>
       </c>
-      <c r="D628" t="n">
+      <c r="D628" s="10" t="n">
         <v>1991</v>
       </c>
-      <c r="E628" t="n">
+      <c r="E628" s="10" t="n">
         <v>4.08</v>
       </c>
-      <c r="F628" t="n">
+      <c r="F628" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="I628" t="n">
+      <c r="I628" s="10" t="n">
         <v>451200000</v>
       </c>
-      <c r="J628" t="b">
-        <v>0</v>
-      </c>
-      <c r="K628" t="n">
+      <c r="J628" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K628" s="10" t="n">
         <v>25000000</v>
       </c>
-      <c r="L628" t="b">
-        <v>0</v>
-      </c>
-      <c r="M628" t="n">
+      <c r="L628" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M628" s="10" t="n">
         <v>84</v>
       </c>
-      <c r="N628" t="n">
+      <c r="N628" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O628" t="n">
-        <v>0</v>
-      </c>
-      <c r="P628" t="b">
+      <c r="O628" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P628" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Pocahontas</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>card_628</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>Mike Gabriel and Eric Goldberg</t>
+        </is>
+      </c>
+      <c r="D629" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E629" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F629" t="n">
+        <v>71</v>
+      </c>
+      <c r="I629" t="n">
+        <v>346100000</v>
+      </c>
+      <c r="J629" t="b">
+        <v>0</v>
+      </c>
+      <c r="K629" t="n">
+        <v>55000000</v>
+      </c>
+      <c r="L629" t="b">
+        <v>0</v>
+      </c>
+      <c r="M629" t="n">
+        <v>81</v>
+      </c>
+      <c r="N629" t="n">
+        <v>2</v>
+      </c>
+      <c r="O629" t="n">
+        <v>0</v>
+      </c>
+      <c r="P629" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>The Hunchback of Notre Dame</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>card_629</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>Gary Trousdale and Kirk Wise</t>
+        </is>
+      </c>
+      <c r="D630" t="n">
+        <v>1996</v>
+      </c>
+      <c r="E630" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="F630" t="n">
+        <v>78</v>
+      </c>
+      <c r="I630" t="n">
+        <v>325000000</v>
+      </c>
+      <c r="J630" t="b">
+        <v>0</v>
+      </c>
+      <c r="K630" t="n">
+        <v>70000000</v>
+      </c>
+      <c r="L630" t="b">
+        <v>0</v>
+      </c>
+      <c r="M630" t="n">
+        <v>91</v>
+      </c>
+      <c r="N630" t="n">
+        <v>0</v>
+      </c>
+      <c r="O630" t="n">
+        <v>0</v>
+      </c>
+      <c r="P630" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Hercules</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>card_630</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>John Musker and Ron Clements</t>
+        </is>
+      </c>
+      <c r="D631" t="n">
+        <v>1997</v>
+      </c>
+      <c r="E631" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="F631" t="n">
+        <v>62</v>
+      </c>
+      <c r="I631" t="n">
+        <v>252700000</v>
+      </c>
+      <c r="J631" t="b">
+        <v>0</v>
+      </c>
+      <c r="K631" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="L631" t="b">
+        <v>0</v>
+      </c>
+      <c r="M631" t="n">
+        <v>93</v>
+      </c>
+      <c r="N631" t="n">
+        <v>0</v>
+      </c>
+      <c r="O631" t="n">
+        <v>0</v>
+      </c>
+      <c r="P631" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Mulan</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>card_631</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Barry Cook and Tony Bancroft</t>
+        </is>
+      </c>
+      <c r="D632" t="n">
+        <v>1998</v>
+      </c>
+      <c r="E632" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="F632" t="n">
+        <v>82</v>
+      </c>
+      <c r="I632" t="n">
+        <v>304000000</v>
+      </c>
+      <c r="J632" t="b">
+        <v>0</v>
+      </c>
+      <c r="K632" t="n">
+        <v>90000000</v>
+      </c>
+      <c r="L632" t="b">
+        <v>0</v>
+      </c>
+      <c r="M632" t="n">
+        <v>88</v>
+      </c>
+      <c r="N632" t="n">
+        <v>0</v>
+      </c>
+      <c r="O632" t="n">
+        <v>0</v>
+      </c>
+      <c r="P632" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Tarzan</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>card_632</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Kevin Lima and Chris Buck</t>
+        </is>
+      </c>
+      <c r="D633" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E633" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="F633" t="n">
+        <v>78</v>
+      </c>
+      <c r="I633" t="n">
+        <v>448200000</v>
+      </c>
+      <c r="J633" t="b">
+        <v>0</v>
+      </c>
+      <c r="K633" t="n">
+        <v>130000000</v>
+      </c>
+      <c r="L633" t="b">
+        <v>0</v>
+      </c>
+      <c r="M633" t="n">
+        <v>88</v>
+      </c>
+      <c r="N633" t="n">
+        <v>1</v>
+      </c>
+      <c r="O633" t="n">
+        <v>0</v>
+      </c>
+      <c r="P633" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Fantasia 2000</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>card_633</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Pixote Hunt, Hendel Butoy and Eric Goldberg</t>
+        </is>
+      </c>
+      <c r="D634" t="n">
+        <v>1999</v>
+      </c>
+      <c r="E634" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="F634" t="n">
+        <v>72</v>
+      </c>
+      <c r="I634" t="n">
+        <v>90900000</v>
+      </c>
+      <c r="J634" t="b">
+        <v>0</v>
+      </c>
+      <c r="K634" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L634" t="b">
+        <v>0</v>
+      </c>
+      <c r="M634" t="n">
+        <v>75</v>
+      </c>
+      <c r="N634" t="n">
+        <v>0</v>
+      </c>
+      <c r="O634" t="n">
+        <v>0</v>
+      </c>
+      <c r="P634" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Dinosaur</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>card_634</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Ralph Zondag and Eric Leighton</t>
+        </is>
+      </c>
+      <c r="D635" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E635" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="F635" t="n">
+        <v>66</v>
+      </c>
+      <c r="I635" t="n">
+        <v>349800000</v>
+      </c>
+      <c r="J635" t="b">
+        <v>0</v>
+      </c>
+      <c r="K635" t="n">
+        <v>127500000</v>
+      </c>
+      <c r="L635" t="b">
+        <v>0</v>
+      </c>
+      <c r="M635" t="n">
+        <v>82</v>
+      </c>
+      <c r="N635" t="n">
+        <v>0</v>
+      </c>
+      <c r="O635" t="n">
+        <v>0</v>
+      </c>
+      <c r="P635" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>The Emperor's New Groove</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>card_635</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Mark Dindal</t>
+        </is>
+      </c>
+      <c r="D636" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E636" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="F636" t="n">
+        <v>79</v>
+      </c>
+      <c r="I636" t="n">
+        <v>169700000</v>
+      </c>
+      <c r="J636" t="b">
+        <v>0</v>
+      </c>
+      <c r="K636" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L636" t="b">
+        <v>0</v>
+      </c>
+      <c r="M636" t="n">
+        <v>78</v>
+      </c>
+      <c r="N636" t="n">
+        <v>0</v>
+      </c>
+      <c r="O636" t="n">
+        <v>0</v>
+      </c>
+      <c r="P636" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Atlantis: The Lost Empire</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>card_636</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>Gary Trousdale and Kirk Wise</t>
+        </is>
+      </c>
+      <c r="D637" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E637" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="F637" t="n">
+        <v>72</v>
+      </c>
+      <c r="I637" t="n">
+        <v>186100000</v>
+      </c>
+      <c r="J637" t="b">
+        <v>0</v>
+      </c>
+      <c r="K637" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L637" t="b">
+        <v>0</v>
+      </c>
+      <c r="M637" t="n">
+        <v>96</v>
+      </c>
+      <c r="N637" t="n">
+        <v>0</v>
+      </c>
+      <c r="O637" t="n">
+        <v>0</v>
+      </c>
+      <c r="P637" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disney animated canon, part 3a: 2002-2009 (card_637-644)
Lilo & Stitch through The Princess and the Frog, 8 films.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P637"/>
+  <dimension ref="A1:P645"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -33045,452 +33045,852 @@
       </c>
     </row>
     <row r="629">
-      <c r="A629" t="inlineStr">
+      <c r="A629" s="10" t="inlineStr">
         <is>
           <t>Pocahontas</t>
         </is>
       </c>
-      <c r="B629" t="inlineStr">
+      <c r="B629" s="10" t="inlineStr">
         <is>
           <t>card_628</t>
         </is>
       </c>
-      <c r="C629" t="inlineStr">
+      <c r="C629" s="10" t="inlineStr">
         <is>
           <t>Mike Gabriel and Eric Goldberg</t>
         </is>
       </c>
-      <c r="D629" t="n">
+      <c r="D629" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E629" t="n">
+      <c r="E629" s="10" t="n">
         <v>3.3</v>
       </c>
-      <c r="F629" t="n">
+      <c r="F629" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I629" t="n">
+      <c r="I629" s="10" t="n">
         <v>346100000</v>
       </c>
-      <c r="J629" t="b">
-        <v>0</v>
-      </c>
-      <c r="K629" t="n">
+      <c r="J629" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K629" s="10" t="n">
         <v>55000000</v>
       </c>
-      <c r="L629" t="b">
-        <v>0</v>
-      </c>
-      <c r="M629" t="n">
+      <c r="L629" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M629" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="N629" t="n">
+      <c r="N629" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O629" t="n">
-        <v>0</v>
-      </c>
-      <c r="P629" t="b">
+      <c r="O629" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P629" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="630">
-      <c r="A630" t="inlineStr">
+      <c r="A630" s="10" t="inlineStr">
         <is>
           <t>The Hunchback of Notre Dame</t>
         </is>
       </c>
-      <c r="B630" t="inlineStr">
+      <c r="B630" s="10" t="inlineStr">
         <is>
           <t>card_629</t>
         </is>
       </c>
-      <c r="C630" t="inlineStr">
+      <c r="C630" s="10" t="inlineStr">
         <is>
           <t>Gary Trousdale and Kirk Wise</t>
         </is>
       </c>
-      <c r="D630" t="n">
+      <c r="D630" s="10" t="n">
         <v>1996</v>
       </c>
-      <c r="E630" t="n">
+      <c r="E630" s="10" t="n">
         <v>3.44</v>
       </c>
-      <c r="F630" t="n">
+      <c r="F630" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I630" t="n">
+      <c r="I630" s="10" t="n">
         <v>325000000</v>
       </c>
-      <c r="J630" t="b">
-        <v>0</v>
-      </c>
-      <c r="K630" t="n">
+      <c r="J630" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K630" s="10" t="n">
         <v>70000000</v>
       </c>
-      <c r="L630" t="b">
-        <v>0</v>
-      </c>
-      <c r="M630" t="n">
+      <c r="L630" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M630" s="10" t="n">
         <v>91</v>
       </c>
-      <c r="N630" t="n">
-        <v>0</v>
-      </c>
-      <c r="O630" t="n">
-        <v>0</v>
-      </c>
-      <c r="P630" t="b">
+      <c r="N630" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O630" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P630" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="631">
-      <c r="A631" t="inlineStr">
+      <c r="A631" s="10" t="inlineStr">
         <is>
           <t>Hercules</t>
         </is>
       </c>
-      <c r="B631" t="inlineStr">
+      <c r="B631" s="10" t="inlineStr">
         <is>
           <t>card_630</t>
         </is>
       </c>
-      <c r="C631" t="inlineStr">
+      <c r="C631" s="10" t="inlineStr">
         <is>
           <t>John Musker and Ron Clements</t>
         </is>
       </c>
-      <c r="D631" t="n">
+      <c r="D631" s="10" t="n">
         <v>1997</v>
       </c>
-      <c r="E631" t="n">
+      <c r="E631" s="10" t="n">
         <v>2.67</v>
       </c>
-      <c r="F631" t="n">
+      <c r="F631" s="10" t="n">
         <v>62</v>
       </c>
-      <c r="I631" t="n">
+      <c r="I631" s="10" t="n">
         <v>252700000</v>
       </c>
-      <c r="J631" t="b">
-        <v>0</v>
-      </c>
-      <c r="K631" t="n">
+      <c r="J631" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K631" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="L631" t="b">
-        <v>0</v>
-      </c>
-      <c r="M631" t="n">
+      <c r="L631" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M631" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N631" t="n">
-        <v>0</v>
-      </c>
-      <c r="O631" t="n">
-        <v>0</v>
-      </c>
-      <c r="P631" t="b">
+      <c r="N631" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O631" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P631" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="632">
-      <c r="A632" t="inlineStr">
+      <c r="A632" s="10" t="inlineStr">
         <is>
           <t>Mulan</t>
         </is>
       </c>
-      <c r="B632" t="inlineStr">
+      <c r="B632" s="10" t="inlineStr">
         <is>
           <t>card_631</t>
         </is>
       </c>
-      <c r="C632" t="inlineStr">
+      <c r="C632" s="10" t="inlineStr">
         <is>
           <t>Barry Cook and Tony Bancroft</t>
         </is>
       </c>
-      <c r="D632" t="n">
+      <c r="D632" s="10" t="n">
         <v>1998</v>
       </c>
-      <c r="E632" t="n">
+      <c r="E632" s="10" t="n">
         <v>4.17</v>
       </c>
-      <c r="F632" t="n">
+      <c r="F632" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="I632" t="n">
+      <c r="I632" s="10" t="n">
         <v>304000000</v>
       </c>
-      <c r="J632" t="b">
-        <v>0</v>
-      </c>
-      <c r="K632" t="n">
+      <c r="J632" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K632" s="10" t="n">
         <v>90000000</v>
       </c>
-      <c r="L632" t="b">
-        <v>0</v>
-      </c>
-      <c r="M632" t="n">
+      <c r="L632" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M632" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N632" t="n">
-        <v>0</v>
-      </c>
-      <c r="O632" t="n">
-        <v>0</v>
-      </c>
-      <c r="P632" t="b">
+      <c r="N632" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O632" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P632" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="633">
-      <c r="A633" t="inlineStr">
+      <c r="A633" s="10" t="inlineStr">
         <is>
           <t>Tarzan</t>
         </is>
       </c>
-      <c r="B633" t="inlineStr">
+      <c r="B633" s="10" t="inlineStr">
         <is>
           <t>card_632</t>
         </is>
       </c>
-      <c r="C633" t="inlineStr">
+      <c r="C633" s="10" t="inlineStr">
         <is>
           <t>Kevin Lima and Chris Buck</t>
         </is>
       </c>
-      <c r="D633" t="n">
+      <c r="D633" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E633" t="n">
+      <c r="E633" s="10" t="n">
         <v>3.74</v>
       </c>
-      <c r="F633" t="n">
+      <c r="F633" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I633" t="n">
+      <c r="I633" s="10" t="n">
         <v>448200000</v>
       </c>
-      <c r="J633" t="b">
-        <v>0</v>
-      </c>
-      <c r="K633" t="n">
+      <c r="J633" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K633" s="10" t="n">
         <v>130000000</v>
       </c>
-      <c r="L633" t="b">
-        <v>0</v>
-      </c>
-      <c r="M633" t="n">
+      <c r="L633" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M633" s="10" t="n">
         <v>88</v>
       </c>
-      <c r="N633" t="n">
+      <c r="N633" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O633" t="n">
-        <v>0</v>
-      </c>
-      <c r="P633" t="b">
+      <c r="O633" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P633" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="634">
-      <c r="A634" t="inlineStr">
+      <c r="A634" s="10" t="inlineStr">
         <is>
           <t>Fantasia 2000</t>
         </is>
       </c>
-      <c r="B634" t="inlineStr">
+      <c r="B634" s="10" t="inlineStr">
         <is>
           <t>card_633</t>
         </is>
       </c>
-      <c r="C634" t="inlineStr">
+      <c r="C634" s="10" t="inlineStr">
         <is>
           <t>Pixote Hunt, Hendel Butoy and Eric Goldberg</t>
         </is>
       </c>
-      <c r="D634" t="n">
+      <c r="D634" s="10" t="n">
         <v>1999</v>
       </c>
-      <c r="E634" t="n">
+      <c r="E634" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="F634" t="n">
+      <c r="F634" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I634" t="n">
+      <c r="I634" s="10" t="n">
         <v>90900000</v>
       </c>
-      <c r="J634" t="b">
-        <v>0</v>
-      </c>
-      <c r="K634" t="n">
+      <c r="J634" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K634" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L634" t="b">
-        <v>0</v>
-      </c>
-      <c r="M634" t="n">
+      <c r="L634" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M634" s="10" t="n">
         <v>75</v>
       </c>
-      <c r="N634" t="n">
-        <v>0</v>
-      </c>
-      <c r="O634" t="n">
-        <v>0</v>
-      </c>
-      <c r="P634" t="b">
+      <c r="N634" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O634" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P634" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="635">
-      <c r="A635" t="inlineStr">
+      <c r="A635" s="10" t="inlineStr">
         <is>
           <t>Dinosaur</t>
         </is>
       </c>
-      <c r="B635" t="inlineStr">
+      <c r="B635" s="10" t="inlineStr">
         <is>
           <t>card_634</t>
         </is>
       </c>
-      <c r="C635" t="inlineStr">
+      <c r="C635" s="10" t="inlineStr">
         <is>
           <t>Ralph Zondag and Eric Leighton</t>
         </is>
       </c>
-      <c r="D635" t="n">
+      <c r="D635" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E635" t="n">
+      <c r="E635" s="10" t="n">
         <v>3.04</v>
       </c>
-      <c r="F635" t="n">
+      <c r="F635" s="10" t="n">
         <v>66</v>
       </c>
-      <c r="I635" t="n">
+      <c r="I635" s="10" t="n">
         <v>349800000</v>
       </c>
-      <c r="J635" t="b">
-        <v>0</v>
-      </c>
-      <c r="K635" t="n">
+      <c r="J635" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K635" s="10" t="n">
         <v>127500000</v>
       </c>
-      <c r="L635" t="b">
-        <v>0</v>
-      </c>
-      <c r="M635" t="n">
+      <c r="L635" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M635" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="N635" t="n">
-        <v>0</v>
-      </c>
-      <c r="O635" t="n">
-        <v>0</v>
-      </c>
-      <c r="P635" t="b">
+      <c r="N635" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O635" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P635" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="636">
-      <c r="A636" t="inlineStr">
+      <c r="A636" s="10" t="inlineStr">
         <is>
           <t>The Emperor's New Groove</t>
         </is>
       </c>
-      <c r="B636" t="inlineStr">
+      <c r="B636" s="10" t="inlineStr">
         <is>
           <t>card_635</t>
         </is>
       </c>
-      <c r="C636" t="inlineStr">
+      <c r="C636" s="10" t="inlineStr">
         <is>
           <t>Mark Dindal</t>
         </is>
       </c>
-      <c r="D636" t="n">
+      <c r="D636" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E636" t="n">
+      <c r="E636" s="10" t="n">
         <v>3.94</v>
       </c>
-      <c r="F636" t="n">
+      <c r="F636" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="I636" t="n">
+      <c r="I636" s="10" t="n">
         <v>169700000</v>
       </c>
-      <c r="J636" t="b">
-        <v>0</v>
-      </c>
-      <c r="K636" t="n">
+      <c r="J636" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K636" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L636" t="b">
-        <v>0</v>
-      </c>
-      <c r="M636" t="n">
+      <c r="L636" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M636" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="N636" t="n">
-        <v>0</v>
-      </c>
-      <c r="O636" t="n">
-        <v>0</v>
-      </c>
-      <c r="P636" t="b">
+      <c r="N636" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O636" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P636" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="637">
-      <c r="A637" t="inlineStr">
+      <c r="A637" s="10" t="inlineStr">
         <is>
           <t>Atlantis: The Lost Empire</t>
         </is>
       </c>
-      <c r="B637" t="inlineStr">
+      <c r="B637" s="10" t="inlineStr">
         <is>
           <t>card_636</t>
         </is>
       </c>
-      <c r="C637" t="inlineStr">
+      <c r="C637" s="10" t="inlineStr">
         <is>
           <t>Gary Trousdale and Kirk Wise</t>
         </is>
       </c>
-      <c r="D637" t="n">
+      <c r="D637" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E637" t="n">
+      <c r="E637" s="10" t="n">
         <v>3.78</v>
       </c>
-      <c r="F637" t="n">
+      <c r="F637" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I637" t="n">
+      <c r="I637" s="10" t="n">
         <v>186100000</v>
       </c>
-      <c r="J637" t="b">
-        <v>0</v>
-      </c>
-      <c r="K637" t="n">
+      <c r="J637" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K637" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L637" t="b">
-        <v>0</v>
-      </c>
-      <c r="M637" t="n">
+      <c r="L637" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M637" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N637" t="n">
-        <v>0</v>
-      </c>
-      <c r="O637" t="n">
-        <v>0</v>
-      </c>
-      <c r="P637" t="b">
+      <c r="N637" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O637" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P637" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Lilo &amp; Stitch</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>card_637</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Chris Sanders and Dean DeBlois</t>
+        </is>
+      </c>
+      <c r="D638" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E638" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="F638" t="n">
+        <v>80</v>
+      </c>
+      <c r="I638" t="n">
+        <v>273100000</v>
+      </c>
+      <c r="J638" t="b">
+        <v>0</v>
+      </c>
+      <c r="K638" t="n">
+        <v>80000000</v>
+      </c>
+      <c r="L638" t="b">
+        <v>0</v>
+      </c>
+      <c r="M638" t="n">
+        <v>85</v>
+      </c>
+      <c r="N638" t="n">
+        <v>0</v>
+      </c>
+      <c r="O638" t="n">
+        <v>0</v>
+      </c>
+      <c r="P638" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Treasure Planet</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>card_638</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>John Musker and Ron Clements</t>
+        </is>
+      </c>
+      <c r="D639" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E639" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="F639" t="n">
+        <v>80</v>
+      </c>
+      <c r="I639" t="n">
+        <v>109600000</v>
+      </c>
+      <c r="J639" t="b">
+        <v>0</v>
+      </c>
+      <c r="K639" t="n">
+        <v>140000000</v>
+      </c>
+      <c r="L639" t="b">
+        <v>0</v>
+      </c>
+      <c r="M639" t="n">
+        <v>95</v>
+      </c>
+      <c r="N639" t="n">
+        <v>0</v>
+      </c>
+      <c r="O639" t="n">
+        <v>0</v>
+      </c>
+      <c r="P639" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Brother Bear</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>card_639</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>Aaron Blaise and Robert Walker</t>
+        </is>
+      </c>
+      <c r="D640" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E640" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="F640" t="n">
+        <v>68</v>
+      </c>
+      <c r="I640" t="n">
+        <v>250400000</v>
+      </c>
+      <c r="J640" t="b">
+        <v>0</v>
+      </c>
+      <c r="K640" t="n">
+        <v>46000000</v>
+      </c>
+      <c r="L640" t="b">
+        <v>0</v>
+      </c>
+      <c r="M640" t="n">
+        <v>85</v>
+      </c>
+      <c r="N640" t="n">
+        <v>0</v>
+      </c>
+      <c r="O640" t="n">
+        <v>0</v>
+      </c>
+      <c r="P640" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Home on the Range</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>card_640</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>Will Finn and John Sanford</t>
+        </is>
+      </c>
+      <c r="D641" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E641" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F641" t="n">
+        <v>50</v>
+      </c>
+      <c r="I641" t="n">
+        <v>145300000</v>
+      </c>
+      <c r="J641" t="b">
+        <v>0</v>
+      </c>
+      <c r="K641" t="n">
+        <v>110000000</v>
+      </c>
+      <c r="L641" t="b">
+        <v>0</v>
+      </c>
+      <c r="M641" t="n">
+        <v>76</v>
+      </c>
+      <c r="N641" t="n">
+        <v>0</v>
+      </c>
+      <c r="O641" t="n">
+        <v>0</v>
+      </c>
+      <c r="P641" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Chicken Little</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>card_641</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Mark Dindal</t>
+        </is>
+      </c>
+      <c r="D642" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E642" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="F642" t="n">
+        <v>52</v>
+      </c>
+      <c r="I642" t="n">
+        <v>314400000</v>
+      </c>
+      <c r="J642" t="b">
+        <v>0</v>
+      </c>
+      <c r="K642" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L642" t="b">
+        <v>0</v>
+      </c>
+      <c r="M642" t="n">
+        <v>81</v>
+      </c>
+      <c r="N642" t="n">
+        <v>0</v>
+      </c>
+      <c r="O642" t="n">
+        <v>0</v>
+      </c>
+      <c r="P642" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Meet the Robinsons</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>card_642</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>Stephen Anderson</t>
+        </is>
+      </c>
+      <c r="D643" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E643" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F643" t="n">
+        <v>68</v>
+      </c>
+      <c r="I643" t="n">
+        <v>170500000</v>
+      </c>
+      <c r="J643" t="b">
+        <v>0</v>
+      </c>
+      <c r="K643" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L643" t="b">
+        <v>0</v>
+      </c>
+      <c r="M643" t="n">
+        <v>95</v>
+      </c>
+      <c r="N643" t="n">
+        <v>0</v>
+      </c>
+      <c r="O643" t="n">
+        <v>0</v>
+      </c>
+      <c r="P643" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>card_643</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>Chris Williams and Byron Howard</t>
+        </is>
+      </c>
+      <c r="D644" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E644" t="n">
+        <v>3.24</v>
+      </c>
+      <c r="F644" t="n">
+        <v>72</v>
+      </c>
+      <c r="I644" t="n">
+        <v>310000000</v>
+      </c>
+      <c r="J644" t="b">
+        <v>0</v>
+      </c>
+      <c r="K644" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L644" t="b">
+        <v>0</v>
+      </c>
+      <c r="M644" t="n">
+        <v>96</v>
+      </c>
+      <c r="N644" t="n">
+        <v>0</v>
+      </c>
+      <c r="O644" t="n">
+        <v>0</v>
+      </c>
+      <c r="P644" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>The Princess and the Frog</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>card_644</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>John Musker and Ron Clements</t>
+        </is>
+      </c>
+      <c r="D645" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E645" t="n">
+        <v>4</v>
+      </c>
+      <c r="F645" t="n">
+        <v>73</v>
+      </c>
+      <c r="I645" t="n">
+        <v>271000000</v>
+      </c>
+      <c r="J645" t="b">
+        <v>0</v>
+      </c>
+      <c r="K645" t="n">
+        <v>105000000</v>
+      </c>
+      <c r="L645" t="b">
+        <v>0</v>
+      </c>
+      <c r="M645" t="n">
+        <v>97</v>
+      </c>
+      <c r="N645" t="n">
+        <v>0</v>
+      </c>
+      <c r="O645" t="n">
+        <v>0</v>
+      </c>
+      <c r="P645" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disney animated canon, part 3b: 2010-2014 (card_645-649)
Tangled, Winnie the Pooh (2011), Wreck-It Ralph, Frozen, Big Hero 6.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P645"/>
+  <dimension ref="A1:P650"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -33495,402 +33495,652 @@
       </c>
     </row>
     <row r="638">
-      <c r="A638" t="inlineStr">
+      <c r="A638" s="10" t="inlineStr">
         <is>
           <t>Lilo &amp; Stitch</t>
         </is>
       </c>
-      <c r="B638" t="inlineStr">
+      <c r="B638" s="10" t="inlineStr">
         <is>
           <t>card_637</t>
         </is>
       </c>
-      <c r="C638" t="inlineStr">
+      <c r="C638" s="10" t="inlineStr">
         <is>
           <t>Chris Sanders and Dean DeBlois</t>
         </is>
       </c>
-      <c r="D638" t="n">
+      <c r="D638" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E638" t="n">
+      <c r="E638" s="10" t="n">
         <v>4.06</v>
       </c>
-      <c r="F638" t="n">
+      <c r="F638" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I638" t="n">
+      <c r="I638" s="10" t="n">
         <v>273100000</v>
       </c>
-      <c r="J638" t="b">
-        <v>0</v>
-      </c>
-      <c r="K638" t="n">
+      <c r="J638" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K638" s="10" t="n">
         <v>80000000</v>
       </c>
-      <c r="L638" t="b">
-        <v>0</v>
-      </c>
-      <c r="M638" t="n">
+      <c r="L638" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M638" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="N638" t="n">
-        <v>0</v>
-      </c>
-      <c r="O638" t="n">
-        <v>0</v>
-      </c>
-      <c r="P638" t="b">
+      <c r="N638" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O638" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P638" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="639">
-      <c r="A639" t="inlineStr">
+      <c r="A639" s="10" t="inlineStr">
         <is>
           <t>Treasure Planet</t>
         </is>
       </c>
-      <c r="B639" t="inlineStr">
+      <c r="B639" s="10" t="inlineStr">
         <is>
           <t>card_638</t>
         </is>
       </c>
-      <c r="C639" t="inlineStr">
+      <c r="C639" s="10" t="inlineStr">
         <is>
           <t>John Musker and Ron Clements</t>
         </is>
       </c>
-      <c r="D639" t="n">
+      <c r="D639" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E639" t="n">
+      <c r="E639" s="10" t="n">
         <v>3.95</v>
       </c>
-      <c r="F639" t="n">
+      <c r="F639" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="I639" t="n">
+      <c r="I639" s="10" t="n">
         <v>109600000</v>
       </c>
-      <c r="J639" t="b">
-        <v>0</v>
-      </c>
-      <c r="K639" t="n">
+      <c r="J639" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K639" s="10" t="n">
         <v>140000000</v>
       </c>
-      <c r="L639" t="b">
-        <v>0</v>
-      </c>
-      <c r="M639" t="n">
+      <c r="L639" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M639" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N639" t="n">
-        <v>0</v>
-      </c>
-      <c r="O639" t="n">
-        <v>0</v>
-      </c>
-      <c r="P639" t="b">
+      <c r="N639" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O639" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P639" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="640">
-      <c r="A640" t="inlineStr">
+      <c r="A640" s="10" t="inlineStr">
         <is>
           <t>Brother Bear</t>
         </is>
       </c>
-      <c r="B640" t="inlineStr">
+      <c r="B640" s="10" t="inlineStr">
         <is>
           <t>card_639</t>
         </is>
       </c>
-      <c r="C640" t="inlineStr">
+      <c r="C640" s="10" t="inlineStr">
         <is>
           <t>Aaron Blaise and Robert Walker</t>
         </is>
       </c>
-      <c r="D640" t="n">
+      <c r="D640" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E640" t="n">
+      <c r="E640" s="10" t="n">
         <v>3.84</v>
       </c>
-      <c r="F640" t="n">
+      <c r="F640" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I640" t="n">
+      <c r="I640" s="10" t="n">
         <v>250400000</v>
       </c>
-      <c r="J640" t="b">
-        <v>0</v>
-      </c>
-      <c r="K640" t="n">
+      <c r="J640" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K640" s="10" t="n">
         <v>46000000</v>
       </c>
-      <c r="L640" t="b">
-        <v>0</v>
-      </c>
-      <c r="M640" t="n">
+      <c r="L640" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M640" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="N640" t="n">
-        <v>0</v>
-      </c>
-      <c r="O640" t="n">
-        <v>0</v>
-      </c>
-      <c r="P640" t="b">
+      <c r="N640" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O640" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P640" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="641">
-      <c r="A641" t="inlineStr">
+      <c r="A641" s="10" t="inlineStr">
         <is>
           <t>Home on the Range</t>
         </is>
       </c>
-      <c r="B641" t="inlineStr">
+      <c r="B641" s="10" t="inlineStr">
         <is>
           <t>card_640</t>
         </is>
       </c>
-      <c r="C641" t="inlineStr">
+      <c r="C641" s="10" t="inlineStr">
         <is>
           <t>Will Finn and John Sanford</t>
         </is>
       </c>
-      <c r="D641" t="n">
+      <c r="D641" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E641" t="n">
+      <c r="E641" s="10" t="n">
         <v>2.8</v>
       </c>
-      <c r="F641" t="n">
+      <c r="F641" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I641" t="n">
+      <c r="I641" s="10" t="n">
         <v>145300000</v>
       </c>
-      <c r="J641" t="b">
-        <v>0</v>
-      </c>
-      <c r="K641" t="n">
+      <c r="J641" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K641" s="10" t="n">
         <v>110000000</v>
       </c>
-      <c r="L641" t="b">
-        <v>0</v>
-      </c>
-      <c r="M641" t="n">
+      <c r="L641" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M641" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="N641" t="n">
-        <v>0</v>
-      </c>
-      <c r="O641" t="n">
-        <v>0</v>
-      </c>
-      <c r="P641" t="b">
+      <c r="N641" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O641" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P641" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="642">
-      <c r="A642" t="inlineStr">
+      <c r="A642" s="10" t="inlineStr">
         <is>
           <t>Chicken Little</t>
         </is>
       </c>
-      <c r="B642" t="inlineStr">
+      <c r="B642" s="10" t="inlineStr">
         <is>
           <t>card_641</t>
         </is>
       </c>
-      <c r="C642" t="inlineStr">
+      <c r="C642" s="10" t="inlineStr">
         <is>
           <t>Mark Dindal</t>
         </is>
       </c>
-      <c r="D642" t="n">
+      <c r="D642" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E642" t="n">
+      <c r="E642" s="10" t="n">
         <v>3.73</v>
       </c>
-      <c r="F642" t="n">
+      <c r="F642" s="10" t="n">
         <v>52</v>
       </c>
-      <c r="I642" t="n">
+      <c r="I642" s="10" t="n">
         <v>314400000</v>
       </c>
-      <c r="J642" t="b">
-        <v>0</v>
-      </c>
-      <c r="K642" t="n">
+      <c r="J642" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K642" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L642" t="b">
-        <v>0</v>
-      </c>
-      <c r="M642" t="n">
+      <c r="L642" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M642" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="N642" t="n">
-        <v>0</v>
-      </c>
-      <c r="O642" t="n">
-        <v>0</v>
-      </c>
-      <c r="P642" t="b">
+      <c r="N642" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O642" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P642" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="643">
-      <c r="A643" t="inlineStr">
+      <c r="A643" s="10" t="inlineStr">
         <is>
           <t>Meet the Robinsons</t>
         </is>
       </c>
-      <c r="B643" t="inlineStr">
+      <c r="B643" s="10" t="inlineStr">
         <is>
           <t>card_642</t>
         </is>
       </c>
-      <c r="C643" t="inlineStr">
+      <c r="C643" s="10" t="inlineStr">
         <is>
           <t>Stephen Anderson</t>
         </is>
       </c>
-      <c r="D643" t="n">
+      <c r="D643" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E643" t="n">
+      <c r="E643" s="10" t="n">
         <v>3.65</v>
       </c>
-      <c r="F643" t="n">
+      <c r="F643" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I643" t="n">
+      <c r="I643" s="10" t="n">
         <v>170500000</v>
       </c>
-      <c r="J643" t="b">
-        <v>0</v>
-      </c>
-      <c r="K643" t="n">
+      <c r="J643" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K643" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L643" t="b">
-        <v>0</v>
-      </c>
-      <c r="M643" t="n">
+      <c r="L643" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M643" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N643" t="n">
-        <v>0</v>
-      </c>
-      <c r="O643" t="n">
-        <v>0</v>
-      </c>
-      <c r="P643" t="b">
+      <c r="N643" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O643" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P643" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="644">
-      <c r="A644" t="inlineStr">
+      <c r="A644" s="10" t="inlineStr">
         <is>
           <t>Bolt</t>
         </is>
       </c>
-      <c r="B644" t="inlineStr">
+      <c r="B644" s="10" t="inlineStr">
         <is>
           <t>card_643</t>
         </is>
       </c>
-      <c r="C644" t="inlineStr">
+      <c r="C644" s="10" t="inlineStr">
         <is>
           <t>Chris Williams and Byron Howard</t>
         </is>
       </c>
-      <c r="D644" t="n">
+      <c r="D644" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E644" t="n">
+      <c r="E644" s="10" t="n">
         <v>3.24</v>
       </c>
-      <c r="F644" t="n">
+      <c r="F644" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I644" t="n">
+      <c r="I644" s="10" t="n">
         <v>310000000</v>
       </c>
-      <c r="J644" t="b">
-        <v>0</v>
-      </c>
-      <c r="K644" t="n">
+      <c r="J644" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K644" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L644" t="b">
-        <v>0</v>
-      </c>
-      <c r="M644" t="n">
+      <c r="L644" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M644" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N644" t="n">
-        <v>0</v>
-      </c>
-      <c r="O644" t="n">
-        <v>0</v>
-      </c>
-      <c r="P644" t="b">
+      <c r="N644" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O644" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P644" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="645">
-      <c r="A645" t="inlineStr">
+      <c r="A645" s="10" t="inlineStr">
         <is>
           <t>The Princess and the Frog</t>
         </is>
       </c>
-      <c r="B645" t="inlineStr">
+      <c r="B645" s="10" t="inlineStr">
         <is>
           <t>card_644</t>
         </is>
       </c>
-      <c r="C645" t="inlineStr">
+      <c r="C645" s="10" t="inlineStr">
         <is>
           <t>John Musker and Ron Clements</t>
         </is>
       </c>
-      <c r="D645" t="n">
+      <c r="D645" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E645" t="n">
+      <c r="E645" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F645" t="n">
+      <c r="F645" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I645" t="n">
+      <c r="I645" s="10" t="n">
         <v>271000000</v>
       </c>
-      <c r="J645" t="b">
-        <v>0</v>
-      </c>
-      <c r="K645" t="n">
+      <c r="J645" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K645" s="10" t="n">
         <v>105000000</v>
       </c>
-      <c r="L645" t="b">
-        <v>0</v>
-      </c>
-      <c r="M645" t="n">
+      <c r="L645" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M645" s="10" t="n">
         <v>97</v>
       </c>
-      <c r="N645" t="n">
-        <v>0</v>
-      </c>
-      <c r="O645" t="n">
-        <v>0</v>
-      </c>
-      <c r="P645" t="b">
+      <c r="N645" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O645" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P645" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Tangled</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>card_645</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Nathan Greno and Byron Howard</t>
+        </is>
+      </c>
+      <c r="D646" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E646" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="F646" t="n">
+        <v>81</v>
+      </c>
+      <c r="I646" t="n">
+        <v>592500000</v>
+      </c>
+      <c r="J646" t="b">
+        <v>0</v>
+      </c>
+      <c r="K646" t="n">
+        <v>260000000</v>
+      </c>
+      <c r="L646" t="b">
+        <v>0</v>
+      </c>
+      <c r="M646" t="n">
+        <v>100</v>
+      </c>
+      <c r="N646" t="n">
+        <v>0</v>
+      </c>
+      <c r="O646" t="n">
+        <v>0</v>
+      </c>
+      <c r="P646" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Winnie the Pooh</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>card_646</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Stephen Anderson and Don Hall</t>
+        </is>
+      </c>
+      <c r="D647" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E647" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="F647" t="n">
+        <v>76</v>
+      </c>
+      <c r="I647" t="n">
+        <v>50100000</v>
+      </c>
+      <c r="J647" t="b">
+        <v>0</v>
+      </c>
+      <c r="K647" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L647" t="b">
+        <v>0</v>
+      </c>
+      <c r="M647" t="n">
+        <v>63</v>
+      </c>
+      <c r="N647" t="n">
+        <v>0</v>
+      </c>
+      <c r="O647" t="n">
+        <v>0</v>
+      </c>
+      <c r="P647" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Wreck-It Ralph</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>card_647</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Rich Moore</t>
+        </is>
+      </c>
+      <c r="D648" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E648" t="n">
+        <v>3.62</v>
+      </c>
+      <c r="F648" t="n">
+        <v>83</v>
+      </c>
+      <c r="I648" t="n">
+        <v>496500000</v>
+      </c>
+      <c r="J648" t="b">
+        <v>0</v>
+      </c>
+      <c r="K648" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="L648" t="b">
+        <v>0</v>
+      </c>
+      <c r="M648" t="n">
+        <v>101</v>
+      </c>
+      <c r="N648" t="n">
+        <v>0</v>
+      </c>
+      <c r="O648" t="n">
+        <v>0</v>
+      </c>
+      <c r="P648" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>card_648</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Chris Buck and Jennifer Lee</t>
+        </is>
+      </c>
+      <c r="D649" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E649" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F649" t="n">
+        <v>74</v>
+      </c>
+      <c r="I649" t="n">
+        <v>1280000000</v>
+      </c>
+      <c r="J649" t="b">
+        <v>0</v>
+      </c>
+      <c r="K649" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L649" t="b">
+        <v>0</v>
+      </c>
+      <c r="M649" t="n">
+        <v>102</v>
+      </c>
+      <c r="N649" t="n">
+        <v>2</v>
+      </c>
+      <c r="O649" t="n">
+        <v>0</v>
+      </c>
+      <c r="P649" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Big Hero 6</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>card_649</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Don Hall and Chris Williams</t>
+        </is>
+      </c>
+      <c r="D650" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E650" t="n">
+        <v>3.86</v>
+      </c>
+      <c r="F650" t="n">
+        <v>78</v>
+      </c>
+      <c r="I650" t="n">
+        <v>657800000</v>
+      </c>
+      <c r="J650" t="b">
+        <v>0</v>
+      </c>
+      <c r="K650" t="n">
+        <v>165000000</v>
+      </c>
+      <c r="L650" t="b">
+        <v>0</v>
+      </c>
+      <c r="M650" t="n">
+        <v>102</v>
+      </c>
+      <c r="N650" t="n">
+        <v>1</v>
+      </c>
+      <c r="O650" t="n">
+        <v>0</v>
+      </c>
+      <c r="P650" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Disney animated canon, part 3c: 2016-2023 (card_650-656)
Moana through Wish. This completes the Disney animated canon since
1960 (Sword in the Stone through Wish), 43 films added across 6
batches. Live-action Disney is far too vast to enumerate exhaustively
and was out of scope for this pass.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P650"/>
+  <dimension ref="A1:P657"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -33895,252 +33895,602 @@
       </c>
     </row>
     <row r="646">
-      <c r="A646" t="inlineStr">
+      <c r="A646" s="10" t="inlineStr">
         <is>
           <t>Tangled</t>
         </is>
       </c>
-      <c r="B646" t="inlineStr">
+      <c r="B646" s="10" t="inlineStr">
         <is>
           <t>card_645</t>
         </is>
       </c>
-      <c r="C646" t="inlineStr">
+      <c r="C646" s="10" t="inlineStr">
         <is>
           <t>Nathan Greno and Byron Howard</t>
         </is>
       </c>
-      <c r="D646" t="n">
+      <c r="D646" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E646" t="n">
+      <c r="E646" s="10" t="n">
         <v>4.07</v>
       </c>
-      <c r="F646" t="n">
+      <c r="F646" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I646" t="n">
+      <c r="I646" s="10" t="n">
         <v>592500000</v>
       </c>
-      <c r="J646" t="b">
-        <v>0</v>
-      </c>
-      <c r="K646" t="n">
+      <c r="J646" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K646" s="10" t="n">
         <v>260000000</v>
       </c>
-      <c r="L646" t="b">
-        <v>0</v>
-      </c>
-      <c r="M646" t="n">
+      <c r="L646" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M646" s="10" t="n">
         <v>100</v>
       </c>
-      <c r="N646" t="n">
-        <v>0</v>
-      </c>
-      <c r="O646" t="n">
-        <v>0</v>
-      </c>
-      <c r="P646" t="b">
+      <c r="N646" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O646" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P646" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="647">
-      <c r="A647" t="inlineStr">
+      <c r="A647" s="10" t="inlineStr">
         <is>
           <t>Winnie the Pooh</t>
         </is>
       </c>
-      <c r="B647" t="inlineStr">
+      <c r="B647" s="10" t="inlineStr">
         <is>
           <t>card_646</t>
         </is>
       </c>
-      <c r="C647" t="inlineStr">
+      <c r="C647" s="10" t="inlineStr">
         <is>
           <t>Stephen Anderson and Don Hall</t>
         </is>
       </c>
-      <c r="D647" t="n">
+      <c r="D647" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E647" t="n">
+      <c r="E647" s="10" t="n">
         <v>3.69</v>
       </c>
-      <c r="F647" t="n">
+      <c r="F647" s="10" t="n">
         <v>76</v>
       </c>
-      <c r="I647" t="n">
+      <c r="I647" s="10" t="n">
         <v>50100000</v>
       </c>
-      <c r="J647" t="b">
-        <v>0</v>
-      </c>
-      <c r="K647" t="n">
+      <c r="J647" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K647" s="10" t="n">
         <v>30000000</v>
       </c>
-      <c r="L647" t="b">
-        <v>0</v>
-      </c>
-      <c r="M647" t="n">
+      <c r="L647" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M647" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="N647" t="n">
-        <v>0</v>
-      </c>
-      <c r="O647" t="n">
-        <v>0</v>
-      </c>
-      <c r="P647" t="b">
+      <c r="N647" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O647" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P647" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="648">
-      <c r="A648" t="inlineStr">
+      <c r="A648" s="10" t="inlineStr">
         <is>
           <t>Wreck-It Ralph</t>
         </is>
       </c>
-      <c r="B648" t="inlineStr">
+      <c r="B648" s="10" t="inlineStr">
         <is>
           <t>card_647</t>
         </is>
       </c>
-      <c r="C648" t="inlineStr">
+      <c r="C648" s="10" t="inlineStr">
         <is>
           <t>Rich Moore</t>
         </is>
       </c>
-      <c r="D648" t="n">
+      <c r="D648" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E648" t="n">
+      <c r="E648" s="10" t="n">
         <v>3.62</v>
       </c>
-      <c r="F648" t="n">
+      <c r="F648" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I648" t="n">
+      <c r="I648" s="10" t="n">
         <v>496500000</v>
       </c>
-      <c r="J648" t="b">
-        <v>0</v>
-      </c>
-      <c r="K648" t="n">
+      <c r="J648" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K648" s="10" t="n">
         <v>165000000</v>
       </c>
-      <c r="L648" t="b">
-        <v>0</v>
-      </c>
-      <c r="M648" t="n">
+      <c r="L648" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M648" s="10" t="n">
         <v>101</v>
       </c>
-      <c r="N648" t="n">
-        <v>0</v>
-      </c>
-      <c r="O648" t="n">
-        <v>0</v>
-      </c>
-      <c r="P648" t="b">
+      <c r="N648" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O648" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P648" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="649">
-      <c r="A649" t="inlineStr">
+      <c r="A649" s="10" t="inlineStr">
         <is>
           <t>Frozen</t>
         </is>
       </c>
-      <c r="B649" t="inlineStr">
+      <c r="B649" s="10" t="inlineStr">
         <is>
           <t>card_648</t>
         </is>
       </c>
-      <c r="C649" t="inlineStr">
+      <c r="C649" s="10" t="inlineStr">
         <is>
           <t>Chris Buck and Jennifer Lee</t>
         </is>
       </c>
-      <c r="D649" t="n">
+      <c r="D649" s="10" t="n">
         <v>2013</v>
       </c>
-      <c r="E649" t="n">
+      <c r="E649" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F649" t="n">
+      <c r="F649" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I649" t="n">
+      <c r="I649" s="10" t="n">
         <v>1280000000</v>
       </c>
-      <c r="J649" t="b">
-        <v>0</v>
-      </c>
-      <c r="K649" t="n">
+      <c r="J649" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K649" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L649" t="b">
-        <v>0</v>
-      </c>
-      <c r="M649" t="n">
+      <c r="L649" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M649" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="N649" t="n">
+      <c r="N649" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="O649" t="n">
-        <v>0</v>
-      </c>
-      <c r="P649" t="b">
+      <c r="O649" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P649" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="650">
-      <c r="A650" t="inlineStr">
+      <c r="A650" s="10" t="inlineStr">
         <is>
           <t>Big Hero 6</t>
         </is>
       </c>
-      <c r="B650" t="inlineStr">
+      <c r="B650" s="10" t="inlineStr">
         <is>
           <t>card_649</t>
         </is>
       </c>
-      <c r="C650" t="inlineStr">
+      <c r="C650" s="10" t="inlineStr">
         <is>
           <t>Don Hall and Chris Williams</t>
         </is>
       </c>
-      <c r="D650" t="n">
+      <c r="D650" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E650" t="n">
+      <c r="E650" s="10" t="n">
         <v>3.86</v>
       </c>
-      <c r="F650" t="n">
+      <c r="F650" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I650" t="n">
+      <c r="I650" s="10" t="n">
         <v>657800000</v>
       </c>
-      <c r="J650" t="b">
-        <v>0</v>
-      </c>
-      <c r="K650" t="n">
+      <c r="J650" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K650" s="10" t="n">
         <v>165000000</v>
       </c>
-      <c r="L650" t="b">
-        <v>0</v>
-      </c>
-      <c r="M650" t="n">
+      <c r="L650" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M650" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="N650" t="n">
+      <c r="N650" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O650" t="n">
-        <v>0</v>
-      </c>
-      <c r="P650" t="b">
+      <c r="O650" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P650" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Moana</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>card_650</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>John Musker and Ron Clements</t>
+        </is>
+      </c>
+      <c r="D651" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E651" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="F651" t="n">
+        <v>78</v>
+      </c>
+      <c r="I651" t="n">
+        <v>687200000</v>
+      </c>
+      <c r="J651" t="b">
+        <v>0</v>
+      </c>
+      <c r="K651" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L651" t="b">
+        <v>0</v>
+      </c>
+      <c r="M651" t="n">
+        <v>113</v>
+      </c>
+      <c r="N651" t="n">
+        <v>0</v>
+      </c>
+      <c r="O651" t="n">
+        <v>0</v>
+      </c>
+      <c r="P651" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Ralph Breaks the Internet</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>card_651</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Rich Moore and Phil Johnston</t>
+        </is>
+      </c>
+      <c r="D652" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E652" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F652" t="n">
+        <v>63</v>
+      </c>
+      <c r="I652" t="n">
+        <v>529300000</v>
+      </c>
+      <c r="J652" t="b">
+        <v>0</v>
+      </c>
+      <c r="K652" t="n">
+        <v>175000000</v>
+      </c>
+      <c r="L652" t="b">
+        <v>0</v>
+      </c>
+      <c r="M652" t="n">
+        <v>112</v>
+      </c>
+      <c r="N652" t="n">
+        <v>0</v>
+      </c>
+      <c r="O652" t="n">
+        <v>0</v>
+      </c>
+      <c r="P652" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Frozen II</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>card_652</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Chris Buck and Jennifer Lee</t>
+        </is>
+      </c>
+      <c r="D653" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E653" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="F653" t="n">
+        <v>67</v>
+      </c>
+      <c r="I653" t="n">
+        <v>1453000000</v>
+      </c>
+      <c r="J653" t="b">
+        <v>0</v>
+      </c>
+      <c r="K653" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L653" t="b">
+        <v>0</v>
+      </c>
+      <c r="M653" t="n">
+        <v>103</v>
+      </c>
+      <c r="N653" t="n">
+        <v>0</v>
+      </c>
+      <c r="O653" t="n">
+        <v>0</v>
+      </c>
+      <c r="P653" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Raya and the Last Dragon</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>card_653</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Don Hall and Carlos Lopez Estrada</t>
+        </is>
+      </c>
+      <c r="D654" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E654" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="F654" t="n">
+        <v>68</v>
+      </c>
+      <c r="I654" t="n">
+        <v>130400000</v>
+      </c>
+      <c r="J654" t="b">
+        <v>0</v>
+      </c>
+      <c r="K654" t="n">
+        <v>100000000</v>
+      </c>
+      <c r="L654" t="b">
+        <v>0</v>
+      </c>
+      <c r="M654" t="n">
+        <v>107</v>
+      </c>
+      <c r="N654" t="n">
+        <v>0</v>
+      </c>
+      <c r="O654" t="n">
+        <v>0</v>
+      </c>
+      <c r="P654" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Encanto</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>card_654</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Jared Bush and Byron Howard</t>
+        </is>
+      </c>
+      <c r="D655" t="n">
+        <v>2021</v>
+      </c>
+      <c r="E655" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="F655" t="n">
+        <v>40</v>
+      </c>
+      <c r="I655" t="n">
+        <v>261300000</v>
+      </c>
+      <c r="J655" t="b">
+        <v>0</v>
+      </c>
+      <c r="K655" t="n">
+        <v>120000000</v>
+      </c>
+      <c r="L655" t="b">
+        <v>0</v>
+      </c>
+      <c r="M655" t="n">
+        <v>102</v>
+      </c>
+      <c r="N655" t="n">
+        <v>1</v>
+      </c>
+      <c r="O655" t="n">
+        <v>0</v>
+      </c>
+      <c r="P655" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Strange World</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>card_655</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Don Hall</t>
+        </is>
+      </c>
+      <c r="D656" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E656" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="F656" t="n">
+        <v>35</v>
+      </c>
+      <c r="I656" t="n">
+        <v>73600000</v>
+      </c>
+      <c r="J656" t="b">
+        <v>0</v>
+      </c>
+      <c r="K656" t="n">
+        <v>180000000</v>
+      </c>
+      <c r="L656" t="b">
+        <v>0</v>
+      </c>
+      <c r="M656" t="n">
+        <v>102</v>
+      </c>
+      <c r="N656" t="n">
+        <v>0</v>
+      </c>
+      <c r="O656" t="n">
+        <v>0</v>
+      </c>
+      <c r="P656" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Wish</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>card_656</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Chris Buck and Fawn Veerasunthorn</t>
+        </is>
+      </c>
+      <c r="D657" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E657" t="n">
+        <v>2.26</v>
+      </c>
+      <c r="F657" t="n">
+        <v>40</v>
+      </c>
+      <c r="I657" t="n">
+        <v>255000000</v>
+      </c>
+      <c r="J657" t="b">
+        <v>0</v>
+      </c>
+      <c r="K657" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L657" t="b">
+        <v>0</v>
+      </c>
+      <c r="M657" t="n">
+        <v>95</v>
+      </c>
+      <c r="N657" t="n">
+        <v>0</v>
+      </c>
+      <c r="O657" t="n">
+        <v>0</v>
+      </c>
+      <c r="P657" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add all Bleach movies (card_657-660)
Memories of Nobody, The DiamondDust Rebellion, Fade to Black, Hell
Verse -- all 4 theatrical Bleach films. Budget/box office are rough
USD conversions of the JPY figures Wikipedia reports (Japan-only
grosses; no exact worldwide totals are documented for these).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P657"/>
+  <dimension ref="A1:P661"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -34145,352 +34145,540 @@
       </c>
     </row>
     <row r="651">
-      <c r="A651" t="inlineStr">
+      <c r="A651" s="10" t="inlineStr">
         <is>
           <t>Moana</t>
         </is>
       </c>
-      <c r="B651" t="inlineStr">
+      <c r="B651" s="10" t="inlineStr">
         <is>
           <t>card_650</t>
         </is>
       </c>
-      <c r="C651" t="inlineStr">
+      <c r="C651" s="10" t="inlineStr">
         <is>
           <t>John Musker and Ron Clements</t>
         </is>
       </c>
-      <c r="D651" t="n">
+      <c r="D651" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E651" t="n">
+      <c r="E651" s="10" t="n">
         <v>3.72</v>
       </c>
-      <c r="F651" t="n">
+      <c r="F651" s="10" t="n">
         <v>78</v>
       </c>
-      <c r="I651" t="n">
+      <c r="I651" s="10" t="n">
         <v>687200000</v>
       </c>
-      <c r="J651" t="b">
-        <v>0</v>
-      </c>
-      <c r="K651" t="n">
+      <c r="J651" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K651" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L651" t="b">
-        <v>0</v>
-      </c>
-      <c r="M651" t="n">
+      <c r="L651" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M651" s="10" t="n">
         <v>113</v>
       </c>
-      <c r="N651" t="n">
-        <v>0</v>
-      </c>
-      <c r="O651" t="n">
-        <v>0</v>
-      </c>
-      <c r="P651" t="b">
+      <c r="N651" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O651" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P651" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="652">
-      <c r="A652" t="inlineStr">
+      <c r="A652" s="10" t="inlineStr">
         <is>
           <t>Ralph Breaks the Internet</t>
         </is>
       </c>
-      <c r="B652" t="inlineStr">
+      <c r="B652" s="10" t="inlineStr">
         <is>
           <t>card_651</t>
         </is>
       </c>
-      <c r="C652" t="inlineStr">
+      <c r="C652" s="10" t="inlineStr">
         <is>
           <t>Rich Moore and Phil Johnston</t>
         </is>
       </c>
-      <c r="D652" t="n">
+      <c r="D652" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E652" t="n">
+      <c r="E652" s="10" t="n">
         <v>2.9</v>
       </c>
-      <c r="F652" t="n">
+      <c r="F652" s="10" t="n">
         <v>63</v>
       </c>
-      <c r="I652" t="n">
+      <c r="I652" s="10" t="n">
         <v>529300000</v>
       </c>
-      <c r="J652" t="b">
-        <v>0</v>
-      </c>
-      <c r="K652" t="n">
+      <c r="J652" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K652" s="10" t="n">
         <v>175000000</v>
       </c>
-      <c r="L652" t="b">
-        <v>0</v>
-      </c>
-      <c r="M652" t="n">
+      <c r="L652" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M652" s="10" t="n">
         <v>112</v>
       </c>
-      <c r="N652" t="n">
-        <v>0</v>
-      </c>
-      <c r="O652" t="n">
-        <v>0</v>
-      </c>
-      <c r="P652" t="b">
+      <c r="N652" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O652" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P652" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="653">
-      <c r="A653" t="inlineStr">
+      <c r="A653" s="10" t="inlineStr">
         <is>
           <t>Frozen II</t>
         </is>
       </c>
-      <c r="B653" t="inlineStr">
+      <c r="B653" s="10" t="inlineStr">
         <is>
           <t>card_652</t>
         </is>
       </c>
-      <c r="C653" t="inlineStr">
+      <c r="C653" s="10" t="inlineStr">
         <is>
           <t>Chris Buck and Jennifer Lee</t>
         </is>
       </c>
-      <c r="D653" t="n">
+      <c r="D653" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E653" t="n">
+      <c r="E653" s="10" t="n">
         <v>3.45</v>
       </c>
-      <c r="F653" t="n">
+      <c r="F653" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="I653" t="n">
+      <c r="I653" s="10" t="n">
         <v>1453000000</v>
       </c>
-      <c r="J653" t="b">
-        <v>0</v>
-      </c>
-      <c r="K653" t="n">
+      <c r="J653" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K653" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L653" t="b">
-        <v>0</v>
-      </c>
-      <c r="M653" t="n">
+      <c r="L653" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M653" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="N653" t="n">
-        <v>0</v>
-      </c>
-      <c r="O653" t="n">
-        <v>0</v>
-      </c>
-      <c r="P653" t="b">
+      <c r="N653" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O653" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P653" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="654">
-      <c r="A654" t="inlineStr">
+      <c r="A654" s="10" t="inlineStr">
         <is>
           <t>Raya and the Last Dragon</t>
         </is>
       </c>
-      <c r="B654" t="inlineStr">
+      <c r="B654" s="10" t="inlineStr">
         <is>
           <t>card_653</t>
         </is>
       </c>
-      <c r="C654" t="inlineStr">
+      <c r="C654" s="10" t="inlineStr">
         <is>
           <t>Don Hall and Carlos Lopez Estrada</t>
         </is>
       </c>
-      <c r="D654" t="n">
+      <c r="D654" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E654" t="n">
+      <c r="E654" s="10" t="n">
         <v>3.2</v>
       </c>
-      <c r="F654" t="n">
+      <c r="F654" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="I654" t="n">
+      <c r="I654" s="10" t="n">
         <v>130400000</v>
       </c>
-      <c r="J654" t="b">
-        <v>0</v>
-      </c>
-      <c r="K654" t="n">
+      <c r="J654" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K654" s="10" t="n">
         <v>100000000</v>
       </c>
-      <c r="L654" t="b">
-        <v>0</v>
-      </c>
-      <c r="M654" t="n">
+      <c r="L654" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M654" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N654" t="n">
-        <v>0</v>
-      </c>
-      <c r="O654" t="n">
-        <v>0</v>
-      </c>
-      <c r="P654" t="b">
+      <c r="N654" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O654" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P654" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="655">
-      <c r="A655" t="inlineStr">
+      <c r="A655" s="10" t="inlineStr">
         <is>
           <t>Encanto</t>
         </is>
       </c>
-      <c r="B655" t="inlineStr">
+      <c r="B655" s="10" t="inlineStr">
         <is>
           <t>card_654</t>
         </is>
       </c>
-      <c r="C655" t="inlineStr">
+      <c r="C655" s="10" t="inlineStr">
         <is>
           <t>Jared Bush and Byron Howard</t>
         </is>
       </c>
-      <c r="D655" t="n">
+      <c r="D655" s="10" t="n">
         <v>2021</v>
       </c>
-      <c r="E655" t="n">
+      <c r="E655" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="F655" t="n">
+      <c r="F655" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="I655" t="n">
+      <c r="I655" s="10" t="n">
         <v>261300000</v>
       </c>
-      <c r="J655" t="b">
-        <v>0</v>
-      </c>
-      <c r="K655" t="n">
+      <c r="J655" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K655" s="10" t="n">
         <v>120000000</v>
       </c>
-      <c r="L655" t="b">
-        <v>0</v>
-      </c>
-      <c r="M655" t="n">
+      <c r="L655" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M655" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="N655" t="n">
+      <c r="N655" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O655" t="n">
-        <v>0</v>
-      </c>
-      <c r="P655" t="b">
+      <c r="O655" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P655" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="656">
-      <c r="A656" t="inlineStr">
+      <c r="A656" s="10" t="inlineStr">
         <is>
           <t>Strange World</t>
         </is>
       </c>
-      <c r="B656" t="inlineStr">
+      <c r="B656" s="10" t="inlineStr">
         <is>
           <t>card_655</t>
         </is>
       </c>
-      <c r="C656" t="inlineStr">
+      <c r="C656" s="10" t="inlineStr">
         <is>
           <t>Don Hall</t>
         </is>
       </c>
-      <c r="D656" t="n">
+      <c r="D656" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E656" t="n">
+      <c r="E656" s="10" t="n">
         <v>3.19</v>
       </c>
-      <c r="F656" t="n">
+      <c r="F656" s="10" t="n">
         <v>35</v>
       </c>
-      <c r="I656" t="n">
+      <c r="I656" s="10" t="n">
         <v>73600000</v>
       </c>
-      <c r="J656" t="b">
-        <v>0</v>
-      </c>
-      <c r="K656" t="n">
+      <c r="J656" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K656" s="10" t="n">
         <v>180000000</v>
       </c>
-      <c r="L656" t="b">
-        <v>0</v>
-      </c>
-      <c r="M656" t="n">
+      <c r="L656" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M656" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="N656" t="n">
-        <v>0</v>
-      </c>
-      <c r="O656" t="n">
-        <v>0</v>
-      </c>
-      <c r="P656" t="b">
+      <c r="N656" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O656" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P656" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="657">
-      <c r="A657" t="inlineStr">
+      <c r="A657" s="10" t="inlineStr">
         <is>
           <t>Wish</t>
         </is>
       </c>
-      <c r="B657" t="inlineStr">
+      <c r="B657" s="10" t="inlineStr">
         <is>
           <t>card_656</t>
         </is>
       </c>
-      <c r="C657" t="inlineStr">
+      <c r="C657" s="10" t="inlineStr">
         <is>
           <t>Chris Buck and Fawn Veerasunthorn</t>
         </is>
       </c>
-      <c r="D657" t="n">
+      <c r="D657" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E657" t="n">
+      <c r="E657" s="10" t="n">
         <v>2.26</v>
       </c>
-      <c r="F657" t="n">
+      <c r="F657" s="10" t="n">
         <v>40</v>
       </c>
-      <c r="I657" t="n">
+      <c r="I657" s="10" t="n">
         <v>255000000</v>
       </c>
-      <c r="J657" t="b">
-        <v>0</v>
-      </c>
-      <c r="K657" t="n">
+      <c r="J657" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K657" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L657" t="b">
-        <v>0</v>
-      </c>
-      <c r="M657" t="n">
+      <c r="L657" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M657" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N657" t="n">
-        <v>0</v>
-      </c>
-      <c r="O657" t="n">
-        <v>0</v>
-      </c>
-      <c r="P657" t="b">
+      <c r="N657" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O657" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P657" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Bleach the Movie: Memories of Nobody</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>card_657</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Noriyuki Abe</t>
+        </is>
+      </c>
+      <c r="D658" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E658" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="I658" t="n">
+        <v>5700000</v>
+      </c>
+      <c r="J658" t="b">
+        <v>1</v>
+      </c>
+      <c r="K658" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L658" t="b">
+        <v>1</v>
+      </c>
+      <c r="M658" t="n">
+        <v>93</v>
+      </c>
+      <c r="N658" t="n">
+        <v>0</v>
+      </c>
+      <c r="O658" t="n">
+        <v>0</v>
+      </c>
+      <c r="P658" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Bleach the Movie: The DiamondDust Rebellion</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>card_658</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Noriyuki Abe</t>
+        </is>
+      </c>
+      <c r="D659" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E659" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="I659" t="n">
+        <v>6800000</v>
+      </c>
+      <c r="J659" t="b">
+        <v>1</v>
+      </c>
+      <c r="K659" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L659" t="b">
+        <v>1</v>
+      </c>
+      <c r="M659" t="n">
+        <v>95</v>
+      </c>
+      <c r="N659" t="n">
+        <v>0</v>
+      </c>
+      <c r="O659" t="n">
+        <v>0</v>
+      </c>
+      <c r="P659" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Bleach the Movie: Fade to Black</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>card_659</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Noriyuki Abe</t>
+        </is>
+      </c>
+      <c r="D660" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E660" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="I660" t="n">
+        <v>6800000</v>
+      </c>
+      <c r="J660" t="b">
+        <v>1</v>
+      </c>
+      <c r="K660" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L660" t="b">
+        <v>1</v>
+      </c>
+      <c r="M660" t="n">
+        <v>95</v>
+      </c>
+      <c r="N660" t="n">
+        <v>0</v>
+      </c>
+      <c r="O660" t="n">
+        <v>0</v>
+      </c>
+      <c r="P660" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Bleach the Movie: Hell Verse</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>card_660</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Noriyuki Abe</t>
+        </is>
+      </c>
+      <c r="D661" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E661" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="I661" t="n">
+        <v>7000000</v>
+      </c>
+      <c r="J661" t="b">
+        <v>1</v>
+      </c>
+      <c r="K661" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L661" t="b">
+        <v>1</v>
+      </c>
+      <c r="M661" t="n">
+        <v>94</v>
+      </c>
+      <c r="N661" t="n">
+        <v>0</v>
+      </c>
+      <c r="O661" t="n">
+        <v>0</v>
+      </c>
+      <c r="P661" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add all Naruto movies (card_661-671)
All 11 theatrical films: Ninja Clash in the Land of Snow through
Boruto: Naruto the Movie. Several directors' birth years aren't
documented anywhere (Toshiyuki Tsuru, Masahiko Murata, Hiroyuki
Yamashita) so those cards' director_age_at_release stays null.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P661"/>
+  <dimension ref="A1:P672"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -34495,190 +34495,707 @@
       </c>
     </row>
     <row r="658">
-      <c r="A658" t="inlineStr">
+      <c r="A658" s="10" t="inlineStr">
         <is>
           <t>Bleach the Movie: Memories of Nobody</t>
         </is>
       </c>
-      <c r="B658" t="inlineStr">
+      <c r="B658" s="10" t="inlineStr">
         <is>
           <t>card_657</t>
         </is>
       </c>
-      <c r="C658" t="inlineStr">
+      <c r="C658" s="10" t="inlineStr">
         <is>
           <t>Noriyuki Abe</t>
         </is>
       </c>
-      <c r="D658" t="n">
+      <c r="D658" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E658" t="n">
+      <c r="E658" s="10" t="n">
         <v>3.35</v>
       </c>
-      <c r="I658" t="n">
+      <c r="I658" s="10" t="n">
         <v>5700000</v>
       </c>
-      <c r="J658" t="b">
+      <c r="J658" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K658" t="n">
+      <c r="K658" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L658" t="b">
+      <c r="L658" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M658" t="n">
+      <c r="M658" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N658" t="n">
-        <v>0</v>
-      </c>
-      <c r="O658" t="n">
-        <v>0</v>
-      </c>
-      <c r="P658" t="b">
+      <c r="N658" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O658" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P658" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="659">
-      <c r="A659" t="inlineStr">
+      <c r="A659" s="10" t="inlineStr">
         <is>
           <t>Bleach the Movie: The DiamondDust Rebellion</t>
         </is>
       </c>
-      <c r="B659" t="inlineStr">
+      <c r="B659" s="10" t="inlineStr">
         <is>
           <t>card_658</t>
         </is>
       </c>
-      <c r="C659" t="inlineStr">
+      <c r="C659" s="10" t="inlineStr">
         <is>
           <t>Noriyuki Abe</t>
         </is>
       </c>
-      <c r="D659" t="n">
+      <c r="D659" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E659" t="n">
+      <c r="E659" s="10" t="n">
         <v>3.21</v>
       </c>
-      <c r="I659" t="n">
+      <c r="I659" s="10" t="n">
         <v>6800000</v>
       </c>
-      <c r="J659" t="b">
+      <c r="J659" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K659" t="n">
+      <c r="K659" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L659" t="b">
+      <c r="L659" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M659" t="n">
+      <c r="M659" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N659" t="n">
-        <v>0</v>
-      </c>
-      <c r="O659" t="n">
-        <v>0</v>
-      </c>
-      <c r="P659" t="b">
+      <c r="N659" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O659" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P659" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="660">
-      <c r="A660" t="inlineStr">
+      <c r="A660" s="10" t="inlineStr">
         <is>
           <t>Bleach the Movie: Fade to Black</t>
         </is>
       </c>
-      <c r="B660" t="inlineStr">
+      <c r="B660" s="10" t="inlineStr">
         <is>
           <t>card_659</t>
         </is>
       </c>
-      <c r="C660" t="inlineStr">
+      <c r="C660" s="10" t="inlineStr">
         <is>
           <t>Noriyuki Abe</t>
         </is>
       </c>
-      <c r="D660" t="n">
+      <c r="D660" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E660" t="n">
+      <c r="E660" s="10" t="n">
         <v>3.31</v>
       </c>
-      <c r="I660" t="n">
+      <c r="I660" s="10" t="n">
         <v>6800000</v>
       </c>
-      <c r="J660" t="b">
+      <c r="J660" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K660" t="n">
+      <c r="K660" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L660" t="b">
+      <c r="L660" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M660" t="n">
+      <c r="M660" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N660" t="n">
-        <v>0</v>
-      </c>
-      <c r="O660" t="n">
-        <v>0</v>
-      </c>
-      <c r="P660" t="b">
+      <c r="N660" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O660" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P660" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="661">
-      <c r="A661" t="inlineStr">
+      <c r="A661" s="10" t="inlineStr">
         <is>
           <t>Bleach the Movie: Hell Verse</t>
         </is>
       </c>
-      <c r="B661" t="inlineStr">
+      <c r="B661" s="10" t="inlineStr">
         <is>
           <t>card_660</t>
         </is>
       </c>
-      <c r="C661" t="inlineStr">
+      <c r="C661" s="10" t="inlineStr">
         <is>
           <t>Noriyuki Abe</t>
         </is>
       </c>
-      <c r="D661" t="n">
+      <c r="D661" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E661" t="n">
+      <c r="E661" s="10" t="n">
         <v>3.43</v>
       </c>
-      <c r="I661" t="n">
+      <c r="I661" s="10" t="n">
         <v>7000000</v>
       </c>
-      <c r="J661" t="b">
+      <c r="J661" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K661" t="n">
+      <c r="K661" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L661" t="b">
+      <c r="L661" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M661" t="n">
+      <c r="M661" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="N661" t="n">
-        <v>0</v>
-      </c>
-      <c r="O661" t="n">
-        <v>0</v>
-      </c>
-      <c r="P661" t="b">
+      <c r="N661" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O661" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P661" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Naruto the Movie: Ninja Clash in the Land of Snow</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>card_661</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>Tensai Okamura</t>
+        </is>
+      </c>
+      <c r="D662" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E662" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="I662" t="n">
+        <v>11100000</v>
+      </c>
+      <c r="J662" t="b">
+        <v>1</v>
+      </c>
+      <c r="K662" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L662" t="b">
+        <v>1</v>
+      </c>
+      <c r="M662" t="n">
+        <v>82</v>
+      </c>
+      <c r="N662" t="n">
+        <v>0</v>
+      </c>
+      <c r="O662" t="n">
+        <v>0</v>
+      </c>
+      <c r="P662" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Naruto the Movie 2: Legend of the Stone of Gelel</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>card_662</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Hirotsugu Kawasaki</t>
+        </is>
+      </c>
+      <c r="D663" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E663" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="I663" t="n">
+        <v>10200000</v>
+      </c>
+      <c r="J663" t="b">
+        <v>0</v>
+      </c>
+      <c r="K663" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L663" t="b">
+        <v>1</v>
+      </c>
+      <c r="M663" t="n">
+        <v>97</v>
+      </c>
+      <c r="N663" t="n">
+        <v>0</v>
+      </c>
+      <c r="O663" t="n">
+        <v>0</v>
+      </c>
+      <c r="P663" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Naruto the Movie 3: Guardians of the Crescent Moon Kingdom</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>card_663</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>Toshiyuki Tsuru</t>
+        </is>
+      </c>
+      <c r="D664" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E664" t="n">
+        <v>2.96</v>
+      </c>
+      <c r="I664" t="n">
+        <v>3224005</v>
+      </c>
+      <c r="J664" t="b">
+        <v>0</v>
+      </c>
+      <c r="K664" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L664" t="b">
+        <v>1</v>
+      </c>
+      <c r="M664" t="n">
+        <v>95</v>
+      </c>
+      <c r="N664" t="n">
+        <v>0</v>
+      </c>
+      <c r="O664" t="n">
+        <v>0</v>
+      </c>
+      <c r="P664" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Naruto Shippuden the Movie</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>card_664</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Hajime Kamegaki</t>
+        </is>
+      </c>
+      <c r="D665" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E665" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="I665" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="J665" t="b">
+        <v>0</v>
+      </c>
+      <c r="K665" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L665" t="b">
+        <v>1</v>
+      </c>
+      <c r="M665" t="n">
+        <v>95</v>
+      </c>
+      <c r="N665" t="n">
+        <v>0</v>
+      </c>
+      <c r="O665" t="n">
+        <v>0</v>
+      </c>
+      <c r="P665" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Naruto Shippuden the Movie: Bonds</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>card_665</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Hajime Kamegaki</t>
+        </is>
+      </c>
+      <c r="D666" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E666" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="I666" t="n">
+        <v>10600000</v>
+      </c>
+      <c r="J666" t="b">
+        <v>0</v>
+      </c>
+      <c r="K666" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L666" t="b">
+        <v>1</v>
+      </c>
+      <c r="M666" t="n">
+        <v>93</v>
+      </c>
+      <c r="N666" t="n">
+        <v>0</v>
+      </c>
+      <c r="O666" t="n">
+        <v>0</v>
+      </c>
+      <c r="P666" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Naruto Shippuden the Movie: The Will of Fire</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>card_666</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>Masahiko Murata</t>
+        </is>
+      </c>
+      <c r="D667" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E667" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="I667" t="n">
+        <v>8100000</v>
+      </c>
+      <c r="J667" t="b">
+        <v>0</v>
+      </c>
+      <c r="K667" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L667" t="b">
+        <v>1</v>
+      </c>
+      <c r="M667" t="n">
+        <v>96</v>
+      </c>
+      <c r="N667" t="n">
+        <v>0</v>
+      </c>
+      <c r="O667" t="n">
+        <v>0</v>
+      </c>
+      <c r="P667" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Naruto Shippuden the Movie: The Lost Tower</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>card_667</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Masahiko Murata</t>
+        </is>
+      </c>
+      <c r="D668" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E668" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="I668" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="J668" t="b">
+        <v>0</v>
+      </c>
+      <c r="K668" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L668" t="b">
+        <v>1</v>
+      </c>
+      <c r="M668" t="n">
+        <v>85</v>
+      </c>
+      <c r="N668" t="n">
+        <v>0</v>
+      </c>
+      <c r="O668" t="n">
+        <v>0</v>
+      </c>
+      <c r="P668" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Naruto Shippuden the Movie: Blood Prison</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>card_668</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Masahiko Murata</t>
+        </is>
+      </c>
+      <c r="D669" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E669" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="I669" t="n">
+        <v>9100000</v>
+      </c>
+      <c r="J669" t="b">
+        <v>0</v>
+      </c>
+      <c r="K669" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="L669" t="b">
+        <v>1</v>
+      </c>
+      <c r="M669" t="n">
+        <v>103</v>
+      </c>
+      <c r="N669" t="n">
+        <v>0</v>
+      </c>
+      <c r="O669" t="n">
+        <v>0</v>
+      </c>
+      <c r="P669" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Road to Ninja: Naruto the Movie</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>card_669</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Hayato Date</t>
+        </is>
+      </c>
+      <c r="D670" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E670" t="n">
+        <v>3.49</v>
+      </c>
+      <c r="I670" t="n">
+        <v>17900000</v>
+      </c>
+      <c r="J670" t="b">
+        <v>0</v>
+      </c>
+      <c r="K670" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L670" t="b">
+        <v>1</v>
+      </c>
+      <c r="M670" t="n">
+        <v>109</v>
+      </c>
+      <c r="N670" t="n">
+        <v>0</v>
+      </c>
+      <c r="O670" t="n">
+        <v>0</v>
+      </c>
+      <c r="P670" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>The Last: Naruto the Movie</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>card_670</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Tsuneo Kobayashi</t>
+        </is>
+      </c>
+      <c r="D671" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E671" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="I671" t="n">
+        <v>19840000</v>
+      </c>
+      <c r="J671" t="b">
+        <v>0</v>
+      </c>
+      <c r="K671" t="n">
+        <v>1010000</v>
+      </c>
+      <c r="L671" t="b">
+        <v>0</v>
+      </c>
+      <c r="M671" t="n">
+        <v>112</v>
+      </c>
+      <c r="N671" t="n">
+        <v>0</v>
+      </c>
+      <c r="O671" t="n">
+        <v>0</v>
+      </c>
+      <c r="P671" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Boruto: Naruto the Movie</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>card_671</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Hiroyuki Yamashita</t>
+        </is>
+      </c>
+      <c r="D672" t="n">
+        <v>2015</v>
+      </c>
+      <c r="E672" t="n">
+        <v>3.22</v>
+      </c>
+      <c r="I672" t="n">
+        <v>38500000</v>
+      </c>
+      <c r="J672" t="b">
+        <v>0</v>
+      </c>
+      <c r="K672" t="n">
+        <v>21000000</v>
+      </c>
+      <c r="L672" t="b">
+        <v>0</v>
+      </c>
+      <c r="M672" t="n">
+        <v>96</v>
+      </c>
+      <c r="N672" t="n">
+        <v>0</v>
+      </c>
+      <c r="O672" t="n">
+        <v>0</v>
+      </c>
+      <c r="P672" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add all core One Piece theatrical films (card_672-683)
12 films: One Piece: The Movie (2000) through One Piece Film: Red
(2022) -- covers the full mainline theatrical series. (Two 2007-2008
specials, Episode of Alabasta and Episode of Chopper Plus, were
TV-special-style releases rather than true theatrical films and are
excluded.) This completes the Bleach/One Piece/Naruto pass: all 4
Bleach films, all 11 Naruto films, and the 12 core One Piece films are
now in the database. Box office for the pre-2009 films is a USD
conversion of Wikipedia's JPY Japan-box-office figures using period
exchange rates (no separate worldwide totals are documented for these);
several directors' birth years aren't documented anywhere and are left
null.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P672"/>
+  <dimension ref="A1:P684"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -34683,519 +34683,1083 @@
       </c>
     </row>
     <row r="662">
-      <c r="A662" t="inlineStr">
+      <c r="A662" s="10" t="inlineStr">
         <is>
           <t>Naruto the Movie: Ninja Clash in the Land of Snow</t>
         </is>
       </c>
-      <c r="B662" t="inlineStr">
+      <c r="B662" s="10" t="inlineStr">
         <is>
           <t>card_661</t>
         </is>
       </c>
-      <c r="C662" t="inlineStr">
+      <c r="C662" s="10" t="inlineStr">
         <is>
           <t>Tensai Okamura</t>
         </is>
       </c>
-      <c r="D662" t="n">
+      <c r="D662" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E662" t="n">
+      <c r="E662" s="10" t="n">
         <v>3.13</v>
       </c>
-      <c r="I662" t="n">
+      <c r="I662" s="10" t="n">
         <v>11100000</v>
       </c>
-      <c r="J662" t="b">
+      <c r="J662" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K662" t="n">
+      <c r="K662" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L662" t="b">
+      <c r="L662" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M662" t="n">
+      <c r="M662" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="N662" t="n">
-        <v>0</v>
-      </c>
-      <c r="O662" t="n">
-        <v>0</v>
-      </c>
-      <c r="P662" t="b">
+      <c r="N662" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O662" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P662" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="663">
-      <c r="A663" t="inlineStr">
+      <c r="A663" s="10" t="inlineStr">
         <is>
           <t>Naruto the Movie 2: Legend of the Stone of Gelel</t>
         </is>
       </c>
-      <c r="B663" t="inlineStr">
+      <c r="B663" s="10" t="inlineStr">
         <is>
           <t>card_662</t>
         </is>
       </c>
-      <c r="C663" t="inlineStr">
+      <c r="C663" s="10" t="inlineStr">
         <is>
           <t>Hirotsugu Kawasaki</t>
         </is>
       </c>
-      <c r="D663" t="n">
+      <c r="D663" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E663" t="n">
+      <c r="E663" s="10" t="n">
         <v>2.81</v>
       </c>
-      <c r="I663" t="n">
+      <c r="I663" s="10" t="n">
         <v>10200000</v>
       </c>
-      <c r="J663" t="b">
-        <v>0</v>
-      </c>
-      <c r="K663" t="n">
+      <c r="J663" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K663" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L663" t="b">
+      <c r="L663" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M663" t="n">
+      <c r="M663" s="10" t="n">
         <v>97</v>
       </c>
-      <c r="N663" t="n">
-        <v>0</v>
-      </c>
-      <c r="O663" t="n">
-        <v>0</v>
-      </c>
-      <c r="P663" t="b">
+      <c r="N663" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O663" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P663" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="664">
-      <c r="A664" t="inlineStr">
+      <c r="A664" s="10" t="inlineStr">
         <is>
           <t>Naruto the Movie 3: Guardians of the Crescent Moon Kingdom</t>
         </is>
       </c>
-      <c r="B664" t="inlineStr">
+      <c r="B664" s="10" t="inlineStr">
         <is>
           <t>card_663</t>
         </is>
       </c>
-      <c r="C664" t="inlineStr">
+      <c r="C664" s="10" t="inlineStr">
         <is>
           <t>Toshiyuki Tsuru</t>
         </is>
       </c>
-      <c r="D664" t="n">
+      <c r="D664" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E664" t="n">
+      <c r="E664" s="10" t="n">
         <v>2.96</v>
       </c>
-      <c r="I664" t="n">
+      <c r="I664" s="10" t="n">
         <v>3224005</v>
       </c>
-      <c r="J664" t="b">
-        <v>0</v>
-      </c>
-      <c r="K664" t="n">
+      <c r="J664" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K664" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L664" t="b">
+      <c r="L664" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M664" t="n">
+      <c r="M664" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N664" t="n">
-        <v>0</v>
-      </c>
-      <c r="O664" t="n">
-        <v>0</v>
-      </c>
-      <c r="P664" t="b">
+      <c r="N664" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O664" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P664" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="665">
-      <c r="A665" t="inlineStr">
+      <c r="A665" s="10" t="inlineStr">
         <is>
           <t>Naruto Shippuden the Movie</t>
         </is>
       </c>
-      <c r="B665" t="inlineStr">
+      <c r="B665" s="10" t="inlineStr">
         <is>
           <t>card_664</t>
         </is>
       </c>
-      <c r="C665" t="inlineStr">
+      <c r="C665" s="10" t="inlineStr">
         <is>
           <t>Hajime Kamegaki</t>
         </is>
       </c>
-      <c r="D665" t="n">
+      <c r="D665" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E665" t="n">
+      <c r="E665" s="10" t="n">
         <v>3.25</v>
       </c>
-      <c r="I665" t="n">
+      <c r="I665" s="10" t="n">
         <v>10000000</v>
       </c>
-      <c r="J665" t="b">
-        <v>0</v>
-      </c>
-      <c r="K665" t="n">
+      <c r="J665" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K665" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L665" t="b">
+      <c r="L665" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M665" t="n">
+      <c r="M665" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N665" t="n">
-        <v>0</v>
-      </c>
-      <c r="O665" t="n">
-        <v>0</v>
-      </c>
-      <c r="P665" t="b">
+      <c r="N665" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O665" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P665" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="666">
-      <c r="A666" t="inlineStr">
+      <c r="A666" s="10" t="inlineStr">
         <is>
           <t>Naruto Shippuden the Movie: Bonds</t>
         </is>
       </c>
-      <c r="B666" t="inlineStr">
+      <c r="B666" s="10" t="inlineStr">
         <is>
           <t>card_665</t>
         </is>
       </c>
-      <c r="C666" t="inlineStr">
+      <c r="C666" s="10" t="inlineStr">
         <is>
           <t>Hajime Kamegaki</t>
         </is>
       </c>
-      <c r="D666" t="n">
+      <c r="D666" s="10" t="n">
         <v>2008</v>
       </c>
-      <c r="E666" t="n">
+      <c r="E666" s="10" t="n">
         <v>3.11</v>
       </c>
-      <c r="I666" t="n">
+      <c r="I666" s="10" t="n">
         <v>10600000</v>
       </c>
-      <c r="J666" t="b">
-        <v>0</v>
-      </c>
-      <c r="K666" t="n">
+      <c r="J666" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K666" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L666" t="b">
+      <c r="L666" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M666" t="n">
+      <c r="M666" s="10" t="n">
         <v>93</v>
       </c>
-      <c r="N666" t="n">
-        <v>0</v>
-      </c>
-      <c r="O666" t="n">
-        <v>0</v>
-      </c>
-      <c r="P666" t="b">
+      <c r="N666" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O666" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P666" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="667">
-      <c r="A667" t="inlineStr">
+      <c r="A667" s="10" t="inlineStr">
         <is>
           <t>Naruto Shippuden the Movie: The Will of Fire</t>
         </is>
       </c>
-      <c r="B667" t="inlineStr">
+      <c r="B667" s="10" t="inlineStr">
         <is>
           <t>card_666</t>
         </is>
       </c>
-      <c r="C667" t="inlineStr">
+      <c r="C667" s="10" t="inlineStr">
         <is>
           <t>Masahiko Murata</t>
         </is>
       </c>
-      <c r="D667" t="n">
+      <c r="D667" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E667" t="n">
+      <c r="E667" s="10" t="n">
         <v>3.19</v>
       </c>
-      <c r="I667" t="n">
+      <c r="I667" s="10" t="n">
         <v>8100000</v>
       </c>
-      <c r="J667" t="b">
-        <v>0</v>
-      </c>
-      <c r="K667" t="n">
+      <c r="J667" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K667" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L667" t="b">
+      <c r="L667" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M667" t="n">
+      <c r="M667" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N667" t="n">
-        <v>0</v>
-      </c>
-      <c r="O667" t="n">
-        <v>0</v>
-      </c>
-      <c r="P667" t="b">
+      <c r="N667" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O667" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P667" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="668">
-      <c r="A668" t="inlineStr">
+      <c r="A668" s="10" t="inlineStr">
         <is>
           <t>Naruto Shippuden the Movie: The Lost Tower</t>
         </is>
       </c>
-      <c r="B668" t="inlineStr">
+      <c r="B668" s="10" t="inlineStr">
         <is>
           <t>card_667</t>
         </is>
       </c>
-      <c r="C668" t="inlineStr">
+      <c r="C668" s="10" t="inlineStr">
         <is>
           <t>Masahiko Murata</t>
         </is>
       </c>
-      <c r="D668" t="n">
+      <c r="D668" s="10" t="n">
         <v>2010</v>
       </c>
-      <c r="E668" t="n">
+      <c r="E668" s="10" t="n">
         <v>3.09</v>
       </c>
-      <c r="I668" t="n">
+      <c r="I668" s="10" t="n">
         <v>8500000</v>
       </c>
-      <c r="J668" t="b">
-        <v>0</v>
-      </c>
-      <c r="K668" t="n">
+      <c r="J668" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K668" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L668" t="b">
+      <c r="L668" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M668" t="n">
+      <c r="M668" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="N668" t="n">
-        <v>0</v>
-      </c>
-      <c r="O668" t="n">
-        <v>0</v>
-      </c>
-      <c r="P668" t="b">
+      <c r="N668" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O668" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P668" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="669">
-      <c r="A669" t="inlineStr">
+      <c r="A669" s="10" t="inlineStr">
         <is>
           <t>Naruto Shippuden the Movie: Blood Prison</t>
         </is>
       </c>
-      <c r="B669" t="inlineStr">
+      <c r="B669" s="10" t="inlineStr">
         <is>
           <t>card_668</t>
         </is>
       </c>
-      <c r="C669" t="inlineStr">
+      <c r="C669" s="10" t="inlineStr">
         <is>
           <t>Masahiko Murata</t>
         </is>
       </c>
-      <c r="D669" t="n">
+      <c r="D669" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E669" t="n">
+      <c r="E669" s="10" t="n">
         <v>3.19</v>
       </c>
-      <c r="I669" t="n">
+      <c r="I669" s="10" t="n">
         <v>9100000</v>
       </c>
-      <c r="J669" t="b">
-        <v>0</v>
-      </c>
-      <c r="K669" t="n">
+      <c r="J669" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K669" s="10" t="n">
         <v>4500000</v>
       </c>
-      <c r="L669" t="b">
+      <c r="L669" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M669" t="n">
+      <c r="M669" s="10" t="n">
         <v>103</v>
       </c>
-      <c r="N669" t="n">
-        <v>0</v>
-      </c>
-      <c r="O669" t="n">
-        <v>0</v>
-      </c>
-      <c r="P669" t="b">
+      <c r="N669" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O669" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P669" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="670">
-      <c r="A670" t="inlineStr">
+      <c r="A670" s="10" t="inlineStr">
         <is>
           <t>Road to Ninja: Naruto the Movie</t>
         </is>
       </c>
-      <c r="B670" t="inlineStr">
+      <c r="B670" s="10" t="inlineStr">
         <is>
           <t>card_669</t>
         </is>
       </c>
-      <c r="C670" t="inlineStr">
+      <c r="C670" s="10" t="inlineStr">
         <is>
           <t>Hayato Date</t>
         </is>
       </c>
-      <c r="D670" t="n">
+      <c r="D670" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E670" t="n">
+      <c r="E670" s="10" t="n">
         <v>3.49</v>
       </c>
-      <c r="I670" t="n">
+      <c r="I670" s="10" t="n">
         <v>17900000</v>
       </c>
-      <c r="J670" t="b">
-        <v>0</v>
-      </c>
-      <c r="K670" t="n">
+      <c r="J670" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K670" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L670" t="b">
+      <c r="L670" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M670" t="n">
+      <c r="M670" s="10" t="n">
         <v>109</v>
       </c>
-      <c r="N670" t="n">
-        <v>0</v>
-      </c>
-      <c r="O670" t="n">
-        <v>0</v>
-      </c>
-      <c r="P670" t="b">
+      <c r="N670" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O670" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P670" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="671">
-      <c r="A671" t="inlineStr">
+      <c r="A671" s="10" t="inlineStr">
         <is>
           <t>The Last: Naruto the Movie</t>
         </is>
       </c>
-      <c r="B671" t="inlineStr">
+      <c r="B671" s="10" t="inlineStr">
         <is>
           <t>card_670</t>
         </is>
       </c>
-      <c r="C671" t="inlineStr">
+      <c r="C671" s="10" t="inlineStr">
         <is>
           <t>Tsuneo Kobayashi</t>
         </is>
       </c>
-      <c r="D671" t="n">
+      <c r="D671" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E671" t="n">
+      <c r="E671" s="10" t="n">
         <v>3.54</v>
       </c>
-      <c r="I671" t="n">
+      <c r="I671" s="10" t="n">
         <v>19840000</v>
       </c>
-      <c r="J671" t="b">
-        <v>0</v>
-      </c>
-      <c r="K671" t="n">
+      <c r="J671" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K671" s="10" t="n">
         <v>1010000</v>
       </c>
-      <c r="L671" t="b">
-        <v>0</v>
-      </c>
-      <c r="M671" t="n">
+      <c r="L671" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M671" s="10" t="n">
         <v>112</v>
       </c>
-      <c r="N671" t="n">
-        <v>0</v>
-      </c>
-      <c r="O671" t="n">
-        <v>0</v>
-      </c>
-      <c r="P671" t="b">
+      <c r="N671" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O671" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P671" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="672">
-      <c r="A672" t="inlineStr">
+      <c r="A672" s="10" t="inlineStr">
         <is>
           <t>Boruto: Naruto the Movie</t>
         </is>
       </c>
-      <c r="B672" t="inlineStr">
+      <c r="B672" s="10" t="inlineStr">
         <is>
           <t>card_671</t>
         </is>
       </c>
-      <c r="C672" t="inlineStr">
+      <c r="C672" s="10" t="inlineStr">
         <is>
           <t>Hiroyuki Yamashita</t>
         </is>
       </c>
-      <c r="D672" t="n">
+      <c r="D672" s="10" t="n">
         <v>2015</v>
       </c>
-      <c r="E672" t="n">
+      <c r="E672" s="10" t="n">
         <v>3.22</v>
       </c>
-      <c r="I672" t="n">
+      <c r="I672" s="10" t="n">
         <v>38500000</v>
       </c>
-      <c r="J672" t="b">
-        <v>0</v>
-      </c>
-      <c r="K672" t="n">
+      <c r="J672" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K672" s="10" t="n">
         <v>21000000</v>
       </c>
-      <c r="L672" t="b">
-        <v>0</v>
-      </c>
-      <c r="M672" t="n">
+      <c r="L672" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M672" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="N672" t="n">
-        <v>0</v>
-      </c>
-      <c r="O672" t="n">
-        <v>0</v>
-      </c>
-      <c r="P672" t="b">
+      <c r="N672" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O672" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P672" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>One Piece: The Movie</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>card_672</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Junji Shimizu</t>
+        </is>
+      </c>
+      <c r="D673" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E673" t="n">
+        <v>3.31</v>
+      </c>
+      <c r="I673" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="J673" t="b">
+        <v>1</v>
+      </c>
+      <c r="K673" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L673" t="b">
+        <v>1</v>
+      </c>
+      <c r="M673" t="n">
+        <v>51</v>
+      </c>
+      <c r="N673" t="n">
+        <v>0</v>
+      </c>
+      <c r="O673" t="n">
+        <v>0</v>
+      </c>
+      <c r="P673" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>One Piece: Clockwork Island Adventure</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>card_673</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Junji Shimizu</t>
+        </is>
+      </c>
+      <c r="D674" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E674" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="I674" t="n">
+        <v>24800000</v>
+      </c>
+      <c r="J674" t="b">
+        <v>1</v>
+      </c>
+      <c r="K674" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L674" t="b">
+        <v>1</v>
+      </c>
+      <c r="M674" t="n">
+        <v>60</v>
+      </c>
+      <c r="N674" t="n">
+        <v>0</v>
+      </c>
+      <c r="O674" t="n">
+        <v>0</v>
+      </c>
+      <c r="P674" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>One Piece: Chopper's Kingdom on the Island of Strange Animals</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>card_674</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Junji Shimizu</t>
+        </is>
+      </c>
+      <c r="D675" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E675" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="I675" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="J675" t="b">
+        <v>1</v>
+      </c>
+      <c r="K675" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="L675" t="b">
+        <v>1</v>
+      </c>
+      <c r="M675" t="n">
+        <v>56</v>
+      </c>
+      <c r="N675" t="n">
+        <v>0</v>
+      </c>
+      <c r="O675" t="n">
+        <v>0</v>
+      </c>
+      <c r="P675" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>One Piece: Dead End Adventure</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>card_675</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Konosuke Uda</t>
+        </is>
+      </c>
+      <c r="D676" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E676" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="I676" t="n">
+        <v>17200000</v>
+      </c>
+      <c r="J676" t="b">
+        <v>1</v>
+      </c>
+      <c r="K676" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="L676" t="b">
+        <v>1</v>
+      </c>
+      <c r="M676" t="n">
+        <v>95</v>
+      </c>
+      <c r="N676" t="n">
+        <v>0</v>
+      </c>
+      <c r="O676" t="n">
+        <v>0</v>
+      </c>
+      <c r="P676" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>One Piece: The Cursed Holy Sword</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>card_676</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Kazuhisa Takenouchi</t>
+        </is>
+      </c>
+      <c r="D677" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E677" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="I677" t="n">
+        <v>16700000</v>
+      </c>
+      <c r="J677" t="b">
+        <v>1</v>
+      </c>
+      <c r="K677" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="L677" t="b">
+        <v>1</v>
+      </c>
+      <c r="M677" t="n">
+        <v>95</v>
+      </c>
+      <c r="N677" t="n">
+        <v>0</v>
+      </c>
+      <c r="O677" t="n">
+        <v>0</v>
+      </c>
+      <c r="P677" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>One Piece: Baron Omatsuri and the Secret Island</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>card_677</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Mamoru Hosoda</t>
+        </is>
+      </c>
+      <c r="D678" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E678" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="I678" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="J678" t="b">
+        <v>0</v>
+      </c>
+      <c r="K678" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="L678" t="b">
+        <v>1</v>
+      </c>
+      <c r="M678" t="n">
+        <v>91</v>
+      </c>
+      <c r="N678" t="n">
+        <v>0</v>
+      </c>
+      <c r="O678" t="n">
+        <v>0</v>
+      </c>
+      <c r="P678" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>One Piece: The Giant Mechanical Soldier of Karakuri Castle</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>card_678</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Konosuke Uda</t>
+        </is>
+      </c>
+      <c r="D679" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E679" t="n">
+        <v>2.87</v>
+      </c>
+      <c r="I679" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="J679" t="b">
+        <v>1</v>
+      </c>
+      <c r="K679" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="L679" t="b">
+        <v>1</v>
+      </c>
+      <c r="M679" t="n">
+        <v>94</v>
+      </c>
+      <c r="N679" t="n">
+        <v>0</v>
+      </c>
+      <c r="O679" t="n">
+        <v>0</v>
+      </c>
+      <c r="P679" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>One Piece Film: Strong World</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>card_679</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Munehisa Sakai</t>
+        </is>
+      </c>
+      <c r="D680" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E680" t="n">
+        <v>3.56</v>
+      </c>
+      <c r="I680" t="n">
+        <v>61200000</v>
+      </c>
+      <c r="J680" t="b">
+        <v>0</v>
+      </c>
+      <c r="K680" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L680" t="b">
+        <v>1</v>
+      </c>
+      <c r="M680" t="n">
+        <v>115</v>
+      </c>
+      <c r="N680" t="n">
+        <v>1</v>
+      </c>
+      <c r="O680" t="n">
+        <v>0</v>
+      </c>
+      <c r="P680" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>One Piece Film: Z</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>card_680</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Tatsuya Nagamine</t>
+        </is>
+      </c>
+      <c r="D681" t="n">
+        <v>2012</v>
+      </c>
+      <c r="E681" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="I681" t="n">
+        <v>85000000</v>
+      </c>
+      <c r="J681" t="b">
+        <v>0</v>
+      </c>
+      <c r="K681" t="n">
+        <v>16000000</v>
+      </c>
+      <c r="L681" t="b">
+        <v>1</v>
+      </c>
+      <c r="M681" t="n">
+        <v>107</v>
+      </c>
+      <c r="N681" t="n">
+        <v>0</v>
+      </c>
+      <c r="O681" t="n">
+        <v>0</v>
+      </c>
+      <c r="P681" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>One Piece Film: Gold</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>card_681</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Hiroaki Miyamoto</t>
+        </is>
+      </c>
+      <c r="D682" t="n">
+        <v>2016</v>
+      </c>
+      <c r="E682" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I682" t="n">
+        <v>70800000</v>
+      </c>
+      <c r="J682" t="b">
+        <v>0</v>
+      </c>
+      <c r="K682" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="L682" t="b">
+        <v>1</v>
+      </c>
+      <c r="M682" t="n">
+        <v>120</v>
+      </c>
+      <c r="N682" t="n">
+        <v>0</v>
+      </c>
+      <c r="O682" t="n">
+        <v>0</v>
+      </c>
+      <c r="P682" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>One Piece: Stampede</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>card_682</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Takashi Otsuka</t>
+        </is>
+      </c>
+      <c r="D683" t="n">
+        <v>2019</v>
+      </c>
+      <c r="E683" t="n">
+        <v>3.58</v>
+      </c>
+      <c r="I683" t="n">
+        <v>94700000</v>
+      </c>
+      <c r="J683" t="b">
+        <v>0</v>
+      </c>
+      <c r="K683" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L683" t="b">
+        <v>1</v>
+      </c>
+      <c r="M683" t="n">
+        <v>120</v>
+      </c>
+      <c r="N683" t="n">
+        <v>0</v>
+      </c>
+      <c r="O683" t="n">
+        <v>0</v>
+      </c>
+      <c r="P683" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>One Piece Film: Red</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>card_683</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Goro Taniguchi</t>
+        </is>
+      </c>
+      <c r="D684" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E684" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="I684" t="n">
+        <v>246500000</v>
+      </c>
+      <c r="J684" t="b">
+        <v>0</v>
+      </c>
+      <c r="K684" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L684" t="b">
+        <v>1</v>
+      </c>
+      <c r="M684" t="n">
+        <v>115</v>
+      </c>
+      <c r="N684" t="n">
+        <v>0</v>
+      </c>
+      <c r="O684" t="n">
+        <v>0</v>
+      </c>
+      <c r="P684" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the Avatar trilogy (card_684-686)
Avatar, The Way of Water, Fire and Ash (2025) -- all three James
Cameron films now in the DB.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P684"/>
+  <dimension ref="A1:P687"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -35200,566 +35200,716 @@
       </c>
     </row>
     <row r="673">
-      <c r="A673" t="inlineStr">
+      <c r="A673" s="10" t="inlineStr">
         <is>
           <t>One Piece: The Movie</t>
         </is>
       </c>
-      <c r="B673" t="inlineStr">
+      <c r="B673" s="10" t="inlineStr">
         <is>
           <t>card_672</t>
         </is>
       </c>
-      <c r="C673" t="inlineStr">
+      <c r="C673" s="10" t="inlineStr">
         <is>
           <t>Junji Shimizu</t>
         </is>
       </c>
-      <c r="D673" t="n">
+      <c r="D673" s="10" t="n">
         <v>2000</v>
       </c>
-      <c r="E673" t="n">
+      <c r="E673" s="10" t="n">
         <v>3.31</v>
       </c>
-      <c r="I673" t="n">
+      <c r="I673" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="J673" t="b">
+      <c r="J673" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K673" t="n">
+      <c r="K673" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L673" t="b">
+      <c r="L673" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M673" t="n">
+      <c r="M673" s="10" t="n">
         <v>51</v>
       </c>
-      <c r="N673" t="n">
-        <v>0</v>
-      </c>
-      <c r="O673" t="n">
-        <v>0</v>
-      </c>
-      <c r="P673" t="b">
+      <c r="N673" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O673" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P673" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="674">
-      <c r="A674" t="inlineStr">
+      <c r="A674" s="10" t="inlineStr">
         <is>
           <t>One Piece: Clockwork Island Adventure</t>
         </is>
       </c>
-      <c r="B674" t="inlineStr">
+      <c r="B674" s="10" t="inlineStr">
         <is>
           <t>card_673</t>
         </is>
       </c>
-      <c r="C674" t="inlineStr">
+      <c r="C674" s="10" t="inlineStr">
         <is>
           <t>Junji Shimizu</t>
         </is>
       </c>
-      <c r="D674" t="n">
+      <c r="D674" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E674" t="n">
+      <c r="E674" s="10" t="n">
         <v>3.08</v>
       </c>
-      <c r="I674" t="n">
+      <c r="I674" s="10" t="n">
         <v>24800000</v>
       </c>
-      <c r="J674" t="b">
+      <c r="J674" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K674" t="n">
+      <c r="K674" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L674" t="b">
+      <c r="L674" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M674" t="n">
+      <c r="M674" s="10" t="n">
         <v>60</v>
       </c>
-      <c r="N674" t="n">
-        <v>0</v>
-      </c>
-      <c r="O674" t="n">
-        <v>0</v>
-      </c>
-      <c r="P674" t="b">
+      <c r="N674" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O674" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P674" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="675">
-      <c r="A675" t="inlineStr">
+      <c r="A675" s="10" t="inlineStr">
         <is>
           <t>One Piece: Chopper's Kingdom on the Island of Strange Animals</t>
         </is>
       </c>
-      <c r="B675" t="inlineStr">
+      <c r="B675" s="10" t="inlineStr">
         <is>
           <t>card_674</t>
         </is>
       </c>
-      <c r="C675" t="inlineStr">
+      <c r="C675" s="10" t="inlineStr">
         <is>
           <t>Junji Shimizu</t>
         </is>
       </c>
-      <c r="D675" t="n">
+      <c r="D675" s="10" t="n">
         <v>2002</v>
       </c>
-      <c r="E675" t="n">
+      <c r="E675" s="10" t="n">
         <v>2.82</v>
       </c>
-      <c r="I675" t="n">
+      <c r="I675" s="10" t="n">
         <v>16000000</v>
       </c>
-      <c r="J675" t="b">
+      <c r="J675" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K675" t="n">
+      <c r="K675" s="10" t="n">
         <v>5000000</v>
       </c>
-      <c r="L675" t="b">
+      <c r="L675" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M675" t="n">
+      <c r="M675" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="N675" t="n">
-        <v>0</v>
-      </c>
-      <c r="O675" t="n">
-        <v>0</v>
-      </c>
-      <c r="P675" t="b">
+      <c r="N675" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O675" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P675" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="676">
-      <c r="A676" t="inlineStr">
+      <c r="A676" s="10" t="inlineStr">
         <is>
           <t>One Piece: Dead End Adventure</t>
         </is>
       </c>
-      <c r="B676" t="inlineStr">
+      <c r="B676" s="10" t="inlineStr">
         <is>
           <t>card_675</t>
         </is>
       </c>
-      <c r="C676" t="inlineStr">
+      <c r="C676" s="10" t="inlineStr">
         <is>
           <t>Konosuke Uda</t>
         </is>
       </c>
-      <c r="D676" t="n">
+      <c r="D676" s="10" t="n">
         <v>2003</v>
       </c>
-      <c r="E676" t="n">
+      <c r="E676" s="10" t="n">
         <v>3.36</v>
       </c>
-      <c r="I676" t="n">
+      <c r="I676" s="10" t="n">
         <v>17200000</v>
       </c>
-      <c r="J676" t="b">
+      <c r="J676" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K676" t="n">
+      <c r="K676" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="L676" t="b">
+      <c r="L676" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M676" t="n">
+      <c r="M676" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N676" t="n">
-        <v>0</v>
-      </c>
-      <c r="O676" t="n">
-        <v>0</v>
-      </c>
-      <c r="P676" t="b">
+      <c r="N676" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O676" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P676" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="677">
-      <c r="A677" t="inlineStr">
+      <c r="A677" s="10" t="inlineStr">
         <is>
           <t>One Piece: The Cursed Holy Sword</t>
         </is>
       </c>
-      <c r="B677" t="inlineStr">
+      <c r="B677" s="10" t="inlineStr">
         <is>
           <t>card_676</t>
         </is>
       </c>
-      <c r="C677" t="inlineStr">
+      <c r="C677" s="10" t="inlineStr">
         <is>
           <t>Kazuhisa Takenouchi</t>
         </is>
       </c>
-      <c r="D677" t="n">
+      <c r="D677" s="10" t="n">
         <v>2004</v>
       </c>
-      <c r="E677" t="n">
+      <c r="E677" s="10" t="n">
         <v>2.9</v>
       </c>
-      <c r="I677" t="n">
+      <c r="I677" s="10" t="n">
         <v>16700000</v>
       </c>
-      <c r="J677" t="b">
+      <c r="J677" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K677" t="n">
+      <c r="K677" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="L677" t="b">
+      <c r="L677" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M677" t="n">
+      <c r="M677" s="10" t="n">
         <v>95</v>
       </c>
-      <c r="N677" t="n">
-        <v>0</v>
-      </c>
-      <c r="O677" t="n">
-        <v>0</v>
-      </c>
-      <c r="P677" t="b">
+      <c r="N677" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O677" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P677" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="678">
-      <c r="A678" t="inlineStr">
+      <c r="A678" s="10" t="inlineStr">
         <is>
           <t>One Piece: Baron Omatsuri and the Secret Island</t>
         </is>
       </c>
-      <c r="B678" t="inlineStr">
+      <c r="B678" s="10" t="inlineStr">
         <is>
           <t>card_677</t>
         </is>
       </c>
-      <c r="C678" t="inlineStr">
+      <c r="C678" s="10" t="inlineStr">
         <is>
           <t>Mamoru Hosoda</t>
         </is>
       </c>
-      <c r="D678" t="n">
+      <c r="D678" s="10" t="n">
         <v>2005</v>
       </c>
-      <c r="E678" t="n">
+      <c r="E678" s="10" t="n">
         <v>4.08</v>
       </c>
-      <c r="I678" t="n">
+      <c r="I678" s="10" t="n">
         <v>10500000</v>
       </c>
-      <c r="J678" t="b">
-        <v>0</v>
-      </c>
-      <c r="K678" t="n">
+      <c r="J678" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K678" s="10" t="n">
         <v>6000000</v>
       </c>
-      <c r="L678" t="b">
+      <c r="L678" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M678" t="n">
+      <c r="M678" s="10" t="n">
         <v>91</v>
       </c>
-      <c r="N678" t="n">
-        <v>0</v>
-      </c>
-      <c r="O678" t="n">
-        <v>0</v>
-      </c>
-      <c r="P678" t="b">
+      <c r="N678" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O678" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P678" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="679">
-      <c r="A679" t="inlineStr">
+      <c r="A679" s="10" t="inlineStr">
         <is>
           <t>One Piece: The Giant Mechanical Soldier of Karakuri Castle</t>
         </is>
       </c>
-      <c r="B679" t="inlineStr">
+      <c r="B679" s="10" t="inlineStr">
         <is>
           <t>card_678</t>
         </is>
       </c>
-      <c r="C679" t="inlineStr">
+      <c r="C679" s="10" t="inlineStr">
         <is>
           <t>Konosuke Uda</t>
         </is>
       </c>
-      <c r="D679" t="n">
+      <c r="D679" s="10" t="n">
         <v>2006</v>
       </c>
-      <c r="E679" t="n">
+      <c r="E679" s="10" t="n">
         <v>2.87</v>
       </c>
-      <c r="I679" t="n">
+      <c r="I679" s="10" t="n">
         <v>8500000</v>
       </c>
-      <c r="J679" t="b">
+      <c r="J679" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K679" t="n">
+      <c r="K679" s="10" t="n">
         <v>6500000</v>
       </c>
-      <c r="L679" t="b">
+      <c r="L679" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M679" t="n">
+      <c r="M679" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="N679" t="n">
-        <v>0</v>
-      </c>
-      <c r="O679" t="n">
-        <v>0</v>
-      </c>
-      <c r="P679" t="b">
+      <c r="N679" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O679" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P679" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="680">
-      <c r="A680" t="inlineStr">
+      <c r="A680" s="10" t="inlineStr">
         <is>
           <t>One Piece Film: Strong World</t>
         </is>
       </c>
-      <c r="B680" t="inlineStr">
+      <c r="B680" s="10" t="inlineStr">
         <is>
           <t>card_679</t>
         </is>
       </c>
-      <c r="C680" t="inlineStr">
+      <c r="C680" s="10" t="inlineStr">
         <is>
           <t>Munehisa Sakai</t>
         </is>
       </c>
-      <c r="D680" t="n">
+      <c r="D680" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E680" t="n">
+      <c r="E680" s="10" t="n">
         <v>3.56</v>
       </c>
-      <c r="I680" t="n">
+      <c r="I680" s="10" t="n">
         <v>61200000</v>
       </c>
-      <c r="J680" t="b">
-        <v>0</v>
-      </c>
-      <c r="K680" t="n">
+      <c r="J680" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K680" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L680" t="b">
+      <c r="L680" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M680" t="n">
+      <c r="M680" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N680" t="n">
+      <c r="N680" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O680" t="n">
-        <v>0</v>
-      </c>
-      <c r="P680" t="b">
+      <c r="O680" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P680" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="681">
-      <c r="A681" t="inlineStr">
+      <c r="A681" s="10" t="inlineStr">
         <is>
           <t>One Piece Film: Z</t>
         </is>
       </c>
-      <c r="B681" t="inlineStr">
+      <c r="B681" s="10" t="inlineStr">
         <is>
           <t>card_680</t>
         </is>
       </c>
-      <c r="C681" t="inlineStr">
+      <c r="C681" s="10" t="inlineStr">
         <is>
           <t>Tatsuya Nagamine</t>
         </is>
       </c>
-      <c r="D681" t="n">
+      <c r="D681" s="10" t="n">
         <v>2012</v>
       </c>
-      <c r="E681" t="n">
+      <c r="E681" s="10" t="n">
         <v>3.64</v>
       </c>
-      <c r="I681" t="n">
+      <c r="I681" s="10" t="n">
         <v>85000000</v>
       </c>
-      <c r="J681" t="b">
-        <v>0</v>
-      </c>
-      <c r="K681" t="n">
+      <c r="J681" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K681" s="10" t="n">
         <v>16000000</v>
       </c>
-      <c r="L681" t="b">
+      <c r="L681" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M681" t="n">
+      <c r="M681" s="10" t="n">
         <v>107</v>
       </c>
-      <c r="N681" t="n">
-        <v>0</v>
-      </c>
-      <c r="O681" t="n">
-        <v>0</v>
-      </c>
-      <c r="P681" t="b">
+      <c r="N681" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O681" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P681" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="682">
-      <c r="A682" t="inlineStr">
+      <c r="A682" s="10" t="inlineStr">
         <is>
           <t>One Piece Film: Gold</t>
         </is>
       </c>
-      <c r="B682" t="inlineStr">
+      <c r="B682" s="10" t="inlineStr">
         <is>
           <t>card_681</t>
         </is>
       </c>
-      <c r="C682" t="inlineStr">
+      <c r="C682" s="10" t="inlineStr">
         <is>
           <t>Hiroaki Miyamoto</t>
         </is>
       </c>
-      <c r="D682" t="n">
+      <c r="D682" s="10" t="n">
         <v>2016</v>
       </c>
-      <c r="E682" t="n">
+      <c r="E682" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="I682" t="n">
+      <c r="I682" s="10" t="n">
         <v>70800000</v>
       </c>
-      <c r="J682" t="b">
-        <v>0</v>
-      </c>
-      <c r="K682" t="n">
+      <c r="J682" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K682" s="10" t="n">
         <v>18000000</v>
       </c>
-      <c r="L682" t="b">
+      <c r="L682" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M682" t="n">
+      <c r="M682" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="N682" t="n">
-        <v>0</v>
-      </c>
-      <c r="O682" t="n">
-        <v>0</v>
-      </c>
-      <c r="P682" t="b">
+      <c r="N682" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O682" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P682" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="683">
-      <c r="A683" t="inlineStr">
+      <c r="A683" s="10" t="inlineStr">
         <is>
           <t>One Piece: Stampede</t>
         </is>
       </c>
-      <c r="B683" t="inlineStr">
+      <c r="B683" s="10" t="inlineStr">
         <is>
           <t>card_682</t>
         </is>
       </c>
-      <c r="C683" t="inlineStr">
+      <c r="C683" s="10" t="inlineStr">
         <is>
           <t>Takashi Otsuka</t>
         </is>
       </c>
-      <c r="D683" t="n">
+      <c r="D683" s="10" t="n">
         <v>2019</v>
       </c>
-      <c r="E683" t="n">
+      <c r="E683" s="10" t="n">
         <v>3.58</v>
       </c>
-      <c r="I683" t="n">
+      <c r="I683" s="10" t="n">
         <v>94700000</v>
       </c>
-      <c r="J683" t="b">
-        <v>0</v>
-      </c>
-      <c r="K683" t="n">
+      <c r="J683" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K683" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L683" t="b">
+      <c r="L683" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M683" t="n">
+      <c r="M683" s="10" t="n">
         <v>120</v>
       </c>
-      <c r="N683" t="n">
-        <v>0</v>
-      </c>
-      <c r="O683" t="n">
-        <v>0</v>
-      </c>
-      <c r="P683" t="b">
+      <c r="N683" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O683" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P683" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="684">
-      <c r="A684" t="inlineStr">
+      <c r="A684" s="10" t="inlineStr">
         <is>
           <t>One Piece Film: Red</t>
         </is>
       </c>
-      <c r="B684" t="inlineStr">
+      <c r="B684" s="10" t="inlineStr">
         <is>
           <t>card_683</t>
         </is>
       </c>
-      <c r="C684" t="inlineStr">
+      <c r="C684" s="10" t="inlineStr">
         <is>
           <t>Goro Taniguchi</t>
         </is>
       </c>
-      <c r="D684" t="n">
+      <c r="D684" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E684" t="n">
+      <c r="E684" s="10" t="n">
         <v>3.33</v>
       </c>
-      <c r="I684" t="n">
+      <c r="I684" s="10" t="n">
         <v>246500000</v>
       </c>
-      <c r="J684" t="b">
-        <v>0</v>
-      </c>
-      <c r="K684" t="n">
+      <c r="J684" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K684" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L684" t="b">
+      <c r="L684" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M684" t="n">
+      <c r="M684" s="10" t="n">
         <v>115</v>
       </c>
-      <c r="N684" t="n">
-        <v>0</v>
-      </c>
-      <c r="O684" t="n">
-        <v>0</v>
-      </c>
-      <c r="P684" t="b">
+      <c r="N684" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O684" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P684" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Avatar</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>card_684</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>James Cameron</t>
+        </is>
+      </c>
+      <c r="D685" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E685" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="F685" t="n">
+        <v>74</v>
+      </c>
+      <c r="I685" t="n">
+        <v>2924000000</v>
+      </c>
+      <c r="J685" t="b">
+        <v>0</v>
+      </c>
+      <c r="K685" t="n">
+        <v>237000000</v>
+      </c>
+      <c r="L685" t="b">
+        <v>0</v>
+      </c>
+      <c r="M685" t="n">
+        <v>162</v>
+      </c>
+      <c r="N685" t="n">
+        <v>3</v>
+      </c>
+      <c r="O685" t="n">
+        <v>0</v>
+      </c>
+      <c r="P685" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Avatar: The Way of Water</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>card_685</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>James Cameron</t>
+        </is>
+      </c>
+      <c r="D686" t="n">
+        <v>2022</v>
+      </c>
+      <c r="E686" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="F686" t="n">
+        <v>72</v>
+      </c>
+      <c r="I686" t="n">
+        <v>2334000000</v>
+      </c>
+      <c r="J686" t="b">
+        <v>0</v>
+      </c>
+      <c r="K686" t="n">
+        <v>400000000</v>
+      </c>
+      <c r="L686" t="b">
+        <v>0</v>
+      </c>
+      <c r="M686" t="n">
+        <v>192</v>
+      </c>
+      <c r="N686" t="n">
+        <v>1</v>
+      </c>
+      <c r="O686" t="n">
+        <v>0</v>
+      </c>
+      <c r="P686" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Avatar: Fire and Ash</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>card_686</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>James Cameron</t>
+        </is>
+      </c>
+      <c r="D687" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E687" t="n">
+        <v>3.55</v>
+      </c>
+      <c r="F687" t="n">
+        <v>69</v>
+      </c>
+      <c r="I687" t="n">
+        <v>1490000000</v>
+      </c>
+      <c r="J687" t="b">
+        <v>0</v>
+      </c>
+      <c r="K687" t="n">
+        <v>375000000</v>
+      </c>
+      <c r="L687" t="b">
+        <v>0</v>
+      </c>
+      <c r="M687" t="n">
+        <v>197</v>
+      </c>
+      <c r="N687" t="n">
+        <v>1</v>
+      </c>
+      <c r="O687" t="n">
+        <v>0</v>
+      </c>
+      <c r="P687" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Transformers series (card_687-693)
All 7 films: Transformers (2007) through Rise of the Beasts (2023),
including Bumblebee.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P687"/>
+  <dimension ref="A1:P694"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -35764,152 +35764,502 @@
       </c>
     </row>
     <row r="685">
-      <c r="A685" t="inlineStr">
+      <c r="A685" s="10" t="inlineStr">
         <is>
           <t>Avatar</t>
         </is>
       </c>
-      <c r="B685" t="inlineStr">
+      <c r="B685" s="10" t="inlineStr">
         <is>
           <t>card_684</t>
         </is>
       </c>
-      <c r="C685" t="inlineStr">
+      <c r="C685" s="10" t="inlineStr">
         <is>
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="D685" t="n">
+      <c r="D685" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E685" t="n">
+      <c r="E685" s="10" t="n">
         <v>3.77</v>
       </c>
-      <c r="F685" t="n">
+      <c r="F685" s="10" t="n">
         <v>74</v>
       </c>
-      <c r="I685" t="n">
+      <c r="I685" s="10" t="n">
         <v>2924000000</v>
       </c>
-      <c r="J685" t="b">
-        <v>0</v>
-      </c>
-      <c r="K685" t="n">
+      <c r="J685" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K685" s="10" t="n">
         <v>237000000</v>
       </c>
-      <c r="L685" t="b">
-        <v>0</v>
-      </c>
-      <c r="M685" t="n">
+      <c r="L685" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M685" s="10" t="n">
         <v>162</v>
       </c>
-      <c r="N685" t="n">
+      <c r="N685" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="O685" t="n">
-        <v>0</v>
-      </c>
-      <c r="P685" t="b">
+      <c r="O685" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P685" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="686">
-      <c r="A686" t="inlineStr">
+      <c r="A686" s="10" t="inlineStr">
         <is>
           <t>Avatar: The Way of Water</t>
         </is>
       </c>
-      <c r="B686" t="inlineStr">
+      <c r="B686" s="10" t="inlineStr">
         <is>
           <t>card_685</t>
         </is>
       </c>
-      <c r="C686" t="inlineStr">
+      <c r="C686" s="10" t="inlineStr">
         <is>
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="D686" t="n">
+      <c r="D686" s="10" t="n">
         <v>2022</v>
       </c>
-      <c r="E686" t="n">
+      <c r="E686" s="10" t="n">
         <v>3.65</v>
       </c>
-      <c r="F686" t="n">
+      <c r="F686" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="I686" t="n">
+      <c r="I686" s="10" t="n">
         <v>2334000000</v>
       </c>
-      <c r="J686" t="b">
-        <v>0</v>
-      </c>
-      <c r="K686" t="n">
+      <c r="J686" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K686" s="10" t="n">
         <v>400000000</v>
       </c>
-      <c r="L686" t="b">
-        <v>0</v>
-      </c>
-      <c r="M686" t="n">
+      <c r="L686" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M686" s="10" t="n">
         <v>192</v>
       </c>
-      <c r="N686" t="n">
+      <c r="N686" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O686" t="n">
-        <v>0</v>
-      </c>
-      <c r="P686" t="b">
+      <c r="O686" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P686" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="687">
-      <c r="A687" t="inlineStr">
+      <c r="A687" s="10" t="inlineStr">
         <is>
           <t>Avatar: Fire and Ash</t>
         </is>
       </c>
-      <c r="B687" t="inlineStr">
+      <c r="B687" s="10" t="inlineStr">
         <is>
           <t>card_686</t>
         </is>
       </c>
-      <c r="C687" t="inlineStr">
+      <c r="C687" s="10" t="inlineStr">
         <is>
           <t>James Cameron</t>
         </is>
       </c>
-      <c r="D687" t="n">
+      <c r="D687" s="10" t="n">
         <v>2025</v>
       </c>
-      <c r="E687" t="n">
+      <c r="E687" s="10" t="n">
         <v>3.55</v>
       </c>
-      <c r="F687" t="n">
+      <c r="F687" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I687" t="n">
+      <c r="I687" s="10" t="n">
         <v>1490000000</v>
       </c>
-      <c r="J687" t="b">
-        <v>0</v>
-      </c>
-      <c r="K687" t="n">
+      <c r="J687" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K687" s="10" t="n">
         <v>375000000</v>
       </c>
-      <c r="L687" t="b">
-        <v>0</v>
-      </c>
-      <c r="M687" t="n">
+      <c r="L687" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M687" s="10" t="n">
         <v>197</v>
       </c>
-      <c r="N687" t="n">
+      <c r="N687" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O687" t="n">
-        <v>0</v>
-      </c>
-      <c r="P687" t="b">
+      <c r="O687" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P687" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Transformers</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>card_687</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Michael Bay</t>
+        </is>
+      </c>
+      <c r="D688" t="n">
+        <v>2007</v>
+      </c>
+      <c r="E688" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F688" t="n">
+        <v>71</v>
+      </c>
+      <c r="I688" t="n">
+        <v>709700000</v>
+      </c>
+      <c r="J688" t="b">
+        <v>0</v>
+      </c>
+      <c r="K688" t="n">
+        <v>150000000</v>
+      </c>
+      <c r="L688" t="b">
+        <v>0</v>
+      </c>
+      <c r="M688" t="n">
+        <v>143</v>
+      </c>
+      <c r="N688" t="n">
+        <v>0</v>
+      </c>
+      <c r="O688" t="n">
+        <v>0</v>
+      </c>
+      <c r="P688" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Transformers: Revenge of the Fallen</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>card_688</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Michael Bay</t>
+        </is>
+      </c>
+      <c r="D689" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E689" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F689" t="n">
+        <v>50</v>
+      </c>
+      <c r="I689" t="n">
+        <v>836500000</v>
+      </c>
+      <c r="J689" t="b">
+        <v>0</v>
+      </c>
+      <c r="K689" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L689" t="b">
+        <v>0</v>
+      </c>
+      <c r="M689" t="n">
+        <v>150</v>
+      </c>
+      <c r="N689" t="n">
+        <v>0</v>
+      </c>
+      <c r="O689" t="n">
+        <v>0</v>
+      </c>
+      <c r="P689" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Transformers: Dark of the Moon</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>card_689</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Michael Bay</t>
+        </is>
+      </c>
+      <c r="D690" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E690" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="F690" t="n">
+        <v>59</v>
+      </c>
+      <c r="I690" t="n">
+        <v>1124000000</v>
+      </c>
+      <c r="J690" t="b">
+        <v>0</v>
+      </c>
+      <c r="K690" t="n">
+        <v>195000000</v>
+      </c>
+      <c r="L690" t="b">
+        <v>0</v>
+      </c>
+      <c r="M690" t="n">
+        <v>154</v>
+      </c>
+      <c r="N690" t="n">
+        <v>0</v>
+      </c>
+      <c r="O690" t="n">
+        <v>0</v>
+      </c>
+      <c r="P690" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Transformers: Age of Extinction</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>card_690</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Michael Bay</t>
+        </is>
+      </c>
+      <c r="D691" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E691" t="n">
+        <v>2.32</v>
+      </c>
+      <c r="F691" t="n">
+        <v>46</v>
+      </c>
+      <c r="I691" t="n">
+        <v>1105000000</v>
+      </c>
+      <c r="J691" t="b">
+        <v>0</v>
+      </c>
+      <c r="K691" t="n">
+        <v>210000000</v>
+      </c>
+      <c r="L691" t="b">
+        <v>0</v>
+      </c>
+      <c r="M691" t="n">
+        <v>165</v>
+      </c>
+      <c r="N691" t="n">
+        <v>0</v>
+      </c>
+      <c r="O691" t="n">
+        <v>0</v>
+      </c>
+      <c r="P691" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Transformers: The Last Knight</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>card_691</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Michael Bay</t>
+        </is>
+      </c>
+      <c r="D692" t="n">
+        <v>2017</v>
+      </c>
+      <c r="E692" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F692" t="n">
+        <v>41</v>
+      </c>
+      <c r="I692" t="n">
+        <v>605400000</v>
+      </c>
+      <c r="J692" t="b">
+        <v>0</v>
+      </c>
+      <c r="K692" t="n">
+        <v>217000000</v>
+      </c>
+      <c r="L692" t="b">
+        <v>0</v>
+      </c>
+      <c r="M692" t="n">
+        <v>149</v>
+      </c>
+      <c r="N692" t="n">
+        <v>0</v>
+      </c>
+      <c r="O692" t="n">
+        <v>0</v>
+      </c>
+      <c r="P692" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Bumblebee</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>card_692</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Travis Knight</t>
+        </is>
+      </c>
+      <c r="D693" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E693" t="n">
+        <v>3.21</v>
+      </c>
+      <c r="F693" t="n">
+        <v>69</v>
+      </c>
+      <c r="I693" t="n">
+        <v>468000000</v>
+      </c>
+      <c r="J693" t="b">
+        <v>0</v>
+      </c>
+      <c r="K693" t="n">
+        <v>135000000</v>
+      </c>
+      <c r="L693" t="b">
+        <v>0</v>
+      </c>
+      <c r="M693" t="n">
+        <v>114</v>
+      </c>
+      <c r="N693" t="n">
+        <v>0</v>
+      </c>
+      <c r="O693" t="n">
+        <v>0</v>
+      </c>
+      <c r="P693" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Transformers: Rise of the Beasts</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>card_693</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Steven Caple Jr.</t>
+        </is>
+      </c>
+      <c r="D694" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E694" t="n">
+        <v>2.68</v>
+      </c>
+      <c r="F694" t="n">
+        <v>55</v>
+      </c>
+      <c r="I694" t="n">
+        <v>441700000</v>
+      </c>
+      <c r="J694" t="b">
+        <v>0</v>
+      </c>
+      <c r="K694" t="n">
+        <v>200000000</v>
+      </c>
+      <c r="L694" t="b">
+        <v>0</v>
+      </c>
+      <c r="M694" t="n">
+        <v>127</v>
+      </c>
+      <c r="N694" t="n">
+        <v>0</v>
+      </c>
+      <c r="O694" t="n">
+        <v>0</v>
+      </c>
+      <c r="P694" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Studio Ghibli films, part 1: 1988-2001 (card_694-700)
Grave of the Fireflies, Kiki's Delivery Service, Only Yesterday, Porco
Rosso, Pom Poko, Whisper of the Heart, Spirited Away.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P694"/>
+  <dimension ref="A1:P701"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -35914,352 +35914,696 @@
       </c>
     </row>
     <row r="688">
-      <c r="A688" t="inlineStr">
+      <c r="A688" s="10" t="inlineStr">
         <is>
           <t>Transformers</t>
         </is>
       </c>
-      <c r="B688" t="inlineStr">
+      <c r="B688" s="10" t="inlineStr">
         <is>
           <t>card_687</t>
         </is>
       </c>
-      <c r="C688" t="inlineStr">
+      <c r="C688" s="10" t="inlineStr">
         <is>
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="D688" t="n">
+      <c r="D688" s="10" t="n">
         <v>2007</v>
       </c>
-      <c r="E688" t="n">
+      <c r="E688" s="10" t="n">
         <v>3.4</v>
       </c>
-      <c r="F688" t="n">
+      <c r="F688" s="10" t="n">
         <v>71</v>
       </c>
-      <c r="I688" t="n">
+      <c r="I688" s="10" t="n">
         <v>709700000</v>
       </c>
-      <c r="J688" t="b">
-        <v>0</v>
-      </c>
-      <c r="K688" t="n">
+      <c r="J688" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K688" s="10" t="n">
         <v>150000000</v>
       </c>
-      <c r="L688" t="b">
-        <v>0</v>
-      </c>
-      <c r="M688" t="n">
+      <c r="L688" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M688" s="10" t="n">
         <v>143</v>
       </c>
-      <c r="N688" t="n">
-        <v>0</v>
-      </c>
-      <c r="O688" t="n">
-        <v>0</v>
-      </c>
-      <c r="P688" t="b">
+      <c r="N688" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O688" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P688" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="689">
-      <c r="A689" t="inlineStr">
+      <c r="A689" s="10" t="inlineStr">
         <is>
           <t>Transformers: Revenge of the Fallen</t>
         </is>
       </c>
-      <c r="B689" t="inlineStr">
+      <c r="B689" s="10" t="inlineStr">
         <is>
           <t>card_688</t>
         </is>
       </c>
-      <c r="C689" t="inlineStr">
+      <c r="C689" s="10" t="inlineStr">
         <is>
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="D689" t="n">
+      <c r="D689" s="10" t="n">
         <v>2009</v>
       </c>
-      <c r="E689" t="n">
+      <c r="E689" s="10" t="n">
         <v>2.77</v>
       </c>
-      <c r="F689" t="n">
+      <c r="F689" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="I689" t="n">
+      <c r="I689" s="10" t="n">
         <v>836500000</v>
       </c>
-      <c r="J689" t="b">
-        <v>0</v>
-      </c>
-      <c r="K689" t="n">
+      <c r="J689" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K689" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L689" t="b">
-        <v>0</v>
-      </c>
-      <c r="M689" t="n">
+      <c r="L689" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M689" s="10" t="n">
         <v>150</v>
       </c>
-      <c r="N689" t="n">
-        <v>0</v>
-      </c>
-      <c r="O689" t="n">
-        <v>0</v>
-      </c>
-      <c r="P689" t="b">
+      <c r="N689" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O689" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P689" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="690">
-      <c r="A690" t="inlineStr">
+      <c r="A690" s="10" t="inlineStr">
         <is>
           <t>Transformers: Dark of the Moon</t>
         </is>
       </c>
-      <c r="B690" t="inlineStr">
+      <c r="B690" s="10" t="inlineStr">
         <is>
           <t>card_689</t>
         </is>
       </c>
-      <c r="C690" t="inlineStr">
+      <c r="C690" s="10" t="inlineStr">
         <is>
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="D690" t="n">
+      <c r="D690" s="10" t="n">
         <v>2011</v>
       </c>
-      <c r="E690" t="n">
+      <c r="E690" s="10" t="n">
         <v>2.88</v>
       </c>
-      <c r="F690" t="n">
+      <c r="F690" s="10" t="n">
         <v>59</v>
       </c>
-      <c r="I690" t="n">
+      <c r="I690" s="10" t="n">
         <v>1124000000</v>
       </c>
-      <c r="J690" t="b">
-        <v>0</v>
-      </c>
-      <c r="K690" t="n">
+      <c r="J690" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K690" s="10" t="n">
         <v>195000000</v>
       </c>
-      <c r="L690" t="b">
-        <v>0</v>
-      </c>
-      <c r="M690" t="n">
+      <c r="L690" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M690" s="10" t="n">
         <v>154</v>
       </c>
-      <c r="N690" t="n">
-        <v>0</v>
-      </c>
-      <c r="O690" t="n">
-        <v>0</v>
-      </c>
-      <c r="P690" t="b">
+      <c r="N690" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O690" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P690" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="691">
-      <c r="A691" t="inlineStr">
+      <c r="A691" s="10" t="inlineStr">
         <is>
           <t>Transformers: Age of Extinction</t>
         </is>
       </c>
-      <c r="B691" t="inlineStr">
+      <c r="B691" s="10" t="inlineStr">
         <is>
           <t>card_690</t>
         </is>
       </c>
-      <c r="C691" t="inlineStr">
+      <c r="C691" s="10" t="inlineStr">
         <is>
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="D691" t="n">
+      <c r="D691" s="10" t="n">
         <v>2014</v>
       </c>
-      <c r="E691" t="n">
+      <c r="E691" s="10" t="n">
         <v>2.32</v>
       </c>
-      <c r="F691" t="n">
+      <c r="F691" s="10" t="n">
         <v>46</v>
       </c>
-      <c r="I691" t="n">
+      <c r="I691" s="10" t="n">
         <v>1105000000</v>
       </c>
-      <c r="J691" t="b">
-        <v>0</v>
-      </c>
-      <c r="K691" t="n">
+      <c r="J691" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K691" s="10" t="n">
         <v>210000000</v>
       </c>
-      <c r="L691" t="b">
-        <v>0</v>
-      </c>
-      <c r="M691" t="n">
+      <c r="L691" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M691" s="10" t="n">
         <v>165</v>
       </c>
-      <c r="N691" t="n">
-        <v>0</v>
-      </c>
-      <c r="O691" t="n">
-        <v>0</v>
-      </c>
-      <c r="P691" t="b">
+      <c r="N691" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O691" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P691" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="692">
-      <c r="A692" t="inlineStr">
+      <c r="A692" s="10" t="inlineStr">
         <is>
           <t>Transformers: The Last Knight</t>
         </is>
       </c>
-      <c r="B692" t="inlineStr">
+      <c r="B692" s="10" t="inlineStr">
         <is>
           <t>card_691</t>
         </is>
       </c>
-      <c r="C692" t="inlineStr">
+      <c r="C692" s="10" t="inlineStr">
         <is>
           <t>Michael Bay</t>
         </is>
       </c>
-      <c r="D692" t="n">
+      <c r="D692" s="10" t="n">
         <v>2017</v>
       </c>
-      <c r="E692" t="n">
+      <c r="E692" s="10" t="n">
         <v>2.13</v>
       </c>
-      <c r="F692" t="n">
+      <c r="F692" s="10" t="n">
         <v>41</v>
       </c>
-      <c r="I692" t="n">
+      <c r="I692" s="10" t="n">
         <v>605400000</v>
       </c>
-      <c r="J692" t="b">
-        <v>0</v>
-      </c>
-      <c r="K692" t="n">
+      <c r="J692" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K692" s="10" t="n">
         <v>217000000</v>
       </c>
-      <c r="L692" t="b">
-        <v>0</v>
-      </c>
-      <c r="M692" t="n">
+      <c r="L692" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M692" s="10" t="n">
         <v>149</v>
       </c>
-      <c r="N692" t="n">
-        <v>0</v>
-      </c>
-      <c r="O692" t="n">
-        <v>0</v>
-      </c>
-      <c r="P692" t="b">
+      <c r="N692" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O692" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P692" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="693">
-      <c r="A693" t="inlineStr">
+      <c r="A693" s="10" t="inlineStr">
         <is>
           <t>Bumblebee</t>
         </is>
       </c>
-      <c r="B693" t="inlineStr">
+      <c r="B693" s="10" t="inlineStr">
         <is>
           <t>card_692</t>
         </is>
       </c>
-      <c r="C693" t="inlineStr">
+      <c r="C693" s="10" t="inlineStr">
         <is>
           <t>Travis Knight</t>
         </is>
       </c>
-      <c r="D693" t="n">
+      <c r="D693" s="10" t="n">
         <v>2018</v>
       </c>
-      <c r="E693" t="n">
+      <c r="E693" s="10" t="n">
         <v>3.21</v>
       </c>
-      <c r="F693" t="n">
+      <c r="F693" s="10" t="n">
         <v>69</v>
       </c>
-      <c r="I693" t="n">
+      <c r="I693" s="10" t="n">
         <v>468000000</v>
       </c>
-      <c r="J693" t="b">
-        <v>0</v>
-      </c>
-      <c r="K693" t="n">
+      <c r="J693" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K693" s="10" t="n">
         <v>135000000</v>
       </c>
-      <c r="L693" t="b">
-        <v>0</v>
-      </c>
-      <c r="M693" t="n">
+      <c r="L693" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M693" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="N693" t="n">
-        <v>0</v>
-      </c>
-      <c r="O693" t="n">
-        <v>0</v>
-      </c>
-      <c r="P693" t="b">
+      <c r="N693" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O693" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P693" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="694">
-      <c r="A694" t="inlineStr">
+      <c r="A694" s="10" t="inlineStr">
         <is>
           <t>Transformers: Rise of the Beasts</t>
         </is>
       </c>
-      <c r="B694" t="inlineStr">
+      <c r="B694" s="10" t="inlineStr">
         <is>
           <t>card_693</t>
         </is>
       </c>
-      <c r="C694" t="inlineStr">
+      <c r="C694" s="10" t="inlineStr">
         <is>
           <t>Steven Caple Jr.</t>
         </is>
       </c>
-      <c r="D694" t="n">
+      <c r="D694" s="10" t="n">
         <v>2023</v>
       </c>
-      <c r="E694" t="n">
+      <c r="E694" s="10" t="n">
         <v>2.68</v>
       </c>
-      <c r="F694" t="n">
+      <c r="F694" s="10" t="n">
         <v>55</v>
       </c>
-      <c r="I694" t="n">
+      <c r="I694" s="10" t="n">
         <v>441700000</v>
       </c>
-      <c r="J694" t="b">
-        <v>0</v>
-      </c>
-      <c r="K694" t="n">
+      <c r="J694" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K694" s="10" t="n">
         <v>200000000</v>
       </c>
-      <c r="L694" t="b">
-        <v>0</v>
-      </c>
-      <c r="M694" t="n">
+      <c r="L694" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M694" s="10" t="n">
         <v>127</v>
       </c>
-      <c r="N694" t="n">
-        <v>0</v>
-      </c>
-      <c r="O694" t="n">
-        <v>0</v>
-      </c>
-      <c r="P694" t="b">
+      <c r="N694" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O694" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P694" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Grave of the Fireflies</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>card_694</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Isao Takahata</t>
+        </is>
+      </c>
+      <c r="D695" t="n">
+        <v>1988</v>
+      </c>
+      <c r="E695" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="I695" t="n">
+        <v>17000000</v>
+      </c>
+      <c r="J695" t="b">
+        <v>1</v>
+      </c>
+      <c r="K695" t="n">
+        <v>3700000</v>
+      </c>
+      <c r="L695" t="b">
+        <v>0</v>
+      </c>
+      <c r="M695" t="n">
+        <v>89</v>
+      </c>
+      <c r="N695" t="n">
+        <v>0</v>
+      </c>
+      <c r="O695" t="n">
+        <v>0</v>
+      </c>
+      <c r="P695" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Kiki's Delivery Service</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>card_695</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D696" t="n">
+        <v>1989</v>
+      </c>
+      <c r="E696" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="F696" t="n">
+        <v>83</v>
+      </c>
+      <c r="I696" t="n">
+        <v>41800000</v>
+      </c>
+      <c r="J696" t="b">
+        <v>0</v>
+      </c>
+      <c r="K696" t="n">
+        <v>6900000</v>
+      </c>
+      <c r="L696" t="b">
+        <v>0</v>
+      </c>
+      <c r="M696" t="n">
+        <v>102</v>
+      </c>
+      <c r="N696" t="n">
+        <v>0</v>
+      </c>
+      <c r="O696" t="n">
+        <v>0</v>
+      </c>
+      <c r="P696" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Only Yesterday</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>card_696</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Isao Takahata</t>
+        </is>
+      </c>
+      <c r="D697" t="n">
+        <v>1991</v>
+      </c>
+      <c r="E697" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="I697" t="n">
+        <v>26500000</v>
+      </c>
+      <c r="J697" t="b">
+        <v>1</v>
+      </c>
+      <c r="K697" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="L697" t="b">
+        <v>1</v>
+      </c>
+      <c r="M697" t="n">
+        <v>118</v>
+      </c>
+      <c r="N697" t="n">
+        <v>0</v>
+      </c>
+      <c r="O697" t="n">
+        <v>0</v>
+      </c>
+      <c r="P697" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Porco Rosso</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>card_697</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D698" t="n">
+        <v>1992</v>
+      </c>
+      <c r="E698" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F698" t="n">
+        <v>81</v>
+      </c>
+      <c r="I698" t="n">
+        <v>44600000</v>
+      </c>
+      <c r="J698" t="b">
+        <v>0</v>
+      </c>
+      <c r="K698" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="L698" t="b">
+        <v>0</v>
+      </c>
+      <c r="M698" t="n">
+        <v>94</v>
+      </c>
+      <c r="N698" t="n">
+        <v>0</v>
+      </c>
+      <c r="O698" t="n">
+        <v>0</v>
+      </c>
+      <c r="P698" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Pom Poko</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>card_698</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Isao Takahata</t>
+        </is>
+      </c>
+      <c r="D699" t="n">
+        <v>1994</v>
+      </c>
+      <c r="E699" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="F699" t="n">
+        <v>73</v>
+      </c>
+      <c r="I699" t="n">
+        <v>41800000</v>
+      </c>
+      <c r="J699" t="b">
+        <v>1</v>
+      </c>
+      <c r="K699" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L699" t="b">
+        <v>1</v>
+      </c>
+      <c r="M699" t="n">
+        <v>119</v>
+      </c>
+      <c r="N699" t="n">
+        <v>0</v>
+      </c>
+      <c r="O699" t="n">
+        <v>0</v>
+      </c>
+      <c r="P699" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Whisper of the Heart</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>card_699</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Yoshifumi Kondo</t>
+        </is>
+      </c>
+      <c r="D700" t="n">
+        <v>1995</v>
+      </c>
+      <c r="E700" t="n">
+        <v>4.19</v>
+      </c>
+      <c r="F700" t="n">
+        <v>81</v>
+      </c>
+      <c r="I700" t="n">
+        <v>34900000</v>
+      </c>
+      <c r="J700" t="b">
+        <v>0</v>
+      </c>
+      <c r="K700" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L700" t="b">
+        <v>1</v>
+      </c>
+      <c r="M700" t="n">
+        <v>111</v>
+      </c>
+      <c r="N700" t="n">
+        <v>0</v>
+      </c>
+      <c r="O700" t="n">
+        <v>0</v>
+      </c>
+      <c r="P700" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Spirited Away</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>card_700</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D701" t="n">
+        <v>2001</v>
+      </c>
+      <c r="E701" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="F701" t="n">
+        <v>90</v>
+      </c>
+      <c r="I701" t="n">
+        <v>396000000</v>
+      </c>
+      <c r="J701" t="b">
+        <v>0</v>
+      </c>
+      <c r="K701" t="n">
+        <v>19200000</v>
+      </c>
+      <c r="L701" t="b">
+        <v>0</v>
+      </c>
+      <c r="M701" t="n">
+        <v>124</v>
+      </c>
+      <c r="N701" t="n">
+        <v>1</v>
+      </c>
+      <c r="O701" t="n">
+        <v>0</v>
+      </c>
+      <c r="P701" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Studio Ghibli films, part 2: 2002-2023 (card_701-707)
The Cat Returns, Ponyo, The Secret World of Arrietty, From Up on
Poppy Hill, The Wind Rises, When Marnie Was There, The Boy and the
Heron. This completes all 46 categories from the original request.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P701"/>
+  <dimension ref="A1:P708"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -36264,346 +36264,693 @@
       </c>
     </row>
     <row r="695">
-      <c r="A695" t="inlineStr">
+      <c r="A695" s="10" t="inlineStr">
         <is>
           <t>Grave of the Fireflies</t>
         </is>
       </c>
-      <c r="B695" t="inlineStr">
+      <c r="B695" s="10" t="inlineStr">
         <is>
           <t>card_694</t>
         </is>
       </c>
-      <c r="C695" t="inlineStr">
+      <c r="C695" s="10" t="inlineStr">
         <is>
           <t>Isao Takahata</t>
         </is>
       </c>
-      <c r="D695" t="n">
+      <c r="D695" s="10" t="n">
         <v>1988</v>
       </c>
-      <c r="E695" t="n">
+      <c r="E695" s="10" t="n">
         <v>4.48</v>
       </c>
-      <c r="I695" t="n">
+      <c r="I695" s="10" t="n">
         <v>17000000</v>
       </c>
-      <c r="J695" t="b">
+      <c r="J695" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K695" t="n">
+      <c r="K695" s="10" t="n">
         <v>3700000</v>
       </c>
-      <c r="L695" t="b">
-        <v>0</v>
-      </c>
-      <c r="M695" t="n">
+      <c r="L695" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M695" s="10" t="n">
         <v>89</v>
       </c>
-      <c r="N695" t="n">
-        <v>0</v>
-      </c>
-      <c r="O695" t="n">
-        <v>0</v>
-      </c>
-      <c r="P695" t="b">
+      <c r="N695" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O695" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P695" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="696">
-      <c r="A696" t="inlineStr">
+      <c r="A696" s="10" t="inlineStr">
         <is>
           <t>Kiki's Delivery Service</t>
         </is>
       </c>
-      <c r="B696" t="inlineStr">
+      <c r="B696" s="10" t="inlineStr">
         <is>
           <t>card_695</t>
         </is>
       </c>
-      <c r="C696" t="inlineStr">
+      <c r="C696" s="10" t="inlineStr">
         <is>
           <t>Hayao Miyazaki</t>
         </is>
       </c>
-      <c r="D696" t="n">
+      <c r="D696" s="10" t="n">
         <v>1989</v>
       </c>
-      <c r="E696" t="n">
+      <c r="E696" s="10" t="n">
         <v>4.15</v>
       </c>
-      <c r="F696" t="n">
+      <c r="F696" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="I696" t="n">
+      <c r="I696" s="10" t="n">
         <v>41800000</v>
       </c>
-      <c r="J696" t="b">
-        <v>0</v>
-      </c>
-      <c r="K696" t="n">
+      <c r="J696" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K696" s="10" t="n">
         <v>6900000</v>
       </c>
-      <c r="L696" t="b">
-        <v>0</v>
-      </c>
-      <c r="M696" t="n">
+      <c r="L696" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M696" s="10" t="n">
         <v>102</v>
       </c>
-      <c r="N696" t="n">
-        <v>0</v>
-      </c>
-      <c r="O696" t="n">
-        <v>0</v>
-      </c>
-      <c r="P696" t="b">
+      <c r="N696" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O696" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P696" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="697">
-      <c r="A697" t="inlineStr">
+      <c r="A697" s="10" t="inlineStr">
         <is>
           <t>Only Yesterday</t>
         </is>
       </c>
-      <c r="B697" t="inlineStr">
+      <c r="B697" s="10" t="inlineStr">
         <is>
           <t>card_696</t>
         </is>
       </c>
-      <c r="C697" t="inlineStr">
+      <c r="C697" s="10" t="inlineStr">
         <is>
           <t>Isao Takahata</t>
         </is>
       </c>
-      <c r="D697" t="n">
+      <c r="D697" s="10" t="n">
         <v>1991</v>
       </c>
-      <c r="E697" t="n">
+      <c r="E697" s="10" t="n">
         <v>3.91</v>
       </c>
-      <c r="I697" t="n">
+      <c r="I697" s="10" t="n">
         <v>26500000</v>
       </c>
-      <c r="J697" t="b">
+      <c r="J697" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K697" t="n">
+      <c r="K697" s="10" t="n">
         <v>4000000</v>
       </c>
-      <c r="L697" t="b">
+      <c r="L697" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M697" t="n">
+      <c r="M697" s="10" t="n">
         <v>118</v>
       </c>
-      <c r="N697" t="n">
-        <v>0</v>
-      </c>
-      <c r="O697" t="n">
-        <v>0</v>
-      </c>
-      <c r="P697" t="b">
+      <c r="N697" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O697" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P697" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="698">
-      <c r="A698" t="inlineStr">
+      <c r="A698" s="10" t="inlineStr">
         <is>
           <t>Porco Rosso</t>
         </is>
       </c>
-      <c r="B698" t="inlineStr">
+      <c r="B698" s="10" t="inlineStr">
         <is>
           <t>card_697</t>
         </is>
       </c>
-      <c r="C698" t="inlineStr">
+      <c r="C698" s="10" t="inlineStr">
         <is>
           <t>Hayao Miyazaki</t>
         </is>
       </c>
-      <c r="D698" t="n">
+      <c r="D698" s="10" t="n">
         <v>1992</v>
       </c>
-      <c r="E698" t="n">
+      <c r="E698" s="10" t="n">
         <v>4.04</v>
       </c>
-      <c r="F698" t="n">
+      <c r="F698" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I698" t="n">
+      <c r="I698" s="10" t="n">
         <v>44600000</v>
       </c>
-      <c r="J698" t="b">
-        <v>0</v>
-      </c>
-      <c r="K698" t="n">
+      <c r="J698" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K698" s="10" t="n">
         <v>1800000</v>
       </c>
-      <c r="L698" t="b">
-        <v>0</v>
-      </c>
-      <c r="M698" t="n">
+      <c r="L698" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M698" s="10" t="n">
         <v>94</v>
       </c>
-      <c r="N698" t="n">
-        <v>0</v>
-      </c>
-      <c r="O698" t="n">
-        <v>0</v>
-      </c>
-      <c r="P698" t="b">
+      <c r="N698" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O698" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P698" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="699">
-      <c r="A699" t="inlineStr">
+      <c r="A699" s="10" t="inlineStr">
         <is>
           <t>Pom Poko</t>
         </is>
       </c>
-      <c r="B699" t="inlineStr">
+      <c r="B699" s="10" t="inlineStr">
         <is>
           <t>card_698</t>
         </is>
       </c>
-      <c r="C699" t="inlineStr">
+      <c r="C699" s="10" t="inlineStr">
         <is>
           <t>Isao Takahata</t>
         </is>
       </c>
-      <c r="D699" t="n">
+      <c r="D699" s="10" t="n">
         <v>1994</v>
       </c>
-      <c r="E699" t="n">
+      <c r="E699" s="10" t="n">
         <v>3.71</v>
       </c>
-      <c r="F699" t="n">
+      <c r="F699" s="10" t="n">
         <v>73</v>
       </c>
-      <c r="I699" t="n">
+      <c r="I699" s="10" t="n">
         <v>41800000</v>
       </c>
-      <c r="J699" t="b">
+      <c r="J699" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K699" t="n">
+      <c r="K699" s="10" t="n">
         <v>20000000</v>
       </c>
-      <c r="L699" t="b">
+      <c r="L699" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M699" t="n">
+      <c r="M699" s="10" t="n">
         <v>119</v>
       </c>
-      <c r="N699" t="n">
-        <v>0</v>
-      </c>
-      <c r="O699" t="n">
-        <v>0</v>
-      </c>
-      <c r="P699" t="b">
+      <c r="N699" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O699" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P699" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="700">
-      <c r="A700" t="inlineStr">
+      <c r="A700" s="10" t="inlineStr">
         <is>
           <t>Whisper of the Heart</t>
         </is>
       </c>
-      <c r="B700" t="inlineStr">
+      <c r="B700" s="10" t="inlineStr">
         <is>
           <t>card_699</t>
         </is>
       </c>
-      <c r="C700" t="inlineStr">
+      <c r="C700" s="10" t="inlineStr">
         <is>
           <t>Yoshifumi Kondo</t>
         </is>
       </c>
-      <c r="D700" t="n">
+      <c r="D700" s="10" t="n">
         <v>1995</v>
       </c>
-      <c r="E700" t="n">
+      <c r="E700" s="10" t="n">
         <v>4.19</v>
       </c>
-      <c r="F700" t="n">
+      <c r="F700" s="10" t="n">
         <v>81</v>
       </c>
-      <c r="I700" t="n">
+      <c r="I700" s="10" t="n">
         <v>34900000</v>
       </c>
-      <c r="J700" t="b">
-        <v>0</v>
-      </c>
-      <c r="K700" t="n">
+      <c r="J700" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K700" s="10" t="n">
         <v>15000000</v>
       </c>
-      <c r="L700" t="b">
+      <c r="L700" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="M700" t="n">
+      <c r="M700" s="10" t="n">
         <v>111</v>
       </c>
-      <c r="N700" t="n">
-        <v>0</v>
-      </c>
-      <c r="O700" t="n">
-        <v>0</v>
-      </c>
-      <c r="P700" t="b">
+      <c r="N700" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O700" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P700" s="10" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="701">
-      <c r="A701" t="inlineStr">
+      <c r="A701" s="10" t="inlineStr">
         <is>
           <t>Spirited Away</t>
         </is>
       </c>
-      <c r="B701" t="inlineStr">
+      <c r="B701" s="10" t="inlineStr">
         <is>
           <t>card_700</t>
         </is>
       </c>
-      <c r="C701" t="inlineStr">
+      <c r="C701" s="10" t="inlineStr">
         <is>
           <t>Hayao Miyazaki</t>
         </is>
       </c>
-      <c r="D701" t="n">
+      <c r="D701" s="10" t="n">
         <v>2001</v>
       </c>
-      <c r="E701" t="n">
+      <c r="E701" s="10" t="n">
         <v>4.43</v>
       </c>
-      <c r="F701" t="n">
+      <c r="F701" s="10" t="n">
         <v>90</v>
       </c>
-      <c r="I701" t="n">
+      <c r="I701" s="10" t="n">
         <v>396000000</v>
       </c>
-      <c r="J701" t="b">
-        <v>0</v>
-      </c>
-      <c r="K701" t="n">
+      <c r="J701" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K701" s="10" t="n">
         <v>19200000</v>
       </c>
-      <c r="L701" t="b">
-        <v>0</v>
-      </c>
-      <c r="M701" t="n">
+      <c r="L701" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M701" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="N701" t="n">
+      <c r="N701" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O701" t="n">
-        <v>0</v>
-      </c>
-      <c r="P701" t="b">
+      <c r="O701" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P701" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>The Cat Returns</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>card_701</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Hiroyuki Morita</t>
+        </is>
+      </c>
+      <c r="D702" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E702" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="I702" t="n">
+        <v>65000000</v>
+      </c>
+      <c r="J702" t="b">
+        <v>0</v>
+      </c>
+      <c r="K702" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="L702" t="b">
+        <v>0</v>
+      </c>
+      <c r="M702" t="n">
+        <v>75</v>
+      </c>
+      <c r="N702" t="n">
+        <v>0</v>
+      </c>
+      <c r="O702" t="n">
+        <v>0</v>
+      </c>
+      <c r="P702" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>Ponyo</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>card_702</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D703" t="n">
+        <v>2008</v>
+      </c>
+      <c r="E703" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="F703" t="n">
+        <v>78</v>
+      </c>
+      <c r="I703" t="n">
+        <v>205900000</v>
+      </c>
+      <c r="J703" t="b">
+        <v>0</v>
+      </c>
+      <c r="K703" t="n">
+        <v>34000000</v>
+      </c>
+      <c r="L703" t="b">
+        <v>0</v>
+      </c>
+      <c r="M703" t="n">
+        <v>101</v>
+      </c>
+      <c r="N703" t="n">
+        <v>0</v>
+      </c>
+      <c r="O703" t="n">
+        <v>0</v>
+      </c>
+      <c r="P703" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>The Secret World of Arrietty</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>card_703</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Hiromasa Yonebayashi</t>
+        </is>
+      </c>
+      <c r="D704" t="n">
+        <v>2010</v>
+      </c>
+      <c r="E704" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="F704" t="n">
+        <v>81</v>
+      </c>
+      <c r="I704" t="n">
+        <v>149000000</v>
+      </c>
+      <c r="J704" t="b">
+        <v>0</v>
+      </c>
+      <c r="K704" t="n">
+        <v>23000000</v>
+      </c>
+      <c r="L704" t="b">
+        <v>0</v>
+      </c>
+      <c r="M704" t="n">
+        <v>95</v>
+      </c>
+      <c r="N704" t="n">
+        <v>0</v>
+      </c>
+      <c r="O704" t="n">
+        <v>0</v>
+      </c>
+      <c r="P704" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>From Up on Poppy Hill</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>card_704</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Goro Miyazaki</t>
+        </is>
+      </c>
+      <c r="D705" t="n">
+        <v>2011</v>
+      </c>
+      <c r="E705" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="F705" t="n">
+        <v>76</v>
+      </c>
+      <c r="I705" t="n">
+        <v>61500000</v>
+      </c>
+      <c r="J705" t="b">
+        <v>0</v>
+      </c>
+      <c r="K705" t="n">
+        <v>22000000</v>
+      </c>
+      <c r="L705" t="b">
+        <v>0</v>
+      </c>
+      <c r="M705" t="n">
+        <v>92</v>
+      </c>
+      <c r="N705" t="n">
+        <v>0</v>
+      </c>
+      <c r="O705" t="n">
+        <v>0</v>
+      </c>
+      <c r="P705" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>The Wind Rises</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>card_705</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D706" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E706" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="F706" t="n">
+        <v>83</v>
+      </c>
+      <c r="I706" t="n">
+        <v>136500000</v>
+      </c>
+      <c r="J706" t="b">
+        <v>0</v>
+      </c>
+      <c r="K706" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="L706" t="b">
+        <v>0</v>
+      </c>
+      <c r="M706" t="n">
+        <v>126</v>
+      </c>
+      <c r="N706" t="n">
+        <v>0</v>
+      </c>
+      <c r="O706" t="n">
+        <v>0</v>
+      </c>
+      <c r="P706" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>When Marnie Was There</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>card_706</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>Hiromasa Yonebayashi</t>
+        </is>
+      </c>
+      <c r="D707" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E707" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="F707" t="n">
+        <v>79</v>
+      </c>
+      <c r="I707" t="n">
+        <v>35700000</v>
+      </c>
+      <c r="J707" t="b">
+        <v>0</v>
+      </c>
+      <c r="K707" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="L707" t="b">
+        <v>0</v>
+      </c>
+      <c r="M707" t="n">
+        <v>103</v>
+      </c>
+      <c r="N707" t="n">
+        <v>0</v>
+      </c>
+      <c r="O707" t="n">
+        <v>0</v>
+      </c>
+      <c r="P707" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>The Boy and the Heron</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>card_707</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D708" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E708" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F708" t="n">
+        <v>78</v>
+      </c>
+      <c r="I708" t="n">
+        <v>294200000</v>
+      </c>
+      <c r="J708" t="b">
+        <v>0</v>
+      </c>
+      <c r="K708" t="n">
+        <v>53000000</v>
+      </c>
+      <c r="L708" t="b">
+        <v>0</v>
+      </c>
+      <c r="M708" t="n">
+        <v>124</v>
+      </c>
+      <c r="N708" t="n">
+        <v>1</v>
+      </c>
+      <c r="O708" t="n">
+        <v>0</v>
+      </c>
+      <c r="P708" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill remaining director birth years, drop undocumented ones
Set estimated birth years for Ralph Zondag (1963), Fawn Veerasunthorn
(1981), Toshiyuki Tsuru (1966), Junji Shimizu (1960), and Hiroaki
Miyamoto (1981, confirmed over the 1881 typo).

Removed the 5 cards whose directors (Masahiko Murata, Hiroyuki
Yamashita, Kazuhisa Takenouchi) have no documented birth year at all:
Naruto Shippuden the Movie: The Will of Fire / The Lost Tower / Blood
Prison, Boruto: Naruto the Movie, and One Piece: The Cursed Holy
Sword. All director_age_at_release values now resolve (702/702).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -394,7 +394,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P708"/>
+  <dimension ref="A1:P703"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38" customWidth="1" style="10" min="1" max="1"/>
@@ -34920,39 +34920,39 @@
     <row r="667">
       <c r="A667" s="10" t="inlineStr">
         <is>
-          <t>Naruto Shippuden the Movie: The Will of Fire</t>
+          <t>Road to Ninja: Naruto the Movie</t>
         </is>
       </c>
       <c r="B667" s="10" t="inlineStr">
         <is>
-          <t>card_666</t>
+          <t>card_669</t>
         </is>
       </c>
       <c r="C667" s="10" t="inlineStr">
         <is>
-          <t>Masahiko Murata</t>
+          <t>Hayato Date</t>
         </is>
       </c>
       <c r="D667" s="10" t="n">
-        <v>2009</v>
+        <v>2012</v>
       </c>
       <c r="E667" s="10" t="n">
-        <v>3.19</v>
+        <v>3.49</v>
       </c>
       <c r="I667" s="10" t="n">
-        <v>8100000</v>
+        <v>17900000</v>
       </c>
       <c r="J667" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K667" s="10" t="n">
-        <v>4500000</v>
+        <v>5000000</v>
       </c>
       <c r="L667" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M667" s="10" t="n">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="N667" s="10" t="n">
         <v>0</v>
@@ -34967,39 +34967,39 @@
     <row r="668">
       <c r="A668" s="10" t="inlineStr">
         <is>
-          <t>Naruto Shippuden the Movie: The Lost Tower</t>
+          <t>The Last: Naruto the Movie</t>
         </is>
       </c>
       <c r="B668" s="10" t="inlineStr">
         <is>
-          <t>card_667</t>
+          <t>card_670</t>
         </is>
       </c>
       <c r="C668" s="10" t="inlineStr">
         <is>
-          <t>Masahiko Murata</t>
+          <t>Tsuneo Kobayashi</t>
         </is>
       </c>
       <c r="D668" s="10" t="n">
-        <v>2010</v>
+        <v>2014</v>
       </c>
       <c r="E668" s="10" t="n">
-        <v>3.09</v>
+        <v>3.54</v>
       </c>
       <c r="I668" s="10" t="n">
-        <v>8500000</v>
+        <v>19840000</v>
       </c>
       <c r="J668" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K668" s="10" t="n">
-        <v>4500000</v>
+        <v>1010000</v>
       </c>
       <c r="L668" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M668" s="10" t="n">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="N668" s="10" t="n">
         <v>0</v>
@@ -35014,39 +35014,39 @@
     <row r="669">
       <c r="A669" s="10" t="inlineStr">
         <is>
-          <t>Naruto Shippuden the Movie: Blood Prison</t>
+          <t>One Piece: The Movie</t>
         </is>
       </c>
       <c r="B669" s="10" t="inlineStr">
         <is>
-          <t>card_668</t>
+          <t>card_672</t>
         </is>
       </c>
       <c r="C669" s="10" t="inlineStr">
         <is>
-          <t>Masahiko Murata</t>
+          <t>Junji Shimizu</t>
         </is>
       </c>
       <c r="D669" s="10" t="n">
-        <v>2011</v>
+        <v>2000</v>
       </c>
       <c r="E669" s="10" t="n">
-        <v>3.19</v>
+        <v>3.31</v>
       </c>
       <c r="I669" s="10" t="n">
-        <v>9100000</v>
+        <v>20000000</v>
       </c>
       <c r="J669" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K669" s="10" t="n">
-        <v>4500000</v>
+        <v>5000000</v>
       </c>
       <c r="L669" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M669" s="10" t="n">
-        <v>103</v>
+        <v>51</v>
       </c>
       <c r="N669" s="10" t="n">
         <v>0</v>
@@ -35061,30 +35061,30 @@
     <row r="670">
       <c r="A670" s="10" t="inlineStr">
         <is>
-          <t>Road to Ninja: Naruto the Movie</t>
+          <t>One Piece: Clockwork Island Adventure</t>
         </is>
       </c>
       <c r="B670" s="10" t="inlineStr">
         <is>
-          <t>card_669</t>
+          <t>card_673</t>
         </is>
       </c>
       <c r="C670" s="10" t="inlineStr">
         <is>
-          <t>Hayato Date</t>
+          <t>Junji Shimizu</t>
         </is>
       </c>
       <c r="D670" s="10" t="n">
-        <v>2012</v>
+        <v>2001</v>
       </c>
       <c r="E670" s="10" t="n">
-        <v>3.49</v>
+        <v>3.08</v>
       </c>
       <c r="I670" s="10" t="n">
-        <v>17900000</v>
+        <v>24800000</v>
       </c>
       <c r="J670" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K670" s="10" t="n">
         <v>5000000</v>
@@ -35093,7 +35093,7 @@
         <v>1</v>
       </c>
       <c r="M670" s="10" t="n">
-        <v>109</v>
+        <v>60</v>
       </c>
       <c r="N670" s="10" t="n">
         <v>0</v>
@@ -35108,39 +35108,39 @@
     <row r="671">
       <c r="A671" s="10" t="inlineStr">
         <is>
-          <t>The Last: Naruto the Movie</t>
+          <t>One Piece: Chopper's Kingdom on the Island of Strange Animals</t>
         </is>
       </c>
       <c r="B671" s="10" t="inlineStr">
         <is>
-          <t>card_670</t>
+          <t>card_674</t>
         </is>
       </c>
       <c r="C671" s="10" t="inlineStr">
         <is>
-          <t>Tsuneo Kobayashi</t>
+          <t>Junji Shimizu</t>
         </is>
       </c>
       <c r="D671" s="10" t="n">
-        <v>2014</v>
+        <v>2002</v>
       </c>
       <c r="E671" s="10" t="n">
-        <v>3.54</v>
+        <v>2.82</v>
       </c>
       <c r="I671" s="10" t="n">
-        <v>19840000</v>
+        <v>16000000</v>
       </c>
       <c r="J671" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K671" s="10" t="n">
-        <v>1010000</v>
+        <v>5000000</v>
       </c>
       <c r="L671" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M671" s="10" t="n">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="N671" s="10" t="n">
         <v>0</v>
@@ -35155,39 +35155,39 @@
     <row r="672">
       <c r="A672" s="10" t="inlineStr">
         <is>
-          <t>Boruto: Naruto the Movie</t>
+          <t>One Piece: Dead End Adventure</t>
         </is>
       </c>
       <c r="B672" s="10" t="inlineStr">
         <is>
-          <t>card_671</t>
+          <t>card_675</t>
         </is>
       </c>
       <c r="C672" s="10" t="inlineStr">
         <is>
-          <t>Hiroyuki Yamashita</t>
+          <t>Konosuke Uda</t>
         </is>
       </c>
       <c r="D672" s="10" t="n">
-        <v>2015</v>
+        <v>2003</v>
       </c>
       <c r="E672" s="10" t="n">
-        <v>3.22</v>
+        <v>3.36</v>
       </c>
       <c r="I672" s="10" t="n">
-        <v>38500000</v>
+        <v>17200000</v>
       </c>
       <c r="J672" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K672" s="10" t="n">
-        <v>21000000</v>
+        <v>6000000</v>
       </c>
       <c r="L672" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M672" s="10" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="N672" s="10" t="n">
         <v>0</v>
@@ -35202,39 +35202,39 @@
     <row r="673">
       <c r="A673" s="10" t="inlineStr">
         <is>
-          <t>One Piece: The Movie</t>
+          <t>One Piece: Baron Omatsuri and the Secret Island</t>
         </is>
       </c>
       <c r="B673" s="10" t="inlineStr">
         <is>
-          <t>card_672</t>
+          <t>card_677</t>
         </is>
       </c>
       <c r="C673" s="10" t="inlineStr">
         <is>
-          <t>Junji Shimizu</t>
+          <t>Mamoru Hosoda</t>
         </is>
       </c>
       <c r="D673" s="10" t="n">
-        <v>2000</v>
+        <v>2005</v>
       </c>
       <c r="E673" s="10" t="n">
-        <v>3.31</v>
+        <v>4.08</v>
       </c>
       <c r="I673" s="10" t="n">
-        <v>20000000</v>
+        <v>10500000</v>
       </c>
       <c r="J673" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K673" s="10" t="n">
-        <v>5000000</v>
+        <v>6000000</v>
       </c>
       <c r="L673" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M673" s="10" t="n">
-        <v>51</v>
+        <v>91</v>
       </c>
       <c r="N673" s="10" t="n">
         <v>0</v>
@@ -35249,39 +35249,39 @@
     <row r="674">
       <c r="A674" s="10" t="inlineStr">
         <is>
-          <t>One Piece: Clockwork Island Adventure</t>
+          <t>One Piece: The Giant Mechanical Soldier of Karakuri Castle</t>
         </is>
       </c>
       <c r="B674" s="10" t="inlineStr">
         <is>
-          <t>card_673</t>
+          <t>card_678</t>
         </is>
       </c>
       <c r="C674" s="10" t="inlineStr">
         <is>
-          <t>Junji Shimizu</t>
+          <t>Konosuke Uda</t>
         </is>
       </c>
       <c r="D674" s="10" t="n">
-        <v>2001</v>
+        <v>2006</v>
       </c>
       <c r="E674" s="10" t="n">
-        <v>3.08</v>
+        <v>2.87</v>
       </c>
       <c r="I674" s="10" t="n">
-        <v>24800000</v>
+        <v>8500000</v>
       </c>
       <c r="J674" s="10" t="b">
         <v>1</v>
       </c>
       <c r="K674" s="10" t="n">
-        <v>5000000</v>
+        <v>6500000</v>
       </c>
       <c r="L674" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M674" s="10" t="n">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="N674" s="10" t="n">
         <v>0</v>
@@ -35296,42 +35296,42 @@
     <row r="675">
       <c r="A675" s="10" t="inlineStr">
         <is>
-          <t>One Piece: Chopper's Kingdom on the Island of Strange Animals</t>
+          <t>One Piece Film: Strong World</t>
         </is>
       </c>
       <c r="B675" s="10" t="inlineStr">
         <is>
-          <t>card_674</t>
+          <t>card_679</t>
         </is>
       </c>
       <c r="C675" s="10" t="inlineStr">
         <is>
-          <t>Junji Shimizu</t>
+          <t>Munehisa Sakai</t>
         </is>
       </c>
       <c r="D675" s="10" t="n">
-        <v>2002</v>
+        <v>2009</v>
       </c>
       <c r="E675" s="10" t="n">
-        <v>2.82</v>
+        <v>3.56</v>
       </c>
       <c r="I675" s="10" t="n">
-        <v>16000000</v>
+        <v>61200000</v>
       </c>
       <c r="J675" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K675" s="10" t="n">
-        <v>5000000</v>
+        <v>15000000</v>
       </c>
       <c r="L675" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M675" s="10" t="n">
-        <v>56</v>
+        <v>115</v>
       </c>
       <c r="N675" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O675" s="10" t="n">
         <v>0</v>
@@ -35343,39 +35343,39 @@
     <row r="676">
       <c r="A676" s="10" t="inlineStr">
         <is>
-          <t>One Piece: Dead End Adventure</t>
+          <t>One Piece Film: Z</t>
         </is>
       </c>
       <c r="B676" s="10" t="inlineStr">
         <is>
-          <t>card_675</t>
+          <t>card_680</t>
         </is>
       </c>
       <c r="C676" s="10" t="inlineStr">
         <is>
-          <t>Konosuke Uda</t>
+          <t>Tatsuya Nagamine</t>
         </is>
       </c>
       <c r="D676" s="10" t="n">
-        <v>2003</v>
+        <v>2012</v>
       </c>
       <c r="E676" s="10" t="n">
-        <v>3.36</v>
+        <v>3.64</v>
       </c>
       <c r="I676" s="10" t="n">
-        <v>17200000</v>
+        <v>85000000</v>
       </c>
       <c r="J676" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K676" s="10" t="n">
-        <v>6000000</v>
+        <v>16000000</v>
       </c>
       <c r="L676" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M676" s="10" t="n">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="N676" s="10" t="n">
         <v>0</v>
@@ -35390,39 +35390,39 @@
     <row r="677">
       <c r="A677" s="10" t="inlineStr">
         <is>
-          <t>One Piece: The Cursed Holy Sword</t>
+          <t>One Piece Film: Gold</t>
         </is>
       </c>
       <c r="B677" s="10" t="inlineStr">
         <is>
-          <t>card_676</t>
+          <t>card_681</t>
         </is>
       </c>
       <c r="C677" s="10" t="inlineStr">
         <is>
-          <t>Kazuhisa Takenouchi</t>
+          <t>Hiroaki Miyamoto</t>
         </is>
       </c>
       <c r="D677" s="10" t="n">
-        <v>2004</v>
+        <v>2016</v>
       </c>
       <c r="E677" s="10" t="n">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
       <c r="I677" s="10" t="n">
-        <v>16700000</v>
+        <v>70800000</v>
       </c>
       <c r="J677" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K677" s="10" t="n">
-        <v>6000000</v>
+        <v>18000000</v>
       </c>
       <c r="L677" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M677" s="10" t="n">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="N677" s="10" t="n">
         <v>0</v>
@@ -35437,39 +35437,39 @@
     <row r="678">
       <c r="A678" s="10" t="inlineStr">
         <is>
-          <t>One Piece: Baron Omatsuri and the Secret Island</t>
+          <t>One Piece: Stampede</t>
         </is>
       </c>
       <c r="B678" s="10" t="inlineStr">
         <is>
-          <t>card_677</t>
+          <t>card_682</t>
         </is>
       </c>
       <c r="C678" s="10" t="inlineStr">
         <is>
-          <t>Mamoru Hosoda</t>
+          <t>Takashi Otsuka</t>
         </is>
       </c>
       <c r="D678" s="10" t="n">
-        <v>2005</v>
+        <v>2019</v>
       </c>
       <c r="E678" s="10" t="n">
-        <v>4.08</v>
+        <v>3.58</v>
       </c>
       <c r="I678" s="10" t="n">
-        <v>10500000</v>
+        <v>94700000</v>
       </c>
       <c r="J678" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K678" s="10" t="n">
-        <v>6000000</v>
+        <v>20000000</v>
       </c>
       <c r="L678" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M678" s="10" t="n">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="N678" s="10" t="n">
         <v>0</v>
@@ -35484,39 +35484,39 @@
     <row r="679">
       <c r="A679" s="10" t="inlineStr">
         <is>
-          <t>One Piece: The Giant Mechanical Soldier of Karakuri Castle</t>
+          <t>One Piece Film: Red</t>
         </is>
       </c>
       <c r="B679" s="10" t="inlineStr">
         <is>
-          <t>card_678</t>
+          <t>card_683</t>
         </is>
       </c>
       <c r="C679" s="10" t="inlineStr">
         <is>
-          <t>Konosuke Uda</t>
+          <t>Goro Taniguchi</t>
         </is>
       </c>
       <c r="D679" s="10" t="n">
-        <v>2006</v>
+        <v>2022</v>
       </c>
       <c r="E679" s="10" t="n">
-        <v>2.87</v>
+        <v>3.33</v>
       </c>
       <c r="I679" s="10" t="n">
-        <v>8500000</v>
+        <v>246500000</v>
       </c>
       <c r="J679" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K679" s="10" t="n">
-        <v>6500000</v>
+        <v>20000000</v>
       </c>
       <c r="L679" s="10" t="b">
         <v>1</v>
       </c>
       <c r="M679" s="10" t="n">
-        <v>94</v>
+        <v>115</v>
       </c>
       <c r="N679" s="10" t="n">
         <v>0</v>
@@ -35531,42 +35531,45 @@
     <row r="680">
       <c r="A680" s="10" t="inlineStr">
         <is>
-          <t>One Piece Film: Strong World</t>
+          <t>Avatar</t>
         </is>
       </c>
       <c r="B680" s="10" t="inlineStr">
         <is>
-          <t>card_679</t>
+          <t>card_684</t>
         </is>
       </c>
       <c r="C680" s="10" t="inlineStr">
         <is>
-          <t>Munehisa Sakai</t>
+          <t>James Cameron</t>
         </is>
       </c>
       <c r="D680" s="10" t="n">
         <v>2009</v>
       </c>
       <c r="E680" s="10" t="n">
-        <v>3.56</v>
+        <v>3.77</v>
+      </c>
+      <c r="F680" s="10" t="n">
+        <v>74</v>
       </c>
       <c r="I680" s="10" t="n">
-        <v>61200000</v>
+        <v>2924000000</v>
       </c>
       <c r="J680" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K680" s="10" t="n">
-        <v>15000000</v>
+        <v>237000000</v>
       </c>
       <c r="L680" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M680" s="10" t="n">
-        <v>115</v>
+        <v>162</v>
       </c>
       <c r="N680" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O680" s="10" t="n">
         <v>0</v>
@@ -35578,42 +35581,45 @@
     <row r="681">
       <c r="A681" s="10" t="inlineStr">
         <is>
-          <t>One Piece Film: Z</t>
+          <t>Avatar: The Way of Water</t>
         </is>
       </c>
       <c r="B681" s="10" t="inlineStr">
         <is>
-          <t>card_680</t>
+          <t>card_685</t>
         </is>
       </c>
       <c r="C681" s="10" t="inlineStr">
         <is>
-          <t>Tatsuya Nagamine</t>
+          <t>James Cameron</t>
         </is>
       </c>
       <c r="D681" s="10" t="n">
-        <v>2012</v>
+        <v>2022</v>
       </c>
       <c r="E681" s="10" t="n">
-        <v>3.64</v>
+        <v>3.65</v>
+      </c>
+      <c r="F681" s="10" t="n">
+        <v>72</v>
       </c>
       <c r="I681" s="10" t="n">
-        <v>85000000</v>
+        <v>2334000000</v>
       </c>
       <c r="J681" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K681" s="10" t="n">
-        <v>16000000</v>
+        <v>400000000</v>
       </c>
       <c r="L681" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M681" s="10" t="n">
+        <v>192</v>
+      </c>
+      <c r="N681" s="10" t="n">
         <v>1</v>
-      </c>
-      <c r="M681" s="10" t="n">
-        <v>107</v>
-      </c>
-      <c r="N681" s="10" t="n">
-        <v>0</v>
       </c>
       <c r="O681" s="10" t="n">
         <v>0</v>
@@ -35625,42 +35631,45 @@
     <row r="682">
       <c r="A682" s="10" t="inlineStr">
         <is>
-          <t>One Piece Film: Gold</t>
+          <t>Avatar: Fire and Ash</t>
         </is>
       </c>
       <c r="B682" s="10" t="inlineStr">
         <is>
-          <t>card_681</t>
+          <t>card_686</t>
         </is>
       </c>
       <c r="C682" s="10" t="inlineStr">
         <is>
-          <t>Hiroaki Miyamoto</t>
+          <t>James Cameron</t>
         </is>
       </c>
       <c r="D682" s="10" t="n">
-        <v>2016</v>
+        <v>2025</v>
       </c>
       <c r="E682" s="10" t="n">
-        <v>3.5</v>
+        <v>3.55</v>
+      </c>
+      <c r="F682" s="10" t="n">
+        <v>69</v>
       </c>
       <c r="I682" s="10" t="n">
-        <v>70800000</v>
+        <v>1490000000</v>
       </c>
       <c r="J682" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K682" s="10" t="n">
-        <v>18000000</v>
+        <v>375000000</v>
       </c>
       <c r="L682" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M682" s="10" t="n">
+        <v>197</v>
+      </c>
+      <c r="N682" s="10" t="n">
         <v>1</v>
-      </c>
-      <c r="M682" s="10" t="n">
-        <v>120</v>
-      </c>
-      <c r="N682" s="10" t="n">
-        <v>0</v>
       </c>
       <c r="O682" s="10" t="n">
         <v>0</v>
@@ -35672,39 +35681,42 @@
     <row r="683">
       <c r="A683" s="10" t="inlineStr">
         <is>
-          <t>One Piece: Stampede</t>
+          <t>Transformers</t>
         </is>
       </c>
       <c r="B683" s="10" t="inlineStr">
         <is>
-          <t>card_682</t>
+          <t>card_687</t>
         </is>
       </c>
       <c r="C683" s="10" t="inlineStr">
         <is>
-          <t>Takashi Otsuka</t>
+          <t>Michael Bay</t>
         </is>
       </c>
       <c r="D683" s="10" t="n">
-        <v>2019</v>
+        <v>2007</v>
       </c>
       <c r="E683" s="10" t="n">
-        <v>3.58</v>
+        <v>3.4</v>
+      </c>
+      <c r="F683" s="10" t="n">
+        <v>71</v>
       </c>
       <c r="I683" s="10" t="n">
-        <v>94700000</v>
+        <v>709700000</v>
       </c>
       <c r="J683" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K683" s="10" t="n">
-        <v>20000000</v>
+        <v>150000000</v>
       </c>
       <c r="L683" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M683" s="10" t="n">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="N683" s="10" t="n">
         <v>0</v>
@@ -35719,39 +35731,42 @@
     <row r="684">
       <c r="A684" s="10" t="inlineStr">
         <is>
-          <t>One Piece Film: Red</t>
+          <t>Transformers: Revenge of the Fallen</t>
         </is>
       </c>
       <c r="B684" s="10" t="inlineStr">
         <is>
-          <t>card_683</t>
+          <t>card_688</t>
         </is>
       </c>
       <c r="C684" s="10" t="inlineStr">
         <is>
-          <t>Goro Taniguchi</t>
+          <t>Michael Bay</t>
         </is>
       </c>
       <c r="D684" s="10" t="n">
-        <v>2022</v>
+        <v>2009</v>
       </c>
       <c r="E684" s="10" t="n">
-        <v>3.33</v>
+        <v>2.77</v>
+      </c>
+      <c r="F684" s="10" t="n">
+        <v>50</v>
       </c>
       <c r="I684" s="10" t="n">
-        <v>246500000</v>
+        <v>836500000</v>
       </c>
       <c r="J684" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K684" s="10" t="n">
-        <v>20000000</v>
+        <v>200000000</v>
       </c>
       <c r="L684" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M684" s="10" t="n">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="N684" s="10" t="n">
         <v>0</v>
@@ -35766,45 +35781,45 @@
     <row r="685">
       <c r="A685" s="10" t="inlineStr">
         <is>
-          <t>Avatar</t>
+          <t>Transformers: Dark of the Moon</t>
         </is>
       </c>
       <c r="B685" s="10" t="inlineStr">
         <is>
-          <t>card_684</t>
+          <t>card_689</t>
         </is>
       </c>
       <c r="C685" s="10" t="inlineStr">
         <is>
-          <t>James Cameron</t>
+          <t>Michael Bay</t>
         </is>
       </c>
       <c r="D685" s="10" t="n">
-        <v>2009</v>
+        <v>2011</v>
       </c>
       <c r="E685" s="10" t="n">
-        <v>3.77</v>
+        <v>2.88</v>
       </c>
       <c r="F685" s="10" t="n">
-        <v>74</v>
+        <v>59</v>
       </c>
       <c r="I685" s="10" t="n">
-        <v>2924000000</v>
+        <v>1124000000</v>
       </c>
       <c r="J685" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K685" s="10" t="n">
-        <v>237000000</v>
+        <v>195000000</v>
       </c>
       <c r="L685" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M685" s="10" t="n">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="N685" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O685" s="10" t="n">
         <v>0</v>
@@ -35816,45 +35831,45 @@
     <row r="686">
       <c r="A686" s="10" t="inlineStr">
         <is>
-          <t>Avatar: The Way of Water</t>
+          <t>Transformers: Age of Extinction</t>
         </is>
       </c>
       <c r="B686" s="10" t="inlineStr">
         <is>
-          <t>card_685</t>
+          <t>card_690</t>
         </is>
       </c>
       <c r="C686" s="10" t="inlineStr">
         <is>
-          <t>James Cameron</t>
+          <t>Michael Bay</t>
         </is>
       </c>
       <c r="D686" s="10" t="n">
-        <v>2022</v>
+        <v>2014</v>
       </c>
       <c r="E686" s="10" t="n">
-        <v>3.65</v>
+        <v>2.32</v>
       </c>
       <c r="F686" s="10" t="n">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="I686" s="10" t="n">
-        <v>2334000000</v>
+        <v>1105000000</v>
       </c>
       <c r="J686" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K686" s="10" t="n">
-        <v>400000000</v>
+        <v>210000000</v>
       </c>
       <c r="L686" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M686" s="10" t="n">
-        <v>192</v>
+        <v>165</v>
       </c>
       <c r="N686" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O686" s="10" t="n">
         <v>0</v>
@@ -35866,45 +35881,45 @@
     <row r="687">
       <c r="A687" s="10" t="inlineStr">
         <is>
-          <t>Avatar: Fire and Ash</t>
+          <t>Transformers: The Last Knight</t>
         </is>
       </c>
       <c r="B687" s="10" t="inlineStr">
         <is>
-          <t>card_686</t>
+          <t>card_691</t>
         </is>
       </c>
       <c r="C687" s="10" t="inlineStr">
         <is>
-          <t>James Cameron</t>
+          <t>Michael Bay</t>
         </is>
       </c>
       <c r="D687" s="10" t="n">
-        <v>2025</v>
+        <v>2017</v>
       </c>
       <c r="E687" s="10" t="n">
-        <v>3.55</v>
+        <v>2.13</v>
       </c>
       <c r="F687" s="10" t="n">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="I687" s="10" t="n">
-        <v>1490000000</v>
+        <v>605400000</v>
       </c>
       <c r="J687" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K687" s="10" t="n">
-        <v>375000000</v>
+        <v>217000000</v>
       </c>
       <c r="L687" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M687" s="10" t="n">
-        <v>197</v>
+        <v>149</v>
       </c>
       <c r="N687" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O687" s="10" t="n">
         <v>0</v>
@@ -35916,42 +35931,42 @@
     <row r="688">
       <c r="A688" s="10" t="inlineStr">
         <is>
-          <t>Transformers</t>
+          <t>Bumblebee</t>
         </is>
       </c>
       <c r="B688" s="10" t="inlineStr">
         <is>
-          <t>card_687</t>
+          <t>card_692</t>
         </is>
       </c>
       <c r="C688" s="10" t="inlineStr">
         <is>
-          <t>Michael Bay</t>
+          <t>Travis Knight</t>
         </is>
       </c>
       <c r="D688" s="10" t="n">
-        <v>2007</v>
+        <v>2018</v>
       </c>
       <c r="E688" s="10" t="n">
-        <v>3.4</v>
+        <v>3.21</v>
       </c>
       <c r="F688" s="10" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="I688" s="10" t="n">
-        <v>709700000</v>
+        <v>468000000</v>
       </c>
       <c r="J688" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K688" s="10" t="n">
-        <v>150000000</v>
+        <v>135000000</v>
       </c>
       <c r="L688" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M688" s="10" t="n">
-        <v>143</v>
+        <v>114</v>
       </c>
       <c r="N688" s="10" t="n">
         <v>0</v>
@@ -35966,30 +35981,30 @@
     <row r="689">
       <c r="A689" s="10" t="inlineStr">
         <is>
-          <t>Transformers: Revenge of the Fallen</t>
+          <t>Transformers: Rise of the Beasts</t>
         </is>
       </c>
       <c r="B689" s="10" t="inlineStr">
         <is>
-          <t>card_688</t>
+          <t>card_693</t>
         </is>
       </c>
       <c r="C689" s="10" t="inlineStr">
         <is>
-          <t>Michael Bay</t>
+          <t>Steven Caple Jr.</t>
         </is>
       </c>
       <c r="D689" s="10" t="n">
-        <v>2009</v>
+        <v>2023</v>
       </c>
       <c r="E689" s="10" t="n">
-        <v>2.77</v>
+        <v>2.68</v>
       </c>
       <c r="F689" s="10" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="I689" s="10" t="n">
-        <v>836500000</v>
+        <v>441700000</v>
       </c>
       <c r="J689" s="10" t="b">
         <v>0</v>
@@ -36001,7 +36016,7 @@
         <v>0</v>
       </c>
       <c r="M689" s="10" t="n">
-        <v>150</v>
+        <v>127</v>
       </c>
       <c r="N689" s="10" t="n">
         <v>0</v>
@@ -36016,42 +36031,39 @@
     <row r="690">
       <c r="A690" s="10" t="inlineStr">
         <is>
-          <t>Transformers: Dark of the Moon</t>
+          <t>Grave of the Fireflies</t>
         </is>
       </c>
       <c r="B690" s="10" t="inlineStr">
         <is>
-          <t>card_689</t>
+          <t>card_694</t>
         </is>
       </c>
       <c r="C690" s="10" t="inlineStr">
         <is>
-          <t>Michael Bay</t>
+          <t>Isao Takahata</t>
         </is>
       </c>
       <c r="D690" s="10" t="n">
-        <v>2011</v>
+        <v>1988</v>
       </c>
       <c r="E690" s="10" t="n">
-        <v>2.88</v>
-      </c>
-      <c r="F690" s="10" t="n">
-        <v>59</v>
+        <v>4.48</v>
       </c>
       <c r="I690" s="10" t="n">
-        <v>1124000000</v>
+        <v>17000000</v>
       </c>
       <c r="J690" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K690" s="10" t="n">
-        <v>195000000</v>
+        <v>3700000</v>
       </c>
       <c r="L690" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M690" s="10" t="n">
-        <v>154</v>
+        <v>89</v>
       </c>
       <c r="N690" s="10" t="n">
         <v>0</v>
@@ -36066,42 +36078,42 @@
     <row r="691">
       <c r="A691" s="10" t="inlineStr">
         <is>
-          <t>Transformers: Age of Extinction</t>
+          <t>Kiki's Delivery Service</t>
         </is>
       </c>
       <c r="B691" s="10" t="inlineStr">
         <is>
-          <t>card_690</t>
+          <t>card_695</t>
         </is>
       </c>
       <c r="C691" s="10" t="inlineStr">
         <is>
-          <t>Michael Bay</t>
+          <t>Hayao Miyazaki</t>
         </is>
       </c>
       <c r="D691" s="10" t="n">
-        <v>2014</v>
+        <v>1989</v>
       </c>
       <c r="E691" s="10" t="n">
-        <v>2.32</v>
+        <v>4.15</v>
       </c>
       <c r="F691" s="10" t="n">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="I691" s="10" t="n">
-        <v>1105000000</v>
+        <v>41800000</v>
       </c>
       <c r="J691" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K691" s="10" t="n">
-        <v>210000000</v>
+        <v>6900000</v>
       </c>
       <c r="L691" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M691" s="10" t="n">
-        <v>165</v>
+        <v>102</v>
       </c>
       <c r="N691" s="10" t="n">
         <v>0</v>
@@ -36116,42 +36128,39 @@
     <row r="692">
       <c r="A692" s="10" t="inlineStr">
         <is>
-          <t>Transformers: The Last Knight</t>
+          <t>Only Yesterday</t>
         </is>
       </c>
       <c r="B692" s="10" t="inlineStr">
         <is>
-          <t>card_691</t>
+          <t>card_696</t>
         </is>
       </c>
       <c r="C692" s="10" t="inlineStr">
         <is>
-          <t>Michael Bay</t>
+          <t>Isao Takahata</t>
         </is>
       </c>
       <c r="D692" s="10" t="n">
-        <v>2017</v>
+        <v>1991</v>
       </c>
       <c r="E692" s="10" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="F692" s="10" t="n">
-        <v>41</v>
+        <v>3.91</v>
       </c>
       <c r="I692" s="10" t="n">
-        <v>605400000</v>
+        <v>26500000</v>
       </c>
       <c r="J692" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K692" s="10" t="n">
-        <v>217000000</v>
+        <v>4000000</v>
       </c>
       <c r="L692" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M692" s="10" t="n">
-        <v>149</v>
+        <v>118</v>
       </c>
       <c r="N692" s="10" t="n">
         <v>0</v>
@@ -36166,42 +36175,42 @@
     <row r="693">
       <c r="A693" s="10" t="inlineStr">
         <is>
-          <t>Bumblebee</t>
+          <t>Porco Rosso</t>
         </is>
       </c>
       <c r="B693" s="10" t="inlineStr">
         <is>
-          <t>card_692</t>
+          <t>card_697</t>
         </is>
       </c>
       <c r="C693" s="10" t="inlineStr">
         <is>
-          <t>Travis Knight</t>
+          <t>Hayao Miyazaki</t>
         </is>
       </c>
       <c r="D693" s="10" t="n">
-        <v>2018</v>
+        <v>1992</v>
       </c>
       <c r="E693" s="10" t="n">
-        <v>3.21</v>
+        <v>4.04</v>
       </c>
       <c r="F693" s="10" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="I693" s="10" t="n">
-        <v>468000000</v>
+        <v>44600000</v>
       </c>
       <c r="J693" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K693" s="10" t="n">
-        <v>135000000</v>
+        <v>1800000</v>
       </c>
       <c r="L693" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M693" s="10" t="n">
-        <v>114</v>
+        <v>94</v>
       </c>
       <c r="N693" s="10" t="n">
         <v>0</v>
@@ -36216,42 +36225,42 @@
     <row r="694">
       <c r="A694" s="10" t="inlineStr">
         <is>
-          <t>Transformers: Rise of the Beasts</t>
+          <t>Pom Poko</t>
         </is>
       </c>
       <c r="B694" s="10" t="inlineStr">
         <is>
-          <t>card_693</t>
+          <t>card_698</t>
         </is>
       </c>
       <c r="C694" s="10" t="inlineStr">
         <is>
-          <t>Steven Caple Jr.</t>
+          <t>Isao Takahata</t>
         </is>
       </c>
       <c r="D694" s="10" t="n">
-        <v>2023</v>
+        <v>1994</v>
       </c>
       <c r="E694" s="10" t="n">
-        <v>2.68</v>
+        <v>3.71</v>
       </c>
       <c r="F694" s="10" t="n">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="I694" s="10" t="n">
-        <v>441700000</v>
+        <v>41800000</v>
       </c>
       <c r="J694" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K694" s="10" t="n">
-        <v>200000000</v>
+        <v>20000000</v>
       </c>
       <c r="L694" s="10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M694" s="10" t="n">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="N694" s="10" t="n">
         <v>0</v>
@@ -36266,39 +36275,42 @@
     <row r="695">
       <c r="A695" s="10" t="inlineStr">
         <is>
-          <t>Grave of the Fireflies</t>
+          <t>Whisper of the Heart</t>
         </is>
       </c>
       <c r="B695" s="10" t="inlineStr">
         <is>
-          <t>card_694</t>
+          <t>card_699</t>
         </is>
       </c>
       <c r="C695" s="10" t="inlineStr">
         <is>
-          <t>Isao Takahata</t>
+          <t>Yoshifumi Kondo</t>
         </is>
       </c>
       <c r="D695" s="10" t="n">
-        <v>1988</v>
+        <v>1995</v>
       </c>
       <c r="E695" s="10" t="n">
-        <v>4.48</v>
+        <v>4.19</v>
+      </c>
+      <c r="F695" s="10" t="n">
+        <v>81</v>
       </c>
       <c r="I695" s="10" t="n">
-        <v>17000000</v>
+        <v>34900000</v>
       </c>
       <c r="J695" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K695" s="10" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="L695" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="K695" s="10" t="n">
-        <v>3700000</v>
-      </c>
-      <c r="L695" s="10" t="b">
-        <v>0</v>
-      </c>
       <c r="M695" s="10" t="n">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="N695" s="10" t="n">
         <v>0</v>
@@ -36313,12 +36325,12 @@
     <row r="696">
       <c r="A696" s="10" t="inlineStr">
         <is>
-          <t>Kiki's Delivery Service</t>
+          <t>Spirited Away</t>
         </is>
       </c>
       <c r="B696" s="10" t="inlineStr">
         <is>
-          <t>card_695</t>
+          <t>card_700</t>
         </is>
       </c>
       <c r="C696" s="10" t="inlineStr">
@@ -36327,31 +36339,31 @@
         </is>
       </c>
       <c r="D696" s="10" t="n">
-        <v>1989</v>
+        <v>2001</v>
       </c>
       <c r="E696" s="10" t="n">
-        <v>4.15</v>
+        <v>4.43</v>
       </c>
       <c r="F696" s="10" t="n">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="I696" s="10" t="n">
-        <v>41800000</v>
+        <v>396000000</v>
       </c>
       <c r="J696" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K696" s="10" t="n">
-        <v>6900000</v>
+        <v>19200000</v>
       </c>
       <c r="L696" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M696" s="10" t="n">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="N696" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O696" s="10" t="n">
         <v>0</v>
@@ -36363,39 +36375,39 @@
     <row r="697">
       <c r="A697" s="10" t="inlineStr">
         <is>
-          <t>Only Yesterday</t>
+          <t>The Cat Returns</t>
         </is>
       </c>
       <c r="B697" s="10" t="inlineStr">
         <is>
-          <t>card_696</t>
+          <t>card_701</t>
         </is>
       </c>
       <c r="C697" s="10" t="inlineStr">
         <is>
-          <t>Isao Takahata</t>
+          <t>Hiroyuki Morita</t>
         </is>
       </c>
       <c r="D697" s="10" t="n">
-        <v>1991</v>
+        <v>2002</v>
       </c>
       <c r="E697" s="10" t="n">
-        <v>3.91</v>
+        <v>3.66</v>
       </c>
       <c r="I697" s="10" t="n">
-        <v>26500000</v>
+        <v>65000000</v>
       </c>
       <c r="J697" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K697" s="10" t="n">
-        <v>4000000</v>
+        <v>20000000</v>
       </c>
       <c r="L697" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M697" s="10" t="n">
-        <v>118</v>
+        <v>75</v>
       </c>
       <c r="N697" s="10" t="n">
         <v>0</v>
@@ -36410,12 +36422,12 @@
     <row r="698">
       <c r="A698" s="10" t="inlineStr">
         <is>
-          <t>Porco Rosso</t>
+          <t>Ponyo</t>
         </is>
       </c>
       <c r="B698" s="10" t="inlineStr">
         <is>
-          <t>card_697</t>
+          <t>card_702</t>
         </is>
       </c>
       <c r="C698" s="10" t="inlineStr">
@@ -36424,28 +36436,28 @@
         </is>
       </c>
       <c r="D698" s="10" t="n">
-        <v>1992</v>
+        <v>2008</v>
       </c>
       <c r="E698" s="10" t="n">
-        <v>4.04</v>
+        <v>4.13</v>
       </c>
       <c r="F698" s="10" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="I698" s="10" t="n">
-        <v>44600000</v>
+        <v>205900000</v>
       </c>
       <c r="J698" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K698" s="10" t="n">
-        <v>1800000</v>
+        <v>34000000</v>
       </c>
       <c r="L698" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M698" s="10" t="n">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="N698" s="10" t="n">
         <v>0</v>
@@ -36460,42 +36472,42 @@
     <row r="699">
       <c r="A699" s="10" t="inlineStr">
         <is>
-          <t>Pom Poko</t>
+          <t>The Secret World of Arrietty</t>
         </is>
       </c>
       <c r="B699" s="10" t="inlineStr">
         <is>
-          <t>card_698</t>
+          <t>card_703</t>
         </is>
       </c>
       <c r="C699" s="10" t="inlineStr">
         <is>
-          <t>Isao Takahata</t>
+          <t>Hiromasa Yonebayashi</t>
         </is>
       </c>
       <c r="D699" s="10" t="n">
-        <v>1994</v>
+        <v>2010</v>
       </c>
       <c r="E699" s="10" t="n">
-        <v>3.71</v>
+        <v>3.88</v>
       </c>
       <c r="F699" s="10" t="n">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="I699" s="10" t="n">
-        <v>41800000</v>
+        <v>149000000</v>
       </c>
       <c r="J699" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K699" s="10" t="n">
-        <v>20000000</v>
+        <v>23000000</v>
       </c>
       <c r="L699" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M699" s="10" t="n">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="N699" s="10" t="n">
         <v>0</v>
@@ -36510,42 +36522,42 @@
     <row r="700">
       <c r="A700" s="10" t="inlineStr">
         <is>
-          <t>Whisper of the Heart</t>
+          <t>From Up on Poppy Hill</t>
         </is>
       </c>
       <c r="B700" s="10" t="inlineStr">
         <is>
-          <t>card_699</t>
+          <t>card_704</t>
         </is>
       </c>
       <c r="C700" s="10" t="inlineStr">
         <is>
-          <t>Yoshifumi Kondo</t>
+          <t>Goro Miyazaki</t>
         </is>
       </c>
       <c r="D700" s="10" t="n">
-        <v>1995</v>
+        <v>2011</v>
       </c>
       <c r="E700" s="10" t="n">
-        <v>4.19</v>
+        <v>3.76</v>
       </c>
       <c r="F700" s="10" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="I700" s="10" t="n">
-        <v>34900000</v>
+        <v>61500000</v>
       </c>
       <c r="J700" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K700" s="10" t="n">
-        <v>15000000</v>
+        <v>22000000</v>
       </c>
       <c r="L700" s="10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M700" s="10" t="n">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="N700" s="10" t="n">
         <v>0</v>
@@ -36560,12 +36572,12 @@
     <row r="701">
       <c r="A701" s="10" t="inlineStr">
         <is>
-          <t>Spirited Away</t>
+          <t>The Wind Rises</t>
         </is>
       </c>
       <c r="B701" s="10" t="inlineStr">
         <is>
-          <t>card_700</t>
+          <t>card_705</t>
         </is>
       </c>
       <c r="C701" s="10" t="inlineStr">
@@ -36574,383 +36586,136 @@
         </is>
       </c>
       <c r="D701" s="10" t="n">
-        <v>2001</v>
+        <v>2013</v>
       </c>
       <c r="E701" s="10" t="n">
-        <v>4.43</v>
+        <v>4.13</v>
       </c>
       <c r="F701" s="10" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="I701" s="10" t="n">
-        <v>396000000</v>
+        <v>136500000</v>
       </c>
       <c r="J701" s="10" t="b">
         <v>0</v>
       </c>
       <c r="K701" s="10" t="n">
-        <v>19200000</v>
+        <v>30000000</v>
       </c>
       <c r="L701" s="10" t="b">
         <v>0</v>
       </c>
       <c r="M701" s="10" t="n">
+        <v>126</v>
+      </c>
+      <c r="N701" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O701" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P701" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="10" t="inlineStr">
+        <is>
+          <t>When Marnie Was There</t>
+        </is>
+      </c>
+      <c r="B702" s="10" t="inlineStr">
+        <is>
+          <t>card_706</t>
+        </is>
+      </c>
+      <c r="C702" s="10" t="inlineStr">
+        <is>
+          <t>Hiromasa Yonebayashi</t>
+        </is>
+      </c>
+      <c r="D702" s="10" t="n">
+        <v>2014</v>
+      </c>
+      <c r="E702" s="10" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="F702" s="10" t="n">
+        <v>79</v>
+      </c>
+      <c r="I702" s="10" t="n">
+        <v>35700000</v>
+      </c>
+      <c r="J702" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K702" s="10" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="L702" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M702" s="10" t="n">
+        <v>103</v>
+      </c>
+      <c r="N702" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O702" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P702" s="10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="10" t="inlineStr">
+        <is>
+          <t>The Boy and the Heron</t>
+        </is>
+      </c>
+      <c r="B703" s="10" t="inlineStr">
+        <is>
+          <t>card_707</t>
+        </is>
+      </c>
+      <c r="C703" s="10" t="inlineStr">
+        <is>
+          <t>Hayao Miyazaki</t>
+        </is>
+      </c>
+      <c r="D703" s="10" t="n">
+        <v>2023</v>
+      </c>
+      <c r="E703" s="10" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F703" s="10" t="n">
+        <v>78</v>
+      </c>
+      <c r="I703" s="10" t="n">
+        <v>294200000</v>
+      </c>
+      <c r="J703" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K703" s="10" t="n">
+        <v>53000000</v>
+      </c>
+      <c r="L703" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M703" s="10" t="n">
         <v>124</v>
       </c>
-      <c r="N701" s="10" t="n">
+      <c r="N703" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="O701" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P701" s="10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="702">
-      <c r="A702" t="inlineStr">
-        <is>
-          <t>The Cat Returns</t>
-        </is>
-      </c>
-      <c r="B702" t="inlineStr">
-        <is>
-          <t>card_701</t>
-        </is>
-      </c>
-      <c r="C702" t="inlineStr">
-        <is>
-          <t>Hiroyuki Morita</t>
-        </is>
-      </c>
-      <c r="D702" t="n">
-        <v>2002</v>
-      </c>
-      <c r="E702" t="n">
-        <v>3.66</v>
-      </c>
-      <c r="I702" t="n">
-        <v>65000000</v>
-      </c>
-      <c r="J702" t="b">
-        <v>0</v>
-      </c>
-      <c r="K702" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="L702" t="b">
-        <v>0</v>
-      </c>
-      <c r="M702" t="n">
-        <v>75</v>
-      </c>
-      <c r="N702" t="n">
-        <v>0</v>
-      </c>
-      <c r="O702" t="n">
-        <v>0</v>
-      </c>
-      <c r="P702" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="703">
-      <c r="A703" t="inlineStr">
-        <is>
-          <t>Ponyo</t>
-        </is>
-      </c>
-      <c r="B703" t="inlineStr">
-        <is>
-          <t>card_702</t>
-        </is>
-      </c>
-      <c r="C703" t="inlineStr">
-        <is>
-          <t>Hayao Miyazaki</t>
-        </is>
-      </c>
-      <c r="D703" t="n">
-        <v>2008</v>
-      </c>
-      <c r="E703" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="F703" t="n">
-        <v>78</v>
-      </c>
-      <c r="I703" t="n">
-        <v>205900000</v>
-      </c>
-      <c r="J703" t="b">
-        <v>0</v>
-      </c>
-      <c r="K703" t="n">
-        <v>34000000</v>
-      </c>
-      <c r="L703" t="b">
-        <v>0</v>
-      </c>
-      <c r="M703" t="n">
-        <v>101</v>
-      </c>
-      <c r="N703" t="n">
-        <v>0</v>
-      </c>
-      <c r="O703" t="n">
-        <v>0</v>
-      </c>
-      <c r="P703" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="704">
-      <c r="A704" t="inlineStr">
-        <is>
-          <t>The Secret World of Arrietty</t>
-        </is>
-      </c>
-      <c r="B704" t="inlineStr">
-        <is>
-          <t>card_703</t>
-        </is>
-      </c>
-      <c r="C704" t="inlineStr">
-        <is>
-          <t>Hiromasa Yonebayashi</t>
-        </is>
-      </c>
-      <c r="D704" t="n">
-        <v>2010</v>
-      </c>
-      <c r="E704" t="n">
-        <v>3.88</v>
-      </c>
-      <c r="F704" t="n">
-        <v>81</v>
-      </c>
-      <c r="I704" t="n">
-        <v>149000000</v>
-      </c>
-      <c r="J704" t="b">
-        <v>0</v>
-      </c>
-      <c r="K704" t="n">
-        <v>23000000</v>
-      </c>
-      <c r="L704" t="b">
-        <v>0</v>
-      </c>
-      <c r="M704" t="n">
-        <v>95</v>
-      </c>
-      <c r="N704" t="n">
-        <v>0</v>
-      </c>
-      <c r="O704" t="n">
-        <v>0</v>
-      </c>
-      <c r="P704" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="705">
-      <c r="A705" t="inlineStr">
-        <is>
-          <t>From Up on Poppy Hill</t>
-        </is>
-      </c>
-      <c r="B705" t="inlineStr">
-        <is>
-          <t>card_704</t>
-        </is>
-      </c>
-      <c r="C705" t="inlineStr">
-        <is>
-          <t>Goro Miyazaki</t>
-        </is>
-      </c>
-      <c r="D705" t="n">
-        <v>2011</v>
-      </c>
-      <c r="E705" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="F705" t="n">
-        <v>76</v>
-      </c>
-      <c r="I705" t="n">
-        <v>61500000</v>
-      </c>
-      <c r="J705" t="b">
-        <v>0</v>
-      </c>
-      <c r="K705" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="L705" t="b">
-        <v>0</v>
-      </c>
-      <c r="M705" t="n">
-        <v>92</v>
-      </c>
-      <c r="N705" t="n">
-        <v>0</v>
-      </c>
-      <c r="O705" t="n">
-        <v>0</v>
-      </c>
-      <c r="P705" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="706">
-      <c r="A706" t="inlineStr">
-        <is>
-          <t>The Wind Rises</t>
-        </is>
-      </c>
-      <c r="B706" t="inlineStr">
-        <is>
-          <t>card_705</t>
-        </is>
-      </c>
-      <c r="C706" t="inlineStr">
-        <is>
-          <t>Hayao Miyazaki</t>
-        </is>
-      </c>
-      <c r="D706" t="n">
-        <v>2013</v>
-      </c>
-      <c r="E706" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="F706" t="n">
-        <v>83</v>
-      </c>
-      <c r="I706" t="n">
-        <v>136500000</v>
-      </c>
-      <c r="J706" t="b">
-        <v>0</v>
-      </c>
-      <c r="K706" t="n">
-        <v>30000000</v>
-      </c>
-      <c r="L706" t="b">
-        <v>0</v>
-      </c>
-      <c r="M706" t="n">
-        <v>126</v>
-      </c>
-      <c r="N706" t="n">
-        <v>0</v>
-      </c>
-      <c r="O706" t="n">
-        <v>0</v>
-      </c>
-      <c r="P706" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="707">
-      <c r="A707" t="inlineStr">
-        <is>
-          <t>When Marnie Was There</t>
-        </is>
-      </c>
-      <c r="B707" t="inlineStr">
-        <is>
-          <t>card_706</t>
-        </is>
-      </c>
-      <c r="C707" t="inlineStr">
-        <is>
-          <t>Hiromasa Yonebayashi</t>
-        </is>
-      </c>
-      <c r="D707" t="n">
-        <v>2014</v>
-      </c>
-      <c r="E707" t="n">
-        <v>3.91</v>
-      </c>
-      <c r="F707" t="n">
-        <v>79</v>
-      </c>
-      <c r="I707" t="n">
-        <v>35700000</v>
-      </c>
-      <c r="J707" t="b">
-        <v>0</v>
-      </c>
-      <c r="K707" t="n">
-        <v>10500000</v>
-      </c>
-      <c r="L707" t="b">
-        <v>0</v>
-      </c>
-      <c r="M707" t="n">
-        <v>103</v>
-      </c>
-      <c r="N707" t="n">
-        <v>0</v>
-      </c>
-      <c r="O707" t="n">
-        <v>0</v>
-      </c>
-      <c r="P707" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="708">
-      <c r="A708" t="inlineStr">
-        <is>
-          <t>The Boy and the Heron</t>
-        </is>
-      </c>
-      <c r="B708" t="inlineStr">
-        <is>
-          <t>card_707</t>
-        </is>
-      </c>
-      <c r="C708" t="inlineStr">
-        <is>
-          <t>Hayao Miyazaki</t>
-        </is>
-      </c>
-      <c r="D708" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E708" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F708" t="n">
-        <v>78</v>
-      </c>
-      <c r="I708" t="n">
-        <v>294200000</v>
-      </c>
-      <c r="J708" t="b">
-        <v>0</v>
-      </c>
-      <c r="K708" t="n">
-        <v>53000000</v>
-      </c>
-      <c r="L708" t="b">
-        <v>0</v>
-      </c>
-      <c r="M708" t="n">
-        <v>124</v>
-      </c>
-      <c r="N708" t="n">
-        <v>1</v>
-      </c>
-      <c r="O708" t="n">
-        <v>0</v>
-      </c>
-      <c r="P708" t="b">
+      <c r="O703" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P703" s="10" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix two mis-recorded Metacritic user scores
One Hundred and One Dalmatians (1961) was 69, actual Metacritic user
score is 8.0/10 (80). Encanto was 40, actual is 6.9/10 (69). Found via
spot-check verification against live Metacritic pages; ~20 other
sampled scores all matched exactly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -32367,7 +32367,7 @@
         <v>3.75</v>
       </c>
       <c r="F615" s="10" t="n">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="I615" s="10" t="n">
         <v>303000000</v>
@@ -34367,7 +34367,7 @@
         <v>3.47</v>
       </c>
       <c r="F655" s="10" t="n">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="I655" s="10" t="n">
         <v>261300000</v>

</xml_diff>

<commit_message>
Fix 6 more mis-recorded Metacritic user scores
Full re-verification of all 352 newly-added Metacritic scores against
live Metacritic pages (search-based slug resolution, not guessed
slugs) turned up 6 more transcription errors beyond the 2 found
earlier:
- West Side Story (2021): 73 -> 69
- John Wick: Chapter 3 - Parabellum: 84 -> 77
- Mission: Impossible - Ghost Protocol: 79 -> 77
- Godzilla x Kong: The New Empire: 70 -> 67
- Robin Hood (1973): 63 -> 74
- Hercules (1997): 62 -> 79

344 of 352 checked scores matched exactly; the remaining 8 had no
Metacritic user-score page reachable and were left as-is.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/Movie_DB.xlsx
+++ b/source_data/Movie_DB.xlsx
@@ -19515,7 +19515,7 @@
         <v>3.63</v>
       </c>
       <c r="F357" s="10" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="I357" s="10" t="n">
         <v>76000000</v>
@@ -23091,7 +23091,7 @@
         <v>3.71</v>
       </c>
       <c r="F429" s="10" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="I429" s="10" t="n">
         <v>328300000</v>
@@ -24041,7 +24041,7 @@
         <v>3.76</v>
       </c>
       <c r="F448" s="10" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I448" s="10" t="n">
         <v>694700000</v>
@@ -27729,7 +27729,7 @@
         <v>2.72</v>
       </c>
       <c r="F522" s="10" t="n">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I522" s="10" t="n">
         <v>572500000</v>
@@ -32567,7 +32567,7 @@
         <v>3.77</v>
       </c>
       <c r="F619" s="10" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="I619" s="10" t="n">
         <v>33000000</v>
@@ -33167,7 +33167,7 @@
         <v>2.67</v>
       </c>
       <c r="F631" s="10" t="n">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="I631" s="10" t="n">
         <v>252700000</v>

</xml_diff>